<commit_message>
Atualização automática: devolucoes (15/09/2026 08:57)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5297,8 +5297,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5314,7 +5322,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5322,12 +5330,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5627,73 +5653,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5728,7 +5754,7 @@
       <c r="J2" t="s">
         <v>1513</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5772,7 +5798,7 @@
       <c r="J3" t="s">
         <v>1513</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5816,7 +5842,7 @@
       <c r="J4" t="s">
         <v>1513</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5834,7 +5860,7 @@
       <c r="R4" t="s">
         <v>1678</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5872,7 +5898,7 @@
       <c r="J5" t="s">
         <v>1514</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5922,7 +5948,7 @@
       <c r="J6" t="s">
         <v>1513</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5969,7 +5995,7 @@
       <c r="J7" t="s">
         <v>1513</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6016,7 +6042,7 @@
       <c r="J8" t="s">
         <v>1513</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6063,7 +6089,7 @@
       <c r="J9" t="s">
         <v>1513</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6110,7 +6136,7 @@
       <c r="J10" t="s">
         <v>1513</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6157,7 +6183,7 @@
       <c r="J11" t="s">
         <v>1513</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6204,7 +6230,7 @@
       <c r="J12" t="s">
         <v>1513</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6248,7 +6274,7 @@
       <c r="J13" t="s">
         <v>1513</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6266,7 +6292,7 @@
       <c r="R13" t="s">
         <v>1679</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6304,7 +6330,7 @@
       <c r="J14" t="s">
         <v>1513</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6322,7 +6348,7 @@
       <c r="R14" t="s">
         <v>1680</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6360,7 +6386,7 @@
       <c r="J15" t="s">
         <v>1513</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6378,7 +6404,7 @@
       <c r="R15" t="s">
         <v>1680</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6416,7 +6442,7 @@
       <c r="J16" t="s">
         <v>1513</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6460,7 +6486,7 @@
       <c r="J17" t="s">
         <v>1513</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6504,7 +6530,7 @@
       <c r="J18" t="s">
         <v>1513</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6522,7 +6548,7 @@
       <c r="R18" t="s">
         <v>1681</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6563,7 +6589,7 @@
       <c r="J19" t="s">
         <v>1513</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6607,7 +6633,7 @@
       <c r="J20" t="s">
         <v>1513</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6651,7 +6677,7 @@
       <c r="J21" t="s">
         <v>1513</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6669,7 +6695,7 @@
       <c r="R21" t="s">
         <v>1680</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6710,7 +6736,7 @@
       <c r="J22" t="s">
         <v>1513</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6728,7 +6754,7 @@
       <c r="R22" t="s">
         <v>1682</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6769,7 +6795,7 @@
       <c r="J23" t="s">
         <v>1513</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6787,7 +6813,7 @@
       <c r="R23" t="s">
         <v>1683</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6828,7 +6854,7 @@
       <c r="J24" t="s">
         <v>1513</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6872,7 +6898,7 @@
       <c r="J25" t="s">
         <v>1513</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6913,7 +6939,7 @@
       <c r="J26" t="s">
         <v>1515</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6931,7 +6957,7 @@
       <c r="R26" t="s">
         <v>1684</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6966,7 +6992,7 @@
       <c r="J27" t="s">
         <v>1513</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6984,7 +7010,7 @@
       <c r="R27" t="s">
         <v>1685</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7025,7 +7051,7 @@
       <c r="J28" t="s">
         <v>1513</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7069,7 +7095,7 @@
       <c r="J29" t="s">
         <v>1513</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7113,7 +7139,7 @@
       <c r="J30" t="s">
         <v>1513</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7157,7 +7183,7 @@
       <c r="J31" t="s">
         <v>1513</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7175,7 +7201,7 @@
       <c r="R31" t="s">
         <v>1686</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7216,7 +7242,7 @@
       <c r="J32" t="s">
         <v>1513</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7260,7 +7286,7 @@
       <c r="J33" t="s">
         <v>1513</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7278,7 +7304,7 @@
       <c r="R33" t="s">
         <v>1687</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7319,7 +7345,7 @@
       <c r="J34" t="s">
         <v>1513</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7363,7 +7389,7 @@
       <c r="J35" t="s">
         <v>1513</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7381,7 +7407,7 @@
       <c r="R35" t="s">
         <v>1688</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7422,7 +7448,7 @@
       <c r="J36" t="s">
         <v>1513</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7440,7 +7466,7 @@
       <c r="R36" t="s">
         <v>1688</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7481,7 +7507,7 @@
       <c r="J37" t="s">
         <v>1513</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7499,7 +7525,7 @@
       <c r="R37" t="s">
         <v>1688</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7540,7 +7566,7 @@
       <c r="J38" t="s">
         <v>1513</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7558,7 +7584,7 @@
       <c r="R38" t="s">
         <v>1688</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7599,7 +7625,7 @@
       <c r="J39" t="s">
         <v>1513</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7617,7 +7643,7 @@
       <c r="R39" t="s">
         <v>1688</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7658,7 +7684,7 @@
       <c r="J40" t="s">
         <v>1513</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7676,7 +7702,7 @@
       <c r="R40" t="s">
         <v>1689</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7717,7 +7743,7 @@
       <c r="J41" t="s">
         <v>1513</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7735,7 +7761,7 @@
       <c r="R41" t="s">
         <v>1680</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7773,7 +7799,7 @@
       <c r="J42" t="s">
         <v>1513</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7791,7 +7817,7 @@
       <c r="R42" t="s">
         <v>1688</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7832,7 +7858,7 @@
       <c r="J43" t="s">
         <v>1513</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7876,7 +7902,7 @@
       <c r="J44" t="s">
         <v>1513</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7894,7 +7920,7 @@
       <c r="R44" t="s">
         <v>1690</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7935,7 +7961,7 @@
       <c r="J45" t="s">
         <v>1513</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7953,7 +7979,7 @@
       <c r="R45" t="s">
         <v>1691</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7991,7 +8017,7 @@
       <c r="J46" t="s">
         <v>1513</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8035,7 +8061,7 @@
       <c r="J47" t="s">
         <v>1513</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8053,7 +8079,7 @@
       <c r="R47" t="s">
         <v>1692</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8094,7 +8120,7 @@
       <c r="J48" t="s">
         <v>1513</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8138,7 +8164,7 @@
       <c r="J49" t="s">
         <v>1513</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8182,7 +8208,7 @@
       <c r="J50" t="s">
         <v>1513</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8226,7 +8252,7 @@
       <c r="J51" t="s">
         <v>1513</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8273,7 +8299,7 @@
       <c r="J52" t="s">
         <v>1513</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8317,7 +8343,7 @@
       <c r="J53" t="s">
         <v>1513</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8361,7 +8387,7 @@
       <c r="J54" t="s">
         <v>1513</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8405,7 +8431,7 @@
       <c r="J55" t="s">
         <v>1513</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8455,7 +8481,7 @@
       <c r="J56" t="s">
         <v>1513</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8508,7 +8534,7 @@
       <c r="J57" t="s">
         <v>1513</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8558,7 +8584,7 @@
       <c r="J58" t="s">
         <v>1513</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8608,7 +8634,7 @@
       <c r="J59" t="s">
         <v>1513</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8626,7 +8652,7 @@
       <c r="R59" t="s">
         <v>1693</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8667,7 +8693,7 @@
       <c r="J60" t="s">
         <v>1513</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8711,7 +8737,7 @@
       <c r="J61" t="s">
         <v>1513</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8755,7 +8781,7 @@
       <c r="J62" t="s">
         <v>1513</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8799,7 +8825,7 @@
       <c r="J63" t="s">
         <v>1513</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8843,7 +8869,7 @@
       <c r="J64" t="s">
         <v>1513</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8887,7 +8913,7 @@
       <c r="J65" t="s">
         <v>1513</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8934,7 +8960,7 @@
       <c r="J66" t="s">
         <v>1513</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8952,7 +8978,7 @@
       <c r="R66" t="s">
         <v>1694</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8990,7 +9016,7 @@
       <c r="J67" t="s">
         <v>1513</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9034,7 +9060,7 @@
       <c r="J68" t="s">
         <v>1513</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9049,7 +9075,7 @@
       <c r="O68" t="s">
         <v>1597</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9093,7 +9119,7 @@
       <c r="J69" t="s">
         <v>1515</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9137,7 +9163,7 @@
       <c r="J70" t="s">
         <v>1513</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9181,7 +9207,7 @@
       <c r="J71" t="s">
         <v>1513</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9225,7 +9251,7 @@
       <c r="J72" t="s">
         <v>1513</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9269,7 +9295,7 @@
       <c r="J73" t="s">
         <v>1513</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9313,7 +9339,7 @@
       <c r="J74" t="s">
         <v>1513</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9357,7 +9383,7 @@
       <c r="J75" t="s">
         <v>1513</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9401,7 +9427,7 @@
       <c r="J76" t="s">
         <v>1513</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9419,7 +9445,7 @@
       <c r="R76" t="s">
         <v>1695</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9457,7 +9483,7 @@
       <c r="J77" t="s">
         <v>1513</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9475,7 +9501,7 @@
       <c r="R77" t="s">
         <v>1695</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9513,7 +9539,7 @@
       <c r="J78" t="s">
         <v>1513</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9531,7 +9557,7 @@
       <c r="R78" t="s">
         <v>1695</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9569,7 +9595,7 @@
       <c r="J79" t="s">
         <v>1513</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9587,7 +9613,7 @@
       <c r="R79" t="s">
         <v>1695</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9625,7 +9651,7 @@
       <c r="J80" t="s">
         <v>1513</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9669,7 +9695,7 @@
       <c r="J81" t="s">
         <v>1513</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9713,7 +9739,7 @@
       <c r="J82" t="s">
         <v>1513</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9757,7 +9783,7 @@
       <c r="J83" t="s">
         <v>1513</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9801,7 +9827,7 @@
       <c r="J84" t="s">
         <v>1513</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9845,7 +9871,7 @@
       <c r="J85" t="s">
         <v>1513</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9863,7 +9889,7 @@
       <c r="R85" t="s">
         <v>1696</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9901,7 +9927,7 @@
       <c r="J86" t="s">
         <v>1513</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9945,7 +9971,7 @@
       <c r="J87" t="s">
         <v>1513</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9963,7 +9989,7 @@
       <c r="R87" t="s">
         <v>1697</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10001,7 +10027,7 @@
       <c r="J88" t="s">
         <v>1513</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10045,7 +10071,7 @@
       <c r="J89" t="s">
         <v>1513</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10063,7 +10089,7 @@
       <c r="R89" t="s">
         <v>1698</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10098,7 +10124,7 @@
       <c r="J90" t="s">
         <v>1513</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10116,7 +10142,7 @@
       <c r="R90" t="s">
         <v>1699</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10151,7 +10177,7 @@
       <c r="J91" t="s">
         <v>1513</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10169,7 +10195,7 @@
       <c r="R91" t="s">
         <v>1683</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10207,7 +10233,7 @@
       <c r="J92" t="s">
         <v>1513</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10228,7 +10254,7 @@
       <c r="R92" t="s">
         <v>1683</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10269,7 +10295,7 @@
       <c r="J93" t="s">
         <v>1513</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10310,7 +10336,7 @@
       <c r="J94" t="s">
         <v>1513</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10354,7 +10380,7 @@
       <c r="J95" t="s">
         <v>1513</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10398,7 +10424,7 @@
       <c r="J96" t="s">
         <v>1513</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10416,7 +10442,7 @@
       <c r="R96" t="s">
         <v>1700</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10454,7 +10480,7 @@
       <c r="J97" t="s">
         <v>1513</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10469,7 +10495,7 @@
       <c r="R97" t="s">
         <v>1700</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10510,7 +10536,7 @@
       <c r="J98" t="s">
         <v>1513</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10528,7 +10554,7 @@
       <c r="R98" t="s">
         <v>1701</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10566,7 +10592,7 @@
       <c r="J99" t="s">
         <v>1513</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10584,7 +10610,7 @@
       <c r="R99" t="s">
         <v>1702</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10622,7 +10648,7 @@
       <c r="J100" t="s">
         <v>1513</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10663,7 +10689,7 @@
       <c r="J101" t="s">
         <v>1513</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10704,7 +10730,7 @@
       <c r="J102" t="s">
         <v>1513</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10745,7 +10771,7 @@
       <c r="J103" t="s">
         <v>1513</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10786,7 +10812,7 @@
       <c r="J104" t="s">
         <v>1513</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10827,7 +10853,7 @@
       <c r="J105" t="s">
         <v>1513</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10868,7 +10894,7 @@
       <c r="J106" t="s">
         <v>1513</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10909,7 +10935,7 @@
       <c r="J107" t="s">
         <v>1513</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10950,7 +10976,7 @@
       <c r="J108" t="s">
         <v>1513</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10991,7 +11017,7 @@
       <c r="J109" t="s">
         <v>1513</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11044,7 +11070,7 @@
       <c r="J110" t="s">
         <v>1513</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11100,7 +11126,7 @@
       <c r="J111" t="s">
         <v>1513</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11118,7 +11144,7 @@
       <c r="R111" t="s">
         <v>1704</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11156,7 +11182,7 @@
       <c r="J112" t="s">
         <v>1513</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11215,7 +11241,7 @@
       <c r="J113" t="s">
         <v>1513</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11259,7 +11285,7 @@
       <c r="J114" t="s">
         <v>1513</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11303,7 +11329,7 @@
       <c r="J115" t="s">
         <v>1513</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11321,7 +11347,7 @@
       <c r="R115" t="s">
         <v>1706</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11359,7 +11385,7 @@
       <c r="J116" t="s">
         <v>1513</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11418,7 +11444,7 @@
       <c r="J117" t="s">
         <v>1513</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11462,7 +11488,7 @@
       <c r="J118" t="s">
         <v>1513</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11509,7 +11535,7 @@
       <c r="J119" t="s">
         <v>1513</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11550,7 +11576,7 @@
       <c r="J120" t="s">
         <v>1513</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11594,7 +11620,7 @@
       <c r="J121" t="s">
         <v>1513</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11641,7 +11667,7 @@
       <c r="J122" t="s">
         <v>1513</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11691,7 +11717,7 @@
       <c r="J123" t="s">
         <v>1513</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11735,7 +11761,7 @@
       <c r="J124" t="s">
         <v>1513</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11779,7 +11805,7 @@
       <c r="J125" t="s">
         <v>1513</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11797,7 +11823,7 @@
       <c r="R125" t="s">
         <v>1708</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11832,7 +11858,7 @@
       <c r="J126" t="s">
         <v>1513</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11850,7 +11876,7 @@
       <c r="R126" t="s">
         <v>1709</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11885,7 +11911,7 @@
       <c r="J127" t="s">
         <v>1513</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11941,7 +11967,7 @@
       <c r="J128" t="s">
         <v>1513</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11982,7 +12008,7 @@
       <c r="J129" t="s">
         <v>1513</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12023,7 +12049,7 @@
       <c r="J130" t="s">
         <v>1513</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12064,7 +12090,7 @@
       <c r="J131" t="s">
         <v>1513</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12108,7 +12134,7 @@
       <c r="J132" t="s">
         <v>1513</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12149,7 +12175,7 @@
       <c r="J133" t="s">
         <v>1513</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12167,7 +12193,7 @@
       <c r="R133" t="s">
         <v>1695</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12202,7 +12228,7 @@
       <c r="J134" t="s">
         <v>1513</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12220,7 +12246,7 @@
       <c r="R134" t="s">
         <v>1695</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12255,7 +12281,7 @@
       <c r="J135" t="s">
         <v>1513</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12296,7 +12322,7 @@
       <c r="J136" t="s">
         <v>1513</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12337,7 +12363,7 @@
       <c r="J137" t="s">
         <v>1513</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12378,7 +12404,7 @@
       <c r="J138" t="s">
         <v>1513</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12419,7 +12445,7 @@
       <c r="J139" t="s">
         <v>1513</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12466,7 +12492,7 @@
       <c r="J140" t="s">
         <v>1513</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12507,7 +12533,7 @@
       <c r="J141" t="s">
         <v>1513</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12548,7 +12574,7 @@
       <c r="J142" t="s">
         <v>1513</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12592,7 +12618,7 @@
       <c r="J143" t="s">
         <v>1513</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12610,7 +12636,7 @@
       <c r="R143" t="s">
         <v>1695</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12645,7 +12671,7 @@
       <c r="J144" t="s">
         <v>1513</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12663,7 +12689,7 @@
       <c r="R144" t="s">
         <v>1695</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12698,7 +12724,7 @@
       <c r="J145" t="s">
         <v>1513</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12716,7 +12742,7 @@
       <c r="R145" t="s">
         <v>1695</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12751,7 +12777,7 @@
       <c r="J146" t="s">
         <v>1513</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12769,7 +12795,7 @@
       <c r="R146" t="s">
         <v>1703</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12804,7 +12830,7 @@
       <c r="J147" t="s">
         <v>1513</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12822,7 +12848,7 @@
       <c r="R147" t="s">
         <v>1710</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12857,7 +12883,7 @@
       <c r="J148" t="s">
         <v>1513</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12898,7 +12924,7 @@
       <c r="J149" t="s">
         <v>1513</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12916,7 +12942,7 @@
       <c r="R149" t="s">
         <v>1695</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12951,7 +12977,7 @@
       <c r="J150" t="s">
         <v>1513</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12969,7 +12995,7 @@
       <c r="R150" t="s">
         <v>1695</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13004,7 +13030,7 @@
       <c r="J151" t="s">
         <v>1513</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13022,7 +13048,7 @@
       <c r="R151" t="s">
         <v>1711</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13057,7 +13083,7 @@
       <c r="J152" t="s">
         <v>1513</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13075,7 +13101,7 @@
       <c r="R152" t="s">
         <v>1712</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13110,7 +13136,7 @@
       <c r="J153" t="s">
         <v>1513</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13119,7 +13145,7 @@
       <c r="M153" t="s">
         <v>1588</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13160,7 +13186,7 @@
       <c r="J154" t="s">
         <v>1513</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13201,7 +13227,7 @@
       <c r="J155" t="s">
         <v>1513</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13242,7 +13268,7 @@
       <c r="J156" t="s">
         <v>1513</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13283,7 +13309,7 @@
       <c r="J157" t="s">
         <v>1513</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13324,7 +13350,7 @@
       <c r="J158" t="s">
         <v>1513</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13365,7 +13391,7 @@
       <c r="J159" t="s">
         <v>1513</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13406,7 +13432,7 @@
       <c r="J160" t="s">
         <v>1513</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13447,7 +13473,7 @@
       <c r="J161" t="s">
         <v>1513</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13488,7 +13514,7 @@
       <c r="J162" t="s">
         <v>1513</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13506,7 +13532,7 @@
       <c r="R162" t="s">
         <v>1698</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13541,7 +13567,7 @@
       <c r="J163" t="s">
         <v>1513</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13559,7 +13585,7 @@
       <c r="R163" t="s">
         <v>1695</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13594,7 +13620,7 @@
       <c r="J164" t="s">
         <v>1513</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13638,7 +13664,7 @@
       <c r="J165" t="s">
         <v>1513</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13679,7 +13705,7 @@
       <c r="J166" t="s">
         <v>1513</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13697,7 +13723,7 @@
       <c r="R166" t="s">
         <v>1713</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13732,7 +13758,7 @@
       <c r="J167" t="s">
         <v>1513</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13776,7 +13802,7 @@
       <c r="J168" t="s">
         <v>1513</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13820,7 +13846,7 @@
       <c r="J169" t="s">
         <v>1513</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13861,7 +13887,7 @@
       <c r="J170" t="s">
         <v>1513</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13902,7 +13928,7 @@
       <c r="J171" t="s">
         <v>1513</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13943,7 +13969,7 @@
       <c r="J172" t="s">
         <v>1513</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13984,7 +14010,7 @@
       <c r="J173" t="s">
         <v>1513</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14025,7 +14051,7 @@
       <c r="J174" t="s">
         <v>1513</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14066,7 +14092,7 @@
       <c r="J175" t="s">
         <v>1513</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14107,7 +14133,7 @@
       <c r="J176" t="s">
         <v>1513</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14148,7 +14174,7 @@
       <c r="J177" t="s">
         <v>1513</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14189,7 +14215,7 @@
       <c r="J178" t="s">
         <v>1513</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14207,7 +14233,7 @@
       <c r="R178" t="s">
         <v>1711</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14242,7 +14268,7 @@
       <c r="J179" t="s">
         <v>1513</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14251,7 +14277,7 @@
       <c r="M179" t="s">
         <v>1585</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14292,7 +14318,7 @@
       <c r="J180" t="s">
         <v>1513</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14333,7 +14359,7 @@
       <c r="J181" t="s">
         <v>1513</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14351,7 +14377,7 @@
       <c r="R181" t="s">
         <v>1695</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14386,7 +14412,7 @@
       <c r="J182" t="s">
         <v>1513</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14427,7 +14453,7 @@
       <c r="J183" t="s">
         <v>1513</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14468,7 +14494,7 @@
       <c r="J184" t="s">
         <v>1513</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14509,7 +14535,7 @@
       <c r="J185" t="s">
         <v>1513</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14550,7 +14576,7 @@
       <c r="J186" t="s">
         <v>1513</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14591,7 +14617,7 @@
       <c r="J187" t="s">
         <v>1513</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14632,7 +14658,7 @@
       <c r="J188" t="s">
         <v>1513</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14673,7 +14699,7 @@
       <c r="J189" t="s">
         <v>1513</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14714,7 +14740,7 @@
       <c r="J190" t="s">
         <v>1513</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14755,7 +14781,7 @@
       <c r="J191" t="s">
         <v>1513</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14796,7 +14822,7 @@
       <c r="J192" t="s">
         <v>1513</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14837,7 +14863,7 @@
       <c r="J193" t="s">
         <v>1513</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14878,7 +14904,7 @@
       <c r="J194" t="s">
         <v>1513</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14919,7 +14945,7 @@
       <c r="J195" t="s">
         <v>1513</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14937,7 +14963,7 @@
       <c r="R195" t="s">
         <v>1704</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14975,7 +15001,7 @@
       <c r="J196" t="s">
         <v>1513</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14993,7 +15019,7 @@
       <c r="R196" t="s">
         <v>1710</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15031,7 +15057,7 @@
       <c r="J197" t="s">
         <v>1513</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15072,7 +15098,7 @@
       <c r="J198" t="s">
         <v>1515</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15113,7 +15139,7 @@
       <c r="J199" t="s">
         <v>1514</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15154,7 +15180,7 @@
       <c r="J200" t="s">
         <v>1513</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15195,7 +15221,7 @@
       <c r="J201" t="s">
         <v>1513</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15236,7 +15262,7 @@
       <c r="J202" t="s">
         <v>1513</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15254,7 +15280,7 @@
       <c r="R202" t="s">
         <v>1695</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15289,7 +15315,7 @@
       <c r="J203" t="s">
         <v>1513</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15307,7 +15333,7 @@
       <c r="R203" t="s">
         <v>1703</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15342,7 +15368,7 @@
       <c r="J204" t="s">
         <v>1513</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15357,7 +15383,7 @@
       <c r="R204" t="s">
         <v>1714</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15395,7 +15421,7 @@
       <c r="J205" t="s">
         <v>1513</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15413,7 +15439,7 @@
       <c r="R205" t="s">
         <v>1715</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15451,7 +15477,7 @@
       <c r="J206" t="s">
         <v>1513</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15469,7 +15495,7 @@
       <c r="R206" t="s">
         <v>1683</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15504,7 +15530,7 @@
       <c r="J207" t="s">
         <v>1513</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15545,7 +15571,7 @@
       <c r="J208" t="s">
         <v>1513</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15586,7 +15612,7 @@
       <c r="J209" t="s">
         <v>1513</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15627,7 +15653,7 @@
       <c r="J210" t="s">
         <v>1513</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15668,7 +15694,7 @@
       <c r="J211" t="s">
         <v>1513</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15709,7 +15735,7 @@
       <c r="J212" t="s">
         <v>1513</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15750,7 +15776,7 @@
       <c r="J213" t="s">
         <v>1513</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15791,7 +15817,7 @@
       <c r="J214" t="s">
         <v>1513</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15809,7 +15835,7 @@
       <c r="R214" t="s">
         <v>1716</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15844,7 +15870,7 @@
       <c r="J215" t="s">
         <v>1513</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15885,7 +15911,7 @@
       <c r="J216" t="s">
         <v>1513</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15926,7 +15952,7 @@
       <c r="J217" t="s">
         <v>1513</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15967,7 +15993,7 @@
       <c r="J218" t="s">
         <v>1513</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16008,7 +16034,7 @@
       <c r="J219" t="s">
         <v>1513</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16049,7 +16075,7 @@
       <c r="J220" t="s">
         <v>1513</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16090,7 +16116,7 @@
       <c r="J221" t="s">
         <v>1513</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16131,7 +16157,7 @@
       <c r="J222" t="s">
         <v>1513</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16172,7 +16198,7 @@
       <c r="J223" t="s">
         <v>1513</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16213,7 +16239,7 @@
       <c r="J224" t="s">
         <v>1513</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16254,7 +16280,7 @@
       <c r="J225" t="s">
         <v>1513</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16295,7 +16321,7 @@
       <c r="J226" t="s">
         <v>1513</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16336,7 +16362,7 @@
       <c r="J227" t="s">
         <v>1513</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16377,7 +16403,7 @@
       <c r="J228" t="s">
         <v>1513</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16418,7 +16444,7 @@
       <c r="J229" t="s">
         <v>1513</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16459,7 +16485,7 @@
       <c r="J230" t="s">
         <v>1513</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16500,7 +16526,7 @@
       <c r="J231" t="s">
         <v>1513</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16541,7 +16567,7 @@
       <c r="J232" t="s">
         <v>1513</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16582,7 +16608,7 @@
       <c r="J233" t="s">
         <v>1513</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16623,7 +16649,7 @@
       <c r="J234" t="s">
         <v>1513</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16664,7 +16690,7 @@
       <c r="J235" t="s">
         <v>1513</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16705,7 +16731,7 @@
       <c r="J236" t="s">
         <v>1513</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16746,7 +16772,7 @@
       <c r="J237" t="s">
         <v>1513</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16787,7 +16813,7 @@
       <c r="J238" t="s">
         <v>1513</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16828,7 +16854,7 @@
       <c r="J239" t="s">
         <v>1513</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16846,7 +16872,7 @@
       <c r="R239" t="s">
         <v>1710</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16881,7 +16907,7 @@
       <c r="J240" t="s">
         <v>1513</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16922,7 +16948,7 @@
       <c r="J241" t="s">
         <v>1513</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16963,7 +16989,7 @@
       <c r="J242" t="s">
         <v>1513</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16981,7 +17007,7 @@
       <c r="R242" t="s">
         <v>1703</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17016,7 +17042,7 @@
       <c r="J243" t="s">
         <v>1513</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17057,7 +17083,7 @@
       <c r="J244" t="s">
         <v>1513</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17098,7 +17124,7 @@
       <c r="J245" t="s">
         <v>1513</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17139,7 +17165,7 @@
       <c r="J246" t="s">
         <v>1513</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17157,7 +17183,7 @@
       <c r="R246" t="s">
         <v>1683</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17192,7 +17218,7 @@
       <c r="J247" t="s">
         <v>1513</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17233,7 +17259,7 @@
       <c r="J248" t="s">
         <v>1513</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17274,7 +17300,7 @@
       <c r="J249" t="s">
         <v>1513</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17315,7 +17341,7 @@
       <c r="J250" t="s">
         <v>1513</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17356,7 +17382,7 @@
       <c r="J251" t="s">
         <v>1513</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17397,7 +17423,7 @@
       <c r="J252" t="s">
         <v>1513</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17438,7 +17464,7 @@
       <c r="J253" t="s">
         <v>1513</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17456,7 +17482,7 @@
       <c r="R253" t="s">
         <v>1713</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17494,7 +17520,7 @@
       <c r="J254" t="s">
         <v>1513</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17535,7 +17561,7 @@
       <c r="J255" t="s">
         <v>1513</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17576,7 +17602,7 @@
       <c r="J256" t="s">
         <v>1513</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17585,7 +17611,7 @@
       <c r="M256" t="s">
         <v>1584</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17623,7 +17649,7 @@
       <c r="J257" t="s">
         <v>1513</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17632,7 +17658,7 @@
       <c r="M257" t="s">
         <v>1585</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17676,7 +17702,7 @@
       <c r="J258" t="s">
         <v>1513</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17694,7 +17720,7 @@
       <c r="R258" t="s">
         <v>1695</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17732,7 +17758,7 @@
       <c r="J259" t="s">
         <v>1513</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17750,7 +17776,7 @@
       <c r="R259" t="s">
         <v>1711</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17788,7 +17814,7 @@
       <c r="J260" t="s">
         <v>1513</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17797,7 +17823,7 @@
       <c r="M260" t="s">
         <v>1579</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17841,7 +17867,7 @@
       <c r="J261" t="s">
         <v>1513</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17859,7 +17885,7 @@
       <c r="R261" t="s">
         <v>1717</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17897,7 +17923,7 @@
       <c r="J262" t="s">
         <v>1513</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17915,7 +17941,7 @@
       <c r="R262" t="s">
         <v>1711</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17953,7 +17979,7 @@
       <c r="J263" t="s">
         <v>1513</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17962,7 +17988,7 @@
       <c r="M263" t="s">
         <v>1579</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18006,7 +18032,7 @@
       <c r="J264" t="s">
         <v>1513</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18047,7 +18073,7 @@
       <c r="J265" t="s">
         <v>1513</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18088,7 +18114,7 @@
       <c r="J266" t="s">
         <v>1513</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18129,7 +18155,7 @@
       <c r="J267" t="s">
         <v>1513</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18173,7 +18199,7 @@
       <c r="J268" t="s">
         <v>1513</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18214,7 +18240,7 @@
       <c r="J269" t="s">
         <v>1513</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18255,7 +18281,7 @@
       <c r="J270" t="s">
         <v>1513</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18296,7 +18322,7 @@
       <c r="J271" t="s">
         <v>1513</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18337,7 +18363,7 @@
       <c r="J272" t="s">
         <v>1513</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18355,7 +18381,7 @@
       <c r="R272" t="s">
         <v>1718</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18393,7 +18419,7 @@
       <c r="J273" t="s">
         <v>1513</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18437,7 +18463,7 @@
       <c r="J274" t="s">
         <v>1513</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18478,7 +18504,7 @@
       <c r="J275" t="s">
         <v>1513</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18519,7 +18545,7 @@
       <c r="J276" t="s">
         <v>1513</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18560,7 +18586,7 @@
       <c r="J277" t="s">
         <v>1513</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18601,7 +18627,7 @@
       <c r="J278" t="s">
         <v>1513</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18642,7 +18668,7 @@
       <c r="J279" t="s">
         <v>1513</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18683,7 +18709,7 @@
       <c r="J280" t="s">
         <v>1513</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18724,7 +18750,7 @@
       <c r="J281" t="s">
         <v>1513</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18765,7 +18791,7 @@
       <c r="J282" t="s">
         <v>1513</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18806,7 +18832,7 @@
       <c r="J283" t="s">
         <v>1513</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18847,7 +18873,7 @@
       <c r="J284" t="s">
         <v>1513</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18888,7 +18914,7 @@
       <c r="J285" t="s">
         <v>1513</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18929,7 +18955,7 @@
       <c r="J286" t="s">
         <v>1513</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18970,7 +18996,7 @@
       <c r="J287" t="s">
         <v>1513</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19011,7 +19037,7 @@
       <c r="J288" t="s">
         <v>1513</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19052,7 +19078,7 @@
       <c r="J289" t="s">
         <v>1513</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19093,7 +19119,7 @@
       <c r="J290" t="s">
         <v>1513</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19134,7 +19160,7 @@
       <c r="J291" t="s">
         <v>1513</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19175,7 +19201,7 @@
       <c r="J292" t="s">
         <v>1513</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19216,7 +19242,7 @@
       <c r="J293" t="s">
         <v>1513</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19257,7 +19283,7 @@
       <c r="J294" t="s">
         <v>1513</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19298,7 +19324,7 @@
       <c r="J295" t="s">
         <v>1513</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19316,7 +19342,7 @@
       <c r="R295" t="s">
         <v>1719</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19354,7 +19380,7 @@
       <c r="J296" t="s">
         <v>1513</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19372,7 +19398,7 @@
       <c r="R296" t="s">
         <v>1695</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19410,7 +19436,7 @@
       <c r="J297" t="s">
         <v>1513</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19451,7 +19477,7 @@
       <c r="J298" t="s">
         <v>1513</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19492,7 +19518,7 @@
       <c r="J299" t="s">
         <v>1514</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19533,7 +19559,7 @@
       <c r="J300" t="s">
         <v>1513</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19574,7 +19600,7 @@
       <c r="J301" t="s">
         <v>1513</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20412,7 +20438,7 @@
       <c r="R321" t="s">
         <v>1681</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20632,7 +20658,7 @@
       <c r="R326" t="s">
         <v>1720</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21467,7 +21493,7 @@
       <c r="R346" t="s">
         <v>1721</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (15/09/2026 14:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5284,7 +5284,7 @@
     <t>O ITEM FOI REVISADO E ENTREGUE PELA EMPRESA VIA  RECIBO 598/FAB/26</t>
   </si>
   <si>
-    <t>ESSE ITEM FOI REVISADO E ENTREGUE AO PAMALS VIA RECIBO</t>
+    <t>O ITEM ENVIADO PARA BAMN NÃO FOI ESSE PN E SIM O PN 200SGL11SQ VIA GMM 202667113025425 E ESSE PN FOI REVISADO E ENTREGUE AO PAMALS VIA RECIBO 438/FAB/26</t>
   </si>
   <si>
     <t>Pendente</t>
@@ -5303,8 +5303,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5320,7 +5328,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5328,12 +5336,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5633,73 +5659,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5734,7 +5760,7 @@
       <c r="J2" t="s">
         <v>1513</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5778,7 +5804,7 @@
       <c r="J3" t="s">
         <v>1513</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5822,7 +5848,7 @@
       <c r="J4" t="s">
         <v>1513</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5840,7 +5866,7 @@
       <c r="R4" t="s">
         <v>1678</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5878,7 +5904,7 @@
       <c r="J5" t="s">
         <v>1514</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5928,7 +5954,7 @@
       <c r="J6" t="s">
         <v>1513</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5975,7 +6001,7 @@
       <c r="J7" t="s">
         <v>1513</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6022,7 +6048,7 @@
       <c r="J8" t="s">
         <v>1513</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6069,7 +6095,7 @@
       <c r="J9" t="s">
         <v>1513</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6116,7 +6142,7 @@
       <c r="J10" t="s">
         <v>1513</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6163,7 +6189,7 @@
       <c r="J11" t="s">
         <v>1513</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6210,7 +6236,7 @@
       <c r="J12" t="s">
         <v>1513</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6254,7 +6280,7 @@
       <c r="J13" t="s">
         <v>1513</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6272,7 +6298,7 @@
       <c r="R13" t="s">
         <v>1679</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6310,7 +6336,7 @@
       <c r="J14" t="s">
         <v>1513</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6328,7 +6354,7 @@
       <c r="R14" t="s">
         <v>1680</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6366,7 +6392,7 @@
       <c r="J15" t="s">
         <v>1513</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6384,7 +6410,7 @@
       <c r="R15" t="s">
         <v>1680</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6422,7 +6448,7 @@
       <c r="J16" t="s">
         <v>1513</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6466,7 +6492,7 @@
       <c r="J17" t="s">
         <v>1513</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6510,7 +6536,7 @@
       <c r="J18" t="s">
         <v>1513</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6528,7 +6554,7 @@
       <c r="R18" t="s">
         <v>1681</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6569,7 +6595,7 @@
       <c r="J19" t="s">
         <v>1513</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6613,7 +6639,7 @@
       <c r="J20" t="s">
         <v>1513</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6657,7 +6683,7 @@
       <c r="J21" t="s">
         <v>1513</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6675,7 +6701,7 @@
       <c r="R21" t="s">
         <v>1680</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6716,7 +6742,7 @@
       <c r="J22" t="s">
         <v>1513</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6734,7 +6760,7 @@
       <c r="R22" t="s">
         <v>1682</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6775,7 +6801,7 @@
       <c r="J23" t="s">
         <v>1513</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6793,7 +6819,7 @@
       <c r="R23" t="s">
         <v>1683</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6834,7 +6860,7 @@
       <c r="J24" t="s">
         <v>1513</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6878,7 +6904,7 @@
       <c r="J25" t="s">
         <v>1513</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6919,7 +6945,7 @@
       <c r="J26" t="s">
         <v>1515</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6937,7 +6963,7 @@
       <c r="R26" t="s">
         <v>1684</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6972,7 +6998,7 @@
       <c r="J27" t="s">
         <v>1513</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6990,7 +7016,7 @@
       <c r="R27" t="s">
         <v>1685</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7031,7 +7057,7 @@
       <c r="J28" t="s">
         <v>1513</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7075,7 +7101,7 @@
       <c r="J29" t="s">
         <v>1513</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7119,7 +7145,7 @@
       <c r="J30" t="s">
         <v>1513</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7163,7 +7189,7 @@
       <c r="J31" t="s">
         <v>1513</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7181,7 +7207,7 @@
       <c r="R31" t="s">
         <v>1686</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7222,7 +7248,7 @@
       <c r="J32" t="s">
         <v>1513</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7266,7 +7292,7 @@
       <c r="J33" t="s">
         <v>1513</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7284,7 +7310,7 @@
       <c r="R33" t="s">
         <v>1687</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7325,7 +7351,7 @@
       <c r="J34" t="s">
         <v>1513</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7369,7 +7395,7 @@
       <c r="J35" t="s">
         <v>1513</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7387,7 +7413,7 @@
       <c r="R35" t="s">
         <v>1688</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7428,7 +7454,7 @@
       <c r="J36" t="s">
         <v>1513</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7446,7 +7472,7 @@
       <c r="R36" t="s">
         <v>1688</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7487,7 +7513,7 @@
       <c r="J37" t="s">
         <v>1513</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7505,7 +7531,7 @@
       <c r="R37" t="s">
         <v>1688</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7546,7 +7572,7 @@
       <c r="J38" t="s">
         <v>1513</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7564,7 +7590,7 @@
       <c r="R38" t="s">
         <v>1688</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7605,7 +7631,7 @@
       <c r="J39" t="s">
         <v>1513</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7623,7 +7649,7 @@
       <c r="R39" t="s">
         <v>1688</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7664,7 +7690,7 @@
       <c r="J40" t="s">
         <v>1513</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7682,7 +7708,7 @@
       <c r="R40" t="s">
         <v>1689</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7723,7 +7749,7 @@
       <c r="J41" t="s">
         <v>1513</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7741,7 +7767,7 @@
       <c r="R41" t="s">
         <v>1680</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7779,7 +7805,7 @@
       <c r="J42" t="s">
         <v>1513</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7797,7 +7823,7 @@
       <c r="R42" t="s">
         <v>1688</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7838,7 +7864,7 @@
       <c r="J43" t="s">
         <v>1513</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7882,7 +7908,7 @@
       <c r="J44" t="s">
         <v>1513</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7900,7 +7926,7 @@
       <c r="R44" t="s">
         <v>1690</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7941,7 +7967,7 @@
       <c r="J45" t="s">
         <v>1513</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7959,7 +7985,7 @@
       <c r="R45" t="s">
         <v>1691</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7997,7 +8023,7 @@
       <c r="J46" t="s">
         <v>1513</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8041,7 +8067,7 @@
       <c r="J47" t="s">
         <v>1513</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8059,7 +8085,7 @@
       <c r="R47" t="s">
         <v>1692</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8100,7 +8126,7 @@
       <c r="J48" t="s">
         <v>1513</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8144,7 +8170,7 @@
       <c r="J49" t="s">
         <v>1513</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8188,7 +8214,7 @@
       <c r="J50" t="s">
         <v>1513</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8232,7 +8258,7 @@
       <c r="J51" t="s">
         <v>1513</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8279,7 +8305,7 @@
       <c r="J52" t="s">
         <v>1513</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8323,7 +8349,7 @@
       <c r="J53" t="s">
         <v>1513</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8367,7 +8393,7 @@
       <c r="J54" t="s">
         <v>1513</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8411,7 +8437,7 @@
       <c r="J55" t="s">
         <v>1513</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8461,7 +8487,7 @@
       <c r="J56" t="s">
         <v>1513</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8514,7 +8540,7 @@
       <c r="J57" t="s">
         <v>1513</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8564,7 +8590,7 @@
       <c r="J58" t="s">
         <v>1513</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8614,7 +8640,7 @@
       <c r="J59" t="s">
         <v>1513</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8632,7 +8658,7 @@
       <c r="R59" t="s">
         <v>1693</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8673,7 +8699,7 @@
       <c r="J60" t="s">
         <v>1513</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8717,7 +8743,7 @@
       <c r="J61" t="s">
         <v>1513</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8761,7 +8787,7 @@
       <c r="J62" t="s">
         <v>1513</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8805,7 +8831,7 @@
       <c r="J63" t="s">
         <v>1513</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8849,7 +8875,7 @@
       <c r="J64" t="s">
         <v>1513</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8893,7 +8919,7 @@
       <c r="J65" t="s">
         <v>1513</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8940,7 +8966,7 @@
       <c r="J66" t="s">
         <v>1513</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8958,7 +8984,7 @@
       <c r="R66" t="s">
         <v>1694</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8996,7 +9022,7 @@
       <c r="J67" t="s">
         <v>1513</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9040,7 +9066,7 @@
       <c r="J68" t="s">
         <v>1513</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9055,7 +9081,7 @@
       <c r="O68" t="s">
         <v>1597</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9099,7 +9125,7 @@
       <c r="J69" t="s">
         <v>1515</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9143,7 +9169,7 @@
       <c r="J70" t="s">
         <v>1513</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9187,7 +9213,7 @@
       <c r="J71" t="s">
         <v>1513</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9231,7 +9257,7 @@
       <c r="J72" t="s">
         <v>1513</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9275,7 +9301,7 @@
       <c r="J73" t="s">
         <v>1513</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9319,7 +9345,7 @@
       <c r="J74" t="s">
         <v>1513</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9363,7 +9389,7 @@
       <c r="J75" t="s">
         <v>1513</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9407,7 +9433,7 @@
       <c r="J76" t="s">
         <v>1513</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9425,7 +9451,7 @@
       <c r="R76" t="s">
         <v>1695</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9463,7 +9489,7 @@
       <c r="J77" t="s">
         <v>1513</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9481,7 +9507,7 @@
       <c r="R77" t="s">
         <v>1695</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9519,7 +9545,7 @@
       <c r="J78" t="s">
         <v>1513</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9537,7 +9563,7 @@
       <c r="R78" t="s">
         <v>1695</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9575,7 +9601,7 @@
       <c r="J79" t="s">
         <v>1513</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9593,7 +9619,7 @@
       <c r="R79" t="s">
         <v>1695</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9631,7 +9657,7 @@
       <c r="J80" t="s">
         <v>1513</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9675,7 +9701,7 @@
       <c r="J81" t="s">
         <v>1513</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9719,7 +9745,7 @@
       <c r="J82" t="s">
         <v>1513</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9763,7 +9789,7 @@
       <c r="J83" t="s">
         <v>1513</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9807,7 +9833,7 @@
       <c r="J84" t="s">
         <v>1513</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9851,7 +9877,7 @@
       <c r="J85" t="s">
         <v>1513</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9869,7 +9895,7 @@
       <c r="R85" t="s">
         <v>1696</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9907,7 +9933,7 @@
       <c r="J86" t="s">
         <v>1513</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9951,7 +9977,7 @@
       <c r="J87" t="s">
         <v>1513</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9969,7 +9995,7 @@
       <c r="R87" t="s">
         <v>1697</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10007,7 +10033,7 @@
       <c r="J88" t="s">
         <v>1513</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10051,7 +10077,7 @@
       <c r="J89" t="s">
         <v>1513</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10069,7 +10095,7 @@
       <c r="R89" t="s">
         <v>1698</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10104,7 +10130,7 @@
       <c r="J90" t="s">
         <v>1513</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10122,7 +10148,7 @@
       <c r="R90" t="s">
         <v>1699</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10157,7 +10183,7 @@
       <c r="J91" t="s">
         <v>1513</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10175,7 +10201,7 @@
       <c r="R91" t="s">
         <v>1683</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10213,7 +10239,7 @@
       <c r="J92" t="s">
         <v>1513</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10234,7 +10260,7 @@
       <c r="R92" t="s">
         <v>1683</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10275,7 +10301,7 @@
       <c r="J93" t="s">
         <v>1513</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10316,7 +10342,7 @@
       <c r="J94" t="s">
         <v>1513</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10360,7 +10386,7 @@
       <c r="J95" t="s">
         <v>1513</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10404,7 +10430,7 @@
       <c r="J96" t="s">
         <v>1513</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10422,7 +10448,7 @@
       <c r="R96" t="s">
         <v>1700</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10460,7 +10486,7 @@
       <c r="J97" t="s">
         <v>1513</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10475,7 +10501,7 @@
       <c r="R97" t="s">
         <v>1700</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10516,7 +10542,7 @@
       <c r="J98" t="s">
         <v>1513</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10534,7 +10560,7 @@
       <c r="R98" t="s">
         <v>1701</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10572,7 +10598,7 @@
       <c r="J99" t="s">
         <v>1513</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10590,7 +10616,7 @@
       <c r="R99" t="s">
         <v>1702</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10628,7 +10654,7 @@
       <c r="J100" t="s">
         <v>1513</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10669,7 +10695,7 @@
       <c r="J101" t="s">
         <v>1513</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10710,7 +10736,7 @@
       <c r="J102" t="s">
         <v>1513</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10751,7 +10777,7 @@
       <c r="J103" t="s">
         <v>1513</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10792,7 +10818,7 @@
       <c r="J104" t="s">
         <v>1513</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10833,7 +10859,7 @@
       <c r="J105" t="s">
         <v>1513</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10874,7 +10900,7 @@
       <c r="J106" t="s">
         <v>1513</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10915,7 +10941,7 @@
       <c r="J107" t="s">
         <v>1513</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10956,7 +10982,7 @@
       <c r="J108" t="s">
         <v>1513</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10997,7 +11023,7 @@
       <c r="J109" t="s">
         <v>1513</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11050,7 +11076,7 @@
       <c r="J110" t="s">
         <v>1513</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11106,7 +11132,7 @@
       <c r="J111" t="s">
         <v>1513</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11124,7 +11150,7 @@
       <c r="R111" t="s">
         <v>1704</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11162,7 +11188,7 @@
       <c r="J112" t="s">
         <v>1513</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11221,7 +11247,7 @@
       <c r="J113" t="s">
         <v>1513</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11265,7 +11291,7 @@
       <c r="J114" t="s">
         <v>1513</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11309,7 +11335,7 @@
       <c r="J115" t="s">
         <v>1513</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11327,7 +11353,7 @@
       <c r="R115" t="s">
         <v>1706</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11365,7 +11391,7 @@
       <c r="J116" t="s">
         <v>1513</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11424,7 +11450,7 @@
       <c r="J117" t="s">
         <v>1513</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11468,7 +11494,7 @@
       <c r="J118" t="s">
         <v>1513</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11515,7 +11541,7 @@
       <c r="J119" t="s">
         <v>1513</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11556,7 +11582,7 @@
       <c r="J120" t="s">
         <v>1513</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11600,7 +11626,7 @@
       <c r="J121" t="s">
         <v>1513</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11647,7 +11673,7 @@
       <c r="J122" t="s">
         <v>1513</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11697,7 +11723,7 @@
       <c r="J123" t="s">
         <v>1513</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11741,7 +11767,7 @@
       <c r="J124" t="s">
         <v>1513</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11785,7 +11811,7 @@
       <c r="J125" t="s">
         <v>1513</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11803,7 +11829,7 @@
       <c r="R125" t="s">
         <v>1708</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11838,7 +11864,7 @@
       <c r="J126" t="s">
         <v>1513</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11856,7 +11882,7 @@
       <c r="R126" t="s">
         <v>1709</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11891,7 +11917,7 @@
       <c r="J127" t="s">
         <v>1513</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11947,7 +11973,7 @@
       <c r="J128" t="s">
         <v>1513</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11988,7 +12014,7 @@
       <c r="J129" t="s">
         <v>1513</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12029,7 +12055,7 @@
       <c r="J130" t="s">
         <v>1513</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12070,7 +12096,7 @@
       <c r="J131" t="s">
         <v>1513</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12114,7 +12140,7 @@
       <c r="J132" t="s">
         <v>1513</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12155,7 +12181,7 @@
       <c r="J133" t="s">
         <v>1513</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12173,7 +12199,7 @@
       <c r="R133" t="s">
         <v>1695</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12208,7 +12234,7 @@
       <c r="J134" t="s">
         <v>1513</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12226,7 +12252,7 @@
       <c r="R134" t="s">
         <v>1695</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12261,7 +12287,7 @@
       <c r="J135" t="s">
         <v>1513</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12302,7 +12328,7 @@
       <c r="J136" t="s">
         <v>1513</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12343,7 +12369,7 @@
       <c r="J137" t="s">
         <v>1513</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12384,7 +12410,7 @@
       <c r="J138" t="s">
         <v>1513</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12425,7 +12451,7 @@
       <c r="J139" t="s">
         <v>1513</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12472,7 +12498,7 @@
       <c r="J140" t="s">
         <v>1513</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12513,7 +12539,7 @@
       <c r="J141" t="s">
         <v>1513</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12554,7 +12580,7 @@
       <c r="J142" t="s">
         <v>1513</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12598,7 +12624,7 @@
       <c r="J143" t="s">
         <v>1513</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12616,7 +12642,7 @@
       <c r="R143" t="s">
         <v>1695</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12651,7 +12677,7 @@
       <c r="J144" t="s">
         <v>1513</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12669,7 +12695,7 @@
       <c r="R144" t="s">
         <v>1695</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12704,7 +12730,7 @@
       <c r="J145" t="s">
         <v>1513</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12722,7 +12748,7 @@
       <c r="R145" t="s">
         <v>1695</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12757,7 +12783,7 @@
       <c r="J146" t="s">
         <v>1513</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12775,7 +12801,7 @@
       <c r="R146" t="s">
         <v>1703</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12810,7 +12836,7 @@
       <c r="J147" t="s">
         <v>1513</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12828,7 +12854,7 @@
       <c r="R147" t="s">
         <v>1710</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12863,7 +12889,7 @@
       <c r="J148" t="s">
         <v>1513</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12904,7 +12930,7 @@
       <c r="J149" t="s">
         <v>1513</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12922,7 +12948,7 @@
       <c r="R149" t="s">
         <v>1695</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12957,7 +12983,7 @@
       <c r="J150" t="s">
         <v>1513</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12975,7 +13001,7 @@
       <c r="R150" t="s">
         <v>1695</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13010,7 +13036,7 @@
       <c r="J151" t="s">
         <v>1513</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13028,7 +13054,7 @@
       <c r="R151" t="s">
         <v>1711</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13063,7 +13089,7 @@
       <c r="J152" t="s">
         <v>1513</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13081,7 +13107,7 @@
       <c r="R152" t="s">
         <v>1712</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13116,7 +13142,7 @@
       <c r="J153" t="s">
         <v>1513</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13125,7 +13151,7 @@
       <c r="M153" t="s">
         <v>1588</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13166,7 +13192,7 @@
       <c r="J154" t="s">
         <v>1513</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13207,7 +13233,7 @@
       <c r="J155" t="s">
         <v>1513</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13248,7 +13274,7 @@
       <c r="J156" t="s">
         <v>1513</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13289,7 +13315,7 @@
       <c r="J157" t="s">
         <v>1513</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13330,7 +13356,7 @@
       <c r="J158" t="s">
         <v>1513</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13371,7 +13397,7 @@
       <c r="J159" t="s">
         <v>1513</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13412,7 +13438,7 @@
       <c r="J160" t="s">
         <v>1513</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13453,7 +13479,7 @@
       <c r="J161" t="s">
         <v>1513</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13494,7 +13520,7 @@
       <c r="J162" t="s">
         <v>1513</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13512,7 +13538,7 @@
       <c r="R162" t="s">
         <v>1698</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13547,7 +13573,7 @@
       <c r="J163" t="s">
         <v>1513</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13565,7 +13591,7 @@
       <c r="R163" t="s">
         <v>1695</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13600,7 +13626,7 @@
       <c r="J164" t="s">
         <v>1513</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13644,7 +13670,7 @@
       <c r="J165" t="s">
         <v>1513</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13685,7 +13711,7 @@
       <c r="J166" t="s">
         <v>1513</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13703,7 +13729,7 @@
       <c r="R166" t="s">
         <v>1713</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13738,7 +13764,7 @@
       <c r="J167" t="s">
         <v>1513</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13782,7 +13808,7 @@
       <c r="J168" t="s">
         <v>1513</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13826,7 +13852,7 @@
       <c r="J169" t="s">
         <v>1513</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13867,7 +13893,7 @@
       <c r="J170" t="s">
         <v>1513</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13908,7 +13934,7 @@
       <c r="J171" t="s">
         <v>1513</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13949,7 +13975,7 @@
       <c r="J172" t="s">
         <v>1513</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13990,7 +14016,7 @@
       <c r="J173" t="s">
         <v>1513</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14031,7 +14057,7 @@
       <c r="J174" t="s">
         <v>1513</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14072,7 +14098,7 @@
       <c r="J175" t="s">
         <v>1513</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14113,7 +14139,7 @@
       <c r="J176" t="s">
         <v>1513</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14154,7 +14180,7 @@
       <c r="J177" t="s">
         <v>1513</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14195,7 +14221,7 @@
       <c r="J178" t="s">
         <v>1513</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14213,7 +14239,7 @@
       <c r="R178" t="s">
         <v>1711</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14248,7 +14274,7 @@
       <c r="J179" t="s">
         <v>1513</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14257,7 +14283,7 @@
       <c r="M179" t="s">
         <v>1585</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14298,7 +14324,7 @@
       <c r="J180" t="s">
         <v>1513</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14339,7 +14365,7 @@
       <c r="J181" t="s">
         <v>1513</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14357,7 +14383,7 @@
       <c r="R181" t="s">
         <v>1695</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14392,7 +14418,7 @@
       <c r="J182" t="s">
         <v>1513</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14433,7 +14459,7 @@
       <c r="J183" t="s">
         <v>1513</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14474,7 +14500,7 @@
       <c r="J184" t="s">
         <v>1513</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14515,7 +14541,7 @@
       <c r="J185" t="s">
         <v>1513</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14556,7 +14582,7 @@
       <c r="J186" t="s">
         <v>1513</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14597,7 +14623,7 @@
       <c r="J187" t="s">
         <v>1513</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14638,7 +14664,7 @@
       <c r="J188" t="s">
         <v>1513</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14679,7 +14705,7 @@
       <c r="J189" t="s">
         <v>1513</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14720,7 +14746,7 @@
       <c r="J190" t="s">
         <v>1513</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14761,7 +14787,7 @@
       <c r="J191" t="s">
         <v>1513</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14802,7 +14828,7 @@
       <c r="J192" t="s">
         <v>1513</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14843,7 +14869,7 @@
       <c r="J193" t="s">
         <v>1513</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14884,7 +14910,7 @@
       <c r="J194" t="s">
         <v>1513</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14925,7 +14951,7 @@
       <c r="J195" t="s">
         <v>1513</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14943,7 +14969,7 @@
       <c r="R195" t="s">
         <v>1704</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14981,7 +15007,7 @@
       <c r="J196" t="s">
         <v>1513</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14999,7 +15025,7 @@
       <c r="R196" t="s">
         <v>1710</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15037,7 +15063,7 @@
       <c r="J197" t="s">
         <v>1513</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15078,7 +15104,7 @@
       <c r="J198" t="s">
         <v>1515</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15119,7 +15145,7 @@
       <c r="J199" t="s">
         <v>1514</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15160,7 +15186,7 @@
       <c r="J200" t="s">
         <v>1513</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15201,7 +15227,7 @@
       <c r="J201" t="s">
         <v>1513</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15242,7 +15268,7 @@
       <c r="J202" t="s">
         <v>1513</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15260,7 +15286,7 @@
       <c r="R202" t="s">
         <v>1695</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15295,7 +15321,7 @@
       <c r="J203" t="s">
         <v>1513</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15313,7 +15339,7 @@
       <c r="R203" t="s">
         <v>1703</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15348,7 +15374,7 @@
       <c r="J204" t="s">
         <v>1513</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15363,7 +15389,7 @@
       <c r="R204" t="s">
         <v>1714</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15401,7 +15427,7 @@
       <c r="J205" t="s">
         <v>1513</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15419,7 +15445,7 @@
       <c r="R205" t="s">
         <v>1715</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15457,7 +15483,7 @@
       <c r="J206" t="s">
         <v>1513</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15475,7 +15501,7 @@
       <c r="R206" t="s">
         <v>1683</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15510,7 +15536,7 @@
       <c r="J207" t="s">
         <v>1513</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15551,7 +15577,7 @@
       <c r="J208" t="s">
         <v>1513</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15592,7 +15618,7 @@
       <c r="J209" t="s">
         <v>1513</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15633,7 +15659,7 @@
       <c r="J210" t="s">
         <v>1513</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15674,7 +15700,7 @@
       <c r="J211" t="s">
         <v>1513</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15715,7 +15741,7 @@
       <c r="J212" t="s">
         <v>1513</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15756,7 +15782,7 @@
       <c r="J213" t="s">
         <v>1513</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15797,7 +15823,7 @@
       <c r="J214" t="s">
         <v>1513</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15815,7 +15841,7 @@
       <c r="R214" t="s">
         <v>1716</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15850,7 +15876,7 @@
       <c r="J215" t="s">
         <v>1513</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15891,7 +15917,7 @@
       <c r="J216" t="s">
         <v>1513</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15932,7 +15958,7 @@
       <c r="J217" t="s">
         <v>1513</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15973,7 +15999,7 @@
       <c r="J218" t="s">
         <v>1513</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16014,7 +16040,7 @@
       <c r="J219" t="s">
         <v>1513</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16055,7 +16081,7 @@
       <c r="J220" t="s">
         <v>1513</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16096,7 +16122,7 @@
       <c r="J221" t="s">
         <v>1513</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16137,7 +16163,7 @@
       <c r="J222" t="s">
         <v>1513</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16178,7 +16204,7 @@
       <c r="J223" t="s">
         <v>1513</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16219,7 +16245,7 @@
       <c r="J224" t="s">
         <v>1513</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16260,7 +16286,7 @@
       <c r="J225" t="s">
         <v>1513</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16301,7 +16327,7 @@
       <c r="J226" t="s">
         <v>1513</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16342,7 +16368,7 @@
       <c r="J227" t="s">
         <v>1513</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16383,7 +16409,7 @@
       <c r="J228" t="s">
         <v>1513</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16424,7 +16450,7 @@
       <c r="J229" t="s">
         <v>1513</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16465,7 +16491,7 @@
       <c r="J230" t="s">
         <v>1513</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16506,7 +16532,7 @@
       <c r="J231" t="s">
         <v>1513</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16547,7 +16573,7 @@
       <c r="J232" t="s">
         <v>1513</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16588,7 +16614,7 @@
       <c r="J233" t="s">
         <v>1513</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16629,7 +16655,7 @@
       <c r="J234" t="s">
         <v>1513</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16670,7 +16696,7 @@
       <c r="J235" t="s">
         <v>1513</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16711,7 +16737,7 @@
       <c r="J236" t="s">
         <v>1513</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16752,7 +16778,7 @@
       <c r="J237" t="s">
         <v>1513</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16793,7 +16819,7 @@
       <c r="J238" t="s">
         <v>1513</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16834,7 +16860,7 @@
       <c r="J239" t="s">
         <v>1513</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16852,7 +16878,7 @@
       <c r="R239" t="s">
         <v>1710</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16887,7 +16913,7 @@
       <c r="J240" t="s">
         <v>1513</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16928,7 +16954,7 @@
       <c r="J241" t="s">
         <v>1513</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16969,7 +16995,7 @@
       <c r="J242" t="s">
         <v>1513</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16987,7 +17013,7 @@
       <c r="R242" t="s">
         <v>1703</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17022,7 +17048,7 @@
       <c r="J243" t="s">
         <v>1513</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17063,7 +17089,7 @@
       <c r="J244" t="s">
         <v>1513</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17104,7 +17130,7 @@
       <c r="J245" t="s">
         <v>1513</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17145,7 +17171,7 @@
       <c r="J246" t="s">
         <v>1513</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17163,7 +17189,7 @@
       <c r="R246" t="s">
         <v>1683</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17198,7 +17224,7 @@
       <c r="J247" t="s">
         <v>1513</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17239,7 +17265,7 @@
       <c r="J248" t="s">
         <v>1513</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17280,7 +17306,7 @@
       <c r="J249" t="s">
         <v>1513</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17321,7 +17347,7 @@
       <c r="J250" t="s">
         <v>1513</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17362,7 +17388,7 @@
       <c r="J251" t="s">
         <v>1513</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17403,7 +17429,7 @@
       <c r="J252" t="s">
         <v>1513</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17444,7 +17470,7 @@
       <c r="J253" t="s">
         <v>1513</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17462,7 +17488,7 @@
       <c r="R253" t="s">
         <v>1713</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17500,7 +17526,7 @@
       <c r="J254" t="s">
         <v>1513</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17541,7 +17567,7 @@
       <c r="J255" t="s">
         <v>1513</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17582,7 +17608,7 @@
       <c r="J256" t="s">
         <v>1513</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17591,7 +17617,7 @@
       <c r="M256" t="s">
         <v>1584</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17629,7 +17655,7 @@
       <c r="J257" t="s">
         <v>1513</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17638,7 +17664,7 @@
       <c r="M257" t="s">
         <v>1585</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17682,7 +17708,7 @@
       <c r="J258" t="s">
         <v>1513</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17700,7 +17726,7 @@
       <c r="R258" t="s">
         <v>1695</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17738,7 +17764,7 @@
       <c r="J259" t="s">
         <v>1513</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17756,7 +17782,7 @@
       <c r="R259" t="s">
         <v>1711</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17794,7 +17820,7 @@
       <c r="J260" t="s">
         <v>1513</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17803,7 +17829,7 @@
       <c r="M260" t="s">
         <v>1579</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17847,7 +17873,7 @@
       <c r="J261" t="s">
         <v>1513</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17865,7 +17891,7 @@
       <c r="R261" t="s">
         <v>1717</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17903,7 +17929,7 @@
       <c r="J262" t="s">
         <v>1513</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17921,7 +17947,7 @@
       <c r="R262" t="s">
         <v>1711</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17959,7 +17985,7 @@
       <c r="J263" t="s">
         <v>1513</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17968,7 +17994,7 @@
       <c r="M263" t="s">
         <v>1579</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18012,7 +18038,7 @@
       <c r="J264" t="s">
         <v>1513</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18053,7 +18079,7 @@
       <c r="J265" t="s">
         <v>1513</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18094,7 +18120,7 @@
       <c r="J266" t="s">
         <v>1513</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18135,7 +18161,7 @@
       <c r="J267" t="s">
         <v>1513</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18179,7 +18205,7 @@
       <c r="J268" t="s">
         <v>1513</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18220,7 +18246,7 @@
       <c r="J269" t="s">
         <v>1513</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18261,7 +18287,7 @@
       <c r="J270" t="s">
         <v>1513</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18302,7 +18328,7 @@
       <c r="J271" t="s">
         <v>1513</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18343,7 +18369,7 @@
       <c r="J272" t="s">
         <v>1513</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18361,7 +18387,7 @@
       <c r="R272" t="s">
         <v>1718</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18399,7 +18425,7 @@
       <c r="J273" t="s">
         <v>1513</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18443,7 +18469,7 @@
       <c r="J274" t="s">
         <v>1513</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18484,7 +18510,7 @@
       <c r="J275" t="s">
         <v>1513</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18525,7 +18551,7 @@
       <c r="J276" t="s">
         <v>1513</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18566,7 +18592,7 @@
       <c r="J277" t="s">
         <v>1513</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18607,7 +18633,7 @@
       <c r="J278" t="s">
         <v>1513</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18648,7 +18674,7 @@
       <c r="J279" t="s">
         <v>1513</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18689,7 +18715,7 @@
       <c r="J280" t="s">
         <v>1513</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18730,7 +18756,7 @@
       <c r="J281" t="s">
         <v>1513</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18771,7 +18797,7 @@
       <c r="J282" t="s">
         <v>1513</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18812,7 +18838,7 @@
       <c r="J283" t="s">
         <v>1513</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18853,7 +18879,7 @@
       <c r="J284" t="s">
         <v>1513</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18894,7 +18920,7 @@
       <c r="J285" t="s">
         <v>1513</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18935,7 +18961,7 @@
       <c r="J286" t="s">
         <v>1513</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18976,7 +19002,7 @@
       <c r="J287" t="s">
         <v>1513</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19017,7 +19043,7 @@
       <c r="J288" t="s">
         <v>1513</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19058,7 +19084,7 @@
       <c r="J289" t="s">
         <v>1513</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19099,7 +19125,7 @@
       <c r="J290" t="s">
         <v>1513</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19140,7 +19166,7 @@
       <c r="J291" t="s">
         <v>1513</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19181,7 +19207,7 @@
       <c r="J292" t="s">
         <v>1513</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19222,7 +19248,7 @@
       <c r="J293" t="s">
         <v>1513</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19263,7 +19289,7 @@
       <c r="J294" t="s">
         <v>1513</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19304,7 +19330,7 @@
       <c r="J295" t="s">
         <v>1513</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19322,7 +19348,7 @@
       <c r="R295" t="s">
         <v>1719</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19360,7 +19386,7 @@
       <c r="J296" t="s">
         <v>1513</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19378,7 +19404,7 @@
       <c r="R296" t="s">
         <v>1695</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19416,7 +19442,7 @@
       <c r="J297" t="s">
         <v>1513</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19457,7 +19483,7 @@
       <c r="J298" t="s">
         <v>1513</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19498,7 +19524,7 @@
       <c r="J299" t="s">
         <v>1514</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19539,7 +19565,7 @@
       <c r="J300" t="s">
         <v>1513</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19580,7 +19606,7 @@
       <c r="J301" t="s">
         <v>1513</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20418,7 +20444,7 @@
       <c r="R321" t="s">
         <v>1681</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20638,7 +20664,7 @@
       <c r="R326" t="s">
         <v>1720</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21473,7 +21499,7 @@
       <c r="R346" t="s">
         <v>1721</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (16/09/2026 12:26)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5303,16 +5303,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5328,7 +5320,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5336,30 +5328,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5659,73 +5633,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5760,7 +5734,7 @@
       <c r="J2" t="s">
         <v>1513</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5804,7 +5778,7 @@
       <c r="J3" t="s">
         <v>1513</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5848,7 +5822,7 @@
       <c r="J4" t="s">
         <v>1513</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5866,7 +5840,7 @@
       <c r="R4" t="s">
         <v>1678</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5904,7 +5878,7 @@
       <c r="J5" t="s">
         <v>1514</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5954,7 +5928,7 @@
       <c r="J6" t="s">
         <v>1513</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6001,7 +5975,7 @@
       <c r="J7" t="s">
         <v>1513</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6048,7 +6022,7 @@
       <c r="J8" t="s">
         <v>1513</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6095,7 +6069,7 @@
       <c r="J9" t="s">
         <v>1513</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6142,7 +6116,7 @@
       <c r="J10" t="s">
         <v>1513</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6189,7 +6163,7 @@
       <c r="J11" t="s">
         <v>1513</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6236,7 +6210,7 @@
       <c r="J12" t="s">
         <v>1513</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6280,7 +6254,7 @@
       <c r="J13" t="s">
         <v>1513</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6298,7 +6272,7 @@
       <c r="R13" t="s">
         <v>1679</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6336,7 +6310,7 @@
       <c r="J14" t="s">
         <v>1513</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6354,7 +6328,7 @@
       <c r="R14" t="s">
         <v>1680</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6392,7 +6366,7 @@
       <c r="J15" t="s">
         <v>1513</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6410,7 +6384,7 @@
       <c r="R15" t="s">
         <v>1680</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6448,7 +6422,7 @@
       <c r="J16" t="s">
         <v>1513</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6492,7 +6466,7 @@
       <c r="J17" t="s">
         <v>1513</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6536,7 +6510,7 @@
       <c r="J18" t="s">
         <v>1513</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6554,7 +6528,7 @@
       <c r="R18" t="s">
         <v>1681</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6595,7 +6569,7 @@
       <c r="J19" t="s">
         <v>1513</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6639,7 +6613,7 @@
       <c r="J20" t="s">
         <v>1513</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6683,7 +6657,7 @@
       <c r="J21" t="s">
         <v>1513</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6701,7 +6675,7 @@
       <c r="R21" t="s">
         <v>1680</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6742,7 +6716,7 @@
       <c r="J22" t="s">
         <v>1513</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6760,7 +6734,7 @@
       <c r="R22" t="s">
         <v>1682</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6801,7 +6775,7 @@
       <c r="J23" t="s">
         <v>1513</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6819,7 +6793,7 @@
       <c r="R23" t="s">
         <v>1683</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6860,7 +6834,7 @@
       <c r="J24" t="s">
         <v>1513</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6904,7 +6878,7 @@
       <c r="J25" t="s">
         <v>1513</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6945,7 +6919,7 @@
       <c r="J26" t="s">
         <v>1515</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6963,7 +6937,7 @@
       <c r="R26" t="s">
         <v>1684</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6998,7 +6972,7 @@
       <c r="J27" t="s">
         <v>1513</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7016,7 +6990,7 @@
       <c r="R27" t="s">
         <v>1685</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7057,7 +7031,7 @@
       <c r="J28" t="s">
         <v>1513</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7101,7 +7075,7 @@
       <c r="J29" t="s">
         <v>1513</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7145,7 +7119,7 @@
       <c r="J30" t="s">
         <v>1513</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7189,7 +7163,7 @@
       <c r="J31" t="s">
         <v>1513</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7207,7 +7181,7 @@
       <c r="R31" t="s">
         <v>1686</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7248,7 +7222,7 @@
       <c r="J32" t="s">
         <v>1513</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7292,7 +7266,7 @@
       <c r="J33" t="s">
         <v>1513</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7310,7 +7284,7 @@
       <c r="R33" t="s">
         <v>1687</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7351,7 +7325,7 @@
       <c r="J34" t="s">
         <v>1513</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7395,7 +7369,7 @@
       <c r="J35" t="s">
         <v>1513</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7413,7 +7387,7 @@
       <c r="R35" t="s">
         <v>1688</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7454,7 +7428,7 @@
       <c r="J36" t="s">
         <v>1513</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7472,7 +7446,7 @@
       <c r="R36" t="s">
         <v>1688</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7513,7 +7487,7 @@
       <c r="J37" t="s">
         <v>1513</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7531,7 +7505,7 @@
       <c r="R37" t="s">
         <v>1688</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7572,7 +7546,7 @@
       <c r="J38" t="s">
         <v>1513</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7590,7 +7564,7 @@
       <c r="R38" t="s">
         <v>1688</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7631,7 +7605,7 @@
       <c r="J39" t="s">
         <v>1513</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7649,7 +7623,7 @@
       <c r="R39" t="s">
         <v>1688</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7690,7 +7664,7 @@
       <c r="J40" t="s">
         <v>1513</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7708,7 +7682,7 @@
       <c r="R40" t="s">
         <v>1689</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7749,7 +7723,7 @@
       <c r="J41" t="s">
         <v>1513</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7767,7 +7741,7 @@
       <c r="R41" t="s">
         <v>1680</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7805,7 +7779,7 @@
       <c r="J42" t="s">
         <v>1513</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7823,7 +7797,7 @@
       <c r="R42" t="s">
         <v>1688</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7864,7 +7838,7 @@
       <c r="J43" t="s">
         <v>1513</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7908,7 +7882,7 @@
       <c r="J44" t="s">
         <v>1513</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7926,7 +7900,7 @@
       <c r="R44" t="s">
         <v>1690</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7967,7 +7941,7 @@
       <c r="J45" t="s">
         <v>1513</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7985,7 +7959,7 @@
       <c r="R45" t="s">
         <v>1691</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8023,7 +7997,7 @@
       <c r="J46" t="s">
         <v>1513</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8067,7 +8041,7 @@
       <c r="J47" t="s">
         <v>1513</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8085,7 +8059,7 @@
       <c r="R47" t="s">
         <v>1692</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8126,7 +8100,7 @@
       <c r="J48" t="s">
         <v>1513</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8170,7 +8144,7 @@
       <c r="J49" t="s">
         <v>1513</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8214,7 +8188,7 @@
       <c r="J50" t="s">
         <v>1513</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8258,7 +8232,7 @@
       <c r="J51" t="s">
         <v>1513</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8305,7 +8279,7 @@
       <c r="J52" t="s">
         <v>1513</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8349,7 +8323,7 @@
       <c r="J53" t="s">
         <v>1513</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8393,7 +8367,7 @@
       <c r="J54" t="s">
         <v>1513</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8437,7 +8411,7 @@
       <c r="J55" t="s">
         <v>1513</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8487,7 +8461,7 @@
       <c r="J56" t="s">
         <v>1513</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8540,7 +8514,7 @@
       <c r="J57" t="s">
         <v>1513</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8590,7 +8564,7 @@
       <c r="J58" t="s">
         <v>1513</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8640,7 +8614,7 @@
       <c r="J59" t="s">
         <v>1513</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8658,7 +8632,7 @@
       <c r="R59" t="s">
         <v>1693</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8699,7 +8673,7 @@
       <c r="J60" t="s">
         <v>1513</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8743,7 +8717,7 @@
       <c r="J61" t="s">
         <v>1513</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8787,7 +8761,7 @@
       <c r="J62" t="s">
         <v>1513</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8831,7 +8805,7 @@
       <c r="J63" t="s">
         <v>1513</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8875,7 +8849,7 @@
       <c r="J64" t="s">
         <v>1513</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8919,7 +8893,7 @@
       <c r="J65" t="s">
         <v>1513</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8966,7 +8940,7 @@
       <c r="J66" t="s">
         <v>1513</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8984,7 +8958,7 @@
       <c r="R66" t="s">
         <v>1694</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9022,7 +8996,7 @@
       <c r="J67" t="s">
         <v>1513</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9066,7 +9040,7 @@
       <c r="J68" t="s">
         <v>1513</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9081,7 +9055,7 @@
       <c r="O68" t="s">
         <v>1597</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9125,7 +9099,7 @@
       <c r="J69" t="s">
         <v>1515</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9169,7 +9143,7 @@
       <c r="J70" t="s">
         <v>1513</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9213,7 +9187,7 @@
       <c r="J71" t="s">
         <v>1513</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9257,7 +9231,7 @@
       <c r="J72" t="s">
         <v>1513</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9301,7 +9275,7 @@
       <c r="J73" t="s">
         <v>1513</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9345,7 +9319,7 @@
       <c r="J74" t="s">
         <v>1513</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9389,7 +9363,7 @@
       <c r="J75" t="s">
         <v>1513</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9433,7 +9407,7 @@
       <c r="J76" t="s">
         <v>1513</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9451,7 +9425,7 @@
       <c r="R76" t="s">
         <v>1695</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9489,7 +9463,7 @@
       <c r="J77" t="s">
         <v>1513</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9507,7 +9481,7 @@
       <c r="R77" t="s">
         <v>1695</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9545,7 +9519,7 @@
       <c r="J78" t="s">
         <v>1513</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9563,7 +9537,7 @@
       <c r="R78" t="s">
         <v>1695</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9601,7 +9575,7 @@
       <c r="J79" t="s">
         <v>1513</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9619,7 +9593,7 @@
       <c r="R79" t="s">
         <v>1695</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9657,7 +9631,7 @@
       <c r="J80" t="s">
         <v>1513</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9701,7 +9675,7 @@
       <c r="J81" t="s">
         <v>1513</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9745,7 +9719,7 @@
       <c r="J82" t="s">
         <v>1513</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9789,7 +9763,7 @@
       <c r="J83" t="s">
         <v>1513</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9833,7 +9807,7 @@
       <c r="J84" t="s">
         <v>1513</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9877,7 +9851,7 @@
       <c r="J85" t="s">
         <v>1513</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9895,7 +9869,7 @@
       <c r="R85" t="s">
         <v>1696</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9933,7 +9907,7 @@
       <c r="J86" t="s">
         <v>1513</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9977,7 +9951,7 @@
       <c r="J87" t="s">
         <v>1513</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9995,7 +9969,7 @@
       <c r="R87" t="s">
         <v>1697</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10033,7 +10007,7 @@
       <c r="J88" t="s">
         <v>1513</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10077,7 +10051,7 @@
       <c r="J89" t="s">
         <v>1513</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10095,7 +10069,7 @@
       <c r="R89" t="s">
         <v>1698</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10130,7 +10104,7 @@
       <c r="J90" t="s">
         <v>1513</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10148,7 +10122,7 @@
       <c r="R90" t="s">
         <v>1699</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10183,7 +10157,7 @@
       <c r="J91" t="s">
         <v>1513</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10201,7 +10175,7 @@
       <c r="R91" t="s">
         <v>1683</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10239,7 +10213,7 @@
       <c r="J92" t="s">
         <v>1513</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10260,7 +10234,7 @@
       <c r="R92" t="s">
         <v>1683</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10301,7 +10275,7 @@
       <c r="J93" t="s">
         <v>1513</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10342,7 +10316,7 @@
       <c r="J94" t="s">
         <v>1513</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10386,7 +10360,7 @@
       <c r="J95" t="s">
         <v>1513</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10430,7 +10404,7 @@
       <c r="J96" t="s">
         <v>1513</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10448,7 +10422,7 @@
       <c r="R96" t="s">
         <v>1700</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10486,7 +10460,7 @@
       <c r="J97" t="s">
         <v>1513</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10501,7 +10475,7 @@
       <c r="R97" t="s">
         <v>1700</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10542,7 +10516,7 @@
       <c r="J98" t="s">
         <v>1513</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10560,7 +10534,7 @@
       <c r="R98" t="s">
         <v>1701</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10598,7 +10572,7 @@
       <c r="J99" t="s">
         <v>1513</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10616,7 +10590,7 @@
       <c r="R99" t="s">
         <v>1702</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10654,7 +10628,7 @@
       <c r="J100" t="s">
         <v>1513</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10695,7 +10669,7 @@
       <c r="J101" t="s">
         <v>1513</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10736,7 +10710,7 @@
       <c r="J102" t="s">
         <v>1513</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10777,7 +10751,7 @@
       <c r="J103" t="s">
         <v>1513</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10818,7 +10792,7 @@
       <c r="J104" t="s">
         <v>1513</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10859,7 +10833,7 @@
       <c r="J105" t="s">
         <v>1513</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10900,7 +10874,7 @@
       <c r="J106" t="s">
         <v>1513</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10941,7 +10915,7 @@
       <c r="J107" t="s">
         <v>1513</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10982,7 +10956,7 @@
       <c r="J108" t="s">
         <v>1513</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11023,7 +10997,7 @@
       <c r="J109" t="s">
         <v>1513</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11076,7 +11050,7 @@
       <c r="J110" t="s">
         <v>1513</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11132,7 +11106,7 @@
       <c r="J111" t="s">
         <v>1513</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11150,7 +11124,7 @@
       <c r="R111" t="s">
         <v>1704</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11188,7 +11162,7 @@
       <c r="J112" t="s">
         <v>1513</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11247,7 +11221,7 @@
       <c r="J113" t="s">
         <v>1513</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11291,7 +11265,7 @@
       <c r="J114" t="s">
         <v>1513</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11335,7 +11309,7 @@
       <c r="J115" t="s">
         <v>1513</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11353,7 +11327,7 @@
       <c r="R115" t="s">
         <v>1706</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11391,7 +11365,7 @@
       <c r="J116" t="s">
         <v>1513</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11450,7 +11424,7 @@
       <c r="J117" t="s">
         <v>1513</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11494,7 +11468,7 @@
       <c r="J118" t="s">
         <v>1513</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11541,7 +11515,7 @@
       <c r="J119" t="s">
         <v>1513</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11582,7 +11556,7 @@
       <c r="J120" t="s">
         <v>1513</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11626,7 +11600,7 @@
       <c r="J121" t="s">
         <v>1513</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11673,7 +11647,7 @@
       <c r="J122" t="s">
         <v>1513</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11723,7 +11697,7 @@
       <c r="J123" t="s">
         <v>1513</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11767,7 +11741,7 @@
       <c r="J124" t="s">
         <v>1513</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11811,7 +11785,7 @@
       <c r="J125" t="s">
         <v>1513</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11829,7 +11803,7 @@
       <c r="R125" t="s">
         <v>1708</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11864,7 +11838,7 @@
       <c r="J126" t="s">
         <v>1513</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11882,7 +11856,7 @@
       <c r="R126" t="s">
         <v>1709</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11917,7 +11891,7 @@
       <c r="J127" t="s">
         <v>1513</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11973,7 +11947,7 @@
       <c r="J128" t="s">
         <v>1513</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12014,7 +11988,7 @@
       <c r="J129" t="s">
         <v>1513</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12055,7 +12029,7 @@
       <c r="J130" t="s">
         <v>1513</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12096,7 +12070,7 @@
       <c r="J131" t="s">
         <v>1513</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12140,7 +12114,7 @@
       <c r="J132" t="s">
         <v>1513</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12181,7 +12155,7 @@
       <c r="J133" t="s">
         <v>1513</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12199,7 +12173,7 @@
       <c r="R133" t="s">
         <v>1695</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12234,7 +12208,7 @@
       <c r="J134" t="s">
         <v>1513</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12252,7 +12226,7 @@
       <c r="R134" t="s">
         <v>1695</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12287,7 +12261,7 @@
       <c r="J135" t="s">
         <v>1513</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12328,7 +12302,7 @@
       <c r="J136" t="s">
         <v>1513</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12369,7 +12343,7 @@
       <c r="J137" t="s">
         <v>1513</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12410,7 +12384,7 @@
       <c r="J138" t="s">
         <v>1513</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12451,7 +12425,7 @@
       <c r="J139" t="s">
         <v>1513</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12498,7 +12472,7 @@
       <c r="J140" t="s">
         <v>1513</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12539,7 +12513,7 @@
       <c r="J141" t="s">
         <v>1513</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12580,7 +12554,7 @@
       <c r="J142" t="s">
         <v>1513</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12624,7 +12598,7 @@
       <c r="J143" t="s">
         <v>1513</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12642,7 +12616,7 @@
       <c r="R143" t="s">
         <v>1695</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12677,7 +12651,7 @@
       <c r="J144" t="s">
         <v>1513</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12695,7 +12669,7 @@
       <c r="R144" t="s">
         <v>1695</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12730,7 +12704,7 @@
       <c r="J145" t="s">
         <v>1513</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12748,7 +12722,7 @@
       <c r="R145" t="s">
         <v>1695</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12783,7 +12757,7 @@
       <c r="J146" t="s">
         <v>1513</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12801,7 +12775,7 @@
       <c r="R146" t="s">
         <v>1703</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12836,7 +12810,7 @@
       <c r="J147" t="s">
         <v>1513</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12854,7 +12828,7 @@
       <c r="R147" t="s">
         <v>1710</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12889,7 +12863,7 @@
       <c r="J148" t="s">
         <v>1513</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12930,7 +12904,7 @@
       <c r="J149" t="s">
         <v>1513</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12948,7 +12922,7 @@
       <c r="R149" t="s">
         <v>1695</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12983,7 +12957,7 @@
       <c r="J150" t="s">
         <v>1513</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13001,7 +12975,7 @@
       <c r="R150" t="s">
         <v>1695</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13036,7 +13010,7 @@
       <c r="J151" t="s">
         <v>1513</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13054,7 +13028,7 @@
       <c r="R151" t="s">
         <v>1711</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13089,7 +13063,7 @@
       <c r="J152" t="s">
         <v>1513</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13107,7 +13081,7 @@
       <c r="R152" t="s">
         <v>1712</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13142,7 +13116,7 @@
       <c r="J153" t="s">
         <v>1513</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13151,7 +13125,7 @@
       <c r="M153" t="s">
         <v>1588</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13192,7 +13166,7 @@
       <c r="J154" t="s">
         <v>1513</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13233,7 +13207,7 @@
       <c r="J155" t="s">
         <v>1513</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13274,7 +13248,7 @@
       <c r="J156" t="s">
         <v>1513</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13315,7 +13289,7 @@
       <c r="J157" t="s">
         <v>1513</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13356,7 +13330,7 @@
       <c r="J158" t="s">
         <v>1513</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13397,7 +13371,7 @@
       <c r="J159" t="s">
         <v>1513</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13438,7 +13412,7 @@
       <c r="J160" t="s">
         <v>1513</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13479,7 +13453,7 @@
       <c r="J161" t="s">
         <v>1513</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13520,7 +13494,7 @@
       <c r="J162" t="s">
         <v>1513</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13538,7 +13512,7 @@
       <c r="R162" t="s">
         <v>1698</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13573,7 +13547,7 @@
       <c r="J163" t="s">
         <v>1513</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13591,7 +13565,7 @@
       <c r="R163" t="s">
         <v>1695</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13626,7 +13600,7 @@
       <c r="J164" t="s">
         <v>1513</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13670,7 +13644,7 @@
       <c r="J165" t="s">
         <v>1513</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13711,7 +13685,7 @@
       <c r="J166" t="s">
         <v>1513</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13729,7 +13703,7 @@
       <c r="R166" t="s">
         <v>1713</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13764,7 +13738,7 @@
       <c r="J167" t="s">
         <v>1513</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13808,7 +13782,7 @@
       <c r="J168" t="s">
         <v>1513</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13852,7 +13826,7 @@
       <c r="J169" t="s">
         <v>1513</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13893,7 +13867,7 @@
       <c r="J170" t="s">
         <v>1513</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13934,7 +13908,7 @@
       <c r="J171" t="s">
         <v>1513</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13975,7 +13949,7 @@
       <c r="J172" t="s">
         <v>1513</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14016,7 +13990,7 @@
       <c r="J173" t="s">
         <v>1513</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14057,7 +14031,7 @@
       <c r="J174" t="s">
         <v>1513</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14098,7 +14072,7 @@
       <c r="J175" t="s">
         <v>1513</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14139,7 +14113,7 @@
       <c r="J176" t="s">
         <v>1513</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14180,7 +14154,7 @@
       <c r="J177" t="s">
         <v>1513</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14221,7 +14195,7 @@
       <c r="J178" t="s">
         <v>1513</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14239,7 +14213,7 @@
       <c r="R178" t="s">
         <v>1711</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14274,7 +14248,7 @@
       <c r="J179" t="s">
         <v>1513</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14283,7 +14257,7 @@
       <c r="M179" t="s">
         <v>1585</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14324,7 +14298,7 @@
       <c r="J180" t="s">
         <v>1513</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14365,7 +14339,7 @@
       <c r="J181" t="s">
         <v>1513</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14383,7 +14357,7 @@
       <c r="R181" t="s">
         <v>1695</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14418,7 +14392,7 @@
       <c r="J182" t="s">
         <v>1513</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14459,7 +14433,7 @@
       <c r="J183" t="s">
         <v>1513</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14500,7 +14474,7 @@
       <c r="J184" t="s">
         <v>1513</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14541,7 +14515,7 @@
       <c r="J185" t="s">
         <v>1513</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14582,7 +14556,7 @@
       <c r="J186" t="s">
         <v>1513</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14623,7 +14597,7 @@
       <c r="J187" t="s">
         <v>1513</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14664,7 +14638,7 @@
       <c r="J188" t="s">
         <v>1513</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14705,7 +14679,7 @@
       <c r="J189" t="s">
         <v>1513</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14746,7 +14720,7 @@
       <c r="J190" t="s">
         <v>1513</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14787,7 +14761,7 @@
       <c r="J191" t="s">
         <v>1513</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14828,7 +14802,7 @@
       <c r="J192" t="s">
         <v>1513</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14869,7 +14843,7 @@
       <c r="J193" t="s">
         <v>1513</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14910,7 +14884,7 @@
       <c r="J194" t="s">
         <v>1513</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14951,7 +14925,7 @@
       <c r="J195" t="s">
         <v>1513</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14969,7 +14943,7 @@
       <c r="R195" t="s">
         <v>1704</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -15007,7 +14981,7 @@
       <c r="J196" t="s">
         <v>1513</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15025,7 +14999,7 @@
       <c r="R196" t="s">
         <v>1710</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15063,7 +15037,7 @@
       <c r="J197" t="s">
         <v>1513</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15104,7 +15078,7 @@
       <c r="J198" t="s">
         <v>1515</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15145,7 +15119,7 @@
       <c r="J199" t="s">
         <v>1514</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15186,7 +15160,7 @@
       <c r="J200" t="s">
         <v>1513</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15227,7 +15201,7 @@
       <c r="J201" t="s">
         <v>1513</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15268,7 +15242,7 @@
       <c r="J202" t="s">
         <v>1513</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15286,7 +15260,7 @@
       <c r="R202" t="s">
         <v>1695</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15321,7 +15295,7 @@
       <c r="J203" t="s">
         <v>1513</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15339,7 +15313,7 @@
       <c r="R203" t="s">
         <v>1703</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15374,7 +15348,7 @@
       <c r="J204" t="s">
         <v>1513</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15389,7 +15363,7 @@
       <c r="R204" t="s">
         <v>1714</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15427,7 +15401,7 @@
       <c r="J205" t="s">
         <v>1513</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15445,7 +15419,7 @@
       <c r="R205" t="s">
         <v>1715</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15483,7 +15457,7 @@
       <c r="J206" t="s">
         <v>1513</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15501,7 +15475,7 @@
       <c r="R206" t="s">
         <v>1683</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15536,7 +15510,7 @@
       <c r="J207" t="s">
         <v>1513</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15577,7 +15551,7 @@
       <c r="J208" t="s">
         <v>1513</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15618,7 +15592,7 @@
       <c r="J209" t="s">
         <v>1513</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15659,7 +15633,7 @@
       <c r="J210" t="s">
         <v>1513</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15700,7 +15674,7 @@
       <c r="J211" t="s">
         <v>1513</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15741,7 +15715,7 @@
       <c r="J212" t="s">
         <v>1513</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15782,7 +15756,7 @@
       <c r="J213" t="s">
         <v>1513</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15823,7 +15797,7 @@
       <c r="J214" t="s">
         <v>1513</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15841,7 +15815,7 @@
       <c r="R214" t="s">
         <v>1716</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15876,7 +15850,7 @@
       <c r="J215" t="s">
         <v>1513</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15917,7 +15891,7 @@
       <c r="J216" t="s">
         <v>1513</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15958,7 +15932,7 @@
       <c r="J217" t="s">
         <v>1513</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15999,7 +15973,7 @@
       <c r="J218" t="s">
         <v>1513</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16040,7 +16014,7 @@
       <c r="J219" t="s">
         <v>1513</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16081,7 +16055,7 @@
       <c r="J220" t="s">
         <v>1513</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16122,7 +16096,7 @@
       <c r="J221" t="s">
         <v>1513</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16163,7 +16137,7 @@
       <c r="J222" t="s">
         <v>1513</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16204,7 +16178,7 @@
       <c r="J223" t="s">
         <v>1513</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16245,7 +16219,7 @@
       <c r="J224" t="s">
         <v>1513</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16286,7 +16260,7 @@
       <c r="J225" t="s">
         <v>1513</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16327,7 +16301,7 @@
       <c r="J226" t="s">
         <v>1513</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16368,7 +16342,7 @@
       <c r="J227" t="s">
         <v>1513</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16409,7 +16383,7 @@
       <c r="J228" t="s">
         <v>1513</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16450,7 +16424,7 @@
       <c r="J229" t="s">
         <v>1513</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16491,7 +16465,7 @@
       <c r="J230" t="s">
         <v>1513</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16532,7 +16506,7 @@
       <c r="J231" t="s">
         <v>1513</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16573,7 +16547,7 @@
       <c r="J232" t="s">
         <v>1513</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16614,7 +16588,7 @@
       <c r="J233" t="s">
         <v>1513</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16655,7 +16629,7 @@
       <c r="J234" t="s">
         <v>1513</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16696,7 +16670,7 @@
       <c r="J235" t="s">
         <v>1513</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16737,7 +16711,7 @@
       <c r="J236" t="s">
         <v>1513</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16778,7 +16752,7 @@
       <c r="J237" t="s">
         <v>1513</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16819,7 +16793,7 @@
       <c r="J238" t="s">
         <v>1513</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16860,7 +16834,7 @@
       <c r="J239" t="s">
         <v>1513</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16878,7 +16852,7 @@
       <c r="R239" t="s">
         <v>1710</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16913,7 +16887,7 @@
       <c r="J240" t="s">
         <v>1513</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16954,7 +16928,7 @@
       <c r="J241" t="s">
         <v>1513</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16995,7 +16969,7 @@
       <c r="J242" t="s">
         <v>1513</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17013,7 +16987,7 @@
       <c r="R242" t="s">
         <v>1703</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17048,7 +17022,7 @@
       <c r="J243" t="s">
         <v>1513</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17089,7 +17063,7 @@
       <c r="J244" t="s">
         <v>1513</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17130,7 +17104,7 @@
       <c r="J245" t="s">
         <v>1513</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17171,7 +17145,7 @@
       <c r="J246" t="s">
         <v>1513</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17189,7 +17163,7 @@
       <c r="R246" t="s">
         <v>1683</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17224,7 +17198,7 @@
       <c r="J247" t="s">
         <v>1513</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17265,7 +17239,7 @@
       <c r="J248" t="s">
         <v>1513</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17306,7 +17280,7 @@
       <c r="J249" t="s">
         <v>1513</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17347,7 +17321,7 @@
       <c r="J250" t="s">
         <v>1513</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17388,7 +17362,7 @@
       <c r="J251" t="s">
         <v>1513</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17429,7 +17403,7 @@
       <c r="J252" t="s">
         <v>1513</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17470,7 +17444,7 @@
       <c r="J253" t="s">
         <v>1513</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17488,7 +17462,7 @@
       <c r="R253" t="s">
         <v>1713</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17526,7 +17500,7 @@
       <c r="J254" t="s">
         <v>1513</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17567,7 +17541,7 @@
       <c r="J255" t="s">
         <v>1513</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17608,7 +17582,7 @@
       <c r="J256" t="s">
         <v>1513</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17617,7 +17591,7 @@
       <c r="M256" t="s">
         <v>1584</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17655,7 +17629,7 @@
       <c r="J257" t="s">
         <v>1513</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17664,7 +17638,7 @@
       <c r="M257" t="s">
         <v>1585</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17708,7 +17682,7 @@
       <c r="J258" t="s">
         <v>1513</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17726,7 +17700,7 @@
       <c r="R258" t="s">
         <v>1695</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17764,7 +17738,7 @@
       <c r="J259" t="s">
         <v>1513</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17782,7 +17756,7 @@
       <c r="R259" t="s">
         <v>1711</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17820,7 +17794,7 @@
       <c r="J260" t="s">
         <v>1513</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17829,7 +17803,7 @@
       <c r="M260" t="s">
         <v>1579</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17873,7 +17847,7 @@
       <c r="J261" t="s">
         <v>1513</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17891,7 +17865,7 @@
       <c r="R261" t="s">
         <v>1717</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17929,7 +17903,7 @@
       <c r="J262" t="s">
         <v>1513</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17947,7 +17921,7 @@
       <c r="R262" t="s">
         <v>1711</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17985,7 +17959,7 @@
       <c r="J263" t="s">
         <v>1513</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17994,7 +17968,7 @@
       <c r="M263" t="s">
         <v>1579</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18038,7 +18012,7 @@
       <c r="J264" t="s">
         <v>1513</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18079,7 +18053,7 @@
       <c r="J265" t="s">
         <v>1513</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18120,7 +18094,7 @@
       <c r="J266" t="s">
         <v>1513</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18161,7 +18135,7 @@
       <c r="J267" t="s">
         <v>1513</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18205,7 +18179,7 @@
       <c r="J268" t="s">
         <v>1513</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18246,7 +18220,7 @@
       <c r="J269" t="s">
         <v>1513</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18287,7 +18261,7 @@
       <c r="J270" t="s">
         <v>1513</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18328,7 +18302,7 @@
       <c r="J271" t="s">
         <v>1513</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18369,7 +18343,7 @@
       <c r="J272" t="s">
         <v>1513</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18387,7 +18361,7 @@
       <c r="R272" t="s">
         <v>1718</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18425,7 +18399,7 @@
       <c r="J273" t="s">
         <v>1513</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18469,7 +18443,7 @@
       <c r="J274" t="s">
         <v>1513</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18510,7 +18484,7 @@
       <c r="J275" t="s">
         <v>1513</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18551,7 +18525,7 @@
       <c r="J276" t="s">
         <v>1513</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18592,7 +18566,7 @@
       <c r="J277" t="s">
         <v>1513</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18633,7 +18607,7 @@
       <c r="J278" t="s">
         <v>1513</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18674,7 +18648,7 @@
       <c r="J279" t="s">
         <v>1513</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18715,7 +18689,7 @@
       <c r="J280" t="s">
         <v>1513</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18756,7 +18730,7 @@
       <c r="J281" t="s">
         <v>1513</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18797,7 +18771,7 @@
       <c r="J282" t="s">
         <v>1513</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18838,7 +18812,7 @@
       <c r="J283" t="s">
         <v>1513</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18879,7 +18853,7 @@
       <c r="J284" t="s">
         <v>1513</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18920,7 +18894,7 @@
       <c r="J285" t="s">
         <v>1513</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18961,7 +18935,7 @@
       <c r="J286" t="s">
         <v>1513</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19002,7 +18976,7 @@
       <c r="J287" t="s">
         <v>1513</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19043,7 +19017,7 @@
       <c r="J288" t="s">
         <v>1513</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19084,7 +19058,7 @@
       <c r="J289" t="s">
         <v>1513</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19125,7 +19099,7 @@
       <c r="J290" t="s">
         <v>1513</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19166,7 +19140,7 @@
       <c r="J291" t="s">
         <v>1513</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19207,7 +19181,7 @@
       <c r="J292" t="s">
         <v>1513</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19248,7 +19222,7 @@
       <c r="J293" t="s">
         <v>1513</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19289,7 +19263,7 @@
       <c r="J294" t="s">
         <v>1513</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19330,7 +19304,7 @@
       <c r="J295" t="s">
         <v>1513</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19348,7 +19322,7 @@
       <c r="R295" t="s">
         <v>1719</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19386,7 +19360,7 @@
       <c r="J296" t="s">
         <v>1513</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19404,7 +19378,7 @@
       <c r="R296" t="s">
         <v>1695</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19442,7 +19416,7 @@
       <c r="J297" t="s">
         <v>1513</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19483,7 +19457,7 @@
       <c r="J298" t="s">
         <v>1513</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19524,7 +19498,7 @@
       <c r="J299" t="s">
         <v>1514</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19565,7 +19539,7 @@
       <c r="J300" t="s">
         <v>1513</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19606,7 +19580,7 @@
       <c r="J301" t="s">
         <v>1513</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20444,7 +20418,7 @@
       <c r="R321" t="s">
         <v>1681</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20664,7 +20638,7 @@
       <c r="R326" t="s">
         <v>1720</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21499,7 +21473,7 @@
       <c r="R346" t="s">
         <v>1721</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (16/09/2026 12:43)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5303,8 +5303,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5320,7 +5328,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5328,12 +5336,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5633,73 +5659,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5734,7 +5760,7 @@
       <c r="J2" t="s">
         <v>1513</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5778,7 +5804,7 @@
       <c r="J3" t="s">
         <v>1513</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5822,7 +5848,7 @@
       <c r="J4" t="s">
         <v>1513</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5840,7 +5866,7 @@
       <c r="R4" t="s">
         <v>1678</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5878,7 +5904,7 @@
       <c r="J5" t="s">
         <v>1514</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5928,7 +5954,7 @@
       <c r="J6" t="s">
         <v>1513</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5975,7 +6001,7 @@
       <c r="J7" t="s">
         <v>1513</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6022,7 +6048,7 @@
       <c r="J8" t="s">
         <v>1513</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6069,7 +6095,7 @@
       <c r="J9" t="s">
         <v>1513</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6116,7 +6142,7 @@
       <c r="J10" t="s">
         <v>1513</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6163,7 +6189,7 @@
       <c r="J11" t="s">
         <v>1513</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6210,7 +6236,7 @@
       <c r="J12" t="s">
         <v>1513</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6254,7 +6280,7 @@
       <c r="J13" t="s">
         <v>1513</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6272,7 +6298,7 @@
       <c r="R13" t="s">
         <v>1679</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6310,7 +6336,7 @@
       <c r="J14" t="s">
         <v>1513</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6328,7 +6354,7 @@
       <c r="R14" t="s">
         <v>1680</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6366,7 +6392,7 @@
       <c r="J15" t="s">
         <v>1513</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6384,7 +6410,7 @@
       <c r="R15" t="s">
         <v>1680</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6422,7 +6448,7 @@
       <c r="J16" t="s">
         <v>1513</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6466,7 +6492,7 @@
       <c r="J17" t="s">
         <v>1513</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6510,7 +6536,7 @@
       <c r="J18" t="s">
         <v>1513</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6528,7 +6554,7 @@
       <c r="R18" t="s">
         <v>1681</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6569,7 +6595,7 @@
       <c r="J19" t="s">
         <v>1513</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6613,7 +6639,7 @@
       <c r="J20" t="s">
         <v>1513</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6657,7 +6683,7 @@
       <c r="J21" t="s">
         <v>1513</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6675,7 +6701,7 @@
       <c r="R21" t="s">
         <v>1680</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6716,7 +6742,7 @@
       <c r="J22" t="s">
         <v>1513</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6734,7 +6760,7 @@
       <c r="R22" t="s">
         <v>1682</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6775,7 +6801,7 @@
       <c r="J23" t="s">
         <v>1513</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6793,7 +6819,7 @@
       <c r="R23" t="s">
         <v>1683</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6834,7 +6860,7 @@
       <c r="J24" t="s">
         <v>1513</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6878,7 +6904,7 @@
       <c r="J25" t="s">
         <v>1513</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6919,7 +6945,7 @@
       <c r="J26" t="s">
         <v>1515</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6937,7 +6963,7 @@
       <c r="R26" t="s">
         <v>1684</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6972,7 +6998,7 @@
       <c r="J27" t="s">
         <v>1513</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6990,7 +7016,7 @@
       <c r="R27" t="s">
         <v>1685</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7031,7 +7057,7 @@
       <c r="J28" t="s">
         <v>1513</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7075,7 +7101,7 @@
       <c r="J29" t="s">
         <v>1513</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7119,7 +7145,7 @@
       <c r="J30" t="s">
         <v>1513</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7163,7 +7189,7 @@
       <c r="J31" t="s">
         <v>1513</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7181,7 +7207,7 @@
       <c r="R31" t="s">
         <v>1686</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7222,7 +7248,7 @@
       <c r="J32" t="s">
         <v>1513</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7266,7 +7292,7 @@
       <c r="J33" t="s">
         <v>1513</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7284,7 +7310,7 @@
       <c r="R33" t="s">
         <v>1687</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7325,7 +7351,7 @@
       <c r="J34" t="s">
         <v>1513</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7369,7 +7395,7 @@
       <c r="J35" t="s">
         <v>1513</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7387,7 +7413,7 @@
       <c r="R35" t="s">
         <v>1688</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7428,7 +7454,7 @@
       <c r="J36" t="s">
         <v>1513</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7446,7 +7472,7 @@
       <c r="R36" t="s">
         <v>1688</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7487,7 +7513,7 @@
       <c r="J37" t="s">
         <v>1513</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7505,7 +7531,7 @@
       <c r="R37" t="s">
         <v>1688</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7546,7 +7572,7 @@
       <c r="J38" t="s">
         <v>1513</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7564,7 +7590,7 @@
       <c r="R38" t="s">
         <v>1688</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7605,7 +7631,7 @@
       <c r="J39" t="s">
         <v>1513</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7623,7 +7649,7 @@
       <c r="R39" t="s">
         <v>1688</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7664,7 +7690,7 @@
       <c r="J40" t="s">
         <v>1513</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7682,7 +7708,7 @@
       <c r="R40" t="s">
         <v>1689</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7723,7 +7749,7 @@
       <c r="J41" t="s">
         <v>1513</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7741,7 +7767,7 @@
       <c r="R41" t="s">
         <v>1680</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7779,7 +7805,7 @@
       <c r="J42" t="s">
         <v>1513</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7797,7 +7823,7 @@
       <c r="R42" t="s">
         <v>1688</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7838,7 +7864,7 @@
       <c r="J43" t="s">
         <v>1513</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7882,7 +7908,7 @@
       <c r="J44" t="s">
         <v>1513</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7900,7 +7926,7 @@
       <c r="R44" t="s">
         <v>1690</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7941,7 +7967,7 @@
       <c r="J45" t="s">
         <v>1513</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7959,7 +7985,7 @@
       <c r="R45" t="s">
         <v>1691</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7997,7 +8023,7 @@
       <c r="J46" t="s">
         <v>1513</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8041,7 +8067,7 @@
       <c r="J47" t="s">
         <v>1513</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8059,7 +8085,7 @@
       <c r="R47" t="s">
         <v>1692</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8100,7 +8126,7 @@
       <c r="J48" t="s">
         <v>1513</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8144,7 +8170,7 @@
       <c r="J49" t="s">
         <v>1513</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8188,7 +8214,7 @@
       <c r="J50" t="s">
         <v>1513</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8232,7 +8258,7 @@
       <c r="J51" t="s">
         <v>1513</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8279,7 +8305,7 @@
       <c r="J52" t="s">
         <v>1513</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8323,7 +8349,7 @@
       <c r="J53" t="s">
         <v>1513</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8367,7 +8393,7 @@
       <c r="J54" t="s">
         <v>1513</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8411,7 +8437,7 @@
       <c r="J55" t="s">
         <v>1513</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8461,7 +8487,7 @@
       <c r="J56" t="s">
         <v>1513</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8514,7 +8540,7 @@
       <c r="J57" t="s">
         <v>1513</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8564,7 +8590,7 @@
       <c r="J58" t="s">
         <v>1513</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8614,7 +8640,7 @@
       <c r="J59" t="s">
         <v>1513</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8632,7 +8658,7 @@
       <c r="R59" t="s">
         <v>1693</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8673,7 +8699,7 @@
       <c r="J60" t="s">
         <v>1513</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8717,7 +8743,7 @@
       <c r="J61" t="s">
         <v>1513</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8761,7 +8787,7 @@
       <c r="J62" t="s">
         <v>1513</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8805,7 +8831,7 @@
       <c r="J63" t="s">
         <v>1513</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8849,7 +8875,7 @@
       <c r="J64" t="s">
         <v>1513</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8893,7 +8919,7 @@
       <c r="J65" t="s">
         <v>1513</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8940,7 +8966,7 @@
       <c r="J66" t="s">
         <v>1513</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8958,7 +8984,7 @@
       <c r="R66" t="s">
         <v>1694</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8996,7 +9022,7 @@
       <c r="J67" t="s">
         <v>1513</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9040,7 +9066,7 @@
       <c r="J68" t="s">
         <v>1513</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9055,7 +9081,7 @@
       <c r="O68" t="s">
         <v>1597</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9099,7 +9125,7 @@
       <c r="J69" t="s">
         <v>1515</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9143,7 +9169,7 @@
       <c r="J70" t="s">
         <v>1513</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9187,7 +9213,7 @@
       <c r="J71" t="s">
         <v>1513</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9231,7 +9257,7 @@
       <c r="J72" t="s">
         <v>1513</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9275,7 +9301,7 @@
       <c r="J73" t="s">
         <v>1513</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9319,7 +9345,7 @@
       <c r="J74" t="s">
         <v>1513</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9363,7 +9389,7 @@
       <c r="J75" t="s">
         <v>1513</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9407,7 +9433,7 @@
       <c r="J76" t="s">
         <v>1513</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9425,7 +9451,7 @@
       <c r="R76" t="s">
         <v>1695</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9463,7 +9489,7 @@
       <c r="J77" t="s">
         <v>1513</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9481,7 +9507,7 @@
       <c r="R77" t="s">
         <v>1695</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9519,7 +9545,7 @@
       <c r="J78" t="s">
         <v>1513</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9537,7 +9563,7 @@
       <c r="R78" t="s">
         <v>1695</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9575,7 +9601,7 @@
       <c r="J79" t="s">
         <v>1513</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9593,7 +9619,7 @@
       <c r="R79" t="s">
         <v>1695</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9631,7 +9657,7 @@
       <c r="J80" t="s">
         <v>1513</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9675,7 +9701,7 @@
       <c r="J81" t="s">
         <v>1513</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9719,7 +9745,7 @@
       <c r="J82" t="s">
         <v>1513</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9763,7 +9789,7 @@
       <c r="J83" t="s">
         <v>1513</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9807,7 +9833,7 @@
       <c r="J84" t="s">
         <v>1513</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9851,7 +9877,7 @@
       <c r="J85" t="s">
         <v>1513</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9869,7 +9895,7 @@
       <c r="R85" t="s">
         <v>1696</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9907,7 +9933,7 @@
       <c r="J86" t="s">
         <v>1513</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9951,7 +9977,7 @@
       <c r="J87" t="s">
         <v>1513</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9969,7 +9995,7 @@
       <c r="R87" t="s">
         <v>1697</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10007,7 +10033,7 @@
       <c r="J88" t="s">
         <v>1513</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10051,7 +10077,7 @@
       <c r="J89" t="s">
         <v>1513</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10069,7 +10095,7 @@
       <c r="R89" t="s">
         <v>1698</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10104,7 +10130,7 @@
       <c r="J90" t="s">
         <v>1513</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10122,7 +10148,7 @@
       <c r="R90" t="s">
         <v>1699</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10157,7 +10183,7 @@
       <c r="J91" t="s">
         <v>1513</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10175,7 +10201,7 @@
       <c r="R91" t="s">
         <v>1683</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10213,7 +10239,7 @@
       <c r="J92" t="s">
         <v>1513</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10234,7 +10260,7 @@
       <c r="R92" t="s">
         <v>1683</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10275,7 +10301,7 @@
       <c r="J93" t="s">
         <v>1513</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10316,7 +10342,7 @@
       <c r="J94" t="s">
         <v>1513</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10360,7 +10386,7 @@
       <c r="J95" t="s">
         <v>1513</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10404,7 +10430,7 @@
       <c r="J96" t="s">
         <v>1513</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10422,7 +10448,7 @@
       <c r="R96" t="s">
         <v>1700</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10460,7 +10486,7 @@
       <c r="J97" t="s">
         <v>1513</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10475,7 +10501,7 @@
       <c r="R97" t="s">
         <v>1700</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10516,7 +10542,7 @@
       <c r="J98" t="s">
         <v>1513</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10534,7 +10560,7 @@
       <c r="R98" t="s">
         <v>1701</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10572,7 +10598,7 @@
       <c r="J99" t="s">
         <v>1513</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10590,7 +10616,7 @@
       <c r="R99" t="s">
         <v>1702</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10628,7 +10654,7 @@
       <c r="J100" t="s">
         <v>1513</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10669,7 +10695,7 @@
       <c r="J101" t="s">
         <v>1513</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10710,7 +10736,7 @@
       <c r="J102" t="s">
         <v>1513</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10751,7 +10777,7 @@
       <c r="J103" t="s">
         <v>1513</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10792,7 +10818,7 @@
       <c r="J104" t="s">
         <v>1513</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10833,7 +10859,7 @@
       <c r="J105" t="s">
         <v>1513</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10874,7 +10900,7 @@
       <c r="J106" t="s">
         <v>1513</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10915,7 +10941,7 @@
       <c r="J107" t="s">
         <v>1513</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10956,7 +10982,7 @@
       <c r="J108" t="s">
         <v>1513</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10997,7 +11023,7 @@
       <c r="J109" t="s">
         <v>1513</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11050,7 +11076,7 @@
       <c r="J110" t="s">
         <v>1513</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11106,7 +11132,7 @@
       <c r="J111" t="s">
         <v>1513</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11124,7 +11150,7 @@
       <c r="R111" t="s">
         <v>1704</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11162,7 +11188,7 @@
       <c r="J112" t="s">
         <v>1513</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11221,7 +11247,7 @@
       <c r="J113" t="s">
         <v>1513</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11265,7 +11291,7 @@
       <c r="J114" t="s">
         <v>1513</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11309,7 +11335,7 @@
       <c r="J115" t="s">
         <v>1513</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11327,7 +11353,7 @@
       <c r="R115" t="s">
         <v>1706</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11365,7 +11391,7 @@
       <c r="J116" t="s">
         <v>1513</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11424,7 +11450,7 @@
       <c r="J117" t="s">
         <v>1513</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11468,7 +11494,7 @@
       <c r="J118" t="s">
         <v>1513</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11515,7 +11541,7 @@
       <c r="J119" t="s">
         <v>1513</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11556,7 +11582,7 @@
       <c r="J120" t="s">
         <v>1513</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11600,7 +11626,7 @@
       <c r="J121" t="s">
         <v>1513</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11647,7 +11673,7 @@
       <c r="J122" t="s">
         <v>1513</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11697,7 +11723,7 @@
       <c r="J123" t="s">
         <v>1513</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11741,7 +11767,7 @@
       <c r="J124" t="s">
         <v>1513</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11785,7 +11811,7 @@
       <c r="J125" t="s">
         <v>1513</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11803,7 +11829,7 @@
       <c r="R125" t="s">
         <v>1708</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11838,7 +11864,7 @@
       <c r="J126" t="s">
         <v>1513</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11856,7 +11882,7 @@
       <c r="R126" t="s">
         <v>1709</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11891,7 +11917,7 @@
       <c r="J127" t="s">
         <v>1513</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11947,7 +11973,7 @@
       <c r="J128" t="s">
         <v>1513</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11988,7 +12014,7 @@
       <c r="J129" t="s">
         <v>1513</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12029,7 +12055,7 @@
       <c r="J130" t="s">
         <v>1513</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12070,7 +12096,7 @@
       <c r="J131" t="s">
         <v>1513</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12114,7 +12140,7 @@
       <c r="J132" t="s">
         <v>1513</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12155,7 +12181,7 @@
       <c r="J133" t="s">
         <v>1513</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12173,7 +12199,7 @@
       <c r="R133" t="s">
         <v>1695</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12208,7 +12234,7 @@
       <c r="J134" t="s">
         <v>1513</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12226,7 +12252,7 @@
       <c r="R134" t="s">
         <v>1695</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12261,7 +12287,7 @@
       <c r="J135" t="s">
         <v>1513</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12302,7 +12328,7 @@
       <c r="J136" t="s">
         <v>1513</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12343,7 +12369,7 @@
       <c r="J137" t="s">
         <v>1513</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12384,7 +12410,7 @@
       <c r="J138" t="s">
         <v>1513</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12425,7 +12451,7 @@
       <c r="J139" t="s">
         <v>1513</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12472,7 +12498,7 @@
       <c r="J140" t="s">
         <v>1513</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12513,7 +12539,7 @@
       <c r="J141" t="s">
         <v>1513</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12554,7 +12580,7 @@
       <c r="J142" t="s">
         <v>1513</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12598,7 +12624,7 @@
       <c r="J143" t="s">
         <v>1513</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12616,7 +12642,7 @@
       <c r="R143" t="s">
         <v>1695</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12651,7 +12677,7 @@
       <c r="J144" t="s">
         <v>1513</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12669,7 +12695,7 @@
       <c r="R144" t="s">
         <v>1695</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12704,7 +12730,7 @@
       <c r="J145" t="s">
         <v>1513</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12722,7 +12748,7 @@
       <c r="R145" t="s">
         <v>1695</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12757,7 +12783,7 @@
       <c r="J146" t="s">
         <v>1513</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12775,7 +12801,7 @@
       <c r="R146" t="s">
         <v>1703</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12810,7 +12836,7 @@
       <c r="J147" t="s">
         <v>1513</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12828,7 +12854,7 @@
       <c r="R147" t="s">
         <v>1710</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12863,7 +12889,7 @@
       <c r="J148" t="s">
         <v>1513</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12904,7 +12930,7 @@
       <c r="J149" t="s">
         <v>1513</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12922,7 +12948,7 @@
       <c r="R149" t="s">
         <v>1695</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12957,7 +12983,7 @@
       <c r="J150" t="s">
         <v>1513</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12975,7 +13001,7 @@
       <c r="R150" t="s">
         <v>1695</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13010,7 +13036,7 @@
       <c r="J151" t="s">
         <v>1513</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13028,7 +13054,7 @@
       <c r="R151" t="s">
         <v>1711</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13063,7 +13089,7 @@
       <c r="J152" t="s">
         <v>1513</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13081,7 +13107,7 @@
       <c r="R152" t="s">
         <v>1712</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13116,7 +13142,7 @@
       <c r="J153" t="s">
         <v>1513</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13125,7 +13151,7 @@
       <c r="M153" t="s">
         <v>1588</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13166,7 +13192,7 @@
       <c r="J154" t="s">
         <v>1513</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13207,7 +13233,7 @@
       <c r="J155" t="s">
         <v>1513</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13248,7 +13274,7 @@
       <c r="J156" t="s">
         <v>1513</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13289,7 +13315,7 @@
       <c r="J157" t="s">
         <v>1513</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13330,7 +13356,7 @@
       <c r="J158" t="s">
         <v>1513</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13371,7 +13397,7 @@
       <c r="J159" t="s">
         <v>1513</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13412,7 +13438,7 @@
       <c r="J160" t="s">
         <v>1513</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13453,7 +13479,7 @@
       <c r="J161" t="s">
         <v>1513</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13494,7 +13520,7 @@
       <c r="J162" t="s">
         <v>1513</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13512,7 +13538,7 @@
       <c r="R162" t="s">
         <v>1698</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13547,7 +13573,7 @@
       <c r="J163" t="s">
         <v>1513</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13565,7 +13591,7 @@
       <c r="R163" t="s">
         <v>1695</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13600,7 +13626,7 @@
       <c r="J164" t="s">
         <v>1513</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13644,7 +13670,7 @@
       <c r="J165" t="s">
         <v>1513</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13685,7 +13711,7 @@
       <c r="J166" t="s">
         <v>1513</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13703,7 +13729,7 @@
       <c r="R166" t="s">
         <v>1713</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13738,7 +13764,7 @@
       <c r="J167" t="s">
         <v>1513</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13782,7 +13808,7 @@
       <c r="J168" t="s">
         <v>1513</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13826,7 +13852,7 @@
       <c r="J169" t="s">
         <v>1513</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13867,7 +13893,7 @@
       <c r="J170" t="s">
         <v>1513</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13908,7 +13934,7 @@
       <c r="J171" t="s">
         <v>1513</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13949,7 +13975,7 @@
       <c r="J172" t="s">
         <v>1513</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13990,7 +14016,7 @@
       <c r="J173" t="s">
         <v>1513</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14031,7 +14057,7 @@
       <c r="J174" t="s">
         <v>1513</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14072,7 +14098,7 @@
       <c r="J175" t="s">
         <v>1513</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14113,7 +14139,7 @@
       <c r="J176" t="s">
         <v>1513</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14154,7 +14180,7 @@
       <c r="J177" t="s">
         <v>1513</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14195,7 +14221,7 @@
       <c r="J178" t="s">
         <v>1513</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14213,7 +14239,7 @@
       <c r="R178" t="s">
         <v>1711</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14248,7 +14274,7 @@
       <c r="J179" t="s">
         <v>1513</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14257,7 +14283,7 @@
       <c r="M179" t="s">
         <v>1585</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14298,7 +14324,7 @@
       <c r="J180" t="s">
         <v>1513</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14339,7 +14365,7 @@
       <c r="J181" t="s">
         <v>1513</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14357,7 +14383,7 @@
       <c r="R181" t="s">
         <v>1695</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14392,7 +14418,7 @@
       <c r="J182" t="s">
         <v>1513</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14433,7 +14459,7 @@
       <c r="J183" t="s">
         <v>1513</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14474,7 +14500,7 @@
       <c r="J184" t="s">
         <v>1513</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14515,7 +14541,7 @@
       <c r="J185" t="s">
         <v>1513</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14556,7 +14582,7 @@
       <c r="J186" t="s">
         <v>1513</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14597,7 +14623,7 @@
       <c r="J187" t="s">
         <v>1513</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14638,7 +14664,7 @@
       <c r="J188" t="s">
         <v>1513</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14679,7 +14705,7 @@
       <c r="J189" t="s">
         <v>1513</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14720,7 +14746,7 @@
       <c r="J190" t="s">
         <v>1513</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14761,7 +14787,7 @@
       <c r="J191" t="s">
         <v>1513</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14802,7 +14828,7 @@
       <c r="J192" t="s">
         <v>1513</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14843,7 +14869,7 @@
       <c r="J193" t="s">
         <v>1513</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14884,7 +14910,7 @@
       <c r="J194" t="s">
         <v>1513</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14925,7 +14951,7 @@
       <c r="J195" t="s">
         <v>1513</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14943,7 +14969,7 @@
       <c r="R195" t="s">
         <v>1704</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14981,7 +15007,7 @@
       <c r="J196" t="s">
         <v>1513</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14999,7 +15025,7 @@
       <c r="R196" t="s">
         <v>1710</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15037,7 +15063,7 @@
       <c r="J197" t="s">
         <v>1513</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15078,7 +15104,7 @@
       <c r="J198" t="s">
         <v>1515</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15119,7 +15145,7 @@
       <c r="J199" t="s">
         <v>1514</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15160,7 +15186,7 @@
       <c r="J200" t="s">
         <v>1513</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15201,7 +15227,7 @@
       <c r="J201" t="s">
         <v>1513</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15242,7 +15268,7 @@
       <c r="J202" t="s">
         <v>1513</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15260,7 +15286,7 @@
       <c r="R202" t="s">
         <v>1695</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15295,7 +15321,7 @@
       <c r="J203" t="s">
         <v>1513</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15313,7 +15339,7 @@
       <c r="R203" t="s">
         <v>1703</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15348,7 +15374,7 @@
       <c r="J204" t="s">
         <v>1513</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15363,7 +15389,7 @@
       <c r="R204" t="s">
         <v>1714</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15401,7 +15427,7 @@
       <c r="J205" t="s">
         <v>1513</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15419,7 +15445,7 @@
       <c r="R205" t="s">
         <v>1715</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15457,7 +15483,7 @@
       <c r="J206" t="s">
         <v>1513</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15475,7 +15501,7 @@
       <c r="R206" t="s">
         <v>1683</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15510,7 +15536,7 @@
       <c r="J207" t="s">
         <v>1513</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15551,7 +15577,7 @@
       <c r="J208" t="s">
         <v>1513</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15592,7 +15618,7 @@
       <c r="J209" t="s">
         <v>1513</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15633,7 +15659,7 @@
       <c r="J210" t="s">
         <v>1513</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15674,7 +15700,7 @@
       <c r="J211" t="s">
         <v>1513</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15715,7 +15741,7 @@
       <c r="J212" t="s">
         <v>1513</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15756,7 +15782,7 @@
       <c r="J213" t="s">
         <v>1513</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15797,7 +15823,7 @@
       <c r="J214" t="s">
         <v>1513</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15815,7 +15841,7 @@
       <c r="R214" t="s">
         <v>1716</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15850,7 +15876,7 @@
       <c r="J215" t="s">
         <v>1513</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15891,7 +15917,7 @@
       <c r="J216" t="s">
         <v>1513</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15932,7 +15958,7 @@
       <c r="J217" t="s">
         <v>1513</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15973,7 +15999,7 @@
       <c r="J218" t="s">
         <v>1513</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16014,7 +16040,7 @@
       <c r="J219" t="s">
         <v>1513</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16055,7 +16081,7 @@
       <c r="J220" t="s">
         <v>1513</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16096,7 +16122,7 @@
       <c r="J221" t="s">
         <v>1513</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16137,7 +16163,7 @@
       <c r="J222" t="s">
         <v>1513</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16178,7 +16204,7 @@
       <c r="J223" t="s">
         <v>1513</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16219,7 +16245,7 @@
       <c r="J224" t="s">
         <v>1513</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16260,7 +16286,7 @@
       <c r="J225" t="s">
         <v>1513</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16301,7 +16327,7 @@
       <c r="J226" t="s">
         <v>1513</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16342,7 +16368,7 @@
       <c r="J227" t="s">
         <v>1513</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16383,7 +16409,7 @@
       <c r="J228" t="s">
         <v>1513</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16424,7 +16450,7 @@
       <c r="J229" t="s">
         <v>1513</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16465,7 +16491,7 @@
       <c r="J230" t="s">
         <v>1513</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16506,7 +16532,7 @@
       <c r="J231" t="s">
         <v>1513</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16547,7 +16573,7 @@
       <c r="J232" t="s">
         <v>1513</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16588,7 +16614,7 @@
       <c r="J233" t="s">
         <v>1513</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16629,7 +16655,7 @@
       <c r="J234" t="s">
         <v>1513</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16670,7 +16696,7 @@
       <c r="J235" t="s">
         <v>1513</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16711,7 +16737,7 @@
       <c r="J236" t="s">
         <v>1513</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16752,7 +16778,7 @@
       <c r="J237" t="s">
         <v>1513</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16793,7 +16819,7 @@
       <c r="J238" t="s">
         <v>1513</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16834,7 +16860,7 @@
       <c r="J239" t="s">
         <v>1513</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16852,7 +16878,7 @@
       <c r="R239" t="s">
         <v>1710</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16887,7 +16913,7 @@
       <c r="J240" t="s">
         <v>1513</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16928,7 +16954,7 @@
       <c r="J241" t="s">
         <v>1513</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16969,7 +16995,7 @@
       <c r="J242" t="s">
         <v>1513</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16987,7 +17013,7 @@
       <c r="R242" t="s">
         <v>1703</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17022,7 +17048,7 @@
       <c r="J243" t="s">
         <v>1513</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17063,7 +17089,7 @@
       <c r="J244" t="s">
         <v>1513</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17104,7 +17130,7 @@
       <c r="J245" t="s">
         <v>1513</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17145,7 +17171,7 @@
       <c r="J246" t="s">
         <v>1513</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17163,7 +17189,7 @@
       <c r="R246" t="s">
         <v>1683</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17198,7 +17224,7 @@
       <c r="J247" t="s">
         <v>1513</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17239,7 +17265,7 @@
       <c r="J248" t="s">
         <v>1513</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17280,7 +17306,7 @@
       <c r="J249" t="s">
         <v>1513</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17321,7 +17347,7 @@
       <c r="J250" t="s">
         <v>1513</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17362,7 +17388,7 @@
       <c r="J251" t="s">
         <v>1513</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17403,7 +17429,7 @@
       <c r="J252" t="s">
         <v>1513</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17444,7 +17470,7 @@
       <c r="J253" t="s">
         <v>1513</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17462,7 +17488,7 @@
       <c r="R253" t="s">
         <v>1713</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17500,7 +17526,7 @@
       <c r="J254" t="s">
         <v>1513</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17541,7 +17567,7 @@
       <c r="J255" t="s">
         <v>1513</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17582,7 +17608,7 @@
       <c r="J256" t="s">
         <v>1513</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17591,7 +17617,7 @@
       <c r="M256" t="s">
         <v>1584</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17629,7 +17655,7 @@
       <c r="J257" t="s">
         <v>1513</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17638,7 +17664,7 @@
       <c r="M257" t="s">
         <v>1585</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17682,7 +17708,7 @@
       <c r="J258" t="s">
         <v>1513</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17700,7 +17726,7 @@
       <c r="R258" t="s">
         <v>1695</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17738,7 +17764,7 @@
       <c r="J259" t="s">
         <v>1513</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17756,7 +17782,7 @@
       <c r="R259" t="s">
         <v>1711</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17794,7 +17820,7 @@
       <c r="J260" t="s">
         <v>1513</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17803,7 +17829,7 @@
       <c r="M260" t="s">
         <v>1579</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17847,7 +17873,7 @@
       <c r="J261" t="s">
         <v>1513</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17865,7 +17891,7 @@
       <c r="R261" t="s">
         <v>1717</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17903,7 +17929,7 @@
       <c r="J262" t="s">
         <v>1513</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17921,7 +17947,7 @@
       <c r="R262" t="s">
         <v>1711</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17959,7 +17985,7 @@
       <c r="J263" t="s">
         <v>1513</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17968,7 +17994,7 @@
       <c r="M263" t="s">
         <v>1579</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18012,7 +18038,7 @@
       <c r="J264" t="s">
         <v>1513</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18053,7 +18079,7 @@
       <c r="J265" t="s">
         <v>1513</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18094,7 +18120,7 @@
       <c r="J266" t="s">
         <v>1513</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18135,7 +18161,7 @@
       <c r="J267" t="s">
         <v>1513</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18179,7 +18205,7 @@
       <c r="J268" t="s">
         <v>1513</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18220,7 +18246,7 @@
       <c r="J269" t="s">
         <v>1513</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18261,7 +18287,7 @@
       <c r="J270" t="s">
         <v>1513</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18302,7 +18328,7 @@
       <c r="J271" t="s">
         <v>1513</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18343,7 +18369,7 @@
       <c r="J272" t="s">
         <v>1513</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18361,7 +18387,7 @@
       <c r="R272" t="s">
         <v>1718</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18399,7 +18425,7 @@
       <c r="J273" t="s">
         <v>1513</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18443,7 +18469,7 @@
       <c r="J274" t="s">
         <v>1513</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18484,7 +18510,7 @@
       <c r="J275" t="s">
         <v>1513</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18525,7 +18551,7 @@
       <c r="J276" t="s">
         <v>1513</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18566,7 +18592,7 @@
       <c r="J277" t="s">
         <v>1513</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18607,7 +18633,7 @@
       <c r="J278" t="s">
         <v>1513</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18648,7 +18674,7 @@
       <c r="J279" t="s">
         <v>1513</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18689,7 +18715,7 @@
       <c r="J280" t="s">
         <v>1513</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18730,7 +18756,7 @@
       <c r="J281" t="s">
         <v>1513</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18771,7 +18797,7 @@
       <c r="J282" t="s">
         <v>1513</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18812,7 +18838,7 @@
       <c r="J283" t="s">
         <v>1513</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18853,7 +18879,7 @@
       <c r="J284" t="s">
         <v>1513</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18894,7 +18920,7 @@
       <c r="J285" t="s">
         <v>1513</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18935,7 +18961,7 @@
       <c r="J286" t="s">
         <v>1513</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18976,7 +19002,7 @@
       <c r="J287" t="s">
         <v>1513</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19017,7 +19043,7 @@
       <c r="J288" t="s">
         <v>1513</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19058,7 +19084,7 @@
       <c r="J289" t="s">
         <v>1513</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19099,7 +19125,7 @@
       <c r="J290" t="s">
         <v>1513</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19140,7 +19166,7 @@
       <c r="J291" t="s">
         <v>1513</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19181,7 +19207,7 @@
       <c r="J292" t="s">
         <v>1513</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19222,7 +19248,7 @@
       <c r="J293" t="s">
         <v>1513</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19263,7 +19289,7 @@
       <c r="J294" t="s">
         <v>1513</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19304,7 +19330,7 @@
       <c r="J295" t="s">
         <v>1513</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19322,7 +19348,7 @@
       <c r="R295" t="s">
         <v>1719</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19360,7 +19386,7 @@
       <c r="J296" t="s">
         <v>1513</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19378,7 +19404,7 @@
       <c r="R296" t="s">
         <v>1695</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19416,7 +19442,7 @@
       <c r="J297" t="s">
         <v>1513</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19457,7 +19483,7 @@
       <c r="J298" t="s">
         <v>1513</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19498,7 +19524,7 @@
       <c r="J299" t="s">
         <v>1514</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19539,7 +19565,7 @@
       <c r="J300" t="s">
         <v>1513</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19580,7 +19606,7 @@
       <c r="J301" t="s">
         <v>1513</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20418,7 +20444,7 @@
       <c r="R321" t="s">
         <v>1681</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20638,7 +20664,7 @@
       <c r="R326" t="s">
         <v>1720</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21473,7 +21499,7 @@
       <c r="R346" t="s">
         <v>1721</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (17/09/2026 12:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5330,8 +5330,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5347,7 +5355,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5355,12 +5363,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5660,73 +5686,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5761,7 +5787,7 @@
       <c r="J2" t="s">
         <v>1520</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5805,7 +5831,7 @@
       <c r="J3" t="s">
         <v>1520</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5849,7 +5875,7 @@
       <c r="J4" t="s">
         <v>1520</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5867,7 +5893,7 @@
       <c r="R4" t="s">
         <v>1687</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5905,7 +5931,7 @@
       <c r="J5" t="s">
         <v>1521</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5955,7 +5981,7 @@
       <c r="J6" t="s">
         <v>1520</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6002,7 +6028,7 @@
       <c r="J7" t="s">
         <v>1520</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6049,7 +6075,7 @@
       <c r="J8" t="s">
         <v>1520</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6096,7 +6122,7 @@
       <c r="J9" t="s">
         <v>1520</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6143,7 +6169,7 @@
       <c r="J10" t="s">
         <v>1520</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6190,7 +6216,7 @@
       <c r="J11" t="s">
         <v>1520</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6237,7 +6263,7 @@
       <c r="J12" t="s">
         <v>1520</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6281,7 +6307,7 @@
       <c r="J13" t="s">
         <v>1520</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6299,7 +6325,7 @@
       <c r="R13" t="s">
         <v>1688</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6337,7 +6363,7 @@
       <c r="J14" t="s">
         <v>1520</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6355,7 +6381,7 @@
       <c r="R14" t="s">
         <v>1689</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6393,7 +6419,7 @@
       <c r="J15" t="s">
         <v>1520</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6411,7 +6437,7 @@
       <c r="R15" t="s">
         <v>1689</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6449,7 +6475,7 @@
       <c r="J16" t="s">
         <v>1520</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6493,7 +6519,7 @@
       <c r="J17" t="s">
         <v>1520</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6537,7 +6563,7 @@
       <c r="J18" t="s">
         <v>1520</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6555,7 +6581,7 @@
       <c r="R18" t="s">
         <v>1690</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6596,7 +6622,7 @@
       <c r="J19" t="s">
         <v>1520</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6640,7 +6666,7 @@
       <c r="J20" t="s">
         <v>1520</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6684,7 +6710,7 @@
       <c r="J21" t="s">
         <v>1520</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6702,7 +6728,7 @@
       <c r="R21" t="s">
         <v>1689</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6743,7 +6769,7 @@
       <c r="J22" t="s">
         <v>1520</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6761,7 +6787,7 @@
       <c r="R22" t="s">
         <v>1691</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6802,7 +6828,7 @@
       <c r="J23" t="s">
         <v>1520</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6820,7 +6846,7 @@
       <c r="R23" t="s">
         <v>1692</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6861,7 +6887,7 @@
       <c r="J24" t="s">
         <v>1520</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6905,7 +6931,7 @@
       <c r="J25" t="s">
         <v>1520</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6946,7 +6972,7 @@
       <c r="J26" t="s">
         <v>1522</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6964,7 +6990,7 @@
       <c r="R26" t="s">
         <v>1693</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6999,7 +7025,7 @@
       <c r="J27" t="s">
         <v>1520</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7017,7 +7043,7 @@
       <c r="R27" t="s">
         <v>1694</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7058,7 +7084,7 @@
       <c r="J28" t="s">
         <v>1520</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7102,7 +7128,7 @@
       <c r="J29" t="s">
         <v>1520</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7146,7 +7172,7 @@
       <c r="J30" t="s">
         <v>1520</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7190,7 +7216,7 @@
       <c r="J31" t="s">
         <v>1520</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7208,7 +7234,7 @@
       <c r="R31" t="s">
         <v>1695</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7249,7 +7275,7 @@
       <c r="J32" t="s">
         <v>1520</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7293,7 +7319,7 @@
       <c r="J33" t="s">
         <v>1520</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7311,7 +7337,7 @@
       <c r="R33" t="s">
         <v>1696</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7352,7 +7378,7 @@
       <c r="J34" t="s">
         <v>1520</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7396,7 +7422,7 @@
       <c r="J35" t="s">
         <v>1520</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7414,7 +7440,7 @@
       <c r="R35" t="s">
         <v>1697</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7455,7 +7481,7 @@
       <c r="J36" t="s">
         <v>1520</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7473,7 +7499,7 @@
       <c r="R36" t="s">
         <v>1697</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7514,7 +7540,7 @@
       <c r="J37" t="s">
         <v>1520</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7532,7 +7558,7 @@
       <c r="R37" t="s">
         <v>1697</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7573,7 +7599,7 @@
       <c r="J38" t="s">
         <v>1520</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7591,7 +7617,7 @@
       <c r="R38" t="s">
         <v>1697</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7632,7 +7658,7 @@
       <c r="J39" t="s">
         <v>1520</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7650,7 +7676,7 @@
       <c r="R39" t="s">
         <v>1697</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7691,7 +7717,7 @@
       <c r="J40" t="s">
         <v>1520</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7709,7 +7735,7 @@
       <c r="R40" t="s">
         <v>1698</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7750,7 +7776,7 @@
       <c r="J41" t="s">
         <v>1520</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7768,7 +7794,7 @@
       <c r="R41" t="s">
         <v>1689</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7806,7 +7832,7 @@
       <c r="J42" t="s">
         <v>1520</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7824,7 +7850,7 @@
       <c r="R42" t="s">
         <v>1697</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7865,7 +7891,7 @@
       <c r="J43" t="s">
         <v>1520</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7909,7 +7935,7 @@
       <c r="J44" t="s">
         <v>1520</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7927,7 +7953,7 @@
       <c r="R44" t="s">
         <v>1699</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7968,7 +7994,7 @@
       <c r="J45" t="s">
         <v>1520</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7986,7 +8012,7 @@
       <c r="R45" t="s">
         <v>1700</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8024,7 +8050,7 @@
       <c r="J46" t="s">
         <v>1520</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8068,7 +8094,7 @@
       <c r="J47" t="s">
         <v>1520</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8086,7 +8112,7 @@
       <c r="R47" t="s">
         <v>1701</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8127,7 +8153,7 @@
       <c r="J48" t="s">
         <v>1520</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8171,7 +8197,7 @@
       <c r="J49" t="s">
         <v>1520</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8215,7 +8241,7 @@
       <c r="J50" t="s">
         <v>1520</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8259,7 +8285,7 @@
       <c r="J51" t="s">
         <v>1520</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8306,7 +8332,7 @@
       <c r="J52" t="s">
         <v>1520</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8350,7 +8376,7 @@
       <c r="J53" t="s">
         <v>1520</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8394,7 +8420,7 @@
       <c r="J54" t="s">
         <v>1520</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8438,7 +8464,7 @@
       <c r="J55" t="s">
         <v>1520</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8488,7 +8514,7 @@
       <c r="J56" t="s">
         <v>1520</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8541,7 +8567,7 @@
       <c r="J57" t="s">
         <v>1520</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8591,7 +8617,7 @@
       <c r="J58" t="s">
         <v>1520</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8641,7 +8667,7 @@
       <c r="J59" t="s">
         <v>1520</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8659,7 +8685,7 @@
       <c r="R59" t="s">
         <v>1702</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8700,7 +8726,7 @@
       <c r="J60" t="s">
         <v>1520</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8744,7 +8770,7 @@
       <c r="J61" t="s">
         <v>1520</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8788,7 +8814,7 @@
       <c r="J62" t="s">
         <v>1520</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8832,7 +8858,7 @@
       <c r="J63" t="s">
         <v>1520</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8876,7 +8902,7 @@
       <c r="J64" t="s">
         <v>1520</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8920,7 +8946,7 @@
       <c r="J65" t="s">
         <v>1520</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8967,7 +8993,7 @@
       <c r="J66" t="s">
         <v>1520</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8985,7 +9011,7 @@
       <c r="R66" t="s">
         <v>1703</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9023,7 +9049,7 @@
       <c r="J67" t="s">
         <v>1520</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9067,7 +9093,7 @@
       <c r="J68" t="s">
         <v>1520</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9082,7 +9108,7 @@
       <c r="O68" t="s">
         <v>1605</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9126,7 +9152,7 @@
       <c r="J69" t="s">
         <v>1522</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9170,7 +9196,7 @@
       <c r="J70" t="s">
         <v>1520</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9214,7 +9240,7 @@
       <c r="J71" t="s">
         <v>1520</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9258,7 +9284,7 @@
       <c r="J72" t="s">
         <v>1520</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9302,7 +9328,7 @@
       <c r="J73" t="s">
         <v>1520</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9346,7 +9372,7 @@
       <c r="J74" t="s">
         <v>1520</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9390,7 +9416,7 @@
       <c r="J75" t="s">
         <v>1520</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9434,7 +9460,7 @@
       <c r="J76" t="s">
         <v>1520</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9452,7 +9478,7 @@
       <c r="R76" t="s">
         <v>1704</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9490,7 +9516,7 @@
       <c r="J77" t="s">
         <v>1520</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9508,7 +9534,7 @@
       <c r="R77" t="s">
         <v>1704</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9546,7 +9572,7 @@
       <c r="J78" t="s">
         <v>1520</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9564,7 +9590,7 @@
       <c r="R78" t="s">
         <v>1704</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9602,7 +9628,7 @@
       <c r="J79" t="s">
         <v>1520</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9620,7 +9646,7 @@
       <c r="R79" t="s">
         <v>1704</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9658,7 +9684,7 @@
       <c r="J80" t="s">
         <v>1520</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9702,7 +9728,7 @@
       <c r="J81" t="s">
         <v>1520</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9746,7 +9772,7 @@
       <c r="J82" t="s">
         <v>1520</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9790,7 +9816,7 @@
       <c r="J83" t="s">
         <v>1520</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9834,7 +9860,7 @@
       <c r="J84" t="s">
         <v>1520</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9878,7 +9904,7 @@
       <c r="J85" t="s">
         <v>1520</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9896,7 +9922,7 @@
       <c r="R85" t="s">
         <v>1705</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9934,7 +9960,7 @@
       <c r="J86" t="s">
         <v>1520</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9978,7 +10004,7 @@
       <c r="J87" t="s">
         <v>1520</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9996,7 +10022,7 @@
       <c r="R87" t="s">
         <v>1706</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10034,7 +10060,7 @@
       <c r="J88" t="s">
         <v>1520</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10078,7 +10104,7 @@
       <c r="J89" t="s">
         <v>1520</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10096,7 +10122,7 @@
       <c r="R89" t="s">
         <v>1707</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10131,7 +10157,7 @@
       <c r="J90" t="s">
         <v>1520</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10149,7 +10175,7 @@
       <c r="R90" t="s">
         <v>1708</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10184,7 +10210,7 @@
       <c r="J91" t="s">
         <v>1520</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10202,7 +10228,7 @@
       <c r="R91" t="s">
         <v>1692</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10240,7 +10266,7 @@
       <c r="J92" t="s">
         <v>1520</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10261,7 +10287,7 @@
       <c r="R92" t="s">
         <v>1692</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10302,7 +10328,7 @@
       <c r="J93" t="s">
         <v>1520</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10343,7 +10369,7 @@
       <c r="J94" t="s">
         <v>1520</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10387,7 +10413,7 @@
       <c r="J95" t="s">
         <v>1520</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10431,7 +10457,7 @@
       <c r="J96" t="s">
         <v>1520</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10449,7 +10475,7 @@
       <c r="R96" t="s">
         <v>1709</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10487,7 +10513,7 @@
       <c r="J97" t="s">
         <v>1520</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10502,7 +10528,7 @@
       <c r="R97" t="s">
         <v>1709</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10543,7 +10569,7 @@
       <c r="J98" t="s">
         <v>1520</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10561,7 +10587,7 @@
       <c r="R98" t="s">
         <v>1710</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10599,7 +10625,7 @@
       <c r="J99" t="s">
         <v>1520</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10617,7 +10643,7 @@
       <c r="R99" t="s">
         <v>1711</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10655,7 +10681,7 @@
       <c r="J100" t="s">
         <v>1520</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10696,7 +10722,7 @@
       <c r="J101" t="s">
         <v>1520</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10737,7 +10763,7 @@
       <c r="J102" t="s">
         <v>1520</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10778,7 +10804,7 @@
       <c r="J103" t="s">
         <v>1520</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10819,7 +10845,7 @@
       <c r="J104" t="s">
         <v>1520</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10860,7 +10886,7 @@
       <c r="J105" t="s">
         <v>1520</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10901,7 +10927,7 @@
       <c r="J106" t="s">
         <v>1520</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10942,7 +10968,7 @@
       <c r="J107" t="s">
         <v>1520</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10983,7 +11009,7 @@
       <c r="J108" t="s">
         <v>1520</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11024,7 +11050,7 @@
       <c r="J109" t="s">
         <v>1520</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11077,7 +11103,7 @@
       <c r="J110" t="s">
         <v>1520</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11133,7 +11159,7 @@
       <c r="J111" t="s">
         <v>1520</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11151,7 +11177,7 @@
       <c r="R111" t="s">
         <v>1713</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11189,7 +11215,7 @@
       <c r="J112" t="s">
         <v>1520</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11248,7 +11274,7 @@
       <c r="J113" t="s">
         <v>1520</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11292,7 +11318,7 @@
       <c r="J114" t="s">
         <v>1520</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11336,7 +11362,7 @@
       <c r="J115" t="s">
         <v>1520</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11354,7 +11380,7 @@
       <c r="R115" t="s">
         <v>1715</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11392,7 +11418,7 @@
       <c r="J116" t="s">
         <v>1520</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11451,7 +11477,7 @@
       <c r="J117" t="s">
         <v>1520</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11495,7 +11521,7 @@
       <c r="J118" t="s">
         <v>1520</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11542,7 +11568,7 @@
       <c r="J119" t="s">
         <v>1520</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11583,7 +11609,7 @@
       <c r="J120" t="s">
         <v>1520</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11627,7 +11653,7 @@
       <c r="J121" t="s">
         <v>1520</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11674,7 +11700,7 @@
       <c r="J122" t="s">
         <v>1520</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11724,7 +11750,7 @@
       <c r="J123" t="s">
         <v>1520</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11768,7 +11794,7 @@
       <c r="J124" t="s">
         <v>1520</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11812,7 +11838,7 @@
       <c r="J125" t="s">
         <v>1520</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11830,7 +11856,7 @@
       <c r="R125" t="s">
         <v>1717</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11865,7 +11891,7 @@
       <c r="J126" t="s">
         <v>1520</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11883,7 +11909,7 @@
       <c r="R126" t="s">
         <v>1718</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11918,7 +11944,7 @@
       <c r="J127" t="s">
         <v>1520</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11974,7 +12000,7 @@
       <c r="J128" t="s">
         <v>1520</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12015,7 +12041,7 @@
       <c r="J129" t="s">
         <v>1520</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12056,7 +12082,7 @@
       <c r="J130" t="s">
         <v>1520</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12097,7 +12123,7 @@
       <c r="J131" t="s">
         <v>1520</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12141,7 +12167,7 @@
       <c r="J132" t="s">
         <v>1520</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12182,7 +12208,7 @@
       <c r="J133" t="s">
         <v>1520</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12200,7 +12226,7 @@
       <c r="R133" t="s">
         <v>1704</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12235,7 +12261,7 @@
       <c r="J134" t="s">
         <v>1520</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12253,7 +12279,7 @@
       <c r="R134" t="s">
         <v>1704</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12288,7 +12314,7 @@
       <c r="J135" t="s">
         <v>1520</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12329,7 +12355,7 @@
       <c r="J136" t="s">
         <v>1520</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12370,7 +12396,7 @@
       <c r="J137" t="s">
         <v>1520</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12411,7 +12437,7 @@
       <c r="J138" t="s">
         <v>1520</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12452,7 +12478,7 @@
       <c r="J139" t="s">
         <v>1520</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12499,7 +12525,7 @@
       <c r="J140" t="s">
         <v>1520</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12540,7 +12566,7 @@
       <c r="J141" t="s">
         <v>1520</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12581,7 +12607,7 @@
       <c r="J142" t="s">
         <v>1520</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12625,7 +12651,7 @@
       <c r="J143" t="s">
         <v>1520</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12643,7 +12669,7 @@
       <c r="R143" t="s">
         <v>1704</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12678,7 +12704,7 @@
       <c r="J144" t="s">
         <v>1520</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12696,7 +12722,7 @@
       <c r="R144" t="s">
         <v>1704</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12731,7 +12757,7 @@
       <c r="J145" t="s">
         <v>1520</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12749,7 +12775,7 @@
       <c r="R145" t="s">
         <v>1704</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12784,7 +12810,7 @@
       <c r="J146" t="s">
         <v>1520</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12802,7 +12828,7 @@
       <c r="R146" t="s">
         <v>1712</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12837,7 +12863,7 @@
       <c r="J147" t="s">
         <v>1520</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12855,7 +12881,7 @@
       <c r="R147" t="s">
         <v>1719</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12890,7 +12916,7 @@
       <c r="J148" t="s">
         <v>1520</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12931,7 +12957,7 @@
       <c r="J149" t="s">
         <v>1520</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12949,7 +12975,7 @@
       <c r="R149" t="s">
         <v>1704</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12984,7 +13010,7 @@
       <c r="J150" t="s">
         <v>1520</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13002,7 +13028,7 @@
       <c r="R150" t="s">
         <v>1704</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13037,7 +13063,7 @@
       <c r="J151" t="s">
         <v>1520</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13055,7 +13081,7 @@
       <c r="R151" t="s">
         <v>1720</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13090,7 +13116,7 @@
       <c r="J152" t="s">
         <v>1520</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13108,7 +13134,7 @@
       <c r="R152" t="s">
         <v>1721</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13143,7 +13169,7 @@
       <c r="J153" t="s">
         <v>1520</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13152,7 +13178,7 @@
       <c r="M153" t="s">
         <v>1596</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13193,7 +13219,7 @@
       <c r="J154" t="s">
         <v>1520</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13234,7 +13260,7 @@
       <c r="J155" t="s">
         <v>1520</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13275,7 +13301,7 @@
       <c r="J156" t="s">
         <v>1520</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13316,7 +13342,7 @@
       <c r="J157" t="s">
         <v>1520</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13357,7 +13383,7 @@
       <c r="J158" t="s">
         <v>1520</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13398,7 +13424,7 @@
       <c r="J159" t="s">
         <v>1520</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13439,7 +13465,7 @@
       <c r="J160" t="s">
         <v>1520</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13480,7 +13506,7 @@
       <c r="J161" t="s">
         <v>1520</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13521,7 +13547,7 @@
       <c r="J162" t="s">
         <v>1520</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13539,7 +13565,7 @@
       <c r="R162" t="s">
         <v>1707</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13574,7 +13600,7 @@
       <c r="J163" t="s">
         <v>1520</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13592,7 +13618,7 @@
       <c r="R163" t="s">
         <v>1704</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13627,7 +13653,7 @@
       <c r="J164" t="s">
         <v>1520</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13671,7 +13697,7 @@
       <c r="J165" t="s">
         <v>1520</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13712,7 +13738,7 @@
       <c r="J166" t="s">
         <v>1520</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13730,7 +13756,7 @@
       <c r="R166" t="s">
         <v>1722</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13765,7 +13791,7 @@
       <c r="J167" t="s">
         <v>1520</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13809,7 +13835,7 @@
       <c r="J168" t="s">
         <v>1520</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13853,7 +13879,7 @@
       <c r="J169" t="s">
         <v>1520</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13894,7 +13920,7 @@
       <c r="J170" t="s">
         <v>1520</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13935,7 +13961,7 @@
       <c r="J171" t="s">
         <v>1520</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13976,7 +14002,7 @@
       <c r="J172" t="s">
         <v>1520</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14017,7 +14043,7 @@
       <c r="J173" t="s">
         <v>1520</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14058,7 +14084,7 @@
       <c r="J174" t="s">
         <v>1520</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14099,7 +14125,7 @@
       <c r="J175" t="s">
         <v>1520</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14140,7 +14166,7 @@
       <c r="J176" t="s">
         <v>1520</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14181,7 +14207,7 @@
       <c r="J177" t="s">
         <v>1520</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14222,7 +14248,7 @@
       <c r="J178" t="s">
         <v>1520</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14240,7 +14266,7 @@
       <c r="R178" t="s">
         <v>1720</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14275,7 +14301,7 @@
       <c r="J179" t="s">
         <v>1520</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14284,7 +14310,7 @@
       <c r="M179" t="s">
         <v>1593</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14325,7 +14351,7 @@
       <c r="J180" t="s">
         <v>1520</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14366,7 +14392,7 @@
       <c r="J181" t="s">
         <v>1520</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14384,7 +14410,7 @@
       <c r="R181" t="s">
         <v>1704</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14419,7 +14445,7 @@
       <c r="J182" t="s">
         <v>1520</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14460,7 +14486,7 @@
       <c r="J183" t="s">
         <v>1520</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14501,7 +14527,7 @@
       <c r="J184" t="s">
         <v>1520</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14542,7 +14568,7 @@
       <c r="J185" t="s">
         <v>1520</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14583,7 +14609,7 @@
       <c r="J186" t="s">
         <v>1520</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14624,7 +14650,7 @@
       <c r="J187" t="s">
         <v>1520</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14665,7 +14691,7 @@
       <c r="J188" t="s">
         <v>1520</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14706,7 +14732,7 @@
       <c r="J189" t="s">
         <v>1520</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14747,7 +14773,7 @@
       <c r="J190" t="s">
         <v>1520</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14788,7 +14814,7 @@
       <c r="J191" t="s">
         <v>1520</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14829,7 +14855,7 @@
       <c r="J192" t="s">
         <v>1520</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14870,7 +14896,7 @@
       <c r="J193" t="s">
         <v>1520</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14911,7 +14937,7 @@
       <c r="J194" t="s">
         <v>1520</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14952,7 +14978,7 @@
       <c r="J195" t="s">
         <v>1520</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14970,7 +14996,7 @@
       <c r="R195" t="s">
         <v>1713</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -15008,7 +15034,7 @@
       <c r="J196" t="s">
         <v>1520</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15026,7 +15052,7 @@
       <c r="R196" t="s">
         <v>1719</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15064,7 +15090,7 @@
       <c r="J197" t="s">
         <v>1520</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15105,7 +15131,7 @@
       <c r="J198" t="s">
         <v>1522</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15146,7 +15172,7 @@
       <c r="J199" t="s">
         <v>1521</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15187,7 +15213,7 @@
       <c r="J200" t="s">
         <v>1520</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15228,7 +15254,7 @@
       <c r="J201" t="s">
         <v>1520</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15269,7 +15295,7 @@
       <c r="J202" t="s">
         <v>1520</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15287,7 +15313,7 @@
       <c r="R202" t="s">
         <v>1704</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15322,7 +15348,7 @@
       <c r="J203" t="s">
         <v>1520</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15340,7 +15366,7 @@
       <c r="R203" t="s">
         <v>1712</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15375,7 +15401,7 @@
       <c r="J204" t="s">
         <v>1520</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15390,7 +15416,7 @@
       <c r="R204" t="s">
         <v>1723</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15428,7 +15454,7 @@
       <c r="J205" t="s">
         <v>1520</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15446,7 +15472,7 @@
       <c r="R205" t="s">
         <v>1724</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15484,7 +15510,7 @@
       <c r="J206" t="s">
         <v>1520</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15502,7 +15528,7 @@
       <c r="R206" t="s">
         <v>1692</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15537,7 +15563,7 @@
       <c r="J207" t="s">
         <v>1520</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15578,7 +15604,7 @@
       <c r="J208" t="s">
         <v>1520</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15619,7 +15645,7 @@
       <c r="J209" t="s">
         <v>1520</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15660,7 +15686,7 @@
       <c r="J210" t="s">
         <v>1520</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15701,7 +15727,7 @@
       <c r="J211" t="s">
         <v>1520</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15742,7 +15768,7 @@
       <c r="J212" t="s">
         <v>1520</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15783,7 +15809,7 @@
       <c r="J213" t="s">
         <v>1520</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15824,7 +15850,7 @@
       <c r="J214" t="s">
         <v>1520</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15842,7 +15868,7 @@
       <c r="R214" t="s">
         <v>1725</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15877,7 +15903,7 @@
       <c r="J215" t="s">
         <v>1520</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15918,7 +15944,7 @@
       <c r="J216" t="s">
         <v>1520</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15959,7 +15985,7 @@
       <c r="J217" t="s">
         <v>1520</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16000,7 +16026,7 @@
       <c r="J218" t="s">
         <v>1520</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16041,7 +16067,7 @@
       <c r="J219" t="s">
         <v>1520</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16082,7 +16108,7 @@
       <c r="J220" t="s">
         <v>1520</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16123,7 +16149,7 @@
       <c r="J221" t="s">
         <v>1520</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16164,7 +16190,7 @@
       <c r="J222" t="s">
         <v>1520</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16205,7 +16231,7 @@
       <c r="J223" t="s">
         <v>1520</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16246,7 +16272,7 @@
       <c r="J224" t="s">
         <v>1520</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16287,7 +16313,7 @@
       <c r="J225" t="s">
         <v>1520</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16328,7 +16354,7 @@
       <c r="J226" t="s">
         <v>1520</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16369,7 +16395,7 @@
       <c r="J227" t="s">
         <v>1520</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16410,7 +16436,7 @@
       <c r="J228" t="s">
         <v>1520</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16451,7 +16477,7 @@
       <c r="J229" t="s">
         <v>1520</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16492,7 +16518,7 @@
       <c r="J230" t="s">
         <v>1520</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16533,7 +16559,7 @@
       <c r="J231" t="s">
         <v>1520</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16574,7 +16600,7 @@
       <c r="J232" t="s">
         <v>1520</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16615,7 +16641,7 @@
       <c r="J233" t="s">
         <v>1520</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16656,7 +16682,7 @@
       <c r="J234" t="s">
         <v>1520</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16697,7 +16723,7 @@
       <c r="J235" t="s">
         <v>1520</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16738,7 +16764,7 @@
       <c r="J236" t="s">
         <v>1520</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16779,7 +16805,7 @@
       <c r="J237" t="s">
         <v>1520</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16820,7 +16846,7 @@
       <c r="J238" t="s">
         <v>1520</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16861,7 +16887,7 @@
       <c r="J239" t="s">
         <v>1520</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16879,7 +16905,7 @@
       <c r="R239" t="s">
         <v>1719</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16914,7 +16940,7 @@
       <c r="J240" t="s">
         <v>1520</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16955,7 +16981,7 @@
       <c r="J241" t="s">
         <v>1520</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16996,7 +17022,7 @@
       <c r="J242" t="s">
         <v>1520</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17014,7 +17040,7 @@
       <c r="R242" t="s">
         <v>1712</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17049,7 +17075,7 @@
       <c r="J243" t="s">
         <v>1520</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17090,7 +17116,7 @@
       <c r="J244" t="s">
         <v>1520</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17131,7 +17157,7 @@
       <c r="J245" t="s">
         <v>1520</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17172,7 +17198,7 @@
       <c r="J246" t="s">
         <v>1520</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17190,7 +17216,7 @@
       <c r="R246" t="s">
         <v>1692</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17225,7 +17251,7 @@
       <c r="J247" t="s">
         <v>1520</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17266,7 +17292,7 @@
       <c r="J248" t="s">
         <v>1520</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17307,7 +17333,7 @@
       <c r="J249" t="s">
         <v>1520</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17348,7 +17374,7 @@
       <c r="J250" t="s">
         <v>1520</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17389,7 +17415,7 @@
       <c r="J251" t="s">
         <v>1520</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17430,7 +17456,7 @@
       <c r="J252" t="s">
         <v>1520</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17471,7 +17497,7 @@
       <c r="J253" t="s">
         <v>1520</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17489,7 +17515,7 @@
       <c r="R253" t="s">
         <v>1722</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17527,7 +17553,7 @@
       <c r="J254" t="s">
         <v>1520</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17568,7 +17594,7 @@
       <c r="J255" t="s">
         <v>1520</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17609,7 +17635,7 @@
       <c r="J256" t="s">
         <v>1520</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17618,7 +17644,7 @@
       <c r="M256" t="s">
         <v>1592</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17656,7 +17682,7 @@
       <c r="J257" t="s">
         <v>1520</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17665,7 +17691,7 @@
       <c r="M257" t="s">
         <v>1593</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17709,7 +17735,7 @@
       <c r="J258" t="s">
         <v>1520</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17727,7 +17753,7 @@
       <c r="R258" t="s">
         <v>1704</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17765,7 +17791,7 @@
       <c r="J259" t="s">
         <v>1520</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17783,7 +17809,7 @@
       <c r="R259" t="s">
         <v>1720</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17821,7 +17847,7 @@
       <c r="J260" t="s">
         <v>1520</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17830,7 +17856,7 @@
       <c r="M260" t="s">
         <v>1587</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17874,7 +17900,7 @@
       <c r="J261" t="s">
         <v>1520</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17892,7 +17918,7 @@
       <c r="R261" t="s">
         <v>1726</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17930,7 +17956,7 @@
       <c r="J262" t="s">
         <v>1520</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17948,7 +17974,7 @@
       <c r="R262" t="s">
         <v>1720</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17986,7 +18012,7 @@
       <c r="J263" t="s">
         <v>1520</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17995,7 +18021,7 @@
       <c r="M263" t="s">
         <v>1587</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18039,7 +18065,7 @@
       <c r="J264" t="s">
         <v>1520</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18080,7 +18106,7 @@
       <c r="J265" t="s">
         <v>1520</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18121,7 +18147,7 @@
       <c r="J266" t="s">
         <v>1520</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18162,7 +18188,7 @@
       <c r="J267" t="s">
         <v>1520</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18206,7 +18232,7 @@
       <c r="J268" t="s">
         <v>1520</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18247,7 +18273,7 @@
       <c r="J269" t="s">
         <v>1520</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18288,7 +18314,7 @@
       <c r="J270" t="s">
         <v>1520</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18329,7 +18355,7 @@
       <c r="J271" t="s">
         <v>1520</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18370,7 +18396,7 @@
       <c r="J272" t="s">
         <v>1520</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18388,7 +18414,7 @@
       <c r="R272" t="s">
         <v>1727</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18426,7 +18452,7 @@
       <c r="J273" t="s">
         <v>1520</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18470,7 +18496,7 @@
       <c r="J274" t="s">
         <v>1520</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18511,7 +18537,7 @@
       <c r="J275" t="s">
         <v>1520</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18552,7 +18578,7 @@
       <c r="J276" t="s">
         <v>1520</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18593,7 +18619,7 @@
       <c r="J277" t="s">
         <v>1520</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18634,7 +18660,7 @@
       <c r="J278" t="s">
         <v>1520</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18675,7 +18701,7 @@
       <c r="J279" t="s">
         <v>1520</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18716,7 +18742,7 @@
       <c r="J280" t="s">
         <v>1520</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18757,7 +18783,7 @@
       <c r="J281" t="s">
         <v>1520</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18798,7 +18824,7 @@
       <c r="J282" t="s">
         <v>1520</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18839,7 +18865,7 @@
       <c r="J283" t="s">
         <v>1520</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18880,7 +18906,7 @@
       <c r="J284" t="s">
         <v>1520</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18921,7 +18947,7 @@
       <c r="J285" t="s">
         <v>1520</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18962,7 +18988,7 @@
       <c r="J286" t="s">
         <v>1520</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19003,7 +19029,7 @@
       <c r="J287" t="s">
         <v>1520</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19044,7 +19070,7 @@
       <c r="J288" t="s">
         <v>1520</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19085,7 +19111,7 @@
       <c r="J289" t="s">
         <v>1520</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19126,7 +19152,7 @@
       <c r="J290" t="s">
         <v>1520</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19167,7 +19193,7 @@
       <c r="J291" t="s">
         <v>1520</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19208,7 +19234,7 @@
       <c r="J292" t="s">
         <v>1520</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19249,7 +19275,7 @@
       <c r="J293" t="s">
         <v>1520</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19290,7 +19316,7 @@
       <c r="J294" t="s">
         <v>1520</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19331,7 +19357,7 @@
       <c r="J295" t="s">
         <v>1520</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19349,7 +19375,7 @@
       <c r="R295" t="s">
         <v>1728</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19387,7 +19413,7 @@
       <c r="J296" t="s">
         <v>1520</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19405,7 +19431,7 @@
       <c r="R296" t="s">
         <v>1704</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19443,7 +19469,7 @@
       <c r="J297" t="s">
         <v>1520</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19484,7 +19510,7 @@
       <c r="J298" t="s">
         <v>1520</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19525,7 +19551,7 @@
       <c r="J299" t="s">
         <v>1521</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19566,7 +19592,7 @@
       <c r="J300" t="s">
         <v>1520</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19607,7 +19633,7 @@
       <c r="J301" t="s">
         <v>1520</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20445,7 +20471,7 @@
       <c r="R321" t="s">
         <v>1690</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20665,7 +20691,7 @@
       <c r="R326" t="s">
         <v>1729</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21500,7 +21526,7 @@
       <c r="R346" t="s">
         <v>1730</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (18/09/2026 16:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5342,8 +5342,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5359,7 +5367,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5367,12 +5375,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5672,73 +5698,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5773,7 +5799,7 @@
       <c r="J2" t="s">
         <v>1523</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5817,7 +5843,7 @@
       <c r="J3" t="s">
         <v>1523</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5861,7 +5887,7 @@
       <c r="J4" t="s">
         <v>1523</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5879,7 +5905,7 @@
       <c r="R4" t="s">
         <v>1690</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5917,7 +5943,7 @@
       <c r="J5" t="s">
         <v>1524</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5967,7 +5993,7 @@
       <c r="J6" t="s">
         <v>1523</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6014,7 +6040,7 @@
       <c r="J7" t="s">
         <v>1523</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6061,7 +6087,7 @@
       <c r="J8" t="s">
         <v>1523</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6108,7 +6134,7 @@
       <c r="J9" t="s">
         <v>1523</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6155,7 +6181,7 @@
       <c r="J10" t="s">
         <v>1523</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6202,7 +6228,7 @@
       <c r="J11" t="s">
         <v>1523</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6249,7 +6275,7 @@
       <c r="J12" t="s">
         <v>1523</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6293,7 +6319,7 @@
       <c r="J13" t="s">
         <v>1523</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6311,7 +6337,7 @@
       <c r="R13" t="s">
         <v>1691</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6349,7 +6375,7 @@
       <c r="J14" t="s">
         <v>1523</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6367,7 +6393,7 @@
       <c r="R14" t="s">
         <v>1692</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6405,7 +6431,7 @@
       <c r="J15" t="s">
         <v>1523</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6423,7 +6449,7 @@
       <c r="R15" t="s">
         <v>1692</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6464,7 +6490,7 @@
       <c r="J16" t="s">
         <v>1523</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6508,7 +6534,7 @@
       <c r="J17" t="s">
         <v>1523</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6552,7 +6578,7 @@
       <c r="J18" t="s">
         <v>1523</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6570,7 +6596,7 @@
       <c r="R18" t="s">
         <v>1693</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6611,7 +6637,7 @@
       <c r="J19" t="s">
         <v>1523</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6655,7 +6681,7 @@
       <c r="J20" t="s">
         <v>1523</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6699,7 +6725,7 @@
       <c r="J21" t="s">
         <v>1523</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6717,7 +6743,7 @@
       <c r="R21" t="s">
         <v>1692</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6758,7 +6784,7 @@
       <c r="J22" t="s">
         <v>1523</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6776,7 +6802,7 @@
       <c r="R22" t="s">
         <v>1694</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6817,7 +6843,7 @@
       <c r="J23" t="s">
         <v>1523</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6835,7 +6861,7 @@
       <c r="R23" t="s">
         <v>1695</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6876,7 +6902,7 @@
       <c r="J24" t="s">
         <v>1523</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6920,7 +6946,7 @@
       <c r="J25" t="s">
         <v>1523</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6961,7 +6987,7 @@
       <c r="J26" t="s">
         <v>1525</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6979,7 +7005,7 @@
       <c r="R26" t="s">
         <v>1696</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -7014,7 +7040,7 @@
       <c r="J27" t="s">
         <v>1523</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7032,7 +7058,7 @@
       <c r="R27" t="s">
         <v>1697</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7073,7 +7099,7 @@
       <c r="J28" t="s">
         <v>1523</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7117,7 +7143,7 @@
       <c r="J29" t="s">
         <v>1523</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7161,7 +7187,7 @@
       <c r="J30" t="s">
         <v>1523</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7205,7 +7231,7 @@
       <c r="J31" t="s">
         <v>1523</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7223,7 +7249,7 @@
       <c r="R31" t="s">
         <v>1698</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7264,7 +7290,7 @@
       <c r="J32" t="s">
         <v>1523</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7308,7 +7334,7 @@
       <c r="J33" t="s">
         <v>1523</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7326,7 +7352,7 @@
       <c r="R33" t="s">
         <v>1699</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7367,7 +7393,7 @@
       <c r="J34" t="s">
         <v>1523</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7411,7 +7437,7 @@
       <c r="J35" t="s">
         <v>1523</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7429,7 +7455,7 @@
       <c r="R35" t="s">
         <v>1700</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7470,7 +7496,7 @@
       <c r="J36" t="s">
         <v>1523</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7488,7 +7514,7 @@
       <c r="R36" t="s">
         <v>1700</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7529,7 +7555,7 @@
       <c r="J37" t="s">
         <v>1523</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7547,7 +7573,7 @@
       <c r="R37" t="s">
         <v>1700</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7588,7 +7614,7 @@
       <c r="J38" t="s">
         <v>1523</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7606,7 +7632,7 @@
       <c r="R38" t="s">
         <v>1700</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7647,7 +7673,7 @@
       <c r="J39" t="s">
         <v>1523</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7665,7 +7691,7 @@
       <c r="R39" t="s">
         <v>1700</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7706,7 +7732,7 @@
       <c r="J40" t="s">
         <v>1523</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7724,7 +7750,7 @@
       <c r="R40" t="s">
         <v>1701</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7765,7 +7791,7 @@
       <c r="J41" t="s">
         <v>1523</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7783,7 +7809,7 @@
       <c r="R41" t="s">
         <v>1692</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -7824,7 +7850,7 @@
       <c r="J42" t="s">
         <v>1523</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7842,7 +7868,7 @@
       <c r="R42" t="s">
         <v>1700</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7883,7 +7909,7 @@
       <c r="J43" t="s">
         <v>1523</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7927,7 +7953,7 @@
       <c r="J44" t="s">
         <v>1523</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7945,7 +7971,7 @@
       <c r="R44" t="s">
         <v>1702</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7986,7 +8012,7 @@
       <c r="J45" t="s">
         <v>1523</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8004,7 +8030,7 @@
       <c r="R45" t="s">
         <v>1703</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8042,7 +8068,7 @@
       <c r="J46" t="s">
         <v>1523</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8086,7 +8112,7 @@
       <c r="J47" t="s">
         <v>1523</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8104,7 +8130,7 @@
       <c r="R47" t="s">
         <v>1704</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8145,7 +8171,7 @@
       <c r="J48" t="s">
         <v>1523</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8189,7 +8215,7 @@
       <c r="J49" t="s">
         <v>1523</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8233,7 +8259,7 @@
       <c r="J50" t="s">
         <v>1523</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8277,7 +8303,7 @@
       <c r="J51" t="s">
         <v>1523</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8324,7 +8350,7 @@
       <c r="J52" t="s">
         <v>1523</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8368,7 +8394,7 @@
       <c r="J53" t="s">
         <v>1523</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8412,7 +8438,7 @@
       <c r="J54" t="s">
         <v>1523</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8456,7 +8482,7 @@
       <c r="J55" t="s">
         <v>1523</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8506,7 +8532,7 @@
       <c r="J56" t="s">
         <v>1523</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8559,7 +8585,7 @@
       <c r="J57" t="s">
         <v>1523</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8609,7 +8635,7 @@
       <c r="J58" t="s">
         <v>1523</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8659,7 +8685,7 @@
       <c r="J59" t="s">
         <v>1523</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8677,7 +8703,7 @@
       <c r="R59" t="s">
         <v>1705</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8718,7 +8744,7 @@
       <c r="J60" t="s">
         <v>1523</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8762,7 +8788,7 @@
       <c r="J61" t="s">
         <v>1523</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8806,7 +8832,7 @@
       <c r="J62" t="s">
         <v>1523</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8850,7 +8876,7 @@
       <c r="J63" t="s">
         <v>1523</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8894,7 +8920,7 @@
       <c r="J64" t="s">
         <v>1523</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8938,7 +8964,7 @@
       <c r="J65" t="s">
         <v>1523</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8985,7 +9011,7 @@
       <c r="J66" t="s">
         <v>1523</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9003,7 +9029,7 @@
       <c r="R66" t="s">
         <v>1706</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9041,7 +9067,7 @@
       <c r="J67" t="s">
         <v>1523</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9085,7 +9111,7 @@
       <c r="J68" t="s">
         <v>1523</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9100,7 +9126,7 @@
       <c r="O68" t="s">
         <v>1608</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9144,7 +9170,7 @@
       <c r="J69" t="s">
         <v>1525</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9188,7 +9214,7 @@
       <c r="J70" t="s">
         <v>1523</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9232,7 +9258,7 @@
       <c r="J71" t="s">
         <v>1523</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9276,7 +9302,7 @@
       <c r="J72" t="s">
         <v>1523</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9320,7 +9346,7 @@
       <c r="J73" t="s">
         <v>1523</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9364,7 +9390,7 @@
       <c r="J74" t="s">
         <v>1523</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9408,7 +9434,7 @@
       <c r="J75" t="s">
         <v>1523</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9452,7 +9478,7 @@
       <c r="J76" t="s">
         <v>1523</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9470,7 +9496,7 @@
       <c r="R76" t="s">
         <v>1707</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9508,7 +9534,7 @@
       <c r="J77" t="s">
         <v>1523</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9526,7 +9552,7 @@
       <c r="R77" t="s">
         <v>1707</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9564,7 +9590,7 @@
       <c r="J78" t="s">
         <v>1523</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9582,7 +9608,7 @@
       <c r="R78" t="s">
         <v>1707</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9620,7 +9646,7 @@
       <c r="J79" t="s">
         <v>1523</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9638,7 +9664,7 @@
       <c r="R79" t="s">
         <v>1707</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9676,7 +9702,7 @@
       <c r="J80" t="s">
         <v>1523</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9720,7 +9746,7 @@
       <c r="J81" t="s">
         <v>1523</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9764,7 +9790,7 @@
       <c r="J82" t="s">
         <v>1523</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9808,7 +9834,7 @@
       <c r="J83" t="s">
         <v>1523</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9852,7 +9878,7 @@
       <c r="J84" t="s">
         <v>1523</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9896,7 +9922,7 @@
       <c r="J85" t="s">
         <v>1523</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9914,7 +9940,7 @@
       <c r="R85" t="s">
         <v>1708</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9952,7 +9978,7 @@
       <c r="J86" t="s">
         <v>1523</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9996,7 +10022,7 @@
       <c r="J87" t="s">
         <v>1523</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10014,7 +10040,7 @@
       <c r="R87" t="s">
         <v>1709</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10052,7 +10078,7 @@
       <c r="J88" t="s">
         <v>1523</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10096,7 +10122,7 @@
       <c r="J89" t="s">
         <v>1523</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10114,7 +10140,7 @@
       <c r="R89" t="s">
         <v>1710</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10149,7 +10175,7 @@
       <c r="J90" t="s">
         <v>1523</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10167,7 +10193,7 @@
       <c r="R90" t="s">
         <v>1711</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10202,7 +10228,7 @@
       <c r="J91" t="s">
         <v>1523</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10220,7 +10246,7 @@
       <c r="R91" t="s">
         <v>1695</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10258,7 +10284,7 @@
       <c r="J92" t="s">
         <v>1523</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10279,7 +10305,7 @@
       <c r="R92" t="s">
         <v>1695</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10320,7 +10346,7 @@
       <c r="J93" t="s">
         <v>1523</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10361,7 +10387,7 @@
       <c r="J94" t="s">
         <v>1523</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10405,7 +10431,7 @@
       <c r="J95" t="s">
         <v>1523</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10449,7 +10475,7 @@
       <c r="J96" t="s">
         <v>1523</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10467,7 +10493,7 @@
       <c r="R96" t="s">
         <v>1712</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10505,7 +10531,7 @@
       <c r="J97" t="s">
         <v>1523</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10520,7 +10546,7 @@
       <c r="R97" t="s">
         <v>1712</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10561,7 +10587,7 @@
       <c r="J98" t="s">
         <v>1523</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10579,7 +10605,7 @@
       <c r="R98" t="s">
         <v>1713</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10617,7 +10643,7 @@
       <c r="J99" t="s">
         <v>1523</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10635,7 +10661,7 @@
       <c r="R99" t="s">
         <v>1714</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10673,7 +10699,7 @@
       <c r="J100" t="s">
         <v>1523</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10714,7 +10740,7 @@
       <c r="J101" t="s">
         <v>1523</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10755,7 +10781,7 @@
       <c r="J102" t="s">
         <v>1523</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10796,7 +10822,7 @@
       <c r="J103" t="s">
         <v>1523</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10837,7 +10863,7 @@
       <c r="J104" t="s">
         <v>1523</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10878,7 +10904,7 @@
       <c r="J105" t="s">
         <v>1523</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10919,7 +10945,7 @@
       <c r="J106" t="s">
         <v>1523</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10960,7 +10986,7 @@
       <c r="J107" t="s">
         <v>1523</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11001,7 +11027,7 @@
       <c r="J108" t="s">
         <v>1523</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11042,7 +11068,7 @@
       <c r="J109" t="s">
         <v>1523</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11095,7 +11121,7 @@
       <c r="J110" t="s">
         <v>1523</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11151,7 +11177,7 @@
       <c r="J111" t="s">
         <v>1523</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11169,7 +11195,7 @@
       <c r="R111" t="s">
         <v>1716</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11207,7 +11233,7 @@
       <c r="J112" t="s">
         <v>1523</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11266,7 +11292,7 @@
       <c r="J113" t="s">
         <v>1523</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11310,7 +11336,7 @@
       <c r="J114" t="s">
         <v>1523</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11354,7 +11380,7 @@
       <c r="J115" t="s">
         <v>1523</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11372,7 +11398,7 @@
       <c r="R115" t="s">
         <v>1718</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11410,7 +11436,7 @@
       <c r="J116" t="s">
         <v>1523</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11469,7 +11495,7 @@
       <c r="J117" t="s">
         <v>1523</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11513,7 +11539,7 @@
       <c r="J118" t="s">
         <v>1523</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11560,7 +11586,7 @@
       <c r="J119" t="s">
         <v>1523</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11601,7 +11627,7 @@
       <c r="J120" t="s">
         <v>1523</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11645,7 +11671,7 @@
       <c r="J121" t="s">
         <v>1523</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11692,7 +11718,7 @@
       <c r="J122" t="s">
         <v>1523</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11742,7 +11768,7 @@
       <c r="J123" t="s">
         <v>1523</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11786,7 +11812,7 @@
       <c r="J124" t="s">
         <v>1523</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11830,7 +11856,7 @@
       <c r="J125" t="s">
         <v>1523</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11848,7 +11874,7 @@
       <c r="R125" t="s">
         <v>1720</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11883,7 +11909,7 @@
       <c r="J126" t="s">
         <v>1523</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11901,7 +11927,7 @@
       <c r="R126" t="s">
         <v>1721</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11936,7 +11962,7 @@
       <c r="J127" t="s">
         <v>1523</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11992,7 +12018,7 @@
       <c r="J128" t="s">
         <v>1523</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12033,7 +12059,7 @@
       <c r="J129" t="s">
         <v>1523</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12074,7 +12100,7 @@
       <c r="J130" t="s">
         <v>1523</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12115,7 +12141,7 @@
       <c r="J131" t="s">
         <v>1523</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12159,7 +12185,7 @@
       <c r="J132" t="s">
         <v>1523</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12200,7 +12226,7 @@
       <c r="J133" t="s">
         <v>1523</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12218,7 +12244,7 @@
       <c r="R133" t="s">
         <v>1707</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12253,7 +12279,7 @@
       <c r="J134" t="s">
         <v>1523</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12271,7 +12297,7 @@
       <c r="R134" t="s">
         <v>1707</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12306,7 +12332,7 @@
       <c r="J135" t="s">
         <v>1523</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12347,7 +12373,7 @@
       <c r="J136" t="s">
         <v>1523</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12388,7 +12414,7 @@
       <c r="J137" t="s">
         <v>1523</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12429,7 +12455,7 @@
       <c r="J138" t="s">
         <v>1523</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12470,7 +12496,7 @@
       <c r="J139" t="s">
         <v>1523</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12517,7 +12543,7 @@
       <c r="J140" t="s">
         <v>1523</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12558,7 +12584,7 @@
       <c r="J141" t="s">
         <v>1523</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12599,7 +12625,7 @@
       <c r="J142" t="s">
         <v>1523</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12643,7 +12669,7 @@
       <c r="J143" t="s">
         <v>1523</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12661,7 +12687,7 @@
       <c r="R143" t="s">
         <v>1707</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12696,7 +12722,7 @@
       <c r="J144" t="s">
         <v>1523</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12714,7 +12740,7 @@
       <c r="R144" t="s">
         <v>1707</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12749,7 +12775,7 @@
       <c r="J145" t="s">
         <v>1523</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12767,7 +12793,7 @@
       <c r="R145" t="s">
         <v>1707</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12802,7 +12828,7 @@
       <c r="J146" t="s">
         <v>1523</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12820,7 +12846,7 @@
       <c r="R146" t="s">
         <v>1715</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12855,7 +12881,7 @@
       <c r="J147" t="s">
         <v>1523</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12873,7 +12899,7 @@
       <c r="R147" t="s">
         <v>1722</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12908,7 +12934,7 @@
       <c r="J148" t="s">
         <v>1523</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12949,7 +12975,7 @@
       <c r="J149" t="s">
         <v>1523</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12967,7 +12993,7 @@
       <c r="R149" t="s">
         <v>1707</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13002,7 +13028,7 @@
       <c r="J150" t="s">
         <v>1523</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13020,7 +13046,7 @@
       <c r="R150" t="s">
         <v>1707</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13055,7 +13081,7 @@
       <c r="J151" t="s">
         <v>1523</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13073,7 +13099,7 @@
       <c r="R151" t="s">
         <v>1723</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13108,7 +13134,7 @@
       <c r="J152" t="s">
         <v>1523</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13126,7 +13152,7 @@
       <c r="R152" t="s">
         <v>1724</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13161,7 +13187,7 @@
       <c r="J153" t="s">
         <v>1523</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13170,7 +13196,7 @@
       <c r="M153" t="s">
         <v>1599</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13211,7 +13237,7 @@
       <c r="J154" t="s">
         <v>1523</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13252,7 +13278,7 @@
       <c r="J155" t="s">
         <v>1523</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13293,7 +13319,7 @@
       <c r="J156" t="s">
         <v>1523</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13334,7 +13360,7 @@
       <c r="J157" t="s">
         <v>1523</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13375,7 +13401,7 @@
       <c r="J158" t="s">
         <v>1523</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13416,7 +13442,7 @@
       <c r="J159" t="s">
         <v>1523</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13457,7 +13483,7 @@
       <c r="J160" t="s">
         <v>1523</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13498,7 +13524,7 @@
       <c r="J161" t="s">
         <v>1523</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13539,7 +13565,7 @@
       <c r="J162" t="s">
         <v>1523</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13557,7 +13583,7 @@
       <c r="R162" t="s">
         <v>1710</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13592,7 +13618,7 @@
       <c r="J163" t="s">
         <v>1523</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13610,7 +13636,7 @@
       <c r="R163" t="s">
         <v>1707</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13645,7 +13671,7 @@
       <c r="J164" t="s">
         <v>1523</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13689,7 +13715,7 @@
       <c r="J165" t="s">
         <v>1523</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13730,7 +13756,7 @@
       <c r="J166" t="s">
         <v>1523</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13748,7 +13774,7 @@
       <c r="R166" t="s">
         <v>1725</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13783,7 +13809,7 @@
       <c r="J167" t="s">
         <v>1523</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13827,7 +13853,7 @@
       <c r="J168" t="s">
         <v>1523</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13871,7 +13897,7 @@
       <c r="J169" t="s">
         <v>1523</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13912,7 +13938,7 @@
       <c r="J170" t="s">
         <v>1523</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13953,7 +13979,7 @@
       <c r="J171" t="s">
         <v>1523</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13994,7 +14020,7 @@
       <c r="J172" t="s">
         <v>1523</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14035,7 +14061,7 @@
       <c r="J173" t="s">
         <v>1523</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14076,7 +14102,7 @@
       <c r="J174" t="s">
         <v>1523</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14117,7 +14143,7 @@
       <c r="J175" t="s">
         <v>1523</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14158,7 +14184,7 @@
       <c r="J176" t="s">
         <v>1523</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14199,7 +14225,7 @@
       <c r="J177" t="s">
         <v>1523</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14240,7 +14266,7 @@
       <c r="J178" t="s">
         <v>1523</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14258,7 +14284,7 @@
       <c r="R178" t="s">
         <v>1723</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14296,7 +14322,7 @@
       <c r="J179" t="s">
         <v>1523</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14305,7 +14331,7 @@
       <c r="M179" t="s">
         <v>1596</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14346,7 +14372,7 @@
       <c r="J180" t="s">
         <v>1523</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14387,7 +14413,7 @@
       <c r="J181" t="s">
         <v>1523</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14405,7 +14431,7 @@
       <c r="R181" t="s">
         <v>1707</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14440,7 +14466,7 @@
       <c r="J182" t="s">
         <v>1523</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14481,7 +14507,7 @@
       <c r="J183" t="s">
         <v>1523</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14522,7 +14548,7 @@
       <c r="J184" t="s">
         <v>1523</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14563,7 +14589,7 @@
       <c r="J185" t="s">
         <v>1523</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14604,7 +14630,7 @@
       <c r="J186" t="s">
         <v>1523</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14645,7 +14671,7 @@
       <c r="J187" t="s">
         <v>1523</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14686,7 +14712,7 @@
       <c r="J188" t="s">
         <v>1523</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14727,7 +14753,7 @@
       <c r="J189" t="s">
         <v>1523</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14768,7 +14794,7 @@
       <c r="J190" t="s">
         <v>1523</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14809,7 +14835,7 @@
       <c r="J191" t="s">
         <v>1523</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14850,7 +14876,7 @@
       <c r="J192" t="s">
         <v>1523</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14891,7 +14917,7 @@
       <c r="J193" t="s">
         <v>1523</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14932,7 +14958,7 @@
       <c r="J194" t="s">
         <v>1523</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14973,7 +14999,7 @@
       <c r="J195" t="s">
         <v>1523</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14991,7 +15017,7 @@
       <c r="R195" t="s">
         <v>1716</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15032,7 +15058,7 @@
       <c r="J196" t="s">
         <v>1523</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15050,7 +15076,7 @@
       <c r="R196" t="s">
         <v>1722</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15088,7 +15114,7 @@
       <c r="J197" t="s">
         <v>1523</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15129,7 +15155,7 @@
       <c r="J198" t="s">
         <v>1525</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15170,7 +15196,7 @@
       <c r="J199" t="s">
         <v>1524</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15211,7 +15237,7 @@
       <c r="J200" t="s">
         <v>1523</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15252,7 +15278,7 @@
       <c r="J201" t="s">
         <v>1523</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15293,7 +15319,7 @@
       <c r="J202" t="s">
         <v>1523</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15311,7 +15337,7 @@
       <c r="R202" t="s">
         <v>1707</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15346,7 +15372,7 @@
       <c r="J203" t="s">
         <v>1523</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15364,7 +15390,7 @@
       <c r="R203" t="s">
         <v>1715</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15399,7 +15425,7 @@
       <c r="J204" t="s">
         <v>1523</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15414,7 +15440,7 @@
       <c r="R204" t="s">
         <v>1726</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15452,7 +15478,7 @@
       <c r="J205" t="s">
         <v>1523</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15470,7 +15496,7 @@
       <c r="R205" t="s">
         <v>1727</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15508,7 +15534,7 @@
       <c r="J206" t="s">
         <v>1523</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15526,7 +15552,7 @@
       <c r="R206" t="s">
         <v>1695</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15561,7 +15587,7 @@
       <c r="J207" t="s">
         <v>1523</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15602,7 +15628,7 @@
       <c r="J208" t="s">
         <v>1523</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15643,7 +15669,7 @@
       <c r="J209" t="s">
         <v>1523</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15684,7 +15710,7 @@
       <c r="J210" t="s">
         <v>1523</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15725,7 +15751,7 @@
       <c r="J211" t="s">
         <v>1523</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15766,7 +15792,7 @@
       <c r="J212" t="s">
         <v>1523</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15807,7 +15833,7 @@
       <c r="J213" t="s">
         <v>1523</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15848,7 +15874,7 @@
       <c r="J214" t="s">
         <v>1523</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15866,7 +15892,7 @@
       <c r="R214" t="s">
         <v>1728</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15901,7 +15927,7 @@
       <c r="J215" t="s">
         <v>1523</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15942,7 +15968,7 @@
       <c r="J216" t="s">
         <v>1523</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15983,7 +16009,7 @@
       <c r="J217" t="s">
         <v>1523</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16024,7 +16050,7 @@
       <c r="J218" t="s">
         <v>1523</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16065,7 +16091,7 @@
       <c r="J219" t="s">
         <v>1523</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16106,7 +16132,7 @@
       <c r="J220" t="s">
         <v>1523</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16147,7 +16173,7 @@
       <c r="J221" t="s">
         <v>1523</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16188,7 +16214,7 @@
       <c r="J222" t="s">
         <v>1523</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16229,7 +16255,7 @@
       <c r="J223" t="s">
         <v>1523</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16270,7 +16296,7 @@
       <c r="J224" t="s">
         <v>1523</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16311,7 +16337,7 @@
       <c r="J225" t="s">
         <v>1523</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16352,7 +16378,7 @@
       <c r="J226" t="s">
         <v>1523</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16393,7 +16419,7 @@
       <c r="J227" t="s">
         <v>1523</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16434,7 +16460,7 @@
       <c r="J228" t="s">
         <v>1523</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16475,7 +16501,7 @@
       <c r="J229" t="s">
         <v>1523</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16516,7 +16542,7 @@
       <c r="J230" t="s">
         <v>1523</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16557,7 +16583,7 @@
       <c r="J231" t="s">
         <v>1523</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16598,7 +16624,7 @@
       <c r="J232" t="s">
         <v>1523</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16639,7 +16665,7 @@
       <c r="J233" t="s">
         <v>1523</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16680,7 +16706,7 @@
       <c r="J234" t="s">
         <v>1523</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16721,7 +16747,7 @@
       <c r="J235" t="s">
         <v>1523</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16762,7 +16788,7 @@
       <c r="J236" t="s">
         <v>1523</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16803,7 +16829,7 @@
       <c r="J237" t="s">
         <v>1523</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16844,7 +16870,7 @@
       <c r="J238" t="s">
         <v>1523</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16885,7 +16911,7 @@
       <c r="J239" t="s">
         <v>1523</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16903,7 +16929,7 @@
       <c r="R239" t="s">
         <v>1722</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -16941,7 +16967,7 @@
       <c r="J240" t="s">
         <v>1523</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16982,7 +17008,7 @@
       <c r="J241" t="s">
         <v>1523</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17023,7 +17049,7 @@
       <c r="J242" t="s">
         <v>1523</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17041,7 +17067,7 @@
       <c r="R242" t="s">
         <v>1715</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17076,7 +17102,7 @@
       <c r="J243" t="s">
         <v>1523</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17117,7 +17143,7 @@
       <c r="J244" t="s">
         <v>1523</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17158,7 +17184,7 @@
       <c r="J245" t="s">
         <v>1523</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17199,7 +17225,7 @@
       <c r="J246" t="s">
         <v>1523</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17217,7 +17243,7 @@
       <c r="R246" t="s">
         <v>1695</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17255,7 +17281,7 @@
       <c r="J247" t="s">
         <v>1523</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17296,7 +17322,7 @@
       <c r="J248" t="s">
         <v>1523</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17337,7 +17363,7 @@
       <c r="J249" t="s">
         <v>1523</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17378,7 +17404,7 @@
       <c r="J250" t="s">
         <v>1523</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17419,7 +17445,7 @@
       <c r="J251" t="s">
         <v>1523</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17460,7 +17486,7 @@
       <c r="J252" t="s">
         <v>1523</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17501,7 +17527,7 @@
       <c r="J253" t="s">
         <v>1523</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17519,7 +17545,7 @@
       <c r="R253" t="s">
         <v>1725</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17557,7 +17583,7 @@
       <c r="J254" t="s">
         <v>1523</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17598,7 +17624,7 @@
       <c r="J255" t="s">
         <v>1523</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17639,7 +17665,7 @@
       <c r="J256" t="s">
         <v>1523</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17648,7 +17674,7 @@
       <c r="M256" t="s">
         <v>1595</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17686,7 +17712,7 @@
       <c r="J257" t="s">
         <v>1523</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17695,7 +17721,7 @@
       <c r="M257" t="s">
         <v>1596</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17739,7 +17765,7 @@
       <c r="J258" t="s">
         <v>1523</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17757,7 +17783,7 @@
       <c r="R258" t="s">
         <v>1707</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17795,7 +17821,7 @@
       <c r="J259" t="s">
         <v>1523</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17813,7 +17839,7 @@
       <c r="R259" t="s">
         <v>1723</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17851,7 +17877,7 @@
       <c r="J260" t="s">
         <v>1523</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17860,7 +17886,7 @@
       <c r="M260" t="s">
         <v>1590</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17904,7 +17930,7 @@
       <c r="J261" t="s">
         <v>1523</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17922,7 +17948,7 @@
       <c r="R261" t="s">
         <v>1729</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17960,7 +17986,7 @@
       <c r="J262" t="s">
         <v>1523</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17978,7 +18004,7 @@
       <c r="R262" t="s">
         <v>1723</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18016,7 +18042,7 @@
       <c r="J263" t="s">
         <v>1523</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18025,7 +18051,7 @@
       <c r="M263" t="s">
         <v>1590</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18069,7 +18095,7 @@
       <c r="J264" t="s">
         <v>1523</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18110,7 +18136,7 @@
       <c r="J265" t="s">
         <v>1523</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18151,7 +18177,7 @@
       <c r="J266" t="s">
         <v>1523</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18192,7 +18218,7 @@
       <c r="J267" t="s">
         <v>1523</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18236,7 +18262,7 @@
       <c r="J268" t="s">
         <v>1523</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18277,7 +18303,7 @@
       <c r="J269" t="s">
         <v>1523</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18318,7 +18344,7 @@
       <c r="J270" t="s">
         <v>1523</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18359,7 +18385,7 @@
       <c r="J271" t="s">
         <v>1523</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18400,7 +18426,7 @@
       <c r="J272" t="s">
         <v>1523</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18418,7 +18444,7 @@
       <c r="R272" t="s">
         <v>1730</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18456,7 +18482,7 @@
       <c r="J273" t="s">
         <v>1523</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18500,7 +18526,7 @@
       <c r="J274" t="s">
         <v>1523</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18541,7 +18567,7 @@
       <c r="J275" t="s">
         <v>1523</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18582,7 +18608,7 @@
       <c r="J276" t="s">
         <v>1523</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18623,7 +18649,7 @@
       <c r="J277" t="s">
         <v>1523</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18664,7 +18690,7 @@
       <c r="J278" t="s">
         <v>1523</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18705,7 +18731,7 @@
       <c r="J279" t="s">
         <v>1523</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18746,7 +18772,7 @@
       <c r="J280" t="s">
         <v>1523</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18787,7 +18813,7 @@
       <c r="J281" t="s">
         <v>1523</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18828,7 +18854,7 @@
       <c r="J282" t="s">
         <v>1523</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18869,7 +18895,7 @@
       <c r="J283" t="s">
         <v>1523</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18910,7 +18936,7 @@
       <c r="J284" t="s">
         <v>1523</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18951,7 +18977,7 @@
       <c r="J285" t="s">
         <v>1523</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18992,7 +19018,7 @@
       <c r="J286" t="s">
         <v>1523</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19033,7 +19059,7 @@
       <c r="J287" t="s">
         <v>1523</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19074,7 +19100,7 @@
       <c r="J288" t="s">
         <v>1523</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19115,7 +19141,7 @@
       <c r="J289" t="s">
         <v>1523</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19156,7 +19182,7 @@
       <c r="J290" t="s">
         <v>1523</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19197,7 +19223,7 @@
       <c r="J291" t="s">
         <v>1523</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19238,7 +19264,7 @@
       <c r="J292" t="s">
         <v>1523</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19279,7 +19305,7 @@
       <c r="J293" t="s">
         <v>1523</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19320,7 +19346,7 @@
       <c r="J294" t="s">
         <v>1523</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19361,7 +19387,7 @@
       <c r="J295" t="s">
         <v>1523</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19379,7 +19405,7 @@
       <c r="R295" t="s">
         <v>1731</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19420,7 +19446,7 @@
       <c r="J296" t="s">
         <v>1523</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19438,7 +19464,7 @@
       <c r="R296" t="s">
         <v>1707</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19476,7 +19502,7 @@
       <c r="J297" t="s">
         <v>1523</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19517,7 +19543,7 @@
       <c r="J298" t="s">
         <v>1523</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19558,7 +19584,7 @@
       <c r="J299" t="s">
         <v>1524</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19599,7 +19625,7 @@
       <c r="J300" t="s">
         <v>1523</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19640,7 +19666,7 @@
       <c r="J301" t="s">
         <v>1523</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20478,7 +20504,7 @@
       <c r="R321" t="s">
         <v>1693</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -20701,7 +20727,7 @@
       <c r="R326" t="s">
         <v>1732</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21536,7 +21562,7 @@
       <c r="R346" t="s">
         <v>1733</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (21/09/2026 14:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5342,16 +5342,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5367,7 +5359,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5375,30 +5367,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5698,73 +5672,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5799,7 +5773,7 @@
       <c r="J2" t="s">
         <v>1523</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5843,7 +5817,7 @@
       <c r="J3" t="s">
         <v>1523</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5887,7 +5861,7 @@
       <c r="J4" t="s">
         <v>1523</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5905,7 +5879,7 @@
       <c r="R4" t="s">
         <v>1690</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5943,7 +5917,7 @@
       <c r="J5" t="s">
         <v>1524</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5993,7 +5967,7 @@
       <c r="J6" t="s">
         <v>1523</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6040,7 +6014,7 @@
       <c r="J7" t="s">
         <v>1523</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6087,7 +6061,7 @@
       <c r="J8" t="s">
         <v>1523</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6134,7 +6108,7 @@
       <c r="J9" t="s">
         <v>1523</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6181,7 +6155,7 @@
       <c r="J10" t="s">
         <v>1523</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6228,7 +6202,7 @@
       <c r="J11" t="s">
         <v>1523</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6275,7 +6249,7 @@
       <c r="J12" t="s">
         <v>1523</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6319,7 +6293,7 @@
       <c r="J13" t="s">
         <v>1523</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6337,7 +6311,7 @@
       <c r="R13" t="s">
         <v>1691</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6375,7 +6349,7 @@
       <c r="J14" t="s">
         <v>1523</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6393,7 +6367,7 @@
       <c r="R14" t="s">
         <v>1692</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6431,7 +6405,7 @@
       <c r="J15" t="s">
         <v>1523</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6449,7 +6423,7 @@
       <c r="R15" t="s">
         <v>1692</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6490,7 +6464,7 @@
       <c r="J16" t="s">
         <v>1523</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6534,7 +6508,7 @@
       <c r="J17" t="s">
         <v>1523</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6578,7 +6552,7 @@
       <c r="J18" t="s">
         <v>1523</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6596,7 +6570,7 @@
       <c r="R18" t="s">
         <v>1693</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6637,7 +6611,7 @@
       <c r="J19" t="s">
         <v>1523</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6681,7 +6655,7 @@
       <c r="J20" t="s">
         <v>1523</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6725,7 +6699,7 @@
       <c r="J21" t="s">
         <v>1523</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6743,7 +6717,7 @@
       <c r="R21" t="s">
         <v>1692</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6784,7 +6758,7 @@
       <c r="J22" t="s">
         <v>1523</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6802,7 +6776,7 @@
       <c r="R22" t="s">
         <v>1694</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6843,7 +6817,7 @@
       <c r="J23" t="s">
         <v>1523</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6861,7 +6835,7 @@
       <c r="R23" t="s">
         <v>1695</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6902,7 +6876,7 @@
       <c r="J24" t="s">
         <v>1523</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6946,7 +6920,7 @@
       <c r="J25" t="s">
         <v>1523</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6987,7 +6961,7 @@
       <c r="J26" t="s">
         <v>1525</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7005,7 +6979,7 @@
       <c r="R26" t="s">
         <v>1696</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -7040,7 +7014,7 @@
       <c r="J27" t="s">
         <v>1523</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7058,7 +7032,7 @@
       <c r="R27" t="s">
         <v>1697</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7099,7 +7073,7 @@
       <c r="J28" t="s">
         <v>1523</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7143,7 +7117,7 @@
       <c r="J29" t="s">
         <v>1523</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7187,7 +7161,7 @@
       <c r="J30" t="s">
         <v>1523</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7231,7 +7205,7 @@
       <c r="J31" t="s">
         <v>1523</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7249,7 +7223,7 @@
       <c r="R31" t="s">
         <v>1698</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7290,7 +7264,7 @@
       <c r="J32" t="s">
         <v>1523</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7334,7 +7308,7 @@
       <c r="J33" t="s">
         <v>1523</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7352,7 +7326,7 @@
       <c r="R33" t="s">
         <v>1699</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7393,7 +7367,7 @@
       <c r="J34" t="s">
         <v>1523</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7437,7 +7411,7 @@
       <c r="J35" t="s">
         <v>1523</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7455,7 +7429,7 @@
       <c r="R35" t="s">
         <v>1700</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7496,7 +7470,7 @@
       <c r="J36" t="s">
         <v>1523</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7514,7 +7488,7 @@
       <c r="R36" t="s">
         <v>1700</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7555,7 +7529,7 @@
       <c r="J37" t="s">
         <v>1523</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7573,7 +7547,7 @@
       <c r="R37" t="s">
         <v>1700</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7614,7 +7588,7 @@
       <c r="J38" t="s">
         <v>1523</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7632,7 +7606,7 @@
       <c r="R38" t="s">
         <v>1700</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7673,7 +7647,7 @@
       <c r="J39" t="s">
         <v>1523</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7691,7 +7665,7 @@
       <c r="R39" t="s">
         <v>1700</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7732,7 +7706,7 @@
       <c r="J40" t="s">
         <v>1523</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7750,7 +7724,7 @@
       <c r="R40" t="s">
         <v>1701</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7791,7 +7765,7 @@
       <c r="J41" t="s">
         <v>1523</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7809,7 +7783,7 @@
       <c r="R41" t="s">
         <v>1692</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -7850,7 +7824,7 @@
       <c r="J42" t="s">
         <v>1523</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7868,7 +7842,7 @@
       <c r="R42" t="s">
         <v>1700</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7909,7 +7883,7 @@
       <c r="J43" t="s">
         <v>1523</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7953,7 +7927,7 @@
       <c r="J44" t="s">
         <v>1523</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7971,7 +7945,7 @@
       <c r="R44" t="s">
         <v>1702</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8012,7 +7986,7 @@
       <c r="J45" t="s">
         <v>1523</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8030,7 +8004,7 @@
       <c r="R45" t="s">
         <v>1703</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8068,7 +8042,7 @@
       <c r="J46" t="s">
         <v>1523</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8112,7 +8086,7 @@
       <c r="J47" t="s">
         <v>1523</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8130,7 +8104,7 @@
       <c r="R47" t="s">
         <v>1704</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8171,7 +8145,7 @@
       <c r="J48" t="s">
         <v>1523</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8215,7 +8189,7 @@
       <c r="J49" t="s">
         <v>1523</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8259,7 +8233,7 @@
       <c r="J50" t="s">
         <v>1523</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8303,7 +8277,7 @@
       <c r="J51" t="s">
         <v>1523</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8350,7 +8324,7 @@
       <c r="J52" t="s">
         <v>1523</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8394,7 +8368,7 @@
       <c r="J53" t="s">
         <v>1523</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8438,7 +8412,7 @@
       <c r="J54" t="s">
         <v>1523</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8482,7 +8456,7 @@
       <c r="J55" t="s">
         <v>1523</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8532,7 +8506,7 @@
       <c r="J56" t="s">
         <v>1523</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8585,7 +8559,7 @@
       <c r="J57" t="s">
         <v>1523</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8635,7 +8609,7 @@
       <c r="J58" t="s">
         <v>1523</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8685,7 +8659,7 @@
       <c r="J59" t="s">
         <v>1523</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8703,7 +8677,7 @@
       <c r="R59" t="s">
         <v>1705</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8744,7 +8718,7 @@
       <c r="J60" t="s">
         <v>1523</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8788,7 +8762,7 @@
       <c r="J61" t="s">
         <v>1523</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8832,7 +8806,7 @@
       <c r="J62" t="s">
         <v>1523</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8876,7 +8850,7 @@
       <c r="J63" t="s">
         <v>1523</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8920,7 +8894,7 @@
       <c r="J64" t="s">
         <v>1523</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8964,7 +8938,7 @@
       <c r="J65" t="s">
         <v>1523</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9011,7 +8985,7 @@
       <c r="J66" t="s">
         <v>1523</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9029,7 +9003,7 @@
       <c r="R66" t="s">
         <v>1706</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9067,7 +9041,7 @@
       <c r="J67" t="s">
         <v>1523</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9111,7 +9085,7 @@
       <c r="J68" t="s">
         <v>1523</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9126,7 +9100,7 @@
       <c r="O68" t="s">
         <v>1608</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9170,7 +9144,7 @@
       <c r="J69" t="s">
         <v>1525</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9214,7 +9188,7 @@
       <c r="J70" t="s">
         <v>1523</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9258,7 +9232,7 @@
       <c r="J71" t="s">
         <v>1523</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9302,7 +9276,7 @@
       <c r="J72" t="s">
         <v>1523</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9346,7 +9320,7 @@
       <c r="J73" t="s">
         <v>1523</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9390,7 +9364,7 @@
       <c r="J74" t="s">
         <v>1523</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9434,7 +9408,7 @@
       <c r="J75" t="s">
         <v>1523</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9478,7 +9452,7 @@
       <c r="J76" t="s">
         <v>1523</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9496,7 +9470,7 @@
       <c r="R76" t="s">
         <v>1707</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9534,7 +9508,7 @@
       <c r="J77" t="s">
         <v>1523</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9552,7 +9526,7 @@
       <c r="R77" t="s">
         <v>1707</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9590,7 +9564,7 @@
       <c r="J78" t="s">
         <v>1523</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9608,7 +9582,7 @@
       <c r="R78" t="s">
         <v>1707</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9646,7 +9620,7 @@
       <c r="J79" t="s">
         <v>1523</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9664,7 +9638,7 @@
       <c r="R79" t="s">
         <v>1707</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9702,7 +9676,7 @@
       <c r="J80" t="s">
         <v>1523</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9746,7 +9720,7 @@
       <c r="J81" t="s">
         <v>1523</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9790,7 +9764,7 @@
       <c r="J82" t="s">
         <v>1523</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9834,7 +9808,7 @@
       <c r="J83" t="s">
         <v>1523</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9878,7 +9852,7 @@
       <c r="J84" t="s">
         <v>1523</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9922,7 +9896,7 @@
       <c r="J85" t="s">
         <v>1523</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9940,7 +9914,7 @@
       <c r="R85" t="s">
         <v>1708</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9978,7 +9952,7 @@
       <c r="J86" t="s">
         <v>1523</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10022,7 +9996,7 @@
       <c r="J87" t="s">
         <v>1523</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10040,7 +10014,7 @@
       <c r="R87" t="s">
         <v>1709</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10078,7 +10052,7 @@
       <c r="J88" t="s">
         <v>1523</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10122,7 +10096,7 @@
       <c r="J89" t="s">
         <v>1523</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10140,7 +10114,7 @@
       <c r="R89" t="s">
         <v>1710</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10175,7 +10149,7 @@
       <c r="J90" t="s">
         <v>1523</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10193,7 +10167,7 @@
       <c r="R90" t="s">
         <v>1711</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10228,7 +10202,7 @@
       <c r="J91" t="s">
         <v>1523</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10246,7 +10220,7 @@
       <c r="R91" t="s">
         <v>1695</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10284,7 +10258,7 @@
       <c r="J92" t="s">
         <v>1523</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10305,7 +10279,7 @@
       <c r="R92" t="s">
         <v>1695</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10346,7 +10320,7 @@
       <c r="J93" t="s">
         <v>1523</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10387,7 +10361,7 @@
       <c r="J94" t="s">
         <v>1523</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10431,7 +10405,7 @@
       <c r="J95" t="s">
         <v>1523</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10475,7 +10449,7 @@
       <c r="J96" t="s">
         <v>1523</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10493,7 +10467,7 @@
       <c r="R96" t="s">
         <v>1712</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10531,7 +10505,7 @@
       <c r="J97" t="s">
         <v>1523</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10546,7 +10520,7 @@
       <c r="R97" t="s">
         <v>1712</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10587,7 +10561,7 @@
       <c r="J98" t="s">
         <v>1523</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10605,7 +10579,7 @@
       <c r="R98" t="s">
         <v>1713</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10643,7 +10617,7 @@
       <c r="J99" t="s">
         <v>1523</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10661,7 +10635,7 @@
       <c r="R99" t="s">
         <v>1714</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10699,7 +10673,7 @@
       <c r="J100" t="s">
         <v>1523</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10740,7 +10714,7 @@
       <c r="J101" t="s">
         <v>1523</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10781,7 +10755,7 @@
       <c r="J102" t="s">
         <v>1523</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10822,7 +10796,7 @@
       <c r="J103" t="s">
         <v>1523</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10863,7 +10837,7 @@
       <c r="J104" t="s">
         <v>1523</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10904,7 +10878,7 @@
       <c r="J105" t="s">
         <v>1523</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10945,7 +10919,7 @@
       <c r="J106" t="s">
         <v>1523</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10986,7 +10960,7 @@
       <c r="J107" t="s">
         <v>1523</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11027,7 +11001,7 @@
       <c r="J108" t="s">
         <v>1523</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11068,7 +11042,7 @@
       <c r="J109" t="s">
         <v>1523</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11121,7 +11095,7 @@
       <c r="J110" t="s">
         <v>1523</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11177,7 +11151,7 @@
       <c r="J111" t="s">
         <v>1523</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11195,7 +11169,7 @@
       <c r="R111" t="s">
         <v>1716</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11233,7 +11207,7 @@
       <c r="J112" t="s">
         <v>1523</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11292,7 +11266,7 @@
       <c r="J113" t="s">
         <v>1523</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11336,7 +11310,7 @@
       <c r="J114" t="s">
         <v>1523</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11380,7 +11354,7 @@
       <c r="J115" t="s">
         <v>1523</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11398,7 +11372,7 @@
       <c r="R115" t="s">
         <v>1718</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11436,7 +11410,7 @@
       <c r="J116" t="s">
         <v>1523</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11495,7 +11469,7 @@
       <c r="J117" t="s">
         <v>1523</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11539,7 +11513,7 @@
       <c r="J118" t="s">
         <v>1523</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11586,7 +11560,7 @@
       <c r="J119" t="s">
         <v>1523</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11627,7 +11601,7 @@
       <c r="J120" t="s">
         <v>1523</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11671,7 +11645,7 @@
       <c r="J121" t="s">
         <v>1523</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11718,7 +11692,7 @@
       <c r="J122" t="s">
         <v>1523</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11768,7 +11742,7 @@
       <c r="J123" t="s">
         <v>1523</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11812,7 +11786,7 @@
       <c r="J124" t="s">
         <v>1523</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11856,7 +11830,7 @@
       <c r="J125" t="s">
         <v>1523</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11874,7 +11848,7 @@
       <c r="R125" t="s">
         <v>1720</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11909,7 +11883,7 @@
       <c r="J126" t="s">
         <v>1523</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11927,7 +11901,7 @@
       <c r="R126" t="s">
         <v>1721</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11962,7 +11936,7 @@
       <c r="J127" t="s">
         <v>1523</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12018,7 +11992,7 @@
       <c r="J128" t="s">
         <v>1523</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12059,7 +12033,7 @@
       <c r="J129" t="s">
         <v>1523</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12100,7 +12074,7 @@
       <c r="J130" t="s">
         <v>1523</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12141,7 +12115,7 @@
       <c r="J131" t="s">
         <v>1523</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12185,7 +12159,7 @@
       <c r="J132" t="s">
         <v>1523</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12226,7 +12200,7 @@
       <c r="J133" t="s">
         <v>1523</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12244,7 +12218,7 @@
       <c r="R133" t="s">
         <v>1707</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12279,7 +12253,7 @@
       <c r="J134" t="s">
         <v>1523</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12297,7 +12271,7 @@
       <c r="R134" t="s">
         <v>1707</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12332,7 +12306,7 @@
       <c r="J135" t="s">
         <v>1523</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12373,7 +12347,7 @@
       <c r="J136" t="s">
         <v>1523</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12414,7 +12388,7 @@
       <c r="J137" t="s">
         <v>1523</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12455,7 +12429,7 @@
       <c r="J138" t="s">
         <v>1523</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12496,7 +12470,7 @@
       <c r="J139" t="s">
         <v>1523</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12543,7 +12517,7 @@
       <c r="J140" t="s">
         <v>1523</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12584,7 +12558,7 @@
       <c r="J141" t="s">
         <v>1523</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12625,7 +12599,7 @@
       <c r="J142" t="s">
         <v>1523</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12669,7 +12643,7 @@
       <c r="J143" t="s">
         <v>1523</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12687,7 +12661,7 @@
       <c r="R143" t="s">
         <v>1707</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12722,7 +12696,7 @@
       <c r="J144" t="s">
         <v>1523</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12740,7 +12714,7 @@
       <c r="R144" t="s">
         <v>1707</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12775,7 +12749,7 @@
       <c r="J145" t="s">
         <v>1523</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12793,7 +12767,7 @@
       <c r="R145" t="s">
         <v>1707</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12828,7 +12802,7 @@
       <c r="J146" t="s">
         <v>1523</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12846,7 +12820,7 @@
       <c r="R146" t="s">
         <v>1715</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12881,7 +12855,7 @@
       <c r="J147" t="s">
         <v>1523</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12899,7 +12873,7 @@
       <c r="R147" t="s">
         <v>1722</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12934,7 +12908,7 @@
       <c r="J148" t="s">
         <v>1523</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12975,7 +12949,7 @@
       <c r="J149" t="s">
         <v>1523</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12993,7 +12967,7 @@
       <c r="R149" t="s">
         <v>1707</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13028,7 +13002,7 @@
       <c r="J150" t="s">
         <v>1523</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13046,7 +13020,7 @@
       <c r="R150" t="s">
         <v>1707</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13081,7 +13055,7 @@
       <c r="J151" t="s">
         <v>1523</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13099,7 +13073,7 @@
       <c r="R151" t="s">
         <v>1723</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13134,7 +13108,7 @@
       <c r="J152" t="s">
         <v>1523</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13152,7 +13126,7 @@
       <c r="R152" t="s">
         <v>1724</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13187,7 +13161,7 @@
       <c r="J153" t="s">
         <v>1523</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13196,7 +13170,7 @@
       <c r="M153" t="s">
         <v>1599</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13237,7 +13211,7 @@
       <c r="J154" t="s">
         <v>1523</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13278,7 +13252,7 @@
       <c r="J155" t="s">
         <v>1523</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13319,7 +13293,7 @@
       <c r="J156" t="s">
         <v>1523</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13360,7 +13334,7 @@
       <c r="J157" t="s">
         <v>1523</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13401,7 +13375,7 @@
       <c r="J158" t="s">
         <v>1523</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13442,7 +13416,7 @@
       <c r="J159" t="s">
         <v>1523</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13483,7 +13457,7 @@
       <c r="J160" t="s">
         <v>1523</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13524,7 +13498,7 @@
       <c r="J161" t="s">
         <v>1523</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13565,7 +13539,7 @@
       <c r="J162" t="s">
         <v>1523</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13583,7 +13557,7 @@
       <c r="R162" t="s">
         <v>1710</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13618,7 +13592,7 @@
       <c r="J163" t="s">
         <v>1523</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13636,7 +13610,7 @@
       <c r="R163" t="s">
         <v>1707</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13671,7 +13645,7 @@
       <c r="J164" t="s">
         <v>1523</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13715,7 +13689,7 @@
       <c r="J165" t="s">
         <v>1523</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13756,7 +13730,7 @@
       <c r="J166" t="s">
         <v>1523</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13774,7 +13748,7 @@
       <c r="R166" t="s">
         <v>1725</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13809,7 +13783,7 @@
       <c r="J167" t="s">
         <v>1523</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13853,7 +13827,7 @@
       <c r="J168" t="s">
         <v>1523</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13897,7 +13871,7 @@
       <c r="J169" t="s">
         <v>1523</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13938,7 +13912,7 @@
       <c r="J170" t="s">
         <v>1523</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13979,7 +13953,7 @@
       <c r="J171" t="s">
         <v>1523</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14020,7 +13994,7 @@
       <c r="J172" t="s">
         <v>1523</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14061,7 +14035,7 @@
       <c r="J173" t="s">
         <v>1523</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14102,7 +14076,7 @@
       <c r="J174" t="s">
         <v>1523</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14143,7 +14117,7 @@
       <c r="J175" t="s">
         <v>1523</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14184,7 +14158,7 @@
       <c r="J176" t="s">
         <v>1523</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14225,7 +14199,7 @@
       <c r="J177" t="s">
         <v>1523</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14266,7 +14240,7 @@
       <c r="J178" t="s">
         <v>1523</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14284,7 +14258,7 @@
       <c r="R178" t="s">
         <v>1723</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14322,7 +14296,7 @@
       <c r="J179" t="s">
         <v>1523</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14331,7 +14305,7 @@
       <c r="M179" t="s">
         <v>1596</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14372,7 +14346,7 @@
       <c r="J180" t="s">
         <v>1523</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14413,7 +14387,7 @@
       <c r="J181" t="s">
         <v>1523</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14431,7 +14405,7 @@
       <c r="R181" t="s">
         <v>1707</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14466,7 +14440,7 @@
       <c r="J182" t="s">
         <v>1523</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14507,7 +14481,7 @@
       <c r="J183" t="s">
         <v>1523</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14548,7 +14522,7 @@
       <c r="J184" t="s">
         <v>1523</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14589,7 +14563,7 @@
       <c r="J185" t="s">
         <v>1523</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14630,7 +14604,7 @@
       <c r="J186" t="s">
         <v>1523</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14671,7 +14645,7 @@
       <c r="J187" t="s">
         <v>1523</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14712,7 +14686,7 @@
       <c r="J188" t="s">
         <v>1523</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14753,7 +14727,7 @@
       <c r="J189" t="s">
         <v>1523</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14794,7 +14768,7 @@
       <c r="J190" t="s">
         <v>1523</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14835,7 +14809,7 @@
       <c r="J191" t="s">
         <v>1523</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14876,7 +14850,7 @@
       <c r="J192" t="s">
         <v>1523</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14917,7 +14891,7 @@
       <c r="J193" t="s">
         <v>1523</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14958,7 +14932,7 @@
       <c r="J194" t="s">
         <v>1523</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14999,7 +14973,7 @@
       <c r="J195" t="s">
         <v>1523</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15017,7 +14991,7 @@
       <c r="R195" t="s">
         <v>1716</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15058,7 +15032,7 @@
       <c r="J196" t="s">
         <v>1523</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15076,7 +15050,7 @@
       <c r="R196" t="s">
         <v>1722</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15114,7 +15088,7 @@
       <c r="J197" t="s">
         <v>1523</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15155,7 +15129,7 @@
       <c r="J198" t="s">
         <v>1525</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15196,7 +15170,7 @@
       <c r="J199" t="s">
         <v>1524</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15237,7 +15211,7 @@
       <c r="J200" t="s">
         <v>1523</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15278,7 +15252,7 @@
       <c r="J201" t="s">
         <v>1523</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15319,7 +15293,7 @@
       <c r="J202" t="s">
         <v>1523</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15337,7 +15311,7 @@
       <c r="R202" t="s">
         <v>1707</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15372,7 +15346,7 @@
       <c r="J203" t="s">
         <v>1523</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15390,7 +15364,7 @@
       <c r="R203" t="s">
         <v>1715</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15425,7 +15399,7 @@
       <c r="J204" t="s">
         <v>1523</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15440,7 +15414,7 @@
       <c r="R204" t="s">
         <v>1726</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15478,7 +15452,7 @@
       <c r="J205" t="s">
         <v>1523</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15496,7 +15470,7 @@
       <c r="R205" t="s">
         <v>1727</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15534,7 +15508,7 @@
       <c r="J206" t="s">
         <v>1523</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15552,7 +15526,7 @@
       <c r="R206" t="s">
         <v>1695</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15587,7 +15561,7 @@
       <c r="J207" t="s">
         <v>1523</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15628,7 +15602,7 @@
       <c r="J208" t="s">
         <v>1523</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15669,7 +15643,7 @@
       <c r="J209" t="s">
         <v>1523</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15710,7 +15684,7 @@
       <c r="J210" t="s">
         <v>1523</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15751,7 +15725,7 @@
       <c r="J211" t="s">
         <v>1523</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15792,7 +15766,7 @@
       <c r="J212" t="s">
         <v>1523</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15833,7 +15807,7 @@
       <c r="J213" t="s">
         <v>1523</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15874,7 +15848,7 @@
       <c r="J214" t="s">
         <v>1523</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15892,7 +15866,7 @@
       <c r="R214" t="s">
         <v>1728</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15927,7 +15901,7 @@
       <c r="J215" t="s">
         <v>1523</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15968,7 +15942,7 @@
       <c r="J216" t="s">
         <v>1523</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16009,7 +15983,7 @@
       <c r="J217" t="s">
         <v>1523</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16050,7 +16024,7 @@
       <c r="J218" t="s">
         <v>1523</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16091,7 +16065,7 @@
       <c r="J219" t="s">
         <v>1523</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16132,7 +16106,7 @@
       <c r="J220" t="s">
         <v>1523</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16173,7 +16147,7 @@
       <c r="J221" t="s">
         <v>1523</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16214,7 +16188,7 @@
       <c r="J222" t="s">
         <v>1523</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16255,7 +16229,7 @@
       <c r="J223" t="s">
         <v>1523</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16296,7 +16270,7 @@
       <c r="J224" t="s">
         <v>1523</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16337,7 +16311,7 @@
       <c r="J225" t="s">
         <v>1523</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16378,7 +16352,7 @@
       <c r="J226" t="s">
         <v>1523</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16419,7 +16393,7 @@
       <c r="J227" t="s">
         <v>1523</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16460,7 +16434,7 @@
       <c r="J228" t="s">
         <v>1523</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16501,7 +16475,7 @@
       <c r="J229" t="s">
         <v>1523</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16542,7 +16516,7 @@
       <c r="J230" t="s">
         <v>1523</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16583,7 +16557,7 @@
       <c r="J231" t="s">
         <v>1523</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16624,7 +16598,7 @@
       <c r="J232" t="s">
         <v>1523</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16665,7 +16639,7 @@
       <c r="J233" t="s">
         <v>1523</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16706,7 +16680,7 @@
       <c r="J234" t="s">
         <v>1523</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16747,7 +16721,7 @@
       <c r="J235" t="s">
         <v>1523</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16788,7 +16762,7 @@
       <c r="J236" t="s">
         <v>1523</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16829,7 +16803,7 @@
       <c r="J237" t="s">
         <v>1523</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16870,7 +16844,7 @@
       <c r="J238" t="s">
         <v>1523</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16911,7 +16885,7 @@
       <c r="J239" t="s">
         <v>1523</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16929,7 +16903,7 @@
       <c r="R239" t="s">
         <v>1722</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -16967,7 +16941,7 @@
       <c r="J240" t="s">
         <v>1523</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17008,7 +16982,7 @@
       <c r="J241" t="s">
         <v>1523</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17049,7 +17023,7 @@
       <c r="J242" t="s">
         <v>1523</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17067,7 +17041,7 @@
       <c r="R242" t="s">
         <v>1715</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17102,7 +17076,7 @@
       <c r="J243" t="s">
         <v>1523</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17143,7 +17117,7 @@
       <c r="J244" t="s">
         <v>1523</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17184,7 +17158,7 @@
       <c r="J245" t="s">
         <v>1523</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17225,7 +17199,7 @@
       <c r="J246" t="s">
         <v>1523</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17243,7 +17217,7 @@
       <c r="R246" t="s">
         <v>1695</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17281,7 +17255,7 @@
       <c r="J247" t="s">
         <v>1523</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17322,7 +17296,7 @@
       <c r="J248" t="s">
         <v>1523</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17363,7 +17337,7 @@
       <c r="J249" t="s">
         <v>1523</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17404,7 +17378,7 @@
       <c r="J250" t="s">
         <v>1523</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17445,7 +17419,7 @@
       <c r="J251" t="s">
         <v>1523</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17486,7 +17460,7 @@
       <c r="J252" t="s">
         <v>1523</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17527,7 +17501,7 @@
       <c r="J253" t="s">
         <v>1523</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17545,7 +17519,7 @@
       <c r="R253" t="s">
         <v>1725</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17583,7 +17557,7 @@
       <c r="J254" t="s">
         <v>1523</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17624,7 +17598,7 @@
       <c r="J255" t="s">
         <v>1523</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17665,7 +17639,7 @@
       <c r="J256" t="s">
         <v>1523</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17674,7 +17648,7 @@
       <c r="M256" t="s">
         <v>1595</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17712,7 +17686,7 @@
       <c r="J257" t="s">
         <v>1523</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17721,7 +17695,7 @@
       <c r="M257" t="s">
         <v>1596</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17765,7 +17739,7 @@
       <c r="J258" t="s">
         <v>1523</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17783,7 +17757,7 @@
       <c r="R258" t="s">
         <v>1707</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17821,7 +17795,7 @@
       <c r="J259" t="s">
         <v>1523</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17839,7 +17813,7 @@
       <c r="R259" t="s">
         <v>1723</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17877,7 +17851,7 @@
       <c r="J260" t="s">
         <v>1523</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17886,7 +17860,7 @@
       <c r="M260" t="s">
         <v>1590</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17930,7 +17904,7 @@
       <c r="J261" t="s">
         <v>1523</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17948,7 +17922,7 @@
       <c r="R261" t="s">
         <v>1729</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17986,7 +17960,7 @@
       <c r="J262" t="s">
         <v>1523</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18004,7 +17978,7 @@
       <c r="R262" t="s">
         <v>1723</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18042,7 +18016,7 @@
       <c r="J263" t="s">
         <v>1523</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18051,7 +18025,7 @@
       <c r="M263" t="s">
         <v>1590</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18095,7 +18069,7 @@
       <c r="J264" t="s">
         <v>1523</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18136,7 +18110,7 @@
       <c r="J265" t="s">
         <v>1523</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18177,7 +18151,7 @@
       <c r="J266" t="s">
         <v>1523</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18218,7 +18192,7 @@
       <c r="J267" t="s">
         <v>1523</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18262,7 +18236,7 @@
       <c r="J268" t="s">
         <v>1523</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18303,7 +18277,7 @@
       <c r="J269" t="s">
         <v>1523</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18344,7 +18318,7 @@
       <c r="J270" t="s">
         <v>1523</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18385,7 +18359,7 @@
       <c r="J271" t="s">
         <v>1523</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18426,7 +18400,7 @@
       <c r="J272" t="s">
         <v>1523</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18444,7 +18418,7 @@
       <c r="R272" t="s">
         <v>1730</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18482,7 +18456,7 @@
       <c r="J273" t="s">
         <v>1523</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18526,7 +18500,7 @@
       <c r="J274" t="s">
         <v>1523</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18567,7 +18541,7 @@
       <c r="J275" t="s">
         <v>1523</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18608,7 +18582,7 @@
       <c r="J276" t="s">
         <v>1523</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18649,7 +18623,7 @@
       <c r="J277" t="s">
         <v>1523</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18690,7 +18664,7 @@
       <c r="J278" t="s">
         <v>1523</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18731,7 +18705,7 @@
       <c r="J279" t="s">
         <v>1523</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18772,7 +18746,7 @@
       <c r="J280" t="s">
         <v>1523</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18813,7 +18787,7 @@
       <c r="J281" t="s">
         <v>1523</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18854,7 +18828,7 @@
       <c r="J282" t="s">
         <v>1523</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18895,7 +18869,7 @@
       <c r="J283" t="s">
         <v>1523</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18936,7 +18910,7 @@
       <c r="J284" t="s">
         <v>1523</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18977,7 +18951,7 @@
       <c r="J285" t="s">
         <v>1523</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19018,7 +18992,7 @@
       <c r="J286" t="s">
         <v>1523</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19059,7 +19033,7 @@
       <c r="J287" t="s">
         <v>1523</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19100,7 +19074,7 @@
       <c r="J288" t="s">
         <v>1523</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19141,7 +19115,7 @@
       <c r="J289" t="s">
         <v>1523</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19182,7 +19156,7 @@
       <c r="J290" t="s">
         <v>1523</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19223,7 +19197,7 @@
       <c r="J291" t="s">
         <v>1523</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19264,7 +19238,7 @@
       <c r="J292" t="s">
         <v>1523</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19305,7 +19279,7 @@
       <c r="J293" t="s">
         <v>1523</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19346,7 +19320,7 @@
       <c r="J294" t="s">
         <v>1523</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19387,7 +19361,7 @@
       <c r="J295" t="s">
         <v>1523</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19405,7 +19379,7 @@
       <c r="R295" t="s">
         <v>1731</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19446,7 +19420,7 @@
       <c r="J296" t="s">
         <v>1523</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19464,7 +19438,7 @@
       <c r="R296" t="s">
         <v>1707</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19502,7 +19476,7 @@
       <c r="J297" t="s">
         <v>1523</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19543,7 +19517,7 @@
       <c r="J298" t="s">
         <v>1523</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19584,7 +19558,7 @@
       <c r="J299" t="s">
         <v>1524</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19625,7 +19599,7 @@
       <c r="J300" t="s">
         <v>1523</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19666,7 +19640,7 @@
       <c r="J301" t="s">
         <v>1523</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20504,7 +20478,7 @@
       <c r="R321" t="s">
         <v>1693</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -20727,7 +20701,7 @@
       <c r="R326" t="s">
         <v>1732</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21562,7 +21536,7 @@
       <c r="R346" t="s">
         <v>1733</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (21/09/2026 14:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5342,8 +5342,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5359,7 +5367,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5367,12 +5375,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5672,73 +5698,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5773,7 +5799,7 @@
       <c r="J2" t="s">
         <v>1523</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5817,7 +5843,7 @@
       <c r="J3" t="s">
         <v>1523</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5861,7 +5887,7 @@
       <c r="J4" t="s">
         <v>1523</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5879,7 +5905,7 @@
       <c r="R4" t="s">
         <v>1690</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5917,7 +5943,7 @@
       <c r="J5" t="s">
         <v>1524</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5967,7 +5993,7 @@
       <c r="J6" t="s">
         <v>1523</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6014,7 +6040,7 @@
       <c r="J7" t="s">
         <v>1523</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6061,7 +6087,7 @@
       <c r="J8" t="s">
         <v>1523</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6108,7 +6134,7 @@
       <c r="J9" t="s">
         <v>1523</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6155,7 +6181,7 @@
       <c r="J10" t="s">
         <v>1523</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6202,7 +6228,7 @@
       <c r="J11" t="s">
         <v>1523</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6249,7 +6275,7 @@
       <c r="J12" t="s">
         <v>1523</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6293,7 +6319,7 @@
       <c r="J13" t="s">
         <v>1523</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6311,7 +6337,7 @@
       <c r="R13" t="s">
         <v>1691</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6349,7 +6375,7 @@
       <c r="J14" t="s">
         <v>1523</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6367,7 +6393,7 @@
       <c r="R14" t="s">
         <v>1692</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6405,7 +6431,7 @@
       <c r="J15" t="s">
         <v>1523</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6423,7 +6449,7 @@
       <c r="R15" t="s">
         <v>1692</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6464,7 +6490,7 @@
       <c r="J16" t="s">
         <v>1523</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6508,7 +6534,7 @@
       <c r="J17" t="s">
         <v>1523</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6552,7 +6578,7 @@
       <c r="J18" t="s">
         <v>1523</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6570,7 +6596,7 @@
       <c r="R18" t="s">
         <v>1693</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6611,7 +6637,7 @@
       <c r="J19" t="s">
         <v>1523</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6655,7 +6681,7 @@
       <c r="J20" t="s">
         <v>1523</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6699,7 +6725,7 @@
       <c r="J21" t="s">
         <v>1523</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6717,7 +6743,7 @@
       <c r="R21" t="s">
         <v>1692</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6758,7 +6784,7 @@
       <c r="J22" t="s">
         <v>1523</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6776,7 +6802,7 @@
       <c r="R22" t="s">
         <v>1694</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6817,7 +6843,7 @@
       <c r="J23" t="s">
         <v>1523</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6835,7 +6861,7 @@
       <c r="R23" t="s">
         <v>1695</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6876,7 +6902,7 @@
       <c r="J24" t="s">
         <v>1523</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6920,7 +6946,7 @@
       <c r="J25" t="s">
         <v>1523</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6961,7 +6987,7 @@
       <c r="J26" t="s">
         <v>1525</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6979,7 +7005,7 @@
       <c r="R26" t="s">
         <v>1696</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -7014,7 +7040,7 @@
       <c r="J27" t="s">
         <v>1523</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7032,7 +7058,7 @@
       <c r="R27" t="s">
         <v>1697</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7073,7 +7099,7 @@
       <c r="J28" t="s">
         <v>1523</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7117,7 +7143,7 @@
       <c r="J29" t="s">
         <v>1523</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7161,7 +7187,7 @@
       <c r="J30" t="s">
         <v>1523</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7205,7 +7231,7 @@
       <c r="J31" t="s">
         <v>1523</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7223,7 +7249,7 @@
       <c r="R31" t="s">
         <v>1698</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7264,7 +7290,7 @@
       <c r="J32" t="s">
         <v>1523</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7308,7 +7334,7 @@
       <c r="J33" t="s">
         <v>1523</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7326,7 +7352,7 @@
       <c r="R33" t="s">
         <v>1699</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7367,7 +7393,7 @@
       <c r="J34" t="s">
         <v>1523</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7411,7 +7437,7 @@
       <c r="J35" t="s">
         <v>1523</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7429,7 +7455,7 @@
       <c r="R35" t="s">
         <v>1700</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7470,7 +7496,7 @@
       <c r="J36" t="s">
         <v>1523</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7488,7 +7514,7 @@
       <c r="R36" t="s">
         <v>1700</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7529,7 +7555,7 @@
       <c r="J37" t="s">
         <v>1523</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7547,7 +7573,7 @@
       <c r="R37" t="s">
         <v>1700</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7588,7 +7614,7 @@
       <c r="J38" t="s">
         <v>1523</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7606,7 +7632,7 @@
       <c r="R38" t="s">
         <v>1700</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7647,7 +7673,7 @@
       <c r="J39" t="s">
         <v>1523</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7665,7 +7691,7 @@
       <c r="R39" t="s">
         <v>1700</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7706,7 +7732,7 @@
       <c r="J40" t="s">
         <v>1523</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7724,7 +7750,7 @@
       <c r="R40" t="s">
         <v>1701</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7765,7 +7791,7 @@
       <c r="J41" t="s">
         <v>1523</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7783,7 +7809,7 @@
       <c r="R41" t="s">
         <v>1692</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -7824,7 +7850,7 @@
       <c r="J42" t="s">
         <v>1523</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7842,7 +7868,7 @@
       <c r="R42" t="s">
         <v>1700</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7883,7 +7909,7 @@
       <c r="J43" t="s">
         <v>1523</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7927,7 +7953,7 @@
       <c r="J44" t="s">
         <v>1523</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7945,7 +7971,7 @@
       <c r="R44" t="s">
         <v>1702</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7986,7 +8012,7 @@
       <c r="J45" t="s">
         <v>1523</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8004,7 +8030,7 @@
       <c r="R45" t="s">
         <v>1703</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8042,7 +8068,7 @@
       <c r="J46" t="s">
         <v>1523</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8086,7 +8112,7 @@
       <c r="J47" t="s">
         <v>1523</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8104,7 +8130,7 @@
       <c r="R47" t="s">
         <v>1704</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8145,7 +8171,7 @@
       <c r="J48" t="s">
         <v>1523</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8189,7 +8215,7 @@
       <c r="J49" t="s">
         <v>1523</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8233,7 +8259,7 @@
       <c r="J50" t="s">
         <v>1523</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8277,7 +8303,7 @@
       <c r="J51" t="s">
         <v>1523</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8324,7 +8350,7 @@
       <c r="J52" t="s">
         <v>1523</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8368,7 +8394,7 @@
       <c r="J53" t="s">
         <v>1523</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8412,7 +8438,7 @@
       <c r="J54" t="s">
         <v>1523</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8456,7 +8482,7 @@
       <c r="J55" t="s">
         <v>1523</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8506,7 +8532,7 @@
       <c r="J56" t="s">
         <v>1523</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8559,7 +8585,7 @@
       <c r="J57" t="s">
         <v>1523</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8609,7 +8635,7 @@
       <c r="J58" t="s">
         <v>1523</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8659,7 +8685,7 @@
       <c r="J59" t="s">
         <v>1523</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8677,7 +8703,7 @@
       <c r="R59" t="s">
         <v>1705</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8718,7 +8744,7 @@
       <c r="J60" t="s">
         <v>1523</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8762,7 +8788,7 @@
       <c r="J61" t="s">
         <v>1523</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8806,7 +8832,7 @@
       <c r="J62" t="s">
         <v>1523</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8850,7 +8876,7 @@
       <c r="J63" t="s">
         <v>1523</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8894,7 +8920,7 @@
       <c r="J64" t="s">
         <v>1523</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8938,7 +8964,7 @@
       <c r="J65" t="s">
         <v>1523</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8985,7 +9011,7 @@
       <c r="J66" t="s">
         <v>1523</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9003,7 +9029,7 @@
       <c r="R66" t="s">
         <v>1706</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9041,7 +9067,7 @@
       <c r="J67" t="s">
         <v>1523</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9085,7 +9111,7 @@
       <c r="J68" t="s">
         <v>1523</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9100,7 +9126,7 @@
       <c r="O68" t="s">
         <v>1608</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9144,7 +9170,7 @@
       <c r="J69" t="s">
         <v>1525</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9188,7 +9214,7 @@
       <c r="J70" t="s">
         <v>1523</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9232,7 +9258,7 @@
       <c r="J71" t="s">
         <v>1523</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9276,7 +9302,7 @@
       <c r="J72" t="s">
         <v>1523</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9320,7 +9346,7 @@
       <c r="J73" t="s">
         <v>1523</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9364,7 +9390,7 @@
       <c r="J74" t="s">
         <v>1523</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9408,7 +9434,7 @@
       <c r="J75" t="s">
         <v>1523</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9452,7 +9478,7 @@
       <c r="J76" t="s">
         <v>1523</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9470,7 +9496,7 @@
       <c r="R76" t="s">
         <v>1707</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9508,7 +9534,7 @@
       <c r="J77" t="s">
         <v>1523</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9526,7 +9552,7 @@
       <c r="R77" t="s">
         <v>1707</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9564,7 +9590,7 @@
       <c r="J78" t="s">
         <v>1523</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9582,7 +9608,7 @@
       <c r="R78" t="s">
         <v>1707</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9620,7 +9646,7 @@
       <c r="J79" t="s">
         <v>1523</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9638,7 +9664,7 @@
       <c r="R79" t="s">
         <v>1707</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9676,7 +9702,7 @@
       <c r="J80" t="s">
         <v>1523</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9720,7 +9746,7 @@
       <c r="J81" t="s">
         <v>1523</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9764,7 +9790,7 @@
       <c r="J82" t="s">
         <v>1523</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9808,7 +9834,7 @@
       <c r="J83" t="s">
         <v>1523</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9852,7 +9878,7 @@
       <c r="J84" t="s">
         <v>1523</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9896,7 +9922,7 @@
       <c r="J85" t="s">
         <v>1523</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9914,7 +9940,7 @@
       <c r="R85" t="s">
         <v>1708</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9952,7 +9978,7 @@
       <c r="J86" t="s">
         <v>1523</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9996,7 +10022,7 @@
       <c r="J87" t="s">
         <v>1523</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10014,7 +10040,7 @@
       <c r="R87" t="s">
         <v>1709</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10052,7 +10078,7 @@
       <c r="J88" t="s">
         <v>1523</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10096,7 +10122,7 @@
       <c r="J89" t="s">
         <v>1523</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10114,7 +10140,7 @@
       <c r="R89" t="s">
         <v>1710</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10149,7 +10175,7 @@
       <c r="J90" t="s">
         <v>1523</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10167,7 +10193,7 @@
       <c r="R90" t="s">
         <v>1711</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10202,7 +10228,7 @@
       <c r="J91" t="s">
         <v>1523</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10220,7 +10246,7 @@
       <c r="R91" t="s">
         <v>1695</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10258,7 +10284,7 @@
       <c r="J92" t="s">
         <v>1523</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10279,7 +10305,7 @@
       <c r="R92" t="s">
         <v>1695</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10320,7 +10346,7 @@
       <c r="J93" t="s">
         <v>1523</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10361,7 +10387,7 @@
       <c r="J94" t="s">
         <v>1523</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10405,7 +10431,7 @@
       <c r="J95" t="s">
         <v>1523</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10449,7 +10475,7 @@
       <c r="J96" t="s">
         <v>1523</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10467,7 +10493,7 @@
       <c r="R96" t="s">
         <v>1712</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10505,7 +10531,7 @@
       <c r="J97" t="s">
         <v>1523</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10520,7 +10546,7 @@
       <c r="R97" t="s">
         <v>1712</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10561,7 +10587,7 @@
       <c r="J98" t="s">
         <v>1523</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10579,7 +10605,7 @@
       <c r="R98" t="s">
         <v>1713</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10617,7 +10643,7 @@
       <c r="J99" t="s">
         <v>1523</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10635,7 +10661,7 @@
       <c r="R99" t="s">
         <v>1714</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10673,7 +10699,7 @@
       <c r="J100" t="s">
         <v>1523</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10714,7 +10740,7 @@
       <c r="J101" t="s">
         <v>1523</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10755,7 +10781,7 @@
       <c r="J102" t="s">
         <v>1523</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10796,7 +10822,7 @@
       <c r="J103" t="s">
         <v>1523</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10837,7 +10863,7 @@
       <c r="J104" t="s">
         <v>1523</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10878,7 +10904,7 @@
       <c r="J105" t="s">
         <v>1523</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10919,7 +10945,7 @@
       <c r="J106" t="s">
         <v>1523</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10960,7 +10986,7 @@
       <c r="J107" t="s">
         <v>1523</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11001,7 +11027,7 @@
       <c r="J108" t="s">
         <v>1523</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11042,7 +11068,7 @@
       <c r="J109" t="s">
         <v>1523</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11095,7 +11121,7 @@
       <c r="J110" t="s">
         <v>1523</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11151,7 +11177,7 @@
       <c r="J111" t="s">
         <v>1523</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11169,7 +11195,7 @@
       <c r="R111" t="s">
         <v>1716</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11207,7 +11233,7 @@
       <c r="J112" t="s">
         <v>1523</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11266,7 +11292,7 @@
       <c r="J113" t="s">
         <v>1523</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11310,7 +11336,7 @@
       <c r="J114" t="s">
         <v>1523</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11354,7 +11380,7 @@
       <c r="J115" t="s">
         <v>1523</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11372,7 +11398,7 @@
       <c r="R115" t="s">
         <v>1718</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11410,7 +11436,7 @@
       <c r="J116" t="s">
         <v>1523</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11469,7 +11495,7 @@
       <c r="J117" t="s">
         <v>1523</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11513,7 +11539,7 @@
       <c r="J118" t="s">
         <v>1523</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11560,7 +11586,7 @@
       <c r="J119" t="s">
         <v>1523</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11601,7 +11627,7 @@
       <c r="J120" t="s">
         <v>1523</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11645,7 +11671,7 @@
       <c r="J121" t="s">
         <v>1523</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11692,7 +11718,7 @@
       <c r="J122" t="s">
         <v>1523</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11742,7 +11768,7 @@
       <c r="J123" t="s">
         <v>1523</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11786,7 +11812,7 @@
       <c r="J124" t="s">
         <v>1523</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11830,7 +11856,7 @@
       <c r="J125" t="s">
         <v>1523</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11848,7 +11874,7 @@
       <c r="R125" t="s">
         <v>1720</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11883,7 +11909,7 @@
       <c r="J126" t="s">
         <v>1523</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11901,7 +11927,7 @@
       <c r="R126" t="s">
         <v>1721</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11936,7 +11962,7 @@
       <c r="J127" t="s">
         <v>1523</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11992,7 +12018,7 @@
       <c r="J128" t="s">
         <v>1523</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12033,7 +12059,7 @@
       <c r="J129" t="s">
         <v>1523</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12074,7 +12100,7 @@
       <c r="J130" t="s">
         <v>1523</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12115,7 +12141,7 @@
       <c r="J131" t="s">
         <v>1523</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12159,7 +12185,7 @@
       <c r="J132" t="s">
         <v>1523</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12200,7 +12226,7 @@
       <c r="J133" t="s">
         <v>1523</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12218,7 +12244,7 @@
       <c r="R133" t="s">
         <v>1707</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12253,7 +12279,7 @@
       <c r="J134" t="s">
         <v>1523</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12271,7 +12297,7 @@
       <c r="R134" t="s">
         <v>1707</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12306,7 +12332,7 @@
       <c r="J135" t="s">
         <v>1523</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12347,7 +12373,7 @@
       <c r="J136" t="s">
         <v>1523</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12388,7 +12414,7 @@
       <c r="J137" t="s">
         <v>1523</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12429,7 +12455,7 @@
       <c r="J138" t="s">
         <v>1523</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12470,7 +12496,7 @@
       <c r="J139" t="s">
         <v>1523</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12517,7 +12543,7 @@
       <c r="J140" t="s">
         <v>1523</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12558,7 +12584,7 @@
       <c r="J141" t="s">
         <v>1523</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12599,7 +12625,7 @@
       <c r="J142" t="s">
         <v>1523</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12643,7 +12669,7 @@
       <c r="J143" t="s">
         <v>1523</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12661,7 +12687,7 @@
       <c r="R143" t="s">
         <v>1707</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12696,7 +12722,7 @@
       <c r="J144" t="s">
         <v>1523</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12714,7 +12740,7 @@
       <c r="R144" t="s">
         <v>1707</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12749,7 +12775,7 @@
       <c r="J145" t="s">
         <v>1523</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12767,7 +12793,7 @@
       <c r="R145" t="s">
         <v>1707</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12802,7 +12828,7 @@
       <c r="J146" t="s">
         <v>1523</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12820,7 +12846,7 @@
       <c r="R146" t="s">
         <v>1715</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12855,7 +12881,7 @@
       <c r="J147" t="s">
         <v>1523</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12873,7 +12899,7 @@
       <c r="R147" t="s">
         <v>1722</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12908,7 +12934,7 @@
       <c r="J148" t="s">
         <v>1523</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12949,7 +12975,7 @@
       <c r="J149" t="s">
         <v>1523</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12967,7 +12993,7 @@
       <c r="R149" t="s">
         <v>1707</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13002,7 +13028,7 @@
       <c r="J150" t="s">
         <v>1523</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13020,7 +13046,7 @@
       <c r="R150" t="s">
         <v>1707</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13055,7 +13081,7 @@
       <c r="J151" t="s">
         <v>1523</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13073,7 +13099,7 @@
       <c r="R151" t="s">
         <v>1723</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13108,7 +13134,7 @@
       <c r="J152" t="s">
         <v>1523</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13126,7 +13152,7 @@
       <c r="R152" t="s">
         <v>1724</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13161,7 +13187,7 @@
       <c r="J153" t="s">
         <v>1523</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13170,7 +13196,7 @@
       <c r="M153" t="s">
         <v>1599</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13211,7 +13237,7 @@
       <c r="J154" t="s">
         <v>1523</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13252,7 +13278,7 @@
       <c r="J155" t="s">
         <v>1523</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13293,7 +13319,7 @@
       <c r="J156" t="s">
         <v>1523</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13334,7 +13360,7 @@
       <c r="J157" t="s">
         <v>1523</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13375,7 +13401,7 @@
       <c r="J158" t="s">
         <v>1523</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13416,7 +13442,7 @@
       <c r="J159" t="s">
         <v>1523</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13457,7 +13483,7 @@
       <c r="J160" t="s">
         <v>1523</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13498,7 +13524,7 @@
       <c r="J161" t="s">
         <v>1523</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13539,7 +13565,7 @@
       <c r="J162" t="s">
         <v>1523</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13557,7 +13583,7 @@
       <c r="R162" t="s">
         <v>1710</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13592,7 +13618,7 @@
       <c r="J163" t="s">
         <v>1523</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13610,7 +13636,7 @@
       <c r="R163" t="s">
         <v>1707</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13645,7 +13671,7 @@
       <c r="J164" t="s">
         <v>1523</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13689,7 +13715,7 @@
       <c r="J165" t="s">
         <v>1523</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13730,7 +13756,7 @@
       <c r="J166" t="s">
         <v>1523</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13748,7 +13774,7 @@
       <c r="R166" t="s">
         <v>1725</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13783,7 +13809,7 @@
       <c r="J167" t="s">
         <v>1523</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13827,7 +13853,7 @@
       <c r="J168" t="s">
         <v>1523</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13871,7 +13897,7 @@
       <c r="J169" t="s">
         <v>1523</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13912,7 +13938,7 @@
       <c r="J170" t="s">
         <v>1523</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13953,7 +13979,7 @@
       <c r="J171" t="s">
         <v>1523</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13994,7 +14020,7 @@
       <c r="J172" t="s">
         <v>1523</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14035,7 +14061,7 @@
       <c r="J173" t="s">
         <v>1523</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14076,7 +14102,7 @@
       <c r="J174" t="s">
         <v>1523</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14117,7 +14143,7 @@
       <c r="J175" t="s">
         <v>1523</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14158,7 +14184,7 @@
       <c r="J176" t="s">
         <v>1523</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14199,7 +14225,7 @@
       <c r="J177" t="s">
         <v>1523</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14240,7 +14266,7 @@
       <c r="J178" t="s">
         <v>1523</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14258,7 +14284,7 @@
       <c r="R178" t="s">
         <v>1723</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14296,7 +14322,7 @@
       <c r="J179" t="s">
         <v>1523</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14305,7 +14331,7 @@
       <c r="M179" t="s">
         <v>1596</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14346,7 +14372,7 @@
       <c r="J180" t="s">
         <v>1523</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14387,7 +14413,7 @@
       <c r="J181" t="s">
         <v>1523</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14405,7 +14431,7 @@
       <c r="R181" t="s">
         <v>1707</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14440,7 +14466,7 @@
       <c r="J182" t="s">
         <v>1523</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14481,7 +14507,7 @@
       <c r="J183" t="s">
         <v>1523</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14522,7 +14548,7 @@
       <c r="J184" t="s">
         <v>1523</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14563,7 +14589,7 @@
       <c r="J185" t="s">
         <v>1523</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14604,7 +14630,7 @@
       <c r="J186" t="s">
         <v>1523</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14645,7 +14671,7 @@
       <c r="J187" t="s">
         <v>1523</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14686,7 +14712,7 @@
       <c r="J188" t="s">
         <v>1523</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14727,7 +14753,7 @@
       <c r="J189" t="s">
         <v>1523</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14768,7 +14794,7 @@
       <c r="J190" t="s">
         <v>1523</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14809,7 +14835,7 @@
       <c r="J191" t="s">
         <v>1523</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14850,7 +14876,7 @@
       <c r="J192" t="s">
         <v>1523</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14891,7 +14917,7 @@
       <c r="J193" t="s">
         <v>1523</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14932,7 +14958,7 @@
       <c r="J194" t="s">
         <v>1523</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14973,7 +14999,7 @@
       <c r="J195" t="s">
         <v>1523</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14991,7 +15017,7 @@
       <c r="R195" t="s">
         <v>1716</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15032,7 +15058,7 @@
       <c r="J196" t="s">
         <v>1523</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15050,7 +15076,7 @@
       <c r="R196" t="s">
         <v>1722</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15088,7 +15114,7 @@
       <c r="J197" t="s">
         <v>1523</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15129,7 +15155,7 @@
       <c r="J198" t="s">
         <v>1525</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15170,7 +15196,7 @@
       <c r="J199" t="s">
         <v>1524</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15211,7 +15237,7 @@
       <c r="J200" t="s">
         <v>1523</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15252,7 +15278,7 @@
       <c r="J201" t="s">
         <v>1523</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15293,7 +15319,7 @@
       <c r="J202" t="s">
         <v>1523</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15311,7 +15337,7 @@
       <c r="R202" t="s">
         <v>1707</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15346,7 +15372,7 @@
       <c r="J203" t="s">
         <v>1523</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15364,7 +15390,7 @@
       <c r="R203" t="s">
         <v>1715</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15399,7 +15425,7 @@
       <c r="J204" t="s">
         <v>1523</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15414,7 +15440,7 @@
       <c r="R204" t="s">
         <v>1726</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15452,7 +15478,7 @@
       <c r="J205" t="s">
         <v>1523</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15470,7 +15496,7 @@
       <c r="R205" t="s">
         <v>1727</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15508,7 +15534,7 @@
       <c r="J206" t="s">
         <v>1523</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15526,7 +15552,7 @@
       <c r="R206" t="s">
         <v>1695</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15561,7 +15587,7 @@
       <c r="J207" t="s">
         <v>1523</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15602,7 +15628,7 @@
       <c r="J208" t="s">
         <v>1523</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15643,7 +15669,7 @@
       <c r="J209" t="s">
         <v>1523</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15684,7 +15710,7 @@
       <c r="J210" t="s">
         <v>1523</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15725,7 +15751,7 @@
       <c r="J211" t="s">
         <v>1523</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15766,7 +15792,7 @@
       <c r="J212" t="s">
         <v>1523</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15807,7 +15833,7 @@
       <c r="J213" t="s">
         <v>1523</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15848,7 +15874,7 @@
       <c r="J214" t="s">
         <v>1523</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15866,7 +15892,7 @@
       <c r="R214" t="s">
         <v>1728</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15901,7 +15927,7 @@
       <c r="J215" t="s">
         <v>1523</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15942,7 +15968,7 @@
       <c r="J216" t="s">
         <v>1523</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15983,7 +16009,7 @@
       <c r="J217" t="s">
         <v>1523</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16024,7 +16050,7 @@
       <c r="J218" t="s">
         <v>1523</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16065,7 +16091,7 @@
       <c r="J219" t="s">
         <v>1523</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16106,7 +16132,7 @@
       <c r="J220" t="s">
         <v>1523</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16147,7 +16173,7 @@
       <c r="J221" t="s">
         <v>1523</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16188,7 +16214,7 @@
       <c r="J222" t="s">
         <v>1523</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16229,7 +16255,7 @@
       <c r="J223" t="s">
         <v>1523</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16270,7 +16296,7 @@
       <c r="J224" t="s">
         <v>1523</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16311,7 +16337,7 @@
       <c r="J225" t="s">
         <v>1523</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16352,7 +16378,7 @@
       <c r="J226" t="s">
         <v>1523</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16393,7 +16419,7 @@
       <c r="J227" t="s">
         <v>1523</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16434,7 +16460,7 @@
       <c r="J228" t="s">
         <v>1523</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16475,7 +16501,7 @@
       <c r="J229" t="s">
         <v>1523</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16516,7 +16542,7 @@
       <c r="J230" t="s">
         <v>1523</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16557,7 +16583,7 @@
       <c r="J231" t="s">
         <v>1523</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16598,7 +16624,7 @@
       <c r="J232" t="s">
         <v>1523</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16639,7 +16665,7 @@
       <c r="J233" t="s">
         <v>1523</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16680,7 +16706,7 @@
       <c r="J234" t="s">
         <v>1523</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16721,7 +16747,7 @@
       <c r="J235" t="s">
         <v>1523</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16762,7 +16788,7 @@
       <c r="J236" t="s">
         <v>1523</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16803,7 +16829,7 @@
       <c r="J237" t="s">
         <v>1523</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16844,7 +16870,7 @@
       <c r="J238" t="s">
         <v>1523</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16885,7 +16911,7 @@
       <c r="J239" t="s">
         <v>1523</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16903,7 +16929,7 @@
       <c r="R239" t="s">
         <v>1722</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -16941,7 +16967,7 @@
       <c r="J240" t="s">
         <v>1523</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16982,7 +17008,7 @@
       <c r="J241" t="s">
         <v>1523</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17023,7 +17049,7 @@
       <c r="J242" t="s">
         <v>1523</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17041,7 +17067,7 @@
       <c r="R242" t="s">
         <v>1715</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17076,7 +17102,7 @@
       <c r="J243" t="s">
         <v>1523</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17117,7 +17143,7 @@
       <c r="J244" t="s">
         <v>1523</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17158,7 +17184,7 @@
       <c r="J245" t="s">
         <v>1523</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17199,7 +17225,7 @@
       <c r="J246" t="s">
         <v>1523</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17217,7 +17243,7 @@
       <c r="R246" t="s">
         <v>1695</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17255,7 +17281,7 @@
       <c r="J247" t="s">
         <v>1523</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17296,7 +17322,7 @@
       <c r="J248" t="s">
         <v>1523</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17337,7 +17363,7 @@
       <c r="J249" t="s">
         <v>1523</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17378,7 +17404,7 @@
       <c r="J250" t="s">
         <v>1523</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17419,7 +17445,7 @@
       <c r="J251" t="s">
         <v>1523</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17460,7 +17486,7 @@
       <c r="J252" t="s">
         <v>1523</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17501,7 +17527,7 @@
       <c r="J253" t="s">
         <v>1523</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17519,7 +17545,7 @@
       <c r="R253" t="s">
         <v>1725</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17557,7 +17583,7 @@
       <c r="J254" t="s">
         <v>1523</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17598,7 +17624,7 @@
       <c r="J255" t="s">
         <v>1523</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17639,7 +17665,7 @@
       <c r="J256" t="s">
         <v>1523</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17648,7 +17674,7 @@
       <c r="M256" t="s">
         <v>1595</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17686,7 +17712,7 @@
       <c r="J257" t="s">
         <v>1523</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17695,7 +17721,7 @@
       <c r="M257" t="s">
         <v>1596</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17739,7 +17765,7 @@
       <c r="J258" t="s">
         <v>1523</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17757,7 +17783,7 @@
       <c r="R258" t="s">
         <v>1707</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17795,7 +17821,7 @@
       <c r="J259" t="s">
         <v>1523</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17813,7 +17839,7 @@
       <c r="R259" t="s">
         <v>1723</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17851,7 +17877,7 @@
       <c r="J260" t="s">
         <v>1523</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17860,7 +17886,7 @@
       <c r="M260" t="s">
         <v>1590</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17904,7 +17930,7 @@
       <c r="J261" t="s">
         <v>1523</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17922,7 +17948,7 @@
       <c r="R261" t="s">
         <v>1729</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17960,7 +17986,7 @@
       <c r="J262" t="s">
         <v>1523</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17978,7 +18004,7 @@
       <c r="R262" t="s">
         <v>1723</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18016,7 +18042,7 @@
       <c r="J263" t="s">
         <v>1523</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18025,7 +18051,7 @@
       <c r="M263" t="s">
         <v>1590</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18069,7 +18095,7 @@
       <c r="J264" t="s">
         <v>1523</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18110,7 +18136,7 @@
       <c r="J265" t="s">
         <v>1523</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18151,7 +18177,7 @@
       <c r="J266" t="s">
         <v>1523</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18192,7 +18218,7 @@
       <c r="J267" t="s">
         <v>1523</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18236,7 +18262,7 @@
       <c r="J268" t="s">
         <v>1523</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18277,7 +18303,7 @@
       <c r="J269" t="s">
         <v>1523</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18318,7 +18344,7 @@
       <c r="J270" t="s">
         <v>1523</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18359,7 +18385,7 @@
       <c r="J271" t="s">
         <v>1523</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18400,7 +18426,7 @@
       <c r="J272" t="s">
         <v>1523</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18418,7 +18444,7 @@
       <c r="R272" t="s">
         <v>1730</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18456,7 +18482,7 @@
       <c r="J273" t="s">
         <v>1523</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18500,7 +18526,7 @@
       <c r="J274" t="s">
         <v>1523</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18541,7 +18567,7 @@
       <c r="J275" t="s">
         <v>1523</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18582,7 +18608,7 @@
       <c r="J276" t="s">
         <v>1523</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18623,7 +18649,7 @@
       <c r="J277" t="s">
         <v>1523</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18664,7 +18690,7 @@
       <c r="J278" t="s">
         <v>1523</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18705,7 +18731,7 @@
       <c r="J279" t="s">
         <v>1523</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18746,7 +18772,7 @@
       <c r="J280" t="s">
         <v>1523</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18787,7 +18813,7 @@
       <c r="J281" t="s">
         <v>1523</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18828,7 +18854,7 @@
       <c r="J282" t="s">
         <v>1523</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18869,7 +18895,7 @@
       <c r="J283" t="s">
         <v>1523</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18910,7 +18936,7 @@
       <c r="J284" t="s">
         <v>1523</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18951,7 +18977,7 @@
       <c r="J285" t="s">
         <v>1523</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18992,7 +19018,7 @@
       <c r="J286" t="s">
         <v>1523</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19033,7 +19059,7 @@
       <c r="J287" t="s">
         <v>1523</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19074,7 +19100,7 @@
       <c r="J288" t="s">
         <v>1523</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19115,7 +19141,7 @@
       <c r="J289" t="s">
         <v>1523</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19156,7 +19182,7 @@
       <c r="J290" t="s">
         <v>1523</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19197,7 +19223,7 @@
       <c r="J291" t="s">
         <v>1523</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19238,7 +19264,7 @@
       <c r="J292" t="s">
         <v>1523</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19279,7 +19305,7 @@
       <c r="J293" t="s">
         <v>1523</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19320,7 +19346,7 @@
       <c r="J294" t="s">
         <v>1523</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19361,7 +19387,7 @@
       <c r="J295" t="s">
         <v>1523</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19379,7 +19405,7 @@
       <c r="R295" t="s">
         <v>1731</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19420,7 +19446,7 @@
       <c r="J296" t="s">
         <v>1523</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19438,7 +19464,7 @@
       <c r="R296" t="s">
         <v>1707</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19476,7 +19502,7 @@
       <c r="J297" t="s">
         <v>1523</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19517,7 +19543,7 @@
       <c r="J298" t="s">
         <v>1523</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19558,7 +19584,7 @@
       <c r="J299" t="s">
         <v>1524</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19599,7 +19625,7 @@
       <c r="J300" t="s">
         <v>1523</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19640,7 +19666,7 @@
       <c r="J301" t="s">
         <v>1523</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20478,7 +20504,7 @@
       <c r="R321" t="s">
         <v>1693</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -20701,7 +20727,7 @@
       <c r="R326" t="s">
         <v>1732</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21536,7 +21562,7 @@
       <c r="R346" t="s">
         <v>1733</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (23/09/2026 12:27)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5381,16 +5381,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5406,7 +5398,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5414,30 +5406,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5737,73 +5711,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5838,7 +5812,7 @@
       <c r="J2" t="s">
         <v>1534</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5882,7 +5856,7 @@
       <c r="J3" t="s">
         <v>1534</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5926,7 +5900,7 @@
       <c r="J4" t="s">
         <v>1534</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5944,7 +5918,7 @@
       <c r="R4" t="s">
         <v>1703</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5982,7 +5956,7 @@
       <c r="J5" t="s">
         <v>1535</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6032,7 +6006,7 @@
       <c r="J6" t="s">
         <v>1534</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6079,7 +6053,7 @@
       <c r="J7" t="s">
         <v>1534</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6126,7 +6100,7 @@
       <c r="J8" t="s">
         <v>1534</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6173,7 +6147,7 @@
       <c r="J9" t="s">
         <v>1534</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6220,7 +6194,7 @@
       <c r="J10" t="s">
         <v>1534</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6267,7 +6241,7 @@
       <c r="J11" t="s">
         <v>1534</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6314,7 +6288,7 @@
       <c r="J12" t="s">
         <v>1534</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6358,7 +6332,7 @@
       <c r="J13" t="s">
         <v>1534</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6376,7 +6350,7 @@
       <c r="R13" t="s">
         <v>1704</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6414,7 +6388,7 @@
       <c r="J14" t="s">
         <v>1534</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6432,7 +6406,7 @@
       <c r="R14" t="s">
         <v>1705</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6470,7 +6444,7 @@
       <c r="J15" t="s">
         <v>1534</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6488,7 +6462,7 @@
       <c r="R15" t="s">
         <v>1705</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6529,7 +6503,7 @@
       <c r="J16" t="s">
         <v>1534</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6573,7 +6547,7 @@
       <c r="J17" t="s">
         <v>1534</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6617,7 +6591,7 @@
       <c r="J18" t="s">
         <v>1534</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6635,7 +6609,7 @@
       <c r="R18" t="s">
         <v>1706</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6676,7 +6650,7 @@
       <c r="J19" t="s">
         <v>1534</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6720,7 +6694,7 @@
       <c r="J20" t="s">
         <v>1534</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6764,7 +6738,7 @@
       <c r="J21" t="s">
         <v>1534</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6782,7 +6756,7 @@
       <c r="R21" t="s">
         <v>1705</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6823,7 +6797,7 @@
       <c r="J22" t="s">
         <v>1534</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6841,7 +6815,7 @@
       <c r="R22" t="s">
         <v>1707</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6882,7 +6856,7 @@
       <c r="J23" t="s">
         <v>1534</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6900,7 +6874,7 @@
       <c r="R23" t="s">
         <v>1708</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6941,7 +6915,7 @@
       <c r="J24" t="s">
         <v>1534</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6985,7 +6959,7 @@
       <c r="J25" t="s">
         <v>1534</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7026,7 +7000,7 @@
       <c r="J26" t="s">
         <v>1536</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7044,7 +7018,7 @@
       <c r="R26" t="s">
         <v>1709</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -7079,7 +7053,7 @@
       <c r="J27" t="s">
         <v>1534</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7097,7 +7071,7 @@
       <c r="R27" t="s">
         <v>1710</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7138,7 +7112,7 @@
       <c r="J28" t="s">
         <v>1534</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7182,7 +7156,7 @@
       <c r="J29" t="s">
         <v>1534</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7226,7 +7200,7 @@
       <c r="J30" t="s">
         <v>1534</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7270,7 +7244,7 @@
       <c r="J31" t="s">
         <v>1534</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7288,7 +7262,7 @@
       <c r="R31" t="s">
         <v>1711</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7329,7 +7303,7 @@
       <c r="J32" t="s">
         <v>1534</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7373,7 +7347,7 @@
       <c r="J33" t="s">
         <v>1534</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7391,7 +7365,7 @@
       <c r="R33" t="s">
         <v>1712</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7432,7 +7406,7 @@
       <c r="J34" t="s">
         <v>1534</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7476,7 +7450,7 @@
       <c r="J35" t="s">
         <v>1534</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7494,7 +7468,7 @@
       <c r="R35" t="s">
         <v>1713</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7535,7 +7509,7 @@
       <c r="J36" t="s">
         <v>1534</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7553,7 +7527,7 @@
       <c r="R36" t="s">
         <v>1713</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7594,7 +7568,7 @@
       <c r="J37" t="s">
         <v>1534</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7612,7 +7586,7 @@
       <c r="R37" t="s">
         <v>1713</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7653,7 +7627,7 @@
       <c r="J38" t="s">
         <v>1534</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7671,7 +7645,7 @@
       <c r="R38" t="s">
         <v>1713</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7712,7 +7686,7 @@
       <c r="J39" t="s">
         <v>1534</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7730,7 +7704,7 @@
       <c r="R39" t="s">
         <v>1713</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7771,7 +7745,7 @@
       <c r="J40" t="s">
         <v>1534</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7789,7 +7763,7 @@
       <c r="R40" t="s">
         <v>1714</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7830,7 +7804,7 @@
       <c r="J41" t="s">
         <v>1534</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7848,7 +7822,7 @@
       <c r="R41" t="s">
         <v>1705</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -7889,7 +7863,7 @@
       <c r="J42" t="s">
         <v>1534</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7907,7 +7881,7 @@
       <c r="R42" t="s">
         <v>1713</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7948,7 +7922,7 @@
       <c r="J43" t="s">
         <v>1534</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7992,7 +7966,7 @@
       <c r="J44" t="s">
         <v>1534</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8010,7 +7984,7 @@
       <c r="R44" t="s">
         <v>1715</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8051,7 +8025,7 @@
       <c r="J45" t="s">
         <v>1534</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8069,7 +8043,7 @@
       <c r="R45" t="s">
         <v>1716</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8107,7 +8081,7 @@
       <c r="J46" t="s">
         <v>1534</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8151,7 +8125,7 @@
       <c r="J47" t="s">
         <v>1534</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8169,7 +8143,7 @@
       <c r="R47" t="s">
         <v>1717</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8210,7 +8184,7 @@
       <c r="J48" t="s">
         <v>1534</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8254,7 +8228,7 @@
       <c r="J49" t="s">
         <v>1534</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8298,7 +8272,7 @@
       <c r="J50" t="s">
         <v>1534</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8342,7 +8316,7 @@
       <c r="J51" t="s">
         <v>1534</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8389,7 +8363,7 @@
       <c r="J52" t="s">
         <v>1534</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8433,7 +8407,7 @@
       <c r="J53" t="s">
         <v>1534</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8477,7 +8451,7 @@
       <c r="J54" t="s">
         <v>1534</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8521,7 +8495,7 @@
       <c r="J55" t="s">
         <v>1534</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8571,7 +8545,7 @@
       <c r="J56" t="s">
         <v>1534</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8624,7 +8598,7 @@
       <c r="J57" t="s">
         <v>1534</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8674,7 +8648,7 @@
       <c r="J58" t="s">
         <v>1534</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8724,7 +8698,7 @@
       <c r="J59" t="s">
         <v>1534</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8742,7 +8716,7 @@
       <c r="R59" t="s">
         <v>1718</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8783,7 +8757,7 @@
       <c r="J60" t="s">
         <v>1534</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8827,7 +8801,7 @@
       <c r="J61" t="s">
         <v>1534</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8871,7 +8845,7 @@
       <c r="J62" t="s">
         <v>1534</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8915,7 +8889,7 @@
       <c r="J63" t="s">
         <v>1534</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8959,7 +8933,7 @@
       <c r="J64" t="s">
         <v>1534</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9003,7 +8977,7 @@
       <c r="J65" t="s">
         <v>1534</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9050,7 +9024,7 @@
       <c r="J66" t="s">
         <v>1534</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9068,7 +9042,7 @@
       <c r="R66" t="s">
         <v>1719</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9106,7 +9080,7 @@
       <c r="J67" t="s">
         <v>1534</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9150,7 +9124,7 @@
       <c r="J68" t="s">
         <v>1534</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9165,7 +9139,7 @@
       <c r="O68" t="s">
         <v>1621</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9209,7 +9183,7 @@
       <c r="J69" t="s">
         <v>1536</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9253,7 +9227,7 @@
       <c r="J70" t="s">
         <v>1534</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9297,7 +9271,7 @@
       <c r="J71" t="s">
         <v>1534</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9341,7 +9315,7 @@
       <c r="J72" t="s">
         <v>1534</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9385,7 +9359,7 @@
       <c r="J73" t="s">
         <v>1534</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9429,7 +9403,7 @@
       <c r="J74" t="s">
         <v>1534</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9473,7 +9447,7 @@
       <c r="J75" t="s">
         <v>1534</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9517,7 +9491,7 @@
       <c r="J76" t="s">
         <v>1534</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9535,7 +9509,7 @@
       <c r="R76" t="s">
         <v>1720</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9573,7 +9547,7 @@
       <c r="J77" t="s">
         <v>1534</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9591,7 +9565,7 @@
       <c r="R77" t="s">
         <v>1720</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9629,7 +9603,7 @@
       <c r="J78" t="s">
         <v>1534</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9647,7 +9621,7 @@
       <c r="R78" t="s">
         <v>1720</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9685,7 +9659,7 @@
       <c r="J79" t="s">
         <v>1534</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9703,7 +9677,7 @@
       <c r="R79" t="s">
         <v>1720</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9741,7 +9715,7 @@
       <c r="J80" t="s">
         <v>1534</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9785,7 +9759,7 @@
       <c r="J81" t="s">
         <v>1534</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9829,7 +9803,7 @@
       <c r="J82" t="s">
         <v>1534</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9873,7 +9847,7 @@
       <c r="J83" t="s">
         <v>1534</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9917,7 +9891,7 @@
       <c r="J84" t="s">
         <v>1534</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9961,7 +9935,7 @@
       <c r="J85" t="s">
         <v>1534</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9979,7 +9953,7 @@
       <c r="R85" t="s">
         <v>1721</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10017,7 +9991,7 @@
       <c r="J86" t="s">
         <v>1534</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10061,7 +10035,7 @@
       <c r="J87" t="s">
         <v>1534</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10079,7 +10053,7 @@
       <c r="R87" t="s">
         <v>1722</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10117,7 +10091,7 @@
       <c r="J88" t="s">
         <v>1534</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10161,7 +10135,7 @@
       <c r="J89" t="s">
         <v>1534</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10179,7 +10153,7 @@
       <c r="R89" t="s">
         <v>1723</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10214,7 +10188,7 @@
       <c r="J90" t="s">
         <v>1534</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10232,7 +10206,7 @@
       <c r="R90" t="s">
         <v>1724</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10267,7 +10241,7 @@
       <c r="J91" t="s">
         <v>1534</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10285,7 +10259,7 @@
       <c r="R91" t="s">
         <v>1708</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10323,7 +10297,7 @@
       <c r="J92" t="s">
         <v>1534</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10344,7 +10318,7 @@
       <c r="R92" t="s">
         <v>1708</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10385,7 +10359,7 @@
       <c r="J93" t="s">
         <v>1534</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10426,7 +10400,7 @@
       <c r="J94" t="s">
         <v>1534</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10470,7 +10444,7 @@
       <c r="J95" t="s">
         <v>1534</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10514,7 +10488,7 @@
       <c r="J96" t="s">
         <v>1534</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10532,7 +10506,7 @@
       <c r="R96" t="s">
         <v>1725</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10570,7 +10544,7 @@
       <c r="J97" t="s">
         <v>1534</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10585,7 +10559,7 @@
       <c r="R97" t="s">
         <v>1725</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10626,7 +10600,7 @@
       <c r="J98" t="s">
         <v>1534</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10644,7 +10618,7 @@
       <c r="R98" t="s">
         <v>1726</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10682,7 +10656,7 @@
       <c r="J99" t="s">
         <v>1534</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10700,7 +10674,7 @@
       <c r="R99" t="s">
         <v>1727</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10738,7 +10712,7 @@
       <c r="J100" t="s">
         <v>1534</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10779,7 +10753,7 @@
       <c r="J101" t="s">
         <v>1534</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10820,7 +10794,7 @@
       <c r="J102" t="s">
         <v>1534</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10861,7 +10835,7 @@
       <c r="J103" t="s">
         <v>1534</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10902,7 +10876,7 @@
       <c r="J104" t="s">
         <v>1534</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10943,7 +10917,7 @@
       <c r="J105" t="s">
         <v>1534</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10984,7 +10958,7 @@
       <c r="J106" t="s">
         <v>1534</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11025,7 +10999,7 @@
       <c r="J107" t="s">
         <v>1534</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11066,7 +11040,7 @@
       <c r="J108" t="s">
         <v>1534</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11107,7 +11081,7 @@
       <c r="J109" t="s">
         <v>1534</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11160,7 +11134,7 @@
       <c r="J110" t="s">
         <v>1534</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11216,7 +11190,7 @@
       <c r="J111" t="s">
         <v>1534</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11234,7 +11208,7 @@
       <c r="R111" t="s">
         <v>1729</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11272,7 +11246,7 @@
       <c r="J112" t="s">
         <v>1534</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11331,7 +11305,7 @@
       <c r="J113" t="s">
         <v>1534</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11375,7 +11349,7 @@
       <c r="J114" t="s">
         <v>1534</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11419,7 +11393,7 @@
       <c r="J115" t="s">
         <v>1534</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11437,7 +11411,7 @@
       <c r="R115" t="s">
         <v>1731</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11475,7 +11449,7 @@
       <c r="J116" t="s">
         <v>1534</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11534,7 +11508,7 @@
       <c r="J117" t="s">
         <v>1534</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11578,7 +11552,7 @@
       <c r="J118" t="s">
         <v>1534</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11625,7 +11599,7 @@
       <c r="J119" t="s">
         <v>1534</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11666,7 +11640,7 @@
       <c r="J120" t="s">
         <v>1534</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11710,7 +11684,7 @@
       <c r="J121" t="s">
         <v>1534</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11757,7 +11731,7 @@
       <c r="J122" t="s">
         <v>1534</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11807,7 +11781,7 @@
       <c r="J123" t="s">
         <v>1534</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11851,7 +11825,7 @@
       <c r="J124" t="s">
         <v>1534</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11895,7 +11869,7 @@
       <c r="J125" t="s">
         <v>1534</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11913,7 +11887,7 @@
       <c r="R125" t="s">
         <v>1733</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11948,7 +11922,7 @@
       <c r="J126" t="s">
         <v>1534</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11966,7 +11940,7 @@
       <c r="R126" t="s">
         <v>1734</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -12001,7 +11975,7 @@
       <c r="J127" t="s">
         <v>1534</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12057,7 +12031,7 @@
       <c r="J128" t="s">
         <v>1534</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12098,7 +12072,7 @@
       <c r="J129" t="s">
         <v>1534</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12139,7 +12113,7 @@
       <c r="J130" t="s">
         <v>1534</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12180,7 +12154,7 @@
       <c r="J131" t="s">
         <v>1534</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12224,7 +12198,7 @@
       <c r="J132" t="s">
         <v>1534</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12265,7 +12239,7 @@
       <c r="J133" t="s">
         <v>1534</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12283,7 +12257,7 @@
       <c r="R133" t="s">
         <v>1720</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12318,7 +12292,7 @@
       <c r="J134" t="s">
         <v>1534</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12336,7 +12310,7 @@
       <c r="R134" t="s">
         <v>1720</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12371,7 +12345,7 @@
       <c r="J135" t="s">
         <v>1534</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12412,7 +12386,7 @@
       <c r="J136" t="s">
         <v>1534</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12453,7 +12427,7 @@
       <c r="J137" t="s">
         <v>1534</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12494,7 +12468,7 @@
       <c r="J138" t="s">
         <v>1534</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12535,7 +12509,7 @@
       <c r="J139" t="s">
         <v>1534</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12582,7 +12556,7 @@
       <c r="J140" t="s">
         <v>1534</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12623,7 +12597,7 @@
       <c r="J141" t="s">
         <v>1534</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12664,7 +12638,7 @@
       <c r="J142" t="s">
         <v>1534</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12708,7 +12682,7 @@
       <c r="J143" t="s">
         <v>1534</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12726,7 +12700,7 @@
       <c r="R143" t="s">
         <v>1720</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12761,7 +12735,7 @@
       <c r="J144" t="s">
         <v>1534</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12779,7 +12753,7 @@
       <c r="R144" t="s">
         <v>1720</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12814,7 +12788,7 @@
       <c r="J145" t="s">
         <v>1534</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12832,7 +12806,7 @@
       <c r="R145" t="s">
         <v>1720</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12867,7 +12841,7 @@
       <c r="J146" t="s">
         <v>1534</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12885,7 +12859,7 @@
       <c r="R146" t="s">
         <v>1728</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12920,7 +12894,7 @@
       <c r="J147" t="s">
         <v>1534</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12938,7 +12912,7 @@
       <c r="R147" t="s">
         <v>1735</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12973,7 +12947,7 @@
       <c r="J148" t="s">
         <v>1534</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13014,7 +12988,7 @@
       <c r="J149" t="s">
         <v>1534</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13032,7 +13006,7 @@
       <c r="R149" t="s">
         <v>1720</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13067,7 +13041,7 @@
       <c r="J150" t="s">
         <v>1534</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13085,7 +13059,7 @@
       <c r="R150" t="s">
         <v>1720</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13120,7 +13094,7 @@
       <c r="J151" t="s">
         <v>1534</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13138,7 +13112,7 @@
       <c r="R151" t="s">
         <v>1736</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13173,7 +13147,7 @@
       <c r="J152" t="s">
         <v>1534</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13191,7 +13165,7 @@
       <c r="R152" t="s">
         <v>1737</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13226,7 +13200,7 @@
       <c r="J153" t="s">
         <v>1534</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13235,7 +13209,7 @@
       <c r="M153" t="s">
         <v>1612</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13276,7 +13250,7 @@
       <c r="J154" t="s">
         <v>1534</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13317,7 +13291,7 @@
       <c r="J155" t="s">
         <v>1534</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13358,7 +13332,7 @@
       <c r="J156" t="s">
         <v>1534</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13399,7 +13373,7 @@
       <c r="J157" t="s">
         <v>1534</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13440,7 +13414,7 @@
       <c r="J158" t="s">
         <v>1534</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13481,7 +13455,7 @@
       <c r="J159" t="s">
         <v>1534</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13522,7 +13496,7 @@
       <c r="J160" t="s">
         <v>1534</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13563,7 +13537,7 @@
       <c r="J161" t="s">
         <v>1534</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13604,7 +13578,7 @@
       <c r="J162" t="s">
         <v>1534</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13622,7 +13596,7 @@
       <c r="R162" t="s">
         <v>1723</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13657,7 +13631,7 @@
       <c r="J163" t="s">
         <v>1534</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13675,7 +13649,7 @@
       <c r="R163" t="s">
         <v>1720</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13710,7 +13684,7 @@
       <c r="J164" t="s">
         <v>1534</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13754,7 +13728,7 @@
       <c r="J165" t="s">
         <v>1534</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13795,7 +13769,7 @@
       <c r="J166" t="s">
         <v>1534</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13813,7 +13787,7 @@
       <c r="R166" t="s">
         <v>1738</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13848,7 +13822,7 @@
       <c r="J167" t="s">
         <v>1534</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13892,7 +13866,7 @@
       <c r="J168" t="s">
         <v>1534</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13936,7 +13910,7 @@
       <c r="J169" t="s">
         <v>1534</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13977,7 +13951,7 @@
       <c r="J170" t="s">
         <v>1534</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14018,7 +13992,7 @@
       <c r="J171" t="s">
         <v>1534</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14059,7 +14033,7 @@
       <c r="J172" t="s">
         <v>1534</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14100,7 +14074,7 @@
       <c r="J173" t="s">
         <v>1534</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14141,7 +14115,7 @@
       <c r="J174" t="s">
         <v>1534</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14182,7 +14156,7 @@
       <c r="J175" t="s">
         <v>1534</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14223,7 +14197,7 @@
       <c r="J176" t="s">
         <v>1534</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14264,7 +14238,7 @@
       <c r="J177" t="s">
         <v>1534</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14305,7 +14279,7 @@
       <c r="J178" t="s">
         <v>1534</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14323,7 +14297,7 @@
       <c r="R178" t="s">
         <v>1736</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14361,7 +14335,7 @@
       <c r="J179" t="s">
         <v>1534</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14370,7 +14344,7 @@
       <c r="M179" t="s">
         <v>1609</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14411,7 +14385,7 @@
       <c r="J180" t="s">
         <v>1534</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14452,7 +14426,7 @@
       <c r="J181" t="s">
         <v>1534</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14470,7 +14444,7 @@
       <c r="R181" t="s">
         <v>1720</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14505,7 +14479,7 @@
       <c r="J182" t="s">
         <v>1534</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14546,7 +14520,7 @@
       <c r="J183" t="s">
         <v>1534</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14587,7 +14561,7 @@
       <c r="J184" t="s">
         <v>1534</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14628,7 +14602,7 @@
       <c r="J185" t="s">
         <v>1534</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14669,7 +14643,7 @@
       <c r="J186" t="s">
         <v>1534</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14710,7 +14684,7 @@
       <c r="J187" t="s">
         <v>1534</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14751,7 +14725,7 @@
       <c r="J188" t="s">
         <v>1534</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14792,7 +14766,7 @@
       <c r="J189" t="s">
         <v>1534</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14833,7 +14807,7 @@
       <c r="J190" t="s">
         <v>1534</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14874,7 +14848,7 @@
       <c r="J191" t="s">
         <v>1534</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14915,7 +14889,7 @@
       <c r="J192" t="s">
         <v>1534</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14956,7 +14930,7 @@
       <c r="J193" t="s">
         <v>1534</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14997,7 +14971,7 @@
       <c r="J194" t="s">
         <v>1534</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15038,7 +15012,7 @@
       <c r="J195" t="s">
         <v>1534</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15056,7 +15030,7 @@
       <c r="R195" t="s">
         <v>1729</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15097,7 +15071,7 @@
       <c r="J196" t="s">
         <v>1534</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15115,7 +15089,7 @@
       <c r="R196" t="s">
         <v>1735</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15153,7 +15127,7 @@
       <c r="J197" t="s">
         <v>1534</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15194,7 +15168,7 @@
       <c r="J198" t="s">
         <v>1536</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15235,7 +15209,7 @@
       <c r="J199" t="s">
         <v>1535</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15276,7 +15250,7 @@
       <c r="J200" t="s">
         <v>1534</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15317,7 +15291,7 @@
       <c r="J201" t="s">
         <v>1534</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15358,7 +15332,7 @@
       <c r="J202" t="s">
         <v>1534</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15376,7 +15350,7 @@
       <c r="R202" t="s">
         <v>1720</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15411,7 +15385,7 @@
       <c r="J203" t="s">
         <v>1534</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15429,7 +15403,7 @@
       <c r="R203" t="s">
         <v>1728</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15464,7 +15438,7 @@
       <c r="J204" t="s">
         <v>1534</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15479,7 +15453,7 @@
       <c r="R204" t="s">
         <v>1739</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15517,7 +15491,7 @@
       <c r="J205" t="s">
         <v>1534</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15535,7 +15509,7 @@
       <c r="R205" t="s">
         <v>1740</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15573,7 +15547,7 @@
       <c r="J206" t="s">
         <v>1534</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15591,7 +15565,7 @@
       <c r="R206" t="s">
         <v>1708</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15626,7 +15600,7 @@
       <c r="J207" t="s">
         <v>1534</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15667,7 +15641,7 @@
       <c r="J208" t="s">
         <v>1534</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15708,7 +15682,7 @@
       <c r="J209" t="s">
         <v>1534</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15749,7 +15723,7 @@
       <c r="J210" t="s">
         <v>1534</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15790,7 +15764,7 @@
       <c r="J211" t="s">
         <v>1534</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15831,7 +15805,7 @@
       <c r="J212" t="s">
         <v>1534</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15872,7 +15846,7 @@
       <c r="J213" t="s">
         <v>1534</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15913,7 +15887,7 @@
       <c r="J214" t="s">
         <v>1534</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15931,7 +15905,7 @@
       <c r="R214" t="s">
         <v>1741</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15966,7 +15940,7 @@
       <c r="J215" t="s">
         <v>1534</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16007,7 +15981,7 @@
       <c r="J216" t="s">
         <v>1534</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16048,7 +16022,7 @@
       <c r="J217" t="s">
         <v>1534</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16089,7 +16063,7 @@
       <c r="J218" t="s">
         <v>1534</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16130,7 +16104,7 @@
       <c r="J219" t="s">
         <v>1534</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16171,7 +16145,7 @@
       <c r="J220" t="s">
         <v>1534</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16212,7 +16186,7 @@
       <c r="J221" t="s">
         <v>1534</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16253,7 +16227,7 @@
       <c r="J222" t="s">
         <v>1534</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16294,7 +16268,7 @@
       <c r="J223" t="s">
         <v>1534</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16335,7 +16309,7 @@
       <c r="J224" t="s">
         <v>1534</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16376,7 +16350,7 @@
       <c r="J225" t="s">
         <v>1534</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16417,7 +16391,7 @@
       <c r="J226" t="s">
         <v>1534</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16458,7 +16432,7 @@
       <c r="J227" t="s">
         <v>1534</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16499,7 +16473,7 @@
       <c r="J228" t="s">
         <v>1534</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16540,7 +16514,7 @@
       <c r="J229" t="s">
         <v>1534</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16581,7 +16555,7 @@
       <c r="J230" t="s">
         <v>1534</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16622,7 +16596,7 @@
       <c r="J231" t="s">
         <v>1534</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16663,7 +16637,7 @@
       <c r="J232" t="s">
         <v>1534</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16704,7 +16678,7 @@
       <c r="J233" t="s">
         <v>1534</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16745,7 +16719,7 @@
       <c r="J234" t="s">
         <v>1534</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16786,7 +16760,7 @@
       <c r="J235" t="s">
         <v>1534</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16827,7 +16801,7 @@
       <c r="J236" t="s">
         <v>1534</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16868,7 +16842,7 @@
       <c r="J237" t="s">
         <v>1534</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16909,7 +16883,7 @@
       <c r="J238" t="s">
         <v>1534</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16950,7 +16924,7 @@
       <c r="J239" t="s">
         <v>1534</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16968,7 +16942,7 @@
       <c r="R239" t="s">
         <v>1735</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17006,7 +16980,7 @@
       <c r="J240" t="s">
         <v>1534</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17047,7 +17021,7 @@
       <c r="J241" t="s">
         <v>1534</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17088,7 +17062,7 @@
       <c r="J242" t="s">
         <v>1534</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17106,7 +17080,7 @@
       <c r="R242" t="s">
         <v>1728</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17141,7 +17115,7 @@
       <c r="J243" t="s">
         <v>1534</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17182,7 +17156,7 @@
       <c r="J244" t="s">
         <v>1534</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17223,7 +17197,7 @@
       <c r="J245" t="s">
         <v>1534</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17264,7 +17238,7 @@
       <c r="J246" t="s">
         <v>1534</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17282,7 +17256,7 @@
       <c r="R246" t="s">
         <v>1708</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17320,7 +17294,7 @@
       <c r="J247" t="s">
         <v>1534</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17361,7 +17335,7 @@
       <c r="J248" t="s">
         <v>1534</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17402,7 +17376,7 @@
       <c r="J249" t="s">
         <v>1534</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17443,7 +17417,7 @@
       <c r="J250" t="s">
         <v>1534</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17484,7 +17458,7 @@
       <c r="J251" t="s">
         <v>1534</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17525,7 +17499,7 @@
       <c r="J252" t="s">
         <v>1534</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17566,7 +17540,7 @@
       <c r="J253" t="s">
         <v>1534</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17584,7 +17558,7 @@
       <c r="R253" t="s">
         <v>1738</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17622,7 +17596,7 @@
       <c r="J254" t="s">
         <v>1534</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17663,7 +17637,7 @@
       <c r="J255" t="s">
         <v>1534</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17704,7 +17678,7 @@
       <c r="J256" t="s">
         <v>1534</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17713,7 +17687,7 @@
       <c r="M256" t="s">
         <v>1608</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17751,7 +17725,7 @@
       <c r="J257" t="s">
         <v>1534</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17760,7 +17734,7 @@
       <c r="M257" t="s">
         <v>1609</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17804,7 +17778,7 @@
       <c r="J258" t="s">
         <v>1534</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17822,7 +17796,7 @@
       <c r="R258" t="s">
         <v>1720</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17860,7 +17834,7 @@
       <c r="J259" t="s">
         <v>1534</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17878,7 +17852,7 @@
       <c r="R259" t="s">
         <v>1736</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17916,7 +17890,7 @@
       <c r="J260" t="s">
         <v>1534</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17925,7 +17899,7 @@
       <c r="M260" t="s">
         <v>1603</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17969,7 +17943,7 @@
       <c r="J261" t="s">
         <v>1534</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17987,7 +17961,7 @@
       <c r="R261" t="s">
         <v>1742</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18025,7 +17999,7 @@
       <c r="J262" t="s">
         <v>1534</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18043,7 +18017,7 @@
       <c r="R262" t="s">
         <v>1736</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18081,7 +18055,7 @@
       <c r="J263" t="s">
         <v>1534</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18090,7 +18064,7 @@
       <c r="M263" t="s">
         <v>1603</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18134,7 +18108,7 @@
       <c r="J264" t="s">
         <v>1534</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18175,7 +18149,7 @@
       <c r="J265" t="s">
         <v>1534</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18216,7 +18190,7 @@
       <c r="J266" t="s">
         <v>1534</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18257,7 +18231,7 @@
       <c r="J267" t="s">
         <v>1534</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18301,7 +18275,7 @@
       <c r="J268" t="s">
         <v>1534</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18342,7 +18316,7 @@
       <c r="J269" t="s">
         <v>1534</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18383,7 +18357,7 @@
       <c r="J270" t="s">
         <v>1534</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18424,7 +18398,7 @@
       <c r="J271" t="s">
         <v>1534</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18465,7 +18439,7 @@
       <c r="J272" t="s">
         <v>1534</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18483,7 +18457,7 @@
       <c r="R272" t="s">
         <v>1743</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18521,7 +18495,7 @@
       <c r="J273" t="s">
         <v>1534</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18565,7 +18539,7 @@
       <c r="J274" t="s">
         <v>1534</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18606,7 +18580,7 @@
       <c r="J275" t="s">
         <v>1534</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18647,7 +18621,7 @@
       <c r="J276" t="s">
         <v>1534</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18688,7 +18662,7 @@
       <c r="J277" t="s">
         <v>1534</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18729,7 +18703,7 @@
       <c r="J278" t="s">
         <v>1534</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18770,7 +18744,7 @@
       <c r="J279" t="s">
         <v>1534</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18811,7 +18785,7 @@
       <c r="J280" t="s">
         <v>1534</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18852,7 +18826,7 @@
       <c r="J281" t="s">
         <v>1534</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18893,7 +18867,7 @@
       <c r="J282" t="s">
         <v>1534</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18934,7 +18908,7 @@
       <c r="J283" t="s">
         <v>1534</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18975,7 +18949,7 @@
       <c r="J284" t="s">
         <v>1534</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19016,7 +18990,7 @@
       <c r="J285" t="s">
         <v>1534</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19057,7 +19031,7 @@
       <c r="J286" t="s">
         <v>1534</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19098,7 +19072,7 @@
       <c r="J287" t="s">
         <v>1534</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19139,7 +19113,7 @@
       <c r="J288" t="s">
         <v>1534</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19180,7 +19154,7 @@
       <c r="J289" t="s">
         <v>1534</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19221,7 +19195,7 @@
       <c r="J290" t="s">
         <v>1534</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19262,7 +19236,7 @@
       <c r="J291" t="s">
         <v>1534</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19303,7 +19277,7 @@
       <c r="J292" t="s">
         <v>1534</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19344,7 +19318,7 @@
       <c r="J293" t="s">
         <v>1534</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19385,7 +19359,7 @@
       <c r="J294" t="s">
         <v>1534</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19426,7 +19400,7 @@
       <c r="J295" t="s">
         <v>1534</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19444,7 +19418,7 @@
       <c r="R295" t="s">
         <v>1744</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19485,7 +19459,7 @@
       <c r="J296" t="s">
         <v>1534</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19503,7 +19477,7 @@
       <c r="R296" t="s">
         <v>1720</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19541,7 +19515,7 @@
       <c r="J297" t="s">
         <v>1534</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19582,7 +19556,7 @@
       <c r="J298" t="s">
         <v>1534</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19623,7 +19597,7 @@
       <c r="J299" t="s">
         <v>1535</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19664,7 +19638,7 @@
       <c r="J300" t="s">
         <v>1534</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19705,7 +19679,7 @@
       <c r="J301" t="s">
         <v>1534</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20543,7 +20517,7 @@
       <c r="R321" t="s">
         <v>1706</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -20766,7 +20740,7 @@
       <c r="R326" t="s">
         <v>1745</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21601,7 +21575,7 @@
       <c r="R346" t="s">
         <v>1746</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (29/09/2026 19:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5558,8 +5558,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5575,7 +5583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5583,12 +5591,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5888,73 +5914,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5989,7 +6015,7 @@
       <c r="J2" t="s">
         <v>1591</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6033,7 +6059,7 @@
       <c r="J3" t="s">
         <v>1591</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6077,7 +6103,7 @@
       <c r="J4" t="s">
         <v>1591</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6095,7 +6121,7 @@
       <c r="R4" t="s">
         <v>1762</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6133,7 +6159,7 @@
       <c r="J5" t="s">
         <v>1592</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6183,7 +6209,7 @@
       <c r="J6" t="s">
         <v>1591</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6230,7 +6256,7 @@
       <c r="J7" t="s">
         <v>1591</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6277,7 +6303,7 @@
       <c r="J8" t="s">
         <v>1591</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6324,7 +6350,7 @@
       <c r="J9" t="s">
         <v>1591</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6371,7 +6397,7 @@
       <c r="J10" t="s">
         <v>1591</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6418,7 +6444,7 @@
       <c r="J11" t="s">
         <v>1591</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6465,7 +6491,7 @@
       <c r="J12" t="s">
         <v>1591</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6509,7 +6535,7 @@
       <c r="J13" t="s">
         <v>1591</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6527,7 +6553,7 @@
       <c r="R13" t="s">
         <v>1763</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6565,7 +6591,7 @@
       <c r="J14" t="s">
         <v>1591</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6583,7 +6609,7 @@
       <c r="R14" t="s">
         <v>1764</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6621,7 +6647,7 @@
       <c r="J15" t="s">
         <v>1591</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6639,7 +6665,7 @@
       <c r="R15" t="s">
         <v>1764</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6680,7 +6706,7 @@
       <c r="J16" t="s">
         <v>1591</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6724,7 +6750,7 @@
       <c r="J17" t="s">
         <v>1591</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6768,7 +6794,7 @@
       <c r="J18" t="s">
         <v>1591</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6786,7 +6812,7 @@
       <c r="R18" t="s">
         <v>1765</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6827,7 +6853,7 @@
       <c r="J19" t="s">
         <v>1591</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6871,7 +6897,7 @@
       <c r="J20" t="s">
         <v>1591</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6915,7 +6941,7 @@
       <c r="J21" t="s">
         <v>1591</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6933,7 +6959,7 @@
       <c r="R21" t="s">
         <v>1764</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6974,7 +7000,7 @@
       <c r="J22" t="s">
         <v>1591</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6992,7 +7018,7 @@
       <c r="R22" t="s">
         <v>1766</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7033,7 +7059,7 @@
       <c r="J23" t="s">
         <v>1591</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7051,7 +7077,7 @@
       <c r="R23" t="s">
         <v>1767</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7092,7 +7118,7 @@
       <c r="J24" t="s">
         <v>1591</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7136,7 +7162,7 @@
       <c r="J25" t="s">
         <v>1591</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7177,7 +7203,7 @@
       <c r="J26" t="s">
         <v>1593</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7195,7 +7221,7 @@
       <c r="R26" t="s">
         <v>1768</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -7230,7 +7256,7 @@
       <c r="J27" t="s">
         <v>1591</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7248,7 +7274,7 @@
       <c r="R27" t="s">
         <v>1769</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7289,7 +7315,7 @@
       <c r="J28" t="s">
         <v>1591</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7333,7 +7359,7 @@
       <c r="J29" t="s">
         <v>1591</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7377,7 +7403,7 @@
       <c r="J30" t="s">
         <v>1591</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7421,7 +7447,7 @@
       <c r="J31" t="s">
         <v>1591</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7439,7 +7465,7 @@
       <c r="R31" t="s">
         <v>1770</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7480,7 +7506,7 @@
       <c r="J32" t="s">
         <v>1591</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7524,7 +7550,7 @@
       <c r="J33" t="s">
         <v>1591</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7542,7 +7568,7 @@
       <c r="R33" t="s">
         <v>1771</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7583,7 +7609,7 @@
       <c r="J34" t="s">
         <v>1591</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7627,7 +7653,7 @@
       <c r="J35" t="s">
         <v>1591</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7645,7 +7671,7 @@
       <c r="R35" t="s">
         <v>1772</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7686,7 +7712,7 @@
       <c r="J36" t="s">
         <v>1591</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7704,7 +7730,7 @@
       <c r="R36" t="s">
         <v>1772</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7745,7 +7771,7 @@
       <c r="J37" t="s">
         <v>1591</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7763,7 +7789,7 @@
       <c r="R37" t="s">
         <v>1772</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7804,7 +7830,7 @@
       <c r="J38" t="s">
         <v>1591</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7822,7 +7848,7 @@
       <c r="R38" t="s">
         <v>1772</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7863,7 +7889,7 @@
       <c r="J39" t="s">
         <v>1591</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7881,7 +7907,7 @@
       <c r="R39" t="s">
         <v>1772</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7922,7 +7948,7 @@
       <c r="J40" t="s">
         <v>1591</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7940,7 +7966,7 @@
       <c r="R40" t="s">
         <v>1773</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7981,7 +8007,7 @@
       <c r="J41" t="s">
         <v>1591</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7999,7 +8025,7 @@
       <c r="R41" t="s">
         <v>1764</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8040,7 +8066,7 @@
       <c r="J42" t="s">
         <v>1591</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8058,7 +8084,7 @@
       <c r="R42" t="s">
         <v>1772</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8099,7 +8125,7 @@
       <c r="J43" t="s">
         <v>1591</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8143,7 +8169,7 @@
       <c r="J44" t="s">
         <v>1591</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8161,7 +8187,7 @@
       <c r="R44" t="s">
         <v>1774</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8202,7 +8228,7 @@
       <c r="J45" t="s">
         <v>1591</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8220,7 +8246,7 @@
       <c r="R45" t="s">
         <v>1775</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8258,7 +8284,7 @@
       <c r="J46" t="s">
         <v>1591</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8302,7 +8328,7 @@
       <c r="J47" t="s">
         <v>1591</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8320,7 +8346,7 @@
       <c r="R47" t="s">
         <v>1776</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8361,7 +8387,7 @@
       <c r="J48" t="s">
         <v>1591</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8405,7 +8431,7 @@
       <c r="J49" t="s">
         <v>1591</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8449,7 +8475,7 @@
       <c r="J50" t="s">
         <v>1591</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8493,7 +8519,7 @@
       <c r="J51" t="s">
         <v>1591</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8540,7 +8566,7 @@
       <c r="J52" t="s">
         <v>1591</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8584,7 +8610,7 @@
       <c r="J53" t="s">
         <v>1591</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8628,7 +8654,7 @@
       <c r="J54" t="s">
         <v>1591</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8672,7 +8698,7 @@
       <c r="J55" t="s">
         <v>1591</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8722,7 +8748,7 @@
       <c r="J56" t="s">
         <v>1591</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8775,7 +8801,7 @@
       <c r="J57" t="s">
         <v>1591</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8825,7 +8851,7 @@
       <c r="J58" t="s">
         <v>1591</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8875,7 +8901,7 @@
       <c r="J59" t="s">
         <v>1591</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8893,7 +8919,7 @@
       <c r="R59" t="s">
         <v>1777</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8934,7 +8960,7 @@
       <c r="J60" t="s">
         <v>1591</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8978,7 +9004,7 @@
       <c r="J61" t="s">
         <v>1591</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9022,7 +9048,7 @@
       <c r="J62" t="s">
         <v>1591</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9066,7 +9092,7 @@
       <c r="J63" t="s">
         <v>1591</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9110,7 +9136,7 @@
       <c r="J64" t="s">
         <v>1591</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9154,7 +9180,7 @@
       <c r="J65" t="s">
         <v>1591</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9201,7 +9227,7 @@
       <c r="J66" t="s">
         <v>1591</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9219,7 +9245,7 @@
       <c r="R66" t="s">
         <v>1778</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9257,7 +9283,7 @@
       <c r="J67" t="s">
         <v>1591</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9301,7 +9327,7 @@
       <c r="J68" t="s">
         <v>1591</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9316,7 +9342,7 @@
       <c r="O68" t="s">
         <v>1682</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9360,7 +9386,7 @@
       <c r="J69" t="s">
         <v>1593</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9404,7 +9430,7 @@
       <c r="J70" t="s">
         <v>1591</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9448,7 +9474,7 @@
       <c r="J71" t="s">
         <v>1591</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9492,7 +9518,7 @@
       <c r="J72" t="s">
         <v>1591</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9536,7 +9562,7 @@
       <c r="J73" t="s">
         <v>1591</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9580,7 +9606,7 @@
       <c r="J74" t="s">
         <v>1591</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9624,7 +9650,7 @@
       <c r="J75" t="s">
         <v>1591</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9668,7 +9694,7 @@
       <c r="J76" t="s">
         <v>1591</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9686,7 +9712,7 @@
       <c r="R76" t="s">
         <v>1779</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9724,7 +9750,7 @@
       <c r="J77" t="s">
         <v>1591</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9742,7 +9768,7 @@
       <c r="R77" t="s">
         <v>1779</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9780,7 +9806,7 @@
       <c r="J78" t="s">
         <v>1591</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9798,7 +9824,7 @@
       <c r="R78" t="s">
         <v>1779</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9836,7 +9862,7 @@
       <c r="J79" t="s">
         <v>1591</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9854,7 +9880,7 @@
       <c r="R79" t="s">
         <v>1779</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9892,7 +9918,7 @@
       <c r="J80" t="s">
         <v>1591</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9936,7 +9962,7 @@
       <c r="J81" t="s">
         <v>1591</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9980,7 +10006,7 @@
       <c r="J82" t="s">
         <v>1591</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10024,7 +10050,7 @@
       <c r="J83" t="s">
         <v>1591</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10068,7 +10094,7 @@
       <c r="J84" t="s">
         <v>1591</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10112,7 +10138,7 @@
       <c r="J85" t="s">
         <v>1591</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10130,7 +10156,7 @@
       <c r="R85" t="s">
         <v>1780</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10168,7 +10194,7 @@
       <c r="J86" t="s">
         <v>1591</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10212,7 +10238,7 @@
       <c r="J87" t="s">
         <v>1591</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10230,7 +10256,7 @@
       <c r="R87" t="s">
         <v>1781</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10268,7 +10294,7 @@
       <c r="J88" t="s">
         <v>1591</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10312,7 +10338,7 @@
       <c r="J89" t="s">
         <v>1591</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10330,7 +10356,7 @@
       <c r="R89" t="s">
         <v>1782</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10365,7 +10391,7 @@
       <c r="J90" t="s">
         <v>1591</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10383,7 +10409,7 @@
       <c r="R90" t="s">
         <v>1783</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10418,7 +10444,7 @@
       <c r="J91" t="s">
         <v>1591</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10436,7 +10462,7 @@
       <c r="R91" t="s">
         <v>1767</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10474,7 +10500,7 @@
       <c r="J92" t="s">
         <v>1591</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10495,7 +10521,7 @@
       <c r="R92" t="s">
         <v>1767</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10536,7 +10562,7 @@
       <c r="J93" t="s">
         <v>1591</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10577,7 +10603,7 @@
       <c r="J94" t="s">
         <v>1591</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10621,7 +10647,7 @@
       <c r="J95" t="s">
         <v>1591</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10665,7 +10691,7 @@
       <c r="J96" t="s">
         <v>1591</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10683,7 +10709,7 @@
       <c r="R96" t="s">
         <v>1784</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10721,7 +10747,7 @@
       <c r="J97" t="s">
         <v>1591</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10736,7 +10762,7 @@
       <c r="R97" t="s">
         <v>1784</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10777,7 +10803,7 @@
       <c r="J98" t="s">
         <v>1591</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10795,7 +10821,7 @@
       <c r="R98" t="s">
         <v>1785</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10833,7 +10859,7 @@
       <c r="J99" t="s">
         <v>1591</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10851,7 +10877,7 @@
       <c r="R99" t="s">
         <v>1786</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10889,7 +10915,7 @@
       <c r="J100" t="s">
         <v>1591</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10930,7 +10956,7 @@
       <c r="J101" t="s">
         <v>1591</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10971,7 +10997,7 @@
       <c r="J102" t="s">
         <v>1591</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11012,7 +11038,7 @@
       <c r="J103" t="s">
         <v>1591</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11053,7 +11079,7 @@
       <c r="J104" t="s">
         <v>1591</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11094,7 +11120,7 @@
       <c r="J105" t="s">
         <v>1591</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11135,7 +11161,7 @@
       <c r="J106" t="s">
         <v>1591</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11176,7 +11202,7 @@
       <c r="J107" t="s">
         <v>1591</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11217,7 +11243,7 @@
       <c r="J108" t="s">
         <v>1591</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11258,7 +11284,7 @@
       <c r="J109" t="s">
         <v>1591</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11311,7 +11337,7 @@
       <c r="J110" t="s">
         <v>1591</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11367,7 +11393,7 @@
       <c r="J111" t="s">
         <v>1591</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11385,7 +11411,7 @@
       <c r="R111" t="s">
         <v>1788</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11423,7 +11449,7 @@
       <c r="J112" t="s">
         <v>1591</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11482,7 +11508,7 @@
       <c r="J113" t="s">
         <v>1591</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11526,7 +11552,7 @@
       <c r="J114" t="s">
         <v>1591</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11570,7 +11596,7 @@
       <c r="J115" t="s">
         <v>1591</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11588,7 +11614,7 @@
       <c r="R115" t="s">
         <v>1790</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11626,7 +11652,7 @@
       <c r="J116" t="s">
         <v>1591</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11685,7 +11711,7 @@
       <c r="J117" t="s">
         <v>1591</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11729,7 +11755,7 @@
       <c r="J118" t="s">
         <v>1591</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11776,7 +11802,7 @@
       <c r="J119" t="s">
         <v>1591</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11817,7 +11843,7 @@
       <c r="J120" t="s">
         <v>1591</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11861,7 +11887,7 @@
       <c r="J121" t="s">
         <v>1591</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11908,7 +11934,7 @@
       <c r="J122" t="s">
         <v>1591</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11958,7 +11984,7 @@
       <c r="J123" t="s">
         <v>1591</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12002,7 +12028,7 @@
       <c r="J124" t="s">
         <v>1591</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12046,7 +12072,7 @@
       <c r="J125" t="s">
         <v>1591</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12064,7 +12090,7 @@
       <c r="R125" t="s">
         <v>1792</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12099,7 +12125,7 @@
       <c r="J126" t="s">
         <v>1591</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12117,7 +12143,7 @@
       <c r="R126" t="s">
         <v>1793</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -12152,7 +12178,7 @@
       <c r="J127" t="s">
         <v>1591</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12208,7 +12234,7 @@
       <c r="J128" t="s">
         <v>1591</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12249,7 +12275,7 @@
       <c r="J129" t="s">
         <v>1591</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12290,7 +12316,7 @@
       <c r="J130" t="s">
         <v>1591</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12331,7 +12357,7 @@
       <c r="J131" t="s">
         <v>1591</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12375,7 +12401,7 @@
       <c r="J132" t="s">
         <v>1591</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12416,7 +12442,7 @@
       <c r="J133" t="s">
         <v>1591</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12434,7 +12460,7 @@
       <c r="R133" t="s">
         <v>1779</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12469,7 +12495,7 @@
       <c r="J134" t="s">
         <v>1591</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12487,7 +12513,7 @@
       <c r="R134" t="s">
         <v>1779</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12522,7 +12548,7 @@
       <c r="J135" t="s">
         <v>1591</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12563,7 +12589,7 @@
       <c r="J136" t="s">
         <v>1591</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12604,7 +12630,7 @@
       <c r="J137" t="s">
         <v>1591</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12645,7 +12671,7 @@
       <c r="J138" t="s">
         <v>1591</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12686,7 +12712,7 @@
       <c r="J139" t="s">
         <v>1591</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12733,7 +12759,7 @@
       <c r="J140" t="s">
         <v>1591</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12774,7 +12800,7 @@
       <c r="J141" t="s">
         <v>1591</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12815,7 +12841,7 @@
       <c r="J142" t="s">
         <v>1591</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12859,7 +12885,7 @@
       <c r="J143" t="s">
         <v>1591</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12877,7 +12903,7 @@
       <c r="R143" t="s">
         <v>1779</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12912,7 +12938,7 @@
       <c r="J144" t="s">
         <v>1591</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12930,7 +12956,7 @@
       <c r="R144" t="s">
         <v>1779</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12965,7 +12991,7 @@
       <c r="J145" t="s">
         <v>1591</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12983,7 +13009,7 @@
       <c r="R145" t="s">
         <v>1779</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13018,7 +13044,7 @@
       <c r="J146" t="s">
         <v>1591</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13036,7 +13062,7 @@
       <c r="R146" t="s">
         <v>1787</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13071,7 +13097,7 @@
       <c r="J147" t="s">
         <v>1591</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13089,7 +13115,7 @@
       <c r="R147" t="s">
         <v>1794</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13124,7 +13150,7 @@
       <c r="J148" t="s">
         <v>1591</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13165,7 +13191,7 @@
       <c r="J149" t="s">
         <v>1591</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13183,7 +13209,7 @@
       <c r="R149" t="s">
         <v>1779</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13218,7 +13244,7 @@
       <c r="J150" t="s">
         <v>1591</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13236,7 +13262,7 @@
       <c r="R150" t="s">
         <v>1779</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -13271,7 +13297,7 @@
       <c r="J151" t="s">
         <v>1591</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13289,7 +13315,7 @@
       <c r="R151" t="s">
         <v>1795</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13324,7 +13350,7 @@
       <c r="J152" t="s">
         <v>1591</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13342,7 +13368,7 @@
       <c r="R152" t="s">
         <v>1796</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13377,7 +13403,7 @@
       <c r="J153" t="s">
         <v>1591</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13386,7 +13412,7 @@
       <c r="M153" t="s">
         <v>1673</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13427,7 +13453,7 @@
       <c r="J154" t="s">
         <v>1591</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13468,7 +13494,7 @@
       <c r="J155" t="s">
         <v>1591</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13509,7 +13535,7 @@
       <c r="J156" t="s">
         <v>1591</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13550,7 +13576,7 @@
       <c r="J157" t="s">
         <v>1591</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13591,7 +13617,7 @@
       <c r="J158" t="s">
         <v>1591</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13632,7 +13658,7 @@
       <c r="J159" t="s">
         <v>1591</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13673,7 +13699,7 @@
       <c r="J160" t="s">
         <v>1591</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13714,7 +13740,7 @@
       <c r="J161" t="s">
         <v>1591</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13755,7 +13781,7 @@
       <c r="J162" t="s">
         <v>1591</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13773,7 +13799,7 @@
       <c r="R162" t="s">
         <v>1782</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13808,7 +13834,7 @@
       <c r="J163" t="s">
         <v>1591</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13826,7 +13852,7 @@
       <c r="R163" t="s">
         <v>1779</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13861,7 +13887,7 @@
       <c r="J164" t="s">
         <v>1591</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13905,7 +13931,7 @@
       <c r="J165" t="s">
         <v>1591</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13946,7 +13972,7 @@
       <c r="J166" t="s">
         <v>1591</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13964,7 +13990,7 @@
       <c r="R166" t="s">
         <v>1797</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13999,7 +14025,7 @@
       <c r="J167" t="s">
         <v>1591</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14043,7 +14069,7 @@
       <c r="J168" t="s">
         <v>1591</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14087,7 +14113,7 @@
       <c r="J169" t="s">
         <v>1591</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14128,7 +14154,7 @@
       <c r="J170" t="s">
         <v>1591</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14169,7 +14195,7 @@
       <c r="J171" t="s">
         <v>1591</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14210,7 +14236,7 @@
       <c r="J172" t="s">
         <v>1591</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14251,7 +14277,7 @@
       <c r="J173" t="s">
         <v>1591</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14292,7 +14318,7 @@
       <c r="J174" t="s">
         <v>1591</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14333,7 +14359,7 @@
       <c r="J175" t="s">
         <v>1591</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14374,7 +14400,7 @@
       <c r="J176" t="s">
         <v>1591</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14415,7 +14441,7 @@
       <c r="J177" t="s">
         <v>1591</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14456,7 +14482,7 @@
       <c r="J178" t="s">
         <v>1591</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14474,7 +14500,7 @@
       <c r="R178" t="s">
         <v>1795</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14512,7 +14538,7 @@
       <c r="J179" t="s">
         <v>1591</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14521,7 +14547,7 @@
       <c r="M179" t="s">
         <v>1670</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14562,7 +14588,7 @@
       <c r="J180" t="s">
         <v>1591</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14603,7 +14629,7 @@
       <c r="J181" t="s">
         <v>1591</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14621,7 +14647,7 @@
       <c r="R181" t="s">
         <v>1779</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14656,7 +14682,7 @@
       <c r="J182" t="s">
         <v>1591</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14697,7 +14723,7 @@
       <c r="J183" t="s">
         <v>1591</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14738,7 +14764,7 @@
       <c r="J184" t="s">
         <v>1591</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14779,7 +14805,7 @@
       <c r="J185" t="s">
         <v>1591</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14820,7 +14846,7 @@
       <c r="J186" t="s">
         <v>1591</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14861,7 +14887,7 @@
       <c r="J187" t="s">
         <v>1591</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14902,7 +14928,7 @@
       <c r="J188" t="s">
         <v>1591</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14943,7 +14969,7 @@
       <c r="J189" t="s">
         <v>1591</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14984,7 +15010,7 @@
       <c r="J190" t="s">
         <v>1591</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15025,7 +15051,7 @@
       <c r="J191" t="s">
         <v>1591</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15066,7 +15092,7 @@
       <c r="J192" t="s">
         <v>1591</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15107,7 +15133,7 @@
       <c r="J193" t="s">
         <v>1591</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15148,7 +15174,7 @@
       <c r="J194" t="s">
         <v>1591</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15189,7 +15215,7 @@
       <c r="J195" t="s">
         <v>1591</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15207,7 +15233,7 @@
       <c r="R195" t="s">
         <v>1788</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15248,7 +15274,7 @@
       <c r="J196" t="s">
         <v>1591</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15266,7 +15292,7 @@
       <c r="R196" t="s">
         <v>1794</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15304,7 +15330,7 @@
       <c r="J197" t="s">
         <v>1591</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15345,7 +15371,7 @@
       <c r="J198" t="s">
         <v>1593</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15386,7 +15412,7 @@
       <c r="J199" t="s">
         <v>1592</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15427,7 +15453,7 @@
       <c r="J200" t="s">
         <v>1591</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15468,7 +15494,7 @@
       <c r="J201" t="s">
         <v>1591</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15509,7 +15535,7 @@
       <c r="J202" t="s">
         <v>1591</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15527,7 +15553,7 @@
       <c r="R202" t="s">
         <v>1779</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15562,7 +15588,7 @@
       <c r="J203" t="s">
         <v>1591</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15580,7 +15606,7 @@
       <c r="R203" t="s">
         <v>1787</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15615,7 +15641,7 @@
       <c r="J204" t="s">
         <v>1591</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15630,7 +15656,7 @@
       <c r="R204" t="s">
         <v>1798</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15668,7 +15694,7 @@
       <c r="J205" t="s">
         <v>1591</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15686,7 +15712,7 @@
       <c r="R205" t="s">
         <v>1799</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15724,7 +15750,7 @@
       <c r="J206" t="s">
         <v>1591</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15742,7 +15768,7 @@
       <c r="R206" t="s">
         <v>1767</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15777,7 +15803,7 @@
       <c r="J207" t="s">
         <v>1591</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15818,7 +15844,7 @@
       <c r="J208" t="s">
         <v>1591</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15859,7 +15885,7 @@
       <c r="J209" t="s">
         <v>1591</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15900,7 +15926,7 @@
       <c r="J210" t="s">
         <v>1591</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15941,7 +15967,7 @@
       <c r="J211" t="s">
         <v>1591</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15982,7 +16008,7 @@
       <c r="J212" t="s">
         <v>1591</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16023,7 +16049,7 @@
       <c r="J213" t="s">
         <v>1591</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16064,7 +16090,7 @@
       <c r="J214" t="s">
         <v>1591</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16082,7 +16108,7 @@
       <c r="R214" t="s">
         <v>1800</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -16117,7 +16143,7 @@
       <c r="J215" t="s">
         <v>1591</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16158,7 +16184,7 @@
       <c r="J216" t="s">
         <v>1591</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16199,7 +16225,7 @@
       <c r="J217" t="s">
         <v>1591</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16240,7 +16266,7 @@
       <c r="J218" t="s">
         <v>1591</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16281,7 +16307,7 @@
       <c r="J219" t="s">
         <v>1591</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16322,7 +16348,7 @@
       <c r="J220" t="s">
         <v>1591</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16363,7 +16389,7 @@
       <c r="J221" t="s">
         <v>1591</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16404,7 +16430,7 @@
       <c r="J222" t="s">
         <v>1591</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16445,7 +16471,7 @@
       <c r="J223" t="s">
         <v>1591</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16486,7 +16512,7 @@
       <c r="J224" t="s">
         <v>1591</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16527,7 +16553,7 @@
       <c r="J225" t="s">
         <v>1591</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16568,7 +16594,7 @@
       <c r="J226" t="s">
         <v>1591</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16609,7 +16635,7 @@
       <c r="J227" t="s">
         <v>1591</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16650,7 +16676,7 @@
       <c r="J228" t="s">
         <v>1591</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16691,7 +16717,7 @@
       <c r="J229" t="s">
         <v>1591</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16732,7 +16758,7 @@
       <c r="J230" t="s">
         <v>1591</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16773,7 +16799,7 @@
       <c r="J231" t="s">
         <v>1591</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16814,7 +16840,7 @@
       <c r="J232" t="s">
         <v>1591</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16855,7 +16881,7 @@
       <c r="J233" t="s">
         <v>1591</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16896,7 +16922,7 @@
       <c r="J234" t="s">
         <v>1591</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16937,7 +16963,7 @@
       <c r="J235" t="s">
         <v>1591</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16978,7 +17004,7 @@
       <c r="J236" t="s">
         <v>1591</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17019,7 +17045,7 @@
       <c r="J237" t="s">
         <v>1591</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17060,7 +17086,7 @@
       <c r="J238" t="s">
         <v>1591</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17101,7 +17127,7 @@
       <c r="J239" t="s">
         <v>1591</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17119,7 +17145,7 @@
       <c r="R239" t="s">
         <v>1794</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17157,7 +17183,7 @@
       <c r="J240" t="s">
         <v>1591</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17198,7 +17224,7 @@
       <c r="J241" t="s">
         <v>1591</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17239,7 +17265,7 @@
       <c r="J242" t="s">
         <v>1591</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17257,7 +17283,7 @@
       <c r="R242" t="s">
         <v>1787</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17292,7 +17318,7 @@
       <c r="J243" t="s">
         <v>1591</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17333,7 +17359,7 @@
       <c r="J244" t="s">
         <v>1591</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17374,7 +17400,7 @@
       <c r="J245" t="s">
         <v>1591</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17415,7 +17441,7 @@
       <c r="J246" t="s">
         <v>1591</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17433,7 +17459,7 @@
       <c r="R246" t="s">
         <v>1767</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17471,7 +17497,7 @@
       <c r="J247" t="s">
         <v>1591</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17512,7 +17538,7 @@
       <c r="J248" t="s">
         <v>1591</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17553,7 +17579,7 @@
       <c r="J249" t="s">
         <v>1591</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17594,7 +17620,7 @@
       <c r="J250" t="s">
         <v>1591</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17635,7 +17661,7 @@
       <c r="J251" t="s">
         <v>1591</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17676,7 +17702,7 @@
       <c r="J252" t="s">
         <v>1591</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17717,7 +17743,7 @@
       <c r="J253" t="s">
         <v>1591</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17735,7 +17761,7 @@
       <c r="R253" t="s">
         <v>1797</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17773,7 +17799,7 @@
       <c r="J254" t="s">
         <v>1591</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17814,7 +17840,7 @@
       <c r="J255" t="s">
         <v>1591</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17855,7 +17881,7 @@
       <c r="J256" t="s">
         <v>1591</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17864,7 +17890,7 @@
       <c r="M256" t="s">
         <v>1669</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17902,7 +17928,7 @@
       <c r="J257" t="s">
         <v>1591</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17911,7 +17937,7 @@
       <c r="M257" t="s">
         <v>1670</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17955,7 +17981,7 @@
       <c r="J258" t="s">
         <v>1591</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17973,7 +17999,7 @@
       <c r="R258" t="s">
         <v>1779</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18011,7 +18037,7 @@
       <c r="J259" t="s">
         <v>1591</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18029,7 +18055,7 @@
       <c r="R259" t="s">
         <v>1795</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18067,7 +18093,7 @@
       <c r="J260" t="s">
         <v>1591</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18076,7 +18102,7 @@
       <c r="M260" t="s">
         <v>1664</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18120,7 +18146,7 @@
       <c r="J261" t="s">
         <v>1591</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18138,7 +18164,7 @@
       <c r="R261" t="s">
         <v>1801</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18176,7 +18202,7 @@
       <c r="J262" t="s">
         <v>1591</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18194,7 +18220,7 @@
       <c r="R262" t="s">
         <v>1795</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18232,7 +18258,7 @@
       <c r="J263" t="s">
         <v>1591</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18241,7 +18267,7 @@
       <c r="M263" t="s">
         <v>1664</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18285,7 +18311,7 @@
       <c r="J264" t="s">
         <v>1591</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18326,7 +18352,7 @@
       <c r="J265" t="s">
         <v>1591</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18367,7 +18393,7 @@
       <c r="J266" t="s">
         <v>1591</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18408,7 +18434,7 @@
       <c r="J267" t="s">
         <v>1591</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18452,7 +18478,7 @@
       <c r="J268" t="s">
         <v>1591</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18493,7 +18519,7 @@
       <c r="J269" t="s">
         <v>1591</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18534,7 +18560,7 @@
       <c r="J270" t="s">
         <v>1591</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18575,7 +18601,7 @@
       <c r="J271" t="s">
         <v>1591</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18616,7 +18642,7 @@
       <c r="J272" t="s">
         <v>1591</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18634,7 +18660,7 @@
       <c r="R272" t="s">
         <v>1802</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18672,7 +18698,7 @@
       <c r="J273" t="s">
         <v>1591</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18716,7 +18742,7 @@
       <c r="J274" t="s">
         <v>1591</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18757,7 +18783,7 @@
       <c r="J275" t="s">
         <v>1591</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18798,7 +18824,7 @@
       <c r="J276" t="s">
         <v>1591</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18839,7 +18865,7 @@
       <c r="J277" t="s">
         <v>1591</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18880,7 +18906,7 @@
       <c r="J278" t="s">
         <v>1591</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18921,7 +18947,7 @@
       <c r="J279" t="s">
         <v>1591</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18962,7 +18988,7 @@
       <c r="J280" t="s">
         <v>1591</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19003,7 +19029,7 @@
       <c r="J281" t="s">
         <v>1591</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19044,7 +19070,7 @@
       <c r="J282" t="s">
         <v>1591</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19085,7 +19111,7 @@
       <c r="J283" t="s">
         <v>1591</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19126,7 +19152,7 @@
       <c r="J284" t="s">
         <v>1591</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19167,7 +19193,7 @@
       <c r="J285" t="s">
         <v>1591</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19208,7 +19234,7 @@
       <c r="J286" t="s">
         <v>1591</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19249,7 +19275,7 @@
       <c r="J287" t="s">
         <v>1591</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19290,7 +19316,7 @@
       <c r="J288" t="s">
         <v>1591</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19331,7 +19357,7 @@
       <c r="J289" t="s">
         <v>1591</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19372,7 +19398,7 @@
       <c r="J290" t="s">
         <v>1591</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19413,7 +19439,7 @@
       <c r="J291" t="s">
         <v>1591</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19454,7 +19480,7 @@
       <c r="J292" t="s">
         <v>1591</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19495,7 +19521,7 @@
       <c r="J293" t="s">
         <v>1591</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19536,7 +19562,7 @@
       <c r="J294" t="s">
         <v>1591</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19577,7 +19603,7 @@
       <c r="J295" t="s">
         <v>1591</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19595,7 +19621,7 @@
       <c r="R295" t="s">
         <v>1803</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19636,7 +19662,7 @@
       <c r="J296" t="s">
         <v>1591</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19654,7 +19680,7 @@
       <c r="R296" t="s">
         <v>1779</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19692,7 +19718,7 @@
       <c r="J297" t="s">
         <v>1591</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19733,7 +19759,7 @@
       <c r="J298" t="s">
         <v>1591</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19774,7 +19800,7 @@
       <c r="J299" t="s">
         <v>1592</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19815,7 +19841,7 @@
       <c r="J300" t="s">
         <v>1591</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19856,7 +19882,7 @@
       <c r="J301" t="s">
         <v>1591</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20694,7 +20720,7 @@
       <c r="R321" t="s">
         <v>1765</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -20917,7 +20943,7 @@
       <c r="R326" t="s">
         <v>1804</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21752,7 +21778,7 @@
       <c r="R346" t="s">
         <v>1805</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (02/10/2026 09:58)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5669,8 +5669,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5686,7 +5694,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5694,12 +5702,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5999,73 +6025,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6100,7 +6126,7 @@
       <c r="J2" t="s">
         <v>1611</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6144,7 +6170,7 @@
       <c r="J3" t="s">
         <v>1611</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6188,7 +6214,7 @@
       <c r="J4" t="s">
         <v>1611</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6206,7 +6232,7 @@
       <c r="R4" t="s">
         <v>1784</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6244,7 +6270,7 @@
       <c r="J5" t="s">
         <v>1612</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6294,7 +6320,7 @@
       <c r="J6" t="s">
         <v>1611</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6341,7 +6367,7 @@
       <c r="J7" t="s">
         <v>1611</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6388,7 +6414,7 @@
       <c r="J8" t="s">
         <v>1611</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6435,7 +6461,7 @@
       <c r="J9" t="s">
         <v>1611</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6482,7 +6508,7 @@
       <c r="J10" t="s">
         <v>1611</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6529,7 +6555,7 @@
       <c r="J11" t="s">
         <v>1611</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6576,7 +6602,7 @@
       <c r="J12" t="s">
         <v>1611</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6620,7 +6646,7 @@
       <c r="J13" t="s">
         <v>1611</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6638,7 +6664,7 @@
       <c r="R13" t="s">
         <v>1785</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6676,7 +6702,7 @@
       <c r="J14" t="s">
         <v>1611</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6694,7 +6720,7 @@
       <c r="R14" t="s">
         <v>1786</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6735,7 +6761,7 @@
       <c r="J15" t="s">
         <v>1611</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6753,7 +6779,7 @@
       <c r="R15" t="s">
         <v>1786</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6794,7 +6820,7 @@
       <c r="J16" t="s">
         <v>1611</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6838,7 +6864,7 @@
       <c r="J17" t="s">
         <v>1611</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6882,7 +6908,7 @@
       <c r="J18" t="s">
         <v>1611</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6900,7 +6926,7 @@
       <c r="R18" t="s">
         <v>1787</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6941,7 +6967,7 @@
       <c r="J19" t="s">
         <v>1611</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6985,7 +7011,7 @@
       <c r="J20" t="s">
         <v>1611</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7029,7 +7055,7 @@
       <c r="J21" t="s">
         <v>1611</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7047,7 +7073,7 @@
       <c r="R21" t="s">
         <v>1786</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7088,7 +7114,7 @@
       <c r="J22" t="s">
         <v>1611</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7106,7 +7132,7 @@
       <c r="R22" t="s">
         <v>1788</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7147,7 +7173,7 @@
       <c r="J23" t="s">
         <v>1611</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7165,7 +7191,7 @@
       <c r="R23" t="s">
         <v>1789</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7206,7 +7232,7 @@
       <c r="J24" t="s">
         <v>1611</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7250,7 +7276,7 @@
       <c r="J25" t="s">
         <v>1611</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7291,7 +7317,7 @@
       <c r="J26" t="s">
         <v>1613</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7309,7 +7335,7 @@
       <c r="R26" t="s">
         <v>1790</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7347,7 +7373,7 @@
       <c r="J27" t="s">
         <v>1611</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7365,7 +7391,7 @@
       <c r="R27" t="s">
         <v>1791</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7406,7 +7432,7 @@
       <c r="J28" t="s">
         <v>1611</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7450,7 +7476,7 @@
       <c r="J29" t="s">
         <v>1611</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7494,7 +7520,7 @@
       <c r="J30" t="s">
         <v>1611</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7538,7 +7564,7 @@
       <c r="J31" t="s">
         <v>1611</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7556,7 +7582,7 @@
       <c r="R31" t="s">
         <v>1792</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7597,7 +7623,7 @@
       <c r="J32" t="s">
         <v>1611</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7641,7 +7667,7 @@
       <c r="J33" t="s">
         <v>1611</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7659,7 +7685,7 @@
       <c r="R33" t="s">
         <v>1793</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7700,7 +7726,7 @@
       <c r="J34" t="s">
         <v>1611</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7744,7 +7770,7 @@
       <c r="J35" t="s">
         <v>1611</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7762,7 +7788,7 @@
       <c r="R35" t="s">
         <v>1794</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7803,7 +7829,7 @@
       <c r="J36" t="s">
         <v>1611</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7821,7 +7847,7 @@
       <c r="R36" t="s">
         <v>1794</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7862,7 +7888,7 @@
       <c r="J37" t="s">
         <v>1611</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7880,7 +7906,7 @@
       <c r="R37" t="s">
         <v>1794</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7921,7 +7947,7 @@
       <c r="J38" t="s">
         <v>1611</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7939,7 +7965,7 @@
       <c r="R38" t="s">
         <v>1794</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7980,7 +8006,7 @@
       <c r="J39" t="s">
         <v>1611</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7998,7 +8024,7 @@
       <c r="R39" t="s">
         <v>1794</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8039,7 +8065,7 @@
       <c r="J40" t="s">
         <v>1611</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8057,7 +8083,7 @@
       <c r="R40" t="s">
         <v>1795</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8098,7 +8124,7 @@
       <c r="J41" t="s">
         <v>1611</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8116,7 +8142,7 @@
       <c r="R41" t="s">
         <v>1786</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8157,7 +8183,7 @@
       <c r="J42" t="s">
         <v>1611</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8175,7 +8201,7 @@
       <c r="R42" t="s">
         <v>1794</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8216,7 +8242,7 @@
       <c r="J43" t="s">
         <v>1611</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8260,7 +8286,7 @@
       <c r="J44" t="s">
         <v>1611</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8278,7 +8304,7 @@
       <c r="R44" t="s">
         <v>1796</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8319,7 +8345,7 @@
       <c r="J45" t="s">
         <v>1611</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8337,7 +8363,7 @@
       <c r="R45" t="s">
         <v>1797</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8375,7 +8401,7 @@
       <c r="J46" t="s">
         <v>1611</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8419,7 +8445,7 @@
       <c r="J47" t="s">
         <v>1611</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8437,7 +8463,7 @@
       <c r="R47" t="s">
         <v>1798</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8478,7 +8504,7 @@
       <c r="J48" t="s">
         <v>1611</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8522,7 +8548,7 @@
       <c r="J49" t="s">
         <v>1611</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8566,7 +8592,7 @@
       <c r="J50" t="s">
         <v>1611</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8610,7 +8636,7 @@
       <c r="J51" t="s">
         <v>1611</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8657,7 +8683,7 @@
       <c r="J52" t="s">
         <v>1611</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8701,7 +8727,7 @@
       <c r="J53" t="s">
         <v>1611</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8745,7 +8771,7 @@
       <c r="J54" t="s">
         <v>1611</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8789,7 +8815,7 @@
       <c r="J55" t="s">
         <v>1611</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8839,7 +8865,7 @@
       <c r="J56" t="s">
         <v>1611</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8892,7 +8918,7 @@
       <c r="J57" t="s">
         <v>1611</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8942,7 +8968,7 @@
       <c r="J58" t="s">
         <v>1611</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8992,7 +9018,7 @@
       <c r="J59" t="s">
         <v>1611</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9010,7 +9036,7 @@
       <c r="R59" t="s">
         <v>1799</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9051,7 +9077,7 @@
       <c r="J60" t="s">
         <v>1611</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9095,7 +9121,7 @@
       <c r="J61" t="s">
         <v>1611</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9139,7 +9165,7 @@
       <c r="J62" t="s">
         <v>1611</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9183,7 +9209,7 @@
       <c r="J63" t="s">
         <v>1611</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9227,7 +9253,7 @@
       <c r="J64" t="s">
         <v>1611</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9271,7 +9297,7 @@
       <c r="J65" t="s">
         <v>1611</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9318,7 +9344,7 @@
       <c r="J66" t="s">
         <v>1611</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9336,7 +9362,7 @@
       <c r="R66" t="s">
         <v>1800</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9374,7 +9400,7 @@
       <c r="J67" t="s">
         <v>1611</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9418,7 +9444,7 @@
       <c r="J68" t="s">
         <v>1611</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9433,7 +9459,7 @@
       <c r="O68" t="s">
         <v>1704</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9477,7 +9503,7 @@
       <c r="J69" t="s">
         <v>1613</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9521,7 +9547,7 @@
       <c r="J70" t="s">
         <v>1611</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9565,7 +9591,7 @@
       <c r="J71" t="s">
         <v>1611</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9609,7 +9635,7 @@
       <c r="J72" t="s">
         <v>1611</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9653,7 +9679,7 @@
       <c r="J73" t="s">
         <v>1611</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9697,7 +9723,7 @@
       <c r="J74" t="s">
         <v>1611</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9741,7 +9767,7 @@
       <c r="J75" t="s">
         <v>1611</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9785,7 +9811,7 @@
       <c r="J76" t="s">
         <v>1611</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9803,7 +9829,7 @@
       <c r="R76" t="s">
         <v>1801</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9841,7 +9867,7 @@
       <c r="J77" t="s">
         <v>1611</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9859,7 +9885,7 @@
       <c r="R77" t="s">
         <v>1801</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9897,7 +9923,7 @@
       <c r="J78" t="s">
         <v>1611</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9915,7 +9941,7 @@
       <c r="R78" t="s">
         <v>1801</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9953,7 +9979,7 @@
       <c r="J79" t="s">
         <v>1611</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9971,7 +9997,7 @@
       <c r="R79" t="s">
         <v>1801</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10009,7 +10035,7 @@
       <c r="J80" t="s">
         <v>1611</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10053,7 +10079,7 @@
       <c r="J81" t="s">
         <v>1611</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10097,7 +10123,7 @@
       <c r="J82" t="s">
         <v>1611</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10141,7 +10167,7 @@
       <c r="J83" t="s">
         <v>1611</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10185,7 +10211,7 @@
       <c r="J84" t="s">
         <v>1611</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10229,7 +10255,7 @@
       <c r="J85" t="s">
         <v>1611</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10247,7 +10273,7 @@
       <c r="R85" t="s">
         <v>1802</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10285,7 +10311,7 @@
       <c r="J86" t="s">
         <v>1611</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10329,7 +10355,7 @@
       <c r="J87" t="s">
         <v>1611</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10347,7 +10373,7 @@
       <c r="R87" t="s">
         <v>1803</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10385,7 +10411,7 @@
       <c r="J88" t="s">
         <v>1611</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10429,7 +10455,7 @@
       <c r="J89" t="s">
         <v>1611</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10447,7 +10473,7 @@
       <c r="R89" t="s">
         <v>1804</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10482,7 +10508,7 @@
       <c r="J90" t="s">
         <v>1611</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10500,7 +10526,7 @@
       <c r="R90" t="s">
         <v>1805</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10535,7 +10561,7 @@
       <c r="J91" t="s">
         <v>1611</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10553,7 +10579,7 @@
       <c r="R91" t="s">
         <v>1789</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10591,7 +10617,7 @@
       <c r="J92" t="s">
         <v>1611</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10612,7 +10638,7 @@
       <c r="R92" t="s">
         <v>1789</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10653,7 +10679,7 @@
       <c r="J93" t="s">
         <v>1611</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10694,7 +10720,7 @@
       <c r="J94" t="s">
         <v>1611</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10738,7 +10764,7 @@
       <c r="J95" t="s">
         <v>1611</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10782,7 +10808,7 @@
       <c r="J96" t="s">
         <v>1611</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10800,7 +10826,7 @@
       <c r="R96" t="s">
         <v>1806</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10841,7 +10867,7 @@
       <c r="J97" t="s">
         <v>1611</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10856,7 +10882,7 @@
       <c r="R97" t="s">
         <v>1806</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10897,7 +10923,7 @@
       <c r="J98" t="s">
         <v>1611</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10915,7 +10941,7 @@
       <c r="R98" t="s">
         <v>1807</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10953,7 +10979,7 @@
       <c r="J99" t="s">
         <v>1611</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10971,7 +10997,7 @@
       <c r="R99" t="s">
         <v>1808</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11009,7 +11035,7 @@
       <c r="J100" t="s">
         <v>1611</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11050,7 +11076,7 @@
       <c r="J101" t="s">
         <v>1611</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11091,7 +11117,7 @@
       <c r="J102" t="s">
         <v>1611</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11132,7 +11158,7 @@
       <c r="J103" t="s">
         <v>1611</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11173,7 +11199,7 @@
       <c r="J104" t="s">
         <v>1611</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11214,7 +11240,7 @@
       <c r="J105" t="s">
         <v>1611</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11255,7 +11281,7 @@
       <c r="J106" t="s">
         <v>1611</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11296,7 +11322,7 @@
       <c r="J107" t="s">
         <v>1611</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11337,7 +11363,7 @@
       <c r="J108" t="s">
         <v>1611</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11378,7 +11404,7 @@
       <c r="J109" t="s">
         <v>1611</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11431,7 +11457,7 @@
       <c r="J110" t="s">
         <v>1611</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11487,7 +11513,7 @@
       <c r="J111" t="s">
         <v>1611</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11505,7 +11531,7 @@
       <c r="R111" t="s">
         <v>1810</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11543,7 +11569,7 @@
       <c r="J112" t="s">
         <v>1611</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11602,7 +11628,7 @@
       <c r="J113" t="s">
         <v>1611</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11646,7 +11672,7 @@
       <c r="J114" t="s">
         <v>1611</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11690,7 +11716,7 @@
       <c r="J115" t="s">
         <v>1611</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11708,7 +11734,7 @@
       <c r="R115" t="s">
         <v>1812</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11749,7 +11775,7 @@
       <c r="J116" t="s">
         <v>1611</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11808,7 +11834,7 @@
       <c r="J117" t="s">
         <v>1611</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11852,7 +11878,7 @@
       <c r="J118" t="s">
         <v>1611</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11899,7 +11925,7 @@
       <c r="J119" t="s">
         <v>1611</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11940,7 +11966,7 @@
       <c r="J120" t="s">
         <v>1611</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11984,7 +12010,7 @@
       <c r="J121" t="s">
         <v>1611</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12031,7 +12057,7 @@
       <c r="J122" t="s">
         <v>1611</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12081,7 +12107,7 @@
       <c r="J123" t="s">
         <v>1611</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12125,7 +12151,7 @@
       <c r="J124" t="s">
         <v>1611</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12169,7 +12195,7 @@
       <c r="J125" t="s">
         <v>1611</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12187,7 +12213,7 @@
       <c r="R125" t="s">
         <v>1814</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12222,7 +12248,7 @@
       <c r="J126" t="s">
         <v>1611</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12240,7 +12266,7 @@
       <c r="R126" t="s">
         <v>1815</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12278,7 +12304,7 @@
       <c r="J127" t="s">
         <v>1611</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12334,7 +12360,7 @@
       <c r="J128" t="s">
         <v>1611</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12375,7 +12401,7 @@
       <c r="J129" t="s">
         <v>1611</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12416,7 +12442,7 @@
       <c r="J130" t="s">
         <v>1611</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12457,7 +12483,7 @@
       <c r="J131" t="s">
         <v>1611</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12501,7 +12527,7 @@
       <c r="J132" t="s">
         <v>1611</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12542,7 +12568,7 @@
       <c r="J133" t="s">
         <v>1611</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12560,7 +12586,7 @@
       <c r="R133" t="s">
         <v>1801</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12598,7 +12624,7 @@
       <c r="J134" t="s">
         <v>1611</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12616,7 +12642,7 @@
       <c r="R134" t="s">
         <v>1801</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12651,7 +12677,7 @@
       <c r="J135" t="s">
         <v>1611</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12692,7 +12718,7 @@
       <c r="J136" t="s">
         <v>1611</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12733,7 +12759,7 @@
       <c r="J137" t="s">
         <v>1611</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12774,7 +12800,7 @@
       <c r="J138" t="s">
         <v>1611</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12815,7 +12841,7 @@
       <c r="J139" t="s">
         <v>1611</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12862,7 +12888,7 @@
       <c r="J140" t="s">
         <v>1611</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12903,7 +12929,7 @@
       <c r="J141" t="s">
         <v>1611</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12944,7 +12970,7 @@
       <c r="J142" t="s">
         <v>1611</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12988,7 +13014,7 @@
       <c r="J143" t="s">
         <v>1611</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13006,7 +13032,7 @@
       <c r="R143" t="s">
         <v>1801</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13041,7 +13067,7 @@
       <c r="J144" t="s">
         <v>1611</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13059,7 +13085,7 @@
       <c r="R144" t="s">
         <v>1801</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13097,7 +13123,7 @@
       <c r="J145" t="s">
         <v>1611</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13115,7 +13141,7 @@
       <c r="R145" t="s">
         <v>1801</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13150,7 +13176,7 @@
       <c r="J146" t="s">
         <v>1611</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13168,7 +13194,7 @@
       <c r="R146" t="s">
         <v>1809</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13203,7 +13229,7 @@
       <c r="J147" t="s">
         <v>1611</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13221,7 +13247,7 @@
       <c r="R147" t="s">
         <v>1816</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13256,7 +13282,7 @@
       <c r="J148" t="s">
         <v>1611</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13297,7 +13323,7 @@
       <c r="J149" t="s">
         <v>1611</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13315,7 +13341,7 @@
       <c r="R149" t="s">
         <v>1801</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13350,7 +13376,7 @@
       <c r="J150" t="s">
         <v>1611</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13368,7 +13394,7 @@
       <c r="R150" t="s">
         <v>1801</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13406,7 +13432,7 @@
       <c r="J151" t="s">
         <v>1611</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13424,7 +13450,7 @@
       <c r="R151" t="s">
         <v>1817</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13459,7 +13485,7 @@
       <c r="J152" t="s">
         <v>1611</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13477,7 +13503,7 @@
       <c r="R152" t="s">
         <v>1818</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13512,7 +13538,7 @@
       <c r="J153" t="s">
         <v>1611</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13521,7 +13547,7 @@
       <c r="M153" t="s">
         <v>1695</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13562,7 +13588,7 @@
       <c r="J154" t="s">
         <v>1611</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13603,7 +13629,7 @@
       <c r="J155" t="s">
         <v>1611</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13644,7 +13670,7 @@
       <c r="J156" t="s">
         <v>1611</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13685,7 +13711,7 @@
       <c r="J157" t="s">
         <v>1611</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13726,7 +13752,7 @@
       <c r="J158" t="s">
         <v>1611</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13767,7 +13793,7 @@
       <c r="J159" t="s">
         <v>1611</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13808,7 +13834,7 @@
       <c r="J160" t="s">
         <v>1611</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13849,7 +13875,7 @@
       <c r="J161" t="s">
         <v>1611</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13890,7 +13916,7 @@
       <c r="J162" t="s">
         <v>1611</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13908,7 +13934,7 @@
       <c r="R162" t="s">
         <v>1804</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13943,7 +13969,7 @@
       <c r="J163" t="s">
         <v>1611</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13961,7 +13987,7 @@
       <c r="R163" t="s">
         <v>1801</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13996,7 +14022,7 @@
       <c r="J164" t="s">
         <v>1611</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14040,7 +14066,7 @@
       <c r="J165" t="s">
         <v>1611</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14081,7 +14107,7 @@
       <c r="J166" t="s">
         <v>1611</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14099,7 +14125,7 @@
       <c r="R166" t="s">
         <v>1819</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14134,7 +14160,7 @@
       <c r="J167" t="s">
         <v>1611</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14178,7 +14204,7 @@
       <c r="J168" t="s">
         <v>1611</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14222,7 +14248,7 @@
       <c r="J169" t="s">
         <v>1611</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14263,7 +14289,7 @@
       <c r="J170" t="s">
         <v>1611</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14304,7 +14330,7 @@
       <c r="J171" t="s">
         <v>1611</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14345,7 +14371,7 @@
       <c r="J172" t="s">
         <v>1611</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14386,7 +14412,7 @@
       <c r="J173" t="s">
         <v>1611</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14427,7 +14453,7 @@
       <c r="J174" t="s">
         <v>1611</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14468,7 +14494,7 @@
       <c r="J175" t="s">
         <v>1611</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14509,7 +14535,7 @@
       <c r="J176" t="s">
         <v>1611</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14550,7 +14576,7 @@
       <c r="J177" t="s">
         <v>1611</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14591,7 +14617,7 @@
       <c r="J178" t="s">
         <v>1611</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14609,7 +14635,7 @@
       <c r="R178" t="s">
         <v>1817</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14647,7 +14673,7 @@
       <c r="J179" t="s">
         <v>1611</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14656,7 +14682,7 @@
       <c r="M179" t="s">
         <v>1692</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14697,7 +14723,7 @@
       <c r="J180" t="s">
         <v>1611</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14738,7 +14764,7 @@
       <c r="J181" t="s">
         <v>1611</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14756,7 +14782,7 @@
       <c r="R181" t="s">
         <v>1801</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14791,7 +14817,7 @@
       <c r="J182" t="s">
         <v>1611</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14832,7 +14858,7 @@
       <c r="J183" t="s">
         <v>1611</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14873,7 +14899,7 @@
       <c r="J184" t="s">
         <v>1611</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14914,7 +14940,7 @@
       <c r="J185" t="s">
         <v>1611</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14955,7 +14981,7 @@
       <c r="J186" t="s">
         <v>1611</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14996,7 +15022,7 @@
       <c r="J187" t="s">
         <v>1611</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15037,7 +15063,7 @@
       <c r="J188" t="s">
         <v>1611</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15078,7 +15104,7 @@
       <c r="J189" t="s">
         <v>1611</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15119,7 +15145,7 @@
       <c r="J190" t="s">
         <v>1611</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15160,7 +15186,7 @@
       <c r="J191" t="s">
         <v>1611</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15201,7 +15227,7 @@
       <c r="J192" t="s">
         <v>1611</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15242,7 +15268,7 @@
       <c r="J193" t="s">
         <v>1611</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15283,7 +15309,7 @@
       <c r="J194" t="s">
         <v>1611</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15324,7 +15350,7 @@
       <c r="J195" t="s">
         <v>1611</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15342,7 +15368,7 @@
       <c r="R195" t="s">
         <v>1810</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15383,7 +15409,7 @@
       <c r="J196" t="s">
         <v>1611</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15401,7 +15427,7 @@
       <c r="R196" t="s">
         <v>1816</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15439,7 +15465,7 @@
       <c r="J197" t="s">
         <v>1611</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15480,7 +15506,7 @@
       <c r="J198" t="s">
         <v>1613</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15521,7 +15547,7 @@
       <c r="J199" t="s">
         <v>1612</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15562,7 +15588,7 @@
       <c r="J200" t="s">
         <v>1611</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15603,7 +15629,7 @@
       <c r="J201" t="s">
         <v>1611</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15644,7 +15670,7 @@
       <c r="J202" t="s">
         <v>1611</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15662,7 +15688,7 @@
       <c r="R202" t="s">
         <v>1801</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15700,7 +15726,7 @@
       <c r="J203" t="s">
         <v>1611</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15718,7 +15744,7 @@
       <c r="R203" t="s">
         <v>1809</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15753,7 +15779,7 @@
       <c r="J204" t="s">
         <v>1611</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15768,7 +15794,7 @@
       <c r="R204" t="s">
         <v>1820</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15806,7 +15832,7 @@
       <c r="J205" t="s">
         <v>1611</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15824,7 +15850,7 @@
       <c r="R205" t="s">
         <v>1821</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15862,7 +15888,7 @@
       <c r="J206" t="s">
         <v>1611</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15880,7 +15906,7 @@
       <c r="R206" t="s">
         <v>1789</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15915,7 +15941,7 @@
       <c r="J207" t="s">
         <v>1611</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15956,7 +15982,7 @@
       <c r="J208" t="s">
         <v>1611</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15997,7 +16023,7 @@
       <c r="J209" t="s">
         <v>1611</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16038,7 +16064,7 @@
       <c r="J210" t="s">
         <v>1611</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16079,7 +16105,7 @@
       <c r="J211" t="s">
         <v>1611</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16120,7 +16146,7 @@
       <c r="J212" t="s">
         <v>1611</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16161,7 +16187,7 @@
       <c r="J213" t="s">
         <v>1611</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16202,7 +16228,7 @@
       <c r="J214" t="s">
         <v>1611</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16220,7 +16246,7 @@
       <c r="R214" t="s">
         <v>1822</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16258,7 +16284,7 @@
       <c r="J215" t="s">
         <v>1611</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16299,7 +16325,7 @@
       <c r="J216" t="s">
         <v>1611</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16340,7 +16366,7 @@
       <c r="J217" t="s">
         <v>1611</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16381,7 +16407,7 @@
       <c r="J218" t="s">
         <v>1611</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16422,7 +16448,7 @@
       <c r="J219" t="s">
         <v>1611</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16463,7 +16489,7 @@
       <c r="J220" t="s">
         <v>1611</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16504,7 +16530,7 @@
       <c r="J221" t="s">
         <v>1611</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16545,7 +16571,7 @@
       <c r="J222" t="s">
         <v>1611</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16586,7 +16612,7 @@
       <c r="J223" t="s">
         <v>1611</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16627,7 +16653,7 @@
       <c r="J224" t="s">
         <v>1611</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16668,7 +16694,7 @@
       <c r="J225" t="s">
         <v>1611</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16709,7 +16735,7 @@
       <c r="J226" t="s">
         <v>1611</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16750,7 +16776,7 @@
       <c r="J227" t="s">
         <v>1611</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16791,7 +16817,7 @@
       <c r="J228" t="s">
         <v>1611</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16832,7 +16858,7 @@
       <c r="J229" t="s">
         <v>1611</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16873,7 +16899,7 @@
       <c r="J230" t="s">
         <v>1611</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16914,7 +16940,7 @@
       <c r="J231" t="s">
         <v>1611</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16955,7 +16981,7 @@
       <c r="J232" t="s">
         <v>1611</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16996,7 +17022,7 @@
       <c r="J233" t="s">
         <v>1611</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17037,7 +17063,7 @@
       <c r="J234" t="s">
         <v>1611</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17078,7 +17104,7 @@
       <c r="J235" t="s">
         <v>1611</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17119,7 +17145,7 @@
       <c r="J236" t="s">
         <v>1611</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17160,7 +17186,7 @@
       <c r="J237" t="s">
         <v>1611</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17201,7 +17227,7 @@
       <c r="J238" t="s">
         <v>1611</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17242,7 +17268,7 @@
       <c r="J239" t="s">
         <v>1611</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17260,7 +17286,7 @@
       <c r="R239" t="s">
         <v>1816</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17298,7 +17324,7 @@
       <c r="J240" t="s">
         <v>1611</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17339,7 +17365,7 @@
       <c r="J241" t="s">
         <v>1611</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17380,7 +17406,7 @@
       <c r="J242" t="s">
         <v>1611</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17398,7 +17424,7 @@
       <c r="R242" t="s">
         <v>1809</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17433,7 +17459,7 @@
       <c r="J243" t="s">
         <v>1611</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17474,7 +17500,7 @@
       <c r="J244" t="s">
         <v>1611</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17515,7 +17541,7 @@
       <c r="J245" t="s">
         <v>1611</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17556,7 +17582,7 @@
       <c r="J246" t="s">
         <v>1611</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17574,7 +17600,7 @@
       <c r="R246" t="s">
         <v>1789</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17612,7 +17638,7 @@
       <c r="J247" t="s">
         <v>1611</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17653,7 +17679,7 @@
       <c r="J248" t="s">
         <v>1611</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17694,7 +17720,7 @@
       <c r="J249" t="s">
         <v>1611</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17735,7 +17761,7 @@
       <c r="J250" t="s">
         <v>1611</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17776,7 +17802,7 @@
       <c r="J251" t="s">
         <v>1611</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17817,7 +17843,7 @@
       <c r="J252" t="s">
         <v>1611</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17858,7 +17884,7 @@
       <c r="J253" t="s">
         <v>1611</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17876,7 +17902,7 @@
       <c r="R253" t="s">
         <v>1819</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -17917,7 +17943,7 @@
       <c r="J254" t="s">
         <v>1611</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17958,7 +17984,7 @@
       <c r="J255" t="s">
         <v>1611</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17999,7 +18025,7 @@
       <c r="J256" t="s">
         <v>1611</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18008,7 +18034,7 @@
       <c r="M256" t="s">
         <v>1691</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18046,7 +18072,7 @@
       <c r="J257" t="s">
         <v>1611</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18055,7 +18081,7 @@
       <c r="M257" t="s">
         <v>1692</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18099,7 +18125,7 @@
       <c r="J258" t="s">
         <v>1611</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18117,7 +18143,7 @@
       <c r="R258" t="s">
         <v>1801</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18155,7 +18181,7 @@
       <c r="J259" t="s">
         <v>1611</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18173,7 +18199,7 @@
       <c r="R259" t="s">
         <v>1817</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18211,7 +18237,7 @@
       <c r="J260" t="s">
         <v>1611</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18220,7 +18246,7 @@
       <c r="M260" t="s">
         <v>1686</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18264,7 +18290,7 @@
       <c r="J261" t="s">
         <v>1611</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18282,7 +18308,7 @@
       <c r="R261" t="s">
         <v>1823</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18320,7 +18346,7 @@
       <c r="J262" t="s">
         <v>1611</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18338,7 +18364,7 @@
       <c r="R262" t="s">
         <v>1817</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18376,7 +18402,7 @@
       <c r="J263" t="s">
         <v>1611</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18385,7 +18411,7 @@
       <c r="M263" t="s">
         <v>1686</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18429,7 +18455,7 @@
       <c r="J264" t="s">
         <v>1611</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18470,7 +18496,7 @@
       <c r="J265" t="s">
         <v>1611</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18511,7 +18537,7 @@
       <c r="J266" t="s">
         <v>1611</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18552,7 +18578,7 @@
       <c r="J267" t="s">
         <v>1611</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18596,7 +18622,7 @@
       <c r="J268" t="s">
         <v>1611</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18637,7 +18663,7 @@
       <c r="J269" t="s">
         <v>1611</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18678,7 +18704,7 @@
       <c r="J270" t="s">
         <v>1611</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18719,7 +18745,7 @@
       <c r="J271" t="s">
         <v>1611</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18760,7 +18786,7 @@
       <c r="J272" t="s">
         <v>1611</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18778,7 +18804,7 @@
       <c r="R272" t="s">
         <v>1824</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18819,7 +18845,7 @@
       <c r="J273" t="s">
         <v>1611</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18863,7 +18889,7 @@
       <c r="J274" t="s">
         <v>1611</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18904,7 +18930,7 @@
       <c r="J275" t="s">
         <v>1611</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18945,7 +18971,7 @@
       <c r="J276" t="s">
         <v>1611</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18986,7 +19012,7 @@
       <c r="J277" t="s">
         <v>1611</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19027,7 +19053,7 @@
       <c r="J278" t="s">
         <v>1611</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19068,7 +19094,7 @@
       <c r="J279" t="s">
         <v>1611</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19109,7 +19135,7 @@
       <c r="J280" t="s">
         <v>1611</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19150,7 +19176,7 @@
       <c r="J281" t="s">
         <v>1611</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19191,7 +19217,7 @@
       <c r="J282" t="s">
         <v>1611</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19232,7 +19258,7 @@
       <c r="J283" t="s">
         <v>1611</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19273,7 +19299,7 @@
       <c r="J284" t="s">
         <v>1611</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19314,7 +19340,7 @@
       <c r="J285" t="s">
         <v>1611</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19355,7 +19381,7 @@
       <c r="J286" t="s">
         <v>1611</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19396,7 +19422,7 @@
       <c r="J287" t="s">
         <v>1611</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19437,7 +19463,7 @@
       <c r="J288" t="s">
         <v>1611</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19478,7 +19504,7 @@
       <c r="J289" t="s">
         <v>1611</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19519,7 +19545,7 @@
       <c r="J290" t="s">
         <v>1611</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19560,7 +19586,7 @@
       <c r="J291" t="s">
         <v>1611</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19601,7 +19627,7 @@
       <c r="J292" t="s">
         <v>1611</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19642,7 +19668,7 @@
       <c r="J293" t="s">
         <v>1611</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19683,7 +19709,7 @@
       <c r="J294" t="s">
         <v>1611</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19724,7 +19750,7 @@
       <c r="J295" t="s">
         <v>1611</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19742,7 +19768,7 @@
       <c r="R295" t="s">
         <v>1825</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19783,7 +19809,7 @@
       <c r="J296" t="s">
         <v>1611</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19801,7 +19827,7 @@
       <c r="R296" t="s">
         <v>1801</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19839,7 +19865,7 @@
       <c r="J297" t="s">
         <v>1611</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19880,7 +19906,7 @@
       <c r="J298" t="s">
         <v>1611</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19921,7 +19947,7 @@
       <c r="J299" t="s">
         <v>1612</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19962,7 +19988,7 @@
       <c r="J300" t="s">
         <v>1611</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20003,7 +20029,7 @@
       <c r="J301" t="s">
         <v>1611</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20841,7 +20867,7 @@
       <c r="R321" t="s">
         <v>1787</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21064,7 +21090,7 @@
       <c r="R326" t="s">
         <v>1826</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21899,7 +21925,7 @@
       <c r="R346" t="s">
         <v>1827</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (05/10/2026 08:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5687,8 +5687,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5704,7 +5712,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5712,12 +5720,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6017,73 +6043,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6118,7 +6144,7 @@
       <c r="J2" t="s">
         <v>1616</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6162,7 +6188,7 @@
       <c r="J3" t="s">
         <v>1616</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6206,7 +6232,7 @@
       <c r="J4" t="s">
         <v>1616</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6224,7 +6250,7 @@
       <c r="R4" t="s">
         <v>1790</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6262,7 +6288,7 @@
       <c r="J5" t="s">
         <v>1617</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6312,7 +6338,7 @@
       <c r="J6" t="s">
         <v>1616</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6359,7 +6385,7 @@
       <c r="J7" t="s">
         <v>1616</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6406,7 +6432,7 @@
       <c r="J8" t="s">
         <v>1616</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6453,7 +6479,7 @@
       <c r="J9" t="s">
         <v>1616</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6500,7 +6526,7 @@
       <c r="J10" t="s">
         <v>1616</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6547,7 +6573,7 @@
       <c r="J11" t="s">
         <v>1616</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6594,7 +6620,7 @@
       <c r="J12" t="s">
         <v>1616</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6638,7 +6664,7 @@
       <c r="J13" t="s">
         <v>1616</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6656,7 +6682,7 @@
       <c r="R13" t="s">
         <v>1791</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6694,7 +6720,7 @@
       <c r="J14" t="s">
         <v>1616</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6712,7 +6738,7 @@
       <c r="R14" t="s">
         <v>1792</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6753,7 +6779,7 @@
       <c r="J15" t="s">
         <v>1616</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6771,7 +6797,7 @@
       <c r="R15" t="s">
         <v>1792</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6812,7 +6838,7 @@
       <c r="J16" t="s">
         <v>1616</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6856,7 +6882,7 @@
       <c r="J17" t="s">
         <v>1616</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6900,7 +6926,7 @@
       <c r="J18" t="s">
         <v>1616</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6918,7 +6944,7 @@
       <c r="R18" t="s">
         <v>1793</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6959,7 +6985,7 @@
       <c r="J19" t="s">
         <v>1616</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7003,7 +7029,7 @@
       <c r="J20" t="s">
         <v>1616</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7047,7 +7073,7 @@
       <c r="J21" t="s">
         <v>1616</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7065,7 +7091,7 @@
       <c r="R21" t="s">
         <v>1792</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7106,7 +7132,7 @@
       <c r="J22" t="s">
         <v>1616</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7124,7 +7150,7 @@
       <c r="R22" t="s">
         <v>1794</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7165,7 +7191,7 @@
       <c r="J23" t="s">
         <v>1616</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7183,7 +7209,7 @@
       <c r="R23" t="s">
         <v>1795</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7224,7 +7250,7 @@
       <c r="J24" t="s">
         <v>1616</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7268,7 +7294,7 @@
       <c r="J25" t="s">
         <v>1616</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7309,7 +7335,7 @@
       <c r="J26" t="s">
         <v>1618</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7327,7 +7353,7 @@
       <c r="R26" t="s">
         <v>1796</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7365,7 +7391,7 @@
       <c r="J27" t="s">
         <v>1616</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7383,7 +7409,7 @@
       <c r="R27" t="s">
         <v>1797</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7424,7 +7450,7 @@
       <c r="J28" t="s">
         <v>1616</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7468,7 +7494,7 @@
       <c r="J29" t="s">
         <v>1616</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7512,7 +7538,7 @@
       <c r="J30" t="s">
         <v>1616</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7556,7 +7582,7 @@
       <c r="J31" t="s">
         <v>1616</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7574,7 +7600,7 @@
       <c r="R31" t="s">
         <v>1798</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7615,7 +7641,7 @@
       <c r="J32" t="s">
         <v>1616</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7659,7 +7685,7 @@
       <c r="J33" t="s">
         <v>1616</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7677,7 +7703,7 @@
       <c r="R33" t="s">
         <v>1799</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7718,7 +7744,7 @@
       <c r="J34" t="s">
         <v>1616</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7762,7 +7788,7 @@
       <c r="J35" t="s">
         <v>1616</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7780,7 +7806,7 @@
       <c r="R35" t="s">
         <v>1800</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7821,7 +7847,7 @@
       <c r="J36" t="s">
         <v>1616</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7839,7 +7865,7 @@
       <c r="R36" t="s">
         <v>1800</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7880,7 +7906,7 @@
       <c r="J37" t="s">
         <v>1616</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7898,7 +7924,7 @@
       <c r="R37" t="s">
         <v>1800</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7939,7 +7965,7 @@
       <c r="J38" t="s">
         <v>1616</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7957,7 +7983,7 @@
       <c r="R38" t="s">
         <v>1800</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7998,7 +8024,7 @@
       <c r="J39" t="s">
         <v>1616</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8016,7 +8042,7 @@
       <c r="R39" t="s">
         <v>1800</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8057,7 +8083,7 @@
       <c r="J40" t="s">
         <v>1616</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8075,7 +8101,7 @@
       <c r="R40" t="s">
         <v>1801</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8116,7 +8142,7 @@
       <c r="J41" t="s">
         <v>1616</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8134,7 +8160,7 @@
       <c r="R41" t="s">
         <v>1792</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8175,7 +8201,7 @@
       <c r="J42" t="s">
         <v>1616</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8193,7 +8219,7 @@
       <c r="R42" t="s">
         <v>1800</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8234,7 +8260,7 @@
       <c r="J43" t="s">
         <v>1616</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8278,7 +8304,7 @@
       <c r="J44" t="s">
         <v>1616</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8296,7 +8322,7 @@
       <c r="R44" t="s">
         <v>1802</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8337,7 +8363,7 @@
       <c r="J45" t="s">
         <v>1616</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8355,7 +8381,7 @@
       <c r="R45" t="s">
         <v>1803</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8393,7 +8419,7 @@
       <c r="J46" t="s">
         <v>1616</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8437,7 +8463,7 @@
       <c r="J47" t="s">
         <v>1616</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8455,7 +8481,7 @@
       <c r="R47" t="s">
         <v>1804</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8496,7 +8522,7 @@
       <c r="J48" t="s">
         <v>1616</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8540,7 +8566,7 @@
       <c r="J49" t="s">
         <v>1616</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8584,7 +8610,7 @@
       <c r="J50" t="s">
         <v>1616</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8628,7 +8654,7 @@
       <c r="J51" t="s">
         <v>1616</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8675,7 +8701,7 @@
       <c r="J52" t="s">
         <v>1616</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8719,7 +8745,7 @@
       <c r="J53" t="s">
         <v>1616</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8763,7 +8789,7 @@
       <c r="J54" t="s">
         <v>1616</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8807,7 +8833,7 @@
       <c r="J55" t="s">
         <v>1616</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8857,7 +8883,7 @@
       <c r="J56" t="s">
         <v>1616</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8910,7 +8936,7 @@
       <c r="J57" t="s">
         <v>1616</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8960,7 +8986,7 @@
       <c r="J58" t="s">
         <v>1616</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9010,7 +9036,7 @@
       <c r="J59" t="s">
         <v>1616</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9028,7 +9054,7 @@
       <c r="R59" t="s">
         <v>1805</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9069,7 +9095,7 @@
       <c r="J60" t="s">
         <v>1616</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9113,7 +9139,7 @@
       <c r="J61" t="s">
         <v>1616</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9157,7 +9183,7 @@
       <c r="J62" t="s">
         <v>1616</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9201,7 +9227,7 @@
       <c r="J63" t="s">
         <v>1616</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9245,7 +9271,7 @@
       <c r="J64" t="s">
         <v>1616</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9289,7 +9315,7 @@
       <c r="J65" t="s">
         <v>1616</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9336,7 +9362,7 @@
       <c r="J66" t="s">
         <v>1616</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9354,7 +9380,7 @@
       <c r="R66" t="s">
         <v>1806</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9392,7 +9418,7 @@
       <c r="J67" t="s">
         <v>1616</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9436,7 +9462,7 @@
       <c r="J68" t="s">
         <v>1616</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9451,7 +9477,7 @@
       <c r="O68" t="s">
         <v>1710</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9495,7 +9521,7 @@
       <c r="J69" t="s">
         <v>1618</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9539,7 +9565,7 @@
       <c r="J70" t="s">
         <v>1616</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9583,7 +9609,7 @@
       <c r="J71" t="s">
         <v>1616</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9627,7 +9653,7 @@
       <c r="J72" t="s">
         <v>1616</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9671,7 +9697,7 @@
       <c r="J73" t="s">
         <v>1616</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9715,7 +9741,7 @@
       <c r="J74" t="s">
         <v>1616</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9759,7 +9785,7 @@
       <c r="J75" t="s">
         <v>1616</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9803,7 +9829,7 @@
       <c r="J76" t="s">
         <v>1616</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9821,7 +9847,7 @@
       <c r="R76" t="s">
         <v>1807</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9859,7 +9885,7 @@
       <c r="J77" t="s">
         <v>1616</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9877,7 +9903,7 @@
       <c r="R77" t="s">
         <v>1807</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9915,7 +9941,7 @@
       <c r="J78" t="s">
         <v>1616</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9933,7 +9959,7 @@
       <c r="R78" t="s">
         <v>1807</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9971,7 +9997,7 @@
       <c r="J79" t="s">
         <v>1616</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9989,7 +10015,7 @@
       <c r="R79" t="s">
         <v>1807</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10027,7 +10053,7 @@
       <c r="J80" t="s">
         <v>1616</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10071,7 +10097,7 @@
       <c r="J81" t="s">
         <v>1616</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10115,7 +10141,7 @@
       <c r="J82" t="s">
         <v>1616</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10159,7 +10185,7 @@
       <c r="J83" t="s">
         <v>1616</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10203,7 +10229,7 @@
       <c r="J84" t="s">
         <v>1616</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10247,7 +10273,7 @@
       <c r="J85" t="s">
         <v>1616</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10265,7 +10291,7 @@
       <c r="R85" t="s">
         <v>1808</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10303,7 +10329,7 @@
       <c r="J86" t="s">
         <v>1616</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10347,7 +10373,7 @@
       <c r="J87" t="s">
         <v>1616</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10365,7 +10391,7 @@
       <c r="R87" t="s">
         <v>1809</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10403,7 +10429,7 @@
       <c r="J88" t="s">
         <v>1616</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10447,7 +10473,7 @@
       <c r="J89" t="s">
         <v>1616</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10465,7 +10491,7 @@
       <c r="R89" t="s">
         <v>1810</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10500,7 +10526,7 @@
       <c r="J90" t="s">
         <v>1616</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10518,7 +10544,7 @@
       <c r="R90" t="s">
         <v>1811</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10553,7 +10579,7 @@
       <c r="J91" t="s">
         <v>1616</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10571,7 +10597,7 @@
       <c r="R91" t="s">
         <v>1795</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10609,7 +10635,7 @@
       <c r="J92" t="s">
         <v>1616</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10630,7 +10656,7 @@
       <c r="R92" t="s">
         <v>1795</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10671,7 +10697,7 @@
       <c r="J93" t="s">
         <v>1616</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10712,7 +10738,7 @@
       <c r="J94" t="s">
         <v>1616</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10756,7 +10782,7 @@
       <c r="J95" t="s">
         <v>1616</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10800,7 +10826,7 @@
       <c r="J96" t="s">
         <v>1616</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10818,7 +10844,7 @@
       <c r="R96" t="s">
         <v>1812</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10859,7 +10885,7 @@
       <c r="J97" t="s">
         <v>1616</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10874,7 +10900,7 @@
       <c r="R97" t="s">
         <v>1812</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10915,7 +10941,7 @@
       <c r="J98" t="s">
         <v>1616</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10933,7 +10959,7 @@
       <c r="R98" t="s">
         <v>1813</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10971,7 +10997,7 @@
       <c r="J99" t="s">
         <v>1616</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10989,7 +11015,7 @@
       <c r="R99" t="s">
         <v>1814</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11027,7 +11053,7 @@
       <c r="J100" t="s">
         <v>1616</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11068,7 +11094,7 @@
       <c r="J101" t="s">
         <v>1616</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11109,7 +11135,7 @@
       <c r="J102" t="s">
         <v>1616</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11150,7 +11176,7 @@
       <c r="J103" t="s">
         <v>1616</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11191,7 +11217,7 @@
       <c r="J104" t="s">
         <v>1616</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11232,7 +11258,7 @@
       <c r="J105" t="s">
         <v>1616</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11273,7 +11299,7 @@
       <c r="J106" t="s">
         <v>1616</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11314,7 +11340,7 @@
       <c r="J107" t="s">
         <v>1616</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11355,7 +11381,7 @@
       <c r="J108" t="s">
         <v>1616</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11396,7 +11422,7 @@
       <c r="J109" t="s">
         <v>1616</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11449,7 +11475,7 @@
       <c r="J110" t="s">
         <v>1616</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11505,7 +11531,7 @@
       <c r="J111" t="s">
         <v>1616</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11523,7 +11549,7 @@
       <c r="R111" t="s">
         <v>1816</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11561,7 +11587,7 @@
       <c r="J112" t="s">
         <v>1616</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11620,7 +11646,7 @@
       <c r="J113" t="s">
         <v>1616</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11664,7 +11690,7 @@
       <c r="J114" t="s">
         <v>1616</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11708,7 +11734,7 @@
       <c r="J115" t="s">
         <v>1616</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11726,7 +11752,7 @@
       <c r="R115" t="s">
         <v>1818</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11767,7 +11793,7 @@
       <c r="J116" t="s">
         <v>1616</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11826,7 +11852,7 @@
       <c r="J117" t="s">
         <v>1616</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11870,7 +11896,7 @@
       <c r="J118" t="s">
         <v>1616</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11917,7 +11943,7 @@
       <c r="J119" t="s">
         <v>1616</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11958,7 +11984,7 @@
       <c r="J120" t="s">
         <v>1616</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12002,7 +12028,7 @@
       <c r="J121" t="s">
         <v>1616</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12049,7 +12075,7 @@
       <c r="J122" t="s">
         <v>1616</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12099,7 +12125,7 @@
       <c r="J123" t="s">
         <v>1616</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12143,7 +12169,7 @@
       <c r="J124" t="s">
         <v>1616</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12187,7 +12213,7 @@
       <c r="J125" t="s">
         <v>1616</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12205,7 +12231,7 @@
       <c r="R125" t="s">
         <v>1820</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12240,7 +12266,7 @@
       <c r="J126" t="s">
         <v>1616</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12258,7 +12284,7 @@
       <c r="R126" t="s">
         <v>1821</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12296,7 +12322,7 @@
       <c r="J127" t="s">
         <v>1616</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12352,7 +12378,7 @@
       <c r="J128" t="s">
         <v>1616</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12393,7 +12419,7 @@
       <c r="J129" t="s">
         <v>1616</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12434,7 +12460,7 @@
       <c r="J130" t="s">
         <v>1616</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12475,7 +12501,7 @@
       <c r="J131" t="s">
         <v>1616</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12519,7 +12545,7 @@
       <c r="J132" t="s">
         <v>1616</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12560,7 +12586,7 @@
       <c r="J133" t="s">
         <v>1616</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12578,7 +12604,7 @@
       <c r="R133" t="s">
         <v>1807</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12616,7 +12642,7 @@
       <c r="J134" t="s">
         <v>1616</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12634,7 +12660,7 @@
       <c r="R134" t="s">
         <v>1807</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12669,7 +12695,7 @@
       <c r="J135" t="s">
         <v>1616</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12710,7 +12736,7 @@
       <c r="J136" t="s">
         <v>1616</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12751,7 +12777,7 @@
       <c r="J137" t="s">
         <v>1616</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12792,7 +12818,7 @@
       <c r="J138" t="s">
         <v>1616</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12833,7 +12859,7 @@
       <c r="J139" t="s">
         <v>1616</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12880,7 +12906,7 @@
       <c r="J140" t="s">
         <v>1616</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12921,7 +12947,7 @@
       <c r="J141" t="s">
         <v>1616</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12962,7 +12988,7 @@
       <c r="J142" t="s">
         <v>1616</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13006,7 +13032,7 @@
       <c r="J143" t="s">
         <v>1616</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13024,7 +13050,7 @@
       <c r="R143" t="s">
         <v>1807</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13059,7 +13085,7 @@
       <c r="J144" t="s">
         <v>1616</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13077,7 +13103,7 @@
       <c r="R144" t="s">
         <v>1807</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13115,7 +13141,7 @@
       <c r="J145" t="s">
         <v>1616</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13133,7 +13159,7 @@
       <c r="R145" t="s">
         <v>1807</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13168,7 +13194,7 @@
       <c r="J146" t="s">
         <v>1616</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13186,7 +13212,7 @@
       <c r="R146" t="s">
         <v>1815</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13221,7 +13247,7 @@
       <c r="J147" t="s">
         <v>1616</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13239,7 +13265,7 @@
       <c r="R147" t="s">
         <v>1822</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13274,7 +13300,7 @@
       <c r="J148" t="s">
         <v>1616</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13315,7 +13341,7 @@
       <c r="J149" t="s">
         <v>1616</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13333,7 +13359,7 @@
       <c r="R149" t="s">
         <v>1807</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13368,7 +13394,7 @@
       <c r="J150" t="s">
         <v>1616</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13386,7 +13412,7 @@
       <c r="R150" t="s">
         <v>1807</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13424,7 +13450,7 @@
       <c r="J151" t="s">
         <v>1616</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13442,7 +13468,7 @@
       <c r="R151" t="s">
         <v>1823</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13477,7 +13503,7 @@
       <c r="J152" t="s">
         <v>1616</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13495,7 +13521,7 @@
       <c r="R152" t="s">
         <v>1824</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13530,7 +13556,7 @@
       <c r="J153" t="s">
         <v>1616</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13539,7 +13565,7 @@
       <c r="M153" t="s">
         <v>1701</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13580,7 +13606,7 @@
       <c r="J154" t="s">
         <v>1616</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13621,7 +13647,7 @@
       <c r="J155" t="s">
         <v>1616</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13662,7 +13688,7 @@
       <c r="J156" t="s">
         <v>1616</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13703,7 +13729,7 @@
       <c r="J157" t="s">
         <v>1616</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13744,7 +13770,7 @@
       <c r="J158" t="s">
         <v>1616</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13785,7 +13811,7 @@
       <c r="J159" t="s">
         <v>1616</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13826,7 +13852,7 @@
       <c r="J160" t="s">
         <v>1616</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13867,7 +13893,7 @@
       <c r="J161" t="s">
         <v>1616</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13908,7 +13934,7 @@
       <c r="J162" t="s">
         <v>1616</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13926,7 +13952,7 @@
       <c r="R162" t="s">
         <v>1810</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13961,7 +13987,7 @@
       <c r="J163" t="s">
         <v>1616</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13979,7 +14005,7 @@
       <c r="R163" t="s">
         <v>1807</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14014,7 +14040,7 @@
       <c r="J164" t="s">
         <v>1616</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14058,7 +14084,7 @@
       <c r="J165" t="s">
         <v>1616</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14099,7 +14125,7 @@
       <c r="J166" t="s">
         <v>1616</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14117,7 +14143,7 @@
       <c r="R166" t="s">
         <v>1825</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14152,7 +14178,7 @@
       <c r="J167" t="s">
         <v>1616</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14196,7 +14222,7 @@
       <c r="J168" t="s">
         <v>1616</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14240,7 +14266,7 @@
       <c r="J169" t="s">
         <v>1616</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14281,7 +14307,7 @@
       <c r="J170" t="s">
         <v>1616</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14322,7 +14348,7 @@
       <c r="J171" t="s">
         <v>1616</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14363,7 +14389,7 @@
       <c r="J172" t="s">
         <v>1616</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14404,7 +14430,7 @@
       <c r="J173" t="s">
         <v>1616</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14445,7 +14471,7 @@
       <c r="J174" t="s">
         <v>1616</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14486,7 +14512,7 @@
       <c r="J175" t="s">
         <v>1616</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14527,7 +14553,7 @@
       <c r="J176" t="s">
         <v>1616</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14568,7 +14594,7 @@
       <c r="J177" t="s">
         <v>1616</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14609,7 +14635,7 @@
       <c r="J178" t="s">
         <v>1616</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14627,7 +14653,7 @@
       <c r="R178" t="s">
         <v>1823</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14665,7 +14691,7 @@
       <c r="J179" t="s">
         <v>1616</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14674,7 +14700,7 @@
       <c r="M179" t="s">
         <v>1698</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14715,7 +14741,7 @@
       <c r="J180" t="s">
         <v>1616</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14756,7 +14782,7 @@
       <c r="J181" t="s">
         <v>1616</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14774,7 +14800,7 @@
       <c r="R181" t="s">
         <v>1807</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14809,7 +14835,7 @@
       <c r="J182" t="s">
         <v>1616</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14850,7 +14876,7 @@
       <c r="J183" t="s">
         <v>1616</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14891,7 +14917,7 @@
       <c r="J184" t="s">
         <v>1616</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14932,7 +14958,7 @@
       <c r="J185" t="s">
         <v>1616</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14973,7 +14999,7 @@
       <c r="J186" t="s">
         <v>1616</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15014,7 +15040,7 @@
       <c r="J187" t="s">
         <v>1616</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15055,7 +15081,7 @@
       <c r="J188" t="s">
         <v>1616</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15096,7 +15122,7 @@
       <c r="J189" t="s">
         <v>1616</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15137,7 +15163,7 @@
       <c r="J190" t="s">
         <v>1616</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15178,7 +15204,7 @@
       <c r="J191" t="s">
         <v>1616</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15219,7 +15245,7 @@
       <c r="J192" t="s">
         <v>1616</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15260,7 +15286,7 @@
       <c r="J193" t="s">
         <v>1616</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15301,7 +15327,7 @@
       <c r="J194" t="s">
         <v>1616</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15342,7 +15368,7 @@
       <c r="J195" t="s">
         <v>1616</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15360,7 +15386,7 @@
       <c r="R195" t="s">
         <v>1816</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15401,7 +15427,7 @@
       <c r="J196" t="s">
         <v>1616</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15419,7 +15445,7 @@
       <c r="R196" t="s">
         <v>1822</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15457,7 +15483,7 @@
       <c r="J197" t="s">
         <v>1616</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15498,7 +15524,7 @@
       <c r="J198" t="s">
         <v>1618</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15539,7 +15565,7 @@
       <c r="J199" t="s">
         <v>1617</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15580,7 +15606,7 @@
       <c r="J200" t="s">
         <v>1616</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15621,7 +15647,7 @@
       <c r="J201" t="s">
         <v>1616</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15662,7 +15688,7 @@
       <c r="J202" t="s">
         <v>1616</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15680,7 +15706,7 @@
       <c r="R202" t="s">
         <v>1807</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15718,7 +15744,7 @@
       <c r="J203" t="s">
         <v>1616</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15736,7 +15762,7 @@
       <c r="R203" t="s">
         <v>1815</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15771,7 +15797,7 @@
       <c r="J204" t="s">
         <v>1616</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15786,7 +15812,7 @@
       <c r="R204" t="s">
         <v>1826</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15824,7 +15850,7 @@
       <c r="J205" t="s">
         <v>1616</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15842,7 +15868,7 @@
       <c r="R205" t="s">
         <v>1827</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15880,7 +15906,7 @@
       <c r="J206" t="s">
         <v>1616</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15898,7 +15924,7 @@
       <c r="R206" t="s">
         <v>1795</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15933,7 +15959,7 @@
       <c r="J207" t="s">
         <v>1616</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15974,7 +16000,7 @@
       <c r="J208" t="s">
         <v>1616</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16015,7 +16041,7 @@
       <c r="J209" t="s">
         <v>1616</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16056,7 +16082,7 @@
       <c r="J210" t="s">
         <v>1616</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16097,7 +16123,7 @@
       <c r="J211" t="s">
         <v>1616</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16138,7 +16164,7 @@
       <c r="J212" t="s">
         <v>1616</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16179,7 +16205,7 @@
       <c r="J213" t="s">
         <v>1616</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16220,7 +16246,7 @@
       <c r="J214" t="s">
         <v>1616</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16238,7 +16264,7 @@
       <c r="R214" t="s">
         <v>1828</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16276,7 +16302,7 @@
       <c r="J215" t="s">
         <v>1616</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16317,7 +16343,7 @@
       <c r="J216" t="s">
         <v>1616</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16358,7 +16384,7 @@
       <c r="J217" t="s">
         <v>1616</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16399,7 +16425,7 @@
       <c r="J218" t="s">
         <v>1616</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16440,7 +16466,7 @@
       <c r="J219" t="s">
         <v>1616</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16481,7 +16507,7 @@
       <c r="J220" t="s">
         <v>1616</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16522,7 +16548,7 @@
       <c r="J221" t="s">
         <v>1616</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16563,7 +16589,7 @@
       <c r="J222" t="s">
         <v>1616</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16604,7 +16630,7 @@
       <c r="J223" t="s">
         <v>1616</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16645,7 +16671,7 @@
       <c r="J224" t="s">
         <v>1616</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16686,7 +16712,7 @@
       <c r="J225" t="s">
         <v>1616</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16727,7 +16753,7 @@
       <c r="J226" t="s">
         <v>1616</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16768,7 +16794,7 @@
       <c r="J227" t="s">
         <v>1616</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16809,7 +16835,7 @@
       <c r="J228" t="s">
         <v>1616</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16850,7 +16876,7 @@
       <c r="J229" t="s">
         <v>1616</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16891,7 +16917,7 @@
       <c r="J230" t="s">
         <v>1616</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16932,7 +16958,7 @@
       <c r="J231" t="s">
         <v>1616</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16973,7 +16999,7 @@
       <c r="J232" t="s">
         <v>1616</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17014,7 +17040,7 @@
       <c r="J233" t="s">
         <v>1616</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17055,7 +17081,7 @@
       <c r="J234" t="s">
         <v>1616</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17096,7 +17122,7 @@
       <c r="J235" t="s">
         <v>1616</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17137,7 +17163,7 @@
       <c r="J236" t="s">
         <v>1616</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17178,7 +17204,7 @@
       <c r="J237" t="s">
         <v>1616</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17219,7 +17245,7 @@
       <c r="J238" t="s">
         <v>1616</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17260,7 +17286,7 @@
       <c r="J239" t="s">
         <v>1616</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17278,7 +17304,7 @@
       <c r="R239" t="s">
         <v>1822</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17316,7 +17342,7 @@
       <c r="J240" t="s">
         <v>1616</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17357,7 +17383,7 @@
       <c r="J241" t="s">
         <v>1616</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17398,7 +17424,7 @@
       <c r="J242" t="s">
         <v>1616</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17416,7 +17442,7 @@
       <c r="R242" t="s">
         <v>1815</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17451,7 +17477,7 @@
       <c r="J243" t="s">
         <v>1616</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17492,7 +17518,7 @@
       <c r="J244" t="s">
         <v>1616</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17533,7 +17559,7 @@
       <c r="J245" t="s">
         <v>1616</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17574,7 +17600,7 @@
       <c r="J246" t="s">
         <v>1616</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17592,7 +17618,7 @@
       <c r="R246" t="s">
         <v>1795</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17630,7 +17656,7 @@
       <c r="J247" t="s">
         <v>1616</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17671,7 +17697,7 @@
       <c r="J248" t="s">
         <v>1616</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17712,7 +17738,7 @@
       <c r="J249" t="s">
         <v>1616</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17753,7 +17779,7 @@
       <c r="J250" t="s">
         <v>1616</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17794,7 +17820,7 @@
       <c r="J251" t="s">
         <v>1616</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17835,7 +17861,7 @@
       <c r="J252" t="s">
         <v>1616</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17876,7 +17902,7 @@
       <c r="J253" t="s">
         <v>1616</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17894,7 +17920,7 @@
       <c r="R253" t="s">
         <v>1825</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -17935,7 +17961,7 @@
       <c r="J254" t="s">
         <v>1616</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17976,7 +18002,7 @@
       <c r="J255" t="s">
         <v>1616</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18017,7 +18043,7 @@
       <c r="J256" t="s">
         <v>1616</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18026,7 +18052,7 @@
       <c r="M256" t="s">
         <v>1697</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18064,7 +18090,7 @@
       <c r="J257" t="s">
         <v>1616</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18073,7 +18099,7 @@
       <c r="M257" t="s">
         <v>1698</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18117,7 +18143,7 @@
       <c r="J258" t="s">
         <v>1616</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18135,7 +18161,7 @@
       <c r="R258" t="s">
         <v>1807</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18173,7 +18199,7 @@
       <c r="J259" t="s">
         <v>1616</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18191,7 +18217,7 @@
       <c r="R259" t="s">
         <v>1823</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18229,7 +18255,7 @@
       <c r="J260" t="s">
         <v>1616</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18238,7 +18264,7 @@
       <c r="M260" t="s">
         <v>1692</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18282,7 +18308,7 @@
       <c r="J261" t="s">
         <v>1616</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18300,7 +18326,7 @@
       <c r="R261" t="s">
         <v>1829</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18338,7 +18364,7 @@
       <c r="J262" t="s">
         <v>1616</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18356,7 +18382,7 @@
       <c r="R262" t="s">
         <v>1823</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18394,7 +18420,7 @@
       <c r="J263" t="s">
         <v>1616</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18403,7 +18429,7 @@
       <c r="M263" t="s">
         <v>1692</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18447,7 +18473,7 @@
       <c r="J264" t="s">
         <v>1616</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18488,7 +18514,7 @@
       <c r="J265" t="s">
         <v>1616</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18529,7 +18555,7 @@
       <c r="J266" t="s">
         <v>1616</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18570,7 +18596,7 @@
       <c r="J267" t="s">
         <v>1616</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18614,7 +18640,7 @@
       <c r="J268" t="s">
         <v>1616</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18655,7 +18681,7 @@
       <c r="J269" t="s">
         <v>1616</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18696,7 +18722,7 @@
       <c r="J270" t="s">
         <v>1616</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18737,7 +18763,7 @@
       <c r="J271" t="s">
         <v>1616</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18778,7 +18804,7 @@
       <c r="J272" t="s">
         <v>1616</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18796,7 +18822,7 @@
       <c r="R272" t="s">
         <v>1830</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18837,7 +18863,7 @@
       <c r="J273" t="s">
         <v>1616</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18881,7 +18907,7 @@
       <c r="J274" t="s">
         <v>1616</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18922,7 +18948,7 @@
       <c r="J275" t="s">
         <v>1616</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18963,7 +18989,7 @@
       <c r="J276" t="s">
         <v>1616</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19004,7 +19030,7 @@
       <c r="J277" t="s">
         <v>1616</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19045,7 +19071,7 @@
       <c r="J278" t="s">
         <v>1616</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19086,7 +19112,7 @@
       <c r="J279" t="s">
         <v>1616</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19127,7 +19153,7 @@
       <c r="J280" t="s">
         <v>1616</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19168,7 +19194,7 @@
       <c r="J281" t="s">
         <v>1616</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19209,7 +19235,7 @@
       <c r="J282" t="s">
         <v>1616</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19250,7 +19276,7 @@
       <c r="J283" t="s">
         <v>1616</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19291,7 +19317,7 @@
       <c r="J284" t="s">
         <v>1616</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19332,7 +19358,7 @@
       <c r="J285" t="s">
         <v>1616</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19373,7 +19399,7 @@
       <c r="J286" t="s">
         <v>1616</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19414,7 +19440,7 @@
       <c r="J287" t="s">
         <v>1616</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19455,7 +19481,7 @@
       <c r="J288" t="s">
         <v>1616</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19496,7 +19522,7 @@
       <c r="J289" t="s">
         <v>1616</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19537,7 +19563,7 @@
       <c r="J290" t="s">
         <v>1616</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19578,7 +19604,7 @@
       <c r="J291" t="s">
         <v>1616</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19619,7 +19645,7 @@
       <c r="J292" t="s">
         <v>1616</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19660,7 +19686,7 @@
       <c r="J293" t="s">
         <v>1616</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19701,7 +19727,7 @@
       <c r="J294" t="s">
         <v>1616</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19742,7 +19768,7 @@
       <c r="J295" t="s">
         <v>1616</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19760,7 +19786,7 @@
       <c r="R295" t="s">
         <v>1831</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19801,7 +19827,7 @@
       <c r="J296" t="s">
         <v>1616</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19819,7 +19845,7 @@
       <c r="R296" t="s">
         <v>1807</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19857,7 +19883,7 @@
       <c r="J297" t="s">
         <v>1616</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19898,7 +19924,7 @@
       <c r="J298" t="s">
         <v>1616</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19939,7 +19965,7 @@
       <c r="J299" t="s">
         <v>1617</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19980,7 +20006,7 @@
       <c r="J300" t="s">
         <v>1616</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20021,7 +20047,7 @@
       <c r="J301" t="s">
         <v>1616</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20859,7 +20885,7 @@
       <c r="R321" t="s">
         <v>1793</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21082,7 +21108,7 @@
       <c r="R326" t="s">
         <v>1832</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21917,7 +21943,7 @@
       <c r="R346" t="s">
         <v>1833</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (06/10/2026 14:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5690,16 +5690,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5715,7 +5707,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5723,30 +5715,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6046,73 +6020,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6147,7 +6121,7 @@
       <c r="J2" t="s">
         <v>1617</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6191,7 +6165,7 @@
       <c r="J3" t="s">
         <v>1617</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6235,7 +6209,7 @@
       <c r="J4" t="s">
         <v>1617</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6253,7 +6227,7 @@
       <c r="R4" t="s">
         <v>1791</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6291,7 +6265,7 @@
       <c r="J5" t="s">
         <v>1618</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6341,7 +6315,7 @@
       <c r="J6" t="s">
         <v>1617</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6388,7 +6362,7 @@
       <c r="J7" t="s">
         <v>1617</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6435,7 +6409,7 @@
       <c r="J8" t="s">
         <v>1617</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6482,7 +6456,7 @@
       <c r="J9" t="s">
         <v>1617</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6529,7 +6503,7 @@
       <c r="J10" t="s">
         <v>1617</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6576,7 +6550,7 @@
       <c r="J11" t="s">
         <v>1617</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6623,7 +6597,7 @@
       <c r="J12" t="s">
         <v>1617</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6667,7 +6641,7 @@
       <c r="J13" t="s">
         <v>1617</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6685,7 +6659,7 @@
       <c r="R13" t="s">
         <v>1792</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6723,7 +6697,7 @@
       <c r="J14" t="s">
         <v>1617</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6741,7 +6715,7 @@
       <c r="R14" t="s">
         <v>1793</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6782,7 +6756,7 @@
       <c r="J15" t="s">
         <v>1617</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6800,7 +6774,7 @@
       <c r="R15" t="s">
         <v>1793</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6841,7 +6815,7 @@
       <c r="J16" t="s">
         <v>1617</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6885,7 +6859,7 @@
       <c r="J17" t="s">
         <v>1617</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6929,7 +6903,7 @@
       <c r="J18" t="s">
         <v>1617</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6947,7 +6921,7 @@
       <c r="R18" t="s">
         <v>1794</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6988,7 +6962,7 @@
       <c r="J19" t="s">
         <v>1617</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7032,7 +7006,7 @@
       <c r="J20" t="s">
         <v>1617</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7076,7 +7050,7 @@
       <c r="J21" t="s">
         <v>1617</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7094,7 +7068,7 @@
       <c r="R21" t="s">
         <v>1793</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7135,7 +7109,7 @@
       <c r="J22" t="s">
         <v>1617</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7153,7 +7127,7 @@
       <c r="R22" t="s">
         <v>1795</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7194,7 +7168,7 @@
       <c r="J23" t="s">
         <v>1617</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7212,7 +7186,7 @@
       <c r="R23" t="s">
         <v>1796</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7253,7 +7227,7 @@
       <c r="J24" t="s">
         <v>1617</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7297,7 +7271,7 @@
       <c r="J25" t="s">
         <v>1617</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7338,7 +7312,7 @@
       <c r="J26" t="s">
         <v>1619</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7356,7 +7330,7 @@
       <c r="R26" t="s">
         <v>1797</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7394,7 +7368,7 @@
       <c r="J27" t="s">
         <v>1617</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7412,7 +7386,7 @@
       <c r="R27" t="s">
         <v>1798</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7453,7 +7427,7 @@
       <c r="J28" t="s">
         <v>1617</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7497,7 +7471,7 @@
       <c r="J29" t="s">
         <v>1617</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7541,7 +7515,7 @@
       <c r="J30" t="s">
         <v>1617</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7585,7 +7559,7 @@
       <c r="J31" t="s">
         <v>1617</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7603,7 +7577,7 @@
       <c r="R31" t="s">
         <v>1799</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7644,7 +7618,7 @@
       <c r="J32" t="s">
         <v>1617</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7688,7 +7662,7 @@
       <c r="J33" t="s">
         <v>1617</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7706,7 +7680,7 @@
       <c r="R33" t="s">
         <v>1800</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7747,7 +7721,7 @@
       <c r="J34" t="s">
         <v>1617</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7791,7 +7765,7 @@
       <c r="J35" t="s">
         <v>1617</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7809,7 +7783,7 @@
       <c r="R35" t="s">
         <v>1801</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7850,7 +7824,7 @@
       <c r="J36" t="s">
         <v>1617</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7868,7 +7842,7 @@
       <c r="R36" t="s">
         <v>1801</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7909,7 +7883,7 @@
       <c r="J37" t="s">
         <v>1617</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7927,7 +7901,7 @@
       <c r="R37" t="s">
         <v>1801</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7968,7 +7942,7 @@
       <c r="J38" t="s">
         <v>1617</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7986,7 +7960,7 @@
       <c r="R38" t="s">
         <v>1801</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8027,7 +8001,7 @@
       <c r="J39" t="s">
         <v>1617</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8045,7 +8019,7 @@
       <c r="R39" t="s">
         <v>1801</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8086,7 +8060,7 @@
       <c r="J40" t="s">
         <v>1617</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8104,7 +8078,7 @@
       <c r="R40" t="s">
         <v>1802</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8145,7 +8119,7 @@
       <c r="J41" t="s">
         <v>1617</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8163,7 +8137,7 @@
       <c r="R41" t="s">
         <v>1793</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8204,7 +8178,7 @@
       <c r="J42" t="s">
         <v>1617</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8222,7 +8196,7 @@
       <c r="R42" t="s">
         <v>1801</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8263,7 +8237,7 @@
       <c r="J43" t="s">
         <v>1617</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8307,7 +8281,7 @@
       <c r="J44" t="s">
         <v>1617</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8325,7 +8299,7 @@
       <c r="R44" t="s">
         <v>1803</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8366,7 +8340,7 @@
       <c r="J45" t="s">
         <v>1617</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8384,7 +8358,7 @@
       <c r="R45" t="s">
         <v>1804</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8422,7 +8396,7 @@
       <c r="J46" t="s">
         <v>1617</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8466,7 +8440,7 @@
       <c r="J47" t="s">
         <v>1617</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8484,7 +8458,7 @@
       <c r="R47" t="s">
         <v>1805</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8525,7 +8499,7 @@
       <c r="J48" t="s">
         <v>1617</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8569,7 +8543,7 @@
       <c r="J49" t="s">
         <v>1617</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8613,7 +8587,7 @@
       <c r="J50" t="s">
         <v>1617</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8657,7 +8631,7 @@
       <c r="J51" t="s">
         <v>1617</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8704,7 +8678,7 @@
       <c r="J52" t="s">
         <v>1617</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8748,7 +8722,7 @@
       <c r="J53" t="s">
         <v>1617</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8792,7 +8766,7 @@
       <c r="J54" t="s">
         <v>1617</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8836,7 +8810,7 @@
       <c r="J55" t="s">
         <v>1617</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8886,7 +8860,7 @@
       <c r="J56" t="s">
         <v>1617</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8939,7 +8913,7 @@
       <c r="J57" t="s">
         <v>1617</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8989,7 +8963,7 @@
       <c r="J58" t="s">
         <v>1617</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9039,7 +9013,7 @@
       <c r="J59" t="s">
         <v>1617</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9057,7 +9031,7 @@
       <c r="R59" t="s">
         <v>1806</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9098,7 +9072,7 @@
       <c r="J60" t="s">
         <v>1617</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9142,7 +9116,7 @@
       <c r="J61" t="s">
         <v>1617</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9186,7 +9160,7 @@
       <c r="J62" t="s">
         <v>1617</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9230,7 +9204,7 @@
       <c r="J63" t="s">
         <v>1617</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9274,7 +9248,7 @@
       <c r="J64" t="s">
         <v>1617</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9318,7 +9292,7 @@
       <c r="J65" t="s">
         <v>1617</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9365,7 +9339,7 @@
       <c r="J66" t="s">
         <v>1617</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9383,7 +9357,7 @@
       <c r="R66" t="s">
         <v>1807</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9421,7 +9395,7 @@
       <c r="J67" t="s">
         <v>1617</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9465,7 +9439,7 @@
       <c r="J68" t="s">
         <v>1617</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9480,7 +9454,7 @@
       <c r="O68" t="s">
         <v>1711</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9524,7 +9498,7 @@
       <c r="J69" t="s">
         <v>1619</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9568,7 +9542,7 @@
       <c r="J70" t="s">
         <v>1617</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9612,7 +9586,7 @@
       <c r="J71" t="s">
         <v>1617</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9656,7 +9630,7 @@
       <c r="J72" t="s">
         <v>1617</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9700,7 +9674,7 @@
       <c r="J73" t="s">
         <v>1617</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9744,7 +9718,7 @@
       <c r="J74" t="s">
         <v>1617</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9788,7 +9762,7 @@
       <c r="J75" t="s">
         <v>1617</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9832,7 +9806,7 @@
       <c r="J76" t="s">
         <v>1617</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9850,7 +9824,7 @@
       <c r="R76" t="s">
         <v>1808</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9888,7 +9862,7 @@
       <c r="J77" t="s">
         <v>1617</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9906,7 +9880,7 @@
       <c r="R77" t="s">
         <v>1808</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9944,7 +9918,7 @@
       <c r="J78" t="s">
         <v>1617</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9962,7 +9936,7 @@
       <c r="R78" t="s">
         <v>1808</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10000,7 +9974,7 @@
       <c r="J79" t="s">
         <v>1617</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10018,7 +9992,7 @@
       <c r="R79" t="s">
         <v>1808</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10056,7 +10030,7 @@
       <c r="J80" t="s">
         <v>1617</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10100,7 +10074,7 @@
       <c r="J81" t="s">
         <v>1617</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10144,7 +10118,7 @@
       <c r="J82" t="s">
         <v>1617</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10188,7 +10162,7 @@
       <c r="J83" t="s">
         <v>1617</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10232,7 +10206,7 @@
       <c r="J84" t="s">
         <v>1617</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10276,7 +10250,7 @@
       <c r="J85" t="s">
         <v>1617</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10294,7 +10268,7 @@
       <c r="R85" t="s">
         <v>1809</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10332,7 +10306,7 @@
       <c r="J86" t="s">
         <v>1617</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10376,7 +10350,7 @@
       <c r="J87" t="s">
         <v>1617</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10394,7 +10368,7 @@
       <c r="R87" t="s">
         <v>1810</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10432,7 +10406,7 @@
       <c r="J88" t="s">
         <v>1617</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10476,7 +10450,7 @@
       <c r="J89" t="s">
         <v>1617</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10494,7 +10468,7 @@
       <c r="R89" t="s">
         <v>1811</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10529,7 +10503,7 @@
       <c r="J90" t="s">
         <v>1617</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10547,7 +10521,7 @@
       <c r="R90" t="s">
         <v>1812</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10582,7 +10556,7 @@
       <c r="J91" t="s">
         <v>1617</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10600,7 +10574,7 @@
       <c r="R91" t="s">
         <v>1796</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10638,7 +10612,7 @@
       <c r="J92" t="s">
         <v>1617</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10659,7 +10633,7 @@
       <c r="R92" t="s">
         <v>1796</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10700,7 +10674,7 @@
       <c r="J93" t="s">
         <v>1617</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10741,7 +10715,7 @@
       <c r="J94" t="s">
         <v>1617</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10785,7 +10759,7 @@
       <c r="J95" t="s">
         <v>1617</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10829,7 +10803,7 @@
       <c r="J96" t="s">
         <v>1617</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10847,7 +10821,7 @@
       <c r="R96" t="s">
         <v>1813</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10888,7 +10862,7 @@
       <c r="J97" t="s">
         <v>1617</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10903,7 +10877,7 @@
       <c r="R97" t="s">
         <v>1813</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10944,7 +10918,7 @@
       <c r="J98" t="s">
         <v>1617</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10962,7 +10936,7 @@
       <c r="R98" t="s">
         <v>1814</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11000,7 +10974,7 @@
       <c r="J99" t="s">
         <v>1617</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11018,7 +10992,7 @@
       <c r="R99" t="s">
         <v>1815</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11056,7 +11030,7 @@
       <c r="J100" t="s">
         <v>1617</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11097,7 +11071,7 @@
       <c r="J101" t="s">
         <v>1617</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11138,7 +11112,7 @@
       <c r="J102" t="s">
         <v>1617</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11179,7 +11153,7 @@
       <c r="J103" t="s">
         <v>1617</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11220,7 +11194,7 @@
       <c r="J104" t="s">
         <v>1617</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11261,7 +11235,7 @@
       <c r="J105" t="s">
         <v>1617</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11302,7 +11276,7 @@
       <c r="J106" t="s">
         <v>1617</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11343,7 +11317,7 @@
       <c r="J107" t="s">
         <v>1617</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11384,7 +11358,7 @@
       <c r="J108" t="s">
         <v>1617</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11425,7 +11399,7 @@
       <c r="J109" t="s">
         <v>1617</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11478,7 +11452,7 @@
       <c r="J110" t="s">
         <v>1617</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11534,7 +11508,7 @@
       <c r="J111" t="s">
         <v>1617</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11552,7 +11526,7 @@
       <c r="R111" t="s">
         <v>1817</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11590,7 +11564,7 @@
       <c r="J112" t="s">
         <v>1617</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11649,7 +11623,7 @@
       <c r="J113" t="s">
         <v>1617</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11693,7 +11667,7 @@
       <c r="J114" t="s">
         <v>1617</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11737,7 +11711,7 @@
       <c r="J115" t="s">
         <v>1617</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11755,7 +11729,7 @@
       <c r="R115" t="s">
         <v>1819</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11796,7 +11770,7 @@
       <c r="J116" t="s">
         <v>1617</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11855,7 +11829,7 @@
       <c r="J117" t="s">
         <v>1617</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11899,7 +11873,7 @@
       <c r="J118" t="s">
         <v>1617</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11946,7 +11920,7 @@
       <c r="J119" t="s">
         <v>1617</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11987,7 +11961,7 @@
       <c r="J120" t="s">
         <v>1617</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12031,7 +12005,7 @@
       <c r="J121" t="s">
         <v>1617</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12078,7 +12052,7 @@
       <c r="J122" t="s">
         <v>1617</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12128,7 +12102,7 @@
       <c r="J123" t="s">
         <v>1617</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12172,7 +12146,7 @@
       <c r="J124" t="s">
         <v>1617</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12216,7 +12190,7 @@
       <c r="J125" t="s">
         <v>1617</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12234,7 +12208,7 @@
       <c r="R125" t="s">
         <v>1821</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12269,7 +12243,7 @@
       <c r="J126" t="s">
         <v>1617</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12287,7 +12261,7 @@
       <c r="R126" t="s">
         <v>1822</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12325,7 +12299,7 @@
       <c r="J127" t="s">
         <v>1617</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12381,7 +12355,7 @@
       <c r="J128" t="s">
         <v>1617</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12422,7 +12396,7 @@
       <c r="J129" t="s">
         <v>1617</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12463,7 +12437,7 @@
       <c r="J130" t="s">
         <v>1617</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12504,7 +12478,7 @@
       <c r="J131" t="s">
         <v>1617</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12548,7 +12522,7 @@
       <c r="J132" t="s">
         <v>1617</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12589,7 +12563,7 @@
       <c r="J133" t="s">
         <v>1617</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12607,7 +12581,7 @@
       <c r="R133" t="s">
         <v>1808</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12645,7 +12619,7 @@
       <c r="J134" t="s">
         <v>1617</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12663,7 +12637,7 @@
       <c r="R134" t="s">
         <v>1808</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12698,7 +12672,7 @@
       <c r="J135" t="s">
         <v>1617</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12739,7 +12713,7 @@
       <c r="J136" t="s">
         <v>1617</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12780,7 +12754,7 @@
       <c r="J137" t="s">
         <v>1617</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12821,7 +12795,7 @@
       <c r="J138" t="s">
         <v>1617</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12862,7 +12836,7 @@
       <c r="J139" t="s">
         <v>1617</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12909,7 +12883,7 @@
       <c r="J140" t="s">
         <v>1617</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12950,7 +12924,7 @@
       <c r="J141" t="s">
         <v>1617</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12991,7 +12965,7 @@
       <c r="J142" t="s">
         <v>1617</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13035,7 +13009,7 @@
       <c r="J143" t="s">
         <v>1617</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13053,7 +13027,7 @@
       <c r="R143" t="s">
         <v>1808</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13088,7 +13062,7 @@
       <c r="J144" t="s">
         <v>1617</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13106,7 +13080,7 @@
       <c r="R144" t="s">
         <v>1808</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13144,7 +13118,7 @@
       <c r="J145" t="s">
         <v>1617</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13162,7 +13136,7 @@
       <c r="R145" t="s">
         <v>1808</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13197,7 +13171,7 @@
       <c r="J146" t="s">
         <v>1617</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13215,7 +13189,7 @@
       <c r="R146" t="s">
         <v>1816</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13250,7 +13224,7 @@
       <c r="J147" t="s">
         <v>1617</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13268,7 +13242,7 @@
       <c r="R147" t="s">
         <v>1823</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13303,7 +13277,7 @@
       <c r="J148" t="s">
         <v>1617</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13344,7 +13318,7 @@
       <c r="J149" t="s">
         <v>1617</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13362,7 +13336,7 @@
       <c r="R149" t="s">
         <v>1808</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13397,7 +13371,7 @@
       <c r="J150" t="s">
         <v>1617</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13415,7 +13389,7 @@
       <c r="R150" t="s">
         <v>1808</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13453,7 +13427,7 @@
       <c r="J151" t="s">
         <v>1617</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13471,7 +13445,7 @@
       <c r="R151" t="s">
         <v>1824</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13506,7 +13480,7 @@
       <c r="J152" t="s">
         <v>1617</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13524,7 +13498,7 @@
       <c r="R152" t="s">
         <v>1825</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13559,7 +13533,7 @@
       <c r="J153" t="s">
         <v>1617</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13568,7 +13542,7 @@
       <c r="M153" t="s">
         <v>1702</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13609,7 +13583,7 @@
       <c r="J154" t="s">
         <v>1617</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13650,7 +13624,7 @@
       <c r="J155" t="s">
         <v>1617</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13691,7 +13665,7 @@
       <c r="J156" t="s">
         <v>1617</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13732,7 +13706,7 @@
       <c r="J157" t="s">
         <v>1617</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13773,7 +13747,7 @@
       <c r="J158" t="s">
         <v>1617</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13814,7 +13788,7 @@
       <c r="J159" t="s">
         <v>1617</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13855,7 +13829,7 @@
       <c r="J160" t="s">
         <v>1617</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13896,7 +13870,7 @@
       <c r="J161" t="s">
         <v>1617</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13937,7 +13911,7 @@
       <c r="J162" t="s">
         <v>1617</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13955,7 +13929,7 @@
       <c r="R162" t="s">
         <v>1811</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13990,7 +13964,7 @@
       <c r="J163" t="s">
         <v>1617</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14008,7 +13982,7 @@
       <c r="R163" t="s">
         <v>1808</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14043,7 +14017,7 @@
       <c r="J164" t="s">
         <v>1617</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14087,7 +14061,7 @@
       <c r="J165" t="s">
         <v>1617</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14128,7 +14102,7 @@
       <c r="J166" t="s">
         <v>1617</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14146,7 +14120,7 @@
       <c r="R166" t="s">
         <v>1826</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14181,7 +14155,7 @@
       <c r="J167" t="s">
         <v>1617</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14225,7 +14199,7 @@
       <c r="J168" t="s">
         <v>1617</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14269,7 +14243,7 @@
       <c r="J169" t="s">
         <v>1617</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14310,7 +14284,7 @@
       <c r="J170" t="s">
         <v>1617</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14351,7 +14325,7 @@
       <c r="J171" t="s">
         <v>1617</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14392,7 +14366,7 @@
       <c r="J172" t="s">
         <v>1617</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14433,7 +14407,7 @@
       <c r="J173" t="s">
         <v>1617</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14474,7 +14448,7 @@
       <c r="J174" t="s">
         <v>1617</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14515,7 +14489,7 @@
       <c r="J175" t="s">
         <v>1617</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14556,7 +14530,7 @@
       <c r="J176" t="s">
         <v>1617</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14597,7 +14571,7 @@
       <c r="J177" t="s">
         <v>1617</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14638,7 +14612,7 @@
       <c r="J178" t="s">
         <v>1617</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14656,7 +14630,7 @@
       <c r="R178" t="s">
         <v>1824</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14694,7 +14668,7 @@
       <c r="J179" t="s">
         <v>1617</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14703,7 +14677,7 @@
       <c r="M179" t="s">
         <v>1699</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14744,7 +14718,7 @@
       <c r="J180" t="s">
         <v>1617</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14785,7 +14759,7 @@
       <c r="J181" t="s">
         <v>1617</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14803,7 +14777,7 @@
       <c r="R181" t="s">
         <v>1808</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14838,7 +14812,7 @@
       <c r="J182" t="s">
         <v>1617</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14879,7 +14853,7 @@
       <c r="J183" t="s">
         <v>1617</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14920,7 +14894,7 @@
       <c r="J184" t="s">
         <v>1617</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14961,7 +14935,7 @@
       <c r="J185" t="s">
         <v>1617</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15002,7 +14976,7 @@
       <c r="J186" t="s">
         <v>1617</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15043,7 +15017,7 @@
       <c r="J187" t="s">
         <v>1617</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15084,7 +15058,7 @@
       <c r="J188" t="s">
         <v>1617</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15125,7 +15099,7 @@
       <c r="J189" t="s">
         <v>1617</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15166,7 +15140,7 @@
       <c r="J190" t="s">
         <v>1617</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15207,7 +15181,7 @@
       <c r="J191" t="s">
         <v>1617</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15248,7 +15222,7 @@
       <c r="J192" t="s">
         <v>1617</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15289,7 +15263,7 @@
       <c r="J193" t="s">
         <v>1617</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15330,7 +15304,7 @@
       <c r="J194" t="s">
         <v>1617</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15371,7 +15345,7 @@
       <c r="J195" t="s">
         <v>1617</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15389,7 +15363,7 @@
       <c r="R195" t="s">
         <v>1817</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15430,7 +15404,7 @@
       <c r="J196" t="s">
         <v>1617</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15448,7 +15422,7 @@
       <c r="R196" t="s">
         <v>1823</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15486,7 +15460,7 @@
       <c r="J197" t="s">
         <v>1617</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15527,7 +15501,7 @@
       <c r="J198" t="s">
         <v>1619</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15568,7 +15542,7 @@
       <c r="J199" t="s">
         <v>1618</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15609,7 +15583,7 @@
       <c r="J200" t="s">
         <v>1617</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15650,7 +15624,7 @@
       <c r="J201" t="s">
         <v>1617</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15691,7 +15665,7 @@
       <c r="J202" t="s">
         <v>1617</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15709,7 +15683,7 @@
       <c r="R202" t="s">
         <v>1808</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15747,7 +15721,7 @@
       <c r="J203" t="s">
         <v>1617</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15765,7 +15739,7 @@
       <c r="R203" t="s">
         <v>1816</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15800,7 +15774,7 @@
       <c r="J204" t="s">
         <v>1617</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15815,7 +15789,7 @@
       <c r="R204" t="s">
         <v>1827</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15853,7 +15827,7 @@
       <c r="J205" t="s">
         <v>1617</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15871,7 +15845,7 @@
       <c r="R205" t="s">
         <v>1828</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15909,7 +15883,7 @@
       <c r="J206" t="s">
         <v>1617</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15927,7 +15901,7 @@
       <c r="R206" t="s">
         <v>1796</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15962,7 +15936,7 @@
       <c r="J207" t="s">
         <v>1617</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16003,7 +15977,7 @@
       <c r="J208" t="s">
         <v>1617</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16044,7 +16018,7 @@
       <c r="J209" t="s">
         <v>1617</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16085,7 +16059,7 @@
       <c r="J210" t="s">
         <v>1617</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16126,7 +16100,7 @@
       <c r="J211" t="s">
         <v>1617</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16167,7 +16141,7 @@
       <c r="J212" t="s">
         <v>1617</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16208,7 +16182,7 @@
       <c r="J213" t="s">
         <v>1617</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16249,7 +16223,7 @@
       <c r="J214" t="s">
         <v>1617</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16267,7 +16241,7 @@
       <c r="R214" t="s">
         <v>1829</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16305,7 +16279,7 @@
       <c r="J215" t="s">
         <v>1617</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16346,7 +16320,7 @@
       <c r="J216" t="s">
         <v>1617</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16387,7 +16361,7 @@
       <c r="J217" t="s">
         <v>1617</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16428,7 +16402,7 @@
       <c r="J218" t="s">
         <v>1617</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16469,7 +16443,7 @@
       <c r="J219" t="s">
         <v>1617</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16510,7 +16484,7 @@
       <c r="J220" t="s">
         <v>1617</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16551,7 +16525,7 @@
       <c r="J221" t="s">
         <v>1617</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16592,7 +16566,7 @@
       <c r="J222" t="s">
         <v>1617</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16633,7 +16607,7 @@
       <c r="J223" t="s">
         <v>1617</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16674,7 +16648,7 @@
       <c r="J224" t="s">
         <v>1617</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16715,7 +16689,7 @@
       <c r="J225" t="s">
         <v>1617</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16756,7 +16730,7 @@
       <c r="J226" t="s">
         <v>1617</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16797,7 +16771,7 @@
       <c r="J227" t="s">
         <v>1617</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16838,7 +16812,7 @@
       <c r="J228" t="s">
         <v>1617</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16879,7 +16853,7 @@
       <c r="J229" t="s">
         <v>1617</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16920,7 +16894,7 @@
       <c r="J230" t="s">
         <v>1617</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16961,7 +16935,7 @@
       <c r="J231" t="s">
         <v>1617</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17002,7 +16976,7 @@
       <c r="J232" t="s">
         <v>1617</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17043,7 +17017,7 @@
       <c r="J233" t="s">
         <v>1617</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17084,7 +17058,7 @@
       <c r="J234" t="s">
         <v>1617</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17125,7 +17099,7 @@
       <c r="J235" t="s">
         <v>1617</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17166,7 +17140,7 @@
       <c r="J236" t="s">
         <v>1617</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17207,7 +17181,7 @@
       <c r="J237" t="s">
         <v>1617</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17248,7 +17222,7 @@
       <c r="J238" t="s">
         <v>1617</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17289,7 +17263,7 @@
       <c r="J239" t="s">
         <v>1617</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17307,7 +17281,7 @@
       <c r="R239" t="s">
         <v>1823</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17345,7 +17319,7 @@
       <c r="J240" t="s">
         <v>1617</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17386,7 +17360,7 @@
       <c r="J241" t="s">
         <v>1617</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17427,7 +17401,7 @@
       <c r="J242" t="s">
         <v>1617</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17445,7 +17419,7 @@
       <c r="R242" t="s">
         <v>1816</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17480,7 +17454,7 @@
       <c r="J243" t="s">
         <v>1617</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17521,7 +17495,7 @@
       <c r="J244" t="s">
         <v>1617</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17562,7 +17536,7 @@
       <c r="J245" t="s">
         <v>1617</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17603,7 +17577,7 @@
       <c r="J246" t="s">
         <v>1617</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17621,7 +17595,7 @@
       <c r="R246" t="s">
         <v>1796</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17659,7 +17633,7 @@
       <c r="J247" t="s">
         <v>1617</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17700,7 +17674,7 @@
       <c r="J248" t="s">
         <v>1617</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17741,7 +17715,7 @@
       <c r="J249" t="s">
         <v>1617</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17782,7 +17756,7 @@
       <c r="J250" t="s">
         <v>1617</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17823,7 +17797,7 @@
       <c r="J251" t="s">
         <v>1617</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17864,7 +17838,7 @@
       <c r="J252" t="s">
         <v>1617</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17905,7 +17879,7 @@
       <c r="J253" t="s">
         <v>1617</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17923,7 +17897,7 @@
       <c r="R253" t="s">
         <v>1826</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -17964,7 +17938,7 @@
       <c r="J254" t="s">
         <v>1617</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18005,7 +17979,7 @@
       <c r="J255" t="s">
         <v>1617</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18046,7 +18020,7 @@
       <c r="J256" t="s">
         <v>1617</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18055,7 +18029,7 @@
       <c r="M256" t="s">
         <v>1698</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18093,7 +18067,7 @@
       <c r="J257" t="s">
         <v>1617</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18102,7 +18076,7 @@
       <c r="M257" t="s">
         <v>1699</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18146,7 +18120,7 @@
       <c r="J258" t="s">
         <v>1617</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18164,7 +18138,7 @@
       <c r="R258" t="s">
         <v>1808</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18202,7 +18176,7 @@
       <c r="J259" t="s">
         <v>1617</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18220,7 +18194,7 @@
       <c r="R259" t="s">
         <v>1824</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18258,7 +18232,7 @@
       <c r="J260" t="s">
         <v>1617</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18267,7 +18241,7 @@
       <c r="M260" t="s">
         <v>1693</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18311,7 +18285,7 @@
       <c r="J261" t="s">
         <v>1617</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18329,7 +18303,7 @@
       <c r="R261" t="s">
         <v>1830</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18367,7 +18341,7 @@
       <c r="J262" t="s">
         <v>1617</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18385,7 +18359,7 @@
       <c r="R262" t="s">
         <v>1824</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18423,7 +18397,7 @@
       <c r="J263" t="s">
         <v>1617</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18432,7 +18406,7 @@
       <c r="M263" t="s">
         <v>1693</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18476,7 +18450,7 @@
       <c r="J264" t="s">
         <v>1617</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18517,7 +18491,7 @@
       <c r="J265" t="s">
         <v>1617</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18558,7 +18532,7 @@
       <c r="J266" t="s">
         <v>1617</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18599,7 +18573,7 @@
       <c r="J267" t="s">
         <v>1617</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18643,7 +18617,7 @@
       <c r="J268" t="s">
         <v>1617</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18684,7 +18658,7 @@
       <c r="J269" t="s">
         <v>1617</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18725,7 +18699,7 @@
       <c r="J270" t="s">
         <v>1617</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18766,7 +18740,7 @@
       <c r="J271" t="s">
         <v>1617</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18807,7 +18781,7 @@
       <c r="J272" t="s">
         <v>1617</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18825,7 +18799,7 @@
       <c r="R272" t="s">
         <v>1831</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18866,7 +18840,7 @@
       <c r="J273" t="s">
         <v>1617</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18910,7 +18884,7 @@
       <c r="J274" t="s">
         <v>1617</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18951,7 +18925,7 @@
       <c r="J275" t="s">
         <v>1617</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18992,7 +18966,7 @@
       <c r="J276" t="s">
         <v>1617</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19033,7 +19007,7 @@
       <c r="J277" t="s">
         <v>1617</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19074,7 +19048,7 @@
       <c r="J278" t="s">
         <v>1617</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19115,7 +19089,7 @@
       <c r="J279" t="s">
         <v>1617</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19156,7 +19130,7 @@
       <c r="J280" t="s">
         <v>1617</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19197,7 +19171,7 @@
       <c r="J281" t="s">
         <v>1617</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19238,7 +19212,7 @@
       <c r="J282" t="s">
         <v>1617</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19279,7 +19253,7 @@
       <c r="J283" t="s">
         <v>1617</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19320,7 +19294,7 @@
       <c r="J284" t="s">
         <v>1617</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19361,7 +19335,7 @@
       <c r="J285" t="s">
         <v>1617</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19402,7 +19376,7 @@
       <c r="J286" t="s">
         <v>1617</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19443,7 +19417,7 @@
       <c r="J287" t="s">
         <v>1617</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19484,7 +19458,7 @@
       <c r="J288" t="s">
         <v>1617</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19525,7 +19499,7 @@
       <c r="J289" t="s">
         <v>1617</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19566,7 +19540,7 @@
       <c r="J290" t="s">
         <v>1617</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19607,7 +19581,7 @@
       <c r="J291" t="s">
         <v>1617</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19648,7 +19622,7 @@
       <c r="J292" t="s">
         <v>1617</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19689,7 +19663,7 @@
       <c r="J293" t="s">
         <v>1617</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19730,7 +19704,7 @@
       <c r="J294" t="s">
         <v>1617</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19771,7 +19745,7 @@
       <c r="J295" t="s">
         <v>1617</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19789,7 +19763,7 @@
       <c r="R295" t="s">
         <v>1832</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19830,7 +19804,7 @@
       <c r="J296" t="s">
         <v>1617</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19848,7 +19822,7 @@
       <c r="R296" t="s">
         <v>1808</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19886,7 +19860,7 @@
       <c r="J297" t="s">
         <v>1617</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19927,7 +19901,7 @@
       <c r="J298" t="s">
         <v>1617</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19968,7 +19942,7 @@
       <c r="J299" t="s">
         <v>1618</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20009,7 +19983,7 @@
       <c r="J300" t="s">
         <v>1617</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20050,7 +20024,7 @@
       <c r="J301" t="s">
         <v>1617</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20888,7 +20862,7 @@
       <c r="R321" t="s">
         <v>1794</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21111,7 +21085,7 @@
       <c r="R326" t="s">
         <v>1833</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21946,7 +21920,7 @@
       <c r="R346" t="s">
         <v>1834</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (07/10/2026 14:48)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5711,16 +5711,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5736,7 +5728,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5744,30 +5736,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6067,73 +6041,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6168,7 +6142,7 @@
       <c r="J2" t="s">
         <v>1623</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6212,7 +6186,7 @@
       <c r="J3" t="s">
         <v>1623</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6256,7 +6230,7 @@
       <c r="J4" t="s">
         <v>1623</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6274,7 +6248,7 @@
       <c r="R4" t="s">
         <v>1798</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6312,7 +6286,7 @@
       <c r="J5" t="s">
         <v>1624</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6362,7 +6336,7 @@
       <c r="J6" t="s">
         <v>1623</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6409,7 +6383,7 @@
       <c r="J7" t="s">
         <v>1623</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6456,7 +6430,7 @@
       <c r="J8" t="s">
         <v>1623</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6503,7 +6477,7 @@
       <c r="J9" t="s">
         <v>1623</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6550,7 +6524,7 @@
       <c r="J10" t="s">
         <v>1623</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6597,7 +6571,7 @@
       <c r="J11" t="s">
         <v>1623</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6644,7 +6618,7 @@
       <c r="J12" t="s">
         <v>1623</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6688,7 +6662,7 @@
       <c r="J13" t="s">
         <v>1623</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6706,7 +6680,7 @@
       <c r="R13" t="s">
         <v>1799</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6744,7 +6718,7 @@
       <c r="J14" t="s">
         <v>1623</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6762,7 +6736,7 @@
       <c r="R14" t="s">
         <v>1800</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6803,7 +6777,7 @@
       <c r="J15" t="s">
         <v>1623</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6821,7 +6795,7 @@
       <c r="R15" t="s">
         <v>1800</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6862,7 +6836,7 @@
       <c r="J16" t="s">
         <v>1623</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6906,7 +6880,7 @@
       <c r="J17" t="s">
         <v>1623</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6950,7 +6924,7 @@
       <c r="J18" t="s">
         <v>1623</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6968,7 +6942,7 @@
       <c r="R18" t="s">
         <v>1801</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7009,7 +6983,7 @@
       <c r="J19" t="s">
         <v>1623</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7053,7 +7027,7 @@
       <c r="J20" t="s">
         <v>1623</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7097,7 +7071,7 @@
       <c r="J21" t="s">
         <v>1623</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7115,7 +7089,7 @@
       <c r="R21" t="s">
         <v>1800</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7156,7 +7130,7 @@
       <c r="J22" t="s">
         <v>1623</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7174,7 +7148,7 @@
       <c r="R22" t="s">
         <v>1802</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7215,7 +7189,7 @@
       <c r="J23" t="s">
         <v>1623</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7233,7 +7207,7 @@
       <c r="R23" t="s">
         <v>1803</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7274,7 +7248,7 @@
       <c r="J24" t="s">
         <v>1623</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7318,7 +7292,7 @@
       <c r="J25" t="s">
         <v>1623</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7359,7 +7333,7 @@
       <c r="J26" t="s">
         <v>1625</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7377,7 +7351,7 @@
       <c r="R26" t="s">
         <v>1804</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7415,7 +7389,7 @@
       <c r="J27" t="s">
         <v>1623</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7433,7 +7407,7 @@
       <c r="R27" t="s">
         <v>1805</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7474,7 +7448,7 @@
       <c r="J28" t="s">
         <v>1623</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7518,7 +7492,7 @@
       <c r="J29" t="s">
         <v>1623</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7562,7 +7536,7 @@
       <c r="J30" t="s">
         <v>1623</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7606,7 +7580,7 @@
       <c r="J31" t="s">
         <v>1623</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7624,7 +7598,7 @@
       <c r="R31" t="s">
         <v>1806</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7665,7 +7639,7 @@
       <c r="J32" t="s">
         <v>1623</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7709,7 +7683,7 @@
       <c r="J33" t="s">
         <v>1623</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7727,7 +7701,7 @@
       <c r="R33" t="s">
         <v>1807</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7768,7 +7742,7 @@
       <c r="J34" t="s">
         <v>1623</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7812,7 +7786,7 @@
       <c r="J35" t="s">
         <v>1623</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7830,7 +7804,7 @@
       <c r="R35" t="s">
         <v>1808</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7871,7 +7845,7 @@
       <c r="J36" t="s">
         <v>1623</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7889,7 +7863,7 @@
       <c r="R36" t="s">
         <v>1808</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7930,7 +7904,7 @@
       <c r="J37" t="s">
         <v>1623</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7948,7 +7922,7 @@
       <c r="R37" t="s">
         <v>1808</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7989,7 +7963,7 @@
       <c r="J38" t="s">
         <v>1623</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8007,7 +7981,7 @@
       <c r="R38" t="s">
         <v>1808</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8048,7 +8022,7 @@
       <c r="J39" t="s">
         <v>1623</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8066,7 +8040,7 @@
       <c r="R39" t="s">
         <v>1808</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8107,7 +8081,7 @@
       <c r="J40" t="s">
         <v>1623</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8125,7 +8099,7 @@
       <c r="R40" t="s">
         <v>1809</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8166,7 +8140,7 @@
       <c r="J41" t="s">
         <v>1623</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8184,7 +8158,7 @@
       <c r="R41" t="s">
         <v>1800</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8225,7 +8199,7 @@
       <c r="J42" t="s">
         <v>1623</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8243,7 +8217,7 @@
       <c r="R42" t="s">
         <v>1808</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8284,7 +8258,7 @@
       <c r="J43" t="s">
         <v>1623</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8328,7 +8302,7 @@
       <c r="J44" t="s">
         <v>1623</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8346,7 +8320,7 @@
       <c r="R44" t="s">
         <v>1810</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8387,7 +8361,7 @@
       <c r="J45" t="s">
         <v>1623</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8405,7 +8379,7 @@
       <c r="R45" t="s">
         <v>1811</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8443,7 +8417,7 @@
       <c r="J46" t="s">
         <v>1623</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8487,7 +8461,7 @@
       <c r="J47" t="s">
         <v>1623</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8505,7 +8479,7 @@
       <c r="R47" t="s">
         <v>1812</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8546,7 +8520,7 @@
       <c r="J48" t="s">
         <v>1623</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8590,7 +8564,7 @@
       <c r="J49" t="s">
         <v>1623</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8634,7 +8608,7 @@
       <c r="J50" t="s">
         <v>1623</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8678,7 +8652,7 @@
       <c r="J51" t="s">
         <v>1623</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8725,7 +8699,7 @@
       <c r="J52" t="s">
         <v>1623</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8769,7 +8743,7 @@
       <c r="J53" t="s">
         <v>1623</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8813,7 +8787,7 @@
       <c r="J54" t="s">
         <v>1623</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8857,7 +8831,7 @@
       <c r="J55" t="s">
         <v>1623</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8907,7 +8881,7 @@
       <c r="J56" t="s">
         <v>1623</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8960,7 +8934,7 @@
       <c r="J57" t="s">
         <v>1623</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9010,7 +8984,7 @@
       <c r="J58" t="s">
         <v>1623</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9060,7 +9034,7 @@
       <c r="J59" t="s">
         <v>1623</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9078,7 +9052,7 @@
       <c r="R59" t="s">
         <v>1813</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9119,7 +9093,7 @@
       <c r="J60" t="s">
         <v>1623</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9163,7 +9137,7 @@
       <c r="J61" t="s">
         <v>1623</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9207,7 +9181,7 @@
       <c r="J62" t="s">
         <v>1623</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9251,7 +9225,7 @@
       <c r="J63" t="s">
         <v>1623</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9295,7 +9269,7 @@
       <c r="J64" t="s">
         <v>1623</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9339,7 +9313,7 @@
       <c r="J65" t="s">
         <v>1623</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9386,7 +9360,7 @@
       <c r="J66" t="s">
         <v>1623</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9404,7 +9378,7 @@
       <c r="R66" t="s">
         <v>1814</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9442,7 +9416,7 @@
       <c r="J67" t="s">
         <v>1623</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9486,7 +9460,7 @@
       <c r="J68" t="s">
         <v>1623</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9501,7 +9475,7 @@
       <c r="O68" t="s">
         <v>1718</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9545,7 +9519,7 @@
       <c r="J69" t="s">
         <v>1625</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9589,7 +9563,7 @@
       <c r="J70" t="s">
         <v>1623</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9633,7 +9607,7 @@
       <c r="J71" t="s">
         <v>1623</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9677,7 +9651,7 @@
       <c r="J72" t="s">
         <v>1623</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9721,7 +9695,7 @@
       <c r="J73" t="s">
         <v>1623</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9765,7 +9739,7 @@
       <c r="J74" t="s">
         <v>1623</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9809,7 +9783,7 @@
       <c r="J75" t="s">
         <v>1623</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9853,7 +9827,7 @@
       <c r="J76" t="s">
         <v>1623</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9871,7 +9845,7 @@
       <c r="R76" t="s">
         <v>1815</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9909,7 +9883,7 @@
       <c r="J77" t="s">
         <v>1623</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9927,7 +9901,7 @@
       <c r="R77" t="s">
         <v>1815</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9965,7 +9939,7 @@
       <c r="J78" t="s">
         <v>1623</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9983,7 +9957,7 @@
       <c r="R78" t="s">
         <v>1815</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10021,7 +9995,7 @@
       <c r="J79" t="s">
         <v>1623</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10039,7 +10013,7 @@
       <c r="R79" t="s">
         <v>1815</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10077,7 +10051,7 @@
       <c r="J80" t="s">
         <v>1623</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10121,7 +10095,7 @@
       <c r="J81" t="s">
         <v>1623</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10165,7 +10139,7 @@
       <c r="J82" t="s">
         <v>1623</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10209,7 +10183,7 @@
       <c r="J83" t="s">
         <v>1623</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10253,7 +10227,7 @@
       <c r="J84" t="s">
         <v>1623</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10297,7 +10271,7 @@
       <c r="J85" t="s">
         <v>1623</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10315,7 +10289,7 @@
       <c r="R85" t="s">
         <v>1816</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10353,7 +10327,7 @@
       <c r="J86" t="s">
         <v>1623</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10397,7 +10371,7 @@
       <c r="J87" t="s">
         <v>1623</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10415,7 +10389,7 @@
       <c r="R87" t="s">
         <v>1817</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10453,7 +10427,7 @@
       <c r="J88" t="s">
         <v>1623</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10497,7 +10471,7 @@
       <c r="J89" t="s">
         <v>1623</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10515,7 +10489,7 @@
       <c r="R89" t="s">
         <v>1818</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10550,7 +10524,7 @@
       <c r="J90" t="s">
         <v>1623</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10568,7 +10542,7 @@
       <c r="R90" t="s">
         <v>1819</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10603,7 +10577,7 @@
       <c r="J91" t="s">
         <v>1623</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10621,7 +10595,7 @@
       <c r="R91" t="s">
         <v>1803</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10659,7 +10633,7 @@
       <c r="J92" t="s">
         <v>1623</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10680,7 +10654,7 @@
       <c r="R92" t="s">
         <v>1803</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10721,7 +10695,7 @@
       <c r="J93" t="s">
         <v>1623</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10762,7 +10736,7 @@
       <c r="J94" t="s">
         <v>1623</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10806,7 +10780,7 @@
       <c r="J95" t="s">
         <v>1623</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10850,7 +10824,7 @@
       <c r="J96" t="s">
         <v>1623</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10868,7 +10842,7 @@
       <c r="R96" t="s">
         <v>1820</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10909,7 +10883,7 @@
       <c r="J97" t="s">
         <v>1623</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10924,7 +10898,7 @@
       <c r="R97" t="s">
         <v>1820</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10965,7 +10939,7 @@
       <c r="J98" t="s">
         <v>1623</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10983,7 +10957,7 @@
       <c r="R98" t="s">
         <v>1821</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11021,7 +10995,7 @@
       <c r="J99" t="s">
         <v>1623</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11039,7 +11013,7 @@
       <c r="R99" t="s">
         <v>1822</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11077,7 +11051,7 @@
       <c r="J100" t="s">
         <v>1623</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11118,7 +11092,7 @@
       <c r="J101" t="s">
         <v>1623</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11159,7 +11133,7 @@
       <c r="J102" t="s">
         <v>1623</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11200,7 +11174,7 @@
       <c r="J103" t="s">
         <v>1623</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11241,7 +11215,7 @@
       <c r="J104" t="s">
         <v>1623</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11282,7 +11256,7 @@
       <c r="J105" t="s">
         <v>1623</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11323,7 +11297,7 @@
       <c r="J106" t="s">
         <v>1623</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11364,7 +11338,7 @@
       <c r="J107" t="s">
         <v>1623</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11405,7 +11379,7 @@
       <c r="J108" t="s">
         <v>1623</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11446,7 +11420,7 @@
       <c r="J109" t="s">
         <v>1623</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11499,7 +11473,7 @@
       <c r="J110" t="s">
         <v>1623</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11555,7 +11529,7 @@
       <c r="J111" t="s">
         <v>1623</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11573,7 +11547,7 @@
       <c r="R111" t="s">
         <v>1824</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11611,7 +11585,7 @@
       <c r="J112" t="s">
         <v>1623</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11670,7 +11644,7 @@
       <c r="J113" t="s">
         <v>1623</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11714,7 +11688,7 @@
       <c r="J114" t="s">
         <v>1623</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11758,7 +11732,7 @@
       <c r="J115" t="s">
         <v>1623</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11776,7 +11750,7 @@
       <c r="R115" t="s">
         <v>1826</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11817,7 +11791,7 @@
       <c r="J116" t="s">
         <v>1623</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11876,7 +11850,7 @@
       <c r="J117" t="s">
         <v>1623</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11920,7 +11894,7 @@
       <c r="J118" t="s">
         <v>1623</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11967,7 +11941,7 @@
       <c r="J119" t="s">
         <v>1623</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12008,7 +11982,7 @@
       <c r="J120" t="s">
         <v>1623</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12052,7 +12026,7 @@
       <c r="J121" t="s">
         <v>1623</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12099,7 +12073,7 @@
       <c r="J122" t="s">
         <v>1623</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12149,7 +12123,7 @@
       <c r="J123" t="s">
         <v>1623</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12193,7 +12167,7 @@
       <c r="J124" t="s">
         <v>1623</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12237,7 +12211,7 @@
       <c r="J125" t="s">
         <v>1623</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12255,7 +12229,7 @@
       <c r="R125" t="s">
         <v>1828</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12290,7 +12264,7 @@
       <c r="J126" t="s">
         <v>1623</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12308,7 +12282,7 @@
       <c r="R126" t="s">
         <v>1829</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12346,7 +12320,7 @@
       <c r="J127" t="s">
         <v>1623</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12402,7 +12376,7 @@
       <c r="J128" t="s">
         <v>1623</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12443,7 +12417,7 @@
       <c r="J129" t="s">
         <v>1623</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12484,7 +12458,7 @@
       <c r="J130" t="s">
         <v>1623</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12525,7 +12499,7 @@
       <c r="J131" t="s">
         <v>1623</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12569,7 +12543,7 @@
       <c r="J132" t="s">
         <v>1623</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12610,7 +12584,7 @@
       <c r="J133" t="s">
         <v>1623</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12628,7 +12602,7 @@
       <c r="R133" t="s">
         <v>1815</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12666,7 +12640,7 @@
       <c r="J134" t="s">
         <v>1623</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12684,7 +12658,7 @@
       <c r="R134" t="s">
         <v>1815</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12719,7 +12693,7 @@
       <c r="J135" t="s">
         <v>1623</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12760,7 +12734,7 @@
       <c r="J136" t="s">
         <v>1623</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12801,7 +12775,7 @@
       <c r="J137" t="s">
         <v>1623</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12842,7 +12816,7 @@
       <c r="J138" t="s">
         <v>1623</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12883,7 +12857,7 @@
       <c r="J139" t="s">
         <v>1623</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12930,7 +12904,7 @@
       <c r="J140" t="s">
         <v>1623</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12971,7 +12945,7 @@
       <c r="J141" t="s">
         <v>1623</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13012,7 +12986,7 @@
       <c r="J142" t="s">
         <v>1623</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13056,7 +13030,7 @@
       <c r="J143" t="s">
         <v>1623</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13074,7 +13048,7 @@
       <c r="R143" t="s">
         <v>1815</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13109,7 +13083,7 @@
       <c r="J144" t="s">
         <v>1623</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13127,7 +13101,7 @@
       <c r="R144" t="s">
         <v>1815</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13165,7 +13139,7 @@
       <c r="J145" t="s">
         <v>1623</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13183,7 +13157,7 @@
       <c r="R145" t="s">
         <v>1815</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13218,7 +13192,7 @@
       <c r="J146" t="s">
         <v>1623</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13236,7 +13210,7 @@
       <c r="R146" t="s">
         <v>1823</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13271,7 +13245,7 @@
       <c r="J147" t="s">
         <v>1623</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13289,7 +13263,7 @@
       <c r="R147" t="s">
         <v>1830</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13324,7 +13298,7 @@
       <c r="J148" t="s">
         <v>1623</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13365,7 +13339,7 @@
       <c r="J149" t="s">
         <v>1623</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13383,7 +13357,7 @@
       <c r="R149" t="s">
         <v>1815</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13418,7 +13392,7 @@
       <c r="J150" t="s">
         <v>1623</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13436,7 +13410,7 @@
       <c r="R150" t="s">
         <v>1815</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13474,7 +13448,7 @@
       <c r="J151" t="s">
         <v>1623</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13492,7 +13466,7 @@
       <c r="R151" t="s">
         <v>1831</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13527,7 +13501,7 @@
       <c r="J152" t="s">
         <v>1623</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13545,7 +13519,7 @@
       <c r="R152" t="s">
         <v>1832</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13580,7 +13554,7 @@
       <c r="J153" t="s">
         <v>1623</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13589,7 +13563,7 @@
       <c r="M153" t="s">
         <v>1709</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13630,7 +13604,7 @@
       <c r="J154" t="s">
         <v>1623</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13671,7 +13645,7 @@
       <c r="J155" t="s">
         <v>1623</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13712,7 +13686,7 @@
       <c r="J156" t="s">
         <v>1623</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13753,7 +13727,7 @@
       <c r="J157" t="s">
         <v>1623</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13794,7 +13768,7 @@
       <c r="J158" t="s">
         <v>1623</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13835,7 +13809,7 @@
       <c r="J159" t="s">
         <v>1623</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13876,7 +13850,7 @@
       <c r="J160" t="s">
         <v>1623</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13917,7 +13891,7 @@
       <c r="J161" t="s">
         <v>1623</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13958,7 +13932,7 @@
       <c r="J162" t="s">
         <v>1623</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13976,7 +13950,7 @@
       <c r="R162" t="s">
         <v>1818</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14011,7 +13985,7 @@
       <c r="J163" t="s">
         <v>1623</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14029,7 +14003,7 @@
       <c r="R163" t="s">
         <v>1815</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14064,7 +14038,7 @@
       <c r="J164" t="s">
         <v>1623</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14108,7 +14082,7 @@
       <c r="J165" t="s">
         <v>1623</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14149,7 +14123,7 @@
       <c r="J166" t="s">
         <v>1623</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14167,7 +14141,7 @@
       <c r="R166" t="s">
         <v>1833</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14202,7 +14176,7 @@
       <c r="J167" t="s">
         <v>1623</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14246,7 +14220,7 @@
       <c r="J168" t="s">
         <v>1623</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14290,7 +14264,7 @@
       <c r="J169" t="s">
         <v>1623</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14331,7 +14305,7 @@
       <c r="J170" t="s">
         <v>1623</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14372,7 +14346,7 @@
       <c r="J171" t="s">
         <v>1623</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14413,7 +14387,7 @@
       <c r="J172" t="s">
         <v>1623</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14454,7 +14428,7 @@
       <c r="J173" t="s">
         <v>1623</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14495,7 +14469,7 @@
       <c r="J174" t="s">
         <v>1623</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14536,7 +14510,7 @@
       <c r="J175" t="s">
         <v>1623</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14577,7 +14551,7 @@
       <c r="J176" t="s">
         <v>1623</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14618,7 +14592,7 @@
       <c r="J177" t="s">
         <v>1623</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14659,7 +14633,7 @@
       <c r="J178" t="s">
         <v>1623</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14677,7 +14651,7 @@
       <c r="R178" t="s">
         <v>1831</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14715,7 +14689,7 @@
       <c r="J179" t="s">
         <v>1623</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14724,7 +14698,7 @@
       <c r="M179" t="s">
         <v>1706</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14765,7 +14739,7 @@
       <c r="J180" t="s">
         <v>1623</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14806,7 +14780,7 @@
       <c r="J181" t="s">
         <v>1623</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14824,7 +14798,7 @@
       <c r="R181" t="s">
         <v>1815</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14859,7 +14833,7 @@
       <c r="J182" t="s">
         <v>1623</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14900,7 +14874,7 @@
       <c r="J183" t="s">
         <v>1623</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14941,7 +14915,7 @@
       <c r="J184" t="s">
         <v>1623</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14982,7 +14956,7 @@
       <c r="J185" t="s">
         <v>1623</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15023,7 +14997,7 @@
       <c r="J186" t="s">
         <v>1623</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15064,7 +15038,7 @@
       <c r="J187" t="s">
         <v>1623</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15105,7 +15079,7 @@
       <c r="J188" t="s">
         <v>1623</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15146,7 +15120,7 @@
       <c r="J189" t="s">
         <v>1623</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15187,7 +15161,7 @@
       <c r="J190" t="s">
         <v>1623</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15228,7 +15202,7 @@
       <c r="J191" t="s">
         <v>1623</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15269,7 +15243,7 @@
       <c r="J192" t="s">
         <v>1623</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15310,7 +15284,7 @@
       <c r="J193" t="s">
         <v>1623</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15351,7 +15325,7 @@
       <c r="J194" t="s">
         <v>1623</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15392,7 +15366,7 @@
       <c r="J195" t="s">
         <v>1623</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15410,7 +15384,7 @@
       <c r="R195" t="s">
         <v>1824</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15451,7 +15425,7 @@
       <c r="J196" t="s">
         <v>1623</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15469,7 +15443,7 @@
       <c r="R196" t="s">
         <v>1830</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15507,7 +15481,7 @@
       <c r="J197" t="s">
         <v>1623</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15548,7 +15522,7 @@
       <c r="J198" t="s">
         <v>1625</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15589,7 +15563,7 @@
       <c r="J199" t="s">
         <v>1624</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15630,7 +15604,7 @@
       <c r="J200" t="s">
         <v>1623</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15671,7 +15645,7 @@
       <c r="J201" t="s">
         <v>1623</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15712,7 +15686,7 @@
       <c r="J202" t="s">
         <v>1623</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15730,7 +15704,7 @@
       <c r="R202" t="s">
         <v>1815</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15768,7 +15742,7 @@
       <c r="J203" t="s">
         <v>1623</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15786,7 +15760,7 @@
       <c r="R203" t="s">
         <v>1823</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15821,7 +15795,7 @@
       <c r="J204" t="s">
         <v>1623</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15836,7 +15810,7 @@
       <c r="R204" t="s">
         <v>1834</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15874,7 +15848,7 @@
       <c r="J205" t="s">
         <v>1623</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15892,7 +15866,7 @@
       <c r="R205" t="s">
         <v>1835</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15930,7 +15904,7 @@
       <c r="J206" t="s">
         <v>1623</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15948,7 +15922,7 @@
       <c r="R206" t="s">
         <v>1803</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15983,7 +15957,7 @@
       <c r="J207" t="s">
         <v>1623</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16024,7 +15998,7 @@
       <c r="J208" t="s">
         <v>1623</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16065,7 +16039,7 @@
       <c r="J209" t="s">
         <v>1623</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16106,7 +16080,7 @@
       <c r="J210" t="s">
         <v>1623</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16147,7 +16121,7 @@
       <c r="J211" t="s">
         <v>1623</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16188,7 +16162,7 @@
       <c r="J212" t="s">
         <v>1623</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16229,7 +16203,7 @@
       <c r="J213" t="s">
         <v>1623</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16270,7 +16244,7 @@
       <c r="J214" t="s">
         <v>1623</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16288,7 +16262,7 @@
       <c r="R214" t="s">
         <v>1836</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16326,7 +16300,7 @@
       <c r="J215" t="s">
         <v>1623</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16367,7 +16341,7 @@
       <c r="J216" t="s">
         <v>1623</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16408,7 +16382,7 @@
       <c r="J217" t="s">
         <v>1623</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16449,7 +16423,7 @@
       <c r="J218" t="s">
         <v>1623</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16490,7 +16464,7 @@
       <c r="J219" t="s">
         <v>1623</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16531,7 +16505,7 @@
       <c r="J220" t="s">
         <v>1623</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16572,7 +16546,7 @@
       <c r="J221" t="s">
         <v>1623</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16613,7 +16587,7 @@
       <c r="J222" t="s">
         <v>1623</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16654,7 +16628,7 @@
       <c r="J223" t="s">
         <v>1623</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16695,7 +16669,7 @@
       <c r="J224" t="s">
         <v>1623</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16736,7 +16710,7 @@
       <c r="J225" t="s">
         <v>1623</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16777,7 +16751,7 @@
       <c r="J226" t="s">
         <v>1623</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16818,7 +16792,7 @@
       <c r="J227" t="s">
         <v>1623</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16859,7 +16833,7 @@
       <c r="J228" t="s">
         <v>1623</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16900,7 +16874,7 @@
       <c r="J229" t="s">
         <v>1623</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16941,7 +16915,7 @@
       <c r="J230" t="s">
         <v>1623</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16982,7 +16956,7 @@
       <c r="J231" t="s">
         <v>1623</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17023,7 +16997,7 @@
       <c r="J232" t="s">
         <v>1623</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17064,7 +17038,7 @@
       <c r="J233" t="s">
         <v>1623</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17105,7 +17079,7 @@
       <c r="J234" t="s">
         <v>1623</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17146,7 +17120,7 @@
       <c r="J235" t="s">
         <v>1623</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17187,7 +17161,7 @@
       <c r="J236" t="s">
         <v>1623</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17228,7 +17202,7 @@
       <c r="J237" t="s">
         <v>1623</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17269,7 +17243,7 @@
       <c r="J238" t="s">
         <v>1623</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17310,7 +17284,7 @@
       <c r="J239" t="s">
         <v>1623</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17328,7 +17302,7 @@
       <c r="R239" t="s">
         <v>1830</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17366,7 +17340,7 @@
       <c r="J240" t="s">
         <v>1623</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17407,7 +17381,7 @@
       <c r="J241" t="s">
         <v>1623</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17448,7 +17422,7 @@
       <c r="J242" t="s">
         <v>1623</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17466,7 +17440,7 @@
       <c r="R242" t="s">
         <v>1823</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17501,7 +17475,7 @@
       <c r="J243" t="s">
         <v>1623</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17542,7 +17516,7 @@
       <c r="J244" t="s">
         <v>1623</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17583,7 +17557,7 @@
       <c r="J245" t="s">
         <v>1623</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17624,7 +17598,7 @@
       <c r="J246" t="s">
         <v>1623</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17642,7 +17616,7 @@
       <c r="R246" t="s">
         <v>1803</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17680,7 +17654,7 @@
       <c r="J247" t="s">
         <v>1623</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17721,7 +17695,7 @@
       <c r="J248" t="s">
         <v>1623</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17762,7 +17736,7 @@
       <c r="J249" t="s">
         <v>1623</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17803,7 +17777,7 @@
       <c r="J250" t="s">
         <v>1623</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17844,7 +17818,7 @@
       <c r="J251" t="s">
         <v>1623</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17885,7 +17859,7 @@
       <c r="J252" t="s">
         <v>1623</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17926,7 +17900,7 @@
       <c r="J253" t="s">
         <v>1623</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17944,7 +17918,7 @@
       <c r="R253" t="s">
         <v>1833</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -17985,7 +17959,7 @@
       <c r="J254" t="s">
         <v>1623</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18026,7 +18000,7 @@
       <c r="J255" t="s">
         <v>1623</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18067,7 +18041,7 @@
       <c r="J256" t="s">
         <v>1623</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18076,7 +18050,7 @@
       <c r="M256" t="s">
         <v>1705</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18114,7 +18088,7 @@
       <c r="J257" t="s">
         <v>1623</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18123,7 +18097,7 @@
       <c r="M257" t="s">
         <v>1706</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18167,7 +18141,7 @@
       <c r="J258" t="s">
         <v>1623</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18185,7 +18159,7 @@
       <c r="R258" t="s">
         <v>1815</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18223,7 +18197,7 @@
       <c r="J259" t="s">
         <v>1623</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18241,7 +18215,7 @@
       <c r="R259" t="s">
         <v>1831</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18279,7 +18253,7 @@
       <c r="J260" t="s">
         <v>1623</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18288,7 +18262,7 @@
       <c r="M260" t="s">
         <v>1700</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18332,7 +18306,7 @@
       <c r="J261" t="s">
         <v>1623</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18350,7 +18324,7 @@
       <c r="R261" t="s">
         <v>1837</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18388,7 +18362,7 @@
       <c r="J262" t="s">
         <v>1623</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18406,7 +18380,7 @@
       <c r="R262" t="s">
         <v>1831</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18444,7 +18418,7 @@
       <c r="J263" t="s">
         <v>1623</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18453,7 +18427,7 @@
       <c r="M263" t="s">
         <v>1700</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18497,7 +18471,7 @@
       <c r="J264" t="s">
         <v>1623</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18538,7 +18512,7 @@
       <c r="J265" t="s">
         <v>1623</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18579,7 +18553,7 @@
       <c r="J266" t="s">
         <v>1623</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18620,7 +18594,7 @@
       <c r="J267" t="s">
         <v>1623</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18664,7 +18638,7 @@
       <c r="J268" t="s">
         <v>1623</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18705,7 +18679,7 @@
       <c r="J269" t="s">
         <v>1623</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18746,7 +18720,7 @@
       <c r="J270" t="s">
         <v>1623</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18787,7 +18761,7 @@
       <c r="J271" t="s">
         <v>1623</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18828,7 +18802,7 @@
       <c r="J272" t="s">
         <v>1623</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18846,7 +18820,7 @@
       <c r="R272" t="s">
         <v>1838</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18887,7 +18861,7 @@
       <c r="J273" t="s">
         <v>1623</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18931,7 +18905,7 @@
       <c r="J274" t="s">
         <v>1623</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18972,7 +18946,7 @@
       <c r="J275" t="s">
         <v>1623</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19013,7 +18987,7 @@
       <c r="J276" t="s">
         <v>1623</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19054,7 +19028,7 @@
       <c r="J277" t="s">
         <v>1623</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19095,7 +19069,7 @@
       <c r="J278" t="s">
         <v>1623</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19136,7 +19110,7 @@
       <c r="J279" t="s">
         <v>1623</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19177,7 +19151,7 @@
       <c r="J280" t="s">
         <v>1623</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19218,7 +19192,7 @@
       <c r="J281" t="s">
         <v>1623</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19259,7 +19233,7 @@
       <c r="J282" t="s">
         <v>1623</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19300,7 +19274,7 @@
       <c r="J283" t="s">
         <v>1623</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19341,7 +19315,7 @@
       <c r="J284" t="s">
         <v>1623</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19382,7 +19356,7 @@
       <c r="J285" t="s">
         <v>1623</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19423,7 +19397,7 @@
       <c r="J286" t="s">
         <v>1623</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19464,7 +19438,7 @@
       <c r="J287" t="s">
         <v>1623</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19505,7 +19479,7 @@
       <c r="J288" t="s">
         <v>1623</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19546,7 +19520,7 @@
       <c r="J289" t="s">
         <v>1623</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19587,7 +19561,7 @@
       <c r="J290" t="s">
         <v>1623</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19628,7 +19602,7 @@
       <c r="J291" t="s">
         <v>1623</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19669,7 +19643,7 @@
       <c r="J292" t="s">
         <v>1623</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19710,7 +19684,7 @@
       <c r="J293" t="s">
         <v>1623</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19751,7 +19725,7 @@
       <c r="J294" t="s">
         <v>1623</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19792,7 +19766,7 @@
       <c r="J295" t="s">
         <v>1623</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19810,7 +19784,7 @@
       <c r="R295" t="s">
         <v>1839</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19851,7 +19825,7 @@
       <c r="J296" t="s">
         <v>1623</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19869,7 +19843,7 @@
       <c r="R296" t="s">
         <v>1815</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19907,7 +19881,7 @@
       <c r="J297" t="s">
         <v>1623</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19948,7 +19922,7 @@
       <c r="J298" t="s">
         <v>1623</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19989,7 +19963,7 @@
       <c r="J299" t="s">
         <v>1624</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20030,7 +20004,7 @@
       <c r="J300" t="s">
         <v>1623</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20071,7 +20045,7 @@
       <c r="J301" t="s">
         <v>1623</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20909,7 +20883,7 @@
       <c r="R321" t="s">
         <v>1801</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21132,7 +21106,7 @@
       <c r="R326" t="s">
         <v>1840</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21967,7 +21941,7 @@
       <c r="R346" t="s">
         <v>1841</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Devolucoes: atualiza do Drive (planilha 'Devolucoes', aba DEVOLUCAO) apos checagem da RMA de setembro/2026 -- 409 itens, nenhuma linha nova de Consumiveis (CAT=C) pendente de auditoria desde a v4 (ver 00_Instrucoes/auditoria_consumiveis_devolucoes.md)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5711,8 +5711,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5728,7 +5736,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5736,12 +5744,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6041,73 +6067,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6142,7 +6168,7 @@
       <c r="J2" t="s">
         <v>1623</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6186,7 +6212,7 @@
       <c r="J3" t="s">
         <v>1623</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6230,7 +6256,7 @@
       <c r="J4" t="s">
         <v>1623</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6248,7 +6274,7 @@
       <c r="R4" t="s">
         <v>1798</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6286,7 +6312,7 @@
       <c r="J5" t="s">
         <v>1624</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6336,7 +6362,7 @@
       <c r="J6" t="s">
         <v>1623</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6383,7 +6409,7 @@
       <c r="J7" t="s">
         <v>1623</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6430,7 +6456,7 @@
       <c r="J8" t="s">
         <v>1623</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6477,7 +6503,7 @@
       <c r="J9" t="s">
         <v>1623</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6524,7 +6550,7 @@
       <c r="J10" t="s">
         <v>1623</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6571,7 +6597,7 @@
       <c r="J11" t="s">
         <v>1623</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6618,7 +6644,7 @@
       <c r="J12" t="s">
         <v>1623</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6662,7 +6688,7 @@
       <c r="J13" t="s">
         <v>1623</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6680,7 +6706,7 @@
       <c r="R13" t="s">
         <v>1799</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6718,7 +6744,7 @@
       <c r="J14" t="s">
         <v>1623</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6736,7 +6762,7 @@
       <c r="R14" t="s">
         <v>1800</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6777,7 +6803,7 @@
       <c r="J15" t="s">
         <v>1623</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6795,7 +6821,7 @@
       <c r="R15" t="s">
         <v>1800</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6836,7 +6862,7 @@
       <c r="J16" t="s">
         <v>1623</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6880,7 +6906,7 @@
       <c r="J17" t="s">
         <v>1623</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6924,7 +6950,7 @@
       <c r="J18" t="s">
         <v>1623</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6942,7 +6968,7 @@
       <c r="R18" t="s">
         <v>1801</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6983,7 +7009,7 @@
       <c r="J19" t="s">
         <v>1623</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7027,7 +7053,7 @@
       <c r="J20" t="s">
         <v>1623</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7071,7 +7097,7 @@
       <c r="J21" t="s">
         <v>1623</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7089,7 +7115,7 @@
       <c r="R21" t="s">
         <v>1800</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7130,7 +7156,7 @@
       <c r="J22" t="s">
         <v>1623</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7148,7 +7174,7 @@
       <c r="R22" t="s">
         <v>1802</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7189,7 +7215,7 @@
       <c r="J23" t="s">
         <v>1623</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7207,7 +7233,7 @@
       <c r="R23" t="s">
         <v>1803</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7248,7 +7274,7 @@
       <c r="J24" t="s">
         <v>1623</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7292,7 +7318,7 @@
       <c r="J25" t="s">
         <v>1623</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7333,7 +7359,7 @@
       <c r="J26" t="s">
         <v>1625</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7351,7 +7377,7 @@
       <c r="R26" t="s">
         <v>1804</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7389,7 +7415,7 @@
       <c r="J27" t="s">
         <v>1623</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7407,7 +7433,7 @@
       <c r="R27" t="s">
         <v>1805</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7448,7 +7474,7 @@
       <c r="J28" t="s">
         <v>1623</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7492,7 +7518,7 @@
       <c r="J29" t="s">
         <v>1623</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7536,7 +7562,7 @@
       <c r="J30" t="s">
         <v>1623</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7580,7 +7606,7 @@
       <c r="J31" t="s">
         <v>1623</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7598,7 +7624,7 @@
       <c r="R31" t="s">
         <v>1806</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7639,7 +7665,7 @@
       <c r="J32" t="s">
         <v>1623</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7683,7 +7709,7 @@
       <c r="J33" t="s">
         <v>1623</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7701,7 +7727,7 @@
       <c r="R33" t="s">
         <v>1807</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7742,7 +7768,7 @@
       <c r="J34" t="s">
         <v>1623</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7786,7 +7812,7 @@
       <c r="J35" t="s">
         <v>1623</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7804,7 +7830,7 @@
       <c r="R35" t="s">
         <v>1808</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7845,7 +7871,7 @@
       <c r="J36" t="s">
         <v>1623</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7863,7 +7889,7 @@
       <c r="R36" t="s">
         <v>1808</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7904,7 +7930,7 @@
       <c r="J37" t="s">
         <v>1623</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7922,7 +7948,7 @@
       <c r="R37" t="s">
         <v>1808</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7963,7 +7989,7 @@
       <c r="J38" t="s">
         <v>1623</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7981,7 +8007,7 @@
       <c r="R38" t="s">
         <v>1808</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8022,7 +8048,7 @@
       <c r="J39" t="s">
         <v>1623</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8040,7 +8066,7 @@
       <c r="R39" t="s">
         <v>1808</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8081,7 +8107,7 @@
       <c r="J40" t="s">
         <v>1623</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8099,7 +8125,7 @@
       <c r="R40" t="s">
         <v>1809</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8140,7 +8166,7 @@
       <c r="J41" t="s">
         <v>1623</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8158,7 +8184,7 @@
       <c r="R41" t="s">
         <v>1800</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8199,7 +8225,7 @@
       <c r="J42" t="s">
         <v>1623</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8217,7 +8243,7 @@
       <c r="R42" t="s">
         <v>1808</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8258,7 +8284,7 @@
       <c r="J43" t="s">
         <v>1623</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8302,7 +8328,7 @@
       <c r="J44" t="s">
         <v>1623</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8320,7 +8346,7 @@
       <c r="R44" t="s">
         <v>1810</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8361,7 +8387,7 @@
       <c r="J45" t="s">
         <v>1623</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8379,7 +8405,7 @@
       <c r="R45" t="s">
         <v>1811</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8417,7 +8443,7 @@
       <c r="J46" t="s">
         <v>1623</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8461,7 +8487,7 @@
       <c r="J47" t="s">
         <v>1623</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8479,7 +8505,7 @@
       <c r="R47" t="s">
         <v>1812</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8520,7 +8546,7 @@
       <c r="J48" t="s">
         <v>1623</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8564,7 +8590,7 @@
       <c r="J49" t="s">
         <v>1623</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8608,7 +8634,7 @@
       <c r="J50" t="s">
         <v>1623</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8652,7 +8678,7 @@
       <c r="J51" t="s">
         <v>1623</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8699,7 +8725,7 @@
       <c r="J52" t="s">
         <v>1623</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8743,7 +8769,7 @@
       <c r="J53" t="s">
         <v>1623</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8787,7 +8813,7 @@
       <c r="J54" t="s">
         <v>1623</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8831,7 +8857,7 @@
       <c r="J55" t="s">
         <v>1623</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8881,7 +8907,7 @@
       <c r="J56" t="s">
         <v>1623</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8934,7 +8960,7 @@
       <c r="J57" t="s">
         <v>1623</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8984,7 +9010,7 @@
       <c r="J58" t="s">
         <v>1623</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9034,7 +9060,7 @@
       <c r="J59" t="s">
         <v>1623</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9052,7 +9078,7 @@
       <c r="R59" t="s">
         <v>1813</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9093,7 +9119,7 @@
       <c r="J60" t="s">
         <v>1623</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9137,7 +9163,7 @@
       <c r="J61" t="s">
         <v>1623</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9181,7 +9207,7 @@
       <c r="J62" t="s">
         <v>1623</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9225,7 +9251,7 @@
       <c r="J63" t="s">
         <v>1623</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9269,7 +9295,7 @@
       <c r="J64" t="s">
         <v>1623</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9313,7 +9339,7 @@
       <c r="J65" t="s">
         <v>1623</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9360,7 +9386,7 @@
       <c r="J66" t="s">
         <v>1623</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9378,7 +9404,7 @@
       <c r="R66" t="s">
         <v>1814</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9416,7 +9442,7 @@
       <c r="J67" t="s">
         <v>1623</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9460,7 +9486,7 @@
       <c r="J68" t="s">
         <v>1623</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9475,7 +9501,7 @@
       <c r="O68" t="s">
         <v>1718</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9519,7 +9545,7 @@
       <c r="J69" t="s">
         <v>1625</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9563,7 +9589,7 @@
       <c r="J70" t="s">
         <v>1623</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9607,7 +9633,7 @@
       <c r="J71" t="s">
         <v>1623</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9651,7 +9677,7 @@
       <c r="J72" t="s">
         <v>1623</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9695,7 +9721,7 @@
       <c r="J73" t="s">
         <v>1623</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9739,7 +9765,7 @@
       <c r="J74" t="s">
         <v>1623</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9783,7 +9809,7 @@
       <c r="J75" t="s">
         <v>1623</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9827,7 +9853,7 @@
       <c r="J76" t="s">
         <v>1623</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9845,7 +9871,7 @@
       <c r="R76" t="s">
         <v>1815</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9883,7 +9909,7 @@
       <c r="J77" t="s">
         <v>1623</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9901,7 +9927,7 @@
       <c r="R77" t="s">
         <v>1815</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9939,7 +9965,7 @@
       <c r="J78" t="s">
         <v>1623</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9957,7 +9983,7 @@
       <c r="R78" t="s">
         <v>1815</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9995,7 +10021,7 @@
       <c r="J79" t="s">
         <v>1623</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10013,7 +10039,7 @@
       <c r="R79" t="s">
         <v>1815</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10051,7 +10077,7 @@
       <c r="J80" t="s">
         <v>1623</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10095,7 +10121,7 @@
       <c r="J81" t="s">
         <v>1623</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10139,7 +10165,7 @@
       <c r="J82" t="s">
         <v>1623</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10183,7 +10209,7 @@
       <c r="J83" t="s">
         <v>1623</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10227,7 +10253,7 @@
       <c r="J84" t="s">
         <v>1623</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10271,7 +10297,7 @@
       <c r="J85" t="s">
         <v>1623</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10289,7 +10315,7 @@
       <c r="R85" t="s">
         <v>1816</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10327,7 +10353,7 @@
       <c r="J86" t="s">
         <v>1623</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10371,7 +10397,7 @@
       <c r="J87" t="s">
         <v>1623</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10389,7 +10415,7 @@
       <c r="R87" t="s">
         <v>1817</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10427,7 +10453,7 @@
       <c r="J88" t="s">
         <v>1623</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10471,7 +10497,7 @@
       <c r="J89" t="s">
         <v>1623</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10489,7 +10515,7 @@
       <c r="R89" t="s">
         <v>1818</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10524,7 +10550,7 @@
       <c r="J90" t="s">
         <v>1623</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10542,7 +10568,7 @@
       <c r="R90" t="s">
         <v>1819</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10577,7 +10603,7 @@
       <c r="J91" t="s">
         <v>1623</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10595,7 +10621,7 @@
       <c r="R91" t="s">
         <v>1803</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10633,7 +10659,7 @@
       <c r="J92" t="s">
         <v>1623</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10654,7 +10680,7 @@
       <c r="R92" t="s">
         <v>1803</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10695,7 +10721,7 @@
       <c r="J93" t="s">
         <v>1623</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10736,7 +10762,7 @@
       <c r="J94" t="s">
         <v>1623</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10780,7 +10806,7 @@
       <c r="J95" t="s">
         <v>1623</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10824,7 +10850,7 @@
       <c r="J96" t="s">
         <v>1623</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10842,7 +10868,7 @@
       <c r="R96" t="s">
         <v>1820</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10883,7 +10909,7 @@
       <c r="J97" t="s">
         <v>1623</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10898,7 +10924,7 @@
       <c r="R97" t="s">
         <v>1820</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10939,7 +10965,7 @@
       <c r="J98" t="s">
         <v>1623</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10957,7 +10983,7 @@
       <c r="R98" t="s">
         <v>1821</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10995,7 +11021,7 @@
       <c r="J99" t="s">
         <v>1623</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11013,7 +11039,7 @@
       <c r="R99" t="s">
         <v>1822</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11051,7 +11077,7 @@
       <c r="J100" t="s">
         <v>1623</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11092,7 +11118,7 @@
       <c r="J101" t="s">
         <v>1623</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11133,7 +11159,7 @@
       <c r="J102" t="s">
         <v>1623</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11174,7 +11200,7 @@
       <c r="J103" t="s">
         <v>1623</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11215,7 +11241,7 @@
       <c r="J104" t="s">
         <v>1623</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11256,7 +11282,7 @@
       <c r="J105" t="s">
         <v>1623</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11297,7 +11323,7 @@
       <c r="J106" t="s">
         <v>1623</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11338,7 +11364,7 @@
       <c r="J107" t="s">
         <v>1623</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11379,7 +11405,7 @@
       <c r="J108" t="s">
         <v>1623</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11420,7 +11446,7 @@
       <c r="J109" t="s">
         <v>1623</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11473,7 +11499,7 @@
       <c r="J110" t="s">
         <v>1623</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11529,7 +11555,7 @@
       <c r="J111" t="s">
         <v>1623</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11547,7 +11573,7 @@
       <c r="R111" t="s">
         <v>1824</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11585,7 +11611,7 @@
       <c r="J112" t="s">
         <v>1623</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11644,7 +11670,7 @@
       <c r="J113" t="s">
         <v>1623</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11688,7 +11714,7 @@
       <c r="J114" t="s">
         <v>1623</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11732,7 +11758,7 @@
       <c r="J115" t="s">
         <v>1623</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11750,7 +11776,7 @@
       <c r="R115" t="s">
         <v>1826</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11791,7 +11817,7 @@
       <c r="J116" t="s">
         <v>1623</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11850,7 +11876,7 @@
       <c r="J117" t="s">
         <v>1623</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11894,7 +11920,7 @@
       <c r="J118" t="s">
         <v>1623</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11941,7 +11967,7 @@
       <c r="J119" t="s">
         <v>1623</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11982,7 +12008,7 @@
       <c r="J120" t="s">
         <v>1623</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12026,7 +12052,7 @@
       <c r="J121" t="s">
         <v>1623</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12073,7 +12099,7 @@
       <c r="J122" t="s">
         <v>1623</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12123,7 +12149,7 @@
       <c r="J123" t="s">
         <v>1623</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12167,7 +12193,7 @@
       <c r="J124" t="s">
         <v>1623</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12211,7 +12237,7 @@
       <c r="J125" t="s">
         <v>1623</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12229,7 +12255,7 @@
       <c r="R125" t="s">
         <v>1828</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12264,7 +12290,7 @@
       <c r="J126" t="s">
         <v>1623</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12282,7 +12308,7 @@
       <c r="R126" t="s">
         <v>1829</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12320,7 +12346,7 @@
       <c r="J127" t="s">
         <v>1623</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12376,7 +12402,7 @@
       <c r="J128" t="s">
         <v>1623</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12417,7 +12443,7 @@
       <c r="J129" t="s">
         <v>1623</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12458,7 +12484,7 @@
       <c r="J130" t="s">
         <v>1623</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12499,7 +12525,7 @@
       <c r="J131" t="s">
         <v>1623</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12543,7 +12569,7 @@
       <c r="J132" t="s">
         <v>1623</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12584,7 +12610,7 @@
       <c r="J133" t="s">
         <v>1623</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12602,7 +12628,7 @@
       <c r="R133" t="s">
         <v>1815</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12640,7 +12666,7 @@
       <c r="J134" t="s">
         <v>1623</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12658,7 +12684,7 @@
       <c r="R134" t="s">
         <v>1815</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12693,7 +12719,7 @@
       <c r="J135" t="s">
         <v>1623</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12734,7 +12760,7 @@
       <c r="J136" t="s">
         <v>1623</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12775,7 +12801,7 @@
       <c r="J137" t="s">
         <v>1623</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12816,7 +12842,7 @@
       <c r="J138" t="s">
         <v>1623</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12857,7 +12883,7 @@
       <c r="J139" t="s">
         <v>1623</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12904,7 +12930,7 @@
       <c r="J140" t="s">
         <v>1623</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12945,7 +12971,7 @@
       <c r="J141" t="s">
         <v>1623</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12986,7 +13012,7 @@
       <c r="J142" t="s">
         <v>1623</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13030,7 +13056,7 @@
       <c r="J143" t="s">
         <v>1623</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13048,7 +13074,7 @@
       <c r="R143" t="s">
         <v>1815</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13083,7 +13109,7 @@
       <c r="J144" t="s">
         <v>1623</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13101,7 +13127,7 @@
       <c r="R144" t="s">
         <v>1815</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13139,7 +13165,7 @@
       <c r="J145" t="s">
         <v>1623</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13157,7 +13183,7 @@
       <c r="R145" t="s">
         <v>1815</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13192,7 +13218,7 @@
       <c r="J146" t="s">
         <v>1623</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13210,7 +13236,7 @@
       <c r="R146" t="s">
         <v>1823</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13245,7 +13271,7 @@
       <c r="J147" t="s">
         <v>1623</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13263,7 +13289,7 @@
       <c r="R147" t="s">
         <v>1830</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13298,7 +13324,7 @@
       <c r="J148" t="s">
         <v>1623</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13339,7 +13365,7 @@
       <c r="J149" t="s">
         <v>1623</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13357,7 +13383,7 @@
       <c r="R149" t="s">
         <v>1815</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13392,7 +13418,7 @@
       <c r="J150" t="s">
         <v>1623</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13410,7 +13436,7 @@
       <c r="R150" t="s">
         <v>1815</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13448,7 +13474,7 @@
       <c r="J151" t="s">
         <v>1623</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13466,7 +13492,7 @@
       <c r="R151" t="s">
         <v>1831</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13501,7 +13527,7 @@
       <c r="J152" t="s">
         <v>1623</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13519,7 +13545,7 @@
       <c r="R152" t="s">
         <v>1832</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13554,7 +13580,7 @@
       <c r="J153" t="s">
         <v>1623</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13563,7 +13589,7 @@
       <c r="M153" t="s">
         <v>1709</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13604,7 +13630,7 @@
       <c r="J154" t="s">
         <v>1623</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13645,7 +13671,7 @@
       <c r="J155" t="s">
         <v>1623</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13686,7 +13712,7 @@
       <c r="J156" t="s">
         <v>1623</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13727,7 +13753,7 @@
       <c r="J157" t="s">
         <v>1623</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13768,7 +13794,7 @@
       <c r="J158" t="s">
         <v>1623</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13809,7 +13835,7 @@
       <c r="J159" t="s">
         <v>1623</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13850,7 +13876,7 @@
       <c r="J160" t="s">
         <v>1623</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13891,7 +13917,7 @@
       <c r="J161" t="s">
         <v>1623</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13932,7 +13958,7 @@
       <c r="J162" t="s">
         <v>1623</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13950,7 +13976,7 @@
       <c r="R162" t="s">
         <v>1818</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13985,7 +14011,7 @@
       <c r="J163" t="s">
         <v>1623</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14003,7 +14029,7 @@
       <c r="R163" t="s">
         <v>1815</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14038,7 +14064,7 @@
       <c r="J164" t="s">
         <v>1623</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14082,7 +14108,7 @@
       <c r="J165" t="s">
         <v>1623</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14123,7 +14149,7 @@
       <c r="J166" t="s">
         <v>1623</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14141,7 +14167,7 @@
       <c r="R166" t="s">
         <v>1833</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14176,7 +14202,7 @@
       <c r="J167" t="s">
         <v>1623</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14220,7 +14246,7 @@
       <c r="J168" t="s">
         <v>1623</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14264,7 +14290,7 @@
       <c r="J169" t="s">
         <v>1623</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14305,7 +14331,7 @@
       <c r="J170" t="s">
         <v>1623</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14346,7 +14372,7 @@
       <c r="J171" t="s">
         <v>1623</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14387,7 +14413,7 @@
       <c r="J172" t="s">
         <v>1623</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14428,7 +14454,7 @@
       <c r="J173" t="s">
         <v>1623</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14469,7 +14495,7 @@
       <c r="J174" t="s">
         <v>1623</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14510,7 +14536,7 @@
       <c r="J175" t="s">
         <v>1623</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14551,7 +14577,7 @@
       <c r="J176" t="s">
         <v>1623</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14592,7 +14618,7 @@
       <c r="J177" t="s">
         <v>1623</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14633,7 +14659,7 @@
       <c r="J178" t="s">
         <v>1623</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14651,7 +14677,7 @@
       <c r="R178" t="s">
         <v>1831</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14689,7 +14715,7 @@
       <c r="J179" t="s">
         <v>1623</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14698,7 +14724,7 @@
       <c r="M179" t="s">
         <v>1706</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14739,7 +14765,7 @@
       <c r="J180" t="s">
         <v>1623</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14780,7 +14806,7 @@
       <c r="J181" t="s">
         <v>1623</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14798,7 +14824,7 @@
       <c r="R181" t="s">
         <v>1815</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14833,7 +14859,7 @@
       <c r="J182" t="s">
         <v>1623</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14874,7 +14900,7 @@
       <c r="J183" t="s">
         <v>1623</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14915,7 +14941,7 @@
       <c r="J184" t="s">
         <v>1623</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14956,7 +14982,7 @@
       <c r="J185" t="s">
         <v>1623</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14997,7 +15023,7 @@
       <c r="J186" t="s">
         <v>1623</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15038,7 +15064,7 @@
       <c r="J187" t="s">
         <v>1623</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15079,7 +15105,7 @@
       <c r="J188" t="s">
         <v>1623</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15120,7 +15146,7 @@
       <c r="J189" t="s">
         <v>1623</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15161,7 +15187,7 @@
       <c r="J190" t="s">
         <v>1623</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15202,7 +15228,7 @@
       <c r="J191" t="s">
         <v>1623</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15243,7 +15269,7 @@
       <c r="J192" t="s">
         <v>1623</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15284,7 +15310,7 @@
       <c r="J193" t="s">
         <v>1623</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15325,7 +15351,7 @@
       <c r="J194" t="s">
         <v>1623</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15366,7 +15392,7 @@
       <c r="J195" t="s">
         <v>1623</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15384,7 +15410,7 @@
       <c r="R195" t="s">
         <v>1824</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15425,7 +15451,7 @@
       <c r="J196" t="s">
         <v>1623</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15443,7 +15469,7 @@
       <c r="R196" t="s">
         <v>1830</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15481,7 +15507,7 @@
       <c r="J197" t="s">
         <v>1623</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15522,7 +15548,7 @@
       <c r="J198" t="s">
         <v>1625</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15563,7 +15589,7 @@
       <c r="J199" t="s">
         <v>1624</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15604,7 +15630,7 @@
       <c r="J200" t="s">
         <v>1623</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15645,7 +15671,7 @@
       <c r="J201" t="s">
         <v>1623</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15686,7 +15712,7 @@
       <c r="J202" t="s">
         <v>1623</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15704,7 +15730,7 @@
       <c r="R202" t="s">
         <v>1815</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15742,7 +15768,7 @@
       <c r="J203" t="s">
         <v>1623</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15760,7 +15786,7 @@
       <c r="R203" t="s">
         <v>1823</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15795,7 +15821,7 @@
       <c r="J204" t="s">
         <v>1623</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15810,7 +15836,7 @@
       <c r="R204" t="s">
         <v>1834</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15848,7 +15874,7 @@
       <c r="J205" t="s">
         <v>1623</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15866,7 +15892,7 @@
       <c r="R205" t="s">
         <v>1835</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15904,7 +15930,7 @@
       <c r="J206" t="s">
         <v>1623</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15922,7 +15948,7 @@
       <c r="R206" t="s">
         <v>1803</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15957,7 +15983,7 @@
       <c r="J207" t="s">
         <v>1623</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15998,7 +16024,7 @@
       <c r="J208" t="s">
         <v>1623</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16039,7 +16065,7 @@
       <c r="J209" t="s">
         <v>1623</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16080,7 +16106,7 @@
       <c r="J210" t="s">
         <v>1623</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16121,7 +16147,7 @@
       <c r="J211" t="s">
         <v>1623</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16162,7 +16188,7 @@
       <c r="J212" t="s">
         <v>1623</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16203,7 +16229,7 @@
       <c r="J213" t="s">
         <v>1623</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16244,7 +16270,7 @@
       <c r="J214" t="s">
         <v>1623</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16262,7 +16288,7 @@
       <c r="R214" t="s">
         <v>1836</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16300,7 +16326,7 @@
       <c r="J215" t="s">
         <v>1623</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16341,7 +16367,7 @@
       <c r="J216" t="s">
         <v>1623</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16382,7 +16408,7 @@
       <c r="J217" t="s">
         <v>1623</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16423,7 +16449,7 @@
       <c r="J218" t="s">
         <v>1623</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16464,7 +16490,7 @@
       <c r="J219" t="s">
         <v>1623</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16505,7 +16531,7 @@
       <c r="J220" t="s">
         <v>1623</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16546,7 +16572,7 @@
       <c r="J221" t="s">
         <v>1623</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16587,7 +16613,7 @@
       <c r="J222" t="s">
         <v>1623</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16628,7 +16654,7 @@
       <c r="J223" t="s">
         <v>1623</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16669,7 +16695,7 @@
       <c r="J224" t="s">
         <v>1623</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16710,7 +16736,7 @@
       <c r="J225" t="s">
         <v>1623</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16751,7 +16777,7 @@
       <c r="J226" t="s">
         <v>1623</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16792,7 +16818,7 @@
       <c r="J227" t="s">
         <v>1623</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16833,7 +16859,7 @@
       <c r="J228" t="s">
         <v>1623</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16874,7 +16900,7 @@
       <c r="J229" t="s">
         <v>1623</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16915,7 +16941,7 @@
       <c r="J230" t="s">
         <v>1623</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16956,7 +16982,7 @@
       <c r="J231" t="s">
         <v>1623</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16997,7 +17023,7 @@
       <c r="J232" t="s">
         <v>1623</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17038,7 +17064,7 @@
       <c r="J233" t="s">
         <v>1623</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17079,7 +17105,7 @@
       <c r="J234" t="s">
         <v>1623</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17120,7 +17146,7 @@
       <c r="J235" t="s">
         <v>1623</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17161,7 +17187,7 @@
       <c r="J236" t="s">
         <v>1623</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17202,7 +17228,7 @@
       <c r="J237" t="s">
         <v>1623</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17243,7 +17269,7 @@
       <c r="J238" t="s">
         <v>1623</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17284,7 +17310,7 @@
       <c r="J239" t="s">
         <v>1623</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17302,7 +17328,7 @@
       <c r="R239" t="s">
         <v>1830</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17340,7 +17366,7 @@
       <c r="J240" t="s">
         <v>1623</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17381,7 +17407,7 @@
       <c r="J241" t="s">
         <v>1623</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17422,7 +17448,7 @@
       <c r="J242" t="s">
         <v>1623</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17440,7 +17466,7 @@
       <c r="R242" t="s">
         <v>1823</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17475,7 +17501,7 @@
       <c r="J243" t="s">
         <v>1623</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17516,7 +17542,7 @@
       <c r="J244" t="s">
         <v>1623</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17557,7 +17583,7 @@
       <c r="J245" t="s">
         <v>1623</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17598,7 +17624,7 @@
       <c r="J246" t="s">
         <v>1623</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17616,7 +17642,7 @@
       <c r="R246" t="s">
         <v>1803</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17654,7 +17680,7 @@
       <c r="J247" t="s">
         <v>1623</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17695,7 +17721,7 @@
       <c r="J248" t="s">
         <v>1623</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17736,7 +17762,7 @@
       <c r="J249" t="s">
         <v>1623</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17777,7 +17803,7 @@
       <c r="J250" t="s">
         <v>1623</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17818,7 +17844,7 @@
       <c r="J251" t="s">
         <v>1623</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17859,7 +17885,7 @@
       <c r="J252" t="s">
         <v>1623</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17900,7 +17926,7 @@
       <c r="J253" t="s">
         <v>1623</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17918,7 +17944,7 @@
       <c r="R253" t="s">
         <v>1833</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -17959,7 +17985,7 @@
       <c r="J254" t="s">
         <v>1623</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18000,7 +18026,7 @@
       <c r="J255" t="s">
         <v>1623</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18041,7 +18067,7 @@
       <c r="J256" t="s">
         <v>1623</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18050,7 +18076,7 @@
       <c r="M256" t="s">
         <v>1705</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18088,7 +18114,7 @@
       <c r="J257" t="s">
         <v>1623</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18097,7 +18123,7 @@
       <c r="M257" t="s">
         <v>1706</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18141,7 +18167,7 @@
       <c r="J258" t="s">
         <v>1623</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18159,7 +18185,7 @@
       <c r="R258" t="s">
         <v>1815</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18197,7 +18223,7 @@
       <c r="J259" t="s">
         <v>1623</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18215,7 +18241,7 @@
       <c r="R259" t="s">
         <v>1831</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18253,7 +18279,7 @@
       <c r="J260" t="s">
         <v>1623</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18262,7 +18288,7 @@
       <c r="M260" t="s">
         <v>1700</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18306,7 +18332,7 @@
       <c r="J261" t="s">
         <v>1623</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18324,7 +18350,7 @@
       <c r="R261" t="s">
         <v>1837</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18362,7 +18388,7 @@
       <c r="J262" t="s">
         <v>1623</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18380,7 +18406,7 @@
       <c r="R262" t="s">
         <v>1831</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18418,7 +18444,7 @@
       <c r="J263" t="s">
         <v>1623</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18427,7 +18453,7 @@
       <c r="M263" t="s">
         <v>1700</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18471,7 +18497,7 @@
       <c r="J264" t="s">
         <v>1623</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18512,7 +18538,7 @@
       <c r="J265" t="s">
         <v>1623</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18553,7 +18579,7 @@
       <c r="J266" t="s">
         <v>1623</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18594,7 +18620,7 @@
       <c r="J267" t="s">
         <v>1623</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18638,7 +18664,7 @@
       <c r="J268" t="s">
         <v>1623</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18679,7 +18705,7 @@
       <c r="J269" t="s">
         <v>1623</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18720,7 +18746,7 @@
       <c r="J270" t="s">
         <v>1623</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18761,7 +18787,7 @@
       <c r="J271" t="s">
         <v>1623</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18802,7 +18828,7 @@
       <c r="J272" t="s">
         <v>1623</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18820,7 +18846,7 @@
       <c r="R272" t="s">
         <v>1838</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18861,7 +18887,7 @@
       <c r="J273" t="s">
         <v>1623</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18905,7 +18931,7 @@
       <c r="J274" t="s">
         <v>1623</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18946,7 +18972,7 @@
       <c r="J275" t="s">
         <v>1623</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18987,7 +19013,7 @@
       <c r="J276" t="s">
         <v>1623</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19028,7 +19054,7 @@
       <c r="J277" t="s">
         <v>1623</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19069,7 +19095,7 @@
       <c r="J278" t="s">
         <v>1623</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19110,7 +19136,7 @@
       <c r="J279" t="s">
         <v>1623</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19151,7 +19177,7 @@
       <c r="J280" t="s">
         <v>1623</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19192,7 +19218,7 @@
       <c r="J281" t="s">
         <v>1623</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19233,7 +19259,7 @@
       <c r="J282" t="s">
         <v>1623</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19274,7 +19300,7 @@
       <c r="J283" t="s">
         <v>1623</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19315,7 +19341,7 @@
       <c r="J284" t="s">
         <v>1623</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19356,7 +19382,7 @@
       <c r="J285" t="s">
         <v>1623</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19397,7 +19423,7 @@
       <c r="J286" t="s">
         <v>1623</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19438,7 +19464,7 @@
       <c r="J287" t="s">
         <v>1623</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19479,7 +19505,7 @@
       <c r="J288" t="s">
         <v>1623</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19520,7 +19546,7 @@
       <c r="J289" t="s">
         <v>1623</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19561,7 +19587,7 @@
       <c r="J290" t="s">
         <v>1623</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19602,7 +19628,7 @@
       <c r="J291" t="s">
         <v>1623</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19643,7 +19669,7 @@
       <c r="J292" t="s">
         <v>1623</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19684,7 +19710,7 @@
       <c r="J293" t="s">
         <v>1623</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19725,7 +19751,7 @@
       <c r="J294" t="s">
         <v>1623</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19766,7 +19792,7 @@
       <c r="J295" t="s">
         <v>1623</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19784,7 +19810,7 @@
       <c r="R295" t="s">
         <v>1839</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19825,7 +19851,7 @@
       <c r="J296" t="s">
         <v>1623</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19843,7 +19869,7 @@
       <c r="R296" t="s">
         <v>1815</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19881,7 +19907,7 @@
       <c r="J297" t="s">
         <v>1623</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19922,7 +19948,7 @@
       <c r="J298" t="s">
         <v>1623</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19963,7 +19989,7 @@
       <c r="J299" t="s">
         <v>1624</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20004,7 +20030,7 @@
       <c r="J300" t="s">
         <v>1623</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20045,7 +20071,7 @@
       <c r="J301" t="s">
         <v>1623</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20883,7 +20909,7 @@
       <c r="R321" t="s">
         <v>1801</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21106,7 +21132,7 @@
       <c r="R326" t="s">
         <v>1840</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21941,7 +21967,7 @@
       <c r="R346" t="s">
         <v>1841</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (13/10/2026 10:15)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5753,8 +5753,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5770,7 +5778,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5778,12 +5786,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6083,73 +6109,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6184,7 +6210,7 @@
       <c r="J2" t="s">
         <v>1635</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6228,7 +6254,7 @@
       <c r="J3" t="s">
         <v>1635</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6272,7 +6298,7 @@
       <c r="J4" t="s">
         <v>1635</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6290,7 +6316,7 @@
       <c r="R4" t="s">
         <v>1812</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6328,7 +6354,7 @@
       <c r="J5" t="s">
         <v>1636</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6378,7 +6404,7 @@
       <c r="J6" t="s">
         <v>1635</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6425,7 +6451,7 @@
       <c r="J7" t="s">
         <v>1635</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6472,7 +6498,7 @@
       <c r="J8" t="s">
         <v>1635</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6519,7 +6545,7 @@
       <c r="J9" t="s">
         <v>1635</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6566,7 +6592,7 @@
       <c r="J10" t="s">
         <v>1635</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6613,7 +6639,7 @@
       <c r="J11" t="s">
         <v>1635</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6660,7 +6686,7 @@
       <c r="J12" t="s">
         <v>1635</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6704,7 +6730,7 @@
       <c r="J13" t="s">
         <v>1635</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6722,7 +6748,7 @@
       <c r="R13" t="s">
         <v>1813</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6760,7 +6786,7 @@
       <c r="J14" t="s">
         <v>1635</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6778,7 +6804,7 @@
       <c r="R14" t="s">
         <v>1814</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6819,7 +6845,7 @@
       <c r="J15" t="s">
         <v>1635</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6837,7 +6863,7 @@
       <c r="R15" t="s">
         <v>1814</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6878,7 +6904,7 @@
       <c r="J16" t="s">
         <v>1635</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6922,7 +6948,7 @@
       <c r="J17" t="s">
         <v>1635</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6966,7 +6992,7 @@
       <c r="J18" t="s">
         <v>1635</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6984,7 +7010,7 @@
       <c r="R18" t="s">
         <v>1815</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7025,7 +7051,7 @@
       <c r="J19" t="s">
         <v>1635</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7069,7 +7095,7 @@
       <c r="J20" t="s">
         <v>1635</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7113,7 +7139,7 @@
       <c r="J21" t="s">
         <v>1635</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7131,7 +7157,7 @@
       <c r="R21" t="s">
         <v>1814</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7172,7 +7198,7 @@
       <c r="J22" t="s">
         <v>1635</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7190,7 +7216,7 @@
       <c r="R22" t="s">
         <v>1816</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7231,7 +7257,7 @@
       <c r="J23" t="s">
         <v>1635</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7249,7 +7275,7 @@
       <c r="R23" t="s">
         <v>1817</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7290,7 +7316,7 @@
       <c r="J24" t="s">
         <v>1635</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7334,7 +7360,7 @@
       <c r="J25" t="s">
         <v>1635</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7375,7 +7401,7 @@
       <c r="J26" t="s">
         <v>1637</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7393,7 +7419,7 @@
       <c r="R26" t="s">
         <v>1818</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7431,7 +7457,7 @@
       <c r="J27" t="s">
         <v>1635</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7449,7 +7475,7 @@
       <c r="R27" t="s">
         <v>1819</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7490,7 +7516,7 @@
       <c r="J28" t="s">
         <v>1635</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7534,7 +7560,7 @@
       <c r="J29" t="s">
         <v>1635</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7578,7 +7604,7 @@
       <c r="J30" t="s">
         <v>1635</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7622,7 +7648,7 @@
       <c r="J31" t="s">
         <v>1635</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7640,7 +7666,7 @@
       <c r="R31" t="s">
         <v>1820</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7681,7 +7707,7 @@
       <c r="J32" t="s">
         <v>1635</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7725,7 +7751,7 @@
       <c r="J33" t="s">
         <v>1635</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7743,7 +7769,7 @@
       <c r="R33" t="s">
         <v>1821</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7784,7 +7810,7 @@
       <c r="J34" t="s">
         <v>1635</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7828,7 +7854,7 @@
       <c r="J35" t="s">
         <v>1635</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7846,7 +7872,7 @@
       <c r="R35" t="s">
         <v>1822</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7887,7 +7913,7 @@
       <c r="J36" t="s">
         <v>1635</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7905,7 +7931,7 @@
       <c r="R36" t="s">
         <v>1822</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7946,7 +7972,7 @@
       <c r="J37" t="s">
         <v>1635</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7964,7 +7990,7 @@
       <c r="R37" t="s">
         <v>1822</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8005,7 +8031,7 @@
       <c r="J38" t="s">
         <v>1635</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8023,7 +8049,7 @@
       <c r="R38" t="s">
         <v>1822</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8064,7 +8090,7 @@
       <c r="J39" t="s">
         <v>1635</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8082,7 +8108,7 @@
       <c r="R39" t="s">
         <v>1822</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8123,7 +8149,7 @@
       <c r="J40" t="s">
         <v>1635</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8141,7 +8167,7 @@
       <c r="R40" t="s">
         <v>1823</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8182,7 +8208,7 @@
       <c r="J41" t="s">
         <v>1635</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8200,7 +8226,7 @@
       <c r="R41" t="s">
         <v>1814</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8241,7 +8267,7 @@
       <c r="J42" t="s">
         <v>1635</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8259,7 +8285,7 @@
       <c r="R42" t="s">
         <v>1822</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8300,7 +8326,7 @@
       <c r="J43" t="s">
         <v>1635</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8344,7 +8370,7 @@
       <c r="J44" t="s">
         <v>1635</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8362,7 +8388,7 @@
       <c r="R44" t="s">
         <v>1824</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8403,7 +8429,7 @@
       <c r="J45" t="s">
         <v>1635</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8421,7 +8447,7 @@
       <c r="R45" t="s">
         <v>1825</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8459,7 +8485,7 @@
       <c r="J46" t="s">
         <v>1635</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8503,7 +8529,7 @@
       <c r="J47" t="s">
         <v>1635</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8521,7 +8547,7 @@
       <c r="R47" t="s">
         <v>1826</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8562,7 +8588,7 @@
       <c r="J48" t="s">
         <v>1635</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8606,7 +8632,7 @@
       <c r="J49" t="s">
         <v>1635</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8650,7 +8676,7 @@
       <c r="J50" t="s">
         <v>1635</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8694,7 +8720,7 @@
       <c r="J51" t="s">
         <v>1635</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8741,7 +8767,7 @@
       <c r="J52" t="s">
         <v>1635</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8785,7 +8811,7 @@
       <c r="J53" t="s">
         <v>1635</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8829,7 +8855,7 @@
       <c r="J54" t="s">
         <v>1635</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8873,7 +8899,7 @@
       <c r="J55" t="s">
         <v>1635</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8923,7 +8949,7 @@
       <c r="J56" t="s">
         <v>1635</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8976,7 +9002,7 @@
       <c r="J57" t="s">
         <v>1635</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9026,7 +9052,7 @@
       <c r="J58" t="s">
         <v>1635</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9076,7 +9102,7 @@
       <c r="J59" t="s">
         <v>1635</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9094,7 +9120,7 @@
       <c r="R59" t="s">
         <v>1827</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9135,7 +9161,7 @@
       <c r="J60" t="s">
         <v>1635</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9179,7 +9205,7 @@
       <c r="J61" t="s">
         <v>1635</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9223,7 +9249,7 @@
       <c r="J62" t="s">
         <v>1635</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9267,7 +9293,7 @@
       <c r="J63" t="s">
         <v>1635</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9311,7 +9337,7 @@
       <c r="J64" t="s">
         <v>1635</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9355,7 +9381,7 @@
       <c r="J65" t="s">
         <v>1635</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9402,7 +9428,7 @@
       <c r="J66" t="s">
         <v>1635</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9420,7 +9446,7 @@
       <c r="R66" t="s">
         <v>1828</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9458,7 +9484,7 @@
       <c r="J67" t="s">
         <v>1635</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9502,7 +9528,7 @@
       <c r="J68" t="s">
         <v>1635</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9517,7 +9543,7 @@
       <c r="O68" t="s">
         <v>1732</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9561,7 +9587,7 @@
       <c r="J69" t="s">
         <v>1637</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9605,7 +9631,7 @@
       <c r="J70" t="s">
         <v>1635</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9649,7 +9675,7 @@
       <c r="J71" t="s">
         <v>1635</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9693,7 +9719,7 @@
       <c r="J72" t="s">
         <v>1635</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9737,7 +9763,7 @@
       <c r="J73" t="s">
         <v>1635</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9781,7 +9807,7 @@
       <c r="J74" t="s">
         <v>1635</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9825,7 +9851,7 @@
       <c r="J75" t="s">
         <v>1635</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9869,7 +9895,7 @@
       <c r="J76" t="s">
         <v>1635</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9887,7 +9913,7 @@
       <c r="R76" t="s">
         <v>1829</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9925,7 +9951,7 @@
       <c r="J77" t="s">
         <v>1635</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9943,7 +9969,7 @@
       <c r="R77" t="s">
         <v>1829</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9981,7 +10007,7 @@
       <c r="J78" t="s">
         <v>1635</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9999,7 +10025,7 @@
       <c r="R78" t="s">
         <v>1829</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10037,7 +10063,7 @@
       <c r="J79" t="s">
         <v>1635</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10055,7 +10081,7 @@
       <c r="R79" t="s">
         <v>1829</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10093,7 +10119,7 @@
       <c r="J80" t="s">
         <v>1635</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10137,7 +10163,7 @@
       <c r="J81" t="s">
         <v>1635</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10181,7 +10207,7 @@
       <c r="J82" t="s">
         <v>1635</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10225,7 +10251,7 @@
       <c r="J83" t="s">
         <v>1635</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10269,7 +10295,7 @@
       <c r="J84" t="s">
         <v>1635</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10313,7 +10339,7 @@
       <c r="J85" t="s">
         <v>1635</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10331,7 +10357,7 @@
       <c r="R85" t="s">
         <v>1830</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10369,7 +10395,7 @@
       <c r="J86" t="s">
         <v>1635</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10413,7 +10439,7 @@
       <c r="J87" t="s">
         <v>1635</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10431,7 +10457,7 @@
       <c r="R87" t="s">
         <v>1831</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10469,7 +10495,7 @@
       <c r="J88" t="s">
         <v>1635</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10513,7 +10539,7 @@
       <c r="J89" t="s">
         <v>1635</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10531,7 +10557,7 @@
       <c r="R89" t="s">
         <v>1832</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10566,7 +10592,7 @@
       <c r="J90" t="s">
         <v>1635</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10584,7 +10610,7 @@
       <c r="R90" t="s">
         <v>1833</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10619,7 +10645,7 @@
       <c r="J91" t="s">
         <v>1635</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10637,7 +10663,7 @@
       <c r="R91" t="s">
         <v>1817</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10675,7 +10701,7 @@
       <c r="J92" t="s">
         <v>1635</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10696,7 +10722,7 @@
       <c r="R92" t="s">
         <v>1817</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10737,7 +10763,7 @@
       <c r="J93" t="s">
         <v>1635</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10778,7 +10804,7 @@
       <c r="J94" t="s">
         <v>1635</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10822,7 +10848,7 @@
       <c r="J95" t="s">
         <v>1635</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10866,7 +10892,7 @@
       <c r="J96" t="s">
         <v>1635</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10884,7 +10910,7 @@
       <c r="R96" t="s">
         <v>1834</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10925,7 +10951,7 @@
       <c r="J97" t="s">
         <v>1635</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10940,7 +10966,7 @@
       <c r="R97" t="s">
         <v>1834</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10981,7 +11007,7 @@
       <c r="J98" t="s">
         <v>1635</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10999,7 +11025,7 @@
       <c r="R98" t="s">
         <v>1835</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11037,7 +11063,7 @@
       <c r="J99" t="s">
         <v>1635</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11055,7 +11081,7 @@
       <c r="R99" t="s">
         <v>1836</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11093,7 +11119,7 @@
       <c r="J100" t="s">
         <v>1635</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11134,7 +11160,7 @@
       <c r="J101" t="s">
         <v>1635</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11175,7 +11201,7 @@
       <c r="J102" t="s">
         <v>1635</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11216,7 +11242,7 @@
       <c r="J103" t="s">
         <v>1635</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11257,7 +11283,7 @@
       <c r="J104" t="s">
         <v>1635</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11298,7 +11324,7 @@
       <c r="J105" t="s">
         <v>1635</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11339,7 +11365,7 @@
       <c r="J106" t="s">
         <v>1635</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11380,7 +11406,7 @@
       <c r="J107" t="s">
         <v>1635</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11421,7 +11447,7 @@
       <c r="J108" t="s">
         <v>1635</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11462,7 +11488,7 @@
       <c r="J109" t="s">
         <v>1635</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11515,7 +11541,7 @@
       <c r="J110" t="s">
         <v>1635</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11571,7 +11597,7 @@
       <c r="J111" t="s">
         <v>1635</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11589,7 +11615,7 @@
       <c r="R111" t="s">
         <v>1838</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11627,7 +11653,7 @@
       <c r="J112" t="s">
         <v>1635</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11686,7 +11712,7 @@
       <c r="J113" t="s">
         <v>1635</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11730,7 +11756,7 @@
       <c r="J114" t="s">
         <v>1635</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11774,7 +11800,7 @@
       <c r="J115" t="s">
         <v>1635</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11792,7 +11818,7 @@
       <c r="R115" t="s">
         <v>1840</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11833,7 +11859,7 @@
       <c r="J116" t="s">
         <v>1635</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11892,7 +11918,7 @@
       <c r="J117" t="s">
         <v>1635</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11936,7 +11962,7 @@
       <c r="J118" t="s">
         <v>1635</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11983,7 +12009,7 @@
       <c r="J119" t="s">
         <v>1635</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12024,7 +12050,7 @@
       <c r="J120" t="s">
         <v>1635</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12068,7 +12094,7 @@
       <c r="J121" t="s">
         <v>1635</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12115,7 +12141,7 @@
       <c r="J122" t="s">
         <v>1635</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12165,7 +12191,7 @@
       <c r="J123" t="s">
         <v>1635</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12209,7 +12235,7 @@
       <c r="J124" t="s">
         <v>1635</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12253,7 +12279,7 @@
       <c r="J125" t="s">
         <v>1635</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12271,7 +12297,7 @@
       <c r="R125" t="s">
         <v>1842</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12306,7 +12332,7 @@
       <c r="J126" t="s">
         <v>1635</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12324,7 +12350,7 @@
       <c r="R126" t="s">
         <v>1843</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12362,7 +12388,7 @@
       <c r="J127" t="s">
         <v>1635</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12418,7 +12444,7 @@
       <c r="J128" t="s">
         <v>1635</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12459,7 +12485,7 @@
       <c r="J129" t="s">
         <v>1635</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12500,7 +12526,7 @@
       <c r="J130" t="s">
         <v>1635</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12541,7 +12567,7 @@
       <c r="J131" t="s">
         <v>1635</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12585,7 +12611,7 @@
       <c r="J132" t="s">
         <v>1635</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12626,7 +12652,7 @@
       <c r="J133" t="s">
         <v>1635</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12644,7 +12670,7 @@
       <c r="R133" t="s">
         <v>1829</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12682,7 +12708,7 @@
       <c r="J134" t="s">
         <v>1635</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12700,7 +12726,7 @@
       <c r="R134" t="s">
         <v>1829</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12735,7 +12761,7 @@
       <c r="J135" t="s">
         <v>1635</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12776,7 +12802,7 @@
       <c r="J136" t="s">
         <v>1635</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12817,7 +12843,7 @@
       <c r="J137" t="s">
         <v>1635</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12858,7 +12884,7 @@
       <c r="J138" t="s">
         <v>1635</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12899,7 +12925,7 @@
       <c r="J139" t="s">
         <v>1635</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12946,7 +12972,7 @@
       <c r="J140" t="s">
         <v>1635</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12987,7 +13013,7 @@
       <c r="J141" t="s">
         <v>1635</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13028,7 +13054,7 @@
       <c r="J142" t="s">
         <v>1635</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13072,7 +13098,7 @@
       <c r="J143" t="s">
         <v>1635</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13090,7 +13116,7 @@
       <c r="R143" t="s">
         <v>1829</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13125,7 +13151,7 @@
       <c r="J144" t="s">
         <v>1635</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13143,7 +13169,7 @@
       <c r="R144" t="s">
         <v>1829</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13181,7 +13207,7 @@
       <c r="J145" t="s">
         <v>1635</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13199,7 +13225,7 @@
       <c r="R145" t="s">
         <v>1829</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13234,7 +13260,7 @@
       <c r="J146" t="s">
         <v>1635</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13252,7 +13278,7 @@
       <c r="R146" t="s">
         <v>1837</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13287,7 +13313,7 @@
       <c r="J147" t="s">
         <v>1635</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13305,7 +13331,7 @@
       <c r="R147" t="s">
         <v>1844</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13340,7 +13366,7 @@
       <c r="J148" t="s">
         <v>1635</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13381,7 +13407,7 @@
       <c r="J149" t="s">
         <v>1635</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13399,7 +13425,7 @@
       <c r="R149" t="s">
         <v>1829</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13434,7 +13460,7 @@
       <c r="J150" t="s">
         <v>1635</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13452,7 +13478,7 @@
       <c r="R150" t="s">
         <v>1829</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13490,7 +13516,7 @@
       <c r="J151" t="s">
         <v>1635</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13508,7 +13534,7 @@
       <c r="R151" t="s">
         <v>1845</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13543,7 +13569,7 @@
       <c r="J152" t="s">
         <v>1635</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13561,7 +13587,7 @@
       <c r="R152" t="s">
         <v>1846</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13596,7 +13622,7 @@
       <c r="J153" t="s">
         <v>1635</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13605,7 +13631,7 @@
       <c r="M153" t="s">
         <v>1723</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13646,7 +13672,7 @@
       <c r="J154" t="s">
         <v>1635</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13687,7 +13713,7 @@
       <c r="J155" t="s">
         <v>1635</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13728,7 +13754,7 @@
       <c r="J156" t="s">
         <v>1635</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13769,7 +13795,7 @@
       <c r="J157" t="s">
         <v>1635</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13810,7 +13836,7 @@
       <c r="J158" t="s">
         <v>1635</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13851,7 +13877,7 @@
       <c r="J159" t="s">
         <v>1635</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13892,7 +13918,7 @@
       <c r="J160" t="s">
         <v>1635</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13933,7 +13959,7 @@
       <c r="J161" t="s">
         <v>1635</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13974,7 +14000,7 @@
       <c r="J162" t="s">
         <v>1635</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13992,7 +14018,7 @@
       <c r="R162" t="s">
         <v>1832</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14027,7 +14053,7 @@
       <c r="J163" t="s">
         <v>1635</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14045,7 +14071,7 @@
       <c r="R163" t="s">
         <v>1829</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14080,7 +14106,7 @@
       <c r="J164" t="s">
         <v>1635</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14124,7 +14150,7 @@
       <c r="J165" t="s">
         <v>1635</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14165,7 +14191,7 @@
       <c r="J166" t="s">
         <v>1635</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14183,7 +14209,7 @@
       <c r="R166" t="s">
         <v>1847</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14218,7 +14244,7 @@
       <c r="J167" t="s">
         <v>1635</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14262,7 +14288,7 @@
       <c r="J168" t="s">
         <v>1635</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14306,7 +14332,7 @@
       <c r="J169" t="s">
         <v>1635</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14347,7 +14373,7 @@
       <c r="J170" t="s">
         <v>1635</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14388,7 +14414,7 @@
       <c r="J171" t="s">
         <v>1635</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14429,7 +14455,7 @@
       <c r="J172" t="s">
         <v>1635</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14470,7 +14496,7 @@
       <c r="J173" t="s">
         <v>1635</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14511,7 +14537,7 @@
       <c r="J174" t="s">
         <v>1635</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14552,7 +14578,7 @@
       <c r="J175" t="s">
         <v>1635</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14593,7 +14619,7 @@
       <c r="J176" t="s">
         <v>1635</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14634,7 +14660,7 @@
       <c r="J177" t="s">
         <v>1635</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14675,7 +14701,7 @@
       <c r="J178" t="s">
         <v>1635</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14693,7 +14719,7 @@
       <c r="R178" t="s">
         <v>1845</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14731,7 +14757,7 @@
       <c r="J179" t="s">
         <v>1635</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14740,7 +14766,7 @@
       <c r="M179" t="s">
         <v>1720</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14781,7 +14807,7 @@
       <c r="J180" t="s">
         <v>1635</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14822,7 +14848,7 @@
       <c r="J181" t="s">
         <v>1635</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14840,7 +14866,7 @@
       <c r="R181" t="s">
         <v>1829</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14875,7 +14901,7 @@
       <c r="J182" t="s">
         <v>1635</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14916,7 +14942,7 @@
       <c r="J183" t="s">
         <v>1635</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14957,7 +14983,7 @@
       <c r="J184" t="s">
         <v>1635</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14998,7 +15024,7 @@
       <c r="J185" t="s">
         <v>1635</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15039,7 +15065,7 @@
       <c r="J186" t="s">
         <v>1635</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15080,7 +15106,7 @@
       <c r="J187" t="s">
         <v>1635</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15121,7 +15147,7 @@
       <c r="J188" t="s">
         <v>1635</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15162,7 +15188,7 @@
       <c r="J189" t="s">
         <v>1635</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15203,7 +15229,7 @@
       <c r="J190" t="s">
         <v>1635</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15244,7 +15270,7 @@
       <c r="J191" t="s">
         <v>1635</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15285,7 +15311,7 @@
       <c r="J192" t="s">
         <v>1635</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15326,7 +15352,7 @@
       <c r="J193" t="s">
         <v>1635</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15367,7 +15393,7 @@
       <c r="J194" t="s">
         <v>1635</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15408,7 +15434,7 @@
       <c r="J195" t="s">
         <v>1635</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15426,7 +15452,7 @@
       <c r="R195" t="s">
         <v>1838</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15467,7 +15493,7 @@
       <c r="J196" t="s">
         <v>1635</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15485,7 +15511,7 @@
       <c r="R196" t="s">
         <v>1844</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15523,7 +15549,7 @@
       <c r="J197" t="s">
         <v>1635</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15564,7 +15590,7 @@
       <c r="J198" t="s">
         <v>1637</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15605,7 +15631,7 @@
       <c r="J199" t="s">
         <v>1636</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15646,7 +15672,7 @@
       <c r="J200" t="s">
         <v>1635</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15687,7 +15713,7 @@
       <c r="J201" t="s">
         <v>1635</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15728,7 +15754,7 @@
       <c r="J202" t="s">
         <v>1635</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15746,7 +15772,7 @@
       <c r="R202" t="s">
         <v>1829</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15784,7 +15810,7 @@
       <c r="J203" t="s">
         <v>1635</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15802,7 +15828,7 @@
       <c r="R203" t="s">
         <v>1837</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15837,7 +15863,7 @@
       <c r="J204" t="s">
         <v>1635</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15852,7 +15878,7 @@
       <c r="R204" t="s">
         <v>1848</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15890,7 +15916,7 @@
       <c r="J205" t="s">
         <v>1635</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15908,7 +15934,7 @@
       <c r="R205" t="s">
         <v>1849</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15946,7 +15972,7 @@
       <c r="J206" t="s">
         <v>1635</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15964,7 +15990,7 @@
       <c r="R206" t="s">
         <v>1817</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15999,7 +16025,7 @@
       <c r="J207" t="s">
         <v>1635</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16040,7 +16066,7 @@
       <c r="J208" t="s">
         <v>1635</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16081,7 +16107,7 @@
       <c r="J209" t="s">
         <v>1635</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16122,7 +16148,7 @@
       <c r="J210" t="s">
         <v>1635</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16163,7 +16189,7 @@
       <c r="J211" t="s">
         <v>1635</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16204,7 +16230,7 @@
       <c r="J212" t="s">
         <v>1635</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16245,7 +16271,7 @@
       <c r="J213" t="s">
         <v>1635</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16286,7 +16312,7 @@
       <c r="J214" t="s">
         <v>1635</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16304,7 +16330,7 @@
       <c r="R214" t="s">
         <v>1850</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16342,7 +16368,7 @@
       <c r="J215" t="s">
         <v>1635</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16383,7 +16409,7 @@
       <c r="J216" t="s">
         <v>1635</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16424,7 +16450,7 @@
       <c r="J217" t="s">
         <v>1635</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16465,7 +16491,7 @@
       <c r="J218" t="s">
         <v>1635</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16506,7 +16532,7 @@
       <c r="J219" t="s">
         <v>1635</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16547,7 +16573,7 @@
       <c r="J220" t="s">
         <v>1635</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16588,7 +16614,7 @@
       <c r="J221" t="s">
         <v>1635</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16629,7 +16655,7 @@
       <c r="J222" t="s">
         <v>1635</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16670,7 +16696,7 @@
       <c r="J223" t="s">
         <v>1635</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16711,7 +16737,7 @@
       <c r="J224" t="s">
         <v>1635</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16752,7 +16778,7 @@
       <c r="J225" t="s">
         <v>1635</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16793,7 +16819,7 @@
       <c r="J226" t="s">
         <v>1635</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16834,7 +16860,7 @@
       <c r="J227" t="s">
         <v>1635</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16875,7 +16901,7 @@
       <c r="J228" t="s">
         <v>1635</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16916,7 +16942,7 @@
       <c r="J229" t="s">
         <v>1635</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16957,7 +16983,7 @@
       <c r="J230" t="s">
         <v>1635</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16998,7 +17024,7 @@
       <c r="J231" t="s">
         <v>1635</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17039,7 +17065,7 @@
       <c r="J232" t="s">
         <v>1635</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17080,7 +17106,7 @@
       <c r="J233" t="s">
         <v>1635</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17121,7 +17147,7 @@
       <c r="J234" t="s">
         <v>1635</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17162,7 +17188,7 @@
       <c r="J235" t="s">
         <v>1635</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17203,7 +17229,7 @@
       <c r="J236" t="s">
         <v>1635</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17244,7 +17270,7 @@
       <c r="J237" t="s">
         <v>1635</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17285,7 +17311,7 @@
       <c r="J238" t="s">
         <v>1635</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17326,7 +17352,7 @@
       <c r="J239" t="s">
         <v>1635</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17344,7 +17370,7 @@
       <c r="R239" t="s">
         <v>1844</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17382,7 +17408,7 @@
       <c r="J240" t="s">
         <v>1635</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17423,7 +17449,7 @@
       <c r="J241" t="s">
         <v>1635</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17464,7 +17490,7 @@
       <c r="J242" t="s">
         <v>1635</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17482,7 +17508,7 @@
       <c r="R242" t="s">
         <v>1837</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17517,7 +17543,7 @@
       <c r="J243" t="s">
         <v>1635</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17558,7 +17584,7 @@
       <c r="J244" t="s">
         <v>1635</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17599,7 +17625,7 @@
       <c r="J245" t="s">
         <v>1635</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17640,7 +17666,7 @@
       <c r="J246" t="s">
         <v>1635</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17658,7 +17684,7 @@
       <c r="R246" t="s">
         <v>1817</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17696,7 +17722,7 @@
       <c r="J247" t="s">
         <v>1635</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17737,7 +17763,7 @@
       <c r="J248" t="s">
         <v>1635</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17778,7 +17804,7 @@
       <c r="J249" t="s">
         <v>1635</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17819,7 +17845,7 @@
       <c r="J250" t="s">
         <v>1635</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17860,7 +17886,7 @@
       <c r="J251" t="s">
         <v>1635</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17901,7 +17927,7 @@
       <c r="J252" t="s">
         <v>1635</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17942,7 +17968,7 @@
       <c r="J253" t="s">
         <v>1635</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17960,7 +17986,7 @@
       <c r="R253" t="s">
         <v>1847</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18001,7 +18027,7 @@
       <c r="J254" t="s">
         <v>1635</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18042,7 +18068,7 @@
       <c r="J255" t="s">
         <v>1635</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18083,7 +18109,7 @@
       <c r="J256" t="s">
         <v>1635</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18092,7 +18118,7 @@
       <c r="M256" t="s">
         <v>1719</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18130,7 +18156,7 @@
       <c r="J257" t="s">
         <v>1635</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18139,7 +18165,7 @@
       <c r="M257" t="s">
         <v>1720</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18183,7 +18209,7 @@
       <c r="J258" t="s">
         <v>1635</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18201,7 +18227,7 @@
       <c r="R258" t="s">
         <v>1829</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18239,7 +18265,7 @@
       <c r="J259" t="s">
         <v>1635</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18257,7 +18283,7 @@
       <c r="R259" t="s">
         <v>1845</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18295,7 +18321,7 @@
       <c r="J260" t="s">
         <v>1635</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18304,7 +18330,7 @@
       <c r="M260" t="s">
         <v>1714</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18348,7 +18374,7 @@
       <c r="J261" t="s">
         <v>1635</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18366,7 +18392,7 @@
       <c r="R261" t="s">
         <v>1851</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18404,7 +18430,7 @@
       <c r="J262" t="s">
         <v>1635</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18422,7 +18448,7 @@
       <c r="R262" t="s">
         <v>1845</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18460,7 +18486,7 @@
       <c r="J263" t="s">
         <v>1635</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18469,7 +18495,7 @@
       <c r="M263" t="s">
         <v>1714</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18513,7 +18539,7 @@
       <c r="J264" t="s">
         <v>1635</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18554,7 +18580,7 @@
       <c r="J265" t="s">
         <v>1635</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18595,7 +18621,7 @@
       <c r="J266" t="s">
         <v>1635</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18636,7 +18662,7 @@
       <c r="J267" t="s">
         <v>1635</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18680,7 +18706,7 @@
       <c r="J268" t="s">
         <v>1635</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18721,7 +18747,7 @@
       <c r="J269" t="s">
         <v>1635</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18762,7 +18788,7 @@
       <c r="J270" t="s">
         <v>1635</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18803,7 +18829,7 @@
       <c r="J271" t="s">
         <v>1635</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18844,7 +18870,7 @@
       <c r="J272" t="s">
         <v>1635</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18862,7 +18888,7 @@
       <c r="R272" t="s">
         <v>1852</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18903,7 +18929,7 @@
       <c r="J273" t="s">
         <v>1635</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18947,7 +18973,7 @@
       <c r="J274" t="s">
         <v>1635</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18988,7 +19014,7 @@
       <c r="J275" t="s">
         <v>1635</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19029,7 +19055,7 @@
       <c r="J276" t="s">
         <v>1635</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19070,7 +19096,7 @@
       <c r="J277" t="s">
         <v>1635</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19111,7 +19137,7 @@
       <c r="J278" t="s">
         <v>1635</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19152,7 +19178,7 @@
       <c r="J279" t="s">
         <v>1635</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19193,7 +19219,7 @@
       <c r="J280" t="s">
         <v>1635</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19234,7 +19260,7 @@
       <c r="J281" t="s">
         <v>1635</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19275,7 +19301,7 @@
       <c r="J282" t="s">
         <v>1635</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19316,7 +19342,7 @@
       <c r="J283" t="s">
         <v>1635</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19357,7 +19383,7 @@
       <c r="J284" t="s">
         <v>1635</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19398,7 +19424,7 @@
       <c r="J285" t="s">
         <v>1635</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19439,7 +19465,7 @@
       <c r="J286" t="s">
         <v>1635</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19480,7 +19506,7 @@
       <c r="J287" t="s">
         <v>1635</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19521,7 +19547,7 @@
       <c r="J288" t="s">
         <v>1635</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19562,7 +19588,7 @@
       <c r="J289" t="s">
         <v>1635</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19603,7 +19629,7 @@
       <c r="J290" t="s">
         <v>1635</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19644,7 +19670,7 @@
       <c r="J291" t="s">
         <v>1635</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19685,7 +19711,7 @@
       <c r="J292" t="s">
         <v>1635</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19726,7 +19752,7 @@
       <c r="J293" t="s">
         <v>1635</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19767,7 +19793,7 @@
       <c r="J294" t="s">
         <v>1635</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19808,7 +19834,7 @@
       <c r="J295" t="s">
         <v>1635</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19826,7 +19852,7 @@
       <c r="R295" t="s">
         <v>1853</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19867,7 +19893,7 @@
       <c r="J296" t="s">
         <v>1635</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19885,7 +19911,7 @@
       <c r="R296" t="s">
         <v>1829</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19923,7 +19949,7 @@
       <c r="J297" t="s">
         <v>1635</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19964,7 +19990,7 @@
       <c r="J298" t="s">
         <v>1635</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20005,7 +20031,7 @@
       <c r="J299" t="s">
         <v>1636</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20046,7 +20072,7 @@
       <c r="J300" t="s">
         <v>1635</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20087,7 +20113,7 @@
       <c r="J301" t="s">
         <v>1635</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20925,7 +20951,7 @@
       <c r="R321" t="s">
         <v>1815</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21148,7 +21174,7 @@
       <c r="R326" t="s">
         <v>1854</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21983,7 +22009,7 @@
       <c r="R346" t="s">
         <v>1855</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (13/10/2026 15:10)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5753,16 +5753,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5778,7 +5770,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5786,30 +5778,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6109,73 +6083,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6210,7 +6184,7 @@
       <c r="J2" t="s">
         <v>1635</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6254,7 +6228,7 @@
       <c r="J3" t="s">
         <v>1635</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6298,7 +6272,7 @@
       <c r="J4" t="s">
         <v>1635</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6316,7 +6290,7 @@
       <c r="R4" t="s">
         <v>1812</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6354,7 +6328,7 @@
       <c r="J5" t="s">
         <v>1636</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6404,7 +6378,7 @@
       <c r="J6" t="s">
         <v>1635</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6451,7 +6425,7 @@
       <c r="J7" t="s">
         <v>1635</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6498,7 +6472,7 @@
       <c r="J8" t="s">
         <v>1635</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6545,7 +6519,7 @@
       <c r="J9" t="s">
         <v>1635</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6592,7 +6566,7 @@
       <c r="J10" t="s">
         <v>1635</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6639,7 +6613,7 @@
       <c r="J11" t="s">
         <v>1635</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6686,7 +6660,7 @@
       <c r="J12" t="s">
         <v>1635</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6730,7 +6704,7 @@
       <c r="J13" t="s">
         <v>1635</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6748,7 +6722,7 @@
       <c r="R13" t="s">
         <v>1813</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6786,7 +6760,7 @@
       <c r="J14" t="s">
         <v>1635</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6804,7 +6778,7 @@
       <c r="R14" t="s">
         <v>1814</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6845,7 +6819,7 @@
       <c r="J15" t="s">
         <v>1635</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6863,7 +6837,7 @@
       <c r="R15" t="s">
         <v>1814</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6904,7 +6878,7 @@
       <c r="J16" t="s">
         <v>1635</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6948,7 +6922,7 @@
       <c r="J17" t="s">
         <v>1635</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6992,7 +6966,7 @@
       <c r="J18" t="s">
         <v>1635</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -7010,7 +6984,7 @@
       <c r="R18" t="s">
         <v>1815</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7051,7 +7025,7 @@
       <c r="J19" t="s">
         <v>1635</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7095,7 +7069,7 @@
       <c r="J20" t="s">
         <v>1635</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7139,7 +7113,7 @@
       <c r="J21" t="s">
         <v>1635</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7157,7 +7131,7 @@
       <c r="R21" t="s">
         <v>1814</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7198,7 +7172,7 @@
       <c r="J22" t="s">
         <v>1635</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7216,7 +7190,7 @@
       <c r="R22" t="s">
         <v>1816</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7257,7 +7231,7 @@
       <c r="J23" t="s">
         <v>1635</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7275,7 +7249,7 @@
       <c r="R23" t="s">
         <v>1817</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7316,7 +7290,7 @@
       <c r="J24" t="s">
         <v>1635</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7360,7 +7334,7 @@
       <c r="J25" t="s">
         <v>1635</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7401,7 +7375,7 @@
       <c r="J26" t="s">
         <v>1637</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7419,7 +7393,7 @@
       <c r="R26" t="s">
         <v>1818</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7457,7 +7431,7 @@
       <c r="J27" t="s">
         <v>1635</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7475,7 +7449,7 @@
       <c r="R27" t="s">
         <v>1819</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7516,7 +7490,7 @@
       <c r="J28" t="s">
         <v>1635</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7560,7 +7534,7 @@
       <c r="J29" t="s">
         <v>1635</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7604,7 +7578,7 @@
       <c r="J30" t="s">
         <v>1635</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7648,7 +7622,7 @@
       <c r="J31" t="s">
         <v>1635</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7666,7 +7640,7 @@
       <c r="R31" t="s">
         <v>1820</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7707,7 +7681,7 @@
       <c r="J32" t="s">
         <v>1635</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7751,7 +7725,7 @@
       <c r="J33" t="s">
         <v>1635</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7769,7 +7743,7 @@
       <c r="R33" t="s">
         <v>1821</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7810,7 +7784,7 @@
       <c r="J34" t="s">
         <v>1635</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7854,7 +7828,7 @@
       <c r="J35" t="s">
         <v>1635</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7872,7 +7846,7 @@
       <c r="R35" t="s">
         <v>1822</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7913,7 +7887,7 @@
       <c r="J36" t="s">
         <v>1635</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7931,7 +7905,7 @@
       <c r="R36" t="s">
         <v>1822</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7972,7 +7946,7 @@
       <c r="J37" t="s">
         <v>1635</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7990,7 +7964,7 @@
       <c r="R37" t="s">
         <v>1822</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8031,7 +8005,7 @@
       <c r="J38" t="s">
         <v>1635</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8049,7 +8023,7 @@
       <c r="R38" t="s">
         <v>1822</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8090,7 +8064,7 @@
       <c r="J39" t="s">
         <v>1635</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8108,7 +8082,7 @@
       <c r="R39" t="s">
         <v>1822</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8149,7 +8123,7 @@
       <c r="J40" t="s">
         <v>1635</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8167,7 +8141,7 @@
       <c r="R40" t="s">
         <v>1823</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8208,7 +8182,7 @@
       <c r="J41" t="s">
         <v>1635</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8226,7 +8200,7 @@
       <c r="R41" t="s">
         <v>1814</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8267,7 +8241,7 @@
       <c r="J42" t="s">
         <v>1635</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8285,7 +8259,7 @@
       <c r="R42" t="s">
         <v>1822</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8326,7 +8300,7 @@
       <c r="J43" t="s">
         <v>1635</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8370,7 +8344,7 @@
       <c r="J44" t="s">
         <v>1635</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8388,7 +8362,7 @@
       <c r="R44" t="s">
         <v>1824</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8429,7 +8403,7 @@
       <c r="J45" t="s">
         <v>1635</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8447,7 +8421,7 @@
       <c r="R45" t="s">
         <v>1825</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8485,7 +8459,7 @@
       <c r="J46" t="s">
         <v>1635</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8529,7 +8503,7 @@
       <c r="J47" t="s">
         <v>1635</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8547,7 +8521,7 @@
       <c r="R47" t="s">
         <v>1826</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8588,7 +8562,7 @@
       <c r="J48" t="s">
         <v>1635</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8632,7 +8606,7 @@
       <c r="J49" t="s">
         <v>1635</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8676,7 +8650,7 @@
       <c r="J50" t="s">
         <v>1635</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8720,7 +8694,7 @@
       <c r="J51" t="s">
         <v>1635</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8767,7 +8741,7 @@
       <c r="J52" t="s">
         <v>1635</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8811,7 +8785,7 @@
       <c r="J53" t="s">
         <v>1635</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8855,7 +8829,7 @@
       <c r="J54" t="s">
         <v>1635</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8899,7 +8873,7 @@
       <c r="J55" t="s">
         <v>1635</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8949,7 +8923,7 @@
       <c r="J56" t="s">
         <v>1635</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -9002,7 +8976,7 @@
       <c r="J57" t="s">
         <v>1635</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9052,7 +9026,7 @@
       <c r="J58" t="s">
         <v>1635</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9102,7 +9076,7 @@
       <c r="J59" t="s">
         <v>1635</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9120,7 +9094,7 @@
       <c r="R59" t="s">
         <v>1827</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9161,7 +9135,7 @@
       <c r="J60" t="s">
         <v>1635</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9205,7 +9179,7 @@
       <c r="J61" t="s">
         <v>1635</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9249,7 +9223,7 @@
       <c r="J62" t="s">
         <v>1635</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9293,7 +9267,7 @@
       <c r="J63" t="s">
         <v>1635</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9337,7 +9311,7 @@
       <c r="J64" t="s">
         <v>1635</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9381,7 +9355,7 @@
       <c r="J65" t="s">
         <v>1635</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9428,7 +9402,7 @@
       <c r="J66" t="s">
         <v>1635</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9446,7 +9420,7 @@
       <c r="R66" t="s">
         <v>1828</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9484,7 +9458,7 @@
       <c r="J67" t="s">
         <v>1635</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9528,7 +9502,7 @@
       <c r="J68" t="s">
         <v>1635</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9543,7 +9517,7 @@
       <c r="O68" t="s">
         <v>1732</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9587,7 +9561,7 @@
       <c r="J69" t="s">
         <v>1637</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9631,7 +9605,7 @@
       <c r="J70" t="s">
         <v>1635</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9675,7 +9649,7 @@
       <c r="J71" t="s">
         <v>1635</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9719,7 +9693,7 @@
       <c r="J72" t="s">
         <v>1635</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9763,7 +9737,7 @@
       <c r="J73" t="s">
         <v>1635</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9807,7 +9781,7 @@
       <c r="J74" t="s">
         <v>1635</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9851,7 +9825,7 @@
       <c r="J75" t="s">
         <v>1635</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9895,7 +9869,7 @@
       <c r="J76" t="s">
         <v>1635</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9913,7 +9887,7 @@
       <c r="R76" t="s">
         <v>1829</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9951,7 +9925,7 @@
       <c r="J77" t="s">
         <v>1635</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9969,7 +9943,7 @@
       <c r="R77" t="s">
         <v>1829</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -10007,7 +9981,7 @@
       <c r="J78" t="s">
         <v>1635</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -10025,7 +9999,7 @@
       <c r="R78" t="s">
         <v>1829</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10063,7 +10037,7 @@
       <c r="J79" t="s">
         <v>1635</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10081,7 +10055,7 @@
       <c r="R79" t="s">
         <v>1829</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10119,7 +10093,7 @@
       <c r="J80" t="s">
         <v>1635</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10163,7 +10137,7 @@
       <c r="J81" t="s">
         <v>1635</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10207,7 +10181,7 @@
       <c r="J82" t="s">
         <v>1635</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10251,7 +10225,7 @@
       <c r="J83" t="s">
         <v>1635</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10295,7 +10269,7 @@
       <c r="J84" t="s">
         <v>1635</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10339,7 +10313,7 @@
       <c r="J85" t="s">
         <v>1635</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10357,7 +10331,7 @@
       <c r="R85" t="s">
         <v>1830</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10395,7 +10369,7 @@
       <c r="J86" t="s">
         <v>1635</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10439,7 +10413,7 @@
       <c r="J87" t="s">
         <v>1635</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10457,7 +10431,7 @@
       <c r="R87" t="s">
         <v>1831</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10495,7 +10469,7 @@
       <c r="J88" t="s">
         <v>1635</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10539,7 +10513,7 @@
       <c r="J89" t="s">
         <v>1635</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10557,7 +10531,7 @@
       <c r="R89" t="s">
         <v>1832</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10592,7 +10566,7 @@
       <c r="J90" t="s">
         <v>1635</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10610,7 +10584,7 @@
       <c r="R90" t="s">
         <v>1833</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10645,7 +10619,7 @@
       <c r="J91" t="s">
         <v>1635</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10663,7 +10637,7 @@
       <c r="R91" t="s">
         <v>1817</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10701,7 +10675,7 @@
       <c r="J92" t="s">
         <v>1635</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10722,7 +10696,7 @@
       <c r="R92" t="s">
         <v>1817</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10763,7 +10737,7 @@
       <c r="J93" t="s">
         <v>1635</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10804,7 +10778,7 @@
       <c r="J94" t="s">
         <v>1635</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10848,7 +10822,7 @@
       <c r="J95" t="s">
         <v>1635</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10892,7 +10866,7 @@
       <c r="J96" t="s">
         <v>1635</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10910,7 +10884,7 @@
       <c r="R96" t="s">
         <v>1834</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10951,7 +10925,7 @@
       <c r="J97" t="s">
         <v>1635</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10966,7 +10940,7 @@
       <c r="R97" t="s">
         <v>1834</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -11007,7 +10981,7 @@
       <c r="J98" t="s">
         <v>1635</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -11025,7 +10999,7 @@
       <c r="R98" t="s">
         <v>1835</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11063,7 +11037,7 @@
       <c r="J99" t="s">
         <v>1635</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11081,7 +11055,7 @@
       <c r="R99" t="s">
         <v>1836</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11119,7 +11093,7 @@
       <c r="J100" t="s">
         <v>1635</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11160,7 +11134,7 @@
       <c r="J101" t="s">
         <v>1635</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11201,7 +11175,7 @@
       <c r="J102" t="s">
         <v>1635</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11242,7 +11216,7 @@
       <c r="J103" t="s">
         <v>1635</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11283,7 +11257,7 @@
       <c r="J104" t="s">
         <v>1635</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11324,7 +11298,7 @@
       <c r="J105" t="s">
         <v>1635</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11365,7 +11339,7 @@
       <c r="J106" t="s">
         <v>1635</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11406,7 +11380,7 @@
       <c r="J107" t="s">
         <v>1635</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11447,7 +11421,7 @@
       <c r="J108" t="s">
         <v>1635</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11488,7 +11462,7 @@
       <c r="J109" t="s">
         <v>1635</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11541,7 +11515,7 @@
       <c r="J110" t="s">
         <v>1635</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11597,7 +11571,7 @@
       <c r="J111" t="s">
         <v>1635</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11615,7 +11589,7 @@
       <c r="R111" t="s">
         <v>1838</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11653,7 +11627,7 @@
       <c r="J112" t="s">
         <v>1635</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11712,7 +11686,7 @@
       <c r="J113" t="s">
         <v>1635</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11756,7 +11730,7 @@
       <c r="J114" t="s">
         <v>1635</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11800,7 +11774,7 @@
       <c r="J115" t="s">
         <v>1635</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11818,7 +11792,7 @@
       <c r="R115" t="s">
         <v>1840</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11859,7 +11833,7 @@
       <c r="J116" t="s">
         <v>1635</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11918,7 +11892,7 @@
       <c r="J117" t="s">
         <v>1635</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11962,7 +11936,7 @@
       <c r="J118" t="s">
         <v>1635</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -12009,7 +11983,7 @@
       <c r="J119" t="s">
         <v>1635</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12050,7 +12024,7 @@
       <c r="J120" t="s">
         <v>1635</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12094,7 +12068,7 @@
       <c r="J121" t="s">
         <v>1635</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12141,7 +12115,7 @@
       <c r="J122" t="s">
         <v>1635</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12191,7 +12165,7 @@
       <c r="J123" t="s">
         <v>1635</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12235,7 +12209,7 @@
       <c r="J124" t="s">
         <v>1635</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12279,7 +12253,7 @@
       <c r="J125" t="s">
         <v>1635</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12297,7 +12271,7 @@
       <c r="R125" t="s">
         <v>1842</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12332,7 +12306,7 @@
       <c r="J126" t="s">
         <v>1635</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12350,7 +12324,7 @@
       <c r="R126" t="s">
         <v>1843</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12388,7 +12362,7 @@
       <c r="J127" t="s">
         <v>1635</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12444,7 +12418,7 @@
       <c r="J128" t="s">
         <v>1635</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12485,7 +12459,7 @@
       <c r="J129" t="s">
         <v>1635</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12526,7 +12500,7 @@
       <c r="J130" t="s">
         <v>1635</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12567,7 +12541,7 @@
       <c r="J131" t="s">
         <v>1635</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12611,7 +12585,7 @@
       <c r="J132" t="s">
         <v>1635</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12652,7 +12626,7 @@
       <c r="J133" t="s">
         <v>1635</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12670,7 +12644,7 @@
       <c r="R133" t="s">
         <v>1829</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12708,7 +12682,7 @@
       <c r="J134" t="s">
         <v>1635</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12726,7 +12700,7 @@
       <c r="R134" t="s">
         <v>1829</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12761,7 +12735,7 @@
       <c r="J135" t="s">
         <v>1635</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12802,7 +12776,7 @@
       <c r="J136" t="s">
         <v>1635</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12843,7 +12817,7 @@
       <c r="J137" t="s">
         <v>1635</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12884,7 +12858,7 @@
       <c r="J138" t="s">
         <v>1635</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12925,7 +12899,7 @@
       <c r="J139" t="s">
         <v>1635</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12972,7 +12946,7 @@
       <c r="J140" t="s">
         <v>1635</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -13013,7 +12987,7 @@
       <c r="J141" t="s">
         <v>1635</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13054,7 +13028,7 @@
       <c r="J142" t="s">
         <v>1635</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13098,7 +13072,7 @@
       <c r="J143" t="s">
         <v>1635</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13116,7 +13090,7 @@
       <c r="R143" t="s">
         <v>1829</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13151,7 +13125,7 @@
       <c r="J144" t="s">
         <v>1635</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13169,7 +13143,7 @@
       <c r="R144" t="s">
         <v>1829</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13207,7 +13181,7 @@
       <c r="J145" t="s">
         <v>1635</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13225,7 +13199,7 @@
       <c r="R145" t="s">
         <v>1829</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13260,7 +13234,7 @@
       <c r="J146" t="s">
         <v>1635</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13278,7 +13252,7 @@
       <c r="R146" t="s">
         <v>1837</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13313,7 +13287,7 @@
       <c r="J147" t="s">
         <v>1635</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13331,7 +13305,7 @@
       <c r="R147" t="s">
         <v>1844</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13366,7 +13340,7 @@
       <c r="J148" t="s">
         <v>1635</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13407,7 +13381,7 @@
       <c r="J149" t="s">
         <v>1635</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13425,7 +13399,7 @@
       <c r="R149" t="s">
         <v>1829</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13460,7 +13434,7 @@
       <c r="J150" t="s">
         <v>1635</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13478,7 +13452,7 @@
       <c r="R150" t="s">
         <v>1829</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13516,7 +13490,7 @@
       <c r="J151" t="s">
         <v>1635</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13534,7 +13508,7 @@
       <c r="R151" t="s">
         <v>1845</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13569,7 +13543,7 @@
       <c r="J152" t="s">
         <v>1635</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13587,7 +13561,7 @@
       <c r="R152" t="s">
         <v>1846</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13622,7 +13596,7 @@
       <c r="J153" t="s">
         <v>1635</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13631,7 +13605,7 @@
       <c r="M153" t="s">
         <v>1723</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13672,7 +13646,7 @@
       <c r="J154" t="s">
         <v>1635</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13713,7 +13687,7 @@
       <c r="J155" t="s">
         <v>1635</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13754,7 +13728,7 @@
       <c r="J156" t="s">
         <v>1635</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13795,7 +13769,7 @@
       <c r="J157" t="s">
         <v>1635</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13836,7 +13810,7 @@
       <c r="J158" t="s">
         <v>1635</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13877,7 +13851,7 @@
       <c r="J159" t="s">
         <v>1635</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13918,7 +13892,7 @@
       <c r="J160" t="s">
         <v>1635</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13959,7 +13933,7 @@
       <c r="J161" t="s">
         <v>1635</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -14000,7 +13974,7 @@
       <c r="J162" t="s">
         <v>1635</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -14018,7 +13992,7 @@
       <c r="R162" t="s">
         <v>1832</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14053,7 +14027,7 @@
       <c r="J163" t="s">
         <v>1635</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14071,7 +14045,7 @@
       <c r="R163" t="s">
         <v>1829</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14106,7 +14080,7 @@
       <c r="J164" t="s">
         <v>1635</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14150,7 +14124,7 @@
       <c r="J165" t="s">
         <v>1635</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14191,7 +14165,7 @@
       <c r="J166" t="s">
         <v>1635</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14209,7 +14183,7 @@
       <c r="R166" t="s">
         <v>1847</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14244,7 +14218,7 @@
       <c r="J167" t="s">
         <v>1635</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14288,7 +14262,7 @@
       <c r="J168" t="s">
         <v>1635</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14332,7 +14306,7 @@
       <c r="J169" t="s">
         <v>1635</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14373,7 +14347,7 @@
       <c r="J170" t="s">
         <v>1635</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14414,7 +14388,7 @@
       <c r="J171" t="s">
         <v>1635</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14455,7 +14429,7 @@
       <c r="J172" t="s">
         <v>1635</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14496,7 +14470,7 @@
       <c r="J173" t="s">
         <v>1635</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14537,7 +14511,7 @@
       <c r="J174" t="s">
         <v>1635</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14578,7 +14552,7 @@
       <c r="J175" t="s">
         <v>1635</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14619,7 +14593,7 @@
       <c r="J176" t="s">
         <v>1635</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14660,7 +14634,7 @@
       <c r="J177" t="s">
         <v>1635</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14701,7 +14675,7 @@
       <c r="J178" t="s">
         <v>1635</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14719,7 +14693,7 @@
       <c r="R178" t="s">
         <v>1845</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14757,7 +14731,7 @@
       <c r="J179" t="s">
         <v>1635</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14766,7 +14740,7 @@
       <c r="M179" t="s">
         <v>1720</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14807,7 +14781,7 @@
       <c r="J180" t="s">
         <v>1635</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14848,7 +14822,7 @@
       <c r="J181" t="s">
         <v>1635</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14866,7 +14840,7 @@
       <c r="R181" t="s">
         <v>1829</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14901,7 +14875,7 @@
       <c r="J182" t="s">
         <v>1635</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14942,7 +14916,7 @@
       <c r="J183" t="s">
         <v>1635</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14983,7 +14957,7 @@
       <c r="J184" t="s">
         <v>1635</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -15024,7 +14998,7 @@
       <c r="J185" t="s">
         <v>1635</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15065,7 +15039,7 @@
       <c r="J186" t="s">
         <v>1635</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15106,7 +15080,7 @@
       <c r="J187" t="s">
         <v>1635</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15147,7 +15121,7 @@
       <c r="J188" t="s">
         <v>1635</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15188,7 +15162,7 @@
       <c r="J189" t="s">
         <v>1635</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15229,7 +15203,7 @@
       <c r="J190" t="s">
         <v>1635</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15270,7 +15244,7 @@
       <c r="J191" t="s">
         <v>1635</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15311,7 +15285,7 @@
       <c r="J192" t="s">
         <v>1635</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15352,7 +15326,7 @@
       <c r="J193" t="s">
         <v>1635</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15393,7 +15367,7 @@
       <c r="J194" t="s">
         <v>1635</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15434,7 +15408,7 @@
       <c r="J195" t="s">
         <v>1635</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15452,7 +15426,7 @@
       <c r="R195" t="s">
         <v>1838</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15493,7 +15467,7 @@
       <c r="J196" t="s">
         <v>1635</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15511,7 +15485,7 @@
       <c r="R196" t="s">
         <v>1844</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15549,7 +15523,7 @@
       <c r="J197" t="s">
         <v>1635</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15590,7 +15564,7 @@
       <c r="J198" t="s">
         <v>1637</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15631,7 +15605,7 @@
       <c r="J199" t="s">
         <v>1636</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15672,7 +15646,7 @@
       <c r="J200" t="s">
         <v>1635</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15713,7 +15687,7 @@
       <c r="J201" t="s">
         <v>1635</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15754,7 +15728,7 @@
       <c r="J202" t="s">
         <v>1635</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15772,7 +15746,7 @@
       <c r="R202" t="s">
         <v>1829</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15810,7 +15784,7 @@
       <c r="J203" t="s">
         <v>1635</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15828,7 +15802,7 @@
       <c r="R203" t="s">
         <v>1837</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15863,7 +15837,7 @@
       <c r="J204" t="s">
         <v>1635</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15878,7 +15852,7 @@
       <c r="R204" t="s">
         <v>1848</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15916,7 +15890,7 @@
       <c r="J205" t="s">
         <v>1635</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15934,7 +15908,7 @@
       <c r="R205" t="s">
         <v>1849</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15972,7 +15946,7 @@
       <c r="J206" t="s">
         <v>1635</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15990,7 +15964,7 @@
       <c r="R206" t="s">
         <v>1817</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -16025,7 +15999,7 @@
       <c r="J207" t="s">
         <v>1635</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16066,7 +16040,7 @@
       <c r="J208" t="s">
         <v>1635</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16107,7 +16081,7 @@
       <c r="J209" t="s">
         <v>1635</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16148,7 +16122,7 @@
       <c r="J210" t="s">
         <v>1635</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16189,7 +16163,7 @@
       <c r="J211" t="s">
         <v>1635</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16230,7 +16204,7 @@
       <c r="J212" t="s">
         <v>1635</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16271,7 +16245,7 @@
       <c r="J213" t="s">
         <v>1635</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16312,7 +16286,7 @@
       <c r="J214" t="s">
         <v>1635</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16330,7 +16304,7 @@
       <c r="R214" t="s">
         <v>1850</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16368,7 +16342,7 @@
       <c r="J215" t="s">
         <v>1635</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16409,7 +16383,7 @@
       <c r="J216" t="s">
         <v>1635</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16450,7 +16424,7 @@
       <c r="J217" t="s">
         <v>1635</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16491,7 +16465,7 @@
       <c r="J218" t="s">
         <v>1635</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16532,7 +16506,7 @@
       <c r="J219" t="s">
         <v>1635</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16573,7 +16547,7 @@
       <c r="J220" t="s">
         <v>1635</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16614,7 +16588,7 @@
       <c r="J221" t="s">
         <v>1635</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16655,7 +16629,7 @@
       <c r="J222" t="s">
         <v>1635</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16696,7 +16670,7 @@
       <c r="J223" t="s">
         <v>1635</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16737,7 +16711,7 @@
       <c r="J224" t="s">
         <v>1635</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16778,7 +16752,7 @@
       <c r="J225" t="s">
         <v>1635</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16819,7 +16793,7 @@
       <c r="J226" t="s">
         <v>1635</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16860,7 +16834,7 @@
       <c r="J227" t="s">
         <v>1635</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16901,7 +16875,7 @@
       <c r="J228" t="s">
         <v>1635</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16942,7 +16916,7 @@
       <c r="J229" t="s">
         <v>1635</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16983,7 +16957,7 @@
       <c r="J230" t="s">
         <v>1635</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -17024,7 +16998,7 @@
       <c r="J231" t="s">
         <v>1635</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17065,7 +17039,7 @@
       <c r="J232" t="s">
         <v>1635</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17106,7 +17080,7 @@
       <c r="J233" t="s">
         <v>1635</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17147,7 +17121,7 @@
       <c r="J234" t="s">
         <v>1635</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17188,7 +17162,7 @@
       <c r="J235" t="s">
         <v>1635</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17229,7 +17203,7 @@
       <c r="J236" t="s">
         <v>1635</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17270,7 +17244,7 @@
       <c r="J237" t="s">
         <v>1635</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17311,7 +17285,7 @@
       <c r="J238" t="s">
         <v>1635</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17352,7 +17326,7 @@
       <c r="J239" t="s">
         <v>1635</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17370,7 +17344,7 @@
       <c r="R239" t="s">
         <v>1844</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17408,7 +17382,7 @@
       <c r="J240" t="s">
         <v>1635</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17449,7 +17423,7 @@
       <c r="J241" t="s">
         <v>1635</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17490,7 +17464,7 @@
       <c r="J242" t="s">
         <v>1635</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17508,7 +17482,7 @@
       <c r="R242" t="s">
         <v>1837</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17543,7 +17517,7 @@
       <c r="J243" t="s">
         <v>1635</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17584,7 +17558,7 @@
       <c r="J244" t="s">
         <v>1635</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17625,7 +17599,7 @@
       <c r="J245" t="s">
         <v>1635</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17666,7 +17640,7 @@
       <c r="J246" t="s">
         <v>1635</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17684,7 +17658,7 @@
       <c r="R246" t="s">
         <v>1817</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17722,7 +17696,7 @@
       <c r="J247" t="s">
         <v>1635</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17763,7 +17737,7 @@
       <c r="J248" t="s">
         <v>1635</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17804,7 +17778,7 @@
       <c r="J249" t="s">
         <v>1635</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17845,7 +17819,7 @@
       <c r="J250" t="s">
         <v>1635</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17886,7 +17860,7 @@
       <c r="J251" t="s">
         <v>1635</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17927,7 +17901,7 @@
       <c r="J252" t="s">
         <v>1635</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17968,7 +17942,7 @@
       <c r="J253" t="s">
         <v>1635</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17986,7 +17960,7 @@
       <c r="R253" t="s">
         <v>1847</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18027,7 +18001,7 @@
       <c r="J254" t="s">
         <v>1635</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18068,7 +18042,7 @@
       <c r="J255" t="s">
         <v>1635</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18109,7 +18083,7 @@
       <c r="J256" t="s">
         <v>1635</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18118,7 +18092,7 @@
       <c r="M256" t="s">
         <v>1719</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18156,7 +18130,7 @@
       <c r="J257" t="s">
         <v>1635</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18165,7 +18139,7 @@
       <c r="M257" t="s">
         <v>1720</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18209,7 +18183,7 @@
       <c r="J258" t="s">
         <v>1635</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18227,7 +18201,7 @@
       <c r="R258" t="s">
         <v>1829</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18265,7 +18239,7 @@
       <c r="J259" t="s">
         <v>1635</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18283,7 +18257,7 @@
       <c r="R259" t="s">
         <v>1845</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18321,7 +18295,7 @@
       <c r="J260" t="s">
         <v>1635</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18330,7 +18304,7 @@
       <c r="M260" t="s">
         <v>1714</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18374,7 +18348,7 @@
       <c r="J261" t="s">
         <v>1635</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18392,7 +18366,7 @@
       <c r="R261" t="s">
         <v>1851</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18430,7 +18404,7 @@
       <c r="J262" t="s">
         <v>1635</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18448,7 +18422,7 @@
       <c r="R262" t="s">
         <v>1845</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18486,7 +18460,7 @@
       <c r="J263" t="s">
         <v>1635</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18495,7 +18469,7 @@
       <c r="M263" t="s">
         <v>1714</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18539,7 +18513,7 @@
       <c r="J264" t="s">
         <v>1635</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18580,7 +18554,7 @@
       <c r="J265" t="s">
         <v>1635</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18621,7 +18595,7 @@
       <c r="J266" t="s">
         <v>1635</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18662,7 +18636,7 @@
       <c r="J267" t="s">
         <v>1635</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18706,7 +18680,7 @@
       <c r="J268" t="s">
         <v>1635</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18747,7 +18721,7 @@
       <c r="J269" t="s">
         <v>1635</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18788,7 +18762,7 @@
       <c r="J270" t="s">
         <v>1635</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18829,7 +18803,7 @@
       <c r="J271" t="s">
         <v>1635</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18870,7 +18844,7 @@
       <c r="J272" t="s">
         <v>1635</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18888,7 +18862,7 @@
       <c r="R272" t="s">
         <v>1852</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18929,7 +18903,7 @@
       <c r="J273" t="s">
         <v>1635</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18973,7 +18947,7 @@
       <c r="J274" t="s">
         <v>1635</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -19014,7 +18988,7 @@
       <c r="J275" t="s">
         <v>1635</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19055,7 +19029,7 @@
       <c r="J276" t="s">
         <v>1635</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19096,7 +19070,7 @@
       <c r="J277" t="s">
         <v>1635</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19137,7 +19111,7 @@
       <c r="J278" t="s">
         <v>1635</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19178,7 +19152,7 @@
       <c r="J279" t="s">
         <v>1635</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19219,7 +19193,7 @@
       <c r="J280" t="s">
         <v>1635</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19260,7 +19234,7 @@
       <c r="J281" t="s">
         <v>1635</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19301,7 +19275,7 @@
       <c r="J282" t="s">
         <v>1635</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19342,7 +19316,7 @@
       <c r="J283" t="s">
         <v>1635</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19383,7 +19357,7 @@
       <c r="J284" t="s">
         <v>1635</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19424,7 +19398,7 @@
       <c r="J285" t="s">
         <v>1635</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19465,7 +19439,7 @@
       <c r="J286" t="s">
         <v>1635</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19506,7 +19480,7 @@
       <c r="J287" t="s">
         <v>1635</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19547,7 +19521,7 @@
       <c r="J288" t="s">
         <v>1635</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19588,7 +19562,7 @@
       <c r="J289" t="s">
         <v>1635</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19629,7 +19603,7 @@
       <c r="J290" t="s">
         <v>1635</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19670,7 +19644,7 @@
       <c r="J291" t="s">
         <v>1635</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19711,7 +19685,7 @@
       <c r="J292" t="s">
         <v>1635</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19752,7 +19726,7 @@
       <c r="J293" t="s">
         <v>1635</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19793,7 +19767,7 @@
       <c r="J294" t="s">
         <v>1635</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19834,7 +19808,7 @@
       <c r="J295" t="s">
         <v>1635</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19852,7 +19826,7 @@
       <c r="R295" t="s">
         <v>1853</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19893,7 +19867,7 @@
       <c r="J296" t="s">
         <v>1635</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19911,7 +19885,7 @@
       <c r="R296" t="s">
         <v>1829</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19949,7 +19923,7 @@
       <c r="J297" t="s">
         <v>1635</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19990,7 +19964,7 @@
       <c r="J298" t="s">
         <v>1635</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20031,7 +20005,7 @@
       <c r="J299" t="s">
         <v>1636</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20072,7 +20046,7 @@
       <c r="J300" t="s">
         <v>1635</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20113,7 +20087,7 @@
       <c r="J301" t="s">
         <v>1635</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20951,7 +20925,7 @@
       <c r="R321" t="s">
         <v>1815</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21174,7 +21148,7 @@
       <c r="R326" t="s">
         <v>1854</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -22009,7 +21983,7 @@
       <c r="R346" t="s">
         <v>1855</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (14/10/2026 13:35)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5753,8 +5753,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5770,7 +5778,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5778,12 +5786,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6083,73 +6109,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6184,7 +6210,7 @@
       <c r="J2" t="s">
         <v>1635</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6228,7 +6254,7 @@
       <c r="J3" t="s">
         <v>1635</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6272,7 +6298,7 @@
       <c r="J4" t="s">
         <v>1635</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6290,7 +6316,7 @@
       <c r="R4" t="s">
         <v>1812</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6328,7 +6354,7 @@
       <c r="J5" t="s">
         <v>1636</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6378,7 +6404,7 @@
       <c r="J6" t="s">
         <v>1635</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6425,7 +6451,7 @@
       <c r="J7" t="s">
         <v>1635</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6472,7 +6498,7 @@
       <c r="J8" t="s">
         <v>1635</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6519,7 +6545,7 @@
       <c r="J9" t="s">
         <v>1635</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6566,7 +6592,7 @@
       <c r="J10" t="s">
         <v>1635</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6613,7 +6639,7 @@
       <c r="J11" t="s">
         <v>1635</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6660,7 +6686,7 @@
       <c r="J12" t="s">
         <v>1635</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6704,7 +6730,7 @@
       <c r="J13" t="s">
         <v>1635</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6722,7 +6748,7 @@
       <c r="R13" t="s">
         <v>1813</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6760,7 +6786,7 @@
       <c r="J14" t="s">
         <v>1635</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6778,7 +6804,7 @@
       <c r="R14" t="s">
         <v>1814</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6819,7 +6845,7 @@
       <c r="J15" t="s">
         <v>1635</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6837,7 +6863,7 @@
       <c r="R15" t="s">
         <v>1814</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6878,7 +6904,7 @@
       <c r="J16" t="s">
         <v>1635</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6922,7 +6948,7 @@
       <c r="J17" t="s">
         <v>1635</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6966,7 +6992,7 @@
       <c r="J18" t="s">
         <v>1635</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6984,7 +7010,7 @@
       <c r="R18" t="s">
         <v>1815</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7025,7 +7051,7 @@
       <c r="J19" t="s">
         <v>1635</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7069,7 +7095,7 @@
       <c r="J20" t="s">
         <v>1635</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7113,7 +7139,7 @@
       <c r="J21" t="s">
         <v>1635</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7131,7 +7157,7 @@
       <c r="R21" t="s">
         <v>1814</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7172,7 +7198,7 @@
       <c r="J22" t="s">
         <v>1635</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7190,7 +7216,7 @@
       <c r="R22" t="s">
         <v>1816</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7231,7 +7257,7 @@
       <c r="J23" t="s">
         <v>1635</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7249,7 +7275,7 @@
       <c r="R23" t="s">
         <v>1817</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7290,7 +7316,7 @@
       <c r="J24" t="s">
         <v>1635</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7334,7 +7360,7 @@
       <c r="J25" t="s">
         <v>1635</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7375,7 +7401,7 @@
       <c r="J26" t="s">
         <v>1637</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7393,7 +7419,7 @@
       <c r="R26" t="s">
         <v>1818</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7431,7 +7457,7 @@
       <c r="J27" t="s">
         <v>1635</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7449,7 +7475,7 @@
       <c r="R27" t="s">
         <v>1819</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7490,7 +7516,7 @@
       <c r="J28" t="s">
         <v>1635</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7534,7 +7560,7 @@
       <c r="J29" t="s">
         <v>1635</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7578,7 +7604,7 @@
       <c r="J30" t="s">
         <v>1635</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7622,7 +7648,7 @@
       <c r="J31" t="s">
         <v>1635</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7640,7 +7666,7 @@
       <c r="R31" t="s">
         <v>1820</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7681,7 +7707,7 @@
       <c r="J32" t="s">
         <v>1635</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7725,7 +7751,7 @@
       <c r="J33" t="s">
         <v>1635</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7743,7 +7769,7 @@
       <c r="R33" t="s">
         <v>1821</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7784,7 +7810,7 @@
       <c r="J34" t="s">
         <v>1635</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7828,7 +7854,7 @@
       <c r="J35" t="s">
         <v>1635</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7846,7 +7872,7 @@
       <c r="R35" t="s">
         <v>1822</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7887,7 +7913,7 @@
       <c r="J36" t="s">
         <v>1635</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7905,7 +7931,7 @@
       <c r="R36" t="s">
         <v>1822</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7946,7 +7972,7 @@
       <c r="J37" t="s">
         <v>1635</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7964,7 +7990,7 @@
       <c r="R37" t="s">
         <v>1822</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8005,7 +8031,7 @@
       <c r="J38" t="s">
         <v>1635</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8023,7 +8049,7 @@
       <c r="R38" t="s">
         <v>1822</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8064,7 +8090,7 @@
       <c r="J39" t="s">
         <v>1635</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8082,7 +8108,7 @@
       <c r="R39" t="s">
         <v>1822</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8123,7 +8149,7 @@
       <c r="J40" t="s">
         <v>1635</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8141,7 +8167,7 @@
       <c r="R40" t="s">
         <v>1823</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8182,7 +8208,7 @@
       <c r="J41" t="s">
         <v>1635</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8200,7 +8226,7 @@
       <c r="R41" t="s">
         <v>1814</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8241,7 +8267,7 @@
       <c r="J42" t="s">
         <v>1635</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8259,7 +8285,7 @@
       <c r="R42" t="s">
         <v>1822</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8300,7 +8326,7 @@
       <c r="J43" t="s">
         <v>1635</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8344,7 +8370,7 @@
       <c r="J44" t="s">
         <v>1635</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8362,7 +8388,7 @@
       <c r="R44" t="s">
         <v>1824</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8403,7 +8429,7 @@
       <c r="J45" t="s">
         <v>1635</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8421,7 +8447,7 @@
       <c r="R45" t="s">
         <v>1825</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8459,7 +8485,7 @@
       <c r="J46" t="s">
         <v>1635</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8503,7 +8529,7 @@
       <c r="J47" t="s">
         <v>1635</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8521,7 +8547,7 @@
       <c r="R47" t="s">
         <v>1826</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8562,7 +8588,7 @@
       <c r="J48" t="s">
         <v>1635</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8606,7 +8632,7 @@
       <c r="J49" t="s">
         <v>1635</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8650,7 +8676,7 @@
       <c r="J50" t="s">
         <v>1635</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8694,7 +8720,7 @@
       <c r="J51" t="s">
         <v>1635</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8741,7 +8767,7 @@
       <c r="J52" t="s">
         <v>1635</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8785,7 +8811,7 @@
       <c r="J53" t="s">
         <v>1635</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8829,7 +8855,7 @@
       <c r="J54" t="s">
         <v>1635</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8873,7 +8899,7 @@
       <c r="J55" t="s">
         <v>1635</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8923,7 +8949,7 @@
       <c r="J56" t="s">
         <v>1635</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8976,7 +9002,7 @@
       <c r="J57" t="s">
         <v>1635</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9026,7 +9052,7 @@
       <c r="J58" t="s">
         <v>1635</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9076,7 +9102,7 @@
       <c r="J59" t="s">
         <v>1635</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9094,7 +9120,7 @@
       <c r="R59" t="s">
         <v>1827</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9135,7 +9161,7 @@
       <c r="J60" t="s">
         <v>1635</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9179,7 +9205,7 @@
       <c r="J61" t="s">
         <v>1635</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9223,7 +9249,7 @@
       <c r="J62" t="s">
         <v>1635</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9267,7 +9293,7 @@
       <c r="J63" t="s">
         <v>1635</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9311,7 +9337,7 @@
       <c r="J64" t="s">
         <v>1635</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9355,7 +9381,7 @@
       <c r="J65" t="s">
         <v>1635</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9402,7 +9428,7 @@
       <c r="J66" t="s">
         <v>1635</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9420,7 +9446,7 @@
       <c r="R66" t="s">
         <v>1828</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9458,7 +9484,7 @@
       <c r="J67" t="s">
         <v>1635</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9502,7 +9528,7 @@
       <c r="J68" t="s">
         <v>1635</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9517,7 +9543,7 @@
       <c r="O68" t="s">
         <v>1732</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9561,7 +9587,7 @@
       <c r="J69" t="s">
         <v>1637</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9605,7 +9631,7 @@
       <c r="J70" t="s">
         <v>1635</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9649,7 +9675,7 @@
       <c r="J71" t="s">
         <v>1635</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9693,7 +9719,7 @@
       <c r="J72" t="s">
         <v>1635</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9737,7 +9763,7 @@
       <c r="J73" t="s">
         <v>1635</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9781,7 +9807,7 @@
       <c r="J74" t="s">
         <v>1635</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9825,7 +9851,7 @@
       <c r="J75" t="s">
         <v>1635</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9869,7 +9895,7 @@
       <c r="J76" t="s">
         <v>1635</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9887,7 +9913,7 @@
       <c r="R76" t="s">
         <v>1829</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9925,7 +9951,7 @@
       <c r="J77" t="s">
         <v>1635</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9943,7 +9969,7 @@
       <c r="R77" t="s">
         <v>1829</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9981,7 +10007,7 @@
       <c r="J78" t="s">
         <v>1635</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9999,7 +10025,7 @@
       <c r="R78" t="s">
         <v>1829</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10037,7 +10063,7 @@
       <c r="J79" t="s">
         <v>1635</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10055,7 +10081,7 @@
       <c r="R79" t="s">
         <v>1829</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10093,7 +10119,7 @@
       <c r="J80" t="s">
         <v>1635</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10137,7 +10163,7 @@
       <c r="J81" t="s">
         <v>1635</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10181,7 +10207,7 @@
       <c r="J82" t="s">
         <v>1635</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10225,7 +10251,7 @@
       <c r="J83" t="s">
         <v>1635</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10269,7 +10295,7 @@
       <c r="J84" t="s">
         <v>1635</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10313,7 +10339,7 @@
       <c r="J85" t="s">
         <v>1635</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10331,7 +10357,7 @@
       <c r="R85" t="s">
         <v>1830</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10369,7 +10395,7 @@
       <c r="J86" t="s">
         <v>1635</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10413,7 +10439,7 @@
       <c r="J87" t="s">
         <v>1635</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10431,7 +10457,7 @@
       <c r="R87" t="s">
         <v>1831</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10469,7 +10495,7 @@
       <c r="J88" t="s">
         <v>1635</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10513,7 +10539,7 @@
       <c r="J89" t="s">
         <v>1635</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10531,7 +10557,7 @@
       <c r="R89" t="s">
         <v>1832</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10566,7 +10592,7 @@
       <c r="J90" t="s">
         <v>1635</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10584,7 +10610,7 @@
       <c r="R90" t="s">
         <v>1833</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10619,7 +10645,7 @@
       <c r="J91" t="s">
         <v>1635</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10637,7 +10663,7 @@
       <c r="R91" t="s">
         <v>1817</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10675,7 +10701,7 @@
       <c r="J92" t="s">
         <v>1635</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10696,7 +10722,7 @@
       <c r="R92" t="s">
         <v>1817</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10737,7 +10763,7 @@
       <c r="J93" t="s">
         <v>1635</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10778,7 +10804,7 @@
       <c r="J94" t="s">
         <v>1635</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10822,7 +10848,7 @@
       <c r="J95" t="s">
         <v>1635</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10866,7 +10892,7 @@
       <c r="J96" t="s">
         <v>1635</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10884,7 +10910,7 @@
       <c r="R96" t="s">
         <v>1834</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10925,7 +10951,7 @@
       <c r="J97" t="s">
         <v>1635</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10940,7 +10966,7 @@
       <c r="R97" t="s">
         <v>1834</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10981,7 +11007,7 @@
       <c r="J98" t="s">
         <v>1635</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10999,7 +11025,7 @@
       <c r="R98" t="s">
         <v>1835</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11037,7 +11063,7 @@
       <c r="J99" t="s">
         <v>1635</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11055,7 +11081,7 @@
       <c r="R99" t="s">
         <v>1836</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11093,7 +11119,7 @@
       <c r="J100" t="s">
         <v>1635</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11134,7 +11160,7 @@
       <c r="J101" t="s">
         <v>1635</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11175,7 +11201,7 @@
       <c r="J102" t="s">
         <v>1635</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11216,7 +11242,7 @@
       <c r="J103" t="s">
         <v>1635</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11257,7 +11283,7 @@
       <c r="J104" t="s">
         <v>1635</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11298,7 +11324,7 @@
       <c r="J105" t="s">
         <v>1635</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11339,7 +11365,7 @@
       <c r="J106" t="s">
         <v>1635</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11380,7 +11406,7 @@
       <c r="J107" t="s">
         <v>1635</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11421,7 +11447,7 @@
       <c r="J108" t="s">
         <v>1635</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11462,7 +11488,7 @@
       <c r="J109" t="s">
         <v>1635</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11515,7 +11541,7 @@
       <c r="J110" t="s">
         <v>1635</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11571,7 +11597,7 @@
       <c r="J111" t="s">
         <v>1635</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11589,7 +11615,7 @@
       <c r="R111" t="s">
         <v>1838</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11627,7 +11653,7 @@
       <c r="J112" t="s">
         <v>1635</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11686,7 +11712,7 @@
       <c r="J113" t="s">
         <v>1635</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11730,7 +11756,7 @@
       <c r="J114" t="s">
         <v>1635</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11774,7 +11800,7 @@
       <c r="J115" t="s">
         <v>1635</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11792,7 +11818,7 @@
       <c r="R115" t="s">
         <v>1840</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11833,7 +11859,7 @@
       <c r="J116" t="s">
         <v>1635</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11892,7 +11918,7 @@
       <c r="J117" t="s">
         <v>1635</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11936,7 +11962,7 @@
       <c r="J118" t="s">
         <v>1635</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11983,7 +12009,7 @@
       <c r="J119" t="s">
         <v>1635</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12024,7 +12050,7 @@
       <c r="J120" t="s">
         <v>1635</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12068,7 +12094,7 @@
       <c r="J121" t="s">
         <v>1635</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12115,7 +12141,7 @@
       <c r="J122" t="s">
         <v>1635</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12165,7 +12191,7 @@
       <c r="J123" t="s">
         <v>1635</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12209,7 +12235,7 @@
       <c r="J124" t="s">
         <v>1635</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12253,7 +12279,7 @@
       <c r="J125" t="s">
         <v>1635</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12271,7 +12297,7 @@
       <c r="R125" t="s">
         <v>1842</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12306,7 +12332,7 @@
       <c r="J126" t="s">
         <v>1635</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12324,7 +12350,7 @@
       <c r="R126" t="s">
         <v>1843</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12362,7 +12388,7 @@
       <c r="J127" t="s">
         <v>1635</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12418,7 +12444,7 @@
       <c r="J128" t="s">
         <v>1635</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12459,7 +12485,7 @@
       <c r="J129" t="s">
         <v>1635</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12500,7 +12526,7 @@
       <c r="J130" t="s">
         <v>1635</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12541,7 +12567,7 @@
       <c r="J131" t="s">
         <v>1635</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12585,7 +12611,7 @@
       <c r="J132" t="s">
         <v>1635</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12626,7 +12652,7 @@
       <c r="J133" t="s">
         <v>1635</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12644,7 +12670,7 @@
       <c r="R133" t="s">
         <v>1829</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12682,7 +12708,7 @@
       <c r="J134" t="s">
         <v>1635</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12700,7 +12726,7 @@
       <c r="R134" t="s">
         <v>1829</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12735,7 +12761,7 @@
       <c r="J135" t="s">
         <v>1635</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12776,7 +12802,7 @@
       <c r="J136" t="s">
         <v>1635</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12817,7 +12843,7 @@
       <c r="J137" t="s">
         <v>1635</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12858,7 +12884,7 @@
       <c r="J138" t="s">
         <v>1635</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12899,7 +12925,7 @@
       <c r="J139" t="s">
         <v>1635</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12946,7 +12972,7 @@
       <c r="J140" t="s">
         <v>1635</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12987,7 +13013,7 @@
       <c r="J141" t="s">
         <v>1635</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13028,7 +13054,7 @@
       <c r="J142" t="s">
         <v>1635</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13072,7 +13098,7 @@
       <c r="J143" t="s">
         <v>1635</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13090,7 +13116,7 @@
       <c r="R143" t="s">
         <v>1829</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13125,7 +13151,7 @@
       <c r="J144" t="s">
         <v>1635</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13143,7 +13169,7 @@
       <c r="R144" t="s">
         <v>1829</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13181,7 +13207,7 @@
       <c r="J145" t="s">
         <v>1635</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13199,7 +13225,7 @@
       <c r="R145" t="s">
         <v>1829</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13234,7 +13260,7 @@
       <c r="J146" t="s">
         <v>1635</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13252,7 +13278,7 @@
       <c r="R146" t="s">
         <v>1837</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13287,7 +13313,7 @@
       <c r="J147" t="s">
         <v>1635</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13305,7 +13331,7 @@
       <c r="R147" t="s">
         <v>1844</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13340,7 +13366,7 @@
       <c r="J148" t="s">
         <v>1635</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13381,7 +13407,7 @@
       <c r="J149" t="s">
         <v>1635</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13399,7 +13425,7 @@
       <c r="R149" t="s">
         <v>1829</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13434,7 +13460,7 @@
       <c r="J150" t="s">
         <v>1635</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13452,7 +13478,7 @@
       <c r="R150" t="s">
         <v>1829</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13490,7 +13516,7 @@
       <c r="J151" t="s">
         <v>1635</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13508,7 +13534,7 @@
       <c r="R151" t="s">
         <v>1845</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13543,7 +13569,7 @@
       <c r="J152" t="s">
         <v>1635</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13561,7 +13587,7 @@
       <c r="R152" t="s">
         <v>1846</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13596,7 +13622,7 @@
       <c r="J153" t="s">
         <v>1635</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13605,7 +13631,7 @@
       <c r="M153" t="s">
         <v>1723</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13646,7 +13672,7 @@
       <c r="J154" t="s">
         <v>1635</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13687,7 +13713,7 @@
       <c r="J155" t="s">
         <v>1635</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13728,7 +13754,7 @@
       <c r="J156" t="s">
         <v>1635</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13769,7 +13795,7 @@
       <c r="J157" t="s">
         <v>1635</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13810,7 +13836,7 @@
       <c r="J158" t="s">
         <v>1635</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13851,7 +13877,7 @@
       <c r="J159" t="s">
         <v>1635</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13892,7 +13918,7 @@
       <c r="J160" t="s">
         <v>1635</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13933,7 +13959,7 @@
       <c r="J161" t="s">
         <v>1635</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13974,7 +14000,7 @@
       <c r="J162" t="s">
         <v>1635</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13992,7 +14018,7 @@
       <c r="R162" t="s">
         <v>1832</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14027,7 +14053,7 @@
       <c r="J163" t="s">
         <v>1635</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14045,7 +14071,7 @@
       <c r="R163" t="s">
         <v>1829</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14080,7 +14106,7 @@
       <c r="J164" t="s">
         <v>1635</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14124,7 +14150,7 @@
       <c r="J165" t="s">
         <v>1635</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14165,7 +14191,7 @@
       <c r="J166" t="s">
         <v>1635</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14183,7 +14209,7 @@
       <c r="R166" t="s">
         <v>1847</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14218,7 +14244,7 @@
       <c r="J167" t="s">
         <v>1635</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14262,7 +14288,7 @@
       <c r="J168" t="s">
         <v>1635</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14306,7 +14332,7 @@
       <c r="J169" t="s">
         <v>1635</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14347,7 +14373,7 @@
       <c r="J170" t="s">
         <v>1635</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14388,7 +14414,7 @@
       <c r="J171" t="s">
         <v>1635</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14429,7 +14455,7 @@
       <c r="J172" t="s">
         <v>1635</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14470,7 +14496,7 @@
       <c r="J173" t="s">
         <v>1635</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14511,7 +14537,7 @@
       <c r="J174" t="s">
         <v>1635</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14552,7 +14578,7 @@
       <c r="J175" t="s">
         <v>1635</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14593,7 +14619,7 @@
       <c r="J176" t="s">
         <v>1635</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14634,7 +14660,7 @@
       <c r="J177" t="s">
         <v>1635</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14675,7 +14701,7 @@
       <c r="J178" t="s">
         <v>1635</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14693,7 +14719,7 @@
       <c r="R178" t="s">
         <v>1845</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14731,7 +14757,7 @@
       <c r="J179" t="s">
         <v>1635</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14740,7 +14766,7 @@
       <c r="M179" t="s">
         <v>1720</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14781,7 +14807,7 @@
       <c r="J180" t="s">
         <v>1635</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14822,7 +14848,7 @@
       <c r="J181" t="s">
         <v>1635</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14840,7 +14866,7 @@
       <c r="R181" t="s">
         <v>1829</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14875,7 +14901,7 @@
       <c r="J182" t="s">
         <v>1635</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14916,7 +14942,7 @@
       <c r="J183" t="s">
         <v>1635</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14957,7 +14983,7 @@
       <c r="J184" t="s">
         <v>1635</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14998,7 +15024,7 @@
       <c r="J185" t="s">
         <v>1635</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15039,7 +15065,7 @@
       <c r="J186" t="s">
         <v>1635</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15080,7 +15106,7 @@
       <c r="J187" t="s">
         <v>1635</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15121,7 +15147,7 @@
       <c r="J188" t="s">
         <v>1635</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15162,7 +15188,7 @@
       <c r="J189" t="s">
         <v>1635</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15203,7 +15229,7 @@
       <c r="J190" t="s">
         <v>1635</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15244,7 +15270,7 @@
       <c r="J191" t="s">
         <v>1635</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15285,7 +15311,7 @@
       <c r="J192" t="s">
         <v>1635</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15326,7 +15352,7 @@
       <c r="J193" t="s">
         <v>1635</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15367,7 +15393,7 @@
       <c r="J194" t="s">
         <v>1635</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15408,7 +15434,7 @@
       <c r="J195" t="s">
         <v>1635</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15426,7 +15452,7 @@
       <c r="R195" t="s">
         <v>1838</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15467,7 +15493,7 @@
       <c r="J196" t="s">
         <v>1635</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15485,7 +15511,7 @@
       <c r="R196" t="s">
         <v>1844</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15523,7 +15549,7 @@
       <c r="J197" t="s">
         <v>1635</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15564,7 +15590,7 @@
       <c r="J198" t="s">
         <v>1637</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15605,7 +15631,7 @@
       <c r="J199" t="s">
         <v>1636</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15646,7 +15672,7 @@
       <c r="J200" t="s">
         <v>1635</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15687,7 +15713,7 @@
       <c r="J201" t="s">
         <v>1635</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15728,7 +15754,7 @@
       <c r="J202" t="s">
         <v>1635</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15746,7 +15772,7 @@
       <c r="R202" t="s">
         <v>1829</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15784,7 +15810,7 @@
       <c r="J203" t="s">
         <v>1635</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15802,7 +15828,7 @@
       <c r="R203" t="s">
         <v>1837</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15837,7 +15863,7 @@
       <c r="J204" t="s">
         <v>1635</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15852,7 +15878,7 @@
       <c r="R204" t="s">
         <v>1848</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15890,7 +15916,7 @@
       <c r="J205" t="s">
         <v>1635</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15908,7 +15934,7 @@
       <c r="R205" t="s">
         <v>1849</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15946,7 +15972,7 @@
       <c r="J206" t="s">
         <v>1635</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15964,7 +15990,7 @@
       <c r="R206" t="s">
         <v>1817</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15999,7 +16025,7 @@
       <c r="J207" t="s">
         <v>1635</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16040,7 +16066,7 @@
       <c r="J208" t="s">
         <v>1635</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16081,7 +16107,7 @@
       <c r="J209" t="s">
         <v>1635</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16122,7 +16148,7 @@
       <c r="J210" t="s">
         <v>1635</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16163,7 +16189,7 @@
       <c r="J211" t="s">
         <v>1635</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16204,7 +16230,7 @@
       <c r="J212" t="s">
         <v>1635</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16245,7 +16271,7 @@
       <c r="J213" t="s">
         <v>1635</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16286,7 +16312,7 @@
       <c r="J214" t="s">
         <v>1635</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16304,7 +16330,7 @@
       <c r="R214" t="s">
         <v>1850</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16342,7 +16368,7 @@
       <c r="J215" t="s">
         <v>1635</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16383,7 +16409,7 @@
       <c r="J216" t="s">
         <v>1635</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16424,7 +16450,7 @@
       <c r="J217" t="s">
         <v>1635</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16465,7 +16491,7 @@
       <c r="J218" t="s">
         <v>1635</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16506,7 +16532,7 @@
       <c r="J219" t="s">
         <v>1635</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16547,7 +16573,7 @@
       <c r="J220" t="s">
         <v>1635</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16588,7 +16614,7 @@
       <c r="J221" t="s">
         <v>1635</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16629,7 +16655,7 @@
       <c r="J222" t="s">
         <v>1635</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16670,7 +16696,7 @@
       <c r="J223" t="s">
         <v>1635</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16711,7 +16737,7 @@
       <c r="J224" t="s">
         <v>1635</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16752,7 +16778,7 @@
       <c r="J225" t="s">
         <v>1635</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16793,7 +16819,7 @@
       <c r="J226" t="s">
         <v>1635</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16834,7 +16860,7 @@
       <c r="J227" t="s">
         <v>1635</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16875,7 +16901,7 @@
       <c r="J228" t="s">
         <v>1635</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16916,7 +16942,7 @@
       <c r="J229" t="s">
         <v>1635</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16957,7 +16983,7 @@
       <c r="J230" t="s">
         <v>1635</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16998,7 +17024,7 @@
       <c r="J231" t="s">
         <v>1635</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17039,7 +17065,7 @@
       <c r="J232" t="s">
         <v>1635</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17080,7 +17106,7 @@
       <c r="J233" t="s">
         <v>1635</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17121,7 +17147,7 @@
       <c r="J234" t="s">
         <v>1635</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17162,7 +17188,7 @@
       <c r="J235" t="s">
         <v>1635</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17203,7 +17229,7 @@
       <c r="J236" t="s">
         <v>1635</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17244,7 +17270,7 @@
       <c r="J237" t="s">
         <v>1635</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17285,7 +17311,7 @@
       <c r="J238" t="s">
         <v>1635</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17326,7 +17352,7 @@
       <c r="J239" t="s">
         <v>1635</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17344,7 +17370,7 @@
       <c r="R239" t="s">
         <v>1844</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17382,7 +17408,7 @@
       <c r="J240" t="s">
         <v>1635</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17423,7 +17449,7 @@
       <c r="J241" t="s">
         <v>1635</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17464,7 +17490,7 @@
       <c r="J242" t="s">
         <v>1635</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17482,7 +17508,7 @@
       <c r="R242" t="s">
         <v>1837</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17517,7 +17543,7 @@
       <c r="J243" t="s">
         <v>1635</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17558,7 +17584,7 @@
       <c r="J244" t="s">
         <v>1635</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17599,7 +17625,7 @@
       <c r="J245" t="s">
         <v>1635</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17640,7 +17666,7 @@
       <c r="J246" t="s">
         <v>1635</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17658,7 +17684,7 @@
       <c r="R246" t="s">
         <v>1817</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17696,7 +17722,7 @@
       <c r="J247" t="s">
         <v>1635</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17737,7 +17763,7 @@
       <c r="J248" t="s">
         <v>1635</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17778,7 +17804,7 @@
       <c r="J249" t="s">
         <v>1635</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17819,7 +17845,7 @@
       <c r="J250" t="s">
         <v>1635</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17860,7 +17886,7 @@
       <c r="J251" t="s">
         <v>1635</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17901,7 +17927,7 @@
       <c r="J252" t="s">
         <v>1635</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17942,7 +17968,7 @@
       <c r="J253" t="s">
         <v>1635</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17960,7 +17986,7 @@
       <c r="R253" t="s">
         <v>1847</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18001,7 +18027,7 @@
       <c r="J254" t="s">
         <v>1635</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18042,7 +18068,7 @@
       <c r="J255" t="s">
         <v>1635</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18083,7 +18109,7 @@
       <c r="J256" t="s">
         <v>1635</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18092,7 +18118,7 @@
       <c r="M256" t="s">
         <v>1719</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18130,7 +18156,7 @@
       <c r="J257" t="s">
         <v>1635</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18139,7 +18165,7 @@
       <c r="M257" t="s">
         <v>1720</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18183,7 +18209,7 @@
       <c r="J258" t="s">
         <v>1635</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18201,7 +18227,7 @@
       <c r="R258" t="s">
         <v>1829</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18239,7 +18265,7 @@
       <c r="J259" t="s">
         <v>1635</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18257,7 +18283,7 @@
       <c r="R259" t="s">
         <v>1845</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18295,7 +18321,7 @@
       <c r="J260" t="s">
         <v>1635</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18304,7 +18330,7 @@
       <c r="M260" t="s">
         <v>1714</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18348,7 +18374,7 @@
       <c r="J261" t="s">
         <v>1635</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18366,7 +18392,7 @@
       <c r="R261" t="s">
         <v>1851</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18404,7 +18430,7 @@
       <c r="J262" t="s">
         <v>1635</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18422,7 +18448,7 @@
       <c r="R262" t="s">
         <v>1845</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18460,7 +18486,7 @@
       <c r="J263" t="s">
         <v>1635</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18469,7 +18495,7 @@
       <c r="M263" t="s">
         <v>1714</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18513,7 +18539,7 @@
       <c r="J264" t="s">
         <v>1635</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18554,7 +18580,7 @@
       <c r="J265" t="s">
         <v>1635</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18595,7 +18621,7 @@
       <c r="J266" t="s">
         <v>1635</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18636,7 +18662,7 @@
       <c r="J267" t="s">
         <v>1635</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18680,7 +18706,7 @@
       <c r="J268" t="s">
         <v>1635</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18721,7 +18747,7 @@
       <c r="J269" t="s">
         <v>1635</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18762,7 +18788,7 @@
       <c r="J270" t="s">
         <v>1635</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18803,7 +18829,7 @@
       <c r="J271" t="s">
         <v>1635</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18844,7 +18870,7 @@
       <c r="J272" t="s">
         <v>1635</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18862,7 +18888,7 @@
       <c r="R272" t="s">
         <v>1852</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18903,7 +18929,7 @@
       <c r="J273" t="s">
         <v>1635</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18947,7 +18973,7 @@
       <c r="J274" t="s">
         <v>1635</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18988,7 +19014,7 @@
       <c r="J275" t="s">
         <v>1635</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19029,7 +19055,7 @@
       <c r="J276" t="s">
         <v>1635</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19070,7 +19096,7 @@
       <c r="J277" t="s">
         <v>1635</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19111,7 +19137,7 @@
       <c r="J278" t="s">
         <v>1635</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19152,7 +19178,7 @@
       <c r="J279" t="s">
         <v>1635</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19193,7 +19219,7 @@
       <c r="J280" t="s">
         <v>1635</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19234,7 +19260,7 @@
       <c r="J281" t="s">
         <v>1635</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19275,7 +19301,7 @@
       <c r="J282" t="s">
         <v>1635</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19316,7 +19342,7 @@
       <c r="J283" t="s">
         <v>1635</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19357,7 +19383,7 @@
       <c r="J284" t="s">
         <v>1635</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19398,7 +19424,7 @@
       <c r="J285" t="s">
         <v>1635</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19439,7 +19465,7 @@
       <c r="J286" t="s">
         <v>1635</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19480,7 +19506,7 @@
       <c r="J287" t="s">
         <v>1635</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19521,7 +19547,7 @@
       <c r="J288" t="s">
         <v>1635</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19562,7 +19588,7 @@
       <c r="J289" t="s">
         <v>1635</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19603,7 +19629,7 @@
       <c r="J290" t="s">
         <v>1635</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19644,7 +19670,7 @@
       <c r="J291" t="s">
         <v>1635</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19685,7 +19711,7 @@
       <c r="J292" t="s">
         <v>1635</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19726,7 +19752,7 @@
       <c r="J293" t="s">
         <v>1635</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19767,7 +19793,7 @@
       <c r="J294" t="s">
         <v>1635</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19808,7 +19834,7 @@
       <c r="J295" t="s">
         <v>1635</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19826,7 +19852,7 @@
       <c r="R295" t="s">
         <v>1853</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19867,7 +19893,7 @@
       <c r="J296" t="s">
         <v>1635</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19885,7 +19911,7 @@
       <c r="R296" t="s">
         <v>1829</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19923,7 +19949,7 @@
       <c r="J297" t="s">
         <v>1635</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19964,7 +19990,7 @@
       <c r="J298" t="s">
         <v>1635</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20005,7 +20031,7 @@
       <c r="J299" t="s">
         <v>1636</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20046,7 +20072,7 @@
       <c r="J300" t="s">
         <v>1635</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20087,7 +20113,7 @@
       <c r="J301" t="s">
         <v>1635</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20925,7 +20951,7 @@
       <c r="R321" t="s">
         <v>1815</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21148,7 +21174,7 @@
       <c r="R326" t="s">
         <v>1854</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21983,7 +22009,7 @@
       <c r="R346" t="s">
         <v>1855</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (15/10/2026 12:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5753,16 +5753,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5778,7 +5770,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5786,30 +5778,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6109,73 +6083,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6210,7 +6184,7 @@
       <c r="J2" t="s">
         <v>1635</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6254,7 +6228,7 @@
       <c r="J3" t="s">
         <v>1635</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6298,7 +6272,7 @@
       <c r="J4" t="s">
         <v>1635</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6316,7 +6290,7 @@
       <c r="R4" t="s">
         <v>1812</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6354,7 +6328,7 @@
       <c r="J5" t="s">
         <v>1636</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6404,7 +6378,7 @@
       <c r="J6" t="s">
         <v>1635</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6451,7 +6425,7 @@
       <c r="J7" t="s">
         <v>1635</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6498,7 +6472,7 @@
       <c r="J8" t="s">
         <v>1635</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6545,7 +6519,7 @@
       <c r="J9" t="s">
         <v>1635</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6592,7 +6566,7 @@
       <c r="J10" t="s">
         <v>1635</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6639,7 +6613,7 @@
       <c r="J11" t="s">
         <v>1635</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6686,7 +6660,7 @@
       <c r="J12" t="s">
         <v>1635</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6730,7 +6704,7 @@
       <c r="J13" t="s">
         <v>1635</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6748,7 +6722,7 @@
       <c r="R13" t="s">
         <v>1813</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6786,7 +6760,7 @@
       <c r="J14" t="s">
         <v>1635</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6804,7 +6778,7 @@
       <c r="R14" t="s">
         <v>1814</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6845,7 +6819,7 @@
       <c r="J15" t="s">
         <v>1635</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6863,7 +6837,7 @@
       <c r="R15" t="s">
         <v>1814</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6904,7 +6878,7 @@
       <c r="J16" t="s">
         <v>1635</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6948,7 +6922,7 @@
       <c r="J17" t="s">
         <v>1635</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6992,7 +6966,7 @@
       <c r="J18" t="s">
         <v>1635</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -7010,7 +6984,7 @@
       <c r="R18" t="s">
         <v>1815</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7051,7 +7025,7 @@
       <c r="J19" t="s">
         <v>1635</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7095,7 +7069,7 @@
       <c r="J20" t="s">
         <v>1635</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7139,7 +7113,7 @@
       <c r="J21" t="s">
         <v>1635</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7157,7 +7131,7 @@
       <c r="R21" t="s">
         <v>1814</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7198,7 +7172,7 @@
       <c r="J22" t="s">
         <v>1635</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7216,7 +7190,7 @@
       <c r="R22" t="s">
         <v>1816</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7257,7 +7231,7 @@
       <c r="J23" t="s">
         <v>1635</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7275,7 +7249,7 @@
       <c r="R23" t="s">
         <v>1817</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7316,7 +7290,7 @@
       <c r="J24" t="s">
         <v>1635</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7360,7 +7334,7 @@
       <c r="J25" t="s">
         <v>1635</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7401,7 +7375,7 @@
       <c r="J26" t="s">
         <v>1637</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7419,7 +7393,7 @@
       <c r="R26" t="s">
         <v>1818</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7457,7 +7431,7 @@
       <c r="J27" t="s">
         <v>1635</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7475,7 +7449,7 @@
       <c r="R27" t="s">
         <v>1819</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7516,7 +7490,7 @@
       <c r="J28" t="s">
         <v>1635</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7560,7 +7534,7 @@
       <c r="J29" t="s">
         <v>1635</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7604,7 +7578,7 @@
       <c r="J30" t="s">
         <v>1635</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7648,7 +7622,7 @@
       <c r="J31" t="s">
         <v>1635</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7666,7 +7640,7 @@
       <c r="R31" t="s">
         <v>1820</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7707,7 +7681,7 @@
       <c r="J32" t="s">
         <v>1635</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7751,7 +7725,7 @@
       <c r="J33" t="s">
         <v>1635</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7769,7 +7743,7 @@
       <c r="R33" t="s">
         <v>1821</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7810,7 +7784,7 @@
       <c r="J34" t="s">
         <v>1635</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7854,7 +7828,7 @@
       <c r="J35" t="s">
         <v>1635</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7872,7 +7846,7 @@
       <c r="R35" t="s">
         <v>1822</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7913,7 +7887,7 @@
       <c r="J36" t="s">
         <v>1635</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7931,7 +7905,7 @@
       <c r="R36" t="s">
         <v>1822</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7972,7 +7946,7 @@
       <c r="J37" t="s">
         <v>1635</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7990,7 +7964,7 @@
       <c r="R37" t="s">
         <v>1822</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8031,7 +8005,7 @@
       <c r="J38" t="s">
         <v>1635</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8049,7 +8023,7 @@
       <c r="R38" t="s">
         <v>1822</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8090,7 +8064,7 @@
       <c r="J39" t="s">
         <v>1635</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8108,7 +8082,7 @@
       <c r="R39" t="s">
         <v>1822</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8149,7 +8123,7 @@
       <c r="J40" t="s">
         <v>1635</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8167,7 +8141,7 @@
       <c r="R40" t="s">
         <v>1823</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8208,7 +8182,7 @@
       <c r="J41" t="s">
         <v>1635</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8226,7 +8200,7 @@
       <c r="R41" t="s">
         <v>1814</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8267,7 +8241,7 @@
       <c r="J42" t="s">
         <v>1635</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8285,7 +8259,7 @@
       <c r="R42" t="s">
         <v>1822</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8326,7 +8300,7 @@
       <c r="J43" t="s">
         <v>1635</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8370,7 +8344,7 @@
       <c r="J44" t="s">
         <v>1635</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8388,7 +8362,7 @@
       <c r="R44" t="s">
         <v>1824</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8429,7 +8403,7 @@
       <c r="J45" t="s">
         <v>1635</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8447,7 +8421,7 @@
       <c r="R45" t="s">
         <v>1825</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8485,7 +8459,7 @@
       <c r="J46" t="s">
         <v>1635</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8529,7 +8503,7 @@
       <c r="J47" t="s">
         <v>1635</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8547,7 +8521,7 @@
       <c r="R47" t="s">
         <v>1826</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8588,7 +8562,7 @@
       <c r="J48" t="s">
         <v>1635</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8632,7 +8606,7 @@
       <c r="J49" t="s">
         <v>1635</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8676,7 +8650,7 @@
       <c r="J50" t="s">
         <v>1635</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8720,7 +8694,7 @@
       <c r="J51" t="s">
         <v>1635</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8767,7 +8741,7 @@
       <c r="J52" t="s">
         <v>1635</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8811,7 +8785,7 @@
       <c r="J53" t="s">
         <v>1635</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8855,7 +8829,7 @@
       <c r="J54" t="s">
         <v>1635</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8899,7 +8873,7 @@
       <c r="J55" t="s">
         <v>1635</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8949,7 +8923,7 @@
       <c r="J56" t="s">
         <v>1635</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -9002,7 +8976,7 @@
       <c r="J57" t="s">
         <v>1635</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9052,7 +9026,7 @@
       <c r="J58" t="s">
         <v>1635</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9102,7 +9076,7 @@
       <c r="J59" t="s">
         <v>1635</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9120,7 +9094,7 @@
       <c r="R59" t="s">
         <v>1827</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9161,7 +9135,7 @@
       <c r="J60" t="s">
         <v>1635</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9205,7 +9179,7 @@
       <c r="J61" t="s">
         <v>1635</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9249,7 +9223,7 @@
       <c r="J62" t="s">
         <v>1635</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9293,7 +9267,7 @@
       <c r="J63" t="s">
         <v>1635</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9337,7 +9311,7 @@
       <c r="J64" t="s">
         <v>1635</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9381,7 +9355,7 @@
       <c r="J65" t="s">
         <v>1635</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9428,7 +9402,7 @@
       <c r="J66" t="s">
         <v>1635</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9446,7 +9420,7 @@
       <c r="R66" t="s">
         <v>1828</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9484,7 +9458,7 @@
       <c r="J67" t="s">
         <v>1635</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9528,7 +9502,7 @@
       <c r="J68" t="s">
         <v>1635</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9543,7 +9517,7 @@
       <c r="O68" t="s">
         <v>1732</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9587,7 +9561,7 @@
       <c r="J69" t="s">
         <v>1637</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9631,7 +9605,7 @@
       <c r="J70" t="s">
         <v>1635</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9675,7 +9649,7 @@
       <c r="J71" t="s">
         <v>1635</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9719,7 +9693,7 @@
       <c r="J72" t="s">
         <v>1635</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9763,7 +9737,7 @@
       <c r="J73" t="s">
         <v>1635</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9807,7 +9781,7 @@
       <c r="J74" t="s">
         <v>1635</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9851,7 +9825,7 @@
       <c r="J75" t="s">
         <v>1635</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9895,7 +9869,7 @@
       <c r="J76" t="s">
         <v>1635</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9913,7 +9887,7 @@
       <c r="R76" t="s">
         <v>1829</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9951,7 +9925,7 @@
       <c r="J77" t="s">
         <v>1635</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9969,7 +9943,7 @@
       <c r="R77" t="s">
         <v>1829</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -10007,7 +9981,7 @@
       <c r="J78" t="s">
         <v>1635</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -10025,7 +9999,7 @@
       <c r="R78" t="s">
         <v>1829</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10063,7 +10037,7 @@
       <c r="J79" t="s">
         <v>1635</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10081,7 +10055,7 @@
       <c r="R79" t="s">
         <v>1829</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10119,7 +10093,7 @@
       <c r="J80" t="s">
         <v>1635</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10163,7 +10137,7 @@
       <c r="J81" t="s">
         <v>1635</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10207,7 +10181,7 @@
       <c r="J82" t="s">
         <v>1635</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10251,7 +10225,7 @@
       <c r="J83" t="s">
         <v>1635</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10295,7 +10269,7 @@
       <c r="J84" t="s">
         <v>1635</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10339,7 +10313,7 @@
       <c r="J85" t="s">
         <v>1635</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10357,7 +10331,7 @@
       <c r="R85" t="s">
         <v>1830</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10395,7 +10369,7 @@
       <c r="J86" t="s">
         <v>1635</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10439,7 +10413,7 @@
       <c r="J87" t="s">
         <v>1635</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10457,7 +10431,7 @@
       <c r="R87" t="s">
         <v>1831</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10495,7 +10469,7 @@
       <c r="J88" t="s">
         <v>1635</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10539,7 +10513,7 @@
       <c r="J89" t="s">
         <v>1635</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10557,7 +10531,7 @@
       <c r="R89" t="s">
         <v>1832</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10592,7 +10566,7 @@
       <c r="J90" t="s">
         <v>1635</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10610,7 +10584,7 @@
       <c r="R90" t="s">
         <v>1833</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10645,7 +10619,7 @@
       <c r="J91" t="s">
         <v>1635</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10663,7 +10637,7 @@
       <c r="R91" t="s">
         <v>1817</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10701,7 +10675,7 @@
       <c r="J92" t="s">
         <v>1635</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10722,7 +10696,7 @@
       <c r="R92" t="s">
         <v>1817</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10763,7 +10737,7 @@
       <c r="J93" t="s">
         <v>1635</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10804,7 +10778,7 @@
       <c r="J94" t="s">
         <v>1635</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10848,7 +10822,7 @@
       <c r="J95" t="s">
         <v>1635</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10892,7 +10866,7 @@
       <c r="J96" t="s">
         <v>1635</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10910,7 +10884,7 @@
       <c r="R96" t="s">
         <v>1834</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10951,7 +10925,7 @@
       <c r="J97" t="s">
         <v>1635</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10966,7 +10940,7 @@
       <c r="R97" t="s">
         <v>1834</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -11007,7 +10981,7 @@
       <c r="J98" t="s">
         <v>1635</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -11025,7 +10999,7 @@
       <c r="R98" t="s">
         <v>1835</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11063,7 +11037,7 @@
       <c r="J99" t="s">
         <v>1635</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11081,7 +11055,7 @@
       <c r="R99" t="s">
         <v>1836</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11119,7 +11093,7 @@
       <c r="J100" t="s">
         <v>1635</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11160,7 +11134,7 @@
       <c r="J101" t="s">
         <v>1635</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11201,7 +11175,7 @@
       <c r="J102" t="s">
         <v>1635</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11242,7 +11216,7 @@
       <c r="J103" t="s">
         <v>1635</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11283,7 +11257,7 @@
       <c r="J104" t="s">
         <v>1635</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11324,7 +11298,7 @@
       <c r="J105" t="s">
         <v>1635</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11365,7 +11339,7 @@
       <c r="J106" t="s">
         <v>1635</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11406,7 +11380,7 @@
       <c r="J107" t="s">
         <v>1635</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11447,7 +11421,7 @@
       <c r="J108" t="s">
         <v>1635</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11488,7 +11462,7 @@
       <c r="J109" t="s">
         <v>1635</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11541,7 +11515,7 @@
       <c r="J110" t="s">
         <v>1635</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11597,7 +11571,7 @@
       <c r="J111" t="s">
         <v>1635</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11615,7 +11589,7 @@
       <c r="R111" t="s">
         <v>1838</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11653,7 +11627,7 @@
       <c r="J112" t="s">
         <v>1635</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11712,7 +11686,7 @@
       <c r="J113" t="s">
         <v>1635</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11756,7 +11730,7 @@
       <c r="J114" t="s">
         <v>1635</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11800,7 +11774,7 @@
       <c r="J115" t="s">
         <v>1635</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11818,7 +11792,7 @@
       <c r="R115" t="s">
         <v>1840</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11859,7 +11833,7 @@
       <c r="J116" t="s">
         <v>1635</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11918,7 +11892,7 @@
       <c r="J117" t="s">
         <v>1635</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11962,7 +11936,7 @@
       <c r="J118" t="s">
         <v>1635</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -12009,7 +11983,7 @@
       <c r="J119" t="s">
         <v>1635</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12050,7 +12024,7 @@
       <c r="J120" t="s">
         <v>1635</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12094,7 +12068,7 @@
       <c r="J121" t="s">
         <v>1635</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12141,7 +12115,7 @@
       <c r="J122" t="s">
         <v>1635</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12191,7 +12165,7 @@
       <c r="J123" t="s">
         <v>1635</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12235,7 +12209,7 @@
       <c r="J124" t="s">
         <v>1635</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12279,7 +12253,7 @@
       <c r="J125" t="s">
         <v>1635</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12297,7 +12271,7 @@
       <c r="R125" t="s">
         <v>1842</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12332,7 +12306,7 @@
       <c r="J126" t="s">
         <v>1635</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12350,7 +12324,7 @@
       <c r="R126" t="s">
         <v>1843</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12388,7 +12362,7 @@
       <c r="J127" t="s">
         <v>1635</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12444,7 +12418,7 @@
       <c r="J128" t="s">
         <v>1635</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12485,7 +12459,7 @@
       <c r="J129" t="s">
         <v>1635</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12526,7 +12500,7 @@
       <c r="J130" t="s">
         <v>1635</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12567,7 +12541,7 @@
       <c r="J131" t="s">
         <v>1635</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12611,7 +12585,7 @@
       <c r="J132" t="s">
         <v>1635</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12652,7 +12626,7 @@
       <c r="J133" t="s">
         <v>1635</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12670,7 +12644,7 @@
       <c r="R133" t="s">
         <v>1829</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12708,7 +12682,7 @@
       <c r="J134" t="s">
         <v>1635</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12726,7 +12700,7 @@
       <c r="R134" t="s">
         <v>1829</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12761,7 +12735,7 @@
       <c r="J135" t="s">
         <v>1635</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12802,7 +12776,7 @@
       <c r="J136" t="s">
         <v>1635</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12843,7 +12817,7 @@
       <c r="J137" t="s">
         <v>1635</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12884,7 +12858,7 @@
       <c r="J138" t="s">
         <v>1635</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12925,7 +12899,7 @@
       <c r="J139" t="s">
         <v>1635</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12972,7 +12946,7 @@
       <c r="J140" t="s">
         <v>1635</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -13013,7 +12987,7 @@
       <c r="J141" t="s">
         <v>1635</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13054,7 +13028,7 @@
       <c r="J142" t="s">
         <v>1635</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13098,7 +13072,7 @@
       <c r="J143" t="s">
         <v>1635</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13116,7 +13090,7 @@
       <c r="R143" t="s">
         <v>1829</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13151,7 +13125,7 @@
       <c r="J144" t="s">
         <v>1635</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13169,7 +13143,7 @@
       <c r="R144" t="s">
         <v>1829</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13207,7 +13181,7 @@
       <c r="J145" t="s">
         <v>1635</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13225,7 +13199,7 @@
       <c r="R145" t="s">
         <v>1829</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13260,7 +13234,7 @@
       <c r="J146" t="s">
         <v>1635</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13278,7 +13252,7 @@
       <c r="R146" t="s">
         <v>1837</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13313,7 +13287,7 @@
       <c r="J147" t="s">
         <v>1635</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13331,7 +13305,7 @@
       <c r="R147" t="s">
         <v>1844</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13366,7 +13340,7 @@
       <c r="J148" t="s">
         <v>1635</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13407,7 +13381,7 @@
       <c r="J149" t="s">
         <v>1635</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13425,7 +13399,7 @@
       <c r="R149" t="s">
         <v>1829</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13460,7 +13434,7 @@
       <c r="J150" t="s">
         <v>1635</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13478,7 +13452,7 @@
       <c r="R150" t="s">
         <v>1829</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13516,7 +13490,7 @@
       <c r="J151" t="s">
         <v>1635</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13534,7 +13508,7 @@
       <c r="R151" t="s">
         <v>1845</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13569,7 +13543,7 @@
       <c r="J152" t="s">
         <v>1635</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13587,7 +13561,7 @@
       <c r="R152" t="s">
         <v>1846</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13622,7 +13596,7 @@
       <c r="J153" t="s">
         <v>1635</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13631,7 +13605,7 @@
       <c r="M153" t="s">
         <v>1723</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13672,7 +13646,7 @@
       <c r="J154" t="s">
         <v>1635</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13713,7 +13687,7 @@
       <c r="J155" t="s">
         <v>1635</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13754,7 +13728,7 @@
       <c r="J156" t="s">
         <v>1635</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13795,7 +13769,7 @@
       <c r="J157" t="s">
         <v>1635</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13836,7 +13810,7 @@
       <c r="J158" t="s">
         <v>1635</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13877,7 +13851,7 @@
       <c r="J159" t="s">
         <v>1635</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13918,7 +13892,7 @@
       <c r="J160" t="s">
         <v>1635</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13959,7 +13933,7 @@
       <c r="J161" t="s">
         <v>1635</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -14000,7 +13974,7 @@
       <c r="J162" t="s">
         <v>1635</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -14018,7 +13992,7 @@
       <c r="R162" t="s">
         <v>1832</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14053,7 +14027,7 @@
       <c r="J163" t="s">
         <v>1635</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14071,7 +14045,7 @@
       <c r="R163" t="s">
         <v>1829</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14106,7 +14080,7 @@
       <c r="J164" t="s">
         <v>1635</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14150,7 +14124,7 @@
       <c r="J165" t="s">
         <v>1635</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14191,7 +14165,7 @@
       <c r="J166" t="s">
         <v>1635</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14209,7 +14183,7 @@
       <c r="R166" t="s">
         <v>1847</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14244,7 +14218,7 @@
       <c r="J167" t="s">
         <v>1635</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14288,7 +14262,7 @@
       <c r="J168" t="s">
         <v>1635</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14332,7 +14306,7 @@
       <c r="J169" t="s">
         <v>1635</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14373,7 +14347,7 @@
       <c r="J170" t="s">
         <v>1635</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14414,7 +14388,7 @@
       <c r="J171" t="s">
         <v>1635</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14455,7 +14429,7 @@
       <c r="J172" t="s">
         <v>1635</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14496,7 +14470,7 @@
       <c r="J173" t="s">
         <v>1635</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14537,7 +14511,7 @@
       <c r="J174" t="s">
         <v>1635</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14578,7 +14552,7 @@
       <c r="J175" t="s">
         <v>1635</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14619,7 +14593,7 @@
       <c r="J176" t="s">
         <v>1635</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14660,7 +14634,7 @@
       <c r="J177" t="s">
         <v>1635</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14701,7 +14675,7 @@
       <c r="J178" t="s">
         <v>1635</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14719,7 +14693,7 @@
       <c r="R178" t="s">
         <v>1845</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14757,7 +14731,7 @@
       <c r="J179" t="s">
         <v>1635</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14766,7 +14740,7 @@
       <c r="M179" t="s">
         <v>1720</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14807,7 +14781,7 @@
       <c r="J180" t="s">
         <v>1635</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14848,7 +14822,7 @@
       <c r="J181" t="s">
         <v>1635</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14866,7 +14840,7 @@
       <c r="R181" t="s">
         <v>1829</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14901,7 +14875,7 @@
       <c r="J182" t="s">
         <v>1635</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14942,7 +14916,7 @@
       <c r="J183" t="s">
         <v>1635</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14983,7 +14957,7 @@
       <c r="J184" t="s">
         <v>1635</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -15024,7 +14998,7 @@
       <c r="J185" t="s">
         <v>1635</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15065,7 +15039,7 @@
       <c r="J186" t="s">
         <v>1635</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15106,7 +15080,7 @@
       <c r="J187" t="s">
         <v>1635</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15147,7 +15121,7 @@
       <c r="J188" t="s">
         <v>1635</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15188,7 +15162,7 @@
       <c r="J189" t="s">
         <v>1635</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15229,7 +15203,7 @@
       <c r="J190" t="s">
         <v>1635</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15270,7 +15244,7 @@
       <c r="J191" t="s">
         <v>1635</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15311,7 +15285,7 @@
       <c r="J192" t="s">
         <v>1635</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15352,7 +15326,7 @@
       <c r="J193" t="s">
         <v>1635</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15393,7 +15367,7 @@
       <c r="J194" t="s">
         <v>1635</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15434,7 +15408,7 @@
       <c r="J195" t="s">
         <v>1635</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15452,7 +15426,7 @@
       <c r="R195" t="s">
         <v>1838</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15493,7 +15467,7 @@
       <c r="J196" t="s">
         <v>1635</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15511,7 +15485,7 @@
       <c r="R196" t="s">
         <v>1844</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15549,7 +15523,7 @@
       <c r="J197" t="s">
         <v>1635</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15590,7 +15564,7 @@
       <c r="J198" t="s">
         <v>1637</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15631,7 +15605,7 @@
       <c r="J199" t="s">
         <v>1636</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15672,7 +15646,7 @@
       <c r="J200" t="s">
         <v>1635</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15713,7 +15687,7 @@
       <c r="J201" t="s">
         <v>1635</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15754,7 +15728,7 @@
       <c r="J202" t="s">
         <v>1635</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15772,7 +15746,7 @@
       <c r="R202" t="s">
         <v>1829</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15810,7 +15784,7 @@
       <c r="J203" t="s">
         <v>1635</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15828,7 +15802,7 @@
       <c r="R203" t="s">
         <v>1837</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15863,7 +15837,7 @@
       <c r="J204" t="s">
         <v>1635</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15878,7 +15852,7 @@
       <c r="R204" t="s">
         <v>1848</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15916,7 +15890,7 @@
       <c r="J205" t="s">
         <v>1635</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15934,7 +15908,7 @@
       <c r="R205" t="s">
         <v>1849</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15972,7 +15946,7 @@
       <c r="J206" t="s">
         <v>1635</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15990,7 +15964,7 @@
       <c r="R206" t="s">
         <v>1817</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -16025,7 +15999,7 @@
       <c r="J207" t="s">
         <v>1635</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16066,7 +16040,7 @@
       <c r="J208" t="s">
         <v>1635</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16107,7 +16081,7 @@
       <c r="J209" t="s">
         <v>1635</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16148,7 +16122,7 @@
       <c r="J210" t="s">
         <v>1635</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16189,7 +16163,7 @@
       <c r="J211" t="s">
         <v>1635</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16230,7 +16204,7 @@
       <c r="J212" t="s">
         <v>1635</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16271,7 +16245,7 @@
       <c r="J213" t="s">
         <v>1635</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16312,7 +16286,7 @@
       <c r="J214" t="s">
         <v>1635</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16330,7 +16304,7 @@
       <c r="R214" t="s">
         <v>1850</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16368,7 +16342,7 @@
       <c r="J215" t="s">
         <v>1635</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16409,7 +16383,7 @@
       <c r="J216" t="s">
         <v>1635</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16450,7 +16424,7 @@
       <c r="J217" t="s">
         <v>1635</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16491,7 +16465,7 @@
       <c r="J218" t="s">
         <v>1635</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16532,7 +16506,7 @@
       <c r="J219" t="s">
         <v>1635</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16573,7 +16547,7 @@
       <c r="J220" t="s">
         <v>1635</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16614,7 +16588,7 @@
       <c r="J221" t="s">
         <v>1635</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16655,7 +16629,7 @@
       <c r="J222" t="s">
         <v>1635</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16696,7 +16670,7 @@
       <c r="J223" t="s">
         <v>1635</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16737,7 +16711,7 @@
       <c r="J224" t="s">
         <v>1635</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16778,7 +16752,7 @@
       <c r="J225" t="s">
         <v>1635</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16819,7 +16793,7 @@
       <c r="J226" t="s">
         <v>1635</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16860,7 +16834,7 @@
       <c r="J227" t="s">
         <v>1635</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16901,7 +16875,7 @@
       <c r="J228" t="s">
         <v>1635</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16942,7 +16916,7 @@
       <c r="J229" t="s">
         <v>1635</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16983,7 +16957,7 @@
       <c r="J230" t="s">
         <v>1635</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -17024,7 +16998,7 @@
       <c r="J231" t="s">
         <v>1635</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17065,7 +17039,7 @@
       <c r="J232" t="s">
         <v>1635</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17106,7 +17080,7 @@
       <c r="J233" t="s">
         <v>1635</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17147,7 +17121,7 @@
       <c r="J234" t="s">
         <v>1635</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17188,7 +17162,7 @@
       <c r="J235" t="s">
         <v>1635</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17229,7 +17203,7 @@
       <c r="J236" t="s">
         <v>1635</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17270,7 +17244,7 @@
       <c r="J237" t="s">
         <v>1635</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17311,7 +17285,7 @@
       <c r="J238" t="s">
         <v>1635</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17352,7 +17326,7 @@
       <c r="J239" t="s">
         <v>1635</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17370,7 +17344,7 @@
       <c r="R239" t="s">
         <v>1844</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17408,7 +17382,7 @@
       <c r="J240" t="s">
         <v>1635</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17449,7 +17423,7 @@
       <c r="J241" t="s">
         <v>1635</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17490,7 +17464,7 @@
       <c r="J242" t="s">
         <v>1635</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17508,7 +17482,7 @@
       <c r="R242" t="s">
         <v>1837</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17543,7 +17517,7 @@
       <c r="J243" t="s">
         <v>1635</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17584,7 +17558,7 @@
       <c r="J244" t="s">
         <v>1635</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17625,7 +17599,7 @@
       <c r="J245" t="s">
         <v>1635</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17666,7 +17640,7 @@
       <c r="J246" t="s">
         <v>1635</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17684,7 +17658,7 @@
       <c r="R246" t="s">
         <v>1817</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17722,7 +17696,7 @@
       <c r="J247" t="s">
         <v>1635</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17763,7 +17737,7 @@
       <c r="J248" t="s">
         <v>1635</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17804,7 +17778,7 @@
       <c r="J249" t="s">
         <v>1635</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17845,7 +17819,7 @@
       <c r="J250" t="s">
         <v>1635</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17886,7 +17860,7 @@
       <c r="J251" t="s">
         <v>1635</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17927,7 +17901,7 @@
       <c r="J252" t="s">
         <v>1635</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17968,7 +17942,7 @@
       <c r="J253" t="s">
         <v>1635</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17986,7 +17960,7 @@
       <c r="R253" t="s">
         <v>1847</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18027,7 +18001,7 @@
       <c r="J254" t="s">
         <v>1635</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18068,7 +18042,7 @@
       <c r="J255" t="s">
         <v>1635</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18109,7 +18083,7 @@
       <c r="J256" t="s">
         <v>1635</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18118,7 +18092,7 @@
       <c r="M256" t="s">
         <v>1719</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18156,7 +18130,7 @@
       <c r="J257" t="s">
         <v>1635</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18165,7 +18139,7 @@
       <c r="M257" t="s">
         <v>1720</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18209,7 +18183,7 @@
       <c r="J258" t="s">
         <v>1635</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18227,7 +18201,7 @@
       <c r="R258" t="s">
         <v>1829</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18265,7 +18239,7 @@
       <c r="J259" t="s">
         <v>1635</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18283,7 +18257,7 @@
       <c r="R259" t="s">
         <v>1845</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18321,7 +18295,7 @@
       <c r="J260" t="s">
         <v>1635</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18330,7 +18304,7 @@
       <c r="M260" t="s">
         <v>1714</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18374,7 +18348,7 @@
       <c r="J261" t="s">
         <v>1635</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18392,7 +18366,7 @@
       <c r="R261" t="s">
         <v>1851</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18430,7 +18404,7 @@
       <c r="J262" t="s">
         <v>1635</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18448,7 +18422,7 @@
       <c r="R262" t="s">
         <v>1845</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18486,7 +18460,7 @@
       <c r="J263" t="s">
         <v>1635</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18495,7 +18469,7 @@
       <c r="M263" t="s">
         <v>1714</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18539,7 +18513,7 @@
       <c r="J264" t="s">
         <v>1635</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18580,7 +18554,7 @@
       <c r="J265" t="s">
         <v>1635</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18621,7 +18595,7 @@
       <c r="J266" t="s">
         <v>1635</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18662,7 +18636,7 @@
       <c r="J267" t="s">
         <v>1635</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18706,7 +18680,7 @@
       <c r="J268" t="s">
         <v>1635</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18747,7 +18721,7 @@
       <c r="J269" t="s">
         <v>1635</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18788,7 +18762,7 @@
       <c r="J270" t="s">
         <v>1635</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18829,7 +18803,7 @@
       <c r="J271" t="s">
         <v>1635</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18870,7 +18844,7 @@
       <c r="J272" t="s">
         <v>1635</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18888,7 +18862,7 @@
       <c r="R272" t="s">
         <v>1852</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18929,7 +18903,7 @@
       <c r="J273" t="s">
         <v>1635</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18973,7 +18947,7 @@
       <c r="J274" t="s">
         <v>1635</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -19014,7 +18988,7 @@
       <c r="J275" t="s">
         <v>1635</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19055,7 +19029,7 @@
       <c r="J276" t="s">
         <v>1635</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19096,7 +19070,7 @@
       <c r="J277" t="s">
         <v>1635</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19137,7 +19111,7 @@
       <c r="J278" t="s">
         <v>1635</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19178,7 +19152,7 @@
       <c r="J279" t="s">
         <v>1635</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19219,7 +19193,7 @@
       <c r="J280" t="s">
         <v>1635</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19260,7 +19234,7 @@
       <c r="J281" t="s">
         <v>1635</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19301,7 +19275,7 @@
       <c r="J282" t="s">
         <v>1635</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19342,7 +19316,7 @@
       <c r="J283" t="s">
         <v>1635</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19383,7 +19357,7 @@
       <c r="J284" t="s">
         <v>1635</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19424,7 +19398,7 @@
       <c r="J285" t="s">
         <v>1635</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19465,7 +19439,7 @@
       <c r="J286" t="s">
         <v>1635</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19506,7 +19480,7 @@
       <c r="J287" t="s">
         <v>1635</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19547,7 +19521,7 @@
       <c r="J288" t="s">
         <v>1635</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19588,7 +19562,7 @@
       <c r="J289" t="s">
         <v>1635</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19629,7 +19603,7 @@
       <c r="J290" t="s">
         <v>1635</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19670,7 +19644,7 @@
       <c r="J291" t="s">
         <v>1635</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19711,7 +19685,7 @@
       <c r="J292" t="s">
         <v>1635</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19752,7 +19726,7 @@
       <c r="J293" t="s">
         <v>1635</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19793,7 +19767,7 @@
       <c r="J294" t="s">
         <v>1635</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19834,7 +19808,7 @@
       <c r="J295" t="s">
         <v>1635</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19852,7 +19826,7 @@
       <c r="R295" t="s">
         <v>1853</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19893,7 +19867,7 @@
       <c r="J296" t="s">
         <v>1635</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19911,7 +19885,7 @@
       <c r="R296" t="s">
         <v>1829</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19949,7 +19923,7 @@
       <c r="J297" t="s">
         <v>1635</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19990,7 +19964,7 @@
       <c r="J298" t="s">
         <v>1635</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20031,7 +20005,7 @@
       <c r="J299" t="s">
         <v>1636</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20072,7 +20046,7 @@
       <c r="J300" t="s">
         <v>1635</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20113,7 +20087,7 @@
       <c r="J301" t="s">
         <v>1635</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20951,7 +20925,7 @@
       <c r="R321" t="s">
         <v>1815</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21174,7 +21148,7 @@
       <c r="R326" t="s">
         <v>1854</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -22009,7 +21983,7 @@
       <c r="R346" t="s">
         <v>1855</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (16/10/2026 12:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5753,8 +5753,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5770,7 +5778,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5778,12 +5786,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6083,73 +6109,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6184,7 +6210,7 @@
       <c r="J2" t="s">
         <v>1635</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6228,7 +6254,7 @@
       <c r="J3" t="s">
         <v>1635</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6272,7 +6298,7 @@
       <c r="J4" t="s">
         <v>1635</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6290,7 +6316,7 @@
       <c r="R4" t="s">
         <v>1812</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6328,7 +6354,7 @@
       <c r="J5" t="s">
         <v>1636</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6378,7 +6404,7 @@
       <c r="J6" t="s">
         <v>1635</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6425,7 +6451,7 @@
       <c r="J7" t="s">
         <v>1635</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6472,7 +6498,7 @@
       <c r="J8" t="s">
         <v>1635</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6519,7 +6545,7 @@
       <c r="J9" t="s">
         <v>1635</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6566,7 +6592,7 @@
       <c r="J10" t="s">
         <v>1635</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6613,7 +6639,7 @@
       <c r="J11" t="s">
         <v>1635</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6660,7 +6686,7 @@
       <c r="J12" t="s">
         <v>1635</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6704,7 +6730,7 @@
       <c r="J13" t="s">
         <v>1635</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6722,7 +6748,7 @@
       <c r="R13" t="s">
         <v>1813</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6760,7 +6786,7 @@
       <c r="J14" t="s">
         <v>1635</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6778,7 +6804,7 @@
       <c r="R14" t="s">
         <v>1814</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6819,7 +6845,7 @@
       <c r="J15" t="s">
         <v>1635</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6837,7 +6863,7 @@
       <c r="R15" t="s">
         <v>1814</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6878,7 +6904,7 @@
       <c r="J16" t="s">
         <v>1635</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6922,7 +6948,7 @@
       <c r="J17" t="s">
         <v>1635</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6966,7 +6992,7 @@
       <c r="J18" t="s">
         <v>1635</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6984,7 +7010,7 @@
       <c r="R18" t="s">
         <v>1815</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7025,7 +7051,7 @@
       <c r="J19" t="s">
         <v>1635</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7069,7 +7095,7 @@
       <c r="J20" t="s">
         <v>1635</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7113,7 +7139,7 @@
       <c r="J21" t="s">
         <v>1635</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7131,7 +7157,7 @@
       <c r="R21" t="s">
         <v>1814</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7172,7 +7198,7 @@
       <c r="J22" t="s">
         <v>1635</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7190,7 +7216,7 @@
       <c r="R22" t="s">
         <v>1816</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7231,7 +7257,7 @@
       <c r="J23" t="s">
         <v>1635</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7249,7 +7275,7 @@
       <c r="R23" t="s">
         <v>1817</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7290,7 +7316,7 @@
       <c r="J24" t="s">
         <v>1635</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7334,7 +7360,7 @@
       <c r="J25" t="s">
         <v>1635</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7375,7 +7401,7 @@
       <c r="J26" t="s">
         <v>1637</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7393,7 +7419,7 @@
       <c r="R26" t="s">
         <v>1818</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7431,7 +7457,7 @@
       <c r="J27" t="s">
         <v>1635</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7449,7 +7475,7 @@
       <c r="R27" t="s">
         <v>1819</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7490,7 +7516,7 @@
       <c r="J28" t="s">
         <v>1635</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7534,7 +7560,7 @@
       <c r="J29" t="s">
         <v>1635</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7578,7 +7604,7 @@
       <c r="J30" t="s">
         <v>1635</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7622,7 +7648,7 @@
       <c r="J31" t="s">
         <v>1635</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7640,7 +7666,7 @@
       <c r="R31" t="s">
         <v>1820</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7681,7 +7707,7 @@
       <c r="J32" t="s">
         <v>1635</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7725,7 +7751,7 @@
       <c r="J33" t="s">
         <v>1635</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7743,7 +7769,7 @@
       <c r="R33" t="s">
         <v>1821</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7784,7 +7810,7 @@
       <c r="J34" t="s">
         <v>1635</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7828,7 +7854,7 @@
       <c r="J35" t="s">
         <v>1635</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7846,7 +7872,7 @@
       <c r="R35" t="s">
         <v>1822</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7887,7 +7913,7 @@
       <c r="J36" t="s">
         <v>1635</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7905,7 +7931,7 @@
       <c r="R36" t="s">
         <v>1822</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7946,7 +7972,7 @@
       <c r="J37" t="s">
         <v>1635</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7964,7 +7990,7 @@
       <c r="R37" t="s">
         <v>1822</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8005,7 +8031,7 @@
       <c r="J38" t="s">
         <v>1635</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8023,7 +8049,7 @@
       <c r="R38" t="s">
         <v>1822</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8064,7 +8090,7 @@
       <c r="J39" t="s">
         <v>1635</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8082,7 +8108,7 @@
       <c r="R39" t="s">
         <v>1822</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8123,7 +8149,7 @@
       <c r="J40" t="s">
         <v>1635</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8141,7 +8167,7 @@
       <c r="R40" t="s">
         <v>1823</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8182,7 +8208,7 @@
       <c r="J41" t="s">
         <v>1635</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8200,7 +8226,7 @@
       <c r="R41" t="s">
         <v>1814</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8241,7 +8267,7 @@
       <c r="J42" t="s">
         <v>1635</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8259,7 +8285,7 @@
       <c r="R42" t="s">
         <v>1822</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8300,7 +8326,7 @@
       <c r="J43" t="s">
         <v>1635</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8344,7 +8370,7 @@
       <c r="J44" t="s">
         <v>1635</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8362,7 +8388,7 @@
       <c r="R44" t="s">
         <v>1824</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8403,7 +8429,7 @@
       <c r="J45" t="s">
         <v>1635</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8421,7 +8447,7 @@
       <c r="R45" t="s">
         <v>1825</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8459,7 +8485,7 @@
       <c r="J46" t="s">
         <v>1635</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8503,7 +8529,7 @@
       <c r="J47" t="s">
         <v>1635</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8521,7 +8547,7 @@
       <c r="R47" t="s">
         <v>1826</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8562,7 +8588,7 @@
       <c r="J48" t="s">
         <v>1635</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8606,7 +8632,7 @@
       <c r="J49" t="s">
         <v>1635</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8650,7 +8676,7 @@
       <c r="J50" t="s">
         <v>1635</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8694,7 +8720,7 @@
       <c r="J51" t="s">
         <v>1635</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8741,7 +8767,7 @@
       <c r="J52" t="s">
         <v>1635</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8785,7 +8811,7 @@
       <c r="J53" t="s">
         <v>1635</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8829,7 +8855,7 @@
       <c r="J54" t="s">
         <v>1635</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8873,7 +8899,7 @@
       <c r="J55" t="s">
         <v>1635</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8923,7 +8949,7 @@
       <c r="J56" t="s">
         <v>1635</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8976,7 +9002,7 @@
       <c r="J57" t="s">
         <v>1635</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9026,7 +9052,7 @@
       <c r="J58" t="s">
         <v>1635</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9076,7 +9102,7 @@
       <c r="J59" t="s">
         <v>1635</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9094,7 +9120,7 @@
       <c r="R59" t="s">
         <v>1827</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9135,7 +9161,7 @@
       <c r="J60" t="s">
         <v>1635</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9179,7 +9205,7 @@
       <c r="J61" t="s">
         <v>1635</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9223,7 +9249,7 @@
       <c r="J62" t="s">
         <v>1635</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9267,7 +9293,7 @@
       <c r="J63" t="s">
         <v>1635</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9311,7 +9337,7 @@
       <c r="J64" t="s">
         <v>1635</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9355,7 +9381,7 @@
       <c r="J65" t="s">
         <v>1635</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9402,7 +9428,7 @@
       <c r="J66" t="s">
         <v>1635</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9420,7 +9446,7 @@
       <c r="R66" t="s">
         <v>1828</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9458,7 +9484,7 @@
       <c r="J67" t="s">
         <v>1635</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9502,7 +9528,7 @@
       <c r="J68" t="s">
         <v>1635</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9517,7 +9543,7 @@
       <c r="O68" t="s">
         <v>1732</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9561,7 +9587,7 @@
       <c r="J69" t="s">
         <v>1637</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9605,7 +9631,7 @@
       <c r="J70" t="s">
         <v>1635</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9649,7 +9675,7 @@
       <c r="J71" t="s">
         <v>1635</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9693,7 +9719,7 @@
       <c r="J72" t="s">
         <v>1635</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9737,7 +9763,7 @@
       <c r="J73" t="s">
         <v>1635</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9781,7 +9807,7 @@
       <c r="J74" t="s">
         <v>1635</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9825,7 +9851,7 @@
       <c r="J75" t="s">
         <v>1635</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9869,7 +9895,7 @@
       <c r="J76" t="s">
         <v>1635</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9887,7 +9913,7 @@
       <c r="R76" t="s">
         <v>1829</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9925,7 +9951,7 @@
       <c r="J77" t="s">
         <v>1635</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9943,7 +9969,7 @@
       <c r="R77" t="s">
         <v>1829</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9981,7 +10007,7 @@
       <c r="J78" t="s">
         <v>1635</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9999,7 +10025,7 @@
       <c r="R78" t="s">
         <v>1829</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10037,7 +10063,7 @@
       <c r="J79" t="s">
         <v>1635</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10055,7 +10081,7 @@
       <c r="R79" t="s">
         <v>1829</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10093,7 +10119,7 @@
       <c r="J80" t="s">
         <v>1635</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10137,7 +10163,7 @@
       <c r="J81" t="s">
         <v>1635</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10181,7 +10207,7 @@
       <c r="J82" t="s">
         <v>1635</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10225,7 +10251,7 @@
       <c r="J83" t="s">
         <v>1635</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10269,7 +10295,7 @@
       <c r="J84" t="s">
         <v>1635</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10313,7 +10339,7 @@
       <c r="J85" t="s">
         <v>1635</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10331,7 +10357,7 @@
       <c r="R85" t="s">
         <v>1830</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10369,7 +10395,7 @@
       <c r="J86" t="s">
         <v>1635</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10413,7 +10439,7 @@
       <c r="J87" t="s">
         <v>1635</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10431,7 +10457,7 @@
       <c r="R87" t="s">
         <v>1831</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10469,7 +10495,7 @@
       <c r="J88" t="s">
         <v>1635</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10513,7 +10539,7 @@
       <c r="J89" t="s">
         <v>1635</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10531,7 +10557,7 @@
       <c r="R89" t="s">
         <v>1832</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10566,7 +10592,7 @@
       <c r="J90" t="s">
         <v>1635</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10584,7 +10610,7 @@
       <c r="R90" t="s">
         <v>1833</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10619,7 +10645,7 @@
       <c r="J91" t="s">
         <v>1635</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10637,7 +10663,7 @@
       <c r="R91" t="s">
         <v>1817</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10675,7 +10701,7 @@
       <c r="J92" t="s">
         <v>1635</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10696,7 +10722,7 @@
       <c r="R92" t="s">
         <v>1817</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10737,7 +10763,7 @@
       <c r="J93" t="s">
         <v>1635</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10778,7 +10804,7 @@
       <c r="J94" t="s">
         <v>1635</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10822,7 +10848,7 @@
       <c r="J95" t="s">
         <v>1635</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10866,7 +10892,7 @@
       <c r="J96" t="s">
         <v>1635</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10884,7 +10910,7 @@
       <c r="R96" t="s">
         <v>1834</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10925,7 +10951,7 @@
       <c r="J97" t="s">
         <v>1635</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10940,7 +10966,7 @@
       <c r="R97" t="s">
         <v>1834</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10981,7 +11007,7 @@
       <c r="J98" t="s">
         <v>1635</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10999,7 +11025,7 @@
       <c r="R98" t="s">
         <v>1835</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11037,7 +11063,7 @@
       <c r="J99" t="s">
         <v>1635</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11055,7 +11081,7 @@
       <c r="R99" t="s">
         <v>1836</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11093,7 +11119,7 @@
       <c r="J100" t="s">
         <v>1635</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11134,7 +11160,7 @@
       <c r="J101" t="s">
         <v>1635</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11175,7 +11201,7 @@
       <c r="J102" t="s">
         <v>1635</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11216,7 +11242,7 @@
       <c r="J103" t="s">
         <v>1635</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11257,7 +11283,7 @@
       <c r="J104" t="s">
         <v>1635</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11298,7 +11324,7 @@
       <c r="J105" t="s">
         <v>1635</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11339,7 +11365,7 @@
       <c r="J106" t="s">
         <v>1635</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11380,7 +11406,7 @@
       <c r="J107" t="s">
         <v>1635</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11421,7 +11447,7 @@
       <c r="J108" t="s">
         <v>1635</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11462,7 +11488,7 @@
       <c r="J109" t="s">
         <v>1635</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11515,7 +11541,7 @@
       <c r="J110" t="s">
         <v>1635</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11571,7 +11597,7 @@
       <c r="J111" t="s">
         <v>1635</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11589,7 +11615,7 @@
       <c r="R111" t="s">
         <v>1838</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11627,7 +11653,7 @@
       <c r="J112" t="s">
         <v>1635</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11686,7 +11712,7 @@
       <c r="J113" t="s">
         <v>1635</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11730,7 +11756,7 @@
       <c r="J114" t="s">
         <v>1635</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11774,7 +11800,7 @@
       <c r="J115" t="s">
         <v>1635</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11792,7 +11818,7 @@
       <c r="R115" t="s">
         <v>1840</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11833,7 +11859,7 @@
       <c r="J116" t="s">
         <v>1635</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11892,7 +11918,7 @@
       <c r="J117" t="s">
         <v>1635</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11936,7 +11962,7 @@
       <c r="J118" t="s">
         <v>1635</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11983,7 +12009,7 @@
       <c r="J119" t="s">
         <v>1635</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12024,7 +12050,7 @@
       <c r="J120" t="s">
         <v>1635</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12068,7 +12094,7 @@
       <c r="J121" t="s">
         <v>1635</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12115,7 +12141,7 @@
       <c r="J122" t="s">
         <v>1635</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12165,7 +12191,7 @@
       <c r="J123" t="s">
         <v>1635</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12209,7 +12235,7 @@
       <c r="J124" t="s">
         <v>1635</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12253,7 +12279,7 @@
       <c r="J125" t="s">
         <v>1635</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12271,7 +12297,7 @@
       <c r="R125" t="s">
         <v>1842</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12306,7 +12332,7 @@
       <c r="J126" t="s">
         <v>1635</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12324,7 +12350,7 @@
       <c r="R126" t="s">
         <v>1843</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12362,7 +12388,7 @@
       <c r="J127" t="s">
         <v>1635</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12418,7 +12444,7 @@
       <c r="J128" t="s">
         <v>1635</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12459,7 +12485,7 @@
       <c r="J129" t="s">
         <v>1635</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12500,7 +12526,7 @@
       <c r="J130" t="s">
         <v>1635</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12541,7 +12567,7 @@
       <c r="J131" t="s">
         <v>1635</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12585,7 +12611,7 @@
       <c r="J132" t="s">
         <v>1635</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12626,7 +12652,7 @@
       <c r="J133" t="s">
         <v>1635</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12644,7 +12670,7 @@
       <c r="R133" t="s">
         <v>1829</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12682,7 +12708,7 @@
       <c r="J134" t="s">
         <v>1635</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12700,7 +12726,7 @@
       <c r="R134" t="s">
         <v>1829</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12735,7 +12761,7 @@
       <c r="J135" t="s">
         <v>1635</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12776,7 +12802,7 @@
       <c r="J136" t="s">
         <v>1635</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12817,7 +12843,7 @@
       <c r="J137" t="s">
         <v>1635</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12858,7 +12884,7 @@
       <c r="J138" t="s">
         <v>1635</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12899,7 +12925,7 @@
       <c r="J139" t="s">
         <v>1635</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12946,7 +12972,7 @@
       <c r="J140" t="s">
         <v>1635</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12987,7 +13013,7 @@
       <c r="J141" t="s">
         <v>1635</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13028,7 +13054,7 @@
       <c r="J142" t="s">
         <v>1635</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13072,7 +13098,7 @@
       <c r="J143" t="s">
         <v>1635</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13090,7 +13116,7 @@
       <c r="R143" t="s">
         <v>1829</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13125,7 +13151,7 @@
       <c r="J144" t="s">
         <v>1635</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13143,7 +13169,7 @@
       <c r="R144" t="s">
         <v>1829</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13181,7 +13207,7 @@
       <c r="J145" t="s">
         <v>1635</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13199,7 +13225,7 @@
       <c r="R145" t="s">
         <v>1829</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13234,7 +13260,7 @@
       <c r="J146" t="s">
         <v>1635</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13252,7 +13278,7 @@
       <c r="R146" t="s">
         <v>1837</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13287,7 +13313,7 @@
       <c r="J147" t="s">
         <v>1635</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13305,7 +13331,7 @@
       <c r="R147" t="s">
         <v>1844</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13340,7 +13366,7 @@
       <c r="J148" t="s">
         <v>1635</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13381,7 +13407,7 @@
       <c r="J149" t="s">
         <v>1635</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13399,7 +13425,7 @@
       <c r="R149" t="s">
         <v>1829</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13434,7 +13460,7 @@
       <c r="J150" t="s">
         <v>1635</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13452,7 +13478,7 @@
       <c r="R150" t="s">
         <v>1829</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13490,7 +13516,7 @@
       <c r="J151" t="s">
         <v>1635</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13508,7 +13534,7 @@
       <c r="R151" t="s">
         <v>1845</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13543,7 +13569,7 @@
       <c r="J152" t="s">
         <v>1635</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13561,7 +13587,7 @@
       <c r="R152" t="s">
         <v>1846</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13596,7 +13622,7 @@
       <c r="J153" t="s">
         <v>1635</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13605,7 +13631,7 @@
       <c r="M153" t="s">
         <v>1723</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13646,7 +13672,7 @@
       <c r="J154" t="s">
         <v>1635</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13687,7 +13713,7 @@
       <c r="J155" t="s">
         <v>1635</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13728,7 +13754,7 @@
       <c r="J156" t="s">
         <v>1635</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13769,7 +13795,7 @@
       <c r="J157" t="s">
         <v>1635</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13810,7 +13836,7 @@
       <c r="J158" t="s">
         <v>1635</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13851,7 +13877,7 @@
       <c r="J159" t="s">
         <v>1635</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13892,7 +13918,7 @@
       <c r="J160" t="s">
         <v>1635</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13933,7 +13959,7 @@
       <c r="J161" t="s">
         <v>1635</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13974,7 +14000,7 @@
       <c r="J162" t="s">
         <v>1635</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13992,7 +14018,7 @@
       <c r="R162" t="s">
         <v>1832</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14027,7 +14053,7 @@
       <c r="J163" t="s">
         <v>1635</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14045,7 +14071,7 @@
       <c r="R163" t="s">
         <v>1829</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14080,7 +14106,7 @@
       <c r="J164" t="s">
         <v>1635</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14124,7 +14150,7 @@
       <c r="J165" t="s">
         <v>1635</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14165,7 +14191,7 @@
       <c r="J166" t="s">
         <v>1635</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14183,7 +14209,7 @@
       <c r="R166" t="s">
         <v>1847</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14218,7 +14244,7 @@
       <c r="J167" t="s">
         <v>1635</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14262,7 +14288,7 @@
       <c r="J168" t="s">
         <v>1635</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14306,7 +14332,7 @@
       <c r="J169" t="s">
         <v>1635</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14347,7 +14373,7 @@
       <c r="J170" t="s">
         <v>1635</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14388,7 +14414,7 @@
       <c r="J171" t="s">
         <v>1635</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14429,7 +14455,7 @@
       <c r="J172" t="s">
         <v>1635</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14470,7 +14496,7 @@
       <c r="J173" t="s">
         <v>1635</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14511,7 +14537,7 @@
       <c r="J174" t="s">
         <v>1635</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14552,7 +14578,7 @@
       <c r="J175" t="s">
         <v>1635</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14593,7 +14619,7 @@
       <c r="J176" t="s">
         <v>1635</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14634,7 +14660,7 @@
       <c r="J177" t="s">
         <v>1635</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14675,7 +14701,7 @@
       <c r="J178" t="s">
         <v>1635</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14693,7 +14719,7 @@
       <c r="R178" t="s">
         <v>1845</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14731,7 +14757,7 @@
       <c r="J179" t="s">
         <v>1635</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14740,7 +14766,7 @@
       <c r="M179" t="s">
         <v>1720</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14781,7 +14807,7 @@
       <c r="J180" t="s">
         <v>1635</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14822,7 +14848,7 @@
       <c r="J181" t="s">
         <v>1635</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14840,7 +14866,7 @@
       <c r="R181" t="s">
         <v>1829</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14875,7 +14901,7 @@
       <c r="J182" t="s">
         <v>1635</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14916,7 +14942,7 @@
       <c r="J183" t="s">
         <v>1635</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14957,7 +14983,7 @@
       <c r="J184" t="s">
         <v>1635</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14998,7 +15024,7 @@
       <c r="J185" t="s">
         <v>1635</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15039,7 +15065,7 @@
       <c r="J186" t="s">
         <v>1635</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15080,7 +15106,7 @@
       <c r="J187" t="s">
         <v>1635</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15121,7 +15147,7 @@
       <c r="J188" t="s">
         <v>1635</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15162,7 +15188,7 @@
       <c r="J189" t="s">
         <v>1635</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15203,7 +15229,7 @@
       <c r="J190" t="s">
         <v>1635</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15244,7 +15270,7 @@
       <c r="J191" t="s">
         <v>1635</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15285,7 +15311,7 @@
       <c r="J192" t="s">
         <v>1635</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15326,7 +15352,7 @@
       <c r="J193" t="s">
         <v>1635</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15367,7 +15393,7 @@
       <c r="J194" t="s">
         <v>1635</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15408,7 +15434,7 @@
       <c r="J195" t="s">
         <v>1635</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15426,7 +15452,7 @@
       <c r="R195" t="s">
         <v>1838</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15467,7 +15493,7 @@
       <c r="J196" t="s">
         <v>1635</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15485,7 +15511,7 @@
       <c r="R196" t="s">
         <v>1844</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15523,7 +15549,7 @@
       <c r="J197" t="s">
         <v>1635</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15564,7 +15590,7 @@
       <c r="J198" t="s">
         <v>1637</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15605,7 +15631,7 @@
       <c r="J199" t="s">
         <v>1636</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15646,7 +15672,7 @@
       <c r="J200" t="s">
         <v>1635</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15687,7 +15713,7 @@
       <c r="J201" t="s">
         <v>1635</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15728,7 +15754,7 @@
       <c r="J202" t="s">
         <v>1635</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15746,7 +15772,7 @@
       <c r="R202" t="s">
         <v>1829</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15784,7 +15810,7 @@
       <c r="J203" t="s">
         <v>1635</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15802,7 +15828,7 @@
       <c r="R203" t="s">
         <v>1837</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15837,7 +15863,7 @@
       <c r="J204" t="s">
         <v>1635</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15852,7 +15878,7 @@
       <c r="R204" t="s">
         <v>1848</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15890,7 +15916,7 @@
       <c r="J205" t="s">
         <v>1635</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15908,7 +15934,7 @@
       <c r="R205" t="s">
         <v>1849</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15946,7 +15972,7 @@
       <c r="J206" t="s">
         <v>1635</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15964,7 +15990,7 @@
       <c r="R206" t="s">
         <v>1817</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15999,7 +16025,7 @@
       <c r="J207" t="s">
         <v>1635</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16040,7 +16066,7 @@
       <c r="J208" t="s">
         <v>1635</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16081,7 +16107,7 @@
       <c r="J209" t="s">
         <v>1635</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16122,7 +16148,7 @@
       <c r="J210" t="s">
         <v>1635</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16163,7 +16189,7 @@
       <c r="J211" t="s">
         <v>1635</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16204,7 +16230,7 @@
       <c r="J212" t="s">
         <v>1635</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16245,7 +16271,7 @@
       <c r="J213" t="s">
         <v>1635</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16286,7 +16312,7 @@
       <c r="J214" t="s">
         <v>1635</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16304,7 +16330,7 @@
       <c r="R214" t="s">
         <v>1850</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16342,7 +16368,7 @@
       <c r="J215" t="s">
         <v>1635</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16383,7 +16409,7 @@
       <c r="J216" t="s">
         <v>1635</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16424,7 +16450,7 @@
       <c r="J217" t="s">
         <v>1635</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16465,7 +16491,7 @@
       <c r="J218" t="s">
         <v>1635</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16506,7 +16532,7 @@
       <c r="J219" t="s">
         <v>1635</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16547,7 +16573,7 @@
       <c r="J220" t="s">
         <v>1635</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16588,7 +16614,7 @@
       <c r="J221" t="s">
         <v>1635</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16629,7 +16655,7 @@
       <c r="J222" t="s">
         <v>1635</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16670,7 +16696,7 @@
       <c r="J223" t="s">
         <v>1635</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16711,7 +16737,7 @@
       <c r="J224" t="s">
         <v>1635</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16752,7 +16778,7 @@
       <c r="J225" t="s">
         <v>1635</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16793,7 +16819,7 @@
       <c r="J226" t="s">
         <v>1635</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16834,7 +16860,7 @@
       <c r="J227" t="s">
         <v>1635</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16875,7 +16901,7 @@
       <c r="J228" t="s">
         <v>1635</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16916,7 +16942,7 @@
       <c r="J229" t="s">
         <v>1635</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16957,7 +16983,7 @@
       <c r="J230" t="s">
         <v>1635</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16998,7 +17024,7 @@
       <c r="J231" t="s">
         <v>1635</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17039,7 +17065,7 @@
       <c r="J232" t="s">
         <v>1635</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17080,7 +17106,7 @@
       <c r="J233" t="s">
         <v>1635</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17121,7 +17147,7 @@
       <c r="J234" t="s">
         <v>1635</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17162,7 +17188,7 @@
       <c r="J235" t="s">
         <v>1635</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17203,7 +17229,7 @@
       <c r="J236" t="s">
         <v>1635</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17244,7 +17270,7 @@
       <c r="J237" t="s">
         <v>1635</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17285,7 +17311,7 @@
       <c r="J238" t="s">
         <v>1635</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17326,7 +17352,7 @@
       <c r="J239" t="s">
         <v>1635</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17344,7 +17370,7 @@
       <c r="R239" t="s">
         <v>1844</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17382,7 +17408,7 @@
       <c r="J240" t="s">
         <v>1635</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17423,7 +17449,7 @@
       <c r="J241" t="s">
         <v>1635</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17464,7 +17490,7 @@
       <c r="J242" t="s">
         <v>1635</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17482,7 +17508,7 @@
       <c r="R242" t="s">
         <v>1837</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17517,7 +17543,7 @@
       <c r="J243" t="s">
         <v>1635</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17558,7 +17584,7 @@
       <c r="J244" t="s">
         <v>1635</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17599,7 +17625,7 @@
       <c r="J245" t="s">
         <v>1635</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17640,7 +17666,7 @@
       <c r="J246" t="s">
         <v>1635</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17658,7 +17684,7 @@
       <c r="R246" t="s">
         <v>1817</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17696,7 +17722,7 @@
       <c r="J247" t="s">
         <v>1635</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17737,7 +17763,7 @@
       <c r="J248" t="s">
         <v>1635</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17778,7 +17804,7 @@
       <c r="J249" t="s">
         <v>1635</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17819,7 +17845,7 @@
       <c r="J250" t="s">
         <v>1635</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17860,7 +17886,7 @@
       <c r="J251" t="s">
         <v>1635</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17901,7 +17927,7 @@
       <c r="J252" t="s">
         <v>1635</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17942,7 +17968,7 @@
       <c r="J253" t="s">
         <v>1635</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17960,7 +17986,7 @@
       <c r="R253" t="s">
         <v>1847</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18001,7 +18027,7 @@
       <c r="J254" t="s">
         <v>1635</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18042,7 +18068,7 @@
       <c r="J255" t="s">
         <v>1635</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18083,7 +18109,7 @@
       <c r="J256" t="s">
         <v>1635</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18092,7 +18118,7 @@
       <c r="M256" t="s">
         <v>1719</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18130,7 +18156,7 @@
       <c r="J257" t="s">
         <v>1635</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18139,7 +18165,7 @@
       <c r="M257" t="s">
         <v>1720</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18183,7 +18209,7 @@
       <c r="J258" t="s">
         <v>1635</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18201,7 +18227,7 @@
       <c r="R258" t="s">
         <v>1829</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18239,7 +18265,7 @@
       <c r="J259" t="s">
         <v>1635</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18257,7 +18283,7 @@
       <c r="R259" t="s">
         <v>1845</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18295,7 +18321,7 @@
       <c r="J260" t="s">
         <v>1635</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18304,7 +18330,7 @@
       <c r="M260" t="s">
         <v>1714</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18348,7 +18374,7 @@
       <c r="J261" t="s">
         <v>1635</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18366,7 +18392,7 @@
       <c r="R261" t="s">
         <v>1851</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18404,7 +18430,7 @@
       <c r="J262" t="s">
         <v>1635</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18422,7 +18448,7 @@
       <c r="R262" t="s">
         <v>1845</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18460,7 +18486,7 @@
       <c r="J263" t="s">
         <v>1635</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18469,7 +18495,7 @@
       <c r="M263" t="s">
         <v>1714</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18513,7 +18539,7 @@
       <c r="J264" t="s">
         <v>1635</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18554,7 +18580,7 @@
       <c r="J265" t="s">
         <v>1635</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18595,7 +18621,7 @@
       <c r="J266" t="s">
         <v>1635</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18636,7 +18662,7 @@
       <c r="J267" t="s">
         <v>1635</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18680,7 +18706,7 @@
       <c r="J268" t="s">
         <v>1635</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18721,7 +18747,7 @@
       <c r="J269" t="s">
         <v>1635</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18762,7 +18788,7 @@
       <c r="J270" t="s">
         <v>1635</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18803,7 +18829,7 @@
       <c r="J271" t="s">
         <v>1635</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18844,7 +18870,7 @@
       <c r="J272" t="s">
         <v>1635</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18862,7 +18888,7 @@
       <c r="R272" t="s">
         <v>1852</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18903,7 +18929,7 @@
       <c r="J273" t="s">
         <v>1635</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18947,7 +18973,7 @@
       <c r="J274" t="s">
         <v>1635</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18988,7 +19014,7 @@
       <c r="J275" t="s">
         <v>1635</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19029,7 +19055,7 @@
       <c r="J276" t="s">
         <v>1635</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19070,7 +19096,7 @@
       <c r="J277" t="s">
         <v>1635</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19111,7 +19137,7 @@
       <c r="J278" t="s">
         <v>1635</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19152,7 +19178,7 @@
       <c r="J279" t="s">
         <v>1635</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19193,7 +19219,7 @@
       <c r="J280" t="s">
         <v>1635</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19234,7 +19260,7 @@
       <c r="J281" t="s">
         <v>1635</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19275,7 +19301,7 @@
       <c r="J282" t="s">
         <v>1635</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19316,7 +19342,7 @@
       <c r="J283" t="s">
         <v>1635</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19357,7 +19383,7 @@
       <c r="J284" t="s">
         <v>1635</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19398,7 +19424,7 @@
       <c r="J285" t="s">
         <v>1635</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19439,7 +19465,7 @@
       <c r="J286" t="s">
         <v>1635</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19480,7 +19506,7 @@
       <c r="J287" t="s">
         <v>1635</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19521,7 +19547,7 @@
       <c r="J288" t="s">
         <v>1635</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19562,7 +19588,7 @@
       <c r="J289" t="s">
         <v>1635</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19603,7 +19629,7 @@
       <c r="J290" t="s">
         <v>1635</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19644,7 +19670,7 @@
       <c r="J291" t="s">
         <v>1635</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19685,7 +19711,7 @@
       <c r="J292" t="s">
         <v>1635</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19726,7 +19752,7 @@
       <c r="J293" t="s">
         <v>1635</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19767,7 +19793,7 @@
       <c r="J294" t="s">
         <v>1635</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19808,7 +19834,7 @@
       <c r="J295" t="s">
         <v>1635</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19826,7 +19852,7 @@
       <c r="R295" t="s">
         <v>1853</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19867,7 +19893,7 @@
       <c r="J296" t="s">
         <v>1635</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19885,7 +19911,7 @@
       <c r="R296" t="s">
         <v>1829</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19923,7 +19949,7 @@
       <c r="J297" t="s">
         <v>1635</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19964,7 +19990,7 @@
       <c r="J298" t="s">
         <v>1635</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20005,7 +20031,7 @@
       <c r="J299" t="s">
         <v>1636</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20046,7 +20072,7 @@
       <c r="J300" t="s">
         <v>1635</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20087,7 +20113,7 @@
       <c r="J301" t="s">
         <v>1635</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20925,7 +20951,7 @@
       <c r="R321" t="s">
         <v>1815</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21148,7 +21174,7 @@
       <c r="R326" t="s">
         <v>1854</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21983,7 +22009,7 @@
       <c r="R346" t="s">
         <v>1855</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (16/10/2026 12:22)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5753,16 +5753,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5778,7 +5770,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5786,30 +5778,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6109,73 +6083,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6210,7 +6184,7 @@
       <c r="J2" t="s">
         <v>1635</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6254,7 +6228,7 @@
       <c r="J3" t="s">
         <v>1635</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6298,7 +6272,7 @@
       <c r="J4" t="s">
         <v>1635</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6316,7 +6290,7 @@
       <c r="R4" t="s">
         <v>1812</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6354,7 +6328,7 @@
       <c r="J5" t="s">
         <v>1636</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6404,7 +6378,7 @@
       <c r="J6" t="s">
         <v>1635</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6451,7 +6425,7 @@
       <c r="J7" t="s">
         <v>1635</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6498,7 +6472,7 @@
       <c r="J8" t="s">
         <v>1635</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6545,7 +6519,7 @@
       <c r="J9" t="s">
         <v>1635</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6592,7 +6566,7 @@
       <c r="J10" t="s">
         <v>1635</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6639,7 +6613,7 @@
       <c r="J11" t="s">
         <v>1635</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6686,7 +6660,7 @@
       <c r="J12" t="s">
         <v>1635</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6730,7 +6704,7 @@
       <c r="J13" t="s">
         <v>1635</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6748,7 +6722,7 @@
       <c r="R13" t="s">
         <v>1813</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6786,7 +6760,7 @@
       <c r="J14" t="s">
         <v>1635</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6804,7 +6778,7 @@
       <c r="R14" t="s">
         <v>1814</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6845,7 +6819,7 @@
       <c r="J15" t="s">
         <v>1635</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6863,7 +6837,7 @@
       <c r="R15" t="s">
         <v>1814</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6904,7 +6878,7 @@
       <c r="J16" t="s">
         <v>1635</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6948,7 +6922,7 @@
       <c r="J17" t="s">
         <v>1635</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6992,7 +6966,7 @@
       <c r="J18" t="s">
         <v>1635</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -7010,7 +6984,7 @@
       <c r="R18" t="s">
         <v>1815</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7051,7 +7025,7 @@
       <c r="J19" t="s">
         <v>1635</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7095,7 +7069,7 @@
       <c r="J20" t="s">
         <v>1635</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7139,7 +7113,7 @@
       <c r="J21" t="s">
         <v>1635</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7157,7 +7131,7 @@
       <c r="R21" t="s">
         <v>1814</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7198,7 +7172,7 @@
       <c r="J22" t="s">
         <v>1635</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7216,7 +7190,7 @@
       <c r="R22" t="s">
         <v>1816</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7257,7 +7231,7 @@
       <c r="J23" t="s">
         <v>1635</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7275,7 +7249,7 @@
       <c r="R23" t="s">
         <v>1817</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7316,7 +7290,7 @@
       <c r="J24" t="s">
         <v>1635</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7360,7 +7334,7 @@
       <c r="J25" t="s">
         <v>1635</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7401,7 +7375,7 @@
       <c r="J26" t="s">
         <v>1637</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7419,7 +7393,7 @@
       <c r="R26" t="s">
         <v>1818</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7457,7 +7431,7 @@
       <c r="J27" t="s">
         <v>1635</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7475,7 +7449,7 @@
       <c r="R27" t="s">
         <v>1819</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7516,7 +7490,7 @@
       <c r="J28" t="s">
         <v>1635</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7560,7 +7534,7 @@
       <c r="J29" t="s">
         <v>1635</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7604,7 +7578,7 @@
       <c r="J30" t="s">
         <v>1635</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7648,7 +7622,7 @@
       <c r="J31" t="s">
         <v>1635</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7666,7 +7640,7 @@
       <c r="R31" t="s">
         <v>1820</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7707,7 +7681,7 @@
       <c r="J32" t="s">
         <v>1635</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7751,7 +7725,7 @@
       <c r="J33" t="s">
         <v>1635</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7769,7 +7743,7 @@
       <c r="R33" t="s">
         <v>1821</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7810,7 +7784,7 @@
       <c r="J34" t="s">
         <v>1635</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7854,7 +7828,7 @@
       <c r="J35" t="s">
         <v>1635</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7872,7 +7846,7 @@
       <c r="R35" t="s">
         <v>1822</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7913,7 +7887,7 @@
       <c r="J36" t="s">
         <v>1635</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7931,7 +7905,7 @@
       <c r="R36" t="s">
         <v>1822</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7972,7 +7946,7 @@
       <c r="J37" t="s">
         <v>1635</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7990,7 +7964,7 @@
       <c r="R37" t="s">
         <v>1822</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8031,7 +8005,7 @@
       <c r="J38" t="s">
         <v>1635</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8049,7 +8023,7 @@
       <c r="R38" t="s">
         <v>1822</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8090,7 +8064,7 @@
       <c r="J39" t="s">
         <v>1635</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8108,7 +8082,7 @@
       <c r="R39" t="s">
         <v>1822</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8149,7 +8123,7 @@
       <c r="J40" t="s">
         <v>1635</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8167,7 +8141,7 @@
       <c r="R40" t="s">
         <v>1823</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8208,7 +8182,7 @@
       <c r="J41" t="s">
         <v>1635</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8226,7 +8200,7 @@
       <c r="R41" t="s">
         <v>1814</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8267,7 +8241,7 @@
       <c r="J42" t="s">
         <v>1635</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8285,7 +8259,7 @@
       <c r="R42" t="s">
         <v>1822</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8326,7 +8300,7 @@
       <c r="J43" t="s">
         <v>1635</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8370,7 +8344,7 @@
       <c r="J44" t="s">
         <v>1635</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8388,7 +8362,7 @@
       <c r="R44" t="s">
         <v>1824</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8429,7 +8403,7 @@
       <c r="J45" t="s">
         <v>1635</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8447,7 +8421,7 @@
       <c r="R45" t="s">
         <v>1825</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8485,7 +8459,7 @@
       <c r="J46" t="s">
         <v>1635</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8529,7 +8503,7 @@
       <c r="J47" t="s">
         <v>1635</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8547,7 +8521,7 @@
       <c r="R47" t="s">
         <v>1826</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8588,7 +8562,7 @@
       <c r="J48" t="s">
         <v>1635</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8632,7 +8606,7 @@
       <c r="J49" t="s">
         <v>1635</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8676,7 +8650,7 @@
       <c r="J50" t="s">
         <v>1635</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8720,7 +8694,7 @@
       <c r="J51" t="s">
         <v>1635</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8767,7 +8741,7 @@
       <c r="J52" t="s">
         <v>1635</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8811,7 +8785,7 @@
       <c r="J53" t="s">
         <v>1635</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8855,7 +8829,7 @@
       <c r="J54" t="s">
         <v>1635</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8899,7 +8873,7 @@
       <c r="J55" t="s">
         <v>1635</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8949,7 +8923,7 @@
       <c r="J56" t="s">
         <v>1635</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -9002,7 +8976,7 @@
       <c r="J57" t="s">
         <v>1635</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9052,7 +9026,7 @@
       <c r="J58" t="s">
         <v>1635</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9102,7 +9076,7 @@
       <c r="J59" t="s">
         <v>1635</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9120,7 +9094,7 @@
       <c r="R59" t="s">
         <v>1827</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9161,7 +9135,7 @@
       <c r="J60" t="s">
         <v>1635</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9205,7 +9179,7 @@
       <c r="J61" t="s">
         <v>1635</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9249,7 +9223,7 @@
       <c r="J62" t="s">
         <v>1635</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9293,7 +9267,7 @@
       <c r="J63" t="s">
         <v>1635</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9337,7 +9311,7 @@
       <c r="J64" t="s">
         <v>1635</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9381,7 +9355,7 @@
       <c r="J65" t="s">
         <v>1635</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9428,7 +9402,7 @@
       <c r="J66" t="s">
         <v>1635</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9446,7 +9420,7 @@
       <c r="R66" t="s">
         <v>1828</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9484,7 +9458,7 @@
       <c r="J67" t="s">
         <v>1635</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9528,7 +9502,7 @@
       <c r="J68" t="s">
         <v>1635</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9543,7 +9517,7 @@
       <c r="O68" t="s">
         <v>1732</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9587,7 +9561,7 @@
       <c r="J69" t="s">
         <v>1637</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9631,7 +9605,7 @@
       <c r="J70" t="s">
         <v>1635</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9675,7 +9649,7 @@
       <c r="J71" t="s">
         <v>1635</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9719,7 +9693,7 @@
       <c r="J72" t="s">
         <v>1635</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9763,7 +9737,7 @@
       <c r="J73" t="s">
         <v>1635</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9807,7 +9781,7 @@
       <c r="J74" t="s">
         <v>1635</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9851,7 +9825,7 @@
       <c r="J75" t="s">
         <v>1635</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9895,7 +9869,7 @@
       <c r="J76" t="s">
         <v>1635</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9913,7 +9887,7 @@
       <c r="R76" t="s">
         <v>1829</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9951,7 +9925,7 @@
       <c r="J77" t="s">
         <v>1635</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9969,7 +9943,7 @@
       <c r="R77" t="s">
         <v>1829</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -10007,7 +9981,7 @@
       <c r="J78" t="s">
         <v>1635</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -10025,7 +9999,7 @@
       <c r="R78" t="s">
         <v>1829</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10063,7 +10037,7 @@
       <c r="J79" t="s">
         <v>1635</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10081,7 +10055,7 @@
       <c r="R79" t="s">
         <v>1829</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10119,7 +10093,7 @@
       <c r="J80" t="s">
         <v>1635</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10163,7 +10137,7 @@
       <c r="J81" t="s">
         <v>1635</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10207,7 +10181,7 @@
       <c r="J82" t="s">
         <v>1635</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10251,7 +10225,7 @@
       <c r="J83" t="s">
         <v>1635</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10295,7 +10269,7 @@
       <c r="J84" t="s">
         <v>1635</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10339,7 +10313,7 @@
       <c r="J85" t="s">
         <v>1635</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10357,7 +10331,7 @@
       <c r="R85" t="s">
         <v>1830</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10395,7 +10369,7 @@
       <c r="J86" t="s">
         <v>1635</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10439,7 +10413,7 @@
       <c r="J87" t="s">
         <v>1635</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10457,7 +10431,7 @@
       <c r="R87" t="s">
         <v>1831</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10495,7 +10469,7 @@
       <c r="J88" t="s">
         <v>1635</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10539,7 +10513,7 @@
       <c r="J89" t="s">
         <v>1635</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10557,7 +10531,7 @@
       <c r="R89" t="s">
         <v>1832</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10592,7 +10566,7 @@
       <c r="J90" t="s">
         <v>1635</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10610,7 +10584,7 @@
       <c r="R90" t="s">
         <v>1833</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10645,7 +10619,7 @@
       <c r="J91" t="s">
         <v>1635</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10663,7 +10637,7 @@
       <c r="R91" t="s">
         <v>1817</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10701,7 +10675,7 @@
       <c r="J92" t="s">
         <v>1635</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10722,7 +10696,7 @@
       <c r="R92" t="s">
         <v>1817</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10763,7 +10737,7 @@
       <c r="J93" t="s">
         <v>1635</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10804,7 +10778,7 @@
       <c r="J94" t="s">
         <v>1635</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10848,7 +10822,7 @@
       <c r="J95" t="s">
         <v>1635</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10892,7 +10866,7 @@
       <c r="J96" t="s">
         <v>1635</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10910,7 +10884,7 @@
       <c r="R96" t="s">
         <v>1834</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10951,7 +10925,7 @@
       <c r="J97" t="s">
         <v>1635</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10966,7 +10940,7 @@
       <c r="R97" t="s">
         <v>1834</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -11007,7 +10981,7 @@
       <c r="J98" t="s">
         <v>1635</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -11025,7 +10999,7 @@
       <c r="R98" t="s">
         <v>1835</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11063,7 +11037,7 @@
       <c r="J99" t="s">
         <v>1635</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11081,7 +11055,7 @@
       <c r="R99" t="s">
         <v>1836</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11119,7 +11093,7 @@
       <c r="J100" t="s">
         <v>1635</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11160,7 +11134,7 @@
       <c r="J101" t="s">
         <v>1635</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11201,7 +11175,7 @@
       <c r="J102" t="s">
         <v>1635</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11242,7 +11216,7 @@
       <c r="J103" t="s">
         <v>1635</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11283,7 +11257,7 @@
       <c r="J104" t="s">
         <v>1635</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11324,7 +11298,7 @@
       <c r="J105" t="s">
         <v>1635</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11365,7 +11339,7 @@
       <c r="J106" t="s">
         <v>1635</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11406,7 +11380,7 @@
       <c r="J107" t="s">
         <v>1635</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11447,7 +11421,7 @@
       <c r="J108" t="s">
         <v>1635</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11488,7 +11462,7 @@
       <c r="J109" t="s">
         <v>1635</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11541,7 +11515,7 @@
       <c r="J110" t="s">
         <v>1635</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11597,7 +11571,7 @@
       <c r="J111" t="s">
         <v>1635</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11615,7 +11589,7 @@
       <c r="R111" t="s">
         <v>1838</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11653,7 +11627,7 @@
       <c r="J112" t="s">
         <v>1635</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11712,7 +11686,7 @@
       <c r="J113" t="s">
         <v>1635</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11756,7 +11730,7 @@
       <c r="J114" t="s">
         <v>1635</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11800,7 +11774,7 @@
       <c r="J115" t="s">
         <v>1635</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11818,7 +11792,7 @@
       <c r="R115" t="s">
         <v>1840</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11859,7 +11833,7 @@
       <c r="J116" t="s">
         <v>1635</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11918,7 +11892,7 @@
       <c r="J117" t="s">
         <v>1635</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11962,7 +11936,7 @@
       <c r="J118" t="s">
         <v>1635</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -12009,7 +11983,7 @@
       <c r="J119" t="s">
         <v>1635</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12050,7 +12024,7 @@
       <c r="J120" t="s">
         <v>1635</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12094,7 +12068,7 @@
       <c r="J121" t="s">
         <v>1635</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12141,7 +12115,7 @@
       <c r="J122" t="s">
         <v>1635</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12191,7 +12165,7 @@
       <c r="J123" t="s">
         <v>1635</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12235,7 +12209,7 @@
       <c r="J124" t="s">
         <v>1635</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12279,7 +12253,7 @@
       <c r="J125" t="s">
         <v>1635</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12297,7 +12271,7 @@
       <c r="R125" t="s">
         <v>1842</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12332,7 +12306,7 @@
       <c r="J126" t="s">
         <v>1635</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12350,7 +12324,7 @@
       <c r="R126" t="s">
         <v>1843</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12388,7 +12362,7 @@
       <c r="J127" t="s">
         <v>1635</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12444,7 +12418,7 @@
       <c r="J128" t="s">
         <v>1635</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12485,7 +12459,7 @@
       <c r="J129" t="s">
         <v>1635</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12526,7 +12500,7 @@
       <c r="J130" t="s">
         <v>1635</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12567,7 +12541,7 @@
       <c r="J131" t="s">
         <v>1635</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12611,7 +12585,7 @@
       <c r="J132" t="s">
         <v>1635</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12652,7 +12626,7 @@
       <c r="J133" t="s">
         <v>1635</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12670,7 +12644,7 @@
       <c r="R133" t="s">
         <v>1829</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12708,7 +12682,7 @@
       <c r="J134" t="s">
         <v>1635</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12726,7 +12700,7 @@
       <c r="R134" t="s">
         <v>1829</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12761,7 +12735,7 @@
       <c r="J135" t="s">
         <v>1635</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12802,7 +12776,7 @@
       <c r="J136" t="s">
         <v>1635</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12843,7 +12817,7 @@
       <c r="J137" t="s">
         <v>1635</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12884,7 +12858,7 @@
       <c r="J138" t="s">
         <v>1635</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12925,7 +12899,7 @@
       <c r="J139" t="s">
         <v>1635</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12972,7 +12946,7 @@
       <c r="J140" t="s">
         <v>1635</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -13013,7 +12987,7 @@
       <c r="J141" t="s">
         <v>1635</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13054,7 +13028,7 @@
       <c r="J142" t="s">
         <v>1635</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13098,7 +13072,7 @@
       <c r="J143" t="s">
         <v>1635</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13116,7 +13090,7 @@
       <c r="R143" t="s">
         <v>1829</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13151,7 +13125,7 @@
       <c r="J144" t="s">
         <v>1635</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13169,7 +13143,7 @@
       <c r="R144" t="s">
         <v>1829</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13207,7 +13181,7 @@
       <c r="J145" t="s">
         <v>1635</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13225,7 +13199,7 @@
       <c r="R145" t="s">
         <v>1829</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13260,7 +13234,7 @@
       <c r="J146" t="s">
         <v>1635</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13278,7 +13252,7 @@
       <c r="R146" t="s">
         <v>1837</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13313,7 +13287,7 @@
       <c r="J147" t="s">
         <v>1635</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13331,7 +13305,7 @@
       <c r="R147" t="s">
         <v>1844</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13366,7 +13340,7 @@
       <c r="J148" t="s">
         <v>1635</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13407,7 +13381,7 @@
       <c r="J149" t="s">
         <v>1635</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13425,7 +13399,7 @@
       <c r="R149" t="s">
         <v>1829</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13460,7 +13434,7 @@
       <c r="J150" t="s">
         <v>1635</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13478,7 +13452,7 @@
       <c r="R150" t="s">
         <v>1829</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13516,7 +13490,7 @@
       <c r="J151" t="s">
         <v>1635</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13534,7 +13508,7 @@
       <c r="R151" t="s">
         <v>1845</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13569,7 +13543,7 @@
       <c r="J152" t="s">
         <v>1635</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13587,7 +13561,7 @@
       <c r="R152" t="s">
         <v>1846</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13622,7 +13596,7 @@
       <c r="J153" t="s">
         <v>1635</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13631,7 +13605,7 @@
       <c r="M153" t="s">
         <v>1723</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13672,7 +13646,7 @@
       <c r="J154" t="s">
         <v>1635</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13713,7 +13687,7 @@
       <c r="J155" t="s">
         <v>1635</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13754,7 +13728,7 @@
       <c r="J156" t="s">
         <v>1635</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13795,7 +13769,7 @@
       <c r="J157" t="s">
         <v>1635</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13836,7 +13810,7 @@
       <c r="J158" t="s">
         <v>1635</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13877,7 +13851,7 @@
       <c r="J159" t="s">
         <v>1635</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13918,7 +13892,7 @@
       <c r="J160" t="s">
         <v>1635</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13959,7 +13933,7 @@
       <c r="J161" t="s">
         <v>1635</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -14000,7 +13974,7 @@
       <c r="J162" t="s">
         <v>1635</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -14018,7 +13992,7 @@
       <c r="R162" t="s">
         <v>1832</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14053,7 +14027,7 @@
       <c r="J163" t="s">
         <v>1635</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14071,7 +14045,7 @@
       <c r="R163" t="s">
         <v>1829</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14106,7 +14080,7 @@
       <c r="J164" t="s">
         <v>1635</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14150,7 +14124,7 @@
       <c r="J165" t="s">
         <v>1635</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14191,7 +14165,7 @@
       <c r="J166" t="s">
         <v>1635</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14209,7 +14183,7 @@
       <c r="R166" t="s">
         <v>1847</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14244,7 +14218,7 @@
       <c r="J167" t="s">
         <v>1635</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14288,7 +14262,7 @@
       <c r="J168" t="s">
         <v>1635</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14332,7 +14306,7 @@
       <c r="J169" t="s">
         <v>1635</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14373,7 +14347,7 @@
       <c r="J170" t="s">
         <v>1635</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14414,7 +14388,7 @@
       <c r="J171" t="s">
         <v>1635</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14455,7 +14429,7 @@
       <c r="J172" t="s">
         <v>1635</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14496,7 +14470,7 @@
       <c r="J173" t="s">
         <v>1635</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14537,7 +14511,7 @@
       <c r="J174" t="s">
         <v>1635</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14578,7 +14552,7 @@
       <c r="J175" t="s">
         <v>1635</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14619,7 +14593,7 @@
       <c r="J176" t="s">
         <v>1635</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14660,7 +14634,7 @@
       <c r="J177" t="s">
         <v>1635</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14701,7 +14675,7 @@
       <c r="J178" t="s">
         <v>1635</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14719,7 +14693,7 @@
       <c r="R178" t="s">
         <v>1845</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14757,7 +14731,7 @@
       <c r="J179" t="s">
         <v>1635</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14766,7 +14740,7 @@
       <c r="M179" t="s">
         <v>1720</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14807,7 +14781,7 @@
       <c r="J180" t="s">
         <v>1635</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14848,7 +14822,7 @@
       <c r="J181" t="s">
         <v>1635</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14866,7 +14840,7 @@
       <c r="R181" t="s">
         <v>1829</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14901,7 +14875,7 @@
       <c r="J182" t="s">
         <v>1635</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14942,7 +14916,7 @@
       <c r="J183" t="s">
         <v>1635</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14983,7 +14957,7 @@
       <c r="J184" t="s">
         <v>1635</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -15024,7 +14998,7 @@
       <c r="J185" t="s">
         <v>1635</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15065,7 +15039,7 @@
       <c r="J186" t="s">
         <v>1635</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15106,7 +15080,7 @@
       <c r="J187" t="s">
         <v>1635</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15147,7 +15121,7 @@
       <c r="J188" t="s">
         <v>1635</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15188,7 +15162,7 @@
       <c r="J189" t="s">
         <v>1635</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15229,7 +15203,7 @@
       <c r="J190" t="s">
         <v>1635</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15270,7 +15244,7 @@
       <c r="J191" t="s">
         <v>1635</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15311,7 +15285,7 @@
       <c r="J192" t="s">
         <v>1635</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15352,7 +15326,7 @@
       <c r="J193" t="s">
         <v>1635</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15393,7 +15367,7 @@
       <c r="J194" t="s">
         <v>1635</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15434,7 +15408,7 @@
       <c r="J195" t="s">
         <v>1635</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15452,7 +15426,7 @@
       <c r="R195" t="s">
         <v>1838</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15493,7 +15467,7 @@
       <c r="J196" t="s">
         <v>1635</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15511,7 +15485,7 @@
       <c r="R196" t="s">
         <v>1844</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15549,7 +15523,7 @@
       <c r="J197" t="s">
         <v>1635</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15590,7 +15564,7 @@
       <c r="J198" t="s">
         <v>1637</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15631,7 +15605,7 @@
       <c r="J199" t="s">
         <v>1636</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15672,7 +15646,7 @@
       <c r="J200" t="s">
         <v>1635</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15713,7 +15687,7 @@
       <c r="J201" t="s">
         <v>1635</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15754,7 +15728,7 @@
       <c r="J202" t="s">
         <v>1635</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15772,7 +15746,7 @@
       <c r="R202" t="s">
         <v>1829</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15810,7 +15784,7 @@
       <c r="J203" t="s">
         <v>1635</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15828,7 +15802,7 @@
       <c r="R203" t="s">
         <v>1837</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15863,7 +15837,7 @@
       <c r="J204" t="s">
         <v>1635</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15878,7 +15852,7 @@
       <c r="R204" t="s">
         <v>1848</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15916,7 +15890,7 @@
       <c r="J205" t="s">
         <v>1635</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15934,7 +15908,7 @@
       <c r="R205" t="s">
         <v>1849</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15972,7 +15946,7 @@
       <c r="J206" t="s">
         <v>1635</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15990,7 +15964,7 @@
       <c r="R206" t="s">
         <v>1817</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -16025,7 +15999,7 @@
       <c r="J207" t="s">
         <v>1635</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16066,7 +16040,7 @@
       <c r="J208" t="s">
         <v>1635</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16107,7 +16081,7 @@
       <c r="J209" t="s">
         <v>1635</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16148,7 +16122,7 @@
       <c r="J210" t="s">
         <v>1635</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16189,7 +16163,7 @@
       <c r="J211" t="s">
         <v>1635</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16230,7 +16204,7 @@
       <c r="J212" t="s">
         <v>1635</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16271,7 +16245,7 @@
       <c r="J213" t="s">
         <v>1635</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16312,7 +16286,7 @@
       <c r="J214" t="s">
         <v>1635</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16330,7 +16304,7 @@
       <c r="R214" t="s">
         <v>1850</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16368,7 +16342,7 @@
       <c r="J215" t="s">
         <v>1635</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16409,7 +16383,7 @@
       <c r="J216" t="s">
         <v>1635</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16450,7 +16424,7 @@
       <c r="J217" t="s">
         <v>1635</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16491,7 +16465,7 @@
       <c r="J218" t="s">
         <v>1635</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16532,7 +16506,7 @@
       <c r="J219" t="s">
         <v>1635</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16573,7 +16547,7 @@
       <c r="J220" t="s">
         <v>1635</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16614,7 +16588,7 @@
       <c r="J221" t="s">
         <v>1635</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16655,7 +16629,7 @@
       <c r="J222" t="s">
         <v>1635</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16696,7 +16670,7 @@
       <c r="J223" t="s">
         <v>1635</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16737,7 +16711,7 @@
       <c r="J224" t="s">
         <v>1635</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16778,7 +16752,7 @@
       <c r="J225" t="s">
         <v>1635</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16819,7 +16793,7 @@
       <c r="J226" t="s">
         <v>1635</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16860,7 +16834,7 @@
       <c r="J227" t="s">
         <v>1635</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16901,7 +16875,7 @@
       <c r="J228" t="s">
         <v>1635</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16942,7 +16916,7 @@
       <c r="J229" t="s">
         <v>1635</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16983,7 +16957,7 @@
       <c r="J230" t="s">
         <v>1635</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -17024,7 +16998,7 @@
       <c r="J231" t="s">
         <v>1635</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17065,7 +17039,7 @@
       <c r="J232" t="s">
         <v>1635</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17106,7 +17080,7 @@
       <c r="J233" t="s">
         <v>1635</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17147,7 +17121,7 @@
       <c r="J234" t="s">
         <v>1635</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17188,7 +17162,7 @@
       <c r="J235" t="s">
         <v>1635</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17229,7 +17203,7 @@
       <c r="J236" t="s">
         <v>1635</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17270,7 +17244,7 @@
       <c r="J237" t="s">
         <v>1635</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17311,7 +17285,7 @@
       <c r="J238" t="s">
         <v>1635</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17352,7 +17326,7 @@
       <c r="J239" t="s">
         <v>1635</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17370,7 +17344,7 @@
       <c r="R239" t="s">
         <v>1844</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17408,7 +17382,7 @@
       <c r="J240" t="s">
         <v>1635</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17449,7 +17423,7 @@
       <c r="J241" t="s">
         <v>1635</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17490,7 +17464,7 @@
       <c r="J242" t="s">
         <v>1635</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17508,7 +17482,7 @@
       <c r="R242" t="s">
         <v>1837</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17543,7 +17517,7 @@
       <c r="J243" t="s">
         <v>1635</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17584,7 +17558,7 @@
       <c r="J244" t="s">
         <v>1635</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17625,7 +17599,7 @@
       <c r="J245" t="s">
         <v>1635</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17666,7 +17640,7 @@
       <c r="J246" t="s">
         <v>1635</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17684,7 +17658,7 @@
       <c r="R246" t="s">
         <v>1817</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17722,7 +17696,7 @@
       <c r="J247" t="s">
         <v>1635</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17763,7 +17737,7 @@
       <c r="J248" t="s">
         <v>1635</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17804,7 +17778,7 @@
       <c r="J249" t="s">
         <v>1635</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17845,7 +17819,7 @@
       <c r="J250" t="s">
         <v>1635</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17886,7 +17860,7 @@
       <c r="J251" t="s">
         <v>1635</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17927,7 +17901,7 @@
       <c r="J252" t="s">
         <v>1635</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17968,7 +17942,7 @@
       <c r="J253" t="s">
         <v>1635</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17986,7 +17960,7 @@
       <c r="R253" t="s">
         <v>1847</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18027,7 +18001,7 @@
       <c r="J254" t="s">
         <v>1635</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18068,7 +18042,7 @@
       <c r="J255" t="s">
         <v>1635</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18109,7 +18083,7 @@
       <c r="J256" t="s">
         <v>1635</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18118,7 +18092,7 @@
       <c r="M256" t="s">
         <v>1719</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18156,7 +18130,7 @@
       <c r="J257" t="s">
         <v>1635</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18165,7 +18139,7 @@
       <c r="M257" t="s">
         <v>1720</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18209,7 +18183,7 @@
       <c r="J258" t="s">
         <v>1635</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18227,7 +18201,7 @@
       <c r="R258" t="s">
         <v>1829</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18265,7 +18239,7 @@
       <c r="J259" t="s">
         <v>1635</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18283,7 +18257,7 @@
       <c r="R259" t="s">
         <v>1845</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18321,7 +18295,7 @@
       <c r="J260" t="s">
         <v>1635</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18330,7 +18304,7 @@
       <c r="M260" t="s">
         <v>1714</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18374,7 +18348,7 @@
       <c r="J261" t="s">
         <v>1635</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18392,7 +18366,7 @@
       <c r="R261" t="s">
         <v>1851</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18430,7 +18404,7 @@
       <c r="J262" t="s">
         <v>1635</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18448,7 +18422,7 @@
       <c r="R262" t="s">
         <v>1845</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18486,7 +18460,7 @@
       <c r="J263" t="s">
         <v>1635</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18495,7 +18469,7 @@
       <c r="M263" t="s">
         <v>1714</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18539,7 +18513,7 @@
       <c r="J264" t="s">
         <v>1635</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18580,7 +18554,7 @@
       <c r="J265" t="s">
         <v>1635</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18621,7 +18595,7 @@
       <c r="J266" t="s">
         <v>1635</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18662,7 +18636,7 @@
       <c r="J267" t="s">
         <v>1635</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18706,7 +18680,7 @@
       <c r="J268" t="s">
         <v>1635</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18747,7 +18721,7 @@
       <c r="J269" t="s">
         <v>1635</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18788,7 +18762,7 @@
       <c r="J270" t="s">
         <v>1635</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18829,7 +18803,7 @@
       <c r="J271" t="s">
         <v>1635</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18870,7 +18844,7 @@
       <c r="J272" t="s">
         <v>1635</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18888,7 +18862,7 @@
       <c r="R272" t="s">
         <v>1852</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18929,7 +18903,7 @@
       <c r="J273" t="s">
         <v>1635</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18973,7 +18947,7 @@
       <c r="J274" t="s">
         <v>1635</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -19014,7 +18988,7 @@
       <c r="J275" t="s">
         <v>1635</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19055,7 +19029,7 @@
       <c r="J276" t="s">
         <v>1635</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19096,7 +19070,7 @@
       <c r="J277" t="s">
         <v>1635</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19137,7 +19111,7 @@
       <c r="J278" t="s">
         <v>1635</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19178,7 +19152,7 @@
       <c r="J279" t="s">
         <v>1635</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19219,7 +19193,7 @@
       <c r="J280" t="s">
         <v>1635</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19260,7 +19234,7 @@
       <c r="J281" t="s">
         <v>1635</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19301,7 +19275,7 @@
       <c r="J282" t="s">
         <v>1635</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19342,7 +19316,7 @@
       <c r="J283" t="s">
         <v>1635</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19383,7 +19357,7 @@
       <c r="J284" t="s">
         <v>1635</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19424,7 +19398,7 @@
       <c r="J285" t="s">
         <v>1635</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19465,7 +19439,7 @@
       <c r="J286" t="s">
         <v>1635</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19506,7 +19480,7 @@
       <c r="J287" t="s">
         <v>1635</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19547,7 +19521,7 @@
       <c r="J288" t="s">
         <v>1635</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19588,7 +19562,7 @@
       <c r="J289" t="s">
         <v>1635</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19629,7 +19603,7 @@
       <c r="J290" t="s">
         <v>1635</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19670,7 +19644,7 @@
       <c r="J291" t="s">
         <v>1635</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19711,7 +19685,7 @@
       <c r="J292" t="s">
         <v>1635</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19752,7 +19726,7 @@
       <c r="J293" t="s">
         <v>1635</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19793,7 +19767,7 @@
       <c r="J294" t="s">
         <v>1635</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19834,7 +19808,7 @@
       <c r="J295" t="s">
         <v>1635</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19852,7 +19826,7 @@
       <c r="R295" t="s">
         <v>1853</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19893,7 +19867,7 @@
       <c r="J296" t="s">
         <v>1635</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19911,7 +19885,7 @@
       <c r="R296" t="s">
         <v>1829</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19949,7 +19923,7 @@
       <c r="J297" t="s">
         <v>1635</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19990,7 +19964,7 @@
       <c r="J298" t="s">
         <v>1635</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20031,7 +20005,7 @@
       <c r="J299" t="s">
         <v>1636</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20072,7 +20046,7 @@
       <c r="J300" t="s">
         <v>1635</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20113,7 +20087,7 @@
       <c r="J301" t="s">
         <v>1635</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20951,7 +20925,7 @@
       <c r="R321" t="s">
         <v>1815</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21174,7 +21148,7 @@
       <c r="R326" t="s">
         <v>1854</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -22009,7 +21983,7 @@
       <c r="R346" t="s">
         <v>1855</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (19/10/2026 13:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5753,8 +5753,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5770,7 +5778,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5778,12 +5786,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6083,73 +6109,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6184,7 +6210,7 @@
       <c r="J2" t="s">
         <v>1635</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6228,7 +6254,7 @@
       <c r="J3" t="s">
         <v>1635</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6272,7 +6298,7 @@
       <c r="J4" t="s">
         <v>1635</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6290,7 +6316,7 @@
       <c r="R4" t="s">
         <v>1812</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6328,7 +6354,7 @@
       <c r="J5" t="s">
         <v>1636</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6378,7 +6404,7 @@
       <c r="J6" t="s">
         <v>1635</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6425,7 +6451,7 @@
       <c r="J7" t="s">
         <v>1635</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6472,7 +6498,7 @@
       <c r="J8" t="s">
         <v>1635</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6519,7 +6545,7 @@
       <c r="J9" t="s">
         <v>1635</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6566,7 +6592,7 @@
       <c r="J10" t="s">
         <v>1635</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6613,7 +6639,7 @@
       <c r="J11" t="s">
         <v>1635</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6660,7 +6686,7 @@
       <c r="J12" t="s">
         <v>1635</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6704,7 +6730,7 @@
       <c r="J13" t="s">
         <v>1635</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6722,7 +6748,7 @@
       <c r="R13" t="s">
         <v>1813</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6760,7 +6786,7 @@
       <c r="J14" t="s">
         <v>1635</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6778,7 +6804,7 @@
       <c r="R14" t="s">
         <v>1814</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6819,7 +6845,7 @@
       <c r="J15" t="s">
         <v>1635</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6837,7 +6863,7 @@
       <c r="R15" t="s">
         <v>1814</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6878,7 +6904,7 @@
       <c r="J16" t="s">
         <v>1635</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6922,7 +6948,7 @@
       <c r="J17" t="s">
         <v>1635</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6966,7 +6992,7 @@
       <c r="J18" t="s">
         <v>1635</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6984,7 +7010,7 @@
       <c r="R18" t="s">
         <v>1815</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7025,7 +7051,7 @@
       <c r="J19" t="s">
         <v>1635</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7069,7 +7095,7 @@
       <c r="J20" t="s">
         <v>1635</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7113,7 +7139,7 @@
       <c r="J21" t="s">
         <v>1635</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7131,7 +7157,7 @@
       <c r="R21" t="s">
         <v>1814</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7172,7 +7198,7 @@
       <c r="J22" t="s">
         <v>1635</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7190,7 +7216,7 @@
       <c r="R22" t="s">
         <v>1816</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7231,7 +7257,7 @@
       <c r="J23" t="s">
         <v>1635</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7249,7 +7275,7 @@
       <c r="R23" t="s">
         <v>1817</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7290,7 +7316,7 @@
       <c r="J24" t="s">
         <v>1635</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7334,7 +7360,7 @@
       <c r="J25" t="s">
         <v>1635</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7375,7 +7401,7 @@
       <c r="J26" t="s">
         <v>1637</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7393,7 +7419,7 @@
       <c r="R26" t="s">
         <v>1818</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7431,7 +7457,7 @@
       <c r="J27" t="s">
         <v>1635</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7449,7 +7475,7 @@
       <c r="R27" t="s">
         <v>1819</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7490,7 +7516,7 @@
       <c r="J28" t="s">
         <v>1635</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7534,7 +7560,7 @@
       <c r="J29" t="s">
         <v>1635</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7578,7 +7604,7 @@
       <c r="J30" t="s">
         <v>1635</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7622,7 +7648,7 @@
       <c r="J31" t="s">
         <v>1635</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7640,7 +7666,7 @@
       <c r="R31" t="s">
         <v>1820</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7681,7 +7707,7 @@
       <c r="J32" t="s">
         <v>1635</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7725,7 +7751,7 @@
       <c r="J33" t="s">
         <v>1635</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7743,7 +7769,7 @@
       <c r="R33" t="s">
         <v>1821</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7784,7 +7810,7 @@
       <c r="J34" t="s">
         <v>1635</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7828,7 +7854,7 @@
       <c r="J35" t="s">
         <v>1635</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7846,7 +7872,7 @@
       <c r="R35" t="s">
         <v>1822</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7887,7 +7913,7 @@
       <c r="J36" t="s">
         <v>1635</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7905,7 +7931,7 @@
       <c r="R36" t="s">
         <v>1822</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7946,7 +7972,7 @@
       <c r="J37" t="s">
         <v>1635</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7964,7 +7990,7 @@
       <c r="R37" t="s">
         <v>1822</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8005,7 +8031,7 @@
       <c r="J38" t="s">
         <v>1635</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8023,7 +8049,7 @@
       <c r="R38" t="s">
         <v>1822</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8064,7 +8090,7 @@
       <c r="J39" t="s">
         <v>1635</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8082,7 +8108,7 @@
       <c r="R39" t="s">
         <v>1822</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8123,7 +8149,7 @@
       <c r="J40" t="s">
         <v>1635</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8141,7 +8167,7 @@
       <c r="R40" t="s">
         <v>1823</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8182,7 +8208,7 @@
       <c r="J41" t="s">
         <v>1635</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8200,7 +8226,7 @@
       <c r="R41" t="s">
         <v>1814</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8241,7 +8267,7 @@
       <c r="J42" t="s">
         <v>1635</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8259,7 +8285,7 @@
       <c r="R42" t="s">
         <v>1822</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8300,7 +8326,7 @@
       <c r="J43" t="s">
         <v>1635</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8344,7 +8370,7 @@
       <c r="J44" t="s">
         <v>1635</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8362,7 +8388,7 @@
       <c r="R44" t="s">
         <v>1824</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8403,7 +8429,7 @@
       <c r="J45" t="s">
         <v>1635</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8421,7 +8447,7 @@
       <c r="R45" t="s">
         <v>1825</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8459,7 +8485,7 @@
       <c r="J46" t="s">
         <v>1635</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8503,7 +8529,7 @@
       <c r="J47" t="s">
         <v>1635</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8521,7 +8547,7 @@
       <c r="R47" t="s">
         <v>1826</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8562,7 +8588,7 @@
       <c r="J48" t="s">
         <v>1635</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8606,7 +8632,7 @@
       <c r="J49" t="s">
         <v>1635</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8650,7 +8676,7 @@
       <c r="J50" t="s">
         <v>1635</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8694,7 +8720,7 @@
       <c r="J51" t="s">
         <v>1635</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8741,7 +8767,7 @@
       <c r="J52" t="s">
         <v>1635</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8785,7 +8811,7 @@
       <c r="J53" t="s">
         <v>1635</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8829,7 +8855,7 @@
       <c r="J54" t="s">
         <v>1635</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8873,7 +8899,7 @@
       <c r="J55" t="s">
         <v>1635</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8923,7 +8949,7 @@
       <c r="J56" t="s">
         <v>1635</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8976,7 +9002,7 @@
       <c r="J57" t="s">
         <v>1635</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9026,7 +9052,7 @@
       <c r="J58" t="s">
         <v>1635</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9076,7 +9102,7 @@
       <c r="J59" t="s">
         <v>1635</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9094,7 +9120,7 @@
       <c r="R59" t="s">
         <v>1827</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9135,7 +9161,7 @@
       <c r="J60" t="s">
         <v>1635</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9179,7 +9205,7 @@
       <c r="J61" t="s">
         <v>1635</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9223,7 +9249,7 @@
       <c r="J62" t="s">
         <v>1635</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9267,7 +9293,7 @@
       <c r="J63" t="s">
         <v>1635</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9311,7 +9337,7 @@
       <c r="J64" t="s">
         <v>1635</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9355,7 +9381,7 @@
       <c r="J65" t="s">
         <v>1635</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9402,7 +9428,7 @@
       <c r="J66" t="s">
         <v>1635</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9420,7 +9446,7 @@
       <c r="R66" t="s">
         <v>1828</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9458,7 +9484,7 @@
       <c r="J67" t="s">
         <v>1635</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9502,7 +9528,7 @@
       <c r="J68" t="s">
         <v>1635</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9517,7 +9543,7 @@
       <c r="O68" t="s">
         <v>1732</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9561,7 +9587,7 @@
       <c r="J69" t="s">
         <v>1637</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9605,7 +9631,7 @@
       <c r="J70" t="s">
         <v>1635</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9649,7 +9675,7 @@
       <c r="J71" t="s">
         <v>1635</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9693,7 +9719,7 @@
       <c r="J72" t="s">
         <v>1635</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9737,7 +9763,7 @@
       <c r="J73" t="s">
         <v>1635</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9781,7 +9807,7 @@
       <c r="J74" t="s">
         <v>1635</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9825,7 +9851,7 @@
       <c r="J75" t="s">
         <v>1635</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9869,7 +9895,7 @@
       <c r="J76" t="s">
         <v>1635</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9887,7 +9913,7 @@
       <c r="R76" t="s">
         <v>1829</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9925,7 +9951,7 @@
       <c r="J77" t="s">
         <v>1635</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9943,7 +9969,7 @@
       <c r="R77" t="s">
         <v>1829</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9981,7 +10007,7 @@
       <c r="J78" t="s">
         <v>1635</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9999,7 +10025,7 @@
       <c r="R78" t="s">
         <v>1829</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10037,7 +10063,7 @@
       <c r="J79" t="s">
         <v>1635</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10055,7 +10081,7 @@
       <c r="R79" t="s">
         <v>1829</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10093,7 +10119,7 @@
       <c r="J80" t="s">
         <v>1635</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10137,7 +10163,7 @@
       <c r="J81" t="s">
         <v>1635</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10181,7 +10207,7 @@
       <c r="J82" t="s">
         <v>1635</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10225,7 +10251,7 @@
       <c r="J83" t="s">
         <v>1635</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10269,7 +10295,7 @@
       <c r="J84" t="s">
         <v>1635</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10313,7 +10339,7 @@
       <c r="J85" t="s">
         <v>1635</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10331,7 +10357,7 @@
       <c r="R85" t="s">
         <v>1830</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10369,7 +10395,7 @@
       <c r="J86" t="s">
         <v>1635</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10413,7 +10439,7 @@
       <c r="J87" t="s">
         <v>1635</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10431,7 +10457,7 @@
       <c r="R87" t="s">
         <v>1831</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10469,7 +10495,7 @@
       <c r="J88" t="s">
         <v>1635</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10513,7 +10539,7 @@
       <c r="J89" t="s">
         <v>1635</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10531,7 +10557,7 @@
       <c r="R89" t="s">
         <v>1832</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10566,7 +10592,7 @@
       <c r="J90" t="s">
         <v>1635</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10584,7 +10610,7 @@
       <c r="R90" t="s">
         <v>1833</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10619,7 +10645,7 @@
       <c r="J91" t="s">
         <v>1635</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10637,7 +10663,7 @@
       <c r="R91" t="s">
         <v>1817</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10675,7 +10701,7 @@
       <c r="J92" t="s">
         <v>1635</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10696,7 +10722,7 @@
       <c r="R92" t="s">
         <v>1817</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10737,7 +10763,7 @@
       <c r="J93" t="s">
         <v>1635</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10778,7 +10804,7 @@
       <c r="J94" t="s">
         <v>1635</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10822,7 +10848,7 @@
       <c r="J95" t="s">
         <v>1635</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10866,7 +10892,7 @@
       <c r="J96" t="s">
         <v>1635</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10884,7 +10910,7 @@
       <c r="R96" t="s">
         <v>1834</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10925,7 +10951,7 @@
       <c r="J97" t="s">
         <v>1635</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10940,7 +10966,7 @@
       <c r="R97" t="s">
         <v>1834</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10981,7 +11007,7 @@
       <c r="J98" t="s">
         <v>1635</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10999,7 +11025,7 @@
       <c r="R98" t="s">
         <v>1835</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11037,7 +11063,7 @@
       <c r="J99" t="s">
         <v>1635</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11055,7 +11081,7 @@
       <c r="R99" t="s">
         <v>1836</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11093,7 +11119,7 @@
       <c r="J100" t="s">
         <v>1635</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11134,7 +11160,7 @@
       <c r="J101" t="s">
         <v>1635</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11175,7 +11201,7 @@
       <c r="J102" t="s">
         <v>1635</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11216,7 +11242,7 @@
       <c r="J103" t="s">
         <v>1635</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11257,7 +11283,7 @@
       <c r="J104" t="s">
         <v>1635</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11298,7 +11324,7 @@
       <c r="J105" t="s">
         <v>1635</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11339,7 +11365,7 @@
       <c r="J106" t="s">
         <v>1635</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11380,7 +11406,7 @@
       <c r="J107" t="s">
         <v>1635</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11421,7 +11447,7 @@
       <c r="J108" t="s">
         <v>1635</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11462,7 +11488,7 @@
       <c r="J109" t="s">
         <v>1635</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11515,7 +11541,7 @@
       <c r="J110" t="s">
         <v>1635</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11571,7 +11597,7 @@
       <c r="J111" t="s">
         <v>1635</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11589,7 +11615,7 @@
       <c r="R111" t="s">
         <v>1838</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11627,7 +11653,7 @@
       <c r="J112" t="s">
         <v>1635</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11686,7 +11712,7 @@
       <c r="J113" t="s">
         <v>1635</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11730,7 +11756,7 @@
       <c r="J114" t="s">
         <v>1635</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11774,7 +11800,7 @@
       <c r="J115" t="s">
         <v>1635</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11792,7 +11818,7 @@
       <c r="R115" t="s">
         <v>1840</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11833,7 +11859,7 @@
       <c r="J116" t="s">
         <v>1635</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11892,7 +11918,7 @@
       <c r="J117" t="s">
         <v>1635</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11936,7 +11962,7 @@
       <c r="J118" t="s">
         <v>1635</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11983,7 +12009,7 @@
       <c r="J119" t="s">
         <v>1635</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12024,7 +12050,7 @@
       <c r="J120" t="s">
         <v>1635</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12068,7 +12094,7 @@
       <c r="J121" t="s">
         <v>1635</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12115,7 +12141,7 @@
       <c r="J122" t="s">
         <v>1635</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12165,7 +12191,7 @@
       <c r="J123" t="s">
         <v>1635</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12209,7 +12235,7 @@
       <c r="J124" t="s">
         <v>1635</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12253,7 +12279,7 @@
       <c r="J125" t="s">
         <v>1635</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12271,7 +12297,7 @@
       <c r="R125" t="s">
         <v>1842</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12306,7 +12332,7 @@
       <c r="J126" t="s">
         <v>1635</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12324,7 +12350,7 @@
       <c r="R126" t="s">
         <v>1843</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12362,7 +12388,7 @@
       <c r="J127" t="s">
         <v>1635</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12418,7 +12444,7 @@
       <c r="J128" t="s">
         <v>1635</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12459,7 +12485,7 @@
       <c r="J129" t="s">
         <v>1635</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12500,7 +12526,7 @@
       <c r="J130" t="s">
         <v>1635</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12541,7 +12567,7 @@
       <c r="J131" t="s">
         <v>1635</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12585,7 +12611,7 @@
       <c r="J132" t="s">
         <v>1635</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12626,7 +12652,7 @@
       <c r="J133" t="s">
         <v>1635</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12644,7 +12670,7 @@
       <c r="R133" t="s">
         <v>1829</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12682,7 +12708,7 @@
       <c r="J134" t="s">
         <v>1635</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12700,7 +12726,7 @@
       <c r="R134" t="s">
         <v>1829</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12735,7 +12761,7 @@
       <c r="J135" t="s">
         <v>1635</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12776,7 +12802,7 @@
       <c r="J136" t="s">
         <v>1635</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12817,7 +12843,7 @@
       <c r="J137" t="s">
         <v>1635</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12858,7 +12884,7 @@
       <c r="J138" t="s">
         <v>1635</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12899,7 +12925,7 @@
       <c r="J139" t="s">
         <v>1635</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12946,7 +12972,7 @@
       <c r="J140" t="s">
         <v>1635</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12987,7 +13013,7 @@
       <c r="J141" t="s">
         <v>1635</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13028,7 +13054,7 @@
       <c r="J142" t="s">
         <v>1635</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13072,7 +13098,7 @@
       <c r="J143" t="s">
         <v>1635</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13090,7 +13116,7 @@
       <c r="R143" t="s">
         <v>1829</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13125,7 +13151,7 @@
       <c r="J144" t="s">
         <v>1635</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13143,7 +13169,7 @@
       <c r="R144" t="s">
         <v>1829</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13181,7 +13207,7 @@
       <c r="J145" t="s">
         <v>1635</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13199,7 +13225,7 @@
       <c r="R145" t="s">
         <v>1829</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13234,7 +13260,7 @@
       <c r="J146" t="s">
         <v>1635</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13252,7 +13278,7 @@
       <c r="R146" t="s">
         <v>1837</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13287,7 +13313,7 @@
       <c r="J147" t="s">
         <v>1635</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13305,7 +13331,7 @@
       <c r="R147" t="s">
         <v>1844</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13340,7 +13366,7 @@
       <c r="J148" t="s">
         <v>1635</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13381,7 +13407,7 @@
       <c r="J149" t="s">
         <v>1635</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13399,7 +13425,7 @@
       <c r="R149" t="s">
         <v>1829</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13434,7 +13460,7 @@
       <c r="J150" t="s">
         <v>1635</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13452,7 +13478,7 @@
       <c r="R150" t="s">
         <v>1829</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13490,7 +13516,7 @@
       <c r="J151" t="s">
         <v>1635</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13508,7 +13534,7 @@
       <c r="R151" t="s">
         <v>1845</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13543,7 +13569,7 @@
       <c r="J152" t="s">
         <v>1635</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13561,7 +13587,7 @@
       <c r="R152" t="s">
         <v>1846</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13596,7 +13622,7 @@
       <c r="J153" t="s">
         <v>1635</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13605,7 +13631,7 @@
       <c r="M153" t="s">
         <v>1723</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13646,7 +13672,7 @@
       <c r="J154" t="s">
         <v>1635</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13687,7 +13713,7 @@
       <c r="J155" t="s">
         <v>1635</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13728,7 +13754,7 @@
       <c r="J156" t="s">
         <v>1635</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13769,7 +13795,7 @@
       <c r="J157" t="s">
         <v>1635</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13810,7 +13836,7 @@
       <c r="J158" t="s">
         <v>1635</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13851,7 +13877,7 @@
       <c r="J159" t="s">
         <v>1635</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13892,7 +13918,7 @@
       <c r="J160" t="s">
         <v>1635</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13933,7 +13959,7 @@
       <c r="J161" t="s">
         <v>1635</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13974,7 +14000,7 @@
       <c r="J162" t="s">
         <v>1635</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13992,7 +14018,7 @@
       <c r="R162" t="s">
         <v>1832</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14027,7 +14053,7 @@
       <c r="J163" t="s">
         <v>1635</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14045,7 +14071,7 @@
       <c r="R163" t="s">
         <v>1829</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14080,7 +14106,7 @@
       <c r="J164" t="s">
         <v>1635</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14124,7 +14150,7 @@
       <c r="J165" t="s">
         <v>1635</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14165,7 +14191,7 @@
       <c r="J166" t="s">
         <v>1635</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14183,7 +14209,7 @@
       <c r="R166" t="s">
         <v>1847</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14218,7 +14244,7 @@
       <c r="J167" t="s">
         <v>1635</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14262,7 +14288,7 @@
       <c r="J168" t="s">
         <v>1635</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14306,7 +14332,7 @@
       <c r="J169" t="s">
         <v>1635</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14347,7 +14373,7 @@
       <c r="J170" t="s">
         <v>1635</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14388,7 +14414,7 @@
       <c r="J171" t="s">
         <v>1635</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14429,7 +14455,7 @@
       <c r="J172" t="s">
         <v>1635</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14470,7 +14496,7 @@
       <c r="J173" t="s">
         <v>1635</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14511,7 +14537,7 @@
       <c r="J174" t="s">
         <v>1635</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14552,7 +14578,7 @@
       <c r="J175" t="s">
         <v>1635</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14593,7 +14619,7 @@
       <c r="J176" t="s">
         <v>1635</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14634,7 +14660,7 @@
       <c r="J177" t="s">
         <v>1635</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14675,7 +14701,7 @@
       <c r="J178" t="s">
         <v>1635</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14693,7 +14719,7 @@
       <c r="R178" t="s">
         <v>1845</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14731,7 +14757,7 @@
       <c r="J179" t="s">
         <v>1635</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14740,7 +14766,7 @@
       <c r="M179" t="s">
         <v>1720</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14781,7 +14807,7 @@
       <c r="J180" t="s">
         <v>1635</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14822,7 +14848,7 @@
       <c r="J181" t="s">
         <v>1635</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14840,7 +14866,7 @@
       <c r="R181" t="s">
         <v>1829</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14875,7 +14901,7 @@
       <c r="J182" t="s">
         <v>1635</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14916,7 +14942,7 @@
       <c r="J183" t="s">
         <v>1635</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14957,7 +14983,7 @@
       <c r="J184" t="s">
         <v>1635</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14998,7 +15024,7 @@
       <c r="J185" t="s">
         <v>1635</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15039,7 +15065,7 @@
       <c r="J186" t="s">
         <v>1635</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15080,7 +15106,7 @@
       <c r="J187" t="s">
         <v>1635</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15121,7 +15147,7 @@
       <c r="J188" t="s">
         <v>1635</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15162,7 +15188,7 @@
       <c r="J189" t="s">
         <v>1635</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15203,7 +15229,7 @@
       <c r="J190" t="s">
         <v>1635</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15244,7 +15270,7 @@
       <c r="J191" t="s">
         <v>1635</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15285,7 +15311,7 @@
       <c r="J192" t="s">
         <v>1635</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15326,7 +15352,7 @@
       <c r="J193" t="s">
         <v>1635</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15367,7 +15393,7 @@
       <c r="J194" t="s">
         <v>1635</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15408,7 +15434,7 @@
       <c r="J195" t="s">
         <v>1635</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15426,7 +15452,7 @@
       <c r="R195" t="s">
         <v>1838</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15467,7 +15493,7 @@
       <c r="J196" t="s">
         <v>1635</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15485,7 +15511,7 @@
       <c r="R196" t="s">
         <v>1844</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15523,7 +15549,7 @@
       <c r="J197" t="s">
         <v>1635</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15564,7 +15590,7 @@
       <c r="J198" t="s">
         <v>1637</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15605,7 +15631,7 @@
       <c r="J199" t="s">
         <v>1636</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15646,7 +15672,7 @@
       <c r="J200" t="s">
         <v>1635</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15687,7 +15713,7 @@
       <c r="J201" t="s">
         <v>1635</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15728,7 +15754,7 @@
       <c r="J202" t="s">
         <v>1635</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15746,7 +15772,7 @@
       <c r="R202" t="s">
         <v>1829</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15784,7 +15810,7 @@
       <c r="J203" t="s">
         <v>1635</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15802,7 +15828,7 @@
       <c r="R203" t="s">
         <v>1837</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15837,7 +15863,7 @@
       <c r="J204" t="s">
         <v>1635</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15852,7 +15878,7 @@
       <c r="R204" t="s">
         <v>1848</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15890,7 +15916,7 @@
       <c r="J205" t="s">
         <v>1635</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15908,7 +15934,7 @@
       <c r="R205" t="s">
         <v>1849</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15946,7 +15972,7 @@
       <c r="J206" t="s">
         <v>1635</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15964,7 +15990,7 @@
       <c r="R206" t="s">
         <v>1817</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15999,7 +16025,7 @@
       <c r="J207" t="s">
         <v>1635</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16040,7 +16066,7 @@
       <c r="J208" t="s">
         <v>1635</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16081,7 +16107,7 @@
       <c r="J209" t="s">
         <v>1635</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16122,7 +16148,7 @@
       <c r="J210" t="s">
         <v>1635</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16163,7 +16189,7 @@
       <c r="J211" t="s">
         <v>1635</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16204,7 +16230,7 @@
       <c r="J212" t="s">
         <v>1635</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16245,7 +16271,7 @@
       <c r="J213" t="s">
         <v>1635</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16286,7 +16312,7 @@
       <c r="J214" t="s">
         <v>1635</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16304,7 +16330,7 @@
       <c r="R214" t="s">
         <v>1850</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16342,7 +16368,7 @@
       <c r="J215" t="s">
         <v>1635</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16383,7 +16409,7 @@
       <c r="J216" t="s">
         <v>1635</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16424,7 +16450,7 @@
       <c r="J217" t="s">
         <v>1635</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16465,7 +16491,7 @@
       <c r="J218" t="s">
         <v>1635</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16506,7 +16532,7 @@
       <c r="J219" t="s">
         <v>1635</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16547,7 +16573,7 @@
       <c r="J220" t="s">
         <v>1635</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16588,7 +16614,7 @@
       <c r="J221" t="s">
         <v>1635</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16629,7 +16655,7 @@
       <c r="J222" t="s">
         <v>1635</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16670,7 +16696,7 @@
       <c r="J223" t="s">
         <v>1635</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16711,7 +16737,7 @@
       <c r="J224" t="s">
         <v>1635</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16752,7 +16778,7 @@
       <c r="J225" t="s">
         <v>1635</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16793,7 +16819,7 @@
       <c r="J226" t="s">
         <v>1635</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16834,7 +16860,7 @@
       <c r="J227" t="s">
         <v>1635</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16875,7 +16901,7 @@
       <c r="J228" t="s">
         <v>1635</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16916,7 +16942,7 @@
       <c r="J229" t="s">
         <v>1635</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16957,7 +16983,7 @@
       <c r="J230" t="s">
         <v>1635</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16998,7 +17024,7 @@
       <c r="J231" t="s">
         <v>1635</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17039,7 +17065,7 @@
       <c r="J232" t="s">
         <v>1635</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17080,7 +17106,7 @@
       <c r="J233" t="s">
         <v>1635</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17121,7 +17147,7 @@
       <c r="J234" t="s">
         <v>1635</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17162,7 +17188,7 @@
       <c r="J235" t="s">
         <v>1635</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17203,7 +17229,7 @@
       <c r="J236" t="s">
         <v>1635</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17244,7 +17270,7 @@
       <c r="J237" t="s">
         <v>1635</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17285,7 +17311,7 @@
       <c r="J238" t="s">
         <v>1635</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17326,7 +17352,7 @@
       <c r="J239" t="s">
         <v>1635</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17344,7 +17370,7 @@
       <c r="R239" t="s">
         <v>1844</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17382,7 +17408,7 @@
       <c r="J240" t="s">
         <v>1635</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17423,7 +17449,7 @@
       <c r="J241" t="s">
         <v>1635</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17464,7 +17490,7 @@
       <c r="J242" t="s">
         <v>1635</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17482,7 +17508,7 @@
       <c r="R242" t="s">
         <v>1837</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17517,7 +17543,7 @@
       <c r="J243" t="s">
         <v>1635</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17558,7 +17584,7 @@
       <c r="J244" t="s">
         <v>1635</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17599,7 +17625,7 @@
       <c r="J245" t="s">
         <v>1635</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17640,7 +17666,7 @@
       <c r="J246" t="s">
         <v>1635</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17658,7 +17684,7 @@
       <c r="R246" t="s">
         <v>1817</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17696,7 +17722,7 @@
       <c r="J247" t="s">
         <v>1635</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17737,7 +17763,7 @@
       <c r="J248" t="s">
         <v>1635</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17778,7 +17804,7 @@
       <c r="J249" t="s">
         <v>1635</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17819,7 +17845,7 @@
       <c r="J250" t="s">
         <v>1635</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17860,7 +17886,7 @@
       <c r="J251" t="s">
         <v>1635</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17901,7 +17927,7 @@
       <c r="J252" t="s">
         <v>1635</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17942,7 +17968,7 @@
       <c r="J253" t="s">
         <v>1635</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17960,7 +17986,7 @@
       <c r="R253" t="s">
         <v>1847</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18001,7 +18027,7 @@
       <c r="J254" t="s">
         <v>1635</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18042,7 +18068,7 @@
       <c r="J255" t="s">
         <v>1635</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18083,7 +18109,7 @@
       <c r="J256" t="s">
         <v>1635</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18092,7 +18118,7 @@
       <c r="M256" t="s">
         <v>1719</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18130,7 +18156,7 @@
       <c r="J257" t="s">
         <v>1635</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18139,7 +18165,7 @@
       <c r="M257" t="s">
         <v>1720</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18183,7 +18209,7 @@
       <c r="J258" t="s">
         <v>1635</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18201,7 +18227,7 @@
       <c r="R258" t="s">
         <v>1829</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18239,7 +18265,7 @@
       <c r="J259" t="s">
         <v>1635</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18257,7 +18283,7 @@
       <c r="R259" t="s">
         <v>1845</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18295,7 +18321,7 @@
       <c r="J260" t="s">
         <v>1635</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18304,7 +18330,7 @@
       <c r="M260" t="s">
         <v>1714</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18348,7 +18374,7 @@
       <c r="J261" t="s">
         <v>1635</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18366,7 +18392,7 @@
       <c r="R261" t="s">
         <v>1851</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18404,7 +18430,7 @@
       <c r="J262" t="s">
         <v>1635</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18422,7 +18448,7 @@
       <c r="R262" t="s">
         <v>1845</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18460,7 +18486,7 @@
       <c r="J263" t="s">
         <v>1635</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18469,7 +18495,7 @@
       <c r="M263" t="s">
         <v>1714</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18513,7 +18539,7 @@
       <c r="J264" t="s">
         <v>1635</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18554,7 +18580,7 @@
       <c r="J265" t="s">
         <v>1635</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18595,7 +18621,7 @@
       <c r="J266" t="s">
         <v>1635</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18636,7 +18662,7 @@
       <c r="J267" t="s">
         <v>1635</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18680,7 +18706,7 @@
       <c r="J268" t="s">
         <v>1635</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18721,7 +18747,7 @@
       <c r="J269" t="s">
         <v>1635</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18762,7 +18788,7 @@
       <c r="J270" t="s">
         <v>1635</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18803,7 +18829,7 @@
       <c r="J271" t="s">
         <v>1635</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18844,7 +18870,7 @@
       <c r="J272" t="s">
         <v>1635</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18862,7 +18888,7 @@
       <c r="R272" t="s">
         <v>1852</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18903,7 +18929,7 @@
       <c r="J273" t="s">
         <v>1635</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18947,7 +18973,7 @@
       <c r="J274" t="s">
         <v>1635</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18988,7 +19014,7 @@
       <c r="J275" t="s">
         <v>1635</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19029,7 +19055,7 @@
       <c r="J276" t="s">
         <v>1635</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19070,7 +19096,7 @@
       <c r="J277" t="s">
         <v>1635</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19111,7 +19137,7 @@
       <c r="J278" t="s">
         <v>1635</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19152,7 +19178,7 @@
       <c r="J279" t="s">
         <v>1635</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19193,7 +19219,7 @@
       <c r="J280" t="s">
         <v>1635</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19234,7 +19260,7 @@
       <c r="J281" t="s">
         <v>1635</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19275,7 +19301,7 @@
       <c r="J282" t="s">
         <v>1635</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19316,7 +19342,7 @@
       <c r="J283" t="s">
         <v>1635</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19357,7 +19383,7 @@
       <c r="J284" t="s">
         <v>1635</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19398,7 +19424,7 @@
       <c r="J285" t="s">
         <v>1635</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19439,7 +19465,7 @@
       <c r="J286" t="s">
         <v>1635</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19480,7 +19506,7 @@
       <c r="J287" t="s">
         <v>1635</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19521,7 +19547,7 @@
       <c r="J288" t="s">
         <v>1635</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19562,7 +19588,7 @@
       <c r="J289" t="s">
         <v>1635</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19603,7 +19629,7 @@
       <c r="J290" t="s">
         <v>1635</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19644,7 +19670,7 @@
       <c r="J291" t="s">
         <v>1635</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19685,7 +19711,7 @@
       <c r="J292" t="s">
         <v>1635</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19726,7 +19752,7 @@
       <c r="J293" t="s">
         <v>1635</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19767,7 +19793,7 @@
       <c r="J294" t="s">
         <v>1635</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19808,7 +19834,7 @@
       <c r="J295" t="s">
         <v>1635</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19826,7 +19852,7 @@
       <c r="R295" t="s">
         <v>1853</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19867,7 +19893,7 @@
       <c r="J296" t="s">
         <v>1635</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19885,7 +19911,7 @@
       <c r="R296" t="s">
         <v>1829</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19923,7 +19949,7 @@
       <c r="J297" t="s">
         <v>1635</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19964,7 +19990,7 @@
       <c r="J298" t="s">
         <v>1635</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20005,7 +20031,7 @@
       <c r="J299" t="s">
         <v>1636</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20046,7 +20072,7 @@
       <c r="J300" t="s">
         <v>1635</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20087,7 +20113,7 @@
       <c r="J301" t="s">
         <v>1635</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20925,7 +20951,7 @@
       <c r="R321" t="s">
         <v>1815</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21148,7 +21174,7 @@
       <c r="R326" t="s">
         <v>1854</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21983,7 +22009,7 @@
       <c r="R346" t="s">
         <v>1855</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (19/10/2026 14:28)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5753,16 +5753,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5778,7 +5770,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5786,30 +5778,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6109,73 +6083,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6210,7 +6184,7 @@
       <c r="J2" t="s">
         <v>1635</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6254,7 +6228,7 @@
       <c r="J3" t="s">
         <v>1635</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6298,7 +6272,7 @@
       <c r="J4" t="s">
         <v>1635</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6316,7 +6290,7 @@
       <c r="R4" t="s">
         <v>1812</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6354,7 +6328,7 @@
       <c r="J5" t="s">
         <v>1636</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6404,7 +6378,7 @@
       <c r="J6" t="s">
         <v>1635</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6451,7 +6425,7 @@
       <c r="J7" t="s">
         <v>1635</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6498,7 +6472,7 @@
       <c r="J8" t="s">
         <v>1635</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6545,7 +6519,7 @@
       <c r="J9" t="s">
         <v>1635</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6592,7 +6566,7 @@
       <c r="J10" t="s">
         <v>1635</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6639,7 +6613,7 @@
       <c r="J11" t="s">
         <v>1635</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6686,7 +6660,7 @@
       <c r="J12" t="s">
         <v>1635</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6730,7 +6704,7 @@
       <c r="J13" t="s">
         <v>1635</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6748,7 +6722,7 @@
       <c r="R13" t="s">
         <v>1813</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6786,7 +6760,7 @@
       <c r="J14" t="s">
         <v>1635</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6804,7 +6778,7 @@
       <c r="R14" t="s">
         <v>1814</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6845,7 +6819,7 @@
       <c r="J15" t="s">
         <v>1635</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6863,7 +6837,7 @@
       <c r="R15" t="s">
         <v>1814</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6904,7 +6878,7 @@
       <c r="J16" t="s">
         <v>1635</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6948,7 +6922,7 @@
       <c r="J17" t="s">
         <v>1635</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6992,7 +6966,7 @@
       <c r="J18" t="s">
         <v>1635</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -7010,7 +6984,7 @@
       <c r="R18" t="s">
         <v>1815</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7051,7 +7025,7 @@
       <c r="J19" t="s">
         <v>1635</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7095,7 +7069,7 @@
       <c r="J20" t="s">
         <v>1635</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7139,7 +7113,7 @@
       <c r="J21" t="s">
         <v>1635</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7157,7 +7131,7 @@
       <c r="R21" t="s">
         <v>1814</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7198,7 +7172,7 @@
       <c r="J22" t="s">
         <v>1635</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7216,7 +7190,7 @@
       <c r="R22" t="s">
         <v>1816</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7257,7 +7231,7 @@
       <c r="J23" t="s">
         <v>1635</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7275,7 +7249,7 @@
       <c r="R23" t="s">
         <v>1817</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7316,7 +7290,7 @@
       <c r="J24" t="s">
         <v>1635</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7360,7 +7334,7 @@
       <c r="J25" t="s">
         <v>1635</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7401,7 +7375,7 @@
       <c r="J26" t="s">
         <v>1637</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7419,7 +7393,7 @@
       <c r="R26" t="s">
         <v>1818</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7457,7 +7431,7 @@
       <c r="J27" t="s">
         <v>1635</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7475,7 +7449,7 @@
       <c r="R27" t="s">
         <v>1819</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7516,7 +7490,7 @@
       <c r="J28" t="s">
         <v>1635</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7560,7 +7534,7 @@
       <c r="J29" t="s">
         <v>1635</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7604,7 +7578,7 @@
       <c r="J30" t="s">
         <v>1635</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7648,7 +7622,7 @@
       <c r="J31" t="s">
         <v>1635</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7666,7 +7640,7 @@
       <c r="R31" t="s">
         <v>1820</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7707,7 +7681,7 @@
       <c r="J32" t="s">
         <v>1635</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7751,7 +7725,7 @@
       <c r="J33" t="s">
         <v>1635</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7769,7 +7743,7 @@
       <c r="R33" t="s">
         <v>1821</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7810,7 +7784,7 @@
       <c r="J34" t="s">
         <v>1635</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7854,7 +7828,7 @@
       <c r="J35" t="s">
         <v>1635</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7872,7 +7846,7 @@
       <c r="R35" t="s">
         <v>1822</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7913,7 +7887,7 @@
       <c r="J36" t="s">
         <v>1635</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7931,7 +7905,7 @@
       <c r="R36" t="s">
         <v>1822</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7972,7 +7946,7 @@
       <c r="J37" t="s">
         <v>1635</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7990,7 +7964,7 @@
       <c r="R37" t="s">
         <v>1822</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8031,7 +8005,7 @@
       <c r="J38" t="s">
         <v>1635</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8049,7 +8023,7 @@
       <c r="R38" t="s">
         <v>1822</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8090,7 +8064,7 @@
       <c r="J39" t="s">
         <v>1635</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8108,7 +8082,7 @@
       <c r="R39" t="s">
         <v>1822</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8149,7 +8123,7 @@
       <c r="J40" t="s">
         <v>1635</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8167,7 +8141,7 @@
       <c r="R40" t="s">
         <v>1823</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8208,7 +8182,7 @@
       <c r="J41" t="s">
         <v>1635</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8226,7 +8200,7 @@
       <c r="R41" t="s">
         <v>1814</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8267,7 +8241,7 @@
       <c r="J42" t="s">
         <v>1635</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8285,7 +8259,7 @@
       <c r="R42" t="s">
         <v>1822</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8326,7 +8300,7 @@
       <c r="J43" t="s">
         <v>1635</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8370,7 +8344,7 @@
       <c r="J44" t="s">
         <v>1635</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8388,7 +8362,7 @@
       <c r="R44" t="s">
         <v>1824</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8429,7 +8403,7 @@
       <c r="J45" t="s">
         <v>1635</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8447,7 +8421,7 @@
       <c r="R45" t="s">
         <v>1825</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8485,7 +8459,7 @@
       <c r="J46" t="s">
         <v>1635</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8529,7 +8503,7 @@
       <c r="J47" t="s">
         <v>1635</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8547,7 +8521,7 @@
       <c r="R47" t="s">
         <v>1826</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8588,7 +8562,7 @@
       <c r="J48" t="s">
         <v>1635</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8632,7 +8606,7 @@
       <c r="J49" t="s">
         <v>1635</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8676,7 +8650,7 @@
       <c r="J50" t="s">
         <v>1635</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8720,7 +8694,7 @@
       <c r="J51" t="s">
         <v>1635</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8767,7 +8741,7 @@
       <c r="J52" t="s">
         <v>1635</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8811,7 +8785,7 @@
       <c r="J53" t="s">
         <v>1635</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8855,7 +8829,7 @@
       <c r="J54" t="s">
         <v>1635</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8899,7 +8873,7 @@
       <c r="J55" t="s">
         <v>1635</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8949,7 +8923,7 @@
       <c r="J56" t="s">
         <v>1635</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -9002,7 +8976,7 @@
       <c r="J57" t="s">
         <v>1635</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9052,7 +9026,7 @@
       <c r="J58" t="s">
         <v>1635</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9102,7 +9076,7 @@
       <c r="J59" t="s">
         <v>1635</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9120,7 +9094,7 @@
       <c r="R59" t="s">
         <v>1827</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9161,7 +9135,7 @@
       <c r="J60" t="s">
         <v>1635</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9205,7 +9179,7 @@
       <c r="J61" t="s">
         <v>1635</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9249,7 +9223,7 @@
       <c r="J62" t="s">
         <v>1635</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9293,7 +9267,7 @@
       <c r="J63" t="s">
         <v>1635</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9337,7 +9311,7 @@
       <c r="J64" t="s">
         <v>1635</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9381,7 +9355,7 @@
       <c r="J65" t="s">
         <v>1635</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9428,7 +9402,7 @@
       <c r="J66" t="s">
         <v>1635</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9446,7 +9420,7 @@
       <c r="R66" t="s">
         <v>1828</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9484,7 +9458,7 @@
       <c r="J67" t="s">
         <v>1635</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9528,7 +9502,7 @@
       <c r="J68" t="s">
         <v>1635</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9543,7 +9517,7 @@
       <c r="O68" t="s">
         <v>1732</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9587,7 +9561,7 @@
       <c r="J69" t="s">
         <v>1637</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9631,7 +9605,7 @@
       <c r="J70" t="s">
         <v>1635</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9675,7 +9649,7 @@
       <c r="J71" t="s">
         <v>1635</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9719,7 +9693,7 @@
       <c r="J72" t="s">
         <v>1635</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9763,7 +9737,7 @@
       <c r="J73" t="s">
         <v>1635</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9807,7 +9781,7 @@
       <c r="J74" t="s">
         <v>1635</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9851,7 +9825,7 @@
       <c r="J75" t="s">
         <v>1635</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9895,7 +9869,7 @@
       <c r="J76" t="s">
         <v>1635</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9913,7 +9887,7 @@
       <c r="R76" t="s">
         <v>1829</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9951,7 +9925,7 @@
       <c r="J77" t="s">
         <v>1635</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9969,7 +9943,7 @@
       <c r="R77" t="s">
         <v>1829</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -10007,7 +9981,7 @@
       <c r="J78" t="s">
         <v>1635</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -10025,7 +9999,7 @@
       <c r="R78" t="s">
         <v>1829</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10063,7 +10037,7 @@
       <c r="J79" t="s">
         <v>1635</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10081,7 +10055,7 @@
       <c r="R79" t="s">
         <v>1829</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10119,7 +10093,7 @@
       <c r="J80" t="s">
         <v>1635</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10163,7 +10137,7 @@
       <c r="J81" t="s">
         <v>1635</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10207,7 +10181,7 @@
       <c r="J82" t="s">
         <v>1635</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10251,7 +10225,7 @@
       <c r="J83" t="s">
         <v>1635</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10295,7 +10269,7 @@
       <c r="J84" t="s">
         <v>1635</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10339,7 +10313,7 @@
       <c r="J85" t="s">
         <v>1635</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10357,7 +10331,7 @@
       <c r="R85" t="s">
         <v>1830</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10395,7 +10369,7 @@
       <c r="J86" t="s">
         <v>1635</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10439,7 +10413,7 @@
       <c r="J87" t="s">
         <v>1635</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10457,7 +10431,7 @@
       <c r="R87" t="s">
         <v>1831</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10495,7 +10469,7 @@
       <c r="J88" t="s">
         <v>1635</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10539,7 +10513,7 @@
       <c r="J89" t="s">
         <v>1635</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10557,7 +10531,7 @@
       <c r="R89" t="s">
         <v>1832</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10592,7 +10566,7 @@
       <c r="J90" t="s">
         <v>1635</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10610,7 +10584,7 @@
       <c r="R90" t="s">
         <v>1833</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10645,7 +10619,7 @@
       <c r="J91" t="s">
         <v>1635</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10663,7 +10637,7 @@
       <c r="R91" t="s">
         <v>1817</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10701,7 +10675,7 @@
       <c r="J92" t="s">
         <v>1635</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10722,7 +10696,7 @@
       <c r="R92" t="s">
         <v>1817</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10763,7 +10737,7 @@
       <c r="J93" t="s">
         <v>1635</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10804,7 +10778,7 @@
       <c r="J94" t="s">
         <v>1635</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10848,7 +10822,7 @@
       <c r="J95" t="s">
         <v>1635</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10892,7 +10866,7 @@
       <c r="J96" t="s">
         <v>1635</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10910,7 +10884,7 @@
       <c r="R96" t="s">
         <v>1834</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10951,7 +10925,7 @@
       <c r="J97" t="s">
         <v>1635</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10966,7 +10940,7 @@
       <c r="R97" t="s">
         <v>1834</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -11007,7 +10981,7 @@
       <c r="J98" t="s">
         <v>1635</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -11025,7 +10999,7 @@
       <c r="R98" t="s">
         <v>1835</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11063,7 +11037,7 @@
       <c r="J99" t="s">
         <v>1635</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11081,7 +11055,7 @@
       <c r="R99" t="s">
         <v>1836</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11119,7 +11093,7 @@
       <c r="J100" t="s">
         <v>1635</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11160,7 +11134,7 @@
       <c r="J101" t="s">
         <v>1635</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11201,7 +11175,7 @@
       <c r="J102" t="s">
         <v>1635</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11242,7 +11216,7 @@
       <c r="J103" t="s">
         <v>1635</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11283,7 +11257,7 @@
       <c r="J104" t="s">
         <v>1635</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11324,7 +11298,7 @@
       <c r="J105" t="s">
         <v>1635</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11365,7 +11339,7 @@
       <c r="J106" t="s">
         <v>1635</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11406,7 +11380,7 @@
       <c r="J107" t="s">
         <v>1635</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11447,7 +11421,7 @@
       <c r="J108" t="s">
         <v>1635</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11488,7 +11462,7 @@
       <c r="J109" t="s">
         <v>1635</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11541,7 +11515,7 @@
       <c r="J110" t="s">
         <v>1635</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11597,7 +11571,7 @@
       <c r="J111" t="s">
         <v>1635</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11615,7 +11589,7 @@
       <c r="R111" t="s">
         <v>1838</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11653,7 +11627,7 @@
       <c r="J112" t="s">
         <v>1635</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11712,7 +11686,7 @@
       <c r="J113" t="s">
         <v>1635</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11756,7 +11730,7 @@
       <c r="J114" t="s">
         <v>1635</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11800,7 +11774,7 @@
       <c r="J115" t="s">
         <v>1635</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11818,7 +11792,7 @@
       <c r="R115" t="s">
         <v>1840</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11859,7 +11833,7 @@
       <c r="J116" t="s">
         <v>1635</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11918,7 +11892,7 @@
       <c r="J117" t="s">
         <v>1635</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11962,7 +11936,7 @@
       <c r="J118" t="s">
         <v>1635</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -12009,7 +11983,7 @@
       <c r="J119" t="s">
         <v>1635</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12050,7 +12024,7 @@
       <c r="J120" t="s">
         <v>1635</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12094,7 +12068,7 @@
       <c r="J121" t="s">
         <v>1635</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12141,7 +12115,7 @@
       <c r="J122" t="s">
         <v>1635</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12191,7 +12165,7 @@
       <c r="J123" t="s">
         <v>1635</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12235,7 +12209,7 @@
       <c r="J124" t="s">
         <v>1635</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12279,7 +12253,7 @@
       <c r="J125" t="s">
         <v>1635</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12297,7 +12271,7 @@
       <c r="R125" t="s">
         <v>1842</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12332,7 +12306,7 @@
       <c r="J126" t="s">
         <v>1635</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12350,7 +12324,7 @@
       <c r="R126" t="s">
         <v>1843</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12388,7 +12362,7 @@
       <c r="J127" t="s">
         <v>1635</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12444,7 +12418,7 @@
       <c r="J128" t="s">
         <v>1635</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12485,7 +12459,7 @@
       <c r="J129" t="s">
         <v>1635</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12526,7 +12500,7 @@
       <c r="J130" t="s">
         <v>1635</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12567,7 +12541,7 @@
       <c r="J131" t="s">
         <v>1635</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12611,7 +12585,7 @@
       <c r="J132" t="s">
         <v>1635</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12652,7 +12626,7 @@
       <c r="J133" t="s">
         <v>1635</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12670,7 +12644,7 @@
       <c r="R133" t="s">
         <v>1829</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12708,7 +12682,7 @@
       <c r="J134" t="s">
         <v>1635</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12726,7 +12700,7 @@
       <c r="R134" t="s">
         <v>1829</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12761,7 +12735,7 @@
       <c r="J135" t="s">
         <v>1635</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12802,7 +12776,7 @@
       <c r="J136" t="s">
         <v>1635</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12843,7 +12817,7 @@
       <c r="J137" t="s">
         <v>1635</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12884,7 +12858,7 @@
       <c r="J138" t="s">
         <v>1635</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12925,7 +12899,7 @@
       <c r="J139" t="s">
         <v>1635</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12972,7 +12946,7 @@
       <c r="J140" t="s">
         <v>1635</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -13013,7 +12987,7 @@
       <c r="J141" t="s">
         <v>1635</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13054,7 +13028,7 @@
       <c r="J142" t="s">
         <v>1635</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13098,7 +13072,7 @@
       <c r="J143" t="s">
         <v>1635</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13116,7 +13090,7 @@
       <c r="R143" t="s">
         <v>1829</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13151,7 +13125,7 @@
       <c r="J144" t="s">
         <v>1635</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13169,7 +13143,7 @@
       <c r="R144" t="s">
         <v>1829</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13207,7 +13181,7 @@
       <c r="J145" t="s">
         <v>1635</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13225,7 +13199,7 @@
       <c r="R145" t="s">
         <v>1829</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13260,7 +13234,7 @@
       <c r="J146" t="s">
         <v>1635</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13278,7 +13252,7 @@
       <c r="R146" t="s">
         <v>1837</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13313,7 +13287,7 @@
       <c r="J147" t="s">
         <v>1635</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13331,7 +13305,7 @@
       <c r="R147" t="s">
         <v>1844</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13366,7 +13340,7 @@
       <c r="J148" t="s">
         <v>1635</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13407,7 +13381,7 @@
       <c r="J149" t="s">
         <v>1635</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13425,7 +13399,7 @@
       <c r="R149" t="s">
         <v>1829</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13460,7 +13434,7 @@
       <c r="J150" t="s">
         <v>1635</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13478,7 +13452,7 @@
       <c r="R150" t="s">
         <v>1829</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13516,7 +13490,7 @@
       <c r="J151" t="s">
         <v>1635</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13534,7 +13508,7 @@
       <c r="R151" t="s">
         <v>1845</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13569,7 +13543,7 @@
       <c r="J152" t="s">
         <v>1635</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13587,7 +13561,7 @@
       <c r="R152" t="s">
         <v>1846</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13622,7 +13596,7 @@
       <c r="J153" t="s">
         <v>1635</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13631,7 +13605,7 @@
       <c r="M153" t="s">
         <v>1723</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13672,7 +13646,7 @@
       <c r="J154" t="s">
         <v>1635</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13713,7 +13687,7 @@
       <c r="J155" t="s">
         <v>1635</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13754,7 +13728,7 @@
       <c r="J156" t="s">
         <v>1635</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13795,7 +13769,7 @@
       <c r="J157" t="s">
         <v>1635</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13836,7 +13810,7 @@
       <c r="J158" t="s">
         <v>1635</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13877,7 +13851,7 @@
       <c r="J159" t="s">
         <v>1635</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13918,7 +13892,7 @@
       <c r="J160" t="s">
         <v>1635</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13959,7 +13933,7 @@
       <c r="J161" t="s">
         <v>1635</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -14000,7 +13974,7 @@
       <c r="J162" t="s">
         <v>1635</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -14018,7 +13992,7 @@
       <c r="R162" t="s">
         <v>1832</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14053,7 +14027,7 @@
       <c r="J163" t="s">
         <v>1635</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14071,7 +14045,7 @@
       <c r="R163" t="s">
         <v>1829</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14106,7 +14080,7 @@
       <c r="J164" t="s">
         <v>1635</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14150,7 +14124,7 @@
       <c r="J165" t="s">
         <v>1635</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14191,7 +14165,7 @@
       <c r="J166" t="s">
         <v>1635</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14209,7 +14183,7 @@
       <c r="R166" t="s">
         <v>1847</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14244,7 +14218,7 @@
       <c r="J167" t="s">
         <v>1635</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14288,7 +14262,7 @@
       <c r="J168" t="s">
         <v>1635</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14332,7 +14306,7 @@
       <c r="J169" t="s">
         <v>1635</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14373,7 +14347,7 @@
       <c r="J170" t="s">
         <v>1635</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14414,7 +14388,7 @@
       <c r="J171" t="s">
         <v>1635</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14455,7 +14429,7 @@
       <c r="J172" t="s">
         <v>1635</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14496,7 +14470,7 @@
       <c r="J173" t="s">
         <v>1635</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14537,7 +14511,7 @@
       <c r="J174" t="s">
         <v>1635</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14578,7 +14552,7 @@
       <c r="J175" t="s">
         <v>1635</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14619,7 +14593,7 @@
       <c r="J176" t="s">
         <v>1635</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14660,7 +14634,7 @@
       <c r="J177" t="s">
         <v>1635</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14701,7 +14675,7 @@
       <c r="J178" t="s">
         <v>1635</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14719,7 +14693,7 @@
       <c r="R178" t="s">
         <v>1845</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14757,7 +14731,7 @@
       <c r="J179" t="s">
         <v>1635</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14766,7 +14740,7 @@
       <c r="M179" t="s">
         <v>1720</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14807,7 +14781,7 @@
       <c r="J180" t="s">
         <v>1635</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14848,7 +14822,7 @@
       <c r="J181" t="s">
         <v>1635</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14866,7 +14840,7 @@
       <c r="R181" t="s">
         <v>1829</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14901,7 +14875,7 @@
       <c r="J182" t="s">
         <v>1635</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14942,7 +14916,7 @@
       <c r="J183" t="s">
         <v>1635</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14983,7 +14957,7 @@
       <c r="J184" t="s">
         <v>1635</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -15024,7 +14998,7 @@
       <c r="J185" t="s">
         <v>1635</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15065,7 +15039,7 @@
       <c r="J186" t="s">
         <v>1635</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15106,7 +15080,7 @@
       <c r="J187" t="s">
         <v>1635</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15147,7 +15121,7 @@
       <c r="J188" t="s">
         <v>1635</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15188,7 +15162,7 @@
       <c r="J189" t="s">
         <v>1635</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15229,7 +15203,7 @@
       <c r="J190" t="s">
         <v>1635</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15270,7 +15244,7 @@
       <c r="J191" t="s">
         <v>1635</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15311,7 +15285,7 @@
       <c r="J192" t="s">
         <v>1635</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15352,7 +15326,7 @@
       <c r="J193" t="s">
         <v>1635</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15393,7 +15367,7 @@
       <c r="J194" t="s">
         <v>1635</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15434,7 +15408,7 @@
       <c r="J195" t="s">
         <v>1635</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15452,7 +15426,7 @@
       <c r="R195" t="s">
         <v>1838</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15493,7 +15467,7 @@
       <c r="J196" t="s">
         <v>1635</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15511,7 +15485,7 @@
       <c r="R196" t="s">
         <v>1844</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15549,7 +15523,7 @@
       <c r="J197" t="s">
         <v>1635</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15590,7 +15564,7 @@
       <c r="J198" t="s">
         <v>1637</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15631,7 +15605,7 @@
       <c r="J199" t="s">
         <v>1636</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15672,7 +15646,7 @@
       <c r="J200" t="s">
         <v>1635</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15713,7 +15687,7 @@
       <c r="J201" t="s">
         <v>1635</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15754,7 +15728,7 @@
       <c r="J202" t="s">
         <v>1635</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15772,7 +15746,7 @@
       <c r="R202" t="s">
         <v>1829</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15810,7 +15784,7 @@
       <c r="J203" t="s">
         <v>1635</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15828,7 +15802,7 @@
       <c r="R203" t="s">
         <v>1837</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15863,7 +15837,7 @@
       <c r="J204" t="s">
         <v>1635</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15878,7 +15852,7 @@
       <c r="R204" t="s">
         <v>1848</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15916,7 +15890,7 @@
       <c r="J205" t="s">
         <v>1635</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15934,7 +15908,7 @@
       <c r="R205" t="s">
         <v>1849</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15972,7 +15946,7 @@
       <c r="J206" t="s">
         <v>1635</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15990,7 +15964,7 @@
       <c r="R206" t="s">
         <v>1817</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -16025,7 +15999,7 @@
       <c r="J207" t="s">
         <v>1635</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16066,7 +16040,7 @@
       <c r="J208" t="s">
         <v>1635</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16107,7 +16081,7 @@
       <c r="J209" t="s">
         <v>1635</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16148,7 +16122,7 @@
       <c r="J210" t="s">
         <v>1635</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16189,7 +16163,7 @@
       <c r="J211" t="s">
         <v>1635</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16230,7 +16204,7 @@
       <c r="J212" t="s">
         <v>1635</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16271,7 +16245,7 @@
       <c r="J213" t="s">
         <v>1635</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16312,7 +16286,7 @@
       <c r="J214" t="s">
         <v>1635</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16330,7 +16304,7 @@
       <c r="R214" t="s">
         <v>1850</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16368,7 +16342,7 @@
       <c r="J215" t="s">
         <v>1635</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16409,7 +16383,7 @@
       <c r="J216" t="s">
         <v>1635</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16450,7 +16424,7 @@
       <c r="J217" t="s">
         <v>1635</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16491,7 +16465,7 @@
       <c r="J218" t="s">
         <v>1635</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16532,7 +16506,7 @@
       <c r="J219" t="s">
         <v>1635</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16573,7 +16547,7 @@
       <c r="J220" t="s">
         <v>1635</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16614,7 +16588,7 @@
       <c r="J221" t="s">
         <v>1635</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16655,7 +16629,7 @@
       <c r="J222" t="s">
         <v>1635</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16696,7 +16670,7 @@
       <c r="J223" t="s">
         <v>1635</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16737,7 +16711,7 @@
       <c r="J224" t="s">
         <v>1635</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16778,7 +16752,7 @@
       <c r="J225" t="s">
         <v>1635</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16819,7 +16793,7 @@
       <c r="J226" t="s">
         <v>1635</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16860,7 +16834,7 @@
       <c r="J227" t="s">
         <v>1635</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16901,7 +16875,7 @@
       <c r="J228" t="s">
         <v>1635</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16942,7 +16916,7 @@
       <c r="J229" t="s">
         <v>1635</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16983,7 +16957,7 @@
       <c r="J230" t="s">
         <v>1635</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -17024,7 +16998,7 @@
       <c r="J231" t="s">
         <v>1635</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17065,7 +17039,7 @@
       <c r="J232" t="s">
         <v>1635</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17106,7 +17080,7 @@
       <c r="J233" t="s">
         <v>1635</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17147,7 +17121,7 @@
       <c r="J234" t="s">
         <v>1635</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17188,7 +17162,7 @@
       <c r="J235" t="s">
         <v>1635</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17229,7 +17203,7 @@
       <c r="J236" t="s">
         <v>1635</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17270,7 +17244,7 @@
       <c r="J237" t="s">
         <v>1635</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17311,7 +17285,7 @@
       <c r="J238" t="s">
         <v>1635</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17352,7 +17326,7 @@
       <c r="J239" t="s">
         <v>1635</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17370,7 +17344,7 @@
       <c r="R239" t="s">
         <v>1844</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17408,7 +17382,7 @@
       <c r="J240" t="s">
         <v>1635</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17449,7 +17423,7 @@
       <c r="J241" t="s">
         <v>1635</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17490,7 +17464,7 @@
       <c r="J242" t="s">
         <v>1635</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17508,7 +17482,7 @@
       <c r="R242" t="s">
         <v>1837</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17543,7 +17517,7 @@
       <c r="J243" t="s">
         <v>1635</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17584,7 +17558,7 @@
       <c r="J244" t="s">
         <v>1635</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17625,7 +17599,7 @@
       <c r="J245" t="s">
         <v>1635</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17666,7 +17640,7 @@
       <c r="J246" t="s">
         <v>1635</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17684,7 +17658,7 @@
       <c r="R246" t="s">
         <v>1817</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17722,7 +17696,7 @@
       <c r="J247" t="s">
         <v>1635</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17763,7 +17737,7 @@
       <c r="J248" t="s">
         <v>1635</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17804,7 +17778,7 @@
       <c r="J249" t="s">
         <v>1635</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17845,7 +17819,7 @@
       <c r="J250" t="s">
         <v>1635</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17886,7 +17860,7 @@
       <c r="J251" t="s">
         <v>1635</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17927,7 +17901,7 @@
       <c r="J252" t="s">
         <v>1635</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17968,7 +17942,7 @@
       <c r="J253" t="s">
         <v>1635</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17986,7 +17960,7 @@
       <c r="R253" t="s">
         <v>1847</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18027,7 +18001,7 @@
       <c r="J254" t="s">
         <v>1635</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18068,7 +18042,7 @@
       <c r="J255" t="s">
         <v>1635</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18109,7 +18083,7 @@
       <c r="J256" t="s">
         <v>1635</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18118,7 +18092,7 @@
       <c r="M256" t="s">
         <v>1719</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18156,7 +18130,7 @@
       <c r="J257" t="s">
         <v>1635</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18165,7 +18139,7 @@
       <c r="M257" t="s">
         <v>1720</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18209,7 +18183,7 @@
       <c r="J258" t="s">
         <v>1635</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18227,7 +18201,7 @@
       <c r="R258" t="s">
         <v>1829</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18265,7 +18239,7 @@
       <c r="J259" t="s">
         <v>1635</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18283,7 +18257,7 @@
       <c r="R259" t="s">
         <v>1845</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18321,7 +18295,7 @@
       <c r="J260" t="s">
         <v>1635</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18330,7 +18304,7 @@
       <c r="M260" t="s">
         <v>1714</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18374,7 +18348,7 @@
       <c r="J261" t="s">
         <v>1635</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18392,7 +18366,7 @@
       <c r="R261" t="s">
         <v>1851</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18430,7 +18404,7 @@
       <c r="J262" t="s">
         <v>1635</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18448,7 +18422,7 @@
       <c r="R262" t="s">
         <v>1845</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18486,7 +18460,7 @@
       <c r="J263" t="s">
         <v>1635</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18495,7 +18469,7 @@
       <c r="M263" t="s">
         <v>1714</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18539,7 +18513,7 @@
       <c r="J264" t="s">
         <v>1635</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18580,7 +18554,7 @@
       <c r="J265" t="s">
         <v>1635</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18621,7 +18595,7 @@
       <c r="J266" t="s">
         <v>1635</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18662,7 +18636,7 @@
       <c r="J267" t="s">
         <v>1635</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18706,7 +18680,7 @@
       <c r="J268" t="s">
         <v>1635</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18747,7 +18721,7 @@
       <c r="J269" t="s">
         <v>1635</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18788,7 +18762,7 @@
       <c r="J270" t="s">
         <v>1635</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18829,7 +18803,7 @@
       <c r="J271" t="s">
         <v>1635</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18870,7 +18844,7 @@
       <c r="J272" t="s">
         <v>1635</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18888,7 +18862,7 @@
       <c r="R272" t="s">
         <v>1852</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18929,7 +18903,7 @@
       <c r="J273" t="s">
         <v>1635</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18973,7 +18947,7 @@
       <c r="J274" t="s">
         <v>1635</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -19014,7 +18988,7 @@
       <c r="J275" t="s">
         <v>1635</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19055,7 +19029,7 @@
       <c r="J276" t="s">
         <v>1635</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19096,7 +19070,7 @@
       <c r="J277" t="s">
         <v>1635</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19137,7 +19111,7 @@
       <c r="J278" t="s">
         <v>1635</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19178,7 +19152,7 @@
       <c r="J279" t="s">
         <v>1635</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19219,7 +19193,7 @@
       <c r="J280" t="s">
         <v>1635</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19260,7 +19234,7 @@
       <c r="J281" t="s">
         <v>1635</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19301,7 +19275,7 @@
       <c r="J282" t="s">
         <v>1635</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19342,7 +19316,7 @@
       <c r="J283" t="s">
         <v>1635</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19383,7 +19357,7 @@
       <c r="J284" t="s">
         <v>1635</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19424,7 +19398,7 @@
       <c r="J285" t="s">
         <v>1635</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19465,7 +19439,7 @@
       <c r="J286" t="s">
         <v>1635</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19506,7 +19480,7 @@
       <c r="J287" t="s">
         <v>1635</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19547,7 +19521,7 @@
       <c r="J288" t="s">
         <v>1635</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19588,7 +19562,7 @@
       <c r="J289" t="s">
         <v>1635</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19629,7 +19603,7 @@
       <c r="J290" t="s">
         <v>1635</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19670,7 +19644,7 @@
       <c r="J291" t="s">
         <v>1635</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19711,7 +19685,7 @@
       <c r="J292" t="s">
         <v>1635</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19752,7 +19726,7 @@
       <c r="J293" t="s">
         <v>1635</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19793,7 +19767,7 @@
       <c r="J294" t="s">
         <v>1635</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19834,7 +19808,7 @@
       <c r="J295" t="s">
         <v>1635</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19852,7 +19826,7 @@
       <c r="R295" t="s">
         <v>1853</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19893,7 +19867,7 @@
       <c r="J296" t="s">
         <v>1635</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19911,7 +19885,7 @@
       <c r="R296" t="s">
         <v>1829</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19949,7 +19923,7 @@
       <c r="J297" t="s">
         <v>1635</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19990,7 +19964,7 @@
       <c r="J298" t="s">
         <v>1635</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20031,7 +20005,7 @@
       <c r="J299" t="s">
         <v>1636</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20072,7 +20046,7 @@
       <c r="J300" t="s">
         <v>1635</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20113,7 +20087,7 @@
       <c r="J301" t="s">
         <v>1635</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20951,7 +20925,7 @@
       <c r="R321" t="s">
         <v>1815</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21174,7 +21148,7 @@
       <c r="R326" t="s">
         <v>1854</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -22009,7 +21983,7 @@
       <c r="R346" t="s">
         <v>1855</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (21/10/2026 14:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5813,8 +5813,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5830,7 +5838,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5838,12 +5846,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6143,73 +6169,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6244,7 +6270,7 @@
       <c r="J2" t="s">
         <v>1654</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6288,7 +6314,7 @@
       <c r="J3" t="s">
         <v>1654</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6332,7 +6358,7 @@
       <c r="J4" t="s">
         <v>1654</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6350,7 +6376,7 @@
       <c r="R4" t="s">
         <v>1832</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6388,7 +6414,7 @@
       <c r="J5" t="s">
         <v>1655</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6438,7 +6464,7 @@
       <c r="J6" t="s">
         <v>1654</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6485,7 +6511,7 @@
       <c r="J7" t="s">
         <v>1654</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6532,7 +6558,7 @@
       <c r="J8" t="s">
         <v>1654</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6579,7 +6605,7 @@
       <c r="J9" t="s">
         <v>1654</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6626,7 +6652,7 @@
       <c r="J10" t="s">
         <v>1654</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6673,7 +6699,7 @@
       <c r="J11" t="s">
         <v>1654</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6720,7 +6746,7 @@
       <c r="J12" t="s">
         <v>1654</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6764,7 +6790,7 @@
       <c r="J13" t="s">
         <v>1654</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6782,7 +6808,7 @@
       <c r="R13" t="s">
         <v>1833</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6820,7 +6846,7 @@
       <c r="J14" t="s">
         <v>1654</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6838,7 +6864,7 @@
       <c r="R14" t="s">
         <v>1834</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6879,7 +6905,7 @@
       <c r="J15" t="s">
         <v>1654</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6897,7 +6923,7 @@
       <c r="R15" t="s">
         <v>1834</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6938,7 +6964,7 @@
       <c r="J16" t="s">
         <v>1654</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6982,7 +7008,7 @@
       <c r="J17" t="s">
         <v>1654</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -7026,7 +7052,7 @@
       <c r="J18" t="s">
         <v>1654</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -7044,7 +7070,7 @@
       <c r="R18" t="s">
         <v>1835</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7085,7 +7111,7 @@
       <c r="J19" t="s">
         <v>1654</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7129,7 +7155,7 @@
       <c r="J20" t="s">
         <v>1654</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7173,7 +7199,7 @@
       <c r="J21" t="s">
         <v>1654</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7191,7 +7217,7 @@
       <c r="R21" t="s">
         <v>1834</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7232,7 +7258,7 @@
       <c r="J22" t="s">
         <v>1654</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7250,7 +7276,7 @@
       <c r="R22" t="s">
         <v>1836</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7291,7 +7317,7 @@
       <c r="J23" t="s">
         <v>1654</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7309,7 +7335,7 @@
       <c r="R23" t="s">
         <v>1837</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7350,7 +7376,7 @@
       <c r="J24" t="s">
         <v>1654</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7394,7 +7420,7 @@
       <c r="J25" t="s">
         <v>1654</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7435,7 +7461,7 @@
       <c r="J26" t="s">
         <v>1656</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7453,7 +7479,7 @@
       <c r="R26" t="s">
         <v>1838</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7491,7 +7517,7 @@
       <c r="J27" t="s">
         <v>1654</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7509,7 +7535,7 @@
       <c r="R27" t="s">
         <v>1839</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7550,7 +7576,7 @@
       <c r="J28" t="s">
         <v>1654</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7594,7 +7620,7 @@
       <c r="J29" t="s">
         <v>1654</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7638,7 +7664,7 @@
       <c r="J30" t="s">
         <v>1654</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7682,7 +7708,7 @@
       <c r="J31" t="s">
         <v>1654</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7700,7 +7726,7 @@
       <c r="R31" t="s">
         <v>1840</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7741,7 +7767,7 @@
       <c r="J32" t="s">
         <v>1654</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7785,7 +7811,7 @@
       <c r="J33" t="s">
         <v>1654</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7803,7 +7829,7 @@
       <c r="R33" t="s">
         <v>1841</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7844,7 +7870,7 @@
       <c r="J34" t="s">
         <v>1654</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7888,7 +7914,7 @@
       <c r="J35" t="s">
         <v>1654</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7906,7 +7932,7 @@
       <c r="R35" t="s">
         <v>1842</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7947,7 +7973,7 @@
       <c r="J36" t="s">
         <v>1654</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7965,7 +7991,7 @@
       <c r="R36" t="s">
         <v>1842</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -8006,7 +8032,7 @@
       <c r="J37" t="s">
         <v>1654</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -8024,7 +8050,7 @@
       <c r="R37" t="s">
         <v>1842</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8065,7 +8091,7 @@
       <c r="J38" t="s">
         <v>1654</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8083,7 +8109,7 @@
       <c r="R38" t="s">
         <v>1842</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8124,7 +8150,7 @@
       <c r="J39" t="s">
         <v>1654</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8142,7 +8168,7 @@
       <c r="R39" t="s">
         <v>1842</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8183,7 +8209,7 @@
       <c r="J40" t="s">
         <v>1654</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8201,7 +8227,7 @@
       <c r="R40" t="s">
         <v>1843</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8242,7 +8268,7 @@
       <c r="J41" t="s">
         <v>1654</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8260,7 +8286,7 @@
       <c r="R41" t="s">
         <v>1834</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8301,7 +8327,7 @@
       <c r="J42" t="s">
         <v>1654</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8319,7 +8345,7 @@
       <c r="R42" t="s">
         <v>1842</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8360,7 +8386,7 @@
       <c r="J43" t="s">
         <v>1654</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8404,7 +8430,7 @@
       <c r="J44" t="s">
         <v>1654</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8422,7 +8448,7 @@
       <c r="R44" t="s">
         <v>1844</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8463,7 +8489,7 @@
       <c r="J45" t="s">
         <v>1654</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8481,7 +8507,7 @@
       <c r="R45" t="s">
         <v>1845</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8519,7 +8545,7 @@
       <c r="J46" t="s">
         <v>1654</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8563,7 +8589,7 @@
       <c r="J47" t="s">
         <v>1654</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8581,7 +8607,7 @@
       <c r="R47" t="s">
         <v>1846</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8622,7 +8648,7 @@
       <c r="J48" t="s">
         <v>1654</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8666,7 +8692,7 @@
       <c r="J49" t="s">
         <v>1654</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8710,7 +8736,7 @@
       <c r="J50" t="s">
         <v>1654</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8754,7 +8780,7 @@
       <c r="J51" t="s">
         <v>1654</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8801,7 +8827,7 @@
       <c r="J52" t="s">
         <v>1654</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8845,7 +8871,7 @@
       <c r="J53" t="s">
         <v>1654</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8889,7 +8915,7 @@
       <c r="J54" t="s">
         <v>1654</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8933,7 +8959,7 @@
       <c r="J55" t="s">
         <v>1654</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8983,7 +9009,7 @@
       <c r="J56" t="s">
         <v>1654</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -9036,7 +9062,7 @@
       <c r="J57" t="s">
         <v>1654</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9086,7 +9112,7 @@
       <c r="J58" t="s">
         <v>1654</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9136,7 +9162,7 @@
       <c r="J59" t="s">
         <v>1654</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9154,7 +9180,7 @@
       <c r="R59" t="s">
         <v>1847</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9195,7 +9221,7 @@
       <c r="J60" t="s">
         <v>1654</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9239,7 +9265,7 @@
       <c r="J61" t="s">
         <v>1654</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9283,7 +9309,7 @@
       <c r="J62" t="s">
         <v>1654</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9327,7 +9353,7 @@
       <c r="J63" t="s">
         <v>1654</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9371,7 +9397,7 @@
       <c r="J64" t="s">
         <v>1654</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9415,7 +9441,7 @@
       <c r="J65" t="s">
         <v>1654</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9462,7 +9488,7 @@
       <c r="J66" t="s">
         <v>1654</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9480,7 +9506,7 @@
       <c r="R66" t="s">
         <v>1848</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9518,7 +9544,7 @@
       <c r="J67" t="s">
         <v>1654</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9562,7 +9588,7 @@
       <c r="J68" t="s">
         <v>1654</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9577,7 +9603,7 @@
       <c r="O68" t="s">
         <v>1752</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9621,7 +9647,7 @@
       <c r="J69" t="s">
         <v>1656</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9665,7 +9691,7 @@
       <c r="J70" t="s">
         <v>1654</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9709,7 +9735,7 @@
       <c r="J71" t="s">
         <v>1654</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9753,7 +9779,7 @@
       <c r="J72" t="s">
         <v>1654</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9797,7 +9823,7 @@
       <c r="J73" t="s">
         <v>1654</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9841,7 +9867,7 @@
       <c r="J74" t="s">
         <v>1654</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9885,7 +9911,7 @@
       <c r="J75" t="s">
         <v>1654</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9929,7 +9955,7 @@
       <c r="J76" t="s">
         <v>1654</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9947,7 +9973,7 @@
       <c r="R76" t="s">
         <v>1849</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9985,7 +10011,7 @@
       <c r="J77" t="s">
         <v>1654</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -10003,7 +10029,7 @@
       <c r="R77" t="s">
         <v>1849</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -10041,7 +10067,7 @@
       <c r="J78" t="s">
         <v>1654</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -10059,7 +10085,7 @@
       <c r="R78" t="s">
         <v>1849</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10097,7 +10123,7 @@
       <c r="J79" t="s">
         <v>1654</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10115,7 +10141,7 @@
       <c r="R79" t="s">
         <v>1849</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10153,7 +10179,7 @@
       <c r="J80" t="s">
         <v>1654</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10197,7 +10223,7 @@
       <c r="J81" t="s">
         <v>1654</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10241,7 +10267,7 @@
       <c r="J82" t="s">
         <v>1654</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10285,7 +10311,7 @@
       <c r="J83" t="s">
         <v>1654</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10329,7 +10355,7 @@
       <c r="J84" t="s">
         <v>1654</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10373,7 +10399,7 @@
       <c r="J85" t="s">
         <v>1654</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10391,7 +10417,7 @@
       <c r="R85" t="s">
         <v>1850</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10429,7 +10455,7 @@
       <c r="J86" t="s">
         <v>1654</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10473,7 +10499,7 @@
       <c r="J87" t="s">
         <v>1654</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10491,7 +10517,7 @@
       <c r="R87" t="s">
         <v>1851</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10529,7 +10555,7 @@
       <c r="J88" t="s">
         <v>1654</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10573,7 +10599,7 @@
       <c r="J89" t="s">
         <v>1654</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10591,7 +10617,7 @@
       <c r="R89" t="s">
         <v>1852</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10626,7 +10652,7 @@
       <c r="J90" t="s">
         <v>1654</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10644,7 +10670,7 @@
       <c r="R90" t="s">
         <v>1853</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10679,7 +10705,7 @@
       <c r="J91" t="s">
         <v>1654</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10697,7 +10723,7 @@
       <c r="R91" t="s">
         <v>1837</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10735,7 +10761,7 @@
       <c r="J92" t="s">
         <v>1654</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10756,7 +10782,7 @@
       <c r="R92" t="s">
         <v>1837</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10797,7 +10823,7 @@
       <c r="J93" t="s">
         <v>1654</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10838,7 +10864,7 @@
       <c r="J94" t="s">
         <v>1654</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10882,7 +10908,7 @@
       <c r="J95" t="s">
         <v>1654</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10926,7 +10952,7 @@
       <c r="J96" t="s">
         <v>1654</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10944,7 +10970,7 @@
       <c r="R96" t="s">
         <v>1854</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -10985,7 +11011,7 @@
       <c r="J97" t="s">
         <v>1654</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -11000,7 +11026,7 @@
       <c r="R97" t="s">
         <v>1854</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -11041,7 +11067,7 @@
       <c r="J98" t="s">
         <v>1654</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -11059,7 +11085,7 @@
       <c r="R98" t="s">
         <v>1855</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11097,7 +11123,7 @@
       <c r="J99" t="s">
         <v>1654</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11115,7 +11141,7 @@
       <c r="R99" t="s">
         <v>1856</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11153,7 +11179,7 @@
       <c r="J100" t="s">
         <v>1654</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11194,7 +11220,7 @@
       <c r="J101" t="s">
         <v>1654</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11235,7 +11261,7 @@
       <c r="J102" t="s">
         <v>1654</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11276,7 +11302,7 @@
       <c r="J103" t="s">
         <v>1654</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11317,7 +11343,7 @@
       <c r="J104" t="s">
         <v>1654</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11358,7 +11384,7 @@
       <c r="J105" t="s">
         <v>1654</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11399,7 +11425,7 @@
       <c r="J106" t="s">
         <v>1654</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11440,7 +11466,7 @@
       <c r="J107" t="s">
         <v>1654</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11481,7 +11507,7 @@
       <c r="J108" t="s">
         <v>1654</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11522,7 +11548,7 @@
       <c r="J109" t="s">
         <v>1654</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11575,7 +11601,7 @@
       <c r="J110" t="s">
         <v>1654</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11631,7 +11657,7 @@
       <c r="J111" t="s">
         <v>1654</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11649,7 +11675,7 @@
       <c r="R111" t="s">
         <v>1858</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11687,7 +11713,7 @@
       <c r="J112" t="s">
         <v>1654</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11746,7 +11772,7 @@
       <c r="J113" t="s">
         <v>1654</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11790,7 +11816,7 @@
       <c r="J114" t="s">
         <v>1654</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11834,7 +11860,7 @@
       <c r="J115" t="s">
         <v>1654</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11852,7 +11878,7 @@
       <c r="R115" t="s">
         <v>1860</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11893,7 +11919,7 @@
       <c r="J116" t="s">
         <v>1654</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11952,7 +11978,7 @@
       <c r="J117" t="s">
         <v>1654</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11996,7 +12022,7 @@
       <c r="J118" t="s">
         <v>1654</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -12043,7 +12069,7 @@
       <c r="J119" t="s">
         <v>1654</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12084,7 +12110,7 @@
       <c r="J120" t="s">
         <v>1654</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12128,7 +12154,7 @@
       <c r="J121" t="s">
         <v>1654</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12175,7 +12201,7 @@
       <c r="J122" t="s">
         <v>1654</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12225,7 +12251,7 @@
       <c r="J123" t="s">
         <v>1654</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12269,7 +12295,7 @@
       <c r="J124" t="s">
         <v>1654</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12313,7 +12339,7 @@
       <c r="J125" t="s">
         <v>1654</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12331,7 +12357,7 @@
       <c r="R125" t="s">
         <v>1862</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12366,7 +12392,7 @@
       <c r="J126" t="s">
         <v>1654</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12384,7 +12410,7 @@
       <c r="R126" t="s">
         <v>1863</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12422,7 +12448,7 @@
       <c r="J127" t="s">
         <v>1654</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12478,7 +12504,7 @@
       <c r="J128" t="s">
         <v>1654</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12519,7 +12545,7 @@
       <c r="J129" t="s">
         <v>1654</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12560,7 +12586,7 @@
       <c r="J130" t="s">
         <v>1654</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12601,7 +12627,7 @@
       <c r="J131" t="s">
         <v>1654</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12645,7 +12671,7 @@
       <c r="J132" t="s">
         <v>1654</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12686,7 +12712,7 @@
       <c r="J133" t="s">
         <v>1654</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12704,7 +12730,7 @@
       <c r="R133" t="s">
         <v>1849</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12742,7 +12768,7 @@
       <c r="J134" t="s">
         <v>1654</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12760,7 +12786,7 @@
       <c r="R134" t="s">
         <v>1849</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12795,7 +12821,7 @@
       <c r="J135" t="s">
         <v>1654</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12836,7 +12862,7 @@
       <c r="J136" t="s">
         <v>1654</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12877,7 +12903,7 @@
       <c r="J137" t="s">
         <v>1654</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12918,7 +12944,7 @@
       <c r="J138" t="s">
         <v>1654</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12959,7 +12985,7 @@
       <c r="J139" t="s">
         <v>1654</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -13006,7 +13032,7 @@
       <c r="J140" t="s">
         <v>1654</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -13047,7 +13073,7 @@
       <c r="J141" t="s">
         <v>1654</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13088,7 +13114,7 @@
       <c r="J142" t="s">
         <v>1654</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13132,7 +13158,7 @@
       <c r="J143" t="s">
         <v>1654</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13150,7 +13176,7 @@
       <c r="R143" t="s">
         <v>1849</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13185,7 +13211,7 @@
       <c r="J144" t="s">
         <v>1654</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13203,7 +13229,7 @@
       <c r="R144" t="s">
         <v>1849</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13241,7 +13267,7 @@
       <c r="J145" t="s">
         <v>1654</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13259,7 +13285,7 @@
       <c r="R145" t="s">
         <v>1849</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13294,7 +13320,7 @@
       <c r="J146" t="s">
         <v>1654</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13312,7 +13338,7 @@
       <c r="R146" t="s">
         <v>1857</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13347,7 +13373,7 @@
       <c r="J147" t="s">
         <v>1654</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13365,7 +13391,7 @@
       <c r="R147" t="s">
         <v>1864</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13400,7 +13426,7 @@
       <c r="J148" t="s">
         <v>1654</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13441,7 +13467,7 @@
       <c r="J149" t="s">
         <v>1654</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13459,7 +13485,7 @@
       <c r="R149" t="s">
         <v>1849</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13494,7 +13520,7 @@
       <c r="J150" t="s">
         <v>1654</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13512,7 +13538,7 @@
       <c r="R150" t="s">
         <v>1849</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13550,7 +13576,7 @@
       <c r="J151" t="s">
         <v>1654</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13568,7 +13594,7 @@
       <c r="R151" t="s">
         <v>1865</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13603,7 +13629,7 @@
       <c r="J152" t="s">
         <v>1654</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13621,7 +13647,7 @@
       <c r="R152" t="s">
         <v>1866</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13656,7 +13682,7 @@
       <c r="J153" t="s">
         <v>1654</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13665,7 +13691,7 @@
       <c r="M153" t="s">
         <v>1743</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13706,7 +13732,7 @@
       <c r="J154" t="s">
         <v>1654</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13747,7 +13773,7 @@
       <c r="J155" t="s">
         <v>1654</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13788,7 +13814,7 @@
       <c r="J156" t="s">
         <v>1654</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13829,7 +13855,7 @@
       <c r="J157" t="s">
         <v>1654</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13870,7 +13896,7 @@
       <c r="J158" t="s">
         <v>1654</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13911,7 +13937,7 @@
       <c r="J159" t="s">
         <v>1654</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13952,7 +13978,7 @@
       <c r="J160" t="s">
         <v>1654</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13993,7 +14019,7 @@
       <c r="J161" t="s">
         <v>1654</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -14034,7 +14060,7 @@
       <c r="J162" t="s">
         <v>1654</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -14052,7 +14078,7 @@
       <c r="R162" t="s">
         <v>1852</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14087,7 +14113,7 @@
       <c r="J163" t="s">
         <v>1654</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14105,7 +14131,7 @@
       <c r="R163" t="s">
         <v>1849</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14140,7 +14166,7 @@
       <c r="J164" t="s">
         <v>1654</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14184,7 +14210,7 @@
       <c r="J165" t="s">
         <v>1654</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14225,7 +14251,7 @@
       <c r="J166" t="s">
         <v>1654</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14243,7 +14269,7 @@
       <c r="R166" t="s">
         <v>1867</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14278,7 +14304,7 @@
       <c r="J167" t="s">
         <v>1654</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14322,7 +14348,7 @@
       <c r="J168" t="s">
         <v>1654</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14366,7 +14392,7 @@
       <c r="J169" t="s">
         <v>1654</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14407,7 +14433,7 @@
       <c r="J170" t="s">
         <v>1654</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14448,7 +14474,7 @@
       <c r="J171" t="s">
         <v>1654</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14489,7 +14515,7 @@
       <c r="J172" t="s">
         <v>1654</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14530,7 +14556,7 @@
       <c r="J173" t="s">
         <v>1654</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14571,7 +14597,7 @@
       <c r="J174" t="s">
         <v>1654</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14612,7 +14638,7 @@
       <c r="J175" t="s">
         <v>1654</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14653,7 +14679,7 @@
       <c r="J176" t="s">
         <v>1654</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14694,7 +14720,7 @@
       <c r="J177" t="s">
         <v>1654</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14735,7 +14761,7 @@
       <c r="J178" t="s">
         <v>1654</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14753,7 +14779,7 @@
       <c r="R178" t="s">
         <v>1865</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14791,7 +14817,7 @@
       <c r="J179" t="s">
         <v>1654</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14800,7 +14826,7 @@
       <c r="M179" t="s">
         <v>1740</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14841,7 +14867,7 @@
       <c r="J180" t="s">
         <v>1654</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14882,7 +14908,7 @@
       <c r="J181" t="s">
         <v>1654</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14900,7 +14926,7 @@
       <c r="R181" t="s">
         <v>1849</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14935,7 +14961,7 @@
       <c r="J182" t="s">
         <v>1654</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14976,7 +15002,7 @@
       <c r="J183" t="s">
         <v>1654</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -15017,7 +15043,7 @@
       <c r="J184" t="s">
         <v>1654</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -15058,7 +15084,7 @@
       <c r="J185" t="s">
         <v>1654</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15099,7 +15125,7 @@
       <c r="J186" t="s">
         <v>1654</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15140,7 +15166,7 @@
       <c r="J187" t="s">
         <v>1654</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15181,7 +15207,7 @@
       <c r="J188" t="s">
         <v>1654</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15222,7 +15248,7 @@
       <c r="J189" t="s">
         <v>1654</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15263,7 +15289,7 @@
       <c r="J190" t="s">
         <v>1654</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15304,7 +15330,7 @@
       <c r="J191" t="s">
         <v>1654</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15345,7 +15371,7 @@
       <c r="J192" t="s">
         <v>1654</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15386,7 +15412,7 @@
       <c r="J193" t="s">
         <v>1654</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15427,7 +15453,7 @@
       <c r="J194" t="s">
         <v>1654</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15468,7 +15494,7 @@
       <c r="J195" t="s">
         <v>1654</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15486,7 +15512,7 @@
       <c r="R195" t="s">
         <v>1858</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15527,7 +15553,7 @@
       <c r="J196" t="s">
         <v>1654</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15545,7 +15571,7 @@
       <c r="R196" t="s">
         <v>1864</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15583,7 +15609,7 @@
       <c r="J197" t="s">
         <v>1654</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15624,7 +15650,7 @@
       <c r="J198" t="s">
         <v>1656</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15665,7 +15691,7 @@
       <c r="J199" t="s">
         <v>1655</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15706,7 +15732,7 @@
       <c r="J200" t="s">
         <v>1654</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15747,7 +15773,7 @@
       <c r="J201" t="s">
         <v>1654</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15788,7 +15814,7 @@
       <c r="J202" t="s">
         <v>1654</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15806,7 +15832,7 @@
       <c r="R202" t="s">
         <v>1849</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15844,7 +15870,7 @@
       <c r="J203" t="s">
         <v>1654</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15862,7 +15888,7 @@
       <c r="R203" t="s">
         <v>1857</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15897,7 +15923,7 @@
       <c r="J204" t="s">
         <v>1654</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15912,7 +15938,7 @@
       <c r="R204" t="s">
         <v>1868</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15950,7 +15976,7 @@
       <c r="J205" t="s">
         <v>1654</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15968,7 +15994,7 @@
       <c r="R205" t="s">
         <v>1869</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -16006,7 +16032,7 @@
       <c r="J206" t="s">
         <v>1654</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -16024,7 +16050,7 @@
       <c r="R206" t="s">
         <v>1837</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -16059,7 +16085,7 @@
       <c r="J207" t="s">
         <v>1654</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16100,7 +16126,7 @@
       <c r="J208" t="s">
         <v>1654</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16141,7 +16167,7 @@
       <c r="J209" t="s">
         <v>1654</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16182,7 +16208,7 @@
       <c r="J210" t="s">
         <v>1654</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16223,7 +16249,7 @@
       <c r="J211" t="s">
         <v>1654</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16264,7 +16290,7 @@
       <c r="J212" t="s">
         <v>1654</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16305,7 +16331,7 @@
       <c r="J213" t="s">
         <v>1654</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16346,7 +16372,7 @@
       <c r="J214" t="s">
         <v>1654</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16364,7 +16390,7 @@
       <c r="R214" t="s">
         <v>1870</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16402,7 +16428,7 @@
       <c r="J215" t="s">
         <v>1654</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16443,7 +16469,7 @@
       <c r="J216" t="s">
         <v>1654</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16484,7 +16510,7 @@
       <c r="J217" t="s">
         <v>1654</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16525,7 +16551,7 @@
       <c r="J218" t="s">
         <v>1654</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16566,7 +16592,7 @@
       <c r="J219" t="s">
         <v>1654</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16607,7 +16633,7 @@
       <c r="J220" t="s">
         <v>1654</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16648,7 +16674,7 @@
       <c r="J221" t="s">
         <v>1654</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16689,7 +16715,7 @@
       <c r="J222" t="s">
         <v>1654</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16730,7 +16756,7 @@
       <c r="J223" t="s">
         <v>1654</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16771,7 +16797,7 @@
       <c r="J224" t="s">
         <v>1654</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16812,7 +16838,7 @@
       <c r="J225" t="s">
         <v>1654</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16853,7 +16879,7 @@
       <c r="J226" t="s">
         <v>1654</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16894,7 +16920,7 @@
       <c r="J227" t="s">
         <v>1654</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16935,7 +16961,7 @@
       <c r="J228" t="s">
         <v>1654</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16976,7 +17002,7 @@
       <c r="J229" t="s">
         <v>1654</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -17017,7 +17043,7 @@
       <c r="J230" t="s">
         <v>1654</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -17058,7 +17084,7 @@
       <c r="J231" t="s">
         <v>1654</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17099,7 +17125,7 @@
       <c r="J232" t="s">
         <v>1654</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17140,7 +17166,7 @@
       <c r="J233" t="s">
         <v>1654</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17181,7 +17207,7 @@
       <c r="J234" t="s">
         <v>1654</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17222,7 +17248,7 @@
       <c r="J235" t="s">
         <v>1654</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17263,7 +17289,7 @@
       <c r="J236" t="s">
         <v>1654</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17304,7 +17330,7 @@
       <c r="J237" t="s">
         <v>1654</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17345,7 +17371,7 @@
       <c r="J238" t="s">
         <v>1654</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17386,7 +17412,7 @@
       <c r="J239" t="s">
         <v>1654</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17404,7 +17430,7 @@
       <c r="R239" t="s">
         <v>1864</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17442,7 +17468,7 @@
       <c r="J240" t="s">
         <v>1654</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17483,7 +17509,7 @@
       <c r="J241" t="s">
         <v>1654</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17524,7 +17550,7 @@
       <c r="J242" t="s">
         <v>1654</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17542,7 +17568,7 @@
       <c r="R242" t="s">
         <v>1857</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17577,7 +17603,7 @@
       <c r="J243" t="s">
         <v>1654</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17618,7 +17644,7 @@
       <c r="J244" t="s">
         <v>1654</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17659,7 +17685,7 @@
       <c r="J245" t="s">
         <v>1654</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17700,7 +17726,7 @@
       <c r="J246" t="s">
         <v>1654</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17718,7 +17744,7 @@
       <c r="R246" t="s">
         <v>1837</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17756,7 +17782,7 @@
       <c r="J247" t="s">
         <v>1654</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17797,7 +17823,7 @@
       <c r="J248" t="s">
         <v>1654</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17838,7 +17864,7 @@
       <c r="J249" t="s">
         <v>1654</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17879,7 +17905,7 @@
       <c r="J250" t="s">
         <v>1654</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17920,7 +17946,7 @@
       <c r="J251" t="s">
         <v>1654</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17961,7 +17987,7 @@
       <c r="J252" t="s">
         <v>1654</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -18002,7 +18028,7 @@
       <c r="J253" t="s">
         <v>1654</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -18020,7 +18046,7 @@
       <c r="R253" t="s">
         <v>1867</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18061,7 +18087,7 @@
       <c r="J254" t="s">
         <v>1654</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18102,7 +18128,7 @@
       <c r="J255" t="s">
         <v>1654</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18143,7 +18169,7 @@
       <c r="J256" t="s">
         <v>1654</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18152,7 +18178,7 @@
       <c r="M256" t="s">
         <v>1739</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18190,7 +18216,7 @@
       <c r="J257" t="s">
         <v>1654</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18199,7 +18225,7 @@
       <c r="M257" t="s">
         <v>1740</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18243,7 +18269,7 @@
       <c r="J258" t="s">
         <v>1654</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18261,7 +18287,7 @@
       <c r="R258" t="s">
         <v>1849</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18299,7 +18325,7 @@
       <c r="J259" t="s">
         <v>1654</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18317,7 +18343,7 @@
       <c r="R259" t="s">
         <v>1865</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18355,7 +18381,7 @@
       <c r="J260" t="s">
         <v>1654</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18364,7 +18390,7 @@
       <c r="M260" t="s">
         <v>1734</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18408,7 +18434,7 @@
       <c r="J261" t="s">
         <v>1654</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18426,7 +18452,7 @@
       <c r="R261" t="s">
         <v>1871</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18464,7 +18490,7 @@
       <c r="J262" t="s">
         <v>1654</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18482,7 +18508,7 @@
       <c r="R262" t="s">
         <v>1865</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18520,7 +18546,7 @@
       <c r="J263" t="s">
         <v>1654</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18529,7 +18555,7 @@
       <c r="M263" t="s">
         <v>1734</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18573,7 +18599,7 @@
       <c r="J264" t="s">
         <v>1654</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18614,7 +18640,7 @@
       <c r="J265" t="s">
         <v>1654</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18655,7 +18681,7 @@
       <c r="J266" t="s">
         <v>1654</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18696,7 +18722,7 @@
       <c r="J267" t="s">
         <v>1654</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18740,7 +18766,7 @@
       <c r="J268" t="s">
         <v>1654</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18781,7 +18807,7 @@
       <c r="J269" t="s">
         <v>1654</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18822,7 +18848,7 @@
       <c r="J270" t="s">
         <v>1654</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18863,7 +18889,7 @@
       <c r="J271" t="s">
         <v>1654</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18904,7 +18930,7 @@
       <c r="J272" t="s">
         <v>1654</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18922,7 +18948,7 @@
       <c r="R272" t="s">
         <v>1872</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18963,7 +18989,7 @@
       <c r="J273" t="s">
         <v>1654</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -19007,7 +19033,7 @@
       <c r="J274" t="s">
         <v>1654</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -19048,7 +19074,7 @@
       <c r="J275" t="s">
         <v>1654</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19089,7 +19115,7 @@
       <c r="J276" t="s">
         <v>1654</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19130,7 +19156,7 @@
       <c r="J277" t="s">
         <v>1654</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19171,7 +19197,7 @@
       <c r="J278" t="s">
         <v>1654</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19212,7 +19238,7 @@
       <c r="J279" t="s">
         <v>1654</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19253,7 +19279,7 @@
       <c r="J280" t="s">
         <v>1654</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19294,7 +19320,7 @@
       <c r="J281" t="s">
         <v>1654</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19335,7 +19361,7 @@
       <c r="J282" t="s">
         <v>1654</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19376,7 +19402,7 @@
       <c r="J283" t="s">
         <v>1654</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19417,7 +19443,7 @@
       <c r="J284" t="s">
         <v>1654</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19458,7 +19484,7 @@
       <c r="J285" t="s">
         <v>1654</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19499,7 +19525,7 @@
       <c r="J286" t="s">
         <v>1654</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19540,7 +19566,7 @@
       <c r="J287" t="s">
         <v>1654</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19581,7 +19607,7 @@
       <c r="J288" t="s">
         <v>1654</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19622,7 +19648,7 @@
       <c r="J289" t="s">
         <v>1654</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19663,7 +19689,7 @@
       <c r="J290" t="s">
         <v>1654</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19704,7 +19730,7 @@
       <c r="J291" t="s">
         <v>1654</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19745,7 +19771,7 @@
       <c r="J292" t="s">
         <v>1654</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19786,7 +19812,7 @@
       <c r="J293" t="s">
         <v>1654</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19827,7 +19853,7 @@
       <c r="J294" t="s">
         <v>1654</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19868,7 +19894,7 @@
       <c r="J295" t="s">
         <v>1654</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19886,7 +19912,7 @@
       <c r="R295" t="s">
         <v>1873</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19927,7 +19953,7 @@
       <c r="J296" t="s">
         <v>1654</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19945,7 +19971,7 @@
       <c r="R296" t="s">
         <v>1849</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19983,7 +20009,7 @@
       <c r="J297" t="s">
         <v>1654</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -20024,7 +20050,7 @@
       <c r="J298" t="s">
         <v>1654</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20065,7 +20091,7 @@
       <c r="J299" t="s">
         <v>1655</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20106,7 +20132,7 @@
       <c r="J300" t="s">
         <v>1654</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20147,7 +20173,7 @@
       <c r="J301" t="s">
         <v>1654</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20985,7 +21011,7 @@
       <c r="R321" t="s">
         <v>1835</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21208,7 +21234,7 @@
       <c r="R326" t="s">
         <v>1874</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -22043,7 +22069,7 @@
       <c r="R346" t="s">
         <v>1875</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (22/10/2026 12:53)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5813,16 +5813,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5838,7 +5830,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5846,30 +5838,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6169,73 +6143,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6270,7 +6244,7 @@
       <c r="J2" t="s">
         <v>1654</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6314,7 +6288,7 @@
       <c r="J3" t="s">
         <v>1654</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6358,7 +6332,7 @@
       <c r="J4" t="s">
         <v>1654</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6376,7 +6350,7 @@
       <c r="R4" t="s">
         <v>1832</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6414,7 +6388,7 @@
       <c r="J5" t="s">
         <v>1655</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6464,7 +6438,7 @@
       <c r="J6" t="s">
         <v>1654</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6511,7 +6485,7 @@
       <c r="J7" t="s">
         <v>1654</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6558,7 +6532,7 @@
       <c r="J8" t="s">
         <v>1654</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6605,7 +6579,7 @@
       <c r="J9" t="s">
         <v>1654</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6652,7 +6626,7 @@
       <c r="J10" t="s">
         <v>1654</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6699,7 +6673,7 @@
       <c r="J11" t="s">
         <v>1654</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6746,7 +6720,7 @@
       <c r="J12" t="s">
         <v>1654</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6790,7 +6764,7 @@
       <c r="J13" t="s">
         <v>1654</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6808,7 +6782,7 @@
       <c r="R13" t="s">
         <v>1833</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6846,7 +6820,7 @@
       <c r="J14" t="s">
         <v>1654</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6864,7 +6838,7 @@
       <c r="R14" t="s">
         <v>1834</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6905,7 +6879,7 @@
       <c r="J15" t="s">
         <v>1654</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6923,7 +6897,7 @@
       <c r="R15" t="s">
         <v>1834</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6964,7 +6938,7 @@
       <c r="J16" t="s">
         <v>1654</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -7008,7 +6982,7 @@
       <c r="J17" t="s">
         <v>1654</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -7052,7 +7026,7 @@
       <c r="J18" t="s">
         <v>1654</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -7070,7 +7044,7 @@
       <c r="R18" t="s">
         <v>1835</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7111,7 +7085,7 @@
       <c r="J19" t="s">
         <v>1654</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7155,7 +7129,7 @@
       <c r="J20" t="s">
         <v>1654</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7199,7 +7173,7 @@
       <c r="J21" t="s">
         <v>1654</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7217,7 +7191,7 @@
       <c r="R21" t="s">
         <v>1834</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7258,7 +7232,7 @@
       <c r="J22" t="s">
         <v>1654</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7276,7 +7250,7 @@
       <c r="R22" t="s">
         <v>1836</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7317,7 +7291,7 @@
       <c r="J23" t="s">
         <v>1654</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7335,7 +7309,7 @@
       <c r="R23" t="s">
         <v>1837</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7376,7 +7350,7 @@
       <c r="J24" t="s">
         <v>1654</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7420,7 +7394,7 @@
       <c r="J25" t="s">
         <v>1654</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7461,7 +7435,7 @@
       <c r="J26" t="s">
         <v>1656</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7479,7 +7453,7 @@
       <c r="R26" t="s">
         <v>1838</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7517,7 +7491,7 @@
       <c r="J27" t="s">
         <v>1654</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7535,7 +7509,7 @@
       <c r="R27" t="s">
         <v>1839</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7576,7 +7550,7 @@
       <c r="J28" t="s">
         <v>1654</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7620,7 +7594,7 @@
       <c r="J29" t="s">
         <v>1654</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7664,7 +7638,7 @@
       <c r="J30" t="s">
         <v>1654</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7708,7 +7682,7 @@
       <c r="J31" t="s">
         <v>1654</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7726,7 +7700,7 @@
       <c r="R31" t="s">
         <v>1840</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7767,7 +7741,7 @@
       <c r="J32" t="s">
         <v>1654</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7811,7 +7785,7 @@
       <c r="J33" t="s">
         <v>1654</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7829,7 +7803,7 @@
       <c r="R33" t="s">
         <v>1841</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7870,7 +7844,7 @@
       <c r="J34" t="s">
         <v>1654</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7914,7 +7888,7 @@
       <c r="J35" t="s">
         <v>1654</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7932,7 +7906,7 @@
       <c r="R35" t="s">
         <v>1842</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7973,7 +7947,7 @@
       <c r="J36" t="s">
         <v>1654</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7991,7 +7965,7 @@
       <c r="R36" t="s">
         <v>1842</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -8032,7 +8006,7 @@
       <c r="J37" t="s">
         <v>1654</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -8050,7 +8024,7 @@
       <c r="R37" t="s">
         <v>1842</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8091,7 +8065,7 @@
       <c r="J38" t="s">
         <v>1654</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8109,7 +8083,7 @@
       <c r="R38" t="s">
         <v>1842</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8150,7 +8124,7 @@
       <c r="J39" t="s">
         <v>1654</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8168,7 +8142,7 @@
       <c r="R39" t="s">
         <v>1842</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8209,7 +8183,7 @@
       <c r="J40" t="s">
         <v>1654</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8227,7 +8201,7 @@
       <c r="R40" t="s">
         <v>1843</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8268,7 +8242,7 @@
       <c r="J41" t="s">
         <v>1654</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8286,7 +8260,7 @@
       <c r="R41" t="s">
         <v>1834</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8327,7 +8301,7 @@
       <c r="J42" t="s">
         <v>1654</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8345,7 +8319,7 @@
       <c r="R42" t="s">
         <v>1842</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8386,7 +8360,7 @@
       <c r="J43" t="s">
         <v>1654</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8430,7 +8404,7 @@
       <c r="J44" t="s">
         <v>1654</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8448,7 +8422,7 @@
       <c r="R44" t="s">
         <v>1844</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8489,7 +8463,7 @@
       <c r="J45" t="s">
         <v>1654</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8507,7 +8481,7 @@
       <c r="R45" t="s">
         <v>1845</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8545,7 +8519,7 @@
       <c r="J46" t="s">
         <v>1654</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8589,7 +8563,7 @@
       <c r="J47" t="s">
         <v>1654</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8607,7 +8581,7 @@
       <c r="R47" t="s">
         <v>1846</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8648,7 +8622,7 @@
       <c r="J48" t="s">
         <v>1654</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8692,7 +8666,7 @@
       <c r="J49" t="s">
         <v>1654</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8736,7 +8710,7 @@
       <c r="J50" t="s">
         <v>1654</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8780,7 +8754,7 @@
       <c r="J51" t="s">
         <v>1654</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8827,7 +8801,7 @@
       <c r="J52" t="s">
         <v>1654</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8871,7 +8845,7 @@
       <c r="J53" t="s">
         <v>1654</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8915,7 +8889,7 @@
       <c r="J54" t="s">
         <v>1654</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8959,7 +8933,7 @@
       <c r="J55" t="s">
         <v>1654</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -9009,7 +8983,7 @@
       <c r="J56" t="s">
         <v>1654</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -9062,7 +9036,7 @@
       <c r="J57" t="s">
         <v>1654</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9112,7 +9086,7 @@
       <c r="J58" t="s">
         <v>1654</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9162,7 +9136,7 @@
       <c r="J59" t="s">
         <v>1654</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9180,7 +9154,7 @@
       <c r="R59" t="s">
         <v>1847</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9221,7 +9195,7 @@
       <c r="J60" t="s">
         <v>1654</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9265,7 +9239,7 @@
       <c r="J61" t="s">
         <v>1654</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9309,7 +9283,7 @@
       <c r="J62" t="s">
         <v>1654</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9353,7 +9327,7 @@
       <c r="J63" t="s">
         <v>1654</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9397,7 +9371,7 @@
       <c r="J64" t="s">
         <v>1654</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9441,7 +9415,7 @@
       <c r="J65" t="s">
         <v>1654</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9488,7 +9462,7 @@
       <c r="J66" t="s">
         <v>1654</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9506,7 +9480,7 @@
       <c r="R66" t="s">
         <v>1848</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9544,7 +9518,7 @@
       <c r="J67" t="s">
         <v>1654</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9588,7 +9562,7 @@
       <c r="J68" t="s">
         <v>1654</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9603,7 +9577,7 @@
       <c r="O68" t="s">
         <v>1752</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9647,7 +9621,7 @@
       <c r="J69" t="s">
         <v>1656</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9691,7 +9665,7 @@
       <c r="J70" t="s">
         <v>1654</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9735,7 +9709,7 @@
       <c r="J71" t="s">
         <v>1654</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9779,7 +9753,7 @@
       <c r="J72" t="s">
         <v>1654</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9823,7 +9797,7 @@
       <c r="J73" t="s">
         <v>1654</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9867,7 +9841,7 @@
       <c r="J74" t="s">
         <v>1654</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9911,7 +9885,7 @@
       <c r="J75" t="s">
         <v>1654</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9955,7 +9929,7 @@
       <c r="J76" t="s">
         <v>1654</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9973,7 +9947,7 @@
       <c r="R76" t="s">
         <v>1849</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -10011,7 +9985,7 @@
       <c r="J77" t="s">
         <v>1654</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -10029,7 +10003,7 @@
       <c r="R77" t="s">
         <v>1849</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -10067,7 +10041,7 @@
       <c r="J78" t="s">
         <v>1654</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -10085,7 +10059,7 @@
       <c r="R78" t="s">
         <v>1849</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10123,7 +10097,7 @@
       <c r="J79" t="s">
         <v>1654</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10141,7 +10115,7 @@
       <c r="R79" t="s">
         <v>1849</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10179,7 +10153,7 @@
       <c r="J80" t="s">
         <v>1654</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10223,7 +10197,7 @@
       <c r="J81" t="s">
         <v>1654</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10267,7 +10241,7 @@
       <c r="J82" t="s">
         <v>1654</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10311,7 +10285,7 @@
       <c r="J83" t="s">
         <v>1654</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10355,7 +10329,7 @@
       <c r="J84" t="s">
         <v>1654</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10399,7 +10373,7 @@
       <c r="J85" t="s">
         <v>1654</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10417,7 +10391,7 @@
       <c r="R85" t="s">
         <v>1850</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10455,7 +10429,7 @@
       <c r="J86" t="s">
         <v>1654</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10499,7 +10473,7 @@
       <c r="J87" t="s">
         <v>1654</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10517,7 +10491,7 @@
       <c r="R87" t="s">
         <v>1851</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10555,7 +10529,7 @@
       <c r="J88" t="s">
         <v>1654</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10599,7 +10573,7 @@
       <c r="J89" t="s">
         <v>1654</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10617,7 +10591,7 @@
       <c r="R89" t="s">
         <v>1852</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10652,7 +10626,7 @@
       <c r="J90" t="s">
         <v>1654</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10670,7 +10644,7 @@
       <c r="R90" t="s">
         <v>1853</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10705,7 +10679,7 @@
       <c r="J91" t="s">
         <v>1654</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10723,7 +10697,7 @@
       <c r="R91" t="s">
         <v>1837</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10761,7 +10735,7 @@
       <c r="J92" t="s">
         <v>1654</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10782,7 +10756,7 @@
       <c r="R92" t="s">
         <v>1837</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10823,7 +10797,7 @@
       <c r="J93" t="s">
         <v>1654</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10864,7 +10838,7 @@
       <c r="J94" t="s">
         <v>1654</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10908,7 +10882,7 @@
       <c r="J95" t="s">
         <v>1654</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10952,7 +10926,7 @@
       <c r="J96" t="s">
         <v>1654</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10970,7 +10944,7 @@
       <c r="R96" t="s">
         <v>1854</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -11011,7 +10985,7 @@
       <c r="J97" t="s">
         <v>1654</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -11026,7 +11000,7 @@
       <c r="R97" t="s">
         <v>1854</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -11067,7 +11041,7 @@
       <c r="J98" t="s">
         <v>1654</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -11085,7 +11059,7 @@
       <c r="R98" t="s">
         <v>1855</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11123,7 +11097,7 @@
       <c r="J99" t="s">
         <v>1654</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11141,7 +11115,7 @@
       <c r="R99" t="s">
         <v>1856</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11179,7 +11153,7 @@
       <c r="J100" t="s">
         <v>1654</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -11220,7 +11194,7 @@
       <c r="J101" t="s">
         <v>1654</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -11261,7 +11235,7 @@
       <c r="J102" t="s">
         <v>1654</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -11302,7 +11276,7 @@
       <c r="J103" t="s">
         <v>1654</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -11343,7 +11317,7 @@
       <c r="J104" t="s">
         <v>1654</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -11384,7 +11358,7 @@
       <c r="J105" t="s">
         <v>1654</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -11425,7 +11399,7 @@
       <c r="J106" t="s">
         <v>1654</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -11466,7 +11440,7 @@
       <c r="J107" t="s">
         <v>1654</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -11507,7 +11481,7 @@
       <c r="J108" t="s">
         <v>1654</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -11548,7 +11522,7 @@
       <c r="J109" t="s">
         <v>1654</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11601,7 +11575,7 @@
       <c r="J110" t="s">
         <v>1654</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11657,7 +11631,7 @@
       <c r="J111" t="s">
         <v>1654</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11675,7 +11649,7 @@
       <c r="R111" t="s">
         <v>1858</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11713,7 +11687,7 @@
       <c r="J112" t="s">
         <v>1654</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11772,7 +11746,7 @@
       <c r="J113" t="s">
         <v>1654</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11816,7 +11790,7 @@
       <c r="J114" t="s">
         <v>1654</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11860,7 +11834,7 @@
       <c r="J115" t="s">
         <v>1654</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11878,7 +11852,7 @@
       <c r="R115" t="s">
         <v>1860</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="U115" t="s">
@@ -11919,7 +11893,7 @@
       <c r="J116" t="s">
         <v>1654</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11978,7 +11952,7 @@
       <c r="J117" t="s">
         <v>1654</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -12022,7 +11996,7 @@
       <c r="J118" t="s">
         <v>1654</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -12069,7 +12043,7 @@
       <c r="J119" t="s">
         <v>1654</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -12110,7 +12084,7 @@
       <c r="J120" t="s">
         <v>1654</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -12154,7 +12128,7 @@
       <c r="J121" t="s">
         <v>1654</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -12201,7 +12175,7 @@
       <c r="J122" t="s">
         <v>1654</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -12251,7 +12225,7 @@
       <c r="J123" t="s">
         <v>1654</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -12295,7 +12269,7 @@
       <c r="J124" t="s">
         <v>1654</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -12339,7 +12313,7 @@
       <c r="J125" t="s">
         <v>1654</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -12357,7 +12331,7 @@
       <c r="R125" t="s">
         <v>1862</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -12392,7 +12366,7 @@
       <c r="J126" t="s">
         <v>1654</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -12410,7 +12384,7 @@
       <c r="R126" t="s">
         <v>1863</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="U126" t="s">
@@ -12448,7 +12422,7 @@
       <c r="J127" t="s">
         <v>1654</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -12504,7 +12478,7 @@
       <c r="J128" t="s">
         <v>1654</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -12545,7 +12519,7 @@
       <c r="J129" t="s">
         <v>1654</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12586,7 +12560,7 @@
       <c r="J130" t="s">
         <v>1654</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12627,7 +12601,7 @@
       <c r="J131" t="s">
         <v>1654</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12671,7 +12645,7 @@
       <c r="J132" t="s">
         <v>1654</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12712,7 +12686,7 @@
       <c r="J133" t="s">
         <v>1654</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12730,7 +12704,7 @@
       <c r="R133" t="s">
         <v>1849</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="U133" t="s">
@@ -12768,7 +12742,7 @@
       <c r="J134" t="s">
         <v>1654</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12786,7 +12760,7 @@
       <c r="R134" t="s">
         <v>1849</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12821,7 +12795,7 @@
       <c r="J135" t="s">
         <v>1654</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12862,7 +12836,7 @@
       <c r="J136" t="s">
         <v>1654</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12903,7 +12877,7 @@
       <c r="J137" t="s">
         <v>1654</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12944,7 +12918,7 @@
       <c r="J138" t="s">
         <v>1654</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12985,7 +12959,7 @@
       <c r="J139" t="s">
         <v>1654</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -13032,7 +13006,7 @@
       <c r="J140" t="s">
         <v>1654</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -13073,7 +13047,7 @@
       <c r="J141" t="s">
         <v>1654</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -13114,7 +13088,7 @@
       <c r="J142" t="s">
         <v>1654</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -13158,7 +13132,7 @@
       <c r="J143" t="s">
         <v>1654</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -13176,7 +13150,7 @@
       <c r="R143" t="s">
         <v>1849</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -13211,7 +13185,7 @@
       <c r="J144" t="s">
         <v>1654</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -13229,7 +13203,7 @@
       <c r="R144" t="s">
         <v>1849</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="U144" t="s">
@@ -13267,7 +13241,7 @@
       <c r="J145" t="s">
         <v>1654</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -13285,7 +13259,7 @@
       <c r="R145" t="s">
         <v>1849</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -13320,7 +13294,7 @@
       <c r="J146" t="s">
         <v>1654</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -13338,7 +13312,7 @@
       <c r="R146" t="s">
         <v>1857</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -13373,7 +13347,7 @@
       <c r="J147" t="s">
         <v>1654</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -13391,7 +13365,7 @@
       <c r="R147" t="s">
         <v>1864</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -13426,7 +13400,7 @@
       <c r="J148" t="s">
         <v>1654</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -13467,7 +13441,7 @@
       <c r="J149" t="s">
         <v>1654</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -13485,7 +13459,7 @@
       <c r="R149" t="s">
         <v>1849</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -13520,7 +13494,7 @@
       <c r="J150" t="s">
         <v>1654</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -13538,7 +13512,7 @@
       <c r="R150" t="s">
         <v>1849</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="U150" t="s">
@@ -13576,7 +13550,7 @@
       <c r="J151" t="s">
         <v>1654</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13594,7 +13568,7 @@
       <c r="R151" t="s">
         <v>1865</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13629,7 +13603,7 @@
       <c r="J152" t="s">
         <v>1654</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13647,7 +13621,7 @@
       <c r="R152" t="s">
         <v>1866</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13682,7 +13656,7 @@
       <c r="J153" t="s">
         <v>1654</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13691,7 +13665,7 @@
       <c r="M153" t="s">
         <v>1743</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13732,7 +13706,7 @@
       <c r="J154" t="s">
         <v>1654</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13773,7 +13747,7 @@
       <c r="J155" t="s">
         <v>1654</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13814,7 +13788,7 @@
       <c r="J156" t="s">
         <v>1654</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13855,7 +13829,7 @@
       <c r="J157" t="s">
         <v>1654</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13896,7 +13870,7 @@
       <c r="J158" t="s">
         <v>1654</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13937,7 +13911,7 @@
       <c r="J159" t="s">
         <v>1654</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13978,7 +13952,7 @@
       <c r="J160" t="s">
         <v>1654</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -14019,7 +13993,7 @@
       <c r="J161" t="s">
         <v>1654</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -14060,7 +14034,7 @@
       <c r="J162" t="s">
         <v>1654</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -14078,7 +14052,7 @@
       <c r="R162" t="s">
         <v>1852</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -14113,7 +14087,7 @@
       <c r="J163" t="s">
         <v>1654</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -14131,7 +14105,7 @@
       <c r="R163" t="s">
         <v>1849</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -14166,7 +14140,7 @@
       <c r="J164" t="s">
         <v>1654</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -14210,7 +14184,7 @@
       <c r="J165" t="s">
         <v>1654</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -14251,7 +14225,7 @@
       <c r="J166" t="s">
         <v>1654</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -14269,7 +14243,7 @@
       <c r="R166" t="s">
         <v>1867</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -14304,7 +14278,7 @@
       <c r="J167" t="s">
         <v>1654</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -14348,7 +14322,7 @@
       <c r="J168" t="s">
         <v>1654</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -14392,7 +14366,7 @@
       <c r="J169" t="s">
         <v>1654</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -14433,7 +14407,7 @@
       <c r="J170" t="s">
         <v>1654</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -14474,7 +14448,7 @@
       <c r="J171" t="s">
         <v>1654</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -14515,7 +14489,7 @@
       <c r="J172" t="s">
         <v>1654</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -14556,7 +14530,7 @@
       <c r="J173" t="s">
         <v>1654</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14597,7 +14571,7 @@
       <c r="J174" t="s">
         <v>1654</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14638,7 +14612,7 @@
       <c r="J175" t="s">
         <v>1654</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14679,7 +14653,7 @@
       <c r="J176" t="s">
         <v>1654</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14720,7 +14694,7 @@
       <c r="J177" t="s">
         <v>1654</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14761,7 +14735,7 @@
       <c r="J178" t="s">
         <v>1654</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14779,7 +14753,7 @@
       <c r="R178" t="s">
         <v>1865</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="U178" t="s">
@@ -14817,7 +14791,7 @@
       <c r="J179" t="s">
         <v>1654</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14826,7 +14800,7 @@
       <c r="M179" t="s">
         <v>1740</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14867,7 +14841,7 @@
       <c r="J180" t="s">
         <v>1654</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14908,7 +14882,7 @@
       <c r="J181" t="s">
         <v>1654</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14926,7 +14900,7 @@
       <c r="R181" t="s">
         <v>1849</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14961,7 +14935,7 @@
       <c r="J182" t="s">
         <v>1654</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -15002,7 +14976,7 @@
       <c r="J183" t="s">
         <v>1654</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -15043,7 +15017,7 @@
       <c r="J184" t="s">
         <v>1654</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -15084,7 +15058,7 @@
       <c r="J185" t="s">
         <v>1654</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -15125,7 +15099,7 @@
       <c r="J186" t="s">
         <v>1654</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -15166,7 +15140,7 @@
       <c r="J187" t="s">
         <v>1654</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -15207,7 +15181,7 @@
       <c r="J188" t="s">
         <v>1654</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -15248,7 +15222,7 @@
       <c r="J189" t="s">
         <v>1654</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -15289,7 +15263,7 @@
       <c r="J190" t="s">
         <v>1654</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -15330,7 +15304,7 @@
       <c r="J191" t="s">
         <v>1654</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -15371,7 +15345,7 @@
       <c r="J192" t="s">
         <v>1654</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -15412,7 +15386,7 @@
       <c r="J193" t="s">
         <v>1654</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -15453,7 +15427,7 @@
       <c r="J194" t="s">
         <v>1654</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -15494,7 +15468,7 @@
       <c r="J195" t="s">
         <v>1654</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -15512,7 +15486,7 @@
       <c r="R195" t="s">
         <v>1858</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="U195" t="s">
@@ -15553,7 +15527,7 @@
       <c r="J196" t="s">
         <v>1654</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -15571,7 +15545,7 @@
       <c r="R196" t="s">
         <v>1864</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15609,7 +15583,7 @@
       <c r="J197" t="s">
         <v>1654</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15650,7 +15624,7 @@
       <c r="J198" t="s">
         <v>1656</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15691,7 +15665,7 @@
       <c r="J199" t="s">
         <v>1655</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15732,7 +15706,7 @@
       <c r="J200" t="s">
         <v>1654</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15773,7 +15747,7 @@
       <c r="J201" t="s">
         <v>1654</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15814,7 +15788,7 @@
       <c r="J202" t="s">
         <v>1654</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15832,7 +15806,7 @@
       <c r="R202" t="s">
         <v>1849</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="U202" t="s">
@@ -15870,7 +15844,7 @@
       <c r="J203" t="s">
         <v>1654</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15888,7 +15862,7 @@
       <c r="R203" t="s">
         <v>1857</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15923,7 +15897,7 @@
       <c r="J204" t="s">
         <v>1654</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15938,7 +15912,7 @@
       <c r="R204" t="s">
         <v>1868</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15976,7 +15950,7 @@
       <c r="J205" t="s">
         <v>1654</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15994,7 +15968,7 @@
       <c r="R205" t="s">
         <v>1869</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -16032,7 +16006,7 @@
       <c r="J206" t="s">
         <v>1654</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -16050,7 +16024,7 @@
       <c r="R206" t="s">
         <v>1837</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -16085,7 +16059,7 @@
       <c r="J207" t="s">
         <v>1654</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -16126,7 +16100,7 @@
       <c r="J208" t="s">
         <v>1654</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -16167,7 +16141,7 @@
       <c r="J209" t="s">
         <v>1654</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -16208,7 +16182,7 @@
       <c r="J210" t="s">
         <v>1654</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -16249,7 +16223,7 @@
       <c r="J211" t="s">
         <v>1654</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -16290,7 +16264,7 @@
       <c r="J212" t="s">
         <v>1654</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -16331,7 +16305,7 @@
       <c r="J213" t="s">
         <v>1654</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -16372,7 +16346,7 @@
       <c r="J214" t="s">
         <v>1654</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -16390,7 +16364,7 @@
       <c r="R214" t="s">
         <v>1870</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="U214" t="s">
@@ -16428,7 +16402,7 @@
       <c r="J215" t="s">
         <v>1654</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -16469,7 +16443,7 @@
       <c r="J216" t="s">
         <v>1654</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -16510,7 +16484,7 @@
       <c r="J217" t="s">
         <v>1654</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -16551,7 +16525,7 @@
       <c r="J218" t="s">
         <v>1654</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -16592,7 +16566,7 @@
       <c r="J219" t="s">
         <v>1654</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16633,7 +16607,7 @@
       <c r="J220" t="s">
         <v>1654</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16674,7 +16648,7 @@
       <c r="J221" t="s">
         <v>1654</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16715,7 +16689,7 @@
       <c r="J222" t="s">
         <v>1654</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16756,7 +16730,7 @@
       <c r="J223" t="s">
         <v>1654</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16797,7 +16771,7 @@
       <c r="J224" t="s">
         <v>1654</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16838,7 +16812,7 @@
       <c r="J225" t="s">
         <v>1654</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16879,7 +16853,7 @@
       <c r="J226" t="s">
         <v>1654</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16920,7 +16894,7 @@
       <c r="J227" t="s">
         <v>1654</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16961,7 +16935,7 @@
       <c r="J228" t="s">
         <v>1654</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -17002,7 +16976,7 @@
       <c r="J229" t="s">
         <v>1654</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -17043,7 +17017,7 @@
       <c r="J230" t="s">
         <v>1654</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -17084,7 +17058,7 @@
       <c r="J231" t="s">
         <v>1654</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -17125,7 +17099,7 @@
       <c r="J232" t="s">
         <v>1654</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -17166,7 +17140,7 @@
       <c r="J233" t="s">
         <v>1654</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -17207,7 +17181,7 @@
       <c r="J234" t="s">
         <v>1654</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -17248,7 +17222,7 @@
       <c r="J235" t="s">
         <v>1654</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -17289,7 +17263,7 @@
       <c r="J236" t="s">
         <v>1654</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -17330,7 +17304,7 @@
       <c r="J237" t="s">
         <v>1654</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -17371,7 +17345,7 @@
       <c r="J238" t="s">
         <v>1654</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -17412,7 +17386,7 @@
       <c r="J239" t="s">
         <v>1654</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -17430,7 +17404,7 @@
       <c r="R239" t="s">
         <v>1864</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="U239" t="s">
@@ -17468,7 +17442,7 @@
       <c r="J240" t="s">
         <v>1654</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -17509,7 +17483,7 @@
       <c r="J241" t="s">
         <v>1654</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -17550,7 +17524,7 @@
       <c r="J242" t="s">
         <v>1654</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -17568,7 +17542,7 @@
       <c r="R242" t="s">
         <v>1857</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17603,7 +17577,7 @@
       <c r="J243" t="s">
         <v>1654</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17644,7 +17618,7 @@
       <c r="J244" t="s">
         <v>1654</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17685,7 +17659,7 @@
       <c r="J245" t="s">
         <v>1654</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17726,7 +17700,7 @@
       <c r="J246" t="s">
         <v>1654</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17744,7 +17718,7 @@
       <c r="R246" t="s">
         <v>1837</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="U246" t="s">
@@ -17782,7 +17756,7 @@
       <c r="J247" t="s">
         <v>1654</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17823,7 +17797,7 @@
       <c r="J248" t="s">
         <v>1654</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17864,7 +17838,7 @@
       <c r="J249" t="s">
         <v>1654</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17905,7 +17879,7 @@
       <c r="J250" t="s">
         <v>1654</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17946,7 +17920,7 @@
       <c r="J251" t="s">
         <v>1654</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17987,7 +17961,7 @@
       <c r="J252" t="s">
         <v>1654</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -18028,7 +18002,7 @@
       <c r="J253" t="s">
         <v>1654</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -18046,7 +18020,7 @@
       <c r="R253" t="s">
         <v>1867</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="U253" t="s">
@@ -18087,7 +18061,7 @@
       <c r="J254" t="s">
         <v>1654</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -18128,7 +18102,7 @@
       <c r="J255" t="s">
         <v>1654</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -18169,7 +18143,7 @@
       <c r="J256" t="s">
         <v>1654</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -18178,7 +18152,7 @@
       <c r="M256" t="s">
         <v>1739</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -18216,7 +18190,7 @@
       <c r="J257" t="s">
         <v>1654</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -18225,7 +18199,7 @@
       <c r="M257" t="s">
         <v>1740</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -18269,7 +18243,7 @@
       <c r="J258" t="s">
         <v>1654</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -18287,7 +18261,7 @@
       <c r="R258" t="s">
         <v>1849</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -18325,7 +18299,7 @@
       <c r="J259" t="s">
         <v>1654</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -18343,7 +18317,7 @@
       <c r="R259" t="s">
         <v>1865</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -18381,7 +18355,7 @@
       <c r="J260" t="s">
         <v>1654</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -18390,7 +18364,7 @@
       <c r="M260" t="s">
         <v>1734</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -18434,7 +18408,7 @@
       <c r="J261" t="s">
         <v>1654</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -18452,7 +18426,7 @@
       <c r="R261" t="s">
         <v>1871</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -18490,7 +18464,7 @@
       <c r="J262" t="s">
         <v>1654</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -18508,7 +18482,7 @@
       <c r="R262" t="s">
         <v>1865</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -18546,7 +18520,7 @@
       <c r="J263" t="s">
         <v>1654</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -18555,7 +18529,7 @@
       <c r="M263" t="s">
         <v>1734</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -18599,7 +18573,7 @@
       <c r="J264" t="s">
         <v>1654</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18640,7 +18614,7 @@
       <c r="J265" t="s">
         <v>1654</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18681,7 +18655,7 @@
       <c r="J266" t="s">
         <v>1654</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18722,7 +18696,7 @@
       <c r="J267" t="s">
         <v>1654</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18766,7 +18740,7 @@
       <c r="J268" t="s">
         <v>1654</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18807,7 +18781,7 @@
       <c r="J269" t="s">
         <v>1654</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18848,7 +18822,7 @@
       <c r="J270" t="s">
         <v>1654</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18889,7 +18863,7 @@
       <c r="J271" t="s">
         <v>1654</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18930,7 +18904,7 @@
       <c r="J272" t="s">
         <v>1654</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18948,7 +18922,7 @@
       <c r="R272" t="s">
         <v>1872</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="U272" t="s">
@@ -18989,7 +18963,7 @@
       <c r="J273" t="s">
         <v>1654</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -19033,7 +19007,7 @@
       <c r="J274" t="s">
         <v>1654</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -19074,7 +19048,7 @@
       <c r="J275" t="s">
         <v>1654</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -19115,7 +19089,7 @@
       <c r="J276" t="s">
         <v>1654</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -19156,7 +19130,7 @@
       <c r="J277" t="s">
         <v>1654</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -19197,7 +19171,7 @@
       <c r="J278" t="s">
         <v>1654</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -19238,7 +19212,7 @@
       <c r="J279" t="s">
         <v>1654</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -19279,7 +19253,7 @@
       <c r="J280" t="s">
         <v>1654</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -19320,7 +19294,7 @@
       <c r="J281" t="s">
         <v>1654</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -19361,7 +19335,7 @@
       <c r="J282" t="s">
         <v>1654</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -19402,7 +19376,7 @@
       <c r="J283" t="s">
         <v>1654</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -19443,7 +19417,7 @@
       <c r="J284" t="s">
         <v>1654</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -19484,7 +19458,7 @@
       <c r="J285" t="s">
         <v>1654</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -19525,7 +19499,7 @@
       <c r="J286" t="s">
         <v>1654</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -19566,7 +19540,7 @@
       <c r="J287" t="s">
         <v>1654</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19607,7 +19581,7 @@
       <c r="J288" t="s">
         <v>1654</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19648,7 +19622,7 @@
       <c r="J289" t="s">
         <v>1654</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19689,7 +19663,7 @@
       <c r="J290" t="s">
         <v>1654</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19730,7 +19704,7 @@
       <c r="J291" t="s">
         <v>1654</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19771,7 +19745,7 @@
       <c r="J292" t="s">
         <v>1654</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19812,7 +19786,7 @@
       <c r="J293" t="s">
         <v>1654</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19853,7 +19827,7 @@
       <c r="J294" t="s">
         <v>1654</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19894,7 +19868,7 @@
       <c r="J295" t="s">
         <v>1654</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19912,7 +19886,7 @@
       <c r="R295" t="s">
         <v>1873</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="U295" t="s">
@@ -19953,7 +19927,7 @@
       <c r="J296" t="s">
         <v>1654</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19971,7 +19945,7 @@
       <c r="R296" t="s">
         <v>1849</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -20009,7 +19983,7 @@
       <c r="J297" t="s">
         <v>1654</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -20050,7 +20024,7 @@
       <c r="J298" t="s">
         <v>1654</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -20091,7 +20065,7 @@
       <c r="J299" t="s">
         <v>1655</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -20132,7 +20106,7 @@
       <c r="J300" t="s">
         <v>1654</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -20173,7 +20147,7 @@
       <c r="J301" t="s">
         <v>1654</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -21011,7 +20985,7 @@
       <c r="R321" t="s">
         <v>1835</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="U321" t="s">
@@ -21234,7 +21208,7 @@
       <c r="R326" t="s">
         <v>1874</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -22069,7 +22043,7 @@
       <c r="R346" t="s">
         <v>1875</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (23/10/2026 14:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5828,8 +5828,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5845,7 +5853,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5853,12 +5861,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6158,73 +6184,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6259,7 +6285,7 @@
       <c r="J2" t="s">
         <v>1658</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -6303,7 +6329,7 @@
       <c r="J3" t="s">
         <v>1658</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -6347,7 +6373,7 @@
       <c r="J4" t="s">
         <v>1658</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -6365,7 +6391,7 @@
       <c r="R4" t="s">
         <v>1837</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -6403,7 +6429,7 @@
       <c r="J5" t="s">
         <v>1659</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -6453,7 +6479,7 @@
       <c r="J6" t="s">
         <v>1658</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -6500,7 +6526,7 @@
       <c r="J7" t="s">
         <v>1658</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6547,7 +6573,7 @@
       <c r="J8" t="s">
         <v>1658</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6594,7 +6620,7 @@
       <c r="J9" t="s">
         <v>1658</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6641,7 +6667,7 @@
       <c r="J10" t="s">
         <v>1658</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6688,7 +6714,7 @@
       <c r="J11" t="s">
         <v>1658</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6735,7 +6761,7 @@
       <c r="J12" t="s">
         <v>1658</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6779,7 +6805,7 @@
       <c r="J13" t="s">
         <v>1658</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6797,7 +6823,7 @@
       <c r="R13" t="s">
         <v>1838</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6835,7 +6861,7 @@
       <c r="J14" t="s">
         <v>1658</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6853,7 +6879,7 @@
       <c r="R14" t="s">
         <v>1839</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="U14" t="s">
@@ -6894,7 +6920,7 @@
       <c r="J15" t="s">
         <v>1658</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6912,7 +6938,7 @@
       <c r="R15" t="s">
         <v>1839</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="U15" t="s">
@@ -6953,7 +6979,7 @@
       <c r="J16" t="s">
         <v>1658</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6997,7 +7023,7 @@
       <c r="J17" t="s">
         <v>1658</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -7041,7 +7067,7 @@
       <c r="J18" t="s">
         <v>1658</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -7059,7 +7085,7 @@
       <c r="R18" t="s">
         <v>1840</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -7100,7 +7126,7 @@
       <c r="J19" t="s">
         <v>1658</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -7144,7 +7170,7 @@
       <c r="J20" t="s">
         <v>1658</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -7188,7 +7214,7 @@
       <c r="J21" t="s">
         <v>1658</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -7206,7 +7232,7 @@
       <c r="R21" t="s">
         <v>1839</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -7247,7 +7273,7 @@
       <c r="J22" t="s">
         <v>1658</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -7265,7 +7291,7 @@
       <c r="R22" t="s">
         <v>1841</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -7306,7 +7332,7 @@
       <c r="J23" t="s">
         <v>1658</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -7324,7 +7350,7 @@
       <c r="R23" t="s">
         <v>1842</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -7365,7 +7391,7 @@
       <c r="J24" t="s">
         <v>1658</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -7409,7 +7435,7 @@
       <c r="J25" t="s">
         <v>1658</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -7450,7 +7476,7 @@
       <c r="J26" t="s">
         <v>1660</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -7468,7 +7494,7 @@
       <c r="R26" t="s">
         <v>1843</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="U26" t="s">
@@ -7506,7 +7532,7 @@
       <c r="J27" t="s">
         <v>1658</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -7524,7 +7550,7 @@
       <c r="R27" t="s">
         <v>1844</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7565,7 +7591,7 @@
       <c r="J28" t="s">
         <v>1658</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7609,7 +7635,7 @@
       <c r="J29" t="s">
         <v>1658</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7653,7 +7679,7 @@
       <c r="J30" t="s">
         <v>1658</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7697,7 +7723,7 @@
       <c r="J31" t="s">
         <v>1658</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7715,7 +7741,7 @@
       <c r="R31" t="s">
         <v>1845</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7756,7 +7782,7 @@
       <c r="J32" t="s">
         <v>1658</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7800,7 +7826,7 @@
       <c r="J33" t="s">
         <v>1658</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7818,7 +7844,7 @@
       <c r="R33" t="s">
         <v>1846</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7859,7 +7885,7 @@
       <c r="J34" t="s">
         <v>1658</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7903,7 +7929,7 @@
       <c r="J35" t="s">
         <v>1658</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7921,7 +7947,7 @@
       <c r="R35" t="s">
         <v>1847</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7962,7 +7988,7 @@
       <c r="J36" t="s">
         <v>1658</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7980,7 +8006,7 @@
       <c r="R36" t="s">
         <v>1847</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -8021,7 +8047,7 @@
       <c r="J37" t="s">
         <v>1658</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -8039,7 +8065,7 @@
       <c r="R37" t="s">
         <v>1847</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -8080,7 +8106,7 @@
       <c r="J38" t="s">
         <v>1658</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -8098,7 +8124,7 @@
       <c r="R38" t="s">
         <v>1847</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -8139,7 +8165,7 @@
       <c r="J39" t="s">
         <v>1658</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -8157,7 +8183,7 @@
       <c r="R39" t="s">
         <v>1847</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -8198,7 +8224,7 @@
       <c r="J40" t="s">
         <v>1658</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -8216,7 +8242,7 @@
       <c r="R40" t="s">
         <v>1848</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -8257,7 +8283,7 @@
       <c r="J41" t="s">
         <v>1658</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -8275,7 +8301,7 @@
       <c r="R41" t="s">
         <v>1839</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="U41" t="s">
@@ -8316,7 +8342,7 @@
       <c r="J42" t="s">
         <v>1658</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -8334,7 +8360,7 @@
       <c r="R42" t="s">
         <v>1847</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -8375,7 +8401,7 @@
       <c r="J43" t="s">
         <v>1658</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -8419,7 +8445,7 @@
       <c r="J44" t="s">
         <v>1658</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -8437,7 +8463,7 @@
       <c r="R44" t="s">
         <v>1849</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -8478,7 +8504,7 @@
       <c r="J45" t="s">
         <v>1658</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -8496,7 +8522,7 @@
       <c r="R45" t="s">
         <v>1850</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -8534,7 +8560,7 @@
       <c r="J46" t="s">
         <v>1658</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8578,7 +8604,7 @@
       <c r="J47" t="s">
         <v>1658</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8596,7 +8622,7 @@
       <c r="R47" t="s">
         <v>1851</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8637,7 +8663,7 @@
       <c r="J48" t="s">
         <v>1658</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8681,7 +8707,7 @@
       <c r="J49" t="s">
         <v>1658</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8725,7 +8751,7 @@
       <c r="J50" t="s">
         <v>1658</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8769,7 +8795,7 @@
       <c r="J51" t="s">
         <v>1658</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8816,7 +8842,7 @@
       <c r="J52" t="s">
         <v>1658</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8860,7 +8886,7 @@
       <c r="J53" t="s">
         <v>1658</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8904,7 +8930,7 @@
       <c r="J54" t="s">
         <v>1658</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8948,7 +8974,7 @@
       <c r="J55" t="s">
         <v>1658</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8998,7 +9024,7 @@
       <c r="J56" t="s">
         <v>1658</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -9051,7 +9077,7 @@
       <c r="J57" t="s">
         <v>1658</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -9101,7 +9127,7 @@
       <c r="J58" t="s">
         <v>1658</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -9151,7 +9177,7 @@
       <c r="J59" t="s">
         <v>1658</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -9169,7 +9195,7 @@
       <c r="R59" t="s">
         <v>1852</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -9210,7 +9236,7 @@
       <c r="J60" t="s">
         <v>1658</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -9254,7 +9280,7 @@
       <c r="J61" t="s">
         <v>1658</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -9298,7 +9324,7 @@
       <c r="J62" t="s">
         <v>1658</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -9342,7 +9368,7 @@
       <c r="J63" t="s">
         <v>1658</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -9386,7 +9412,7 @@
       <c r="J64" t="s">
         <v>1658</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -9430,7 +9456,7 @@
       <c r="J65" t="s">
         <v>1658</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -9477,7 +9503,7 @@
       <c r="J66" t="s">
         <v>1658</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -9495,7 +9521,7 @@
       <c r="R66" t="s">
         <v>1853</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -9533,7 +9559,7 @@
       <c r="J67" t="s">
         <v>1658</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9577,7 +9603,7 @@
       <c r="J68" t="s">
         <v>1658</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9592,7 +9618,7 @@
       <c r="O68" t="s">
         <v>1757</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9636,7 +9662,7 @@
       <c r="J69" t="s">
         <v>1660</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9680,7 +9706,7 @@
       <c r="J70" t="s">
         <v>1658</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9724,7 +9750,7 @@
       <c r="J71" t="s">
         <v>1658</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9768,7 +9794,7 @@
       <c r="J72" t="s">
         <v>1658</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9812,7 +9838,7 @@
       <c r="J73" t="s">
         <v>1658</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9856,7 +9882,7 @@
       <c r="J74" t="s">
         <v>1658</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9900,7 +9926,7 @@
       <c r="J75" t="s">
         <v>1658</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9944,7 +9970,7 @@
       <c r="J76" t="s">
         <v>1658</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9962,7 +9988,7 @@
       <c r="R76" t="s">
         <v>1854</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -10000,7 +10026,7 @@
       <c r="J77" t="s">
         <v>1658</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -10018,7 +10044,7 @@
       <c r="R77" t="s">
         <v>1854</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -10056,7 +10082,7 @@
       <c r="J78" t="s">
         <v>1658</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -10074,7 +10100,7 @@
       <c r="R78" t="s">
         <v>1854</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -10112,7 +10138,7 @@
       <c r="J79" t="s">
         <v>1658</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -10130,7 +10156,7 @@
       <c r="R79" t="s">
         <v>1854</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -10168,7 +10194,7 @@
       <c r="J80" t="s">
         <v>1658</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -10212,7 +10238,7 @@
       <c r="J81" t="s">
         <v>1658</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -10256,7 +10282,7 @@
       <c r="J82" t="s">
         <v>1658</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -10300,7 +10326,7 @@
       <c r="J83" t="s">
         <v>1658</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -10344,7 +10370,7 @@
       <c r="J84" t="s">
         <v>1658</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -10388,7 +10414,7 @@
       <c r="J85" t="s">
         <v>1658</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -10406,7 +10432,7 @@
       <c r="R85" t="s">
         <v>1855</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -10444,7 +10470,7 @@
       <c r="J86" t="s">
         <v>1658</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -10488,7 +10514,7 @@
       <c r="J87" t="s">
         <v>1658</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -10506,7 +10532,7 @@
       <c r="R87" t="s">
         <v>1856</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -10544,7 +10570,7 @@
       <c r="J88" t="s">
         <v>1658</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10588,7 +10614,7 @@
       <c r="J89" t="s">
         <v>1658</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10606,7 +10632,7 @@
       <c r="R89" t="s">
         <v>1857</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10641,7 +10667,7 @@
       <c r="J90" t="s">
         <v>1658</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10659,7 +10685,7 @@
       <c r="R90" t="s">
         <v>1858</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10694,7 +10720,7 @@
       <c r="J91" t="s">
         <v>1658</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10712,7 +10738,7 @@
       <c r="R91" t="s">
         <v>1842</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10750,7 +10776,7 @@
       <c r="J92" t="s">
         <v>1658</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10771,7 +10797,7 @@
       <c r="R92" t="s">
         <v>1842</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10812,7 +10838,7 @@
       <c r="J93" t="s">
         <v>1658</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10853,7 +10879,7 @@
       <c r="J94" t="s">
         <v>1658</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10897,7 +10923,7 @@
       <c r="J95" t="s">
         <v>1658</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10941,7 +10967,7 @@
       <c r="J96" t="s">
         <v>1658</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10959,7 +10985,7 @@
       <c r="R96" t="s">
         <v>1859</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="U96" t="s">
@@ -11000,7 +11026,7 @@
       <c r="J97" t="s">
         <v>1658</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -11015,7 +11041,7 @@
       <c r="R97" t="s">
         <v>1859</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -11056,7 +11082,7 @@
       <c r="J98" t="s">
         <v>1658</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -11074,7 +11100,7 @@
       <c r="R98" t="s">
         <v>1860</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -11112,7 +11138,7 @@
       <c r="J99" t="s">
         <v>1658</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -11130,7 +11156,7 @@
       <c r="R99" t="s">
         <v>1861</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -11168,7 +11194,7 @@
       <c r="J100" t="s">
         <v>1658</v>
       </c>
-      <c r="K100" s="1